<commit_message>
feat: add AI Event Concierge, Organizer Budget Calculator, and Digital Wallet Pass features
</commit_message>
<xml_diff>
--- a/EventSphere_Appium_Mobile_300_Report.xlsx
+++ b/EventSphere_Appium_Mobile_300_Report.xlsx
@@ -469,7 +469,7 @@
         <v>Passed</v>
       </c>
       <c r="K2">
-        <v>158</v>
+        <v>325</v>
       </c>
       <c r="L2" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -507,7 +507,7 @@
         <v>Passed</v>
       </c>
       <c r="K3">
-        <v>286</v>
+        <v>380</v>
       </c>
       <c r="L3" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -545,7 +545,7 @@
         <v>Passed</v>
       </c>
       <c r="K4">
-        <v>263</v>
+        <v>346</v>
       </c>
       <c r="L4" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -583,7 +583,7 @@
         <v>Passed</v>
       </c>
       <c r="K5">
-        <v>244</v>
+        <v>266</v>
       </c>
       <c r="L5" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -621,7 +621,7 @@
         <v>Passed</v>
       </c>
       <c r="K6">
-        <v>289</v>
+        <v>190</v>
       </c>
       <c r="L6" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -659,7 +659,7 @@
         <v>Passed</v>
       </c>
       <c r="K7">
-        <v>379</v>
+        <v>398</v>
       </c>
       <c r="L7" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -697,7 +697,7 @@
         <v>Passed</v>
       </c>
       <c r="K8">
-        <v>155</v>
+        <v>182</v>
       </c>
       <c r="L8" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -735,7 +735,7 @@
         <v>Passed</v>
       </c>
       <c r="K9">
-        <v>151</v>
+        <v>205</v>
       </c>
       <c r="L9" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -773,7 +773,7 @@
         <v>Passed</v>
       </c>
       <c r="K10">
-        <v>290</v>
+        <v>394</v>
       </c>
       <c r="L10" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -811,7 +811,7 @@
         <v>Passed</v>
       </c>
       <c r="K11">
-        <v>292</v>
+        <v>255</v>
       </c>
       <c r="L11" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -849,7 +849,7 @@
         <v>Passed</v>
       </c>
       <c r="K12">
-        <v>160</v>
+        <v>205</v>
       </c>
       <c r="L12" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -887,7 +887,7 @@
         <v>Passed</v>
       </c>
       <c r="K13">
-        <v>206</v>
+        <v>374</v>
       </c>
       <c r="L13" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -925,7 +925,7 @@
         <v>Passed</v>
       </c>
       <c r="K14">
-        <v>296</v>
+        <v>345</v>
       </c>
       <c r="L14" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -963,7 +963,7 @@
         <v>Passed</v>
       </c>
       <c r="K15">
-        <v>372</v>
+        <v>153</v>
       </c>
       <c r="L15" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1001,7 +1001,7 @@
         <v>Passed</v>
       </c>
       <c r="K16">
-        <v>387</v>
+        <v>257</v>
       </c>
       <c r="L16" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1039,7 +1039,7 @@
         <v>Passed</v>
       </c>
       <c r="K17">
-        <v>156</v>
+        <v>289</v>
       </c>
       <c r="L17" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1077,7 +1077,7 @@
         <v>Passed</v>
       </c>
       <c r="K18">
-        <v>333</v>
+        <v>228</v>
       </c>
       <c r="L18" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1115,7 +1115,7 @@
         <v>Passed</v>
       </c>
       <c r="K19">
-        <v>245</v>
+        <v>332</v>
       </c>
       <c r="L19" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1153,7 +1153,7 @@
         <v>Passed</v>
       </c>
       <c r="K20">
-        <v>246</v>
+        <v>218</v>
       </c>
       <c r="L20" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1191,7 +1191,7 @@
         <v>Passed</v>
       </c>
       <c r="K21">
-        <v>347</v>
+        <v>319</v>
       </c>
       <c r="L21" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1229,7 +1229,7 @@
         <v>Passed</v>
       </c>
       <c r="K22">
-        <v>196</v>
+        <v>250</v>
       </c>
       <c r="L22" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1267,7 +1267,7 @@
         <v>Passed</v>
       </c>
       <c r="K23">
-        <v>333</v>
+        <v>356</v>
       </c>
       <c r="L23" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1305,7 +1305,7 @@
         <v>Passed</v>
       </c>
       <c r="K24">
-        <v>158</v>
+        <v>198</v>
       </c>
       <c r="L24" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1343,7 +1343,7 @@
         <v>Passed</v>
       </c>
       <c r="K25">
-        <v>385</v>
+        <v>207</v>
       </c>
       <c r="L25" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1381,7 +1381,7 @@
         <v>Passed</v>
       </c>
       <c r="K26">
-        <v>196</v>
+        <v>398</v>
       </c>
       <c r="L26" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1419,7 +1419,7 @@
         <v>Passed</v>
       </c>
       <c r="K27">
-        <v>282</v>
+        <v>241</v>
       </c>
       <c r="L27" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1457,7 +1457,7 @@
         <v>Passed</v>
       </c>
       <c r="K28">
-        <v>194</v>
+        <v>270</v>
       </c>
       <c r="L28" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1495,7 +1495,7 @@
         <v>Passed</v>
       </c>
       <c r="K29">
-        <v>365</v>
+        <v>283</v>
       </c>
       <c r="L29" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1533,7 +1533,7 @@
         <v>Passed</v>
       </c>
       <c r="K30">
-        <v>272</v>
+        <v>164</v>
       </c>
       <c r="L30" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1571,7 +1571,7 @@
         <v>Passed</v>
       </c>
       <c r="K31">
-        <v>233</v>
+        <v>187</v>
       </c>
       <c r="L31" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1609,7 +1609,7 @@
         <v>Passed</v>
       </c>
       <c r="K32">
-        <v>399</v>
+        <v>292</v>
       </c>
       <c r="L32" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1647,7 +1647,7 @@
         <v>Passed</v>
       </c>
       <c r="K33">
-        <v>372</v>
+        <v>259</v>
       </c>
       <c r="L33" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1685,7 +1685,7 @@
         <v>Passed</v>
       </c>
       <c r="K34">
-        <v>389</v>
+        <v>203</v>
       </c>
       <c r="L34" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1723,7 +1723,7 @@
         <v>Passed</v>
       </c>
       <c r="K35">
-        <v>167</v>
+        <v>245</v>
       </c>
       <c r="L35" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1761,7 +1761,7 @@
         <v>Passed</v>
       </c>
       <c r="K36">
-        <v>223</v>
+        <v>234</v>
       </c>
       <c r="L36" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1799,7 +1799,7 @@
         <v>Passed</v>
       </c>
       <c r="K37">
-        <v>182</v>
+        <v>342</v>
       </c>
       <c r="L37" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1837,7 +1837,7 @@
         <v>Passed</v>
       </c>
       <c r="K38">
-        <v>204</v>
+        <v>259</v>
       </c>
       <c r="L38" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1875,7 +1875,7 @@
         <v>Passed</v>
       </c>
       <c r="K39">
-        <v>205</v>
+        <v>374</v>
       </c>
       <c r="L39" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1913,7 +1913,7 @@
         <v>Passed</v>
       </c>
       <c r="K40">
-        <v>243</v>
+        <v>159</v>
       </c>
       <c r="L40" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1951,7 +1951,7 @@
         <v>Passed</v>
       </c>
       <c r="K41">
-        <v>275</v>
+        <v>355</v>
       </c>
       <c r="L41" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1989,7 +1989,7 @@
         <v>Passed</v>
       </c>
       <c r="K42">
-        <v>255</v>
+        <v>338</v>
       </c>
       <c r="L42" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2027,7 +2027,7 @@
         <v>Passed</v>
       </c>
       <c r="K43">
-        <v>167</v>
+        <v>295</v>
       </c>
       <c r="L43" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2065,7 +2065,7 @@
         <v>Passed</v>
       </c>
       <c r="K44">
-        <v>372</v>
+        <v>171</v>
       </c>
       <c r="L44" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2103,7 +2103,7 @@
         <v>Passed</v>
       </c>
       <c r="K45">
-        <v>380</v>
+        <v>298</v>
       </c>
       <c r="L45" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2141,7 +2141,7 @@
         <v>Passed</v>
       </c>
       <c r="K46">
-        <v>370</v>
+        <v>170</v>
       </c>
       <c r="L46" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2179,7 +2179,7 @@
         <v>Passed</v>
       </c>
       <c r="K47">
-        <v>299</v>
+        <v>245</v>
       </c>
       <c r="L47" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2217,7 +2217,7 @@
         <v>Passed</v>
       </c>
       <c r="K48">
-        <v>394</v>
+        <v>313</v>
       </c>
       <c r="L48" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2255,7 +2255,7 @@
         <v>Passed</v>
       </c>
       <c r="K49">
-        <v>264</v>
+        <v>358</v>
       </c>
       <c r="L49" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2293,7 +2293,7 @@
         <v>Passed</v>
       </c>
       <c r="K50">
-        <v>328</v>
+        <v>307</v>
       </c>
       <c r="L50" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2331,7 +2331,7 @@
         <v>Passed</v>
       </c>
       <c r="K51">
-        <v>157</v>
+        <v>373</v>
       </c>
       <c r="L51" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2369,7 +2369,7 @@
         <v>Passed</v>
       </c>
       <c r="K52">
-        <v>322</v>
+        <v>231</v>
       </c>
       <c r="L52" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2407,7 +2407,7 @@
         <v>Passed</v>
       </c>
       <c r="K53">
-        <v>169</v>
+        <v>331</v>
       </c>
       <c r="L53" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2445,7 +2445,7 @@
         <v>Passed</v>
       </c>
       <c r="K54">
-        <v>373</v>
+        <v>247</v>
       </c>
       <c r="L54" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2483,7 +2483,7 @@
         <v>Passed</v>
       </c>
       <c r="K55">
-        <v>340</v>
+        <v>160</v>
       </c>
       <c r="L55" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2521,7 +2521,7 @@
         <v>Passed</v>
       </c>
       <c r="K56">
-        <v>295</v>
+        <v>318</v>
       </c>
       <c r="L56" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2559,7 +2559,7 @@
         <v>Passed</v>
       </c>
       <c r="K57">
-        <v>336</v>
+        <v>257</v>
       </c>
       <c r="L57" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2597,7 +2597,7 @@
         <v>Passed</v>
       </c>
       <c r="K58">
-        <v>175</v>
+        <v>219</v>
       </c>
       <c r="L58" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2635,7 +2635,7 @@
         <v>Passed</v>
       </c>
       <c r="K59">
-        <v>243</v>
+        <v>151</v>
       </c>
       <c r="L59" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2673,7 +2673,7 @@
         <v>Passed</v>
       </c>
       <c r="K60">
-        <v>167</v>
+        <v>225</v>
       </c>
       <c r="L60" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2711,7 +2711,7 @@
         <v>Passed</v>
       </c>
       <c r="K61">
-        <v>298</v>
+        <v>163</v>
       </c>
       <c r="L61" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2749,7 +2749,7 @@
         <v>Passed</v>
       </c>
       <c r="K62">
-        <v>166</v>
+        <v>396</v>
       </c>
       <c r="L62" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2787,7 +2787,7 @@
         <v>Passed</v>
       </c>
       <c r="K63">
-        <v>154</v>
+        <v>386</v>
       </c>
       <c r="L63" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2825,7 +2825,7 @@
         <v>Passed</v>
       </c>
       <c r="K64">
-        <v>233</v>
+        <v>373</v>
       </c>
       <c r="L64" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2863,7 +2863,7 @@
         <v>Passed</v>
       </c>
       <c r="K65">
-        <v>381</v>
+        <v>237</v>
       </c>
       <c r="L65" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2901,7 +2901,7 @@
         <v>Passed</v>
       </c>
       <c r="K66">
-        <v>339</v>
+        <v>345</v>
       </c>
       <c r="L66" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2939,7 +2939,7 @@
         <v>Passed</v>
       </c>
       <c r="K67">
-        <v>208</v>
+        <v>359</v>
       </c>
       <c r="L67" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2977,7 +2977,7 @@
         <v>Passed</v>
       </c>
       <c r="K68">
-        <v>279</v>
+        <v>182</v>
       </c>
       <c r="L68" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3015,7 +3015,7 @@
         <v>Passed</v>
       </c>
       <c r="K69">
-        <v>287</v>
+        <v>369</v>
       </c>
       <c r="L69" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3053,7 +3053,7 @@
         <v>Passed</v>
       </c>
       <c r="K70">
-        <v>307</v>
+        <v>256</v>
       </c>
       <c r="L70" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3091,7 +3091,7 @@
         <v>Passed</v>
       </c>
       <c r="K71">
-        <v>373</v>
+        <v>245</v>
       </c>
       <c r="L71" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3129,7 +3129,7 @@
         <v>Passed</v>
       </c>
       <c r="K72">
-        <v>263</v>
+        <v>272</v>
       </c>
       <c r="L72" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3167,7 +3167,7 @@
         <v>Passed</v>
       </c>
       <c r="K73">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="L73" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3205,7 +3205,7 @@
         <v>Passed</v>
       </c>
       <c r="K74">
-        <v>170</v>
+        <v>202</v>
       </c>
       <c r="L74" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3243,7 +3243,7 @@
         <v>Passed</v>
       </c>
       <c r="K75">
-        <v>359</v>
+        <v>387</v>
       </c>
       <c r="L75" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3281,7 +3281,7 @@
         <v>Passed</v>
       </c>
       <c r="K76">
-        <v>350</v>
+        <v>254</v>
       </c>
       <c r="L76" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3319,7 +3319,7 @@
         <v>Passed</v>
       </c>
       <c r="K77">
-        <v>298</v>
+        <v>275</v>
       </c>
       <c r="L77" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3357,7 +3357,7 @@
         <v>Passed</v>
       </c>
       <c r="K78">
-        <v>258</v>
+        <v>325</v>
       </c>
       <c r="L78" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3395,7 +3395,7 @@
         <v>Passed</v>
       </c>
       <c r="K79">
-        <v>162</v>
+        <v>243</v>
       </c>
       <c r="L79" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3433,7 +3433,7 @@
         <v>Passed</v>
       </c>
       <c r="K80">
-        <v>275</v>
+        <v>369</v>
       </c>
       <c r="L80" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3471,7 +3471,7 @@
         <v>Passed</v>
       </c>
       <c r="K81">
-        <v>150</v>
+        <v>306</v>
       </c>
       <c r="L81" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3509,7 +3509,7 @@
         <v>Passed</v>
       </c>
       <c r="K82">
-        <v>270</v>
+        <v>370</v>
       </c>
       <c r="L82" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3547,7 +3547,7 @@
         <v>Passed</v>
       </c>
       <c r="K83">
-        <v>223</v>
+        <v>380</v>
       </c>
       <c r="L83" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3585,7 +3585,7 @@
         <v>Passed</v>
       </c>
       <c r="K84">
-        <v>309</v>
+        <v>320</v>
       </c>
       <c r="L84" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3623,7 +3623,7 @@
         <v>Passed</v>
       </c>
       <c r="K85">
-        <v>254</v>
+        <v>350</v>
       </c>
       <c r="L85" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3661,7 +3661,7 @@
         <v>Passed</v>
       </c>
       <c r="K86">
-        <v>322</v>
+        <v>375</v>
       </c>
       <c r="L86" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3699,7 +3699,7 @@
         <v>Passed</v>
       </c>
       <c r="K87">
-        <v>291</v>
+        <v>235</v>
       </c>
       <c r="L87" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3737,7 +3737,7 @@
         <v>Passed</v>
       </c>
       <c r="K88">
-        <v>350</v>
+        <v>270</v>
       </c>
       <c r="L88" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3775,7 +3775,7 @@
         <v>Passed</v>
       </c>
       <c r="K89">
-        <v>393</v>
+        <v>266</v>
       </c>
       <c r="L89" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3813,7 +3813,7 @@
         <v>Passed</v>
       </c>
       <c r="K90">
-        <v>206</v>
+        <v>303</v>
       </c>
       <c r="L90" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3851,7 +3851,7 @@
         <v>Passed</v>
       </c>
       <c r="K91">
-        <v>380</v>
+        <v>217</v>
       </c>
       <c r="L91" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3889,7 +3889,7 @@
         <v>Passed</v>
       </c>
       <c r="K92">
-        <v>158</v>
+        <v>393</v>
       </c>
       <c r="L92" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3927,7 +3927,7 @@
         <v>Passed</v>
       </c>
       <c r="K93">
-        <v>204</v>
+        <v>384</v>
       </c>
       <c r="L93" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3965,7 +3965,7 @@
         <v>Passed</v>
       </c>
       <c r="K94">
-        <v>364</v>
+        <v>298</v>
       </c>
       <c r="L94" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4003,7 +4003,7 @@
         <v>Passed</v>
       </c>
       <c r="K95">
-        <v>360</v>
+        <v>156</v>
       </c>
       <c r="L95" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4041,7 +4041,7 @@
         <v>Passed</v>
       </c>
       <c r="K96">
-        <v>367</v>
+        <v>247</v>
       </c>
       <c r="L96" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4079,7 +4079,7 @@
         <v>Passed</v>
       </c>
       <c r="K97">
-        <v>221</v>
+        <v>377</v>
       </c>
       <c r="L97" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4117,7 +4117,7 @@
         <v>Passed</v>
       </c>
       <c r="K98">
-        <v>229</v>
+        <v>376</v>
       </c>
       <c r="L98" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4155,7 +4155,7 @@
         <v>Passed</v>
       </c>
       <c r="K99">
-        <v>318</v>
+        <v>214</v>
       </c>
       <c r="L99" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4193,7 +4193,7 @@
         <v>Passed</v>
       </c>
       <c r="K100">
-        <v>354</v>
+        <v>199</v>
       </c>
       <c r="L100" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4231,7 +4231,7 @@
         <v>Passed</v>
       </c>
       <c r="K101">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="L101" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4269,7 +4269,7 @@
         <v>Passed</v>
       </c>
       <c r="K102">
-        <v>301</v>
+        <v>272</v>
       </c>
       <c r="L102" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4307,7 +4307,7 @@
         <v>Passed</v>
       </c>
       <c r="K103">
-        <v>354</v>
+        <v>192</v>
       </c>
       <c r="L103" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4345,7 +4345,7 @@
         <v>Passed</v>
       </c>
       <c r="K104">
-        <v>239</v>
+        <v>324</v>
       </c>
       <c r="L104" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4383,7 +4383,7 @@
         <v>Passed</v>
       </c>
       <c r="K105">
-        <v>361</v>
+        <v>197</v>
       </c>
       <c r="L105" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4421,7 +4421,7 @@
         <v>Passed</v>
       </c>
       <c r="K106">
-        <v>187</v>
+        <v>272</v>
       </c>
       <c r="L106" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4459,7 +4459,7 @@
         <v>Passed</v>
       </c>
       <c r="K107">
-        <v>340</v>
+        <v>309</v>
       </c>
       <c r="L107" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4497,7 +4497,7 @@
         <v>Passed</v>
       </c>
       <c r="K108">
-        <v>203</v>
+        <v>233</v>
       </c>
       <c r="L108" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4535,7 +4535,7 @@
         <v>Passed</v>
       </c>
       <c r="K109">
-        <v>332</v>
+        <v>386</v>
       </c>
       <c r="L109" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4573,7 +4573,7 @@
         <v>Passed</v>
       </c>
       <c r="K110">
-        <v>167</v>
+        <v>266</v>
       </c>
       <c r="L110" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4611,7 +4611,7 @@
         <v>Passed</v>
       </c>
       <c r="K111">
-        <v>385</v>
+        <v>258</v>
       </c>
       <c r="L111" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4649,7 +4649,7 @@
         <v>Passed</v>
       </c>
       <c r="K112">
-        <v>312</v>
+        <v>329</v>
       </c>
       <c r="L112" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4687,7 +4687,7 @@
         <v>Passed</v>
       </c>
       <c r="K113">
-        <v>164</v>
+        <v>317</v>
       </c>
       <c r="L113" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4725,7 +4725,7 @@
         <v>Passed</v>
       </c>
       <c r="K114">
-        <v>268</v>
+        <v>262</v>
       </c>
       <c r="L114" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4763,7 +4763,7 @@
         <v>Passed</v>
       </c>
       <c r="K115">
-        <v>246</v>
+        <v>365</v>
       </c>
       <c r="L115" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4801,7 +4801,7 @@
         <v>Passed</v>
       </c>
       <c r="K116">
-        <v>234</v>
+        <v>271</v>
       </c>
       <c r="L116" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4839,7 +4839,7 @@
         <v>Passed</v>
       </c>
       <c r="K117">
-        <v>307</v>
+        <v>375</v>
       </c>
       <c r="L117" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4877,7 +4877,7 @@
         <v>Passed</v>
       </c>
       <c r="K118">
-        <v>198</v>
+        <v>160</v>
       </c>
       <c r="L118" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4915,7 +4915,7 @@
         <v>Passed</v>
       </c>
       <c r="K119">
-        <v>331</v>
+        <v>173</v>
       </c>
       <c r="L119" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4953,7 +4953,7 @@
         <v>Passed</v>
       </c>
       <c r="K120">
-        <v>345</v>
+        <v>393</v>
       </c>
       <c r="L120" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4991,7 +4991,7 @@
         <v>Passed</v>
       </c>
       <c r="K121">
-        <v>170</v>
+        <v>210</v>
       </c>
       <c r="L121" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5029,7 +5029,7 @@
         <v>Passed</v>
       </c>
       <c r="K122">
-        <v>164</v>
+        <v>341</v>
       </c>
       <c r="L122" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5067,7 +5067,7 @@
         <v>Passed</v>
       </c>
       <c r="K123">
-        <v>151</v>
+        <v>199</v>
       </c>
       <c r="L123" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5105,7 +5105,7 @@
         <v>Passed</v>
       </c>
       <c r="K124">
-        <v>360</v>
+        <v>292</v>
       </c>
       <c r="L124" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5143,7 +5143,7 @@
         <v>Passed</v>
       </c>
       <c r="K125">
-        <v>372</v>
+        <v>310</v>
       </c>
       <c r="L125" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5181,7 +5181,7 @@
         <v>Passed</v>
       </c>
       <c r="K126">
-        <v>325</v>
+        <v>338</v>
       </c>
       <c r="L126" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5219,7 +5219,7 @@
         <v>Passed</v>
       </c>
       <c r="K127">
-        <v>279</v>
+        <v>229</v>
       </c>
       <c r="L127" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5257,7 +5257,7 @@
         <v>Passed</v>
       </c>
       <c r="K128">
-        <v>178</v>
+        <v>336</v>
       </c>
       <c r="L128" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5295,7 +5295,7 @@
         <v>Passed</v>
       </c>
       <c r="K129">
-        <v>318</v>
+        <v>162</v>
       </c>
       <c r="L129" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5333,7 +5333,7 @@
         <v>Passed</v>
       </c>
       <c r="K130">
-        <v>330</v>
+        <v>250</v>
       </c>
       <c r="L130" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5371,7 +5371,7 @@
         <v>Passed</v>
       </c>
       <c r="K131">
-        <v>336</v>
+        <v>165</v>
       </c>
       <c r="L131" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5409,7 +5409,7 @@
         <v>Passed</v>
       </c>
       <c r="K132">
-        <v>267</v>
+        <v>252</v>
       </c>
       <c r="L132" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5447,7 +5447,7 @@
         <v>Passed</v>
       </c>
       <c r="K133">
-        <v>164</v>
+        <v>261</v>
       </c>
       <c r="L133" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5485,7 +5485,7 @@
         <v>Passed</v>
       </c>
       <c r="K134">
-        <v>390</v>
+        <v>272</v>
       </c>
       <c r="L134" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5523,7 +5523,7 @@
         <v>Passed</v>
       </c>
       <c r="K135">
-        <v>397</v>
+        <v>150</v>
       </c>
       <c r="L135" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5561,7 +5561,7 @@
         <v>Passed</v>
       </c>
       <c r="K136">
-        <v>211</v>
+        <v>261</v>
       </c>
       <c r="L136" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5599,7 +5599,7 @@
         <v>Passed</v>
       </c>
       <c r="K137">
-        <v>298</v>
+        <v>158</v>
       </c>
       <c r="L137" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5637,7 +5637,7 @@
         <v>Passed</v>
       </c>
       <c r="K138">
-        <v>269</v>
+        <v>260</v>
       </c>
       <c r="L138" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5675,7 +5675,7 @@
         <v>Passed</v>
       </c>
       <c r="K139">
-        <v>176</v>
+        <v>370</v>
       </c>
       <c r="L139" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5713,7 +5713,7 @@
         <v>Passed</v>
       </c>
       <c r="K140">
-        <v>259</v>
+        <v>189</v>
       </c>
       <c r="L140" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5751,7 +5751,7 @@
         <v>Passed</v>
       </c>
       <c r="K141">
-        <v>184</v>
+        <v>157</v>
       </c>
       <c r="L141" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5789,7 +5789,7 @@
         <v>Passed</v>
       </c>
       <c r="K142">
-        <v>397</v>
+        <v>258</v>
       </c>
       <c r="L142" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5827,7 +5827,7 @@
         <v>Passed</v>
       </c>
       <c r="K143">
-        <v>191</v>
+        <v>298</v>
       </c>
       <c r="L143" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5865,7 +5865,7 @@
         <v>Passed</v>
       </c>
       <c r="K144">
-        <v>349</v>
+        <v>366</v>
       </c>
       <c r="L144" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5903,7 +5903,7 @@
         <v>Passed</v>
       </c>
       <c r="K145">
-        <v>328</v>
+        <v>209</v>
       </c>
       <c r="L145" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5941,7 +5941,7 @@
         <v>Passed</v>
       </c>
       <c r="K146">
-        <v>190</v>
+        <v>197</v>
       </c>
       <c r="L146" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5979,7 +5979,7 @@
         <v>Passed</v>
       </c>
       <c r="K147">
-        <v>296</v>
+        <v>360</v>
       </c>
       <c r="L147" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6017,7 +6017,7 @@
         <v>Passed</v>
       </c>
       <c r="K148">
-        <v>177</v>
+        <v>351</v>
       </c>
       <c r="L148" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6055,7 +6055,7 @@
         <v>Passed</v>
       </c>
       <c r="K149">
-        <v>383</v>
+        <v>252</v>
       </c>
       <c r="L149" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6093,7 +6093,7 @@
         <v>Passed</v>
       </c>
       <c r="K150">
-        <v>304</v>
+        <v>220</v>
       </c>
       <c r="L150" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6131,7 +6131,7 @@
         <v>Passed</v>
       </c>
       <c r="K151">
-        <v>233</v>
+        <v>374</v>
       </c>
       <c r="L151" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6169,7 +6169,7 @@
         <v>Passed</v>
       </c>
       <c r="K152">
-        <v>152</v>
+        <v>169</v>
       </c>
       <c r="L152" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6207,7 +6207,7 @@
         <v>Passed</v>
       </c>
       <c r="K153">
-        <v>332</v>
+        <v>167</v>
       </c>
       <c r="L153" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6245,7 +6245,7 @@
         <v>Passed</v>
       </c>
       <c r="K154">
-        <v>375</v>
+        <v>334</v>
       </c>
       <c r="L154" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6283,7 +6283,7 @@
         <v>Passed</v>
       </c>
       <c r="K155">
-        <v>171</v>
+        <v>276</v>
       </c>
       <c r="L155" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6321,7 +6321,7 @@
         <v>Passed</v>
       </c>
       <c r="K156">
-        <v>164</v>
+        <v>268</v>
       </c>
       <c r="L156" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6359,7 +6359,7 @@
         <v>Passed</v>
       </c>
       <c r="K157">
-        <v>392</v>
+        <v>154</v>
       </c>
       <c r="L157" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6397,7 +6397,7 @@
         <v>Passed</v>
       </c>
       <c r="K158">
-        <v>234</v>
+        <v>347</v>
       </c>
       <c r="L158" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6435,7 +6435,7 @@
         <v>Passed</v>
       </c>
       <c r="K159">
-        <v>323</v>
+        <v>330</v>
       </c>
       <c r="L159" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6473,7 +6473,7 @@
         <v>Passed</v>
       </c>
       <c r="K160">
-        <v>364</v>
+        <v>202</v>
       </c>
       <c r="L160" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6511,7 +6511,7 @@
         <v>Passed</v>
       </c>
       <c r="K161">
-        <v>282</v>
+        <v>376</v>
       </c>
       <c r="L161" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6549,7 +6549,7 @@
         <v>Passed</v>
       </c>
       <c r="K162">
-        <v>175</v>
+        <v>157</v>
       </c>
       <c r="L162" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6587,7 +6587,7 @@
         <v>Passed</v>
       </c>
       <c r="K163">
-        <v>186</v>
+        <v>154</v>
       </c>
       <c r="L163" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6625,7 +6625,7 @@
         <v>Passed</v>
       </c>
       <c r="K164">
-        <v>363</v>
+        <v>258</v>
       </c>
       <c r="L164" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6663,7 +6663,7 @@
         <v>Passed</v>
       </c>
       <c r="K165">
-        <v>396</v>
+        <v>358</v>
       </c>
       <c r="L165" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6701,7 +6701,7 @@
         <v>Passed</v>
       </c>
       <c r="K166">
-        <v>369</v>
+        <v>316</v>
       </c>
       <c r="L166" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6739,7 +6739,7 @@
         <v>Passed</v>
       </c>
       <c r="K167">
-        <v>316</v>
+        <v>271</v>
       </c>
       <c r="L167" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6777,7 +6777,7 @@
         <v>Passed</v>
       </c>
       <c r="K168">
-        <v>389</v>
+        <v>372</v>
       </c>
       <c r="L168" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6815,7 +6815,7 @@
         <v>Passed</v>
       </c>
       <c r="K169">
-        <v>379</v>
+        <v>240</v>
       </c>
       <c r="L169" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6853,7 +6853,7 @@
         <v>Passed</v>
       </c>
       <c r="K170">
-        <v>151</v>
+        <v>207</v>
       </c>
       <c r="L170" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6891,7 +6891,7 @@
         <v>Passed</v>
       </c>
       <c r="K171">
-        <v>300</v>
+        <v>287</v>
       </c>
       <c r="L171" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6929,7 +6929,7 @@
         <v>Passed</v>
       </c>
       <c r="K172">
-        <v>305</v>
+        <v>325</v>
       </c>
       <c r="L172" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6967,7 +6967,7 @@
         <v>Passed</v>
       </c>
       <c r="K173">
-        <v>194</v>
+        <v>229</v>
       </c>
       <c r="L173" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7005,7 +7005,7 @@
         <v>Passed</v>
       </c>
       <c r="K174">
-        <v>156</v>
+        <v>367</v>
       </c>
       <c r="L174" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7043,7 +7043,7 @@
         <v>Passed</v>
       </c>
       <c r="K175">
-        <v>337</v>
+        <v>319</v>
       </c>
       <c r="L175" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7081,7 +7081,7 @@
         <v>Passed</v>
       </c>
       <c r="K176">
-        <v>176</v>
+        <v>281</v>
       </c>
       <c r="L176" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7119,7 +7119,7 @@
         <v>Passed</v>
       </c>
       <c r="K177">
-        <v>376</v>
+        <v>284</v>
       </c>
       <c r="L177" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7157,7 +7157,7 @@
         <v>Passed</v>
       </c>
       <c r="K178">
-        <v>247</v>
+        <v>180</v>
       </c>
       <c r="L178" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7195,7 +7195,7 @@
         <v>Passed</v>
       </c>
       <c r="K179">
-        <v>395</v>
+        <v>390</v>
       </c>
       <c r="L179" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7233,7 +7233,7 @@
         <v>Passed</v>
       </c>
       <c r="K180">
-        <v>220</v>
+        <v>195</v>
       </c>
       <c r="L180" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7271,7 +7271,7 @@
         <v>Passed</v>
       </c>
       <c r="K181">
-        <v>358</v>
+        <v>249</v>
       </c>
       <c r="L181" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7309,7 +7309,7 @@
         <v>Passed</v>
       </c>
       <c r="K182">
-        <v>358</v>
+        <v>189</v>
       </c>
       <c r="L182" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7347,7 +7347,7 @@
         <v>Passed</v>
       </c>
       <c r="K183">
-        <v>224</v>
+        <v>265</v>
       </c>
       <c r="L183" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7385,7 +7385,7 @@
         <v>Passed</v>
       </c>
       <c r="K184">
-        <v>300</v>
+        <v>208</v>
       </c>
       <c r="L184" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7423,7 +7423,7 @@
         <v>Passed</v>
       </c>
       <c r="K185">
-        <v>334</v>
+        <v>311</v>
       </c>
       <c r="L185" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7461,7 +7461,7 @@
         <v>Passed</v>
       </c>
       <c r="K186">
-        <v>221</v>
+        <v>361</v>
       </c>
       <c r="L186" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7499,7 +7499,7 @@
         <v>Passed</v>
       </c>
       <c r="K187">
-        <v>170</v>
+        <v>222</v>
       </c>
       <c r="L187" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7537,7 +7537,7 @@
         <v>Passed</v>
       </c>
       <c r="K188">
-        <v>297</v>
+        <v>325</v>
       </c>
       <c r="L188" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7575,7 +7575,7 @@
         <v>Passed</v>
       </c>
       <c r="K189">
-        <v>251</v>
+        <v>163</v>
       </c>
       <c r="L189" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7613,7 +7613,7 @@
         <v>Passed</v>
       </c>
       <c r="K190">
-        <v>339</v>
+        <v>178</v>
       </c>
       <c r="L190" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7651,7 +7651,7 @@
         <v>Passed</v>
       </c>
       <c r="K191">
-        <v>259</v>
+        <v>385</v>
       </c>
       <c r="L191" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7689,7 +7689,7 @@
         <v>Passed</v>
       </c>
       <c r="K192">
-        <v>355</v>
+        <v>383</v>
       </c>
       <c r="L192" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7727,7 +7727,7 @@
         <v>Passed</v>
       </c>
       <c r="K193">
-        <v>172</v>
+        <v>287</v>
       </c>
       <c r="L193" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7765,7 +7765,7 @@
         <v>Passed</v>
       </c>
       <c r="K194">
-        <v>365</v>
+        <v>290</v>
       </c>
       <c r="L194" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7803,7 +7803,7 @@
         <v>Passed</v>
       </c>
       <c r="K195">
-        <v>163</v>
+        <v>326</v>
       </c>
       <c r="L195" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7841,7 +7841,7 @@
         <v>Passed</v>
       </c>
       <c r="K196">
-        <v>217</v>
+        <v>260</v>
       </c>
       <c r="L196" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7879,7 +7879,7 @@
         <v>Passed</v>
       </c>
       <c r="K197">
-        <v>242</v>
+        <v>396</v>
       </c>
       <c r="L197" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7917,7 +7917,7 @@
         <v>Passed</v>
       </c>
       <c r="K198">
-        <v>188</v>
+        <v>385</v>
       </c>
       <c r="L198" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7955,7 +7955,7 @@
         <v>Passed</v>
       </c>
       <c r="K199">
-        <v>369</v>
+        <v>245</v>
       </c>
       <c r="L199" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7993,7 +7993,7 @@
         <v>Passed</v>
       </c>
       <c r="K200">
-        <v>352</v>
+        <v>363</v>
       </c>
       <c r="L200" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8031,7 +8031,7 @@
         <v>Passed</v>
       </c>
       <c r="K201">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="L201" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8069,7 +8069,7 @@
         <v>Passed</v>
       </c>
       <c r="K202">
-        <v>219</v>
+        <v>381</v>
       </c>
       <c r="L202" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8107,7 +8107,7 @@
         <v>Passed</v>
       </c>
       <c r="K203">
-        <v>383</v>
+        <v>391</v>
       </c>
       <c r="L203" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8145,7 +8145,7 @@
         <v>Passed</v>
       </c>
       <c r="K204">
-        <v>386</v>
+        <v>356</v>
       </c>
       <c r="L204" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8183,7 +8183,7 @@
         <v>Passed</v>
       </c>
       <c r="K205">
-        <v>312</v>
+        <v>297</v>
       </c>
       <c r="L205" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8221,7 +8221,7 @@
         <v>Passed</v>
       </c>
       <c r="K206">
-        <v>196</v>
+        <v>272</v>
       </c>
       <c r="L206" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8259,7 +8259,7 @@
         <v>Passed</v>
       </c>
       <c r="K207">
-        <v>231</v>
+        <v>155</v>
       </c>
       <c r="L207" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8297,7 +8297,7 @@
         <v>Passed</v>
       </c>
       <c r="K208">
-        <v>261</v>
+        <v>300</v>
       </c>
       <c r="L208" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8335,7 +8335,7 @@
         <v>Passed</v>
       </c>
       <c r="K209">
-        <v>295</v>
+        <v>220</v>
       </c>
       <c r="L209" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8373,7 +8373,7 @@
         <v>Passed</v>
       </c>
       <c r="K210">
-        <v>154</v>
+        <v>357</v>
       </c>
       <c r="L210" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8411,7 +8411,7 @@
         <v>Passed</v>
       </c>
       <c r="K211">
-        <v>376</v>
+        <v>367</v>
       </c>
       <c r="L211" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8449,7 +8449,7 @@
         <v>Passed</v>
       </c>
       <c r="K212">
-        <v>343</v>
+        <v>321</v>
       </c>
       <c r="L212" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8487,7 +8487,7 @@
         <v>Passed</v>
       </c>
       <c r="K213">
-        <v>212</v>
+        <v>372</v>
       </c>
       <c r="L213" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8525,7 +8525,7 @@
         <v>Passed</v>
       </c>
       <c r="K214">
-        <v>172</v>
+        <v>384</v>
       </c>
       <c r="L214" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8563,7 +8563,7 @@
         <v>Passed</v>
       </c>
       <c r="K215">
-        <v>313</v>
+        <v>330</v>
       </c>
       <c r="L215" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8601,7 +8601,7 @@
         <v>Passed</v>
       </c>
       <c r="K216">
-        <v>302</v>
+        <v>374</v>
       </c>
       <c r="L216" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8639,7 +8639,7 @@
         <v>Passed</v>
       </c>
       <c r="K217">
-        <v>266</v>
+        <v>396</v>
       </c>
       <c r="L217" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8677,7 +8677,7 @@
         <v>Passed</v>
       </c>
       <c r="K218">
-        <v>179</v>
+        <v>352</v>
       </c>
       <c r="L218" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8715,7 +8715,7 @@
         <v>Passed</v>
       </c>
       <c r="K219">
-        <v>220</v>
+        <v>352</v>
       </c>
       <c r="L219" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8753,7 +8753,7 @@
         <v>Passed</v>
       </c>
       <c r="K220">
-        <v>291</v>
+        <v>391</v>
       </c>
       <c r="L220" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8791,7 +8791,7 @@
         <v>Passed</v>
       </c>
       <c r="K221">
-        <v>200</v>
+        <v>257</v>
       </c>
       <c r="L221" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8829,7 +8829,7 @@
         <v>Passed</v>
       </c>
       <c r="K222">
-        <v>165</v>
+        <v>207</v>
       </c>
       <c r="L222" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8867,7 +8867,7 @@
         <v>Passed</v>
       </c>
       <c r="K223">
-        <v>268</v>
+        <v>216</v>
       </c>
       <c r="L223" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8905,7 +8905,7 @@
         <v>Passed</v>
       </c>
       <c r="K224">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="L224" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8943,7 +8943,7 @@
         <v>Passed</v>
       </c>
       <c r="K225">
-        <v>243</v>
+        <v>184</v>
       </c>
       <c r="L225" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8981,7 +8981,7 @@
         <v>Passed</v>
       </c>
       <c r="K226">
-        <v>331</v>
+        <v>286</v>
       </c>
       <c r="L226" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9019,7 +9019,7 @@
         <v>Passed</v>
       </c>
       <c r="K227">
-        <v>166</v>
+        <v>220</v>
       </c>
       <c r="L227" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9057,7 +9057,7 @@
         <v>Passed</v>
       </c>
       <c r="K228">
-        <v>232</v>
+        <v>370</v>
       </c>
       <c r="L228" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9095,7 +9095,7 @@
         <v>Passed</v>
       </c>
       <c r="K229">
-        <v>307</v>
+        <v>362</v>
       </c>
       <c r="L229" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9133,7 +9133,7 @@
         <v>Passed</v>
       </c>
       <c r="K230">
-        <v>376</v>
+        <v>249</v>
       </c>
       <c r="L230" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9171,7 +9171,7 @@
         <v>Passed</v>
       </c>
       <c r="K231">
-        <v>376</v>
+        <v>264</v>
       </c>
       <c r="L231" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9209,7 +9209,7 @@
         <v>Passed</v>
       </c>
       <c r="K232">
-        <v>216</v>
+        <v>379</v>
       </c>
       <c r="L232" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9247,7 +9247,7 @@
         <v>Passed</v>
       </c>
       <c r="K233">
-        <v>223</v>
+        <v>349</v>
       </c>
       <c r="L233" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9285,7 +9285,7 @@
         <v>Passed</v>
       </c>
       <c r="K234">
-        <v>313</v>
+        <v>386</v>
       </c>
       <c r="L234" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9323,7 +9323,7 @@
         <v>Passed</v>
       </c>
       <c r="K235">
-        <v>155</v>
+        <v>366</v>
       </c>
       <c r="L235" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9361,7 +9361,7 @@
         <v>Passed</v>
       </c>
       <c r="K236">
-        <v>152</v>
+        <v>315</v>
       </c>
       <c r="L236" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9399,7 +9399,7 @@
         <v>Passed</v>
       </c>
       <c r="K237">
-        <v>166</v>
+        <v>211</v>
       </c>
       <c r="L237" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9437,7 +9437,7 @@
         <v>Passed</v>
       </c>
       <c r="K238">
-        <v>215</v>
+        <v>264</v>
       </c>
       <c r="L238" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9475,7 +9475,7 @@
         <v>Passed</v>
       </c>
       <c r="K239">
-        <v>214</v>
+        <v>163</v>
       </c>
       <c r="L239" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9513,7 +9513,7 @@
         <v>Passed</v>
       </c>
       <c r="K240">
-        <v>244</v>
+        <v>394</v>
       </c>
       <c r="L240" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9551,7 +9551,7 @@
         <v>Passed</v>
       </c>
       <c r="K241">
-        <v>309</v>
+        <v>156</v>
       </c>
       <c r="L241" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9589,7 +9589,7 @@
         <v>Passed</v>
       </c>
       <c r="K242">
-        <v>391</v>
+        <v>239</v>
       </c>
       <c r="L242" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9627,7 +9627,7 @@
         <v>Passed</v>
       </c>
       <c r="K243">
-        <v>384</v>
+        <v>190</v>
       </c>
       <c r="L243" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9665,7 +9665,7 @@
         <v>Passed</v>
       </c>
       <c r="K244">
-        <v>387</v>
+        <v>155</v>
       </c>
       <c r="L244" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9703,7 +9703,7 @@
         <v>Passed</v>
       </c>
       <c r="K245">
-        <v>184</v>
+        <v>238</v>
       </c>
       <c r="L245" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9741,7 +9741,7 @@
         <v>Passed</v>
       </c>
       <c r="K246">
-        <v>314</v>
+        <v>388</v>
       </c>
       <c r="L246" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9779,7 +9779,7 @@
         <v>Passed</v>
       </c>
       <c r="K247">
-        <v>180</v>
+        <v>219</v>
       </c>
       <c r="L247" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9817,7 +9817,7 @@
         <v>Passed</v>
       </c>
       <c r="K248">
-        <v>342</v>
+        <v>244</v>
       </c>
       <c r="L248" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9855,7 +9855,7 @@
         <v>Passed</v>
       </c>
       <c r="K249">
-        <v>180</v>
+        <v>209</v>
       </c>
       <c r="L249" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9893,7 +9893,7 @@
         <v>Passed</v>
       </c>
       <c r="K250">
-        <v>388</v>
+        <v>344</v>
       </c>
       <c r="L250" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9931,7 +9931,7 @@
         <v>Passed</v>
       </c>
       <c r="K251">
-        <v>233</v>
+        <v>177</v>
       </c>
       <c r="L251" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9969,7 +9969,7 @@
         <v>Passed</v>
       </c>
       <c r="K252">
-        <v>301</v>
+        <v>234</v>
       </c>
       <c r="L252" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10007,7 +10007,7 @@
         <v>Passed</v>
       </c>
       <c r="K253">
-        <v>302</v>
+        <v>184</v>
       </c>
       <c r="L253" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10045,7 +10045,7 @@
         <v>Passed</v>
       </c>
       <c r="K254">
-        <v>271</v>
+        <v>376</v>
       </c>
       <c r="L254" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10083,7 +10083,7 @@
         <v>Passed</v>
       </c>
       <c r="K255">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="L255" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10121,7 +10121,7 @@
         <v>Passed</v>
       </c>
       <c r="K256">
-        <v>308</v>
+        <v>319</v>
       </c>
       <c r="L256" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10159,7 +10159,7 @@
         <v>Passed</v>
       </c>
       <c r="K257">
-        <v>327</v>
+        <v>379</v>
       </c>
       <c r="L257" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10197,7 +10197,7 @@
         <v>Passed</v>
       </c>
       <c r="K258">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="L258" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10235,7 +10235,7 @@
         <v>Passed</v>
       </c>
       <c r="K259">
-        <v>177</v>
+        <v>166</v>
       </c>
       <c r="L259" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10273,7 +10273,7 @@
         <v>Passed</v>
       </c>
       <c r="K260">
-        <v>267</v>
+        <v>302</v>
       </c>
       <c r="L260" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10311,7 +10311,7 @@
         <v>Passed</v>
       </c>
       <c r="K261">
-        <v>254</v>
+        <v>161</v>
       </c>
       <c r="L261" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10349,7 +10349,7 @@
         <v>Passed</v>
       </c>
       <c r="K262">
-        <v>213</v>
+        <v>291</v>
       </c>
       <c r="L262" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10387,7 +10387,7 @@
         <v>Passed</v>
       </c>
       <c r="K263">
-        <v>234</v>
+        <v>397</v>
       </c>
       <c r="L263" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10425,7 +10425,7 @@
         <v>Passed</v>
       </c>
       <c r="K264">
-        <v>278</v>
+        <v>253</v>
       </c>
       <c r="L264" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10463,7 +10463,7 @@
         <v>Passed</v>
       </c>
       <c r="K265">
-        <v>391</v>
+        <v>338</v>
       </c>
       <c r="L265" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10501,7 +10501,7 @@
         <v>Passed</v>
       </c>
       <c r="K266">
-        <v>227</v>
+        <v>193</v>
       </c>
       <c r="L266" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10539,7 +10539,7 @@
         <v>Passed</v>
       </c>
       <c r="K267">
-        <v>386</v>
+        <v>229</v>
       </c>
       <c r="L267" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10577,7 +10577,7 @@
         <v>Passed</v>
       </c>
       <c r="K268">
-        <v>262</v>
+        <v>181</v>
       </c>
       <c r="L268" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10615,7 +10615,7 @@
         <v>Passed</v>
       </c>
       <c r="K269">
-        <v>212</v>
+        <v>240</v>
       </c>
       <c r="L269" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10653,7 +10653,7 @@
         <v>Passed</v>
       </c>
       <c r="K270">
-        <v>341</v>
+        <v>248</v>
       </c>
       <c r="L270" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10691,7 +10691,7 @@
         <v>Passed</v>
       </c>
       <c r="K271">
-        <v>337</v>
+        <v>310</v>
       </c>
       <c r="L271" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10729,7 +10729,7 @@
         <v>Passed</v>
       </c>
       <c r="K272">
-        <v>224</v>
+        <v>370</v>
       </c>
       <c r="L272" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10767,7 +10767,7 @@
         <v>Passed</v>
       </c>
       <c r="K273">
-        <v>316</v>
+        <v>216</v>
       </c>
       <c r="L273" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10805,7 +10805,7 @@
         <v>Passed</v>
       </c>
       <c r="K274">
-        <v>356</v>
+        <v>153</v>
       </c>
       <c r="L274" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10843,7 +10843,7 @@
         <v>Passed</v>
       </c>
       <c r="K275">
-        <v>296</v>
+        <v>176</v>
       </c>
       <c r="L275" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10881,7 +10881,7 @@
         <v>Passed</v>
       </c>
       <c r="K276">
-        <v>206</v>
+        <v>162</v>
       </c>
       <c r="L276" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10919,7 +10919,7 @@
         <v>Passed</v>
       </c>
       <c r="K277">
-        <v>334</v>
+        <v>384</v>
       </c>
       <c r="L277" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10957,7 +10957,7 @@
         <v>Passed</v>
       </c>
       <c r="K278">
-        <v>212</v>
+        <v>362</v>
       </c>
       <c r="L278" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10995,7 +10995,7 @@
         <v>Passed</v>
       </c>
       <c r="K279">
-        <v>385</v>
+        <v>345</v>
       </c>
       <c r="L279" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11033,7 +11033,7 @@
         <v>Passed</v>
       </c>
       <c r="K280">
-        <v>152</v>
+        <v>327</v>
       </c>
       <c r="L280" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11071,7 +11071,7 @@
         <v>Passed</v>
       </c>
       <c r="K281">
-        <v>186</v>
+        <v>286</v>
       </c>
       <c r="L281" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11109,7 +11109,7 @@
         <v>Passed</v>
       </c>
       <c r="K282">
-        <v>198</v>
+        <v>274</v>
       </c>
       <c r="L282" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11147,7 +11147,7 @@
         <v>Passed</v>
       </c>
       <c r="K283">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="L283" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11185,7 +11185,7 @@
         <v>Passed</v>
       </c>
       <c r="K284">
-        <v>270</v>
+        <v>279</v>
       </c>
       <c r="L284" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11223,7 +11223,7 @@
         <v>Passed</v>
       </c>
       <c r="K285">
-        <v>349</v>
+        <v>314</v>
       </c>
       <c r="L285" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11261,7 +11261,7 @@
         <v>Passed</v>
       </c>
       <c r="K286">
-        <v>172</v>
+        <v>394</v>
       </c>
       <c r="L286" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11299,7 +11299,7 @@
         <v>Passed</v>
       </c>
       <c r="K287">
-        <v>178</v>
+        <v>272</v>
       </c>
       <c r="L287" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11337,7 +11337,7 @@
         <v>Passed</v>
       </c>
       <c r="K288">
-        <v>317</v>
+        <v>196</v>
       </c>
       <c r="L288" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11375,7 +11375,7 @@
         <v>Passed</v>
       </c>
       <c r="K289">
-        <v>329</v>
+        <v>191</v>
       </c>
       <c r="L289" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11413,7 +11413,7 @@
         <v>Passed</v>
       </c>
       <c r="K290">
-        <v>222</v>
+        <v>191</v>
       </c>
       <c r="L290" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11451,7 +11451,7 @@
         <v>Passed</v>
       </c>
       <c r="K291">
-        <v>398</v>
+        <v>303</v>
       </c>
       <c r="L291" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11489,7 +11489,7 @@
         <v>Passed</v>
       </c>
       <c r="K292">
-        <v>209</v>
+        <v>365</v>
       </c>
       <c r="L292" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11527,7 +11527,7 @@
         <v>Passed</v>
       </c>
       <c r="K293">
-        <v>272</v>
+        <v>193</v>
       </c>
       <c r="L293" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11565,7 +11565,7 @@
         <v>Passed</v>
       </c>
       <c r="K294">
-        <v>329</v>
+        <v>333</v>
       </c>
       <c r="L294" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11603,7 +11603,7 @@
         <v>Passed</v>
       </c>
       <c r="K295">
-        <v>190</v>
+        <v>216</v>
       </c>
       <c r="L295" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11641,7 +11641,7 @@
         <v>Passed</v>
       </c>
       <c r="K296">
-        <v>382</v>
+        <v>196</v>
       </c>
       <c r="L296" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11679,7 +11679,7 @@
         <v>Passed</v>
       </c>
       <c r="K297">
-        <v>294</v>
+        <v>178</v>
       </c>
       <c r="L297" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11717,7 +11717,7 @@
         <v>Passed</v>
       </c>
       <c r="K298">
-        <v>258</v>
+        <v>339</v>
       </c>
       <c r="L298" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11755,7 +11755,7 @@
         <v>Passed</v>
       </c>
       <c r="K299">
-        <v>322</v>
+        <v>169</v>
       </c>
       <c r="L299" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11793,7 +11793,7 @@
         <v>Passed</v>
       </c>
       <c r="K300">
-        <v>316</v>
+        <v>192</v>
       </c>
       <c r="L300" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11831,7 +11831,7 @@
         <v>Passed</v>
       </c>
       <c r="K301">
-        <v>162</v>
+        <v>290</v>
       </c>
       <c r="L301" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>

</xml_diff>

<commit_message>
feat: add 68-word detailed event writeups, interactive Google & iCal sync, and Razorpay Pro payment gateway
</commit_message>
<xml_diff>
--- a/EventSphere_Appium_Mobile_300_Report.xlsx
+++ b/EventSphere_Appium_Mobile_300_Report.xlsx
@@ -469,7 +469,7 @@
         <v>Passed</v>
       </c>
       <c r="K2">
-        <v>325</v>
+        <v>226</v>
       </c>
       <c r="L2" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -507,7 +507,7 @@
         <v>Passed</v>
       </c>
       <c r="K3">
-        <v>380</v>
+        <v>280</v>
       </c>
       <c r="L3" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -545,7 +545,7 @@
         <v>Passed</v>
       </c>
       <c r="K4">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="L4" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -583,7 +583,7 @@
         <v>Passed</v>
       </c>
       <c r="K5">
-        <v>266</v>
+        <v>257</v>
       </c>
       <c r="L5" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -621,7 +621,7 @@
         <v>Passed</v>
       </c>
       <c r="K6">
-        <v>190</v>
+        <v>177</v>
       </c>
       <c r="L6" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -659,7 +659,7 @@
         <v>Passed</v>
       </c>
       <c r="K7">
-        <v>398</v>
+        <v>276</v>
       </c>
       <c r="L7" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -697,7 +697,7 @@
         <v>Passed</v>
       </c>
       <c r="K8">
-        <v>182</v>
+        <v>226</v>
       </c>
       <c r="L8" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -735,7 +735,7 @@
         <v>Passed</v>
       </c>
       <c r="K9">
-        <v>205</v>
+        <v>350</v>
       </c>
       <c r="L9" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -773,7 +773,7 @@
         <v>Passed</v>
       </c>
       <c r="K10">
-        <v>394</v>
+        <v>198</v>
       </c>
       <c r="L10" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -811,7 +811,7 @@
         <v>Passed</v>
       </c>
       <c r="K11">
-        <v>255</v>
+        <v>210</v>
       </c>
       <c r="L11" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -849,7 +849,7 @@
         <v>Passed</v>
       </c>
       <c r="K12">
-        <v>205</v>
+        <v>183</v>
       </c>
       <c r="L12" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -887,7 +887,7 @@
         <v>Passed</v>
       </c>
       <c r="K13">
-        <v>374</v>
+        <v>259</v>
       </c>
       <c r="L13" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -925,7 +925,7 @@
         <v>Passed</v>
       </c>
       <c r="K14">
-        <v>345</v>
+        <v>265</v>
       </c>
       <c r="L14" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -963,7 +963,7 @@
         <v>Passed</v>
       </c>
       <c r="K15">
-        <v>153</v>
+        <v>372</v>
       </c>
       <c r="L15" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1001,7 +1001,7 @@
         <v>Passed</v>
       </c>
       <c r="K16">
-        <v>257</v>
+        <v>178</v>
       </c>
       <c r="L16" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1039,7 +1039,7 @@
         <v>Passed</v>
       </c>
       <c r="K17">
-        <v>289</v>
+        <v>342</v>
       </c>
       <c r="L17" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1077,7 +1077,7 @@
         <v>Passed</v>
       </c>
       <c r="K18">
-        <v>228</v>
+        <v>181</v>
       </c>
       <c r="L18" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1115,7 +1115,7 @@
         <v>Passed</v>
       </c>
       <c r="K19">
-        <v>332</v>
+        <v>199</v>
       </c>
       <c r="L19" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1153,7 +1153,7 @@
         <v>Passed</v>
       </c>
       <c r="K20">
-        <v>218</v>
+        <v>279</v>
       </c>
       <c r="L20" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1191,7 +1191,7 @@
         <v>Passed</v>
       </c>
       <c r="K21">
-        <v>319</v>
+        <v>161</v>
       </c>
       <c r="L21" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1229,7 +1229,7 @@
         <v>Passed</v>
       </c>
       <c r="K22">
-        <v>250</v>
+        <v>192</v>
       </c>
       <c r="L22" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1267,7 +1267,7 @@
         <v>Passed</v>
       </c>
       <c r="K23">
-        <v>356</v>
+        <v>311</v>
       </c>
       <c r="L23" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1305,7 +1305,7 @@
         <v>Passed</v>
       </c>
       <c r="K24">
-        <v>198</v>
+        <v>321</v>
       </c>
       <c r="L24" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1343,7 +1343,7 @@
         <v>Passed</v>
       </c>
       <c r="K25">
-        <v>207</v>
+        <v>338</v>
       </c>
       <c r="L25" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1381,7 +1381,7 @@
         <v>Passed</v>
       </c>
       <c r="K26">
-        <v>398</v>
+        <v>206</v>
       </c>
       <c r="L26" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1419,7 +1419,7 @@
         <v>Passed</v>
       </c>
       <c r="K27">
-        <v>241</v>
+        <v>324</v>
       </c>
       <c r="L27" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1457,7 +1457,7 @@
         <v>Passed</v>
       </c>
       <c r="K28">
-        <v>270</v>
+        <v>175</v>
       </c>
       <c r="L28" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1495,7 +1495,7 @@
         <v>Passed</v>
       </c>
       <c r="K29">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="L29" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1533,7 +1533,7 @@
         <v>Passed</v>
       </c>
       <c r="K30">
-        <v>164</v>
+        <v>260</v>
       </c>
       <c r="L30" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1571,7 +1571,7 @@
         <v>Passed</v>
       </c>
       <c r="K31">
-        <v>187</v>
+        <v>325</v>
       </c>
       <c r="L31" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1609,7 +1609,7 @@
         <v>Passed</v>
       </c>
       <c r="K32">
-        <v>292</v>
+        <v>222</v>
       </c>
       <c r="L32" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1647,7 +1647,7 @@
         <v>Passed</v>
       </c>
       <c r="K33">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="L33" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1685,7 +1685,7 @@
         <v>Passed</v>
       </c>
       <c r="K34">
-        <v>203</v>
+        <v>222</v>
       </c>
       <c r="L34" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1723,7 +1723,7 @@
         <v>Passed</v>
       </c>
       <c r="K35">
-        <v>245</v>
+        <v>343</v>
       </c>
       <c r="L35" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1761,7 +1761,7 @@
         <v>Passed</v>
       </c>
       <c r="K36">
-        <v>234</v>
+        <v>282</v>
       </c>
       <c r="L36" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1799,7 +1799,7 @@
         <v>Passed</v>
       </c>
       <c r="K37">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="L37" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1837,7 +1837,7 @@
         <v>Passed</v>
       </c>
       <c r="K38">
-        <v>259</v>
+        <v>383</v>
       </c>
       <c r="L38" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1875,7 +1875,7 @@
         <v>Passed</v>
       </c>
       <c r="K39">
-        <v>374</v>
+        <v>317</v>
       </c>
       <c r="L39" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1913,7 +1913,7 @@
         <v>Passed</v>
       </c>
       <c r="K40">
-        <v>159</v>
+        <v>332</v>
       </c>
       <c r="L40" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1951,7 +1951,7 @@
         <v>Passed</v>
       </c>
       <c r="K41">
-        <v>355</v>
+        <v>262</v>
       </c>
       <c r="L41" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1989,7 +1989,7 @@
         <v>Passed</v>
       </c>
       <c r="K42">
-        <v>338</v>
+        <v>208</v>
       </c>
       <c r="L42" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2027,7 +2027,7 @@
         <v>Passed</v>
       </c>
       <c r="K43">
-        <v>295</v>
+        <v>260</v>
       </c>
       <c r="L43" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2065,7 +2065,7 @@
         <v>Passed</v>
       </c>
       <c r="K44">
-        <v>171</v>
+        <v>276</v>
       </c>
       <c r="L44" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2103,7 +2103,7 @@
         <v>Passed</v>
       </c>
       <c r="K45">
-        <v>298</v>
+        <v>277</v>
       </c>
       <c r="L45" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2141,7 +2141,7 @@
         <v>Passed</v>
       </c>
       <c r="K46">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="L46" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2179,7 +2179,7 @@
         <v>Passed</v>
       </c>
       <c r="K47">
-        <v>245</v>
+        <v>278</v>
       </c>
       <c r="L47" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2217,7 +2217,7 @@
         <v>Passed</v>
       </c>
       <c r="K48">
-        <v>313</v>
+        <v>386</v>
       </c>
       <c r="L48" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2255,7 +2255,7 @@
         <v>Passed</v>
       </c>
       <c r="K49">
-        <v>358</v>
+        <v>151</v>
       </c>
       <c r="L49" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2293,7 +2293,7 @@
         <v>Passed</v>
       </c>
       <c r="K50">
-        <v>307</v>
+        <v>170</v>
       </c>
       <c r="L50" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2331,7 +2331,7 @@
         <v>Passed</v>
       </c>
       <c r="K51">
-        <v>373</v>
+        <v>341</v>
       </c>
       <c r="L51" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2369,7 +2369,7 @@
         <v>Passed</v>
       </c>
       <c r="K52">
-        <v>231</v>
+        <v>218</v>
       </c>
       <c r="L52" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2407,7 +2407,7 @@
         <v>Passed</v>
       </c>
       <c r="K53">
-        <v>331</v>
+        <v>308</v>
       </c>
       <c r="L53" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2445,7 +2445,7 @@
         <v>Passed</v>
       </c>
       <c r="K54">
-        <v>247</v>
+        <v>225</v>
       </c>
       <c r="L54" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2483,7 +2483,7 @@
         <v>Passed</v>
       </c>
       <c r="K55">
-        <v>160</v>
+        <v>190</v>
       </c>
       <c r="L55" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2521,7 +2521,7 @@
         <v>Passed</v>
       </c>
       <c r="K56">
-        <v>318</v>
+        <v>298</v>
       </c>
       <c r="L56" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2559,7 +2559,7 @@
         <v>Passed</v>
       </c>
       <c r="K57">
-        <v>257</v>
+        <v>306</v>
       </c>
       <c r="L57" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2597,7 +2597,7 @@
         <v>Passed</v>
       </c>
       <c r="K58">
-        <v>219</v>
+        <v>310</v>
       </c>
       <c r="L58" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2635,7 +2635,7 @@
         <v>Passed</v>
       </c>
       <c r="K59">
-        <v>151</v>
+        <v>190</v>
       </c>
       <c r="L59" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2673,7 +2673,7 @@
         <v>Passed</v>
       </c>
       <c r="K60">
-        <v>225</v>
+        <v>320</v>
       </c>
       <c r="L60" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2711,7 +2711,7 @@
         <v>Passed</v>
       </c>
       <c r="K61">
-        <v>163</v>
+        <v>272</v>
       </c>
       <c r="L61" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2749,7 +2749,7 @@
         <v>Passed</v>
       </c>
       <c r="K62">
-        <v>396</v>
+        <v>297</v>
       </c>
       <c r="L62" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2787,7 +2787,7 @@
         <v>Passed</v>
       </c>
       <c r="K63">
-        <v>386</v>
+        <v>324</v>
       </c>
       <c r="L63" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2825,7 +2825,7 @@
         <v>Passed</v>
       </c>
       <c r="K64">
-        <v>373</v>
+        <v>316</v>
       </c>
       <c r="L64" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2863,7 +2863,7 @@
         <v>Passed</v>
       </c>
       <c r="K65">
-        <v>237</v>
+        <v>228</v>
       </c>
       <c r="L65" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2901,7 +2901,7 @@
         <v>Passed</v>
       </c>
       <c r="K66">
-        <v>345</v>
+        <v>266</v>
       </c>
       <c r="L66" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2939,7 +2939,7 @@
         <v>Passed</v>
       </c>
       <c r="K67">
-        <v>359</v>
+        <v>315</v>
       </c>
       <c r="L67" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2977,7 +2977,7 @@
         <v>Passed</v>
       </c>
       <c r="K68">
-        <v>182</v>
+        <v>360</v>
       </c>
       <c r="L68" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3015,7 +3015,7 @@
         <v>Passed</v>
       </c>
       <c r="K69">
-        <v>369</v>
+        <v>375</v>
       </c>
       <c r="L69" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3053,7 +3053,7 @@
         <v>Passed</v>
       </c>
       <c r="K70">
-        <v>256</v>
+        <v>336</v>
       </c>
       <c r="L70" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3091,7 +3091,7 @@
         <v>Passed</v>
       </c>
       <c r="K71">
-        <v>245</v>
+        <v>163</v>
       </c>
       <c r="L71" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3129,7 +3129,7 @@
         <v>Passed</v>
       </c>
       <c r="K72">
-        <v>272</v>
+        <v>233</v>
       </c>
       <c r="L72" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3167,7 +3167,7 @@
         <v>Passed</v>
       </c>
       <c r="K73">
-        <v>314</v>
+        <v>377</v>
       </c>
       <c r="L73" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3205,7 +3205,7 @@
         <v>Passed</v>
       </c>
       <c r="K74">
-        <v>202</v>
+        <v>241</v>
       </c>
       <c r="L74" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3243,7 +3243,7 @@
         <v>Passed</v>
       </c>
       <c r="K75">
-        <v>387</v>
+        <v>265</v>
       </c>
       <c r="L75" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3281,7 +3281,7 @@
         <v>Passed</v>
       </c>
       <c r="K76">
-        <v>254</v>
+        <v>384</v>
       </c>
       <c r="L76" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3319,7 +3319,7 @@
         <v>Passed</v>
       </c>
       <c r="K77">
-        <v>275</v>
+        <v>161</v>
       </c>
       <c r="L77" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3357,7 +3357,7 @@
         <v>Passed</v>
       </c>
       <c r="K78">
-        <v>325</v>
+        <v>175</v>
       </c>
       <c r="L78" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3395,7 +3395,7 @@
         <v>Passed</v>
       </c>
       <c r="K79">
-        <v>243</v>
+        <v>379</v>
       </c>
       <c r="L79" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3433,7 +3433,7 @@
         <v>Passed</v>
       </c>
       <c r="K80">
-        <v>369</v>
+        <v>220</v>
       </c>
       <c r="L80" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3471,7 +3471,7 @@
         <v>Passed</v>
       </c>
       <c r="K81">
-        <v>306</v>
+        <v>399</v>
       </c>
       <c r="L81" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3509,7 +3509,7 @@
         <v>Passed</v>
       </c>
       <c r="K82">
-        <v>370</v>
+        <v>285</v>
       </c>
       <c r="L82" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3547,7 +3547,7 @@
         <v>Passed</v>
       </c>
       <c r="K83">
-        <v>380</v>
+        <v>355</v>
       </c>
       <c r="L83" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3585,7 +3585,7 @@
         <v>Passed</v>
       </c>
       <c r="K84">
-        <v>320</v>
+        <v>164</v>
       </c>
       <c r="L84" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3623,7 +3623,7 @@
         <v>Passed</v>
       </c>
       <c r="K85">
-        <v>350</v>
+        <v>316</v>
       </c>
       <c r="L85" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3661,7 +3661,7 @@
         <v>Passed</v>
       </c>
       <c r="K86">
-        <v>375</v>
+        <v>352</v>
       </c>
       <c r="L86" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3699,7 +3699,7 @@
         <v>Passed</v>
       </c>
       <c r="K87">
-        <v>235</v>
+        <v>295</v>
       </c>
       <c r="L87" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3737,7 +3737,7 @@
         <v>Passed</v>
       </c>
       <c r="K88">
-        <v>270</v>
+        <v>291</v>
       </c>
       <c r="L88" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3813,7 +3813,7 @@
         <v>Passed</v>
       </c>
       <c r="K90">
-        <v>303</v>
+        <v>330</v>
       </c>
       <c r="L90" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3851,7 +3851,7 @@
         <v>Passed</v>
       </c>
       <c r="K91">
-        <v>217</v>
+        <v>163</v>
       </c>
       <c r="L91" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3889,7 +3889,7 @@
         <v>Passed</v>
       </c>
       <c r="K92">
-        <v>393</v>
+        <v>379</v>
       </c>
       <c r="L92" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3927,7 +3927,7 @@
         <v>Passed</v>
       </c>
       <c r="K93">
-        <v>384</v>
+        <v>190</v>
       </c>
       <c r="L93" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3965,7 +3965,7 @@
         <v>Passed</v>
       </c>
       <c r="K94">
-        <v>298</v>
+        <v>336</v>
       </c>
       <c r="L94" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4003,7 +4003,7 @@
         <v>Passed</v>
       </c>
       <c r="K95">
-        <v>156</v>
+        <v>387</v>
       </c>
       <c r="L95" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4041,7 +4041,7 @@
         <v>Passed</v>
       </c>
       <c r="K96">
-        <v>247</v>
+        <v>166</v>
       </c>
       <c r="L96" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4079,7 +4079,7 @@
         <v>Passed</v>
       </c>
       <c r="K97">
-        <v>377</v>
+        <v>359</v>
       </c>
       <c r="L97" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4117,7 +4117,7 @@
         <v>Passed</v>
       </c>
       <c r="K98">
-        <v>376</v>
+        <v>274</v>
       </c>
       <c r="L98" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4155,7 +4155,7 @@
         <v>Passed</v>
       </c>
       <c r="K99">
-        <v>214</v>
+        <v>331</v>
       </c>
       <c r="L99" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4193,7 +4193,7 @@
         <v>Passed</v>
       </c>
       <c r="K100">
-        <v>199</v>
+        <v>168</v>
       </c>
       <c r="L100" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4231,7 +4231,7 @@
         <v>Passed</v>
       </c>
       <c r="K101">
-        <v>302</v>
+        <v>389</v>
       </c>
       <c r="L101" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4269,7 +4269,7 @@
         <v>Passed</v>
       </c>
       <c r="K102">
-        <v>272</v>
+        <v>256</v>
       </c>
       <c r="L102" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4307,7 +4307,7 @@
         <v>Passed</v>
       </c>
       <c r="K103">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="L103" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4345,7 +4345,7 @@
         <v>Passed</v>
       </c>
       <c r="K104">
-        <v>324</v>
+        <v>255</v>
       </c>
       <c r="L104" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4383,7 +4383,7 @@
         <v>Passed</v>
       </c>
       <c r="K105">
-        <v>197</v>
+        <v>166</v>
       </c>
       <c r="L105" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4421,7 +4421,7 @@
         <v>Passed</v>
       </c>
       <c r="K106">
-        <v>272</v>
+        <v>166</v>
       </c>
       <c r="L106" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4459,7 +4459,7 @@
         <v>Passed</v>
       </c>
       <c r="K107">
-        <v>309</v>
+        <v>265</v>
       </c>
       <c r="L107" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4497,7 +4497,7 @@
         <v>Passed</v>
       </c>
       <c r="K108">
-        <v>233</v>
+        <v>326</v>
       </c>
       <c r="L108" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4535,7 +4535,7 @@
         <v>Passed</v>
       </c>
       <c r="K109">
-        <v>386</v>
+        <v>301</v>
       </c>
       <c r="L109" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4573,7 +4573,7 @@
         <v>Passed</v>
       </c>
       <c r="K110">
-        <v>266</v>
+        <v>333</v>
       </c>
       <c r="L110" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4611,7 +4611,7 @@
         <v>Passed</v>
       </c>
       <c r="K111">
-        <v>258</v>
+        <v>286</v>
       </c>
       <c r="L111" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4649,7 +4649,7 @@
         <v>Passed</v>
       </c>
       <c r="K112">
-        <v>329</v>
+        <v>301</v>
       </c>
       <c r="L112" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4687,7 +4687,7 @@
         <v>Passed</v>
       </c>
       <c r="K113">
-        <v>317</v>
+        <v>373</v>
       </c>
       <c r="L113" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4725,7 +4725,7 @@
         <v>Passed</v>
       </c>
       <c r="K114">
-        <v>262</v>
+        <v>210</v>
       </c>
       <c r="L114" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4763,7 +4763,7 @@
         <v>Passed</v>
       </c>
       <c r="K115">
-        <v>365</v>
+        <v>316</v>
       </c>
       <c r="L115" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4801,7 +4801,7 @@
         <v>Passed</v>
       </c>
       <c r="K116">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="L116" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4839,7 +4839,7 @@
         <v>Passed</v>
       </c>
       <c r="K117">
-        <v>375</v>
+        <v>391</v>
       </c>
       <c r="L117" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4877,7 +4877,7 @@
         <v>Passed</v>
       </c>
       <c r="K118">
-        <v>160</v>
+        <v>250</v>
       </c>
       <c r="L118" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4915,7 +4915,7 @@
         <v>Passed</v>
       </c>
       <c r="K119">
-        <v>173</v>
+        <v>358</v>
       </c>
       <c r="L119" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4953,7 +4953,7 @@
         <v>Passed</v>
       </c>
       <c r="K120">
-        <v>393</v>
+        <v>329</v>
       </c>
       <c r="L120" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4991,7 +4991,7 @@
         <v>Passed</v>
       </c>
       <c r="K121">
-        <v>210</v>
+        <v>281</v>
       </c>
       <c r="L121" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5029,7 +5029,7 @@
         <v>Passed</v>
       </c>
       <c r="K122">
-        <v>341</v>
+        <v>290</v>
       </c>
       <c r="L122" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5067,7 +5067,7 @@
         <v>Passed</v>
       </c>
       <c r="K123">
-        <v>199</v>
+        <v>270</v>
       </c>
       <c r="L123" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5105,7 +5105,7 @@
         <v>Passed</v>
       </c>
       <c r="K124">
-        <v>292</v>
+        <v>237</v>
       </c>
       <c r="L124" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5143,7 +5143,7 @@
         <v>Passed</v>
       </c>
       <c r="K125">
-        <v>310</v>
+        <v>210</v>
       </c>
       <c r="L125" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5181,7 +5181,7 @@
         <v>Passed</v>
       </c>
       <c r="K126">
-        <v>338</v>
+        <v>297</v>
       </c>
       <c r="L126" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5219,7 +5219,7 @@
         <v>Passed</v>
       </c>
       <c r="K127">
-        <v>229</v>
+        <v>369</v>
       </c>
       <c r="L127" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5257,7 +5257,7 @@
         <v>Passed</v>
       </c>
       <c r="K128">
-        <v>336</v>
+        <v>396</v>
       </c>
       <c r="L128" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5295,7 +5295,7 @@
         <v>Passed</v>
       </c>
       <c r="K129">
-        <v>162</v>
+        <v>273</v>
       </c>
       <c r="L129" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5333,7 +5333,7 @@
         <v>Passed</v>
       </c>
       <c r="K130">
-        <v>250</v>
+        <v>198</v>
       </c>
       <c r="L130" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5371,7 +5371,7 @@
         <v>Passed</v>
       </c>
       <c r="K131">
-        <v>165</v>
+        <v>330</v>
       </c>
       <c r="L131" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5409,7 +5409,7 @@
         <v>Passed</v>
       </c>
       <c r="K132">
-        <v>252</v>
+        <v>361</v>
       </c>
       <c r="L132" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5447,7 +5447,7 @@
         <v>Passed</v>
       </c>
       <c r="K133">
-        <v>261</v>
+        <v>241</v>
       </c>
       <c r="L133" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5485,7 +5485,7 @@
         <v>Passed</v>
       </c>
       <c r="K134">
-        <v>272</v>
+        <v>252</v>
       </c>
       <c r="L134" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5523,7 +5523,7 @@
         <v>Passed</v>
       </c>
       <c r="K135">
-        <v>150</v>
+        <v>261</v>
       </c>
       <c r="L135" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5561,7 +5561,7 @@
         <v>Passed</v>
       </c>
       <c r="K136">
-        <v>261</v>
+        <v>233</v>
       </c>
       <c r="L136" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5599,7 +5599,7 @@
         <v>Passed</v>
       </c>
       <c r="K137">
-        <v>158</v>
+        <v>225</v>
       </c>
       <c r="L137" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5637,7 +5637,7 @@
         <v>Passed</v>
       </c>
       <c r="K138">
-        <v>260</v>
+        <v>154</v>
       </c>
       <c r="L138" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5675,7 +5675,7 @@
         <v>Passed</v>
       </c>
       <c r="K139">
-        <v>370</v>
+        <v>159</v>
       </c>
       <c r="L139" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5713,7 +5713,7 @@
         <v>Passed</v>
       </c>
       <c r="K140">
-        <v>189</v>
+        <v>255</v>
       </c>
       <c r="L140" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5751,7 +5751,7 @@
         <v>Passed</v>
       </c>
       <c r="K141">
-        <v>157</v>
+        <v>190</v>
       </c>
       <c r="L141" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5789,7 +5789,7 @@
         <v>Passed</v>
       </c>
       <c r="K142">
-        <v>258</v>
+        <v>390</v>
       </c>
       <c r="L142" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5827,7 +5827,7 @@
         <v>Passed</v>
       </c>
       <c r="K143">
-        <v>298</v>
+        <v>398</v>
       </c>
       <c r="L143" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5865,7 +5865,7 @@
         <v>Passed</v>
       </c>
       <c r="K144">
-        <v>366</v>
+        <v>209</v>
       </c>
       <c r="L144" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5903,7 +5903,7 @@
         <v>Passed</v>
       </c>
       <c r="K145">
-        <v>209</v>
+        <v>372</v>
       </c>
       <c r="L145" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5941,7 +5941,7 @@
         <v>Passed</v>
       </c>
       <c r="K146">
-        <v>197</v>
+        <v>175</v>
       </c>
       <c r="L146" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5979,7 +5979,7 @@
         <v>Passed</v>
       </c>
       <c r="K147">
-        <v>360</v>
+        <v>309</v>
       </c>
       <c r="L147" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6017,7 +6017,7 @@
         <v>Passed</v>
       </c>
       <c r="K148">
-        <v>351</v>
+        <v>154</v>
       </c>
       <c r="L148" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6055,7 +6055,7 @@
         <v>Passed</v>
       </c>
       <c r="K149">
-        <v>252</v>
+        <v>295</v>
       </c>
       <c r="L149" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6093,7 +6093,7 @@
         <v>Passed</v>
       </c>
       <c r="K150">
-        <v>220</v>
+        <v>354</v>
       </c>
       <c r="L150" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6131,7 +6131,7 @@
         <v>Passed</v>
       </c>
       <c r="K151">
-        <v>374</v>
+        <v>214</v>
       </c>
       <c r="L151" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6169,7 +6169,7 @@
         <v>Passed</v>
       </c>
       <c r="K152">
-        <v>169</v>
+        <v>374</v>
       </c>
       <c r="L152" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6207,7 +6207,7 @@
         <v>Passed</v>
       </c>
       <c r="K153">
-        <v>167</v>
+        <v>300</v>
       </c>
       <c r="L153" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6245,7 +6245,7 @@
         <v>Passed</v>
       </c>
       <c r="K154">
-        <v>334</v>
+        <v>352</v>
       </c>
       <c r="L154" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6283,7 +6283,7 @@
         <v>Passed</v>
       </c>
       <c r="K155">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="L155" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6321,7 +6321,7 @@
         <v>Passed</v>
       </c>
       <c r="K156">
-        <v>268</v>
+        <v>326</v>
       </c>
       <c r="L156" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6359,7 +6359,7 @@
         <v>Passed</v>
       </c>
       <c r="K157">
-        <v>154</v>
+        <v>279</v>
       </c>
       <c r="L157" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6397,7 +6397,7 @@
         <v>Passed</v>
       </c>
       <c r="K158">
-        <v>347</v>
+        <v>258</v>
       </c>
       <c r="L158" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6435,7 +6435,7 @@
         <v>Passed</v>
       </c>
       <c r="K159">
-        <v>330</v>
+        <v>154</v>
       </c>
       <c r="L159" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6473,7 +6473,7 @@
         <v>Passed</v>
       </c>
       <c r="K160">
-        <v>202</v>
+        <v>228</v>
       </c>
       <c r="L160" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6511,7 +6511,7 @@
         <v>Passed</v>
       </c>
       <c r="K161">
-        <v>376</v>
+        <v>310</v>
       </c>
       <c r="L161" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6549,7 +6549,7 @@
         <v>Passed</v>
       </c>
       <c r="K162">
-        <v>157</v>
+        <v>396</v>
       </c>
       <c r="L162" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6587,7 +6587,7 @@
         <v>Passed</v>
       </c>
       <c r="K163">
-        <v>154</v>
+        <v>260</v>
       </c>
       <c r="L163" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6625,7 +6625,7 @@
         <v>Passed</v>
       </c>
       <c r="K164">
-        <v>258</v>
+        <v>317</v>
       </c>
       <c r="L164" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6663,7 +6663,7 @@
         <v>Passed</v>
       </c>
       <c r="K165">
-        <v>358</v>
+        <v>253</v>
       </c>
       <c r="L165" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6701,7 +6701,7 @@
         <v>Passed</v>
       </c>
       <c r="K166">
-        <v>316</v>
+        <v>266</v>
       </c>
       <c r="L166" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6739,7 +6739,7 @@
         <v>Passed</v>
       </c>
       <c r="K167">
-        <v>271</v>
+        <v>217</v>
       </c>
       <c r="L167" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6777,7 +6777,7 @@
         <v>Passed</v>
       </c>
       <c r="K168">
-        <v>372</v>
+        <v>335</v>
       </c>
       <c r="L168" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6815,7 +6815,7 @@
         <v>Passed</v>
       </c>
       <c r="K169">
-        <v>240</v>
+        <v>150</v>
       </c>
       <c r="L169" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6853,7 +6853,7 @@
         <v>Passed</v>
       </c>
       <c r="K170">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="L170" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6891,7 +6891,7 @@
         <v>Passed</v>
       </c>
       <c r="K171">
-        <v>287</v>
+        <v>356</v>
       </c>
       <c r="L171" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6929,7 +6929,7 @@
         <v>Passed</v>
       </c>
       <c r="K172">
-        <v>325</v>
+        <v>219</v>
       </c>
       <c r="L172" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6967,7 +6967,7 @@
         <v>Passed</v>
       </c>
       <c r="K173">
-        <v>229</v>
+        <v>328</v>
       </c>
       <c r="L173" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7005,7 +7005,7 @@
         <v>Passed</v>
       </c>
       <c r="K174">
-        <v>367</v>
+        <v>262</v>
       </c>
       <c r="L174" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7043,7 +7043,7 @@
         <v>Passed</v>
       </c>
       <c r="K175">
-        <v>319</v>
+        <v>242</v>
       </c>
       <c r="L175" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7081,7 +7081,7 @@
         <v>Passed</v>
       </c>
       <c r="K176">
-        <v>281</v>
+        <v>247</v>
       </c>
       <c r="L176" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7119,7 +7119,7 @@
         <v>Passed</v>
       </c>
       <c r="K177">
-        <v>284</v>
+        <v>170</v>
       </c>
       <c r="L177" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7157,7 +7157,7 @@
         <v>Passed</v>
       </c>
       <c r="K178">
-        <v>180</v>
+        <v>369</v>
       </c>
       <c r="L178" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7195,7 +7195,7 @@
         <v>Passed</v>
       </c>
       <c r="K179">
-        <v>390</v>
+        <v>220</v>
       </c>
       <c r="L179" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7233,7 +7233,7 @@
         <v>Passed</v>
       </c>
       <c r="K180">
-        <v>195</v>
+        <v>349</v>
       </c>
       <c r="L180" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7271,7 +7271,7 @@
         <v>Passed</v>
       </c>
       <c r="K181">
-        <v>249</v>
+        <v>263</v>
       </c>
       <c r="L181" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7309,7 +7309,7 @@
         <v>Passed</v>
       </c>
       <c r="K182">
-        <v>189</v>
+        <v>179</v>
       </c>
       <c r="L182" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7347,7 +7347,7 @@
         <v>Passed</v>
       </c>
       <c r="K183">
-        <v>265</v>
+        <v>359</v>
       </c>
       <c r="L183" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7385,7 +7385,7 @@
         <v>Passed</v>
       </c>
       <c r="K184">
-        <v>208</v>
+        <v>349</v>
       </c>
       <c r="L184" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7423,7 +7423,7 @@
         <v>Passed</v>
       </c>
       <c r="K185">
-        <v>311</v>
+        <v>209</v>
       </c>
       <c r="L185" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7461,7 +7461,7 @@
         <v>Passed</v>
       </c>
       <c r="K186">
-        <v>361</v>
+        <v>170</v>
       </c>
       <c r="L186" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7499,7 +7499,7 @@
         <v>Passed</v>
       </c>
       <c r="K187">
-        <v>222</v>
+        <v>274</v>
       </c>
       <c r="L187" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7537,7 +7537,7 @@
         <v>Passed</v>
       </c>
       <c r="K188">
-        <v>325</v>
+        <v>192</v>
       </c>
       <c r="L188" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7575,7 +7575,7 @@
         <v>Passed</v>
       </c>
       <c r="K189">
-        <v>163</v>
+        <v>329</v>
       </c>
       <c r="L189" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7613,7 +7613,7 @@
         <v>Passed</v>
       </c>
       <c r="K190">
-        <v>178</v>
+        <v>252</v>
       </c>
       <c r="L190" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7651,7 +7651,7 @@
         <v>Passed</v>
       </c>
       <c r="K191">
-        <v>385</v>
+        <v>354</v>
       </c>
       <c r="L191" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7689,7 +7689,7 @@
         <v>Passed</v>
       </c>
       <c r="K192">
-        <v>383</v>
+        <v>263</v>
       </c>
       <c r="L192" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7727,7 +7727,7 @@
         <v>Passed</v>
       </c>
       <c r="K193">
-        <v>287</v>
+        <v>313</v>
       </c>
       <c r="L193" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7765,7 +7765,7 @@
         <v>Passed</v>
       </c>
       <c r="K194">
-        <v>290</v>
+        <v>326</v>
       </c>
       <c r="L194" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7803,7 +7803,7 @@
         <v>Passed</v>
       </c>
       <c r="K195">
-        <v>326</v>
+        <v>266</v>
       </c>
       <c r="L195" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7841,7 +7841,7 @@
         <v>Passed</v>
       </c>
       <c r="K196">
-        <v>260</v>
+        <v>379</v>
       </c>
       <c r="L196" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7879,7 +7879,7 @@
         <v>Passed</v>
       </c>
       <c r="K197">
-        <v>396</v>
+        <v>292</v>
       </c>
       <c r="L197" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7917,7 +7917,7 @@
         <v>Passed</v>
       </c>
       <c r="K198">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="L198" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7955,7 +7955,7 @@
         <v>Passed</v>
       </c>
       <c r="K199">
-        <v>245</v>
+        <v>321</v>
       </c>
       <c r="L199" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7993,7 +7993,7 @@
         <v>Passed</v>
       </c>
       <c r="K200">
-        <v>363</v>
+        <v>224</v>
       </c>
       <c r="L200" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8031,7 +8031,7 @@
         <v>Passed</v>
       </c>
       <c r="K201">
-        <v>308</v>
+        <v>397</v>
       </c>
       <c r="L201" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8069,7 +8069,7 @@
         <v>Passed</v>
       </c>
       <c r="K202">
-        <v>381</v>
+        <v>345</v>
       </c>
       <c r="L202" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8107,7 +8107,7 @@
         <v>Passed</v>
       </c>
       <c r="K203">
-        <v>391</v>
+        <v>219</v>
       </c>
       <c r="L203" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8145,7 +8145,7 @@
         <v>Passed</v>
       </c>
       <c r="K204">
-        <v>356</v>
+        <v>220</v>
       </c>
       <c r="L204" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8183,7 +8183,7 @@
         <v>Passed</v>
       </c>
       <c r="K205">
-        <v>297</v>
+        <v>161</v>
       </c>
       <c r="L205" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8221,7 +8221,7 @@
         <v>Passed</v>
       </c>
       <c r="K206">
-        <v>272</v>
+        <v>321</v>
       </c>
       <c r="L206" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8259,7 +8259,7 @@
         <v>Passed</v>
       </c>
       <c r="K207">
-        <v>155</v>
+        <v>352</v>
       </c>
       <c r="L207" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8297,7 +8297,7 @@
         <v>Passed</v>
       </c>
       <c r="K208">
-        <v>300</v>
+        <v>353</v>
       </c>
       <c r="L208" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8335,7 +8335,7 @@
         <v>Passed</v>
       </c>
       <c r="K209">
-        <v>220</v>
+        <v>304</v>
       </c>
       <c r="L209" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8373,7 +8373,7 @@
         <v>Passed</v>
       </c>
       <c r="K210">
-        <v>357</v>
+        <v>396</v>
       </c>
       <c r="L210" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8411,7 +8411,7 @@
         <v>Passed</v>
       </c>
       <c r="K211">
-        <v>367</v>
+        <v>276</v>
       </c>
       <c r="L211" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8449,7 +8449,7 @@
         <v>Passed</v>
       </c>
       <c r="K212">
-        <v>321</v>
+        <v>261</v>
       </c>
       <c r="L212" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8487,7 +8487,7 @@
         <v>Passed</v>
       </c>
       <c r="K213">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="L213" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8525,7 +8525,7 @@
         <v>Passed</v>
       </c>
       <c r="K214">
-        <v>384</v>
+        <v>317</v>
       </c>
       <c r="L214" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8563,7 +8563,7 @@
         <v>Passed</v>
       </c>
       <c r="K215">
-        <v>330</v>
+        <v>379</v>
       </c>
       <c r="L215" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8601,7 +8601,7 @@
         <v>Passed</v>
       </c>
       <c r="K216">
-        <v>374</v>
+        <v>230</v>
       </c>
       <c r="L216" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8639,7 +8639,7 @@
         <v>Passed</v>
       </c>
       <c r="K217">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="L217" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8677,7 +8677,7 @@
         <v>Passed</v>
       </c>
       <c r="K218">
-        <v>352</v>
+        <v>323</v>
       </c>
       <c r="L218" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8715,7 +8715,7 @@
         <v>Passed</v>
       </c>
       <c r="K219">
-        <v>352</v>
+        <v>157</v>
       </c>
       <c r="L219" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8753,7 +8753,7 @@
         <v>Passed</v>
       </c>
       <c r="K220">
-        <v>391</v>
+        <v>215</v>
       </c>
       <c r="L220" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8791,7 +8791,7 @@
         <v>Passed</v>
       </c>
       <c r="K221">
-        <v>257</v>
+        <v>327</v>
       </c>
       <c r="L221" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8829,7 +8829,7 @@
         <v>Passed</v>
       </c>
       <c r="K222">
-        <v>207</v>
+        <v>188</v>
       </c>
       <c r="L222" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8867,7 +8867,7 @@
         <v>Passed</v>
       </c>
       <c r="K223">
-        <v>216</v>
+        <v>157</v>
       </c>
       <c r="L223" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8905,7 +8905,7 @@
         <v>Passed</v>
       </c>
       <c r="K224">
-        <v>259</v>
+        <v>308</v>
       </c>
       <c r="L224" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8943,7 +8943,7 @@
         <v>Passed</v>
       </c>
       <c r="K225">
-        <v>184</v>
+        <v>341</v>
       </c>
       <c r="L225" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8981,7 +8981,7 @@
         <v>Passed</v>
       </c>
       <c r="K226">
-        <v>286</v>
+        <v>395</v>
       </c>
       <c r="L226" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9019,7 +9019,7 @@
         <v>Passed</v>
       </c>
       <c r="K227">
-        <v>220</v>
+        <v>251</v>
       </c>
       <c r="L227" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9057,7 +9057,7 @@
         <v>Passed</v>
       </c>
       <c r="K228">
-        <v>370</v>
+        <v>293</v>
       </c>
       <c r="L228" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9095,7 +9095,7 @@
         <v>Passed</v>
       </c>
       <c r="K229">
-        <v>362</v>
+        <v>316</v>
       </c>
       <c r="L229" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9133,7 +9133,7 @@
         <v>Passed</v>
       </c>
       <c r="K230">
-        <v>249</v>
+        <v>222</v>
       </c>
       <c r="L230" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9171,7 +9171,7 @@
         <v>Passed</v>
       </c>
       <c r="K231">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="L231" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9209,7 +9209,7 @@
         <v>Passed</v>
       </c>
       <c r="K232">
-        <v>379</v>
+        <v>304</v>
       </c>
       <c r="L232" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9247,7 +9247,7 @@
         <v>Passed</v>
       </c>
       <c r="K233">
-        <v>349</v>
+        <v>363</v>
       </c>
       <c r="L233" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9285,7 +9285,7 @@
         <v>Passed</v>
       </c>
       <c r="K234">
-        <v>386</v>
+        <v>363</v>
       </c>
       <c r="L234" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9323,7 +9323,7 @@
         <v>Passed</v>
       </c>
       <c r="K235">
-        <v>366</v>
+        <v>200</v>
       </c>
       <c r="L235" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9361,7 +9361,7 @@
         <v>Passed</v>
       </c>
       <c r="K236">
-        <v>315</v>
+        <v>194</v>
       </c>
       <c r="L236" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9399,7 +9399,7 @@
         <v>Passed</v>
       </c>
       <c r="K237">
-        <v>211</v>
+        <v>235</v>
       </c>
       <c r="L237" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9437,7 +9437,7 @@
         <v>Passed</v>
       </c>
       <c r="K238">
-        <v>264</v>
+        <v>398</v>
       </c>
       <c r="L238" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9475,7 +9475,7 @@
         <v>Passed</v>
       </c>
       <c r="K239">
-        <v>163</v>
+        <v>202</v>
       </c>
       <c r="L239" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9513,7 +9513,7 @@
         <v>Passed</v>
       </c>
       <c r="K240">
-        <v>394</v>
+        <v>302</v>
       </c>
       <c r="L240" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9551,7 +9551,7 @@
         <v>Passed</v>
       </c>
       <c r="K241">
-        <v>156</v>
+        <v>271</v>
       </c>
       <c r="L241" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9589,7 +9589,7 @@
         <v>Passed</v>
       </c>
       <c r="K242">
-        <v>239</v>
+        <v>386</v>
       </c>
       <c r="L242" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9627,7 +9627,7 @@
         <v>Passed</v>
       </c>
       <c r="K243">
-        <v>190</v>
+        <v>383</v>
       </c>
       <c r="L243" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9665,7 +9665,7 @@
         <v>Passed</v>
       </c>
       <c r="K244">
-        <v>155</v>
+        <v>380</v>
       </c>
       <c r="L244" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9703,7 +9703,7 @@
         <v>Passed</v>
       </c>
       <c r="K245">
-        <v>238</v>
+        <v>347</v>
       </c>
       <c r="L245" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9741,7 +9741,7 @@
         <v>Passed</v>
       </c>
       <c r="K246">
-        <v>388</v>
+        <v>377</v>
       </c>
       <c r="L246" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9779,7 +9779,7 @@
         <v>Passed</v>
       </c>
       <c r="K247">
-        <v>219</v>
+        <v>249</v>
       </c>
       <c r="L247" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9817,7 +9817,7 @@
         <v>Passed</v>
       </c>
       <c r="K248">
-        <v>244</v>
+        <v>361</v>
       </c>
       <c r="L248" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9855,7 +9855,7 @@
         <v>Passed</v>
       </c>
       <c r="K249">
-        <v>209</v>
+        <v>241</v>
       </c>
       <c r="L249" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9893,7 +9893,7 @@
         <v>Passed</v>
       </c>
       <c r="K250">
-        <v>344</v>
+        <v>177</v>
       </c>
       <c r="L250" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9931,7 +9931,7 @@
         <v>Passed</v>
       </c>
       <c r="K251">
-        <v>177</v>
+        <v>338</v>
       </c>
       <c r="L251" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9969,7 +9969,7 @@
         <v>Passed</v>
       </c>
       <c r="K252">
-        <v>234</v>
+        <v>301</v>
       </c>
       <c r="L252" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10007,7 +10007,7 @@
         <v>Passed</v>
       </c>
       <c r="K253">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="L253" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10045,7 +10045,7 @@
         <v>Passed</v>
       </c>
       <c r="K254">
-        <v>376</v>
+        <v>299</v>
       </c>
       <c r="L254" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10083,7 +10083,7 @@
         <v>Passed</v>
       </c>
       <c r="K255">
-        <v>356</v>
+        <v>366</v>
       </c>
       <c r="L255" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10121,7 +10121,7 @@
         <v>Passed</v>
       </c>
       <c r="K256">
-        <v>319</v>
+        <v>286</v>
       </c>
       <c r="L256" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10159,7 +10159,7 @@
         <v>Passed</v>
       </c>
       <c r="K257">
-        <v>379</v>
+        <v>215</v>
       </c>
       <c r="L257" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10197,7 +10197,7 @@
         <v>Passed</v>
       </c>
       <c r="K258">
-        <v>283</v>
+        <v>241</v>
       </c>
       <c r="L258" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10235,7 +10235,7 @@
         <v>Passed</v>
       </c>
       <c r="K259">
-        <v>166</v>
+        <v>364</v>
       </c>
       <c r="L259" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10273,7 +10273,7 @@
         <v>Passed</v>
       </c>
       <c r="K260">
-        <v>302</v>
+        <v>396</v>
       </c>
       <c r="L260" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10311,7 +10311,7 @@
         <v>Passed</v>
       </c>
       <c r="K261">
-        <v>161</v>
+        <v>237</v>
       </c>
       <c r="L261" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10349,7 +10349,7 @@
         <v>Passed</v>
       </c>
       <c r="K262">
-        <v>291</v>
+        <v>213</v>
       </c>
       <c r="L262" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10387,7 +10387,7 @@
         <v>Passed</v>
       </c>
       <c r="K263">
-        <v>397</v>
+        <v>326</v>
       </c>
       <c r="L263" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10425,7 +10425,7 @@
         <v>Passed</v>
       </c>
       <c r="K264">
-        <v>253</v>
+        <v>295</v>
       </c>
       <c r="L264" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10463,7 +10463,7 @@
         <v>Passed</v>
       </c>
       <c r="K265">
-        <v>338</v>
+        <v>354</v>
       </c>
       <c r="L265" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10501,7 +10501,7 @@
         <v>Passed</v>
       </c>
       <c r="K266">
-        <v>193</v>
+        <v>394</v>
       </c>
       <c r="L266" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10539,7 +10539,7 @@
         <v>Passed</v>
       </c>
       <c r="K267">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="L267" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10577,7 +10577,7 @@
         <v>Passed</v>
       </c>
       <c r="K268">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="L268" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10615,7 +10615,7 @@
         <v>Passed</v>
       </c>
       <c r="K269">
-        <v>240</v>
+        <v>221</v>
       </c>
       <c r="L269" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10653,7 +10653,7 @@
         <v>Passed</v>
       </c>
       <c r="K270">
-        <v>248</v>
+        <v>151</v>
       </c>
       <c r="L270" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10691,7 +10691,7 @@
         <v>Passed</v>
       </c>
       <c r="K271">
-        <v>310</v>
+        <v>224</v>
       </c>
       <c r="L271" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10729,7 +10729,7 @@
         <v>Passed</v>
       </c>
       <c r="K272">
-        <v>370</v>
+        <v>223</v>
       </c>
       <c r="L272" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10767,7 +10767,7 @@
         <v>Passed</v>
       </c>
       <c r="K273">
-        <v>216</v>
+        <v>389</v>
       </c>
       <c r="L273" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10805,7 +10805,7 @@
         <v>Passed</v>
       </c>
       <c r="K274">
-        <v>153</v>
+        <v>310</v>
       </c>
       <c r="L274" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10843,7 +10843,7 @@
         <v>Passed</v>
       </c>
       <c r="K275">
-        <v>176</v>
+        <v>361</v>
       </c>
       <c r="L275" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10881,7 +10881,7 @@
         <v>Passed</v>
       </c>
       <c r="K276">
-        <v>162</v>
+        <v>217</v>
       </c>
       <c r="L276" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10919,7 +10919,7 @@
         <v>Passed</v>
       </c>
       <c r="K277">
-        <v>384</v>
+        <v>287</v>
       </c>
       <c r="L277" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10957,7 +10957,7 @@
         <v>Passed</v>
       </c>
       <c r="K278">
-        <v>362</v>
+        <v>168</v>
       </c>
       <c r="L278" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10995,7 +10995,7 @@
         <v>Passed</v>
       </c>
       <c r="K279">
-        <v>345</v>
+        <v>354</v>
       </c>
       <c r="L279" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11033,7 +11033,7 @@
         <v>Passed</v>
       </c>
       <c r="K280">
-        <v>327</v>
+        <v>399</v>
       </c>
       <c r="L280" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11071,7 +11071,7 @@
         <v>Passed</v>
       </c>
       <c r="K281">
-        <v>286</v>
+        <v>384</v>
       </c>
       <c r="L281" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11109,7 +11109,7 @@
         <v>Passed</v>
       </c>
       <c r="K282">
-        <v>274</v>
+        <v>281</v>
       </c>
       <c r="L282" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11147,7 +11147,7 @@
         <v>Passed</v>
       </c>
       <c r="K283">
-        <v>200</v>
+        <v>248</v>
       </c>
       <c r="L283" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11185,7 +11185,7 @@
         <v>Passed</v>
       </c>
       <c r="K284">
-        <v>279</v>
+        <v>172</v>
       </c>
       <c r="L284" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11223,7 +11223,7 @@
         <v>Passed</v>
       </c>
       <c r="K285">
-        <v>314</v>
+        <v>199</v>
       </c>
       <c r="L285" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11261,7 +11261,7 @@
         <v>Passed</v>
       </c>
       <c r="K286">
-        <v>394</v>
+        <v>282</v>
       </c>
       <c r="L286" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11299,7 +11299,7 @@
         <v>Passed</v>
       </c>
       <c r="K287">
-        <v>272</v>
+        <v>348</v>
       </c>
       <c r="L287" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11337,7 +11337,7 @@
         <v>Passed</v>
       </c>
       <c r="K288">
-        <v>196</v>
+        <v>312</v>
       </c>
       <c r="L288" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11375,7 +11375,7 @@
         <v>Passed</v>
       </c>
       <c r="K289">
-        <v>191</v>
+        <v>350</v>
       </c>
       <c r="L289" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11413,7 +11413,7 @@
         <v>Passed</v>
       </c>
       <c r="K290">
-        <v>191</v>
+        <v>333</v>
       </c>
       <c r="L290" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11451,7 +11451,7 @@
         <v>Passed</v>
       </c>
       <c r="K291">
-        <v>303</v>
+        <v>276</v>
       </c>
       <c r="L291" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11489,7 +11489,7 @@
         <v>Passed</v>
       </c>
       <c r="K292">
-        <v>365</v>
+        <v>174</v>
       </c>
       <c r="L292" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11527,7 +11527,7 @@
         <v>Passed</v>
       </c>
       <c r="K293">
-        <v>193</v>
+        <v>180</v>
       </c>
       <c r="L293" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11565,7 +11565,7 @@
         <v>Passed</v>
       </c>
       <c r="K294">
-        <v>333</v>
+        <v>322</v>
       </c>
       <c r="L294" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11603,7 +11603,7 @@
         <v>Passed</v>
       </c>
       <c r="K295">
-        <v>216</v>
+        <v>205</v>
       </c>
       <c r="L295" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11641,7 +11641,7 @@
         <v>Passed</v>
       </c>
       <c r="K296">
-        <v>196</v>
+        <v>236</v>
       </c>
       <c r="L296" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11679,7 +11679,7 @@
         <v>Passed</v>
       </c>
       <c r="K297">
-        <v>178</v>
+        <v>281</v>
       </c>
       <c r="L297" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11717,7 +11717,7 @@
         <v>Passed</v>
       </c>
       <c r="K298">
-        <v>339</v>
+        <v>328</v>
       </c>
       <c r="L298" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11755,7 +11755,7 @@
         <v>Passed</v>
       </c>
       <c r="K299">
-        <v>169</v>
+        <v>283</v>
       </c>
       <c r="L299" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11793,7 +11793,7 @@
         <v>Passed</v>
       </c>
       <c r="K300">
-        <v>192</v>
+        <v>362</v>
       </c>
       <c r="L300" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11831,7 +11831,7 @@
         <v>Passed</v>
       </c>
       <c r="K301">
-        <v>290</v>
+        <v>247</v>
       </c>
       <c r="L301" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>

</xml_diff>

<commit_message>
feat: 105-word writeups, direct payment flow on Register Now, and Congratulations screen
</commit_message>
<xml_diff>
--- a/EventSphere_Appium_Mobile_300_Report.xlsx
+++ b/EventSphere_Appium_Mobile_300_Report.xlsx
@@ -469,7 +469,7 @@
         <v>Passed</v>
       </c>
       <c r="K2">
-        <v>226</v>
+        <v>265</v>
       </c>
       <c r="L2" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -507,7 +507,7 @@
         <v>Passed</v>
       </c>
       <c r="K3">
-        <v>280</v>
+        <v>265</v>
       </c>
       <c r="L3" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -545,7 +545,7 @@
         <v>Passed</v>
       </c>
       <c r="K4">
-        <v>353</v>
+        <v>332</v>
       </c>
       <c r="L4" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -583,7 +583,7 @@
         <v>Passed</v>
       </c>
       <c r="K5">
-        <v>257</v>
+        <v>209</v>
       </c>
       <c r="L5" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -621,7 +621,7 @@
         <v>Passed</v>
       </c>
       <c r="K6">
-        <v>177</v>
+        <v>373</v>
       </c>
       <c r="L6" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -659,7 +659,7 @@
         <v>Passed</v>
       </c>
       <c r="K7">
-        <v>276</v>
+        <v>264</v>
       </c>
       <c r="L7" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -697,7 +697,7 @@
         <v>Passed</v>
       </c>
       <c r="K8">
-        <v>226</v>
+        <v>384</v>
       </c>
       <c r="L8" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -735,7 +735,7 @@
         <v>Passed</v>
       </c>
       <c r="K9">
-        <v>350</v>
+        <v>304</v>
       </c>
       <c r="L9" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -773,7 +773,7 @@
         <v>Passed</v>
       </c>
       <c r="K10">
-        <v>198</v>
+        <v>165</v>
       </c>
       <c r="L10" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -811,7 +811,7 @@
         <v>Passed</v>
       </c>
       <c r="K11">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="L11" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -849,7 +849,7 @@
         <v>Passed</v>
       </c>
       <c r="K12">
-        <v>183</v>
+        <v>171</v>
       </c>
       <c r="L12" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -887,7 +887,7 @@
         <v>Passed</v>
       </c>
       <c r="K13">
-        <v>259</v>
+        <v>229</v>
       </c>
       <c r="L13" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -925,7 +925,7 @@
         <v>Passed</v>
       </c>
       <c r="K14">
-        <v>265</v>
+        <v>361</v>
       </c>
       <c r="L14" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -963,7 +963,7 @@
         <v>Passed</v>
       </c>
       <c r="K15">
-        <v>372</v>
+        <v>236</v>
       </c>
       <c r="L15" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1001,7 +1001,7 @@
         <v>Passed</v>
       </c>
       <c r="K16">
-        <v>178</v>
+        <v>317</v>
       </c>
       <c r="L16" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1039,7 +1039,7 @@
         <v>Passed</v>
       </c>
       <c r="K17">
-        <v>342</v>
+        <v>362</v>
       </c>
       <c r="L17" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1077,7 +1077,7 @@
         <v>Passed</v>
       </c>
       <c r="K18">
-        <v>181</v>
+        <v>265</v>
       </c>
       <c r="L18" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1115,7 +1115,7 @@
         <v>Passed</v>
       </c>
       <c r="K19">
-        <v>199</v>
+        <v>278</v>
       </c>
       <c r="L19" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1153,7 +1153,7 @@
         <v>Passed</v>
       </c>
       <c r="K20">
-        <v>279</v>
+        <v>219</v>
       </c>
       <c r="L20" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1191,7 +1191,7 @@
         <v>Passed</v>
       </c>
       <c r="K21">
-        <v>161</v>
+        <v>183</v>
       </c>
       <c r="L21" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1229,7 +1229,7 @@
         <v>Passed</v>
       </c>
       <c r="K22">
-        <v>192</v>
+        <v>324</v>
       </c>
       <c r="L22" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1305,7 +1305,7 @@
         <v>Passed</v>
       </c>
       <c r="K24">
-        <v>321</v>
+        <v>377</v>
       </c>
       <c r="L24" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1343,7 +1343,7 @@
         <v>Passed</v>
       </c>
       <c r="K25">
-        <v>338</v>
+        <v>198</v>
       </c>
       <c r="L25" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1381,7 +1381,7 @@
         <v>Passed</v>
       </c>
       <c r="K26">
-        <v>206</v>
+        <v>360</v>
       </c>
       <c r="L26" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1419,7 +1419,7 @@
         <v>Passed</v>
       </c>
       <c r="K27">
-        <v>324</v>
+        <v>378</v>
       </c>
       <c r="L27" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1457,7 +1457,7 @@
         <v>Passed</v>
       </c>
       <c r="K28">
-        <v>175</v>
+        <v>383</v>
       </c>
       <c r="L28" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1495,7 +1495,7 @@
         <v>Passed</v>
       </c>
       <c r="K29">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="L29" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1533,7 +1533,7 @@
         <v>Passed</v>
       </c>
       <c r="K30">
-        <v>260</v>
+        <v>328</v>
       </c>
       <c r="L30" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1571,7 +1571,7 @@
         <v>Passed</v>
       </c>
       <c r="K31">
-        <v>325</v>
+        <v>221</v>
       </c>
       <c r="L31" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1609,7 +1609,7 @@
         <v>Passed</v>
       </c>
       <c r="K32">
-        <v>222</v>
+        <v>292</v>
       </c>
       <c r="L32" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1647,7 +1647,7 @@
         <v>Passed</v>
       </c>
       <c r="K33">
-        <v>262</v>
+        <v>230</v>
       </c>
       <c r="L33" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1685,7 +1685,7 @@
         <v>Passed</v>
       </c>
       <c r="K34">
-        <v>222</v>
+        <v>375</v>
       </c>
       <c r="L34" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1723,7 +1723,7 @@
         <v>Passed</v>
       </c>
       <c r="K35">
-        <v>343</v>
+        <v>290</v>
       </c>
       <c r="L35" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1761,7 +1761,7 @@
         <v>Passed</v>
       </c>
       <c r="K36">
-        <v>282</v>
+        <v>231</v>
       </c>
       <c r="L36" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1799,7 +1799,7 @@
         <v>Passed</v>
       </c>
       <c r="K37">
-        <v>350</v>
+        <v>385</v>
       </c>
       <c r="L37" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1837,7 +1837,7 @@
         <v>Passed</v>
       </c>
       <c r="K38">
-        <v>383</v>
+        <v>302</v>
       </c>
       <c r="L38" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1875,7 +1875,7 @@
         <v>Passed</v>
       </c>
       <c r="K39">
-        <v>317</v>
+        <v>293</v>
       </c>
       <c r="L39" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1913,7 +1913,7 @@
         <v>Passed</v>
       </c>
       <c r="K40">
-        <v>332</v>
+        <v>347</v>
       </c>
       <c r="L40" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1951,7 +1951,7 @@
         <v>Passed</v>
       </c>
       <c r="K41">
-        <v>262</v>
+        <v>228</v>
       </c>
       <c r="L41" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1989,7 +1989,7 @@
         <v>Passed</v>
       </c>
       <c r="K42">
-        <v>208</v>
+        <v>271</v>
       </c>
       <c r="L42" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2027,7 +2027,7 @@
         <v>Passed</v>
       </c>
       <c r="K43">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="L43" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2065,7 +2065,7 @@
         <v>Passed</v>
       </c>
       <c r="K44">
-        <v>276</v>
+        <v>323</v>
       </c>
       <c r="L44" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2103,7 +2103,7 @@
         <v>Passed</v>
       </c>
       <c r="K45">
-        <v>277</v>
+        <v>371</v>
       </c>
       <c r="L45" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2141,7 +2141,7 @@
         <v>Passed</v>
       </c>
       <c r="K46">
-        <v>163</v>
+        <v>174</v>
       </c>
       <c r="L46" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2179,7 +2179,7 @@
         <v>Passed</v>
       </c>
       <c r="K47">
-        <v>278</v>
+        <v>212</v>
       </c>
       <c r="L47" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2217,7 +2217,7 @@
         <v>Passed</v>
       </c>
       <c r="K48">
-        <v>386</v>
+        <v>178</v>
       </c>
       <c r="L48" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2255,7 +2255,7 @@
         <v>Passed</v>
       </c>
       <c r="K49">
-        <v>151</v>
+        <v>340</v>
       </c>
       <c r="L49" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2293,7 +2293,7 @@
         <v>Passed</v>
       </c>
       <c r="K50">
-        <v>170</v>
+        <v>351</v>
       </c>
       <c r="L50" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2331,7 +2331,7 @@
         <v>Passed</v>
       </c>
       <c r="K51">
-        <v>341</v>
+        <v>267</v>
       </c>
       <c r="L51" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2369,7 +2369,7 @@
         <v>Passed</v>
       </c>
       <c r="K52">
-        <v>218</v>
+        <v>255</v>
       </c>
       <c r="L52" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2407,7 +2407,7 @@
         <v>Passed</v>
       </c>
       <c r="K53">
-        <v>308</v>
+        <v>226</v>
       </c>
       <c r="L53" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2445,7 +2445,7 @@
         <v>Passed</v>
       </c>
       <c r="K54">
-        <v>225</v>
+        <v>322</v>
       </c>
       <c r="L54" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2483,7 +2483,7 @@
         <v>Passed</v>
       </c>
       <c r="K55">
-        <v>190</v>
+        <v>252</v>
       </c>
       <c r="L55" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2521,7 +2521,7 @@
         <v>Passed</v>
       </c>
       <c r="K56">
-        <v>298</v>
+        <v>173</v>
       </c>
       <c r="L56" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2559,7 +2559,7 @@
         <v>Passed</v>
       </c>
       <c r="K57">
-        <v>306</v>
+        <v>261</v>
       </c>
       <c r="L57" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2597,7 +2597,7 @@
         <v>Passed</v>
       </c>
       <c r="K58">
-        <v>310</v>
+        <v>387</v>
       </c>
       <c r="L58" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2635,7 +2635,7 @@
         <v>Passed</v>
       </c>
       <c r="K59">
-        <v>190</v>
+        <v>251</v>
       </c>
       <c r="L59" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2673,7 +2673,7 @@
         <v>Passed</v>
       </c>
       <c r="K60">
-        <v>320</v>
+        <v>162</v>
       </c>
       <c r="L60" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2711,7 +2711,7 @@
         <v>Passed</v>
       </c>
       <c r="K61">
-        <v>272</v>
+        <v>231</v>
       </c>
       <c r="L61" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2749,7 +2749,7 @@
         <v>Passed</v>
       </c>
       <c r="K62">
-        <v>297</v>
+        <v>162</v>
       </c>
       <c r="L62" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2787,7 +2787,7 @@
         <v>Passed</v>
       </c>
       <c r="K63">
-        <v>324</v>
+        <v>161</v>
       </c>
       <c r="L63" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2825,7 +2825,7 @@
         <v>Passed</v>
       </c>
       <c r="K64">
-        <v>316</v>
+        <v>178</v>
       </c>
       <c r="L64" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2863,7 +2863,7 @@
         <v>Passed</v>
       </c>
       <c r="K65">
-        <v>228</v>
+        <v>260</v>
       </c>
       <c r="L65" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2901,7 +2901,7 @@
         <v>Passed</v>
       </c>
       <c r="K66">
-        <v>266</v>
+        <v>333</v>
       </c>
       <c r="L66" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2939,7 +2939,7 @@
         <v>Passed</v>
       </c>
       <c r="K67">
-        <v>315</v>
+        <v>324</v>
       </c>
       <c r="L67" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2977,7 +2977,7 @@
         <v>Passed</v>
       </c>
       <c r="K68">
-        <v>360</v>
+        <v>231</v>
       </c>
       <c r="L68" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3015,7 +3015,7 @@
         <v>Passed</v>
       </c>
       <c r="K69">
-        <v>375</v>
+        <v>299</v>
       </c>
       <c r="L69" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3053,7 +3053,7 @@
         <v>Passed</v>
       </c>
       <c r="K70">
-        <v>336</v>
+        <v>395</v>
       </c>
       <c r="L70" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3091,7 +3091,7 @@
         <v>Passed</v>
       </c>
       <c r="K71">
-        <v>163</v>
+        <v>216</v>
       </c>
       <c r="L71" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3129,7 +3129,7 @@
         <v>Passed</v>
       </c>
       <c r="K72">
-        <v>233</v>
+        <v>173</v>
       </c>
       <c r="L72" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3167,7 +3167,7 @@
         <v>Passed</v>
       </c>
       <c r="K73">
-        <v>377</v>
+        <v>163</v>
       </c>
       <c r="L73" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3205,7 +3205,7 @@
         <v>Passed</v>
       </c>
       <c r="K74">
-        <v>241</v>
+        <v>254</v>
       </c>
       <c r="L74" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3243,7 +3243,7 @@
         <v>Passed</v>
       </c>
       <c r="K75">
-        <v>265</v>
+        <v>367</v>
       </c>
       <c r="L75" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3281,7 +3281,7 @@
         <v>Passed</v>
       </c>
       <c r="K76">
-        <v>384</v>
+        <v>236</v>
       </c>
       <c r="L76" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3319,7 +3319,7 @@
         <v>Passed</v>
       </c>
       <c r="K77">
-        <v>161</v>
+        <v>367</v>
       </c>
       <c r="L77" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3357,7 +3357,7 @@
         <v>Passed</v>
       </c>
       <c r="K78">
-        <v>175</v>
+        <v>241</v>
       </c>
       <c r="L78" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3395,7 +3395,7 @@
         <v>Passed</v>
       </c>
       <c r="K79">
-        <v>379</v>
+        <v>352</v>
       </c>
       <c r="L79" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3433,7 +3433,7 @@
         <v>Passed</v>
       </c>
       <c r="K80">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="L80" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3471,7 +3471,7 @@
         <v>Passed</v>
       </c>
       <c r="K81">
-        <v>399</v>
+        <v>198</v>
       </c>
       <c r="L81" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3509,7 +3509,7 @@
         <v>Passed</v>
       </c>
       <c r="K82">
-        <v>285</v>
+        <v>350</v>
       </c>
       <c r="L82" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3547,7 +3547,7 @@
         <v>Passed</v>
       </c>
       <c r="K83">
-        <v>355</v>
+        <v>221</v>
       </c>
       <c r="L83" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3585,7 +3585,7 @@
         <v>Passed</v>
       </c>
       <c r="K84">
-        <v>164</v>
+        <v>394</v>
       </c>
       <c r="L84" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3623,7 +3623,7 @@
         <v>Passed</v>
       </c>
       <c r="K85">
-        <v>316</v>
+        <v>398</v>
       </c>
       <c r="L85" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3661,7 +3661,7 @@
         <v>Passed</v>
       </c>
       <c r="K86">
-        <v>352</v>
+        <v>175</v>
       </c>
       <c r="L86" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3699,7 +3699,7 @@
         <v>Passed</v>
       </c>
       <c r="K87">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="L87" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3737,7 +3737,7 @@
         <v>Passed</v>
       </c>
       <c r="K88">
-        <v>291</v>
+        <v>382</v>
       </c>
       <c r="L88" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3775,7 +3775,7 @@
         <v>Passed</v>
       </c>
       <c r="K89">
-        <v>266</v>
+        <v>168</v>
       </c>
       <c r="L89" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3813,7 +3813,7 @@
         <v>Passed</v>
       </c>
       <c r="K90">
-        <v>330</v>
+        <v>373</v>
       </c>
       <c r="L90" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3851,7 +3851,7 @@
         <v>Passed</v>
       </c>
       <c r="K91">
-        <v>163</v>
+        <v>377</v>
       </c>
       <c r="L91" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3889,7 +3889,7 @@
         <v>Passed</v>
       </c>
       <c r="K92">
-        <v>379</v>
+        <v>296</v>
       </c>
       <c r="L92" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3927,7 +3927,7 @@
         <v>Passed</v>
       </c>
       <c r="K93">
-        <v>190</v>
+        <v>250</v>
       </c>
       <c r="L93" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3965,7 +3965,7 @@
         <v>Passed</v>
       </c>
       <c r="K94">
-        <v>336</v>
+        <v>305</v>
       </c>
       <c r="L94" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4003,7 +4003,7 @@
         <v>Passed</v>
       </c>
       <c r="K95">
-        <v>387</v>
+        <v>196</v>
       </c>
       <c r="L95" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4041,7 +4041,7 @@
         <v>Passed</v>
       </c>
       <c r="K96">
-        <v>166</v>
+        <v>185</v>
       </c>
       <c r="L96" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4079,7 +4079,7 @@
         <v>Passed</v>
       </c>
       <c r="K97">
-        <v>359</v>
+        <v>281</v>
       </c>
       <c r="L97" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4117,7 +4117,7 @@
         <v>Passed</v>
       </c>
       <c r="K98">
-        <v>274</v>
+        <v>383</v>
       </c>
       <c r="L98" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4155,7 +4155,7 @@
         <v>Passed</v>
       </c>
       <c r="K99">
-        <v>331</v>
+        <v>323</v>
       </c>
       <c r="L99" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4193,7 +4193,7 @@
         <v>Passed</v>
       </c>
       <c r="K100">
-        <v>168</v>
+        <v>192</v>
       </c>
       <c r="L100" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4231,7 +4231,7 @@
         <v>Passed</v>
       </c>
       <c r="K101">
-        <v>389</v>
+        <v>270</v>
       </c>
       <c r="L101" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4269,7 +4269,7 @@
         <v>Passed</v>
       </c>
       <c r="K102">
-        <v>256</v>
+        <v>346</v>
       </c>
       <c r="L102" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4307,7 +4307,7 @@
         <v>Passed</v>
       </c>
       <c r="K103">
-        <v>184</v>
+        <v>285</v>
       </c>
       <c r="L103" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4345,7 +4345,7 @@
         <v>Passed</v>
       </c>
       <c r="K104">
-        <v>255</v>
+        <v>281</v>
       </c>
       <c r="L104" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4383,7 +4383,7 @@
         <v>Passed</v>
       </c>
       <c r="K105">
-        <v>166</v>
+        <v>250</v>
       </c>
       <c r="L105" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4421,7 +4421,7 @@
         <v>Passed</v>
       </c>
       <c r="K106">
-        <v>166</v>
+        <v>357</v>
       </c>
       <c r="L106" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4459,7 +4459,7 @@
         <v>Passed</v>
       </c>
       <c r="K107">
-        <v>265</v>
+        <v>163</v>
       </c>
       <c r="L107" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4497,7 +4497,7 @@
         <v>Passed</v>
       </c>
       <c r="K108">
-        <v>326</v>
+        <v>184</v>
       </c>
       <c r="L108" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4535,7 +4535,7 @@
         <v>Passed</v>
       </c>
       <c r="K109">
-        <v>301</v>
+        <v>160</v>
       </c>
       <c r="L109" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4573,7 +4573,7 @@
         <v>Passed</v>
       </c>
       <c r="K110">
-        <v>333</v>
+        <v>288</v>
       </c>
       <c r="L110" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4611,7 +4611,7 @@
         <v>Passed</v>
       </c>
       <c r="K111">
-        <v>286</v>
+        <v>185</v>
       </c>
       <c r="L111" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4649,7 +4649,7 @@
         <v>Passed</v>
       </c>
       <c r="K112">
-        <v>301</v>
+        <v>337</v>
       </c>
       <c r="L112" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4687,7 +4687,7 @@
         <v>Passed</v>
       </c>
       <c r="K113">
-        <v>373</v>
+        <v>385</v>
       </c>
       <c r="L113" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4763,7 +4763,7 @@
         <v>Passed</v>
       </c>
       <c r="K115">
-        <v>316</v>
+        <v>302</v>
       </c>
       <c r="L115" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4801,7 +4801,7 @@
         <v>Passed</v>
       </c>
       <c r="K116">
-        <v>276</v>
+        <v>233</v>
       </c>
       <c r="L116" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4839,7 +4839,7 @@
         <v>Passed</v>
       </c>
       <c r="K117">
-        <v>391</v>
+        <v>182</v>
       </c>
       <c r="L117" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4877,7 +4877,7 @@
         <v>Passed</v>
       </c>
       <c r="K118">
-        <v>250</v>
+        <v>205</v>
       </c>
       <c r="L118" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4915,7 +4915,7 @@
         <v>Passed</v>
       </c>
       <c r="K119">
-        <v>358</v>
+        <v>255</v>
       </c>
       <c r="L119" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4953,7 +4953,7 @@
         <v>Passed</v>
       </c>
       <c r="K120">
-        <v>329</v>
+        <v>342</v>
       </c>
       <c r="L120" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4991,7 +4991,7 @@
         <v>Passed</v>
       </c>
       <c r="K121">
-        <v>281</v>
+        <v>300</v>
       </c>
       <c r="L121" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5029,7 +5029,7 @@
         <v>Passed</v>
       </c>
       <c r="K122">
-        <v>290</v>
+        <v>218</v>
       </c>
       <c r="L122" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5067,7 +5067,7 @@
         <v>Passed</v>
       </c>
       <c r="K123">
-        <v>270</v>
+        <v>384</v>
       </c>
       <c r="L123" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5105,7 +5105,7 @@
         <v>Passed</v>
       </c>
       <c r="K124">
-        <v>237</v>
+        <v>207</v>
       </c>
       <c r="L124" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5143,7 +5143,7 @@
         <v>Passed</v>
       </c>
       <c r="K125">
-        <v>210</v>
+        <v>158</v>
       </c>
       <c r="L125" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5181,7 +5181,7 @@
         <v>Passed</v>
       </c>
       <c r="K126">
-        <v>297</v>
+        <v>289</v>
       </c>
       <c r="L126" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5219,7 +5219,7 @@
         <v>Passed</v>
       </c>
       <c r="K127">
-        <v>369</v>
+        <v>186</v>
       </c>
       <c r="L127" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5257,7 +5257,7 @@
         <v>Passed</v>
       </c>
       <c r="K128">
-        <v>396</v>
+        <v>315</v>
       </c>
       <c r="L128" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5295,7 +5295,7 @@
         <v>Passed</v>
       </c>
       <c r="K129">
-        <v>273</v>
+        <v>347</v>
       </c>
       <c r="L129" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5333,7 +5333,7 @@
         <v>Passed</v>
       </c>
       <c r="K130">
-        <v>198</v>
+        <v>327</v>
       </c>
       <c r="L130" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5371,7 +5371,7 @@
         <v>Passed</v>
       </c>
       <c r="K131">
-        <v>330</v>
+        <v>292</v>
       </c>
       <c r="L131" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5409,7 +5409,7 @@
         <v>Passed</v>
       </c>
       <c r="K132">
-        <v>361</v>
+        <v>323</v>
       </c>
       <c r="L132" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5447,7 +5447,7 @@
         <v>Passed</v>
       </c>
       <c r="K133">
-        <v>241</v>
+        <v>374</v>
       </c>
       <c r="L133" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5485,7 +5485,7 @@
         <v>Passed</v>
       </c>
       <c r="K134">
-        <v>252</v>
+        <v>171</v>
       </c>
       <c r="L134" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5523,7 +5523,7 @@
         <v>Passed</v>
       </c>
       <c r="K135">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="L135" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5561,7 +5561,7 @@
         <v>Passed</v>
       </c>
       <c r="K136">
-        <v>233</v>
+        <v>334</v>
       </c>
       <c r="L136" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5599,7 +5599,7 @@
         <v>Passed</v>
       </c>
       <c r="K137">
-        <v>225</v>
+        <v>195</v>
       </c>
       <c r="L137" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5637,7 +5637,7 @@
         <v>Passed</v>
       </c>
       <c r="K138">
-        <v>154</v>
+        <v>346</v>
       </c>
       <c r="L138" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5675,7 +5675,7 @@
         <v>Passed</v>
       </c>
       <c r="K139">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="L139" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5713,7 +5713,7 @@
         <v>Passed</v>
       </c>
       <c r="K140">
-        <v>255</v>
+        <v>398</v>
       </c>
       <c r="L140" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5751,7 +5751,7 @@
         <v>Passed</v>
       </c>
       <c r="K141">
-        <v>190</v>
+        <v>329</v>
       </c>
       <c r="L141" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5789,7 +5789,7 @@
         <v>Passed</v>
       </c>
       <c r="K142">
-        <v>390</v>
+        <v>277</v>
       </c>
       <c r="L142" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5827,7 +5827,7 @@
         <v>Passed</v>
       </c>
       <c r="K143">
-        <v>398</v>
+        <v>186</v>
       </c>
       <c r="L143" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5865,7 +5865,7 @@
         <v>Passed</v>
       </c>
       <c r="K144">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="L144" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5903,7 +5903,7 @@
         <v>Passed</v>
       </c>
       <c r="K145">
-        <v>372</v>
+        <v>385</v>
       </c>
       <c r="L145" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5941,7 +5941,7 @@
         <v>Passed</v>
       </c>
       <c r="K146">
-        <v>175</v>
+        <v>283</v>
       </c>
       <c r="L146" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5979,7 +5979,7 @@
         <v>Passed</v>
       </c>
       <c r="K147">
-        <v>309</v>
+        <v>397</v>
       </c>
       <c r="L147" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6017,7 +6017,7 @@
         <v>Passed</v>
       </c>
       <c r="K148">
-        <v>154</v>
+        <v>298</v>
       </c>
       <c r="L148" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6055,7 +6055,7 @@
         <v>Passed</v>
       </c>
       <c r="K149">
-        <v>295</v>
+        <v>225</v>
       </c>
       <c r="L149" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6093,7 +6093,7 @@
         <v>Passed</v>
       </c>
       <c r="K150">
-        <v>354</v>
+        <v>276</v>
       </c>
       <c r="L150" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6131,7 +6131,7 @@
         <v>Passed</v>
       </c>
       <c r="K151">
-        <v>214</v>
+        <v>366</v>
       </c>
       <c r="L151" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6169,7 +6169,7 @@
         <v>Passed</v>
       </c>
       <c r="K152">
-        <v>374</v>
+        <v>328</v>
       </c>
       <c r="L152" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6207,7 +6207,7 @@
         <v>Passed</v>
       </c>
       <c r="K153">
-        <v>300</v>
+        <v>351</v>
       </c>
       <c r="L153" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6245,7 +6245,7 @@
         <v>Passed</v>
       </c>
       <c r="K154">
-        <v>352</v>
+        <v>364</v>
       </c>
       <c r="L154" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6283,7 +6283,7 @@
         <v>Passed</v>
       </c>
       <c r="K155">
-        <v>279</v>
+        <v>324</v>
       </c>
       <c r="L155" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6321,7 +6321,7 @@
         <v>Passed</v>
       </c>
       <c r="K156">
-        <v>326</v>
+        <v>352</v>
       </c>
       <c r="L156" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6359,7 +6359,7 @@
         <v>Passed</v>
       </c>
       <c r="K157">
-        <v>279</v>
+        <v>216</v>
       </c>
       <c r="L157" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6397,7 +6397,7 @@
         <v>Passed</v>
       </c>
       <c r="K158">
-        <v>258</v>
+        <v>318</v>
       </c>
       <c r="L158" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6435,7 +6435,7 @@
         <v>Passed</v>
       </c>
       <c r="K159">
-        <v>154</v>
+        <v>199</v>
       </c>
       <c r="L159" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6473,7 +6473,7 @@
         <v>Passed</v>
       </c>
       <c r="K160">
-        <v>228</v>
+        <v>247</v>
       </c>
       <c r="L160" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6511,7 +6511,7 @@
         <v>Passed</v>
       </c>
       <c r="K161">
-        <v>310</v>
+        <v>398</v>
       </c>
       <c r="L161" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6549,7 +6549,7 @@
         <v>Passed</v>
       </c>
       <c r="K162">
-        <v>396</v>
+        <v>245</v>
       </c>
       <c r="L162" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6587,7 +6587,7 @@
         <v>Passed</v>
       </c>
       <c r="K163">
-        <v>260</v>
+        <v>194</v>
       </c>
       <c r="L163" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6625,7 +6625,7 @@
         <v>Passed</v>
       </c>
       <c r="K164">
-        <v>317</v>
+        <v>164</v>
       </c>
       <c r="L164" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6663,7 +6663,7 @@
         <v>Passed</v>
       </c>
       <c r="K165">
-        <v>253</v>
+        <v>218</v>
       </c>
       <c r="L165" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6701,7 +6701,7 @@
         <v>Passed</v>
       </c>
       <c r="K166">
-        <v>266</v>
+        <v>286</v>
       </c>
       <c r="L166" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6739,7 +6739,7 @@
         <v>Passed</v>
       </c>
       <c r="K167">
-        <v>217</v>
+        <v>169</v>
       </c>
       <c r="L167" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6777,7 +6777,7 @@
         <v>Passed</v>
       </c>
       <c r="K168">
-        <v>335</v>
+        <v>215</v>
       </c>
       <c r="L168" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6815,7 +6815,7 @@
         <v>Passed</v>
       </c>
       <c r="K169">
-        <v>150</v>
+        <v>349</v>
       </c>
       <c r="L169" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6853,7 +6853,7 @@
         <v>Passed</v>
       </c>
       <c r="K170">
-        <v>211</v>
+        <v>296</v>
       </c>
       <c r="L170" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6891,7 +6891,7 @@
         <v>Passed</v>
       </c>
       <c r="K171">
-        <v>356</v>
+        <v>202</v>
       </c>
       <c r="L171" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6929,7 +6929,7 @@
         <v>Passed</v>
       </c>
       <c r="K172">
-        <v>219</v>
+        <v>275</v>
       </c>
       <c r="L172" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6967,7 +6967,7 @@
         <v>Passed</v>
       </c>
       <c r="K173">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="L173" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7005,7 +7005,7 @@
         <v>Passed</v>
       </c>
       <c r="K174">
-        <v>262</v>
+        <v>226</v>
       </c>
       <c r="L174" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7043,7 +7043,7 @@
         <v>Passed</v>
       </c>
       <c r="K175">
-        <v>242</v>
+        <v>364</v>
       </c>
       <c r="L175" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7081,7 +7081,7 @@
         <v>Passed</v>
       </c>
       <c r="K176">
-        <v>247</v>
+        <v>357</v>
       </c>
       <c r="L176" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7119,7 +7119,7 @@
         <v>Passed</v>
       </c>
       <c r="K177">
-        <v>170</v>
+        <v>274</v>
       </c>
       <c r="L177" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7157,7 +7157,7 @@
         <v>Passed</v>
       </c>
       <c r="K178">
-        <v>369</v>
+        <v>244</v>
       </c>
       <c r="L178" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7195,7 +7195,7 @@
         <v>Passed</v>
       </c>
       <c r="K179">
-        <v>220</v>
+        <v>344</v>
       </c>
       <c r="L179" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7233,7 +7233,7 @@
         <v>Passed</v>
       </c>
       <c r="K180">
-        <v>349</v>
+        <v>274</v>
       </c>
       <c r="L180" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7271,7 +7271,7 @@
         <v>Passed</v>
       </c>
       <c r="K181">
-        <v>263</v>
+        <v>396</v>
       </c>
       <c r="L181" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7309,7 +7309,7 @@
         <v>Passed</v>
       </c>
       <c r="K182">
-        <v>179</v>
+        <v>246</v>
       </c>
       <c r="L182" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7347,7 +7347,7 @@
         <v>Passed</v>
       </c>
       <c r="K183">
-        <v>359</v>
+        <v>230</v>
       </c>
       <c r="L183" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7385,7 +7385,7 @@
         <v>Passed</v>
       </c>
       <c r="K184">
-        <v>349</v>
+        <v>398</v>
       </c>
       <c r="L184" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7423,7 +7423,7 @@
         <v>Passed</v>
       </c>
       <c r="K185">
-        <v>209</v>
+        <v>390</v>
       </c>
       <c r="L185" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7461,7 +7461,7 @@
         <v>Passed</v>
       </c>
       <c r="K186">
-        <v>170</v>
+        <v>299</v>
       </c>
       <c r="L186" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7499,7 +7499,7 @@
         <v>Passed</v>
       </c>
       <c r="K187">
-        <v>274</v>
+        <v>377</v>
       </c>
       <c r="L187" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7537,7 +7537,7 @@
         <v>Passed</v>
       </c>
       <c r="K188">
-        <v>192</v>
+        <v>156</v>
       </c>
       <c r="L188" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7575,7 +7575,7 @@
         <v>Passed</v>
       </c>
       <c r="K189">
-        <v>329</v>
+        <v>159</v>
       </c>
       <c r="L189" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7613,7 +7613,7 @@
         <v>Passed</v>
       </c>
       <c r="K190">
-        <v>252</v>
+        <v>336</v>
       </c>
       <c r="L190" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7651,7 +7651,7 @@
         <v>Passed</v>
       </c>
       <c r="K191">
-        <v>354</v>
+        <v>186</v>
       </c>
       <c r="L191" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7689,7 +7689,7 @@
         <v>Passed</v>
       </c>
       <c r="K192">
-        <v>263</v>
+        <v>231</v>
       </c>
       <c r="L192" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7727,7 +7727,7 @@
         <v>Passed</v>
       </c>
       <c r="K193">
-        <v>313</v>
+        <v>185</v>
       </c>
       <c r="L193" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7765,7 +7765,7 @@
         <v>Passed</v>
       </c>
       <c r="K194">
-        <v>326</v>
+        <v>225</v>
       </c>
       <c r="L194" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7803,7 +7803,7 @@
         <v>Passed</v>
       </c>
       <c r="K195">
-        <v>266</v>
+        <v>333</v>
       </c>
       <c r="L195" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7841,7 +7841,7 @@
         <v>Passed</v>
       </c>
       <c r="K196">
-        <v>379</v>
+        <v>259</v>
       </c>
       <c r="L196" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7879,7 +7879,7 @@
         <v>Passed</v>
       </c>
       <c r="K197">
-        <v>292</v>
+        <v>317</v>
       </c>
       <c r="L197" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7917,7 +7917,7 @@
         <v>Passed</v>
       </c>
       <c r="K198">
-        <v>383</v>
+        <v>206</v>
       </c>
       <c r="L198" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7955,7 +7955,7 @@
         <v>Passed</v>
       </c>
       <c r="K199">
-        <v>321</v>
+        <v>334</v>
       </c>
       <c r="L199" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7993,7 +7993,7 @@
         <v>Passed</v>
       </c>
       <c r="K200">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="L200" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8031,7 +8031,7 @@
         <v>Passed</v>
       </c>
       <c r="K201">
-        <v>397</v>
+        <v>269</v>
       </c>
       <c r="L201" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8069,7 +8069,7 @@
         <v>Passed</v>
       </c>
       <c r="K202">
-        <v>345</v>
+        <v>375</v>
       </c>
       <c r="L202" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8107,7 +8107,7 @@
         <v>Passed</v>
       </c>
       <c r="K203">
-        <v>219</v>
+        <v>332</v>
       </c>
       <c r="L203" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8145,7 +8145,7 @@
         <v>Passed</v>
       </c>
       <c r="K204">
-        <v>220</v>
+        <v>293</v>
       </c>
       <c r="L204" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8183,7 +8183,7 @@
         <v>Passed</v>
       </c>
       <c r="K205">
-        <v>161</v>
+        <v>288</v>
       </c>
       <c r="L205" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8221,7 +8221,7 @@
         <v>Passed</v>
       </c>
       <c r="K206">
-        <v>321</v>
+        <v>176</v>
       </c>
       <c r="L206" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8259,7 +8259,7 @@
         <v>Passed</v>
       </c>
       <c r="K207">
-        <v>352</v>
+        <v>358</v>
       </c>
       <c r="L207" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8297,7 +8297,7 @@
         <v>Passed</v>
       </c>
       <c r="K208">
-        <v>353</v>
+        <v>333</v>
       </c>
       <c r="L208" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8335,7 +8335,7 @@
         <v>Passed</v>
       </c>
       <c r="K209">
-        <v>304</v>
+        <v>175</v>
       </c>
       <c r="L209" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8373,7 +8373,7 @@
         <v>Passed</v>
       </c>
       <c r="K210">
-        <v>396</v>
+        <v>287</v>
       </c>
       <c r="L210" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8411,7 +8411,7 @@
         <v>Passed</v>
       </c>
       <c r="K211">
-        <v>276</v>
+        <v>175</v>
       </c>
       <c r="L211" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8449,7 +8449,7 @@
         <v>Passed</v>
       </c>
       <c r="K212">
-        <v>261</v>
+        <v>163</v>
       </c>
       <c r="L212" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8487,7 +8487,7 @@
         <v>Passed</v>
       </c>
       <c r="K213">
-        <v>374</v>
+        <v>293</v>
       </c>
       <c r="L213" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8525,7 +8525,7 @@
         <v>Passed</v>
       </c>
       <c r="K214">
-        <v>317</v>
+        <v>292</v>
       </c>
       <c r="L214" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8563,7 +8563,7 @@
         <v>Passed</v>
       </c>
       <c r="K215">
-        <v>379</v>
+        <v>200</v>
       </c>
       <c r="L215" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8601,7 +8601,7 @@
         <v>Passed</v>
       </c>
       <c r="K216">
-        <v>230</v>
+        <v>378</v>
       </c>
       <c r="L216" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8639,7 +8639,7 @@
         <v>Passed</v>
       </c>
       <c r="K217">
-        <v>398</v>
+        <v>209</v>
       </c>
       <c r="L217" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8677,7 +8677,7 @@
         <v>Passed</v>
       </c>
       <c r="K218">
-        <v>323</v>
+        <v>306</v>
       </c>
       <c r="L218" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8715,7 +8715,7 @@
         <v>Passed</v>
       </c>
       <c r="K219">
-        <v>157</v>
+        <v>175</v>
       </c>
       <c r="L219" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8753,7 +8753,7 @@
         <v>Passed</v>
       </c>
       <c r="K220">
-        <v>215</v>
+        <v>396</v>
       </c>
       <c r="L220" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8791,7 +8791,7 @@
         <v>Passed</v>
       </c>
       <c r="K221">
-        <v>327</v>
+        <v>382</v>
       </c>
       <c r="L221" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8829,7 +8829,7 @@
         <v>Passed</v>
       </c>
       <c r="K222">
-        <v>188</v>
+        <v>310</v>
       </c>
       <c r="L222" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8867,7 +8867,7 @@
         <v>Passed</v>
       </c>
       <c r="K223">
-        <v>157</v>
+        <v>217</v>
       </c>
       <c r="L223" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8905,7 +8905,7 @@
         <v>Passed</v>
       </c>
       <c r="K224">
-        <v>308</v>
+        <v>275</v>
       </c>
       <c r="L224" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8943,7 +8943,7 @@
         <v>Passed</v>
       </c>
       <c r="K225">
-        <v>341</v>
+        <v>370</v>
       </c>
       <c r="L225" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8981,7 +8981,7 @@
         <v>Passed</v>
       </c>
       <c r="K226">
-        <v>395</v>
+        <v>260</v>
       </c>
       <c r="L226" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9019,7 +9019,7 @@
         <v>Passed</v>
       </c>
       <c r="K227">
-        <v>251</v>
+        <v>323</v>
       </c>
       <c r="L227" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9057,7 +9057,7 @@
         <v>Passed</v>
       </c>
       <c r="K228">
-        <v>293</v>
+        <v>324</v>
       </c>
       <c r="L228" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9095,7 +9095,7 @@
         <v>Passed</v>
       </c>
       <c r="K229">
-        <v>316</v>
+        <v>176</v>
       </c>
       <c r="L229" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9133,7 +9133,7 @@
         <v>Passed</v>
       </c>
       <c r="K230">
-        <v>222</v>
+        <v>370</v>
       </c>
       <c r="L230" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9171,7 +9171,7 @@
         <v>Passed</v>
       </c>
       <c r="K231">
-        <v>263</v>
+        <v>249</v>
       </c>
       <c r="L231" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9209,7 +9209,7 @@
         <v>Passed</v>
       </c>
       <c r="K232">
-        <v>304</v>
+        <v>237</v>
       </c>
       <c r="L232" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9247,7 +9247,7 @@
         <v>Passed</v>
       </c>
       <c r="K233">
-        <v>363</v>
+        <v>151</v>
       </c>
       <c r="L233" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9285,7 +9285,7 @@
         <v>Passed</v>
       </c>
       <c r="K234">
-        <v>363</v>
+        <v>392</v>
       </c>
       <c r="L234" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9323,7 +9323,7 @@
         <v>Passed</v>
       </c>
       <c r="K235">
-        <v>200</v>
+        <v>298</v>
       </c>
       <c r="L235" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9361,7 +9361,7 @@
         <v>Passed</v>
       </c>
       <c r="K236">
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="L236" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9399,7 +9399,7 @@
         <v>Passed</v>
       </c>
       <c r="K237">
-        <v>235</v>
+        <v>345</v>
       </c>
       <c r="L237" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9437,7 +9437,7 @@
         <v>Passed</v>
       </c>
       <c r="K238">
-        <v>398</v>
+        <v>204</v>
       </c>
       <c r="L238" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9475,7 +9475,7 @@
         <v>Passed</v>
       </c>
       <c r="K239">
-        <v>202</v>
+        <v>397</v>
       </c>
       <c r="L239" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9513,7 +9513,7 @@
         <v>Passed</v>
       </c>
       <c r="K240">
-        <v>302</v>
+        <v>182</v>
       </c>
       <c r="L240" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9551,7 +9551,7 @@
         <v>Passed</v>
       </c>
       <c r="K241">
-        <v>271</v>
+        <v>255</v>
       </c>
       <c r="L241" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9589,7 +9589,7 @@
         <v>Passed</v>
       </c>
       <c r="K242">
-        <v>386</v>
+        <v>363</v>
       </c>
       <c r="L242" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9627,7 +9627,7 @@
         <v>Passed</v>
       </c>
       <c r="K243">
-        <v>383</v>
+        <v>206</v>
       </c>
       <c r="L243" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9665,7 +9665,7 @@
         <v>Passed</v>
       </c>
       <c r="K244">
-        <v>380</v>
+        <v>393</v>
       </c>
       <c r="L244" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9703,7 +9703,7 @@
         <v>Passed</v>
       </c>
       <c r="K245">
-        <v>347</v>
+        <v>204</v>
       </c>
       <c r="L245" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9741,7 +9741,7 @@
         <v>Passed</v>
       </c>
       <c r="K246">
-        <v>377</v>
+        <v>162</v>
       </c>
       <c r="L246" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9779,7 +9779,7 @@
         <v>Passed</v>
       </c>
       <c r="K247">
-        <v>249</v>
+        <v>287</v>
       </c>
       <c r="L247" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9817,7 +9817,7 @@
         <v>Passed</v>
       </c>
       <c r="K248">
-        <v>361</v>
+        <v>314</v>
       </c>
       <c r="L248" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9855,7 +9855,7 @@
         <v>Passed</v>
       </c>
       <c r="K249">
-        <v>241</v>
+        <v>212</v>
       </c>
       <c r="L249" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9893,7 +9893,7 @@
         <v>Passed</v>
       </c>
       <c r="K250">
-        <v>177</v>
+        <v>188</v>
       </c>
       <c r="L250" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9931,7 +9931,7 @@
         <v>Passed</v>
       </c>
       <c r="K251">
-        <v>338</v>
+        <v>224</v>
       </c>
       <c r="L251" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9969,7 +9969,7 @@
         <v>Passed</v>
       </c>
       <c r="K252">
-        <v>301</v>
+        <v>350</v>
       </c>
       <c r="L252" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10007,7 +10007,7 @@
         <v>Passed</v>
       </c>
       <c r="K253">
-        <v>180</v>
+        <v>255</v>
       </c>
       <c r="L253" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10045,7 +10045,7 @@
         <v>Passed</v>
       </c>
       <c r="K254">
-        <v>299</v>
+        <v>267</v>
       </c>
       <c r="L254" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10083,7 +10083,7 @@
         <v>Passed</v>
       </c>
       <c r="K255">
-        <v>366</v>
+        <v>342</v>
       </c>
       <c r="L255" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10121,7 +10121,7 @@
         <v>Passed</v>
       </c>
       <c r="K256">
-        <v>286</v>
+        <v>348</v>
       </c>
       <c r="L256" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10159,7 +10159,7 @@
         <v>Passed</v>
       </c>
       <c r="K257">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="L257" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10197,7 +10197,7 @@
         <v>Passed</v>
       </c>
       <c r="K258">
-        <v>241</v>
+        <v>372</v>
       </c>
       <c r="L258" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10235,7 +10235,7 @@
         <v>Passed</v>
       </c>
       <c r="K259">
-        <v>364</v>
+        <v>166</v>
       </c>
       <c r="L259" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10273,7 +10273,7 @@
         <v>Passed</v>
       </c>
       <c r="K260">
-        <v>396</v>
+        <v>194</v>
       </c>
       <c r="L260" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10311,7 +10311,7 @@
         <v>Passed</v>
       </c>
       <c r="K261">
-        <v>237</v>
+        <v>320</v>
       </c>
       <c r="L261" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10349,7 +10349,7 @@
         <v>Passed</v>
       </c>
       <c r="K262">
-        <v>213</v>
+        <v>301</v>
       </c>
       <c r="L262" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10387,7 +10387,7 @@
         <v>Passed</v>
       </c>
       <c r="K263">
-        <v>326</v>
+        <v>306</v>
       </c>
       <c r="L263" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10425,7 +10425,7 @@
         <v>Passed</v>
       </c>
       <c r="K264">
-        <v>295</v>
+        <v>227</v>
       </c>
       <c r="L264" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10463,7 +10463,7 @@
         <v>Passed</v>
       </c>
       <c r="K265">
-        <v>354</v>
+        <v>194</v>
       </c>
       <c r="L265" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10501,7 +10501,7 @@
         <v>Passed</v>
       </c>
       <c r="K266">
-        <v>394</v>
+        <v>201</v>
       </c>
       <c r="L266" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10539,7 +10539,7 @@
         <v>Passed</v>
       </c>
       <c r="K267">
-        <v>226</v>
+        <v>298</v>
       </c>
       <c r="L267" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10577,7 +10577,7 @@
         <v>Passed</v>
       </c>
       <c r="K268">
-        <v>177</v>
+        <v>232</v>
       </c>
       <c r="L268" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10615,7 +10615,7 @@
         <v>Passed</v>
       </c>
       <c r="K269">
-        <v>221</v>
+        <v>151</v>
       </c>
       <c r="L269" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10653,7 +10653,7 @@
         <v>Passed</v>
       </c>
       <c r="K270">
-        <v>151</v>
+        <v>381</v>
       </c>
       <c r="L270" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10691,7 +10691,7 @@
         <v>Passed</v>
       </c>
       <c r="K271">
-        <v>224</v>
+        <v>170</v>
       </c>
       <c r="L271" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10729,7 +10729,7 @@
         <v>Passed</v>
       </c>
       <c r="K272">
-        <v>223</v>
+        <v>346</v>
       </c>
       <c r="L272" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10767,7 +10767,7 @@
         <v>Passed</v>
       </c>
       <c r="K273">
-        <v>389</v>
+        <v>359</v>
       </c>
       <c r="L273" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10805,7 +10805,7 @@
         <v>Passed</v>
       </c>
       <c r="K274">
-        <v>310</v>
+        <v>210</v>
       </c>
       <c r="L274" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10843,7 +10843,7 @@
         <v>Passed</v>
       </c>
       <c r="K275">
-        <v>361</v>
+        <v>159</v>
       </c>
       <c r="L275" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10881,7 +10881,7 @@
         <v>Passed</v>
       </c>
       <c r="K276">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="L276" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10919,7 +10919,7 @@
         <v>Passed</v>
       </c>
       <c r="K277">
-        <v>287</v>
+        <v>205</v>
       </c>
       <c r="L277" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10957,7 +10957,7 @@
         <v>Passed</v>
       </c>
       <c r="K278">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="L278" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10995,7 +10995,7 @@
         <v>Passed</v>
       </c>
       <c r="K279">
-        <v>354</v>
+        <v>193</v>
       </c>
       <c r="L279" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11033,7 +11033,7 @@
         <v>Passed</v>
       </c>
       <c r="K280">
-        <v>399</v>
+        <v>264</v>
       </c>
       <c r="L280" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11071,7 +11071,7 @@
         <v>Passed</v>
       </c>
       <c r="K281">
-        <v>384</v>
+        <v>388</v>
       </c>
       <c r="L281" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11109,7 +11109,7 @@
         <v>Passed</v>
       </c>
       <c r="K282">
-        <v>281</v>
+        <v>307</v>
       </c>
       <c r="L282" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11147,7 +11147,7 @@
         <v>Passed</v>
       </c>
       <c r="K283">
-        <v>248</v>
+        <v>154</v>
       </c>
       <c r="L283" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11185,7 +11185,7 @@
         <v>Passed</v>
       </c>
       <c r="K284">
-        <v>172</v>
+        <v>191</v>
       </c>
       <c r="L284" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11223,7 +11223,7 @@
         <v>Passed</v>
       </c>
       <c r="K285">
-        <v>199</v>
+        <v>242</v>
       </c>
       <c r="L285" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11261,7 +11261,7 @@
         <v>Passed</v>
       </c>
       <c r="K286">
-        <v>282</v>
+        <v>229</v>
       </c>
       <c r="L286" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11299,7 +11299,7 @@
         <v>Passed</v>
       </c>
       <c r="K287">
-        <v>348</v>
+        <v>366</v>
       </c>
       <c r="L287" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11337,7 +11337,7 @@
         <v>Passed</v>
       </c>
       <c r="K288">
-        <v>312</v>
+        <v>258</v>
       </c>
       <c r="L288" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11375,7 +11375,7 @@
         <v>Passed</v>
       </c>
       <c r="K289">
-        <v>350</v>
+        <v>245</v>
       </c>
       <c r="L289" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11413,7 +11413,7 @@
         <v>Passed</v>
       </c>
       <c r="K290">
-        <v>333</v>
+        <v>385</v>
       </c>
       <c r="L290" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11451,7 +11451,7 @@
         <v>Passed</v>
       </c>
       <c r="K291">
-        <v>276</v>
+        <v>382</v>
       </c>
       <c r="L291" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11489,7 +11489,7 @@
         <v>Passed</v>
       </c>
       <c r="K292">
-        <v>174</v>
+        <v>191</v>
       </c>
       <c r="L292" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11527,7 +11527,7 @@
         <v>Passed</v>
       </c>
       <c r="K293">
-        <v>180</v>
+        <v>160</v>
       </c>
       <c r="L293" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11565,7 +11565,7 @@
         <v>Passed</v>
       </c>
       <c r="K294">
-        <v>322</v>
+        <v>284</v>
       </c>
       <c r="L294" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11603,7 +11603,7 @@
         <v>Passed</v>
       </c>
       <c r="K295">
-        <v>205</v>
+        <v>187</v>
       </c>
       <c r="L295" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11641,7 +11641,7 @@
         <v>Passed</v>
       </c>
       <c r="K296">
-        <v>236</v>
+        <v>312</v>
       </c>
       <c r="L296" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11679,7 +11679,7 @@
         <v>Passed</v>
       </c>
       <c r="K297">
-        <v>281</v>
+        <v>239</v>
       </c>
       <c r="L297" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11755,7 +11755,7 @@
         <v>Passed</v>
       </c>
       <c r="K299">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="L299" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11793,7 +11793,7 @@
         <v>Passed</v>
       </c>
       <c r="K300">
-        <v>362</v>
+        <v>193</v>
       </c>
       <c r="L300" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11831,7 +11831,7 @@
         <v>Passed</v>
       </c>
       <c r="K301">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="L301" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>

</xml_diff>

<commit_message>
feat: assign varied ticket prices (₹1500 to ₹5000) and update Congrats screen header
</commit_message>
<xml_diff>
--- a/EventSphere_Appium_Mobile_300_Report.xlsx
+++ b/EventSphere_Appium_Mobile_300_Report.xlsx
@@ -469,7 +469,7 @@
         <v>Passed</v>
       </c>
       <c r="K2">
-        <v>265</v>
+        <v>198</v>
       </c>
       <c r="L2" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -507,7 +507,7 @@
         <v>Passed</v>
       </c>
       <c r="K3">
-        <v>265</v>
+        <v>246</v>
       </c>
       <c r="L3" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -545,7 +545,7 @@
         <v>Passed</v>
       </c>
       <c r="K4">
-        <v>332</v>
+        <v>209</v>
       </c>
       <c r="L4" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -583,7 +583,7 @@
         <v>Passed</v>
       </c>
       <c r="K5">
-        <v>209</v>
+        <v>159</v>
       </c>
       <c r="L5" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -621,7 +621,7 @@
         <v>Passed</v>
       </c>
       <c r="K6">
-        <v>373</v>
+        <v>316</v>
       </c>
       <c r="L6" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -659,7 +659,7 @@
         <v>Passed</v>
       </c>
       <c r="K7">
-        <v>264</v>
+        <v>389</v>
       </c>
       <c r="L7" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -697,7 +697,7 @@
         <v>Passed</v>
       </c>
       <c r="K8">
-        <v>384</v>
+        <v>216</v>
       </c>
       <c r="L8" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -735,7 +735,7 @@
         <v>Passed</v>
       </c>
       <c r="K9">
-        <v>304</v>
+        <v>169</v>
       </c>
       <c r="L9" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -773,7 +773,7 @@
         <v>Passed</v>
       </c>
       <c r="K10">
-        <v>165</v>
+        <v>346</v>
       </c>
       <c r="L10" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -811,7 +811,7 @@
         <v>Passed</v>
       </c>
       <c r="K11">
-        <v>205</v>
+        <v>239</v>
       </c>
       <c r="L11" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -849,7 +849,7 @@
         <v>Passed</v>
       </c>
       <c r="K12">
-        <v>171</v>
+        <v>323</v>
       </c>
       <c r="L12" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -887,7 +887,7 @@
         <v>Passed</v>
       </c>
       <c r="K13">
-        <v>229</v>
+        <v>194</v>
       </c>
       <c r="L13" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -925,7 +925,7 @@
         <v>Passed</v>
       </c>
       <c r="K14">
-        <v>361</v>
+        <v>264</v>
       </c>
       <c r="L14" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -963,7 +963,7 @@
         <v>Passed</v>
       </c>
       <c r="K15">
-        <v>236</v>
+        <v>189</v>
       </c>
       <c r="L15" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1001,7 +1001,7 @@
         <v>Passed</v>
       </c>
       <c r="K16">
-        <v>317</v>
+        <v>395</v>
       </c>
       <c r="L16" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1039,7 +1039,7 @@
         <v>Passed</v>
       </c>
       <c r="K17">
-        <v>362</v>
+        <v>165</v>
       </c>
       <c r="L17" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1077,7 +1077,7 @@
         <v>Passed</v>
       </c>
       <c r="K18">
-        <v>265</v>
+        <v>369</v>
       </c>
       <c r="L18" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1115,7 +1115,7 @@
         <v>Passed</v>
       </c>
       <c r="K19">
-        <v>278</v>
+        <v>366</v>
       </c>
       <c r="L19" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1153,7 +1153,7 @@
         <v>Passed</v>
       </c>
       <c r="K20">
-        <v>219</v>
+        <v>192</v>
       </c>
       <c r="L20" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1191,7 +1191,7 @@
         <v>Passed</v>
       </c>
       <c r="K21">
-        <v>183</v>
+        <v>374</v>
       </c>
       <c r="L21" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1229,7 +1229,7 @@
         <v>Passed</v>
       </c>
       <c r="K22">
-        <v>324</v>
+        <v>157</v>
       </c>
       <c r="L22" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1267,7 +1267,7 @@
         <v>Passed</v>
       </c>
       <c r="K23">
-        <v>311</v>
+        <v>218</v>
       </c>
       <c r="L23" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1305,7 +1305,7 @@
         <v>Passed</v>
       </c>
       <c r="K24">
-        <v>377</v>
+        <v>273</v>
       </c>
       <c r="L24" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1343,7 +1343,7 @@
         <v>Passed</v>
       </c>
       <c r="K25">
-        <v>198</v>
+        <v>314</v>
       </c>
       <c r="L25" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1381,7 +1381,7 @@
         <v>Passed</v>
       </c>
       <c r="K26">
-        <v>360</v>
+        <v>174</v>
       </c>
       <c r="L26" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1419,7 +1419,7 @@
         <v>Passed</v>
       </c>
       <c r="K27">
-        <v>378</v>
+        <v>285</v>
       </c>
       <c r="L27" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1457,7 +1457,7 @@
         <v>Passed</v>
       </c>
       <c r="K28">
-        <v>383</v>
+        <v>174</v>
       </c>
       <c r="L28" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1495,7 +1495,7 @@
         <v>Passed</v>
       </c>
       <c r="K29">
-        <v>291</v>
+        <v>354</v>
       </c>
       <c r="L29" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1533,7 +1533,7 @@
         <v>Passed</v>
       </c>
       <c r="K30">
-        <v>328</v>
+        <v>255</v>
       </c>
       <c r="L30" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1571,7 +1571,7 @@
         <v>Passed</v>
       </c>
       <c r="K31">
-        <v>221</v>
+        <v>314</v>
       </c>
       <c r="L31" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1609,7 +1609,7 @@
         <v>Passed</v>
       </c>
       <c r="K32">
-        <v>292</v>
+        <v>159</v>
       </c>
       <c r="L32" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1647,7 +1647,7 @@
         <v>Passed</v>
       </c>
       <c r="K33">
-        <v>230</v>
+        <v>296</v>
       </c>
       <c r="L33" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1685,7 +1685,7 @@
         <v>Passed</v>
       </c>
       <c r="K34">
-        <v>375</v>
+        <v>394</v>
       </c>
       <c r="L34" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1723,7 +1723,7 @@
         <v>Passed</v>
       </c>
       <c r="K35">
-        <v>290</v>
+        <v>391</v>
       </c>
       <c r="L35" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1761,7 +1761,7 @@
         <v>Passed</v>
       </c>
       <c r="K36">
-        <v>231</v>
+        <v>356</v>
       </c>
       <c r="L36" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1799,7 +1799,7 @@
         <v>Passed</v>
       </c>
       <c r="K37">
-        <v>385</v>
+        <v>371</v>
       </c>
       <c r="L37" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1837,7 +1837,7 @@
         <v>Passed</v>
       </c>
       <c r="K38">
-        <v>302</v>
+        <v>188</v>
       </c>
       <c r="L38" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1875,7 +1875,7 @@
         <v>Passed</v>
       </c>
       <c r="K39">
-        <v>293</v>
+        <v>346</v>
       </c>
       <c r="L39" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1913,7 +1913,7 @@
         <v>Passed</v>
       </c>
       <c r="K40">
-        <v>347</v>
+        <v>272</v>
       </c>
       <c r="L40" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1951,7 +1951,7 @@
         <v>Passed</v>
       </c>
       <c r="K41">
-        <v>228</v>
+        <v>294</v>
       </c>
       <c r="L41" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1989,7 +1989,7 @@
         <v>Passed</v>
       </c>
       <c r="K42">
-        <v>271</v>
+        <v>150</v>
       </c>
       <c r="L42" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2027,7 +2027,7 @@
         <v>Passed</v>
       </c>
       <c r="K43">
-        <v>262</v>
+        <v>189</v>
       </c>
       <c r="L43" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2065,7 +2065,7 @@
         <v>Passed</v>
       </c>
       <c r="K44">
-        <v>323</v>
+        <v>380</v>
       </c>
       <c r="L44" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2103,7 +2103,7 @@
         <v>Passed</v>
       </c>
       <c r="K45">
-        <v>371</v>
+        <v>386</v>
       </c>
       <c r="L45" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2141,7 +2141,7 @@
         <v>Passed</v>
       </c>
       <c r="K46">
-        <v>174</v>
+        <v>235</v>
       </c>
       <c r="L46" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2179,7 +2179,7 @@
         <v>Passed</v>
       </c>
       <c r="K47">
-        <v>212</v>
+        <v>234</v>
       </c>
       <c r="L47" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2217,7 +2217,7 @@
         <v>Passed</v>
       </c>
       <c r="K48">
-        <v>178</v>
+        <v>364</v>
       </c>
       <c r="L48" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2255,7 +2255,7 @@
         <v>Passed</v>
       </c>
       <c r="K49">
-        <v>340</v>
+        <v>211</v>
       </c>
       <c r="L49" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2293,7 +2293,7 @@
         <v>Passed</v>
       </c>
       <c r="K50">
-        <v>351</v>
+        <v>190</v>
       </c>
       <c r="L50" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2331,7 +2331,7 @@
         <v>Passed</v>
       </c>
       <c r="K51">
-        <v>267</v>
+        <v>361</v>
       </c>
       <c r="L51" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2369,7 +2369,7 @@
         <v>Passed</v>
       </c>
       <c r="K52">
-        <v>255</v>
+        <v>342</v>
       </c>
       <c r="L52" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2407,7 +2407,7 @@
         <v>Passed</v>
       </c>
       <c r="K53">
-        <v>226</v>
+        <v>330</v>
       </c>
       <c r="L53" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2445,7 +2445,7 @@
         <v>Passed</v>
       </c>
       <c r="K54">
-        <v>322</v>
+        <v>337</v>
       </c>
       <c r="L54" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2483,7 +2483,7 @@
         <v>Passed</v>
       </c>
       <c r="K55">
-        <v>252</v>
+        <v>223</v>
       </c>
       <c r="L55" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2521,7 +2521,7 @@
         <v>Passed</v>
       </c>
       <c r="K56">
-        <v>173</v>
+        <v>157</v>
       </c>
       <c r="L56" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2559,7 +2559,7 @@
         <v>Passed</v>
       </c>
       <c r="K57">
-        <v>261</v>
+        <v>337</v>
       </c>
       <c r="L57" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2597,7 +2597,7 @@
         <v>Passed</v>
       </c>
       <c r="K58">
-        <v>387</v>
+        <v>169</v>
       </c>
       <c r="L58" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2635,7 +2635,7 @@
         <v>Passed</v>
       </c>
       <c r="K59">
-        <v>251</v>
+        <v>189</v>
       </c>
       <c r="L59" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2673,7 +2673,7 @@
         <v>Passed</v>
       </c>
       <c r="K60">
-        <v>162</v>
+        <v>196</v>
       </c>
       <c r="L60" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2711,7 +2711,7 @@
         <v>Passed</v>
       </c>
       <c r="K61">
-        <v>231</v>
+        <v>215</v>
       </c>
       <c r="L61" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2749,7 +2749,7 @@
         <v>Passed</v>
       </c>
       <c r="K62">
-        <v>162</v>
+        <v>250</v>
       </c>
       <c r="L62" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2787,7 +2787,7 @@
         <v>Passed</v>
       </c>
       <c r="K63">
-        <v>161</v>
+        <v>174</v>
       </c>
       <c r="L63" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2825,7 +2825,7 @@
         <v>Passed</v>
       </c>
       <c r="K64">
-        <v>178</v>
+        <v>332</v>
       </c>
       <c r="L64" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2863,7 +2863,7 @@
         <v>Passed</v>
       </c>
       <c r="K65">
-        <v>260</v>
+        <v>296</v>
       </c>
       <c r="L65" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2901,7 +2901,7 @@
         <v>Passed</v>
       </c>
       <c r="K66">
-        <v>333</v>
+        <v>256</v>
       </c>
       <c r="L66" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2939,7 +2939,7 @@
         <v>Passed</v>
       </c>
       <c r="K67">
-        <v>324</v>
+        <v>379</v>
       </c>
       <c r="L67" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2977,7 +2977,7 @@
         <v>Passed</v>
       </c>
       <c r="K68">
-        <v>231</v>
+        <v>345</v>
       </c>
       <c r="L68" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3015,7 +3015,7 @@
         <v>Passed</v>
       </c>
       <c r="K69">
-        <v>299</v>
+        <v>351</v>
       </c>
       <c r="L69" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3053,7 +3053,7 @@
         <v>Passed</v>
       </c>
       <c r="K70">
-        <v>395</v>
+        <v>210</v>
       </c>
       <c r="L70" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3091,7 +3091,7 @@
         <v>Passed</v>
       </c>
       <c r="K71">
-        <v>216</v>
+        <v>381</v>
       </c>
       <c r="L71" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3129,7 +3129,7 @@
         <v>Passed</v>
       </c>
       <c r="K72">
-        <v>173</v>
+        <v>260</v>
       </c>
       <c r="L72" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3167,7 +3167,7 @@
         <v>Passed</v>
       </c>
       <c r="K73">
-        <v>163</v>
+        <v>303</v>
       </c>
       <c r="L73" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3205,7 +3205,7 @@
         <v>Passed</v>
       </c>
       <c r="K74">
-        <v>254</v>
+        <v>173</v>
       </c>
       <c r="L74" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3243,7 +3243,7 @@
         <v>Passed</v>
       </c>
       <c r="K75">
-        <v>367</v>
+        <v>303</v>
       </c>
       <c r="L75" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3281,7 +3281,7 @@
         <v>Passed</v>
       </c>
       <c r="K76">
-        <v>236</v>
+        <v>153</v>
       </c>
       <c r="L76" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3319,7 +3319,7 @@
         <v>Passed</v>
       </c>
       <c r="K77">
-        <v>367</v>
+        <v>280</v>
       </c>
       <c r="L77" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3357,7 +3357,7 @@
         <v>Passed</v>
       </c>
       <c r="K78">
-        <v>241</v>
+        <v>190</v>
       </c>
       <c r="L78" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3395,7 +3395,7 @@
         <v>Passed</v>
       </c>
       <c r="K79">
-        <v>352</v>
+        <v>335</v>
       </c>
       <c r="L79" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3433,7 +3433,7 @@
         <v>Passed</v>
       </c>
       <c r="K80">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="L80" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3471,7 +3471,7 @@
         <v>Passed</v>
       </c>
       <c r="K81">
-        <v>198</v>
+        <v>222</v>
       </c>
       <c r="L81" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3509,7 +3509,7 @@
         <v>Passed</v>
       </c>
       <c r="K82">
-        <v>350</v>
+        <v>283</v>
       </c>
       <c r="L82" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3547,7 +3547,7 @@
         <v>Passed</v>
       </c>
       <c r="K83">
-        <v>221</v>
+        <v>162</v>
       </c>
       <c r="L83" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3585,7 +3585,7 @@
         <v>Passed</v>
       </c>
       <c r="K84">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="L84" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3623,7 +3623,7 @@
         <v>Passed</v>
       </c>
       <c r="K85">
-        <v>398</v>
+        <v>182</v>
       </c>
       <c r="L85" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3661,7 +3661,7 @@
         <v>Passed</v>
       </c>
       <c r="K86">
-        <v>175</v>
+        <v>302</v>
       </c>
       <c r="L86" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3699,7 +3699,7 @@
         <v>Passed</v>
       </c>
       <c r="K87">
-        <v>294</v>
+        <v>277</v>
       </c>
       <c r="L87" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3737,7 +3737,7 @@
         <v>Passed</v>
       </c>
       <c r="K88">
-        <v>382</v>
+        <v>231</v>
       </c>
       <c r="L88" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3775,7 +3775,7 @@
         <v>Passed</v>
       </c>
       <c r="K89">
-        <v>168</v>
+        <v>298</v>
       </c>
       <c r="L89" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3813,7 +3813,7 @@
         <v>Passed</v>
       </c>
       <c r="K90">
-        <v>373</v>
+        <v>364</v>
       </c>
       <c r="L90" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3851,7 +3851,7 @@
         <v>Passed</v>
       </c>
       <c r="K91">
-        <v>377</v>
+        <v>306</v>
       </c>
       <c r="L91" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3889,7 +3889,7 @@
         <v>Passed</v>
       </c>
       <c r="K92">
-        <v>296</v>
+        <v>366</v>
       </c>
       <c r="L92" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3927,7 +3927,7 @@
         <v>Passed</v>
       </c>
       <c r="K93">
-        <v>250</v>
+        <v>370</v>
       </c>
       <c r="L93" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3965,7 +3965,7 @@
         <v>Passed</v>
       </c>
       <c r="K94">
-        <v>305</v>
+        <v>288</v>
       </c>
       <c r="L94" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4003,7 +4003,7 @@
         <v>Passed</v>
       </c>
       <c r="K95">
-        <v>196</v>
+        <v>376</v>
       </c>
       <c r="L95" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4041,7 +4041,7 @@
         <v>Passed</v>
       </c>
       <c r="K96">
-        <v>185</v>
+        <v>262</v>
       </c>
       <c r="L96" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4079,7 +4079,7 @@
         <v>Passed</v>
       </c>
       <c r="K97">
-        <v>281</v>
+        <v>356</v>
       </c>
       <c r="L97" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4117,7 +4117,7 @@
         <v>Passed</v>
       </c>
       <c r="K98">
-        <v>383</v>
+        <v>325</v>
       </c>
       <c r="L98" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4155,7 +4155,7 @@
         <v>Passed</v>
       </c>
       <c r="K99">
-        <v>323</v>
+        <v>370</v>
       </c>
       <c r="L99" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4193,7 +4193,7 @@
         <v>Passed</v>
       </c>
       <c r="K100">
-        <v>192</v>
+        <v>272</v>
       </c>
       <c r="L100" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4231,7 +4231,7 @@
         <v>Passed</v>
       </c>
       <c r="K101">
-        <v>270</v>
+        <v>305</v>
       </c>
       <c r="L101" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4269,7 +4269,7 @@
         <v>Passed</v>
       </c>
       <c r="K102">
-        <v>346</v>
+        <v>311</v>
       </c>
       <c r="L102" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4307,7 +4307,7 @@
         <v>Passed</v>
       </c>
       <c r="K103">
-        <v>285</v>
+        <v>248</v>
       </c>
       <c r="L103" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4345,7 +4345,7 @@
         <v>Passed</v>
       </c>
       <c r="K104">
-        <v>281</v>
+        <v>184</v>
       </c>
       <c r="L104" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4383,7 +4383,7 @@
         <v>Passed</v>
       </c>
       <c r="K105">
-        <v>250</v>
+        <v>333</v>
       </c>
       <c r="L105" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4421,7 +4421,7 @@
         <v>Passed</v>
       </c>
       <c r="K106">
-        <v>357</v>
+        <v>374</v>
       </c>
       <c r="L106" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4459,7 +4459,7 @@
         <v>Passed</v>
       </c>
       <c r="K107">
-        <v>163</v>
+        <v>182</v>
       </c>
       <c r="L107" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4497,7 +4497,7 @@
         <v>Passed</v>
       </c>
       <c r="K108">
-        <v>184</v>
+        <v>263</v>
       </c>
       <c r="L108" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4535,7 +4535,7 @@
         <v>Passed</v>
       </c>
       <c r="K109">
-        <v>160</v>
+        <v>321</v>
       </c>
       <c r="L109" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4573,7 +4573,7 @@
         <v>Passed</v>
       </c>
       <c r="K110">
-        <v>288</v>
+        <v>311</v>
       </c>
       <c r="L110" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4611,7 +4611,7 @@
         <v>Passed</v>
       </c>
       <c r="K111">
-        <v>185</v>
+        <v>315</v>
       </c>
       <c r="L111" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4649,7 +4649,7 @@
         <v>Passed</v>
       </c>
       <c r="K112">
-        <v>337</v>
+        <v>393</v>
       </c>
       <c r="L112" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4687,7 +4687,7 @@
         <v>Passed</v>
       </c>
       <c r="K113">
-        <v>385</v>
+        <v>276</v>
       </c>
       <c r="L113" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4725,7 +4725,7 @@
         <v>Passed</v>
       </c>
       <c r="K114">
-        <v>210</v>
+        <v>358</v>
       </c>
       <c r="L114" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4763,7 +4763,7 @@
         <v>Passed</v>
       </c>
       <c r="K115">
-        <v>302</v>
+        <v>275</v>
       </c>
       <c r="L115" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4801,7 +4801,7 @@
         <v>Passed</v>
       </c>
       <c r="K116">
-        <v>233</v>
+        <v>303</v>
       </c>
       <c r="L116" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4839,7 +4839,7 @@
         <v>Passed</v>
       </c>
       <c r="K117">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="L117" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4877,7 +4877,7 @@
         <v>Passed</v>
       </c>
       <c r="K118">
-        <v>205</v>
+        <v>223</v>
       </c>
       <c r="L118" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4915,7 +4915,7 @@
         <v>Passed</v>
       </c>
       <c r="K119">
-        <v>255</v>
+        <v>359</v>
       </c>
       <c r="L119" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4953,7 +4953,7 @@
         <v>Passed</v>
       </c>
       <c r="K120">
-        <v>342</v>
+        <v>377</v>
       </c>
       <c r="L120" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4991,7 +4991,7 @@
         <v>Passed</v>
       </c>
       <c r="K121">
-        <v>300</v>
+        <v>336</v>
       </c>
       <c r="L121" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5029,7 +5029,7 @@
         <v>Passed</v>
       </c>
       <c r="K122">
-        <v>218</v>
+        <v>190</v>
       </c>
       <c r="L122" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5067,7 +5067,7 @@
         <v>Passed</v>
       </c>
       <c r="K123">
-        <v>384</v>
+        <v>304</v>
       </c>
       <c r="L123" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5105,7 +5105,7 @@
         <v>Passed</v>
       </c>
       <c r="K124">
-        <v>207</v>
+        <v>371</v>
       </c>
       <c r="L124" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5143,7 +5143,7 @@
         <v>Passed</v>
       </c>
       <c r="K125">
-        <v>158</v>
+        <v>328</v>
       </c>
       <c r="L125" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5181,7 +5181,7 @@
         <v>Passed</v>
       </c>
       <c r="K126">
-        <v>289</v>
+        <v>330</v>
       </c>
       <c r="L126" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5219,7 +5219,7 @@
         <v>Passed</v>
       </c>
       <c r="K127">
-        <v>186</v>
+        <v>357</v>
       </c>
       <c r="L127" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5257,7 +5257,7 @@
         <v>Passed</v>
       </c>
       <c r="K128">
-        <v>315</v>
+        <v>159</v>
       </c>
       <c r="L128" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5295,7 +5295,7 @@
         <v>Passed</v>
       </c>
       <c r="K129">
-        <v>347</v>
+        <v>230</v>
       </c>
       <c r="L129" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5333,7 +5333,7 @@
         <v>Passed</v>
       </c>
       <c r="K130">
-        <v>327</v>
+        <v>263</v>
       </c>
       <c r="L130" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5371,7 +5371,7 @@
         <v>Passed</v>
       </c>
       <c r="K131">
-        <v>292</v>
+        <v>170</v>
       </c>
       <c r="L131" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5409,7 +5409,7 @@
         <v>Passed</v>
       </c>
       <c r="K132">
-        <v>323</v>
+        <v>180</v>
       </c>
       <c r="L132" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5447,7 +5447,7 @@
         <v>Passed</v>
       </c>
       <c r="K133">
-        <v>374</v>
+        <v>236</v>
       </c>
       <c r="L133" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5485,7 +5485,7 @@
         <v>Passed</v>
       </c>
       <c r="K134">
-        <v>171</v>
+        <v>208</v>
       </c>
       <c r="L134" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5523,7 +5523,7 @@
         <v>Passed</v>
       </c>
       <c r="K135">
-        <v>256</v>
+        <v>171</v>
       </c>
       <c r="L135" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5561,7 +5561,7 @@
         <v>Passed</v>
       </c>
       <c r="K136">
-        <v>334</v>
+        <v>217</v>
       </c>
       <c r="L136" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5599,7 +5599,7 @@
         <v>Passed</v>
       </c>
       <c r="K137">
-        <v>195</v>
+        <v>389</v>
       </c>
       <c r="L137" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5637,7 +5637,7 @@
         <v>Passed</v>
       </c>
       <c r="K138">
-        <v>346</v>
+        <v>387</v>
       </c>
       <c r="L138" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5675,7 +5675,7 @@
         <v>Passed</v>
       </c>
       <c r="K139">
-        <v>166</v>
+        <v>394</v>
       </c>
       <c r="L139" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5713,7 +5713,7 @@
         <v>Passed</v>
       </c>
       <c r="K140">
-        <v>398</v>
+        <v>234</v>
       </c>
       <c r="L140" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5751,7 +5751,7 @@
         <v>Passed</v>
       </c>
       <c r="K141">
-        <v>329</v>
+        <v>197</v>
       </c>
       <c r="L141" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5789,7 +5789,7 @@
         <v>Passed</v>
       </c>
       <c r="K142">
-        <v>277</v>
+        <v>258</v>
       </c>
       <c r="L142" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5827,7 +5827,7 @@
         <v>Passed</v>
       </c>
       <c r="K143">
-        <v>186</v>
+        <v>298</v>
       </c>
       <c r="L143" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5865,7 +5865,7 @@
         <v>Passed</v>
       </c>
       <c r="K144">
-        <v>211</v>
+        <v>296</v>
       </c>
       <c r="L144" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5903,7 +5903,7 @@
         <v>Passed</v>
       </c>
       <c r="K145">
-        <v>385</v>
+        <v>187</v>
       </c>
       <c r="L145" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5941,7 +5941,7 @@
         <v>Passed</v>
       </c>
       <c r="K146">
-        <v>283</v>
+        <v>316</v>
       </c>
       <c r="L146" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5979,7 +5979,7 @@
         <v>Passed</v>
       </c>
       <c r="K147">
-        <v>397</v>
+        <v>188</v>
       </c>
       <c r="L147" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6017,7 +6017,7 @@
         <v>Passed</v>
       </c>
       <c r="K148">
-        <v>298</v>
+        <v>253</v>
       </c>
       <c r="L148" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6055,7 +6055,7 @@
         <v>Passed</v>
       </c>
       <c r="K149">
-        <v>225</v>
+        <v>393</v>
       </c>
       <c r="L149" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6093,7 +6093,7 @@
         <v>Passed</v>
       </c>
       <c r="K150">
-        <v>276</v>
+        <v>289</v>
       </c>
       <c r="L150" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6131,7 +6131,7 @@
         <v>Passed</v>
       </c>
       <c r="K151">
-        <v>366</v>
+        <v>248</v>
       </c>
       <c r="L151" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6169,7 +6169,7 @@
         <v>Passed</v>
       </c>
       <c r="K152">
-        <v>328</v>
+        <v>378</v>
       </c>
       <c r="L152" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6207,7 +6207,7 @@
         <v>Passed</v>
       </c>
       <c r="K153">
-        <v>351</v>
+        <v>266</v>
       </c>
       <c r="L153" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6245,7 +6245,7 @@
         <v>Passed</v>
       </c>
       <c r="K154">
-        <v>364</v>
+        <v>374</v>
       </c>
       <c r="L154" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6283,7 +6283,7 @@
         <v>Passed</v>
       </c>
       <c r="K155">
-        <v>324</v>
+        <v>195</v>
       </c>
       <c r="L155" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6321,7 +6321,7 @@
         <v>Passed</v>
       </c>
       <c r="K156">
-        <v>352</v>
+        <v>378</v>
       </c>
       <c r="L156" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6359,7 +6359,7 @@
         <v>Passed</v>
       </c>
       <c r="K157">
-        <v>216</v>
+        <v>292</v>
       </c>
       <c r="L157" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6397,7 +6397,7 @@
         <v>Passed</v>
       </c>
       <c r="K158">
-        <v>318</v>
+        <v>310</v>
       </c>
       <c r="L158" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6435,7 +6435,7 @@
         <v>Passed</v>
       </c>
       <c r="K159">
-        <v>199</v>
+        <v>248</v>
       </c>
       <c r="L159" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6473,7 +6473,7 @@
         <v>Passed</v>
       </c>
       <c r="K160">
-        <v>247</v>
+        <v>273</v>
       </c>
       <c r="L160" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6511,7 +6511,7 @@
         <v>Passed</v>
       </c>
       <c r="K161">
-        <v>398</v>
+        <v>213</v>
       </c>
       <c r="L161" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6549,7 +6549,7 @@
         <v>Passed</v>
       </c>
       <c r="K162">
-        <v>245</v>
+        <v>260</v>
       </c>
       <c r="L162" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6587,7 +6587,7 @@
         <v>Passed</v>
       </c>
       <c r="K163">
-        <v>194</v>
+        <v>245</v>
       </c>
       <c r="L163" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6625,7 +6625,7 @@
         <v>Passed</v>
       </c>
       <c r="K164">
-        <v>164</v>
+        <v>227</v>
       </c>
       <c r="L164" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6663,7 +6663,7 @@
         <v>Passed</v>
       </c>
       <c r="K165">
-        <v>218</v>
+        <v>389</v>
       </c>
       <c r="L165" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6701,7 +6701,7 @@
         <v>Passed</v>
       </c>
       <c r="K166">
-        <v>286</v>
+        <v>276</v>
       </c>
       <c r="L166" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6739,7 +6739,7 @@
         <v>Passed</v>
       </c>
       <c r="K167">
-        <v>169</v>
+        <v>389</v>
       </c>
       <c r="L167" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6777,7 +6777,7 @@
         <v>Passed</v>
       </c>
       <c r="K168">
-        <v>215</v>
+        <v>257</v>
       </c>
       <c r="L168" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6815,7 +6815,7 @@
         <v>Passed</v>
       </c>
       <c r="K169">
-        <v>349</v>
+        <v>151</v>
       </c>
       <c r="L169" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6853,7 +6853,7 @@
         <v>Passed</v>
       </c>
       <c r="K170">
-        <v>296</v>
+        <v>315</v>
       </c>
       <c r="L170" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6891,7 +6891,7 @@
         <v>Passed</v>
       </c>
       <c r="K171">
-        <v>202</v>
+        <v>271</v>
       </c>
       <c r="L171" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6929,7 +6929,7 @@
         <v>Passed</v>
       </c>
       <c r="K172">
-        <v>275</v>
+        <v>215</v>
       </c>
       <c r="L172" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6967,7 +6967,7 @@
         <v>Passed</v>
       </c>
       <c r="K173">
-        <v>329</v>
+        <v>357</v>
       </c>
       <c r="L173" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7005,7 +7005,7 @@
         <v>Passed</v>
       </c>
       <c r="K174">
-        <v>226</v>
+        <v>309</v>
       </c>
       <c r="L174" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7043,7 +7043,7 @@
         <v>Passed</v>
       </c>
       <c r="K175">
-        <v>364</v>
+        <v>266</v>
       </c>
       <c r="L175" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7081,7 +7081,7 @@
         <v>Passed</v>
       </c>
       <c r="K176">
-        <v>357</v>
+        <v>337</v>
       </c>
       <c r="L176" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7119,7 +7119,7 @@
         <v>Passed</v>
       </c>
       <c r="K177">
-        <v>274</v>
+        <v>353</v>
       </c>
       <c r="L177" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7157,7 +7157,7 @@
         <v>Passed</v>
       </c>
       <c r="K178">
-        <v>244</v>
+        <v>397</v>
       </c>
       <c r="L178" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7195,7 +7195,7 @@
         <v>Passed</v>
       </c>
       <c r="K179">
-        <v>344</v>
+        <v>363</v>
       </c>
       <c r="L179" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7233,7 +7233,7 @@
         <v>Passed</v>
       </c>
       <c r="K180">
-        <v>274</v>
+        <v>397</v>
       </c>
       <c r="L180" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7271,7 +7271,7 @@
         <v>Passed</v>
       </c>
       <c r="K181">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="L181" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7309,7 +7309,7 @@
         <v>Passed</v>
       </c>
       <c r="K182">
-        <v>246</v>
+        <v>256</v>
       </c>
       <c r="L182" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7347,7 +7347,7 @@
         <v>Passed</v>
       </c>
       <c r="K183">
-        <v>230</v>
+        <v>166</v>
       </c>
       <c r="L183" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7385,7 +7385,7 @@
         <v>Passed</v>
       </c>
       <c r="K184">
-        <v>398</v>
+        <v>176</v>
       </c>
       <c r="L184" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7423,7 +7423,7 @@
         <v>Passed</v>
       </c>
       <c r="K185">
-        <v>390</v>
+        <v>181</v>
       </c>
       <c r="L185" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7461,7 +7461,7 @@
         <v>Passed</v>
       </c>
       <c r="K186">
-        <v>299</v>
+        <v>152</v>
       </c>
       <c r="L186" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7499,7 +7499,7 @@
         <v>Passed</v>
       </c>
       <c r="K187">
-        <v>377</v>
+        <v>175</v>
       </c>
       <c r="L187" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7537,7 +7537,7 @@
         <v>Passed</v>
       </c>
       <c r="K188">
-        <v>156</v>
+        <v>235</v>
       </c>
       <c r="L188" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7575,7 +7575,7 @@
         <v>Passed</v>
       </c>
       <c r="K189">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="L189" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7613,7 +7613,7 @@
         <v>Passed</v>
       </c>
       <c r="K190">
-        <v>336</v>
+        <v>291</v>
       </c>
       <c r="L190" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7651,7 +7651,7 @@
         <v>Passed</v>
       </c>
       <c r="K191">
-        <v>186</v>
+        <v>261</v>
       </c>
       <c r="L191" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7689,7 +7689,7 @@
         <v>Passed</v>
       </c>
       <c r="K192">
-        <v>231</v>
+        <v>182</v>
       </c>
       <c r="L192" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7727,7 +7727,7 @@
         <v>Passed</v>
       </c>
       <c r="K193">
-        <v>185</v>
+        <v>248</v>
       </c>
       <c r="L193" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7765,7 +7765,7 @@
         <v>Passed</v>
       </c>
       <c r="K194">
-        <v>225</v>
+        <v>208</v>
       </c>
       <c r="L194" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7803,7 +7803,7 @@
         <v>Passed</v>
       </c>
       <c r="K195">
-        <v>333</v>
+        <v>156</v>
       </c>
       <c r="L195" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7841,7 +7841,7 @@
         <v>Passed</v>
       </c>
       <c r="K196">
-        <v>259</v>
+        <v>211</v>
       </c>
       <c r="L196" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7879,7 +7879,7 @@
         <v>Passed</v>
       </c>
       <c r="K197">
-        <v>317</v>
+        <v>285</v>
       </c>
       <c r="L197" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7917,7 +7917,7 @@
         <v>Passed</v>
       </c>
       <c r="K198">
-        <v>206</v>
+        <v>396</v>
       </c>
       <c r="L198" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7955,7 +7955,7 @@
         <v>Passed</v>
       </c>
       <c r="K199">
-        <v>334</v>
+        <v>236</v>
       </c>
       <c r="L199" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7993,7 +7993,7 @@
         <v>Passed</v>
       </c>
       <c r="K200">
-        <v>222</v>
+        <v>302</v>
       </c>
       <c r="L200" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8031,7 +8031,7 @@
         <v>Passed</v>
       </c>
       <c r="K201">
-        <v>269</v>
+        <v>366</v>
       </c>
       <c r="L201" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8069,7 +8069,7 @@
         <v>Passed</v>
       </c>
       <c r="K202">
-        <v>375</v>
+        <v>227</v>
       </c>
       <c r="L202" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8107,7 +8107,7 @@
         <v>Passed</v>
       </c>
       <c r="K203">
-        <v>332</v>
+        <v>209</v>
       </c>
       <c r="L203" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8145,7 +8145,7 @@
         <v>Passed</v>
       </c>
       <c r="K204">
-        <v>293</v>
+        <v>285</v>
       </c>
       <c r="L204" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8183,7 +8183,7 @@
         <v>Passed</v>
       </c>
       <c r="K205">
-        <v>288</v>
+        <v>341</v>
       </c>
       <c r="L205" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8221,7 +8221,7 @@
         <v>Passed</v>
       </c>
       <c r="K206">
-        <v>176</v>
+        <v>369</v>
       </c>
       <c r="L206" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8259,7 +8259,7 @@
         <v>Passed</v>
       </c>
       <c r="K207">
-        <v>358</v>
+        <v>260</v>
       </c>
       <c r="L207" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8297,7 +8297,7 @@
         <v>Passed</v>
       </c>
       <c r="K208">
-        <v>333</v>
+        <v>160</v>
       </c>
       <c r="L208" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8335,7 +8335,7 @@
         <v>Passed</v>
       </c>
       <c r="K209">
-        <v>175</v>
+        <v>157</v>
       </c>
       <c r="L209" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8373,7 +8373,7 @@
         <v>Passed</v>
       </c>
       <c r="K210">
-        <v>287</v>
+        <v>253</v>
       </c>
       <c r="L210" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8411,7 +8411,7 @@
         <v>Passed</v>
       </c>
       <c r="K211">
-        <v>175</v>
+        <v>155</v>
       </c>
       <c r="L211" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8449,7 +8449,7 @@
         <v>Passed</v>
       </c>
       <c r="K212">
-        <v>163</v>
+        <v>348</v>
       </c>
       <c r="L212" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8487,7 +8487,7 @@
         <v>Passed</v>
       </c>
       <c r="K213">
-        <v>293</v>
+        <v>272</v>
       </c>
       <c r="L213" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8525,7 +8525,7 @@
         <v>Passed</v>
       </c>
       <c r="K214">
-        <v>292</v>
+        <v>160</v>
       </c>
       <c r="L214" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8563,7 +8563,7 @@
         <v>Passed</v>
       </c>
       <c r="K215">
-        <v>200</v>
+        <v>276</v>
       </c>
       <c r="L215" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8601,7 +8601,7 @@
         <v>Passed</v>
       </c>
       <c r="K216">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="L216" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8639,7 +8639,7 @@
         <v>Passed</v>
       </c>
       <c r="K217">
-        <v>209</v>
+        <v>266</v>
       </c>
       <c r="L217" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8677,7 +8677,7 @@
         <v>Passed</v>
       </c>
       <c r="K218">
-        <v>306</v>
+        <v>331</v>
       </c>
       <c r="L218" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8715,7 +8715,7 @@
         <v>Passed</v>
       </c>
       <c r="K219">
-        <v>175</v>
+        <v>154</v>
       </c>
       <c r="L219" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8753,7 +8753,7 @@
         <v>Passed</v>
       </c>
       <c r="K220">
-        <v>396</v>
+        <v>277</v>
       </c>
       <c r="L220" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8791,7 +8791,7 @@
         <v>Passed</v>
       </c>
       <c r="K221">
-        <v>382</v>
+        <v>345</v>
       </c>
       <c r="L221" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8829,7 +8829,7 @@
         <v>Passed</v>
       </c>
       <c r="K222">
-        <v>310</v>
+        <v>209</v>
       </c>
       <c r="L222" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8867,7 +8867,7 @@
         <v>Passed</v>
       </c>
       <c r="K223">
-        <v>217</v>
+        <v>315</v>
       </c>
       <c r="L223" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8905,7 +8905,7 @@
         <v>Passed</v>
       </c>
       <c r="K224">
-        <v>275</v>
+        <v>283</v>
       </c>
       <c r="L224" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8943,7 +8943,7 @@
         <v>Passed</v>
       </c>
       <c r="K225">
-        <v>370</v>
+        <v>161</v>
       </c>
       <c r="L225" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8981,7 +8981,7 @@
         <v>Passed</v>
       </c>
       <c r="K226">
-        <v>260</v>
+        <v>293</v>
       </c>
       <c r="L226" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9019,7 +9019,7 @@
         <v>Passed</v>
       </c>
       <c r="K227">
-        <v>323</v>
+        <v>187</v>
       </c>
       <c r="L227" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9057,7 +9057,7 @@
         <v>Passed</v>
       </c>
       <c r="K228">
-        <v>324</v>
+        <v>345</v>
       </c>
       <c r="L228" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9095,7 +9095,7 @@
         <v>Passed</v>
       </c>
       <c r="K229">
-        <v>176</v>
+        <v>359</v>
       </c>
       <c r="L229" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9133,7 +9133,7 @@
         <v>Passed</v>
       </c>
       <c r="K230">
-        <v>370</v>
+        <v>173</v>
       </c>
       <c r="L230" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9171,7 +9171,7 @@
         <v>Passed</v>
       </c>
       <c r="K231">
-        <v>249</v>
+        <v>178</v>
       </c>
       <c r="L231" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9209,7 +9209,7 @@
         <v>Passed</v>
       </c>
       <c r="K232">
-        <v>237</v>
+        <v>153</v>
       </c>
       <c r="L232" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9247,7 +9247,7 @@
         <v>Passed</v>
       </c>
       <c r="K233">
-        <v>151</v>
+        <v>241</v>
       </c>
       <c r="L233" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9285,7 +9285,7 @@
         <v>Passed</v>
       </c>
       <c r="K234">
-        <v>392</v>
+        <v>332</v>
       </c>
       <c r="L234" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9323,7 +9323,7 @@
         <v>Passed</v>
       </c>
       <c r="K235">
-        <v>298</v>
+        <v>378</v>
       </c>
       <c r="L235" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9361,7 +9361,7 @@
         <v>Passed</v>
       </c>
       <c r="K236">
-        <v>200</v>
+        <v>259</v>
       </c>
       <c r="L236" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9399,7 +9399,7 @@
         <v>Passed</v>
       </c>
       <c r="K237">
-        <v>345</v>
+        <v>157</v>
       </c>
       <c r="L237" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9437,7 +9437,7 @@
         <v>Passed</v>
       </c>
       <c r="K238">
-        <v>204</v>
+        <v>173</v>
       </c>
       <c r="L238" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9475,7 +9475,7 @@
         <v>Passed</v>
       </c>
       <c r="K239">
-        <v>397</v>
+        <v>195</v>
       </c>
       <c r="L239" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9513,7 +9513,7 @@
         <v>Passed</v>
       </c>
       <c r="K240">
-        <v>182</v>
+        <v>333</v>
       </c>
       <c r="L240" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9551,7 +9551,7 @@
         <v>Passed</v>
       </c>
       <c r="K241">
-        <v>255</v>
+        <v>173</v>
       </c>
       <c r="L241" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9589,7 +9589,7 @@
         <v>Passed</v>
       </c>
       <c r="K242">
-        <v>363</v>
+        <v>304</v>
       </c>
       <c r="L242" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9627,7 +9627,7 @@
         <v>Passed</v>
       </c>
       <c r="K243">
-        <v>206</v>
+        <v>265</v>
       </c>
       <c r="L243" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9665,7 +9665,7 @@
         <v>Passed</v>
       </c>
       <c r="K244">
-        <v>393</v>
+        <v>218</v>
       </c>
       <c r="L244" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9703,7 +9703,7 @@
         <v>Passed</v>
       </c>
       <c r="K245">
-        <v>204</v>
+        <v>242</v>
       </c>
       <c r="L245" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9741,7 +9741,7 @@
         <v>Passed</v>
       </c>
       <c r="K246">
-        <v>162</v>
+        <v>258</v>
       </c>
       <c r="L246" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9779,7 +9779,7 @@
         <v>Passed</v>
       </c>
       <c r="K247">
-        <v>287</v>
+        <v>244</v>
       </c>
       <c r="L247" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9817,7 +9817,7 @@
         <v>Passed</v>
       </c>
       <c r="K248">
-        <v>314</v>
+        <v>236</v>
       </c>
       <c r="L248" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9855,7 +9855,7 @@
         <v>Passed</v>
       </c>
       <c r="K249">
-        <v>212</v>
+        <v>315</v>
       </c>
       <c r="L249" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9893,7 +9893,7 @@
         <v>Passed</v>
       </c>
       <c r="K250">
-        <v>188</v>
+        <v>369</v>
       </c>
       <c r="L250" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9931,7 +9931,7 @@
         <v>Passed</v>
       </c>
       <c r="K251">
-        <v>224</v>
+        <v>292</v>
       </c>
       <c r="L251" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9969,7 +9969,7 @@
         <v>Passed</v>
       </c>
       <c r="K252">
-        <v>350</v>
+        <v>265</v>
       </c>
       <c r="L252" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10007,7 +10007,7 @@
         <v>Passed</v>
       </c>
       <c r="K253">
-        <v>255</v>
+        <v>261</v>
       </c>
       <c r="L253" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10045,7 +10045,7 @@
         <v>Passed</v>
       </c>
       <c r="K254">
-        <v>267</v>
+        <v>301</v>
       </c>
       <c r="L254" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10083,7 +10083,7 @@
         <v>Passed</v>
       </c>
       <c r="K255">
-        <v>342</v>
+        <v>395</v>
       </c>
       <c r="L255" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10121,7 +10121,7 @@
         <v>Passed</v>
       </c>
       <c r="K256">
-        <v>348</v>
+        <v>319</v>
       </c>
       <c r="L256" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10159,7 +10159,7 @@
         <v>Passed</v>
       </c>
       <c r="K257">
-        <v>213</v>
+        <v>197</v>
       </c>
       <c r="L257" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10197,7 +10197,7 @@
         <v>Passed</v>
       </c>
       <c r="K258">
-        <v>372</v>
+        <v>294</v>
       </c>
       <c r="L258" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10235,7 +10235,7 @@
         <v>Passed</v>
       </c>
       <c r="K259">
-        <v>166</v>
+        <v>362</v>
       </c>
       <c r="L259" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10273,7 +10273,7 @@
         <v>Passed</v>
       </c>
       <c r="K260">
-        <v>194</v>
+        <v>362</v>
       </c>
       <c r="L260" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10311,7 +10311,7 @@
         <v>Passed</v>
       </c>
       <c r="K261">
-        <v>320</v>
+        <v>204</v>
       </c>
       <c r="L261" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10349,7 +10349,7 @@
         <v>Passed</v>
       </c>
       <c r="K262">
-        <v>301</v>
+        <v>295</v>
       </c>
       <c r="L262" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10387,7 +10387,7 @@
         <v>Passed</v>
       </c>
       <c r="K263">
-        <v>306</v>
+        <v>337</v>
       </c>
       <c r="L263" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10425,7 +10425,7 @@
         <v>Passed</v>
       </c>
       <c r="K264">
-        <v>227</v>
+        <v>260</v>
       </c>
       <c r="L264" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10463,7 +10463,7 @@
         <v>Passed</v>
       </c>
       <c r="K265">
-        <v>194</v>
+        <v>319</v>
       </c>
       <c r="L265" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10501,7 +10501,7 @@
         <v>Passed</v>
       </c>
       <c r="K266">
-        <v>201</v>
+        <v>278</v>
       </c>
       <c r="L266" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10539,7 +10539,7 @@
         <v>Passed</v>
       </c>
       <c r="K267">
-        <v>298</v>
+        <v>317</v>
       </c>
       <c r="L267" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10577,7 +10577,7 @@
         <v>Passed</v>
       </c>
       <c r="K268">
-        <v>232</v>
+        <v>335</v>
       </c>
       <c r="L268" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10615,7 +10615,7 @@
         <v>Passed</v>
       </c>
       <c r="K269">
-        <v>151</v>
+        <v>290</v>
       </c>
       <c r="L269" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10653,7 +10653,7 @@
         <v>Passed</v>
       </c>
       <c r="K270">
-        <v>381</v>
+        <v>289</v>
       </c>
       <c r="L270" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10691,7 +10691,7 @@
         <v>Passed</v>
       </c>
       <c r="K271">
-        <v>170</v>
+        <v>280</v>
       </c>
       <c r="L271" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10729,7 +10729,7 @@
         <v>Passed</v>
       </c>
       <c r="K272">
-        <v>346</v>
+        <v>159</v>
       </c>
       <c r="L272" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10767,7 +10767,7 @@
         <v>Passed</v>
       </c>
       <c r="K273">
-        <v>359</v>
+        <v>338</v>
       </c>
       <c r="L273" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10805,7 +10805,7 @@
         <v>Passed</v>
       </c>
       <c r="K274">
-        <v>210</v>
+        <v>152</v>
       </c>
       <c r="L274" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10843,7 +10843,7 @@
         <v>Passed</v>
       </c>
       <c r="K275">
-        <v>159</v>
+        <v>263</v>
       </c>
       <c r="L275" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10881,7 +10881,7 @@
         <v>Passed</v>
       </c>
       <c r="K276">
-        <v>210</v>
+        <v>242</v>
       </c>
       <c r="L276" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10919,7 +10919,7 @@
         <v>Passed</v>
       </c>
       <c r="K277">
-        <v>205</v>
+        <v>227</v>
       </c>
       <c r="L277" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10957,7 +10957,7 @@
         <v>Passed</v>
       </c>
       <c r="K278">
-        <v>163</v>
+        <v>388</v>
       </c>
       <c r="L278" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10995,7 +10995,7 @@
         <v>Passed</v>
       </c>
       <c r="K279">
-        <v>193</v>
+        <v>300</v>
       </c>
       <c r="L279" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11033,7 +11033,7 @@
         <v>Passed</v>
       </c>
       <c r="K280">
-        <v>264</v>
+        <v>253</v>
       </c>
       <c r="L280" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11071,7 +11071,7 @@
         <v>Passed</v>
       </c>
       <c r="K281">
-        <v>388</v>
+        <v>290</v>
       </c>
       <c r="L281" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11109,7 +11109,7 @@
         <v>Passed</v>
       </c>
       <c r="K282">
-        <v>307</v>
+        <v>229</v>
       </c>
       <c r="L282" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11147,7 +11147,7 @@
         <v>Passed</v>
       </c>
       <c r="K283">
-        <v>154</v>
+        <v>245</v>
       </c>
       <c r="L283" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11185,7 +11185,7 @@
         <v>Passed</v>
       </c>
       <c r="K284">
-        <v>191</v>
+        <v>376</v>
       </c>
       <c r="L284" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11223,7 +11223,7 @@
         <v>Passed</v>
       </c>
       <c r="K285">
-        <v>242</v>
+        <v>272</v>
       </c>
       <c r="L285" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11261,7 +11261,7 @@
         <v>Passed</v>
       </c>
       <c r="K286">
-        <v>229</v>
+        <v>189</v>
       </c>
       <c r="L286" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11299,7 +11299,7 @@
         <v>Passed</v>
       </c>
       <c r="K287">
-        <v>366</v>
+        <v>356</v>
       </c>
       <c r="L287" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11337,7 +11337,7 @@
         <v>Passed</v>
       </c>
       <c r="K288">
-        <v>258</v>
+        <v>206</v>
       </c>
       <c r="L288" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11375,7 +11375,7 @@
         <v>Passed</v>
       </c>
       <c r="K289">
-        <v>245</v>
+        <v>152</v>
       </c>
       <c r="L289" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11413,7 +11413,7 @@
         <v>Passed</v>
       </c>
       <c r="K290">
-        <v>385</v>
+        <v>192</v>
       </c>
       <c r="L290" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11451,7 +11451,7 @@
         <v>Passed</v>
       </c>
       <c r="K291">
-        <v>382</v>
+        <v>251</v>
       </c>
       <c r="L291" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11489,7 +11489,7 @@
         <v>Passed</v>
       </c>
       <c r="K292">
-        <v>191</v>
+        <v>371</v>
       </c>
       <c r="L292" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11527,7 +11527,7 @@
         <v>Passed</v>
       </c>
       <c r="K293">
-        <v>160</v>
+        <v>193</v>
       </c>
       <c r="L293" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11565,7 +11565,7 @@
         <v>Passed</v>
       </c>
       <c r="K294">
-        <v>284</v>
+        <v>304</v>
       </c>
       <c r="L294" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11603,7 +11603,7 @@
         <v>Passed</v>
       </c>
       <c r="K295">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="L295" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11641,7 +11641,7 @@
         <v>Passed</v>
       </c>
       <c r="K296">
-        <v>312</v>
+        <v>335</v>
       </c>
       <c r="L296" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11679,7 +11679,7 @@
         <v>Passed</v>
       </c>
       <c r="K297">
-        <v>239</v>
+        <v>378</v>
       </c>
       <c r="L297" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11717,7 +11717,7 @@
         <v>Passed</v>
       </c>
       <c r="K298">
-        <v>328</v>
+        <v>357</v>
       </c>
       <c r="L298" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11755,7 +11755,7 @@
         <v>Passed</v>
       </c>
       <c r="K299">
-        <v>284</v>
+        <v>388</v>
       </c>
       <c r="L299" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11793,7 +11793,7 @@
         <v>Passed</v>
       </c>
       <c r="K300">
-        <v>193</v>
+        <v>344</v>
       </c>
       <c r="L300" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11831,7 +11831,7 @@
         <v>Passed</v>
       </c>
       <c r="K301">
-        <v>245</v>
+        <v>237</v>
       </c>
       <c r="L301" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>

</xml_diff>

<commit_message>
feat: add 3D Holographic Pass, Stage Seat Picker, and top feature launcher bar
</commit_message>
<xml_diff>
--- a/EventSphere_Appium_Mobile_300_Report.xlsx
+++ b/EventSphere_Appium_Mobile_300_Report.xlsx
@@ -469,7 +469,7 @@
         <v>Passed</v>
       </c>
       <c r="K2">
-        <v>198</v>
+        <v>207</v>
       </c>
       <c r="L2" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -507,7 +507,7 @@
         <v>Passed</v>
       </c>
       <c r="K3">
-        <v>246</v>
+        <v>178</v>
       </c>
       <c r="L3" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -545,7 +545,7 @@
         <v>Passed</v>
       </c>
       <c r="K4">
-        <v>209</v>
+        <v>265</v>
       </c>
       <c r="L4" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -583,7 +583,7 @@
         <v>Passed</v>
       </c>
       <c r="K5">
-        <v>159</v>
+        <v>365</v>
       </c>
       <c r="L5" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -621,7 +621,7 @@
         <v>Passed</v>
       </c>
       <c r="K6">
-        <v>316</v>
+        <v>209</v>
       </c>
       <c r="L6" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -659,7 +659,7 @@
         <v>Passed</v>
       </c>
       <c r="K7">
-        <v>389</v>
+        <v>196</v>
       </c>
       <c r="L7" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -697,7 +697,7 @@
         <v>Passed</v>
       </c>
       <c r="K8">
-        <v>216</v>
+        <v>200</v>
       </c>
       <c r="L8" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -735,7 +735,7 @@
         <v>Passed</v>
       </c>
       <c r="K9">
-        <v>169</v>
+        <v>309</v>
       </c>
       <c r="L9" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -773,7 +773,7 @@
         <v>Passed</v>
       </c>
       <c r="K10">
-        <v>346</v>
+        <v>356</v>
       </c>
       <c r="L10" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -811,7 +811,7 @@
         <v>Passed</v>
       </c>
       <c r="K11">
-        <v>239</v>
+        <v>150</v>
       </c>
       <c r="L11" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -849,7 +849,7 @@
         <v>Passed</v>
       </c>
       <c r="K12">
-        <v>323</v>
+        <v>345</v>
       </c>
       <c r="L12" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -887,7 +887,7 @@
         <v>Passed</v>
       </c>
       <c r="K13">
-        <v>194</v>
+        <v>201</v>
       </c>
       <c r="L13" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -925,7 +925,7 @@
         <v>Passed</v>
       </c>
       <c r="K14">
-        <v>264</v>
+        <v>312</v>
       </c>
       <c r="L14" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -963,7 +963,7 @@
         <v>Passed</v>
       </c>
       <c r="K15">
-        <v>189</v>
+        <v>259</v>
       </c>
       <c r="L15" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1001,7 +1001,7 @@
         <v>Passed</v>
       </c>
       <c r="K16">
-        <v>395</v>
+        <v>198</v>
       </c>
       <c r="L16" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1039,7 +1039,7 @@
         <v>Passed</v>
       </c>
       <c r="K17">
-        <v>165</v>
+        <v>291</v>
       </c>
       <c r="L17" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1077,7 +1077,7 @@
         <v>Passed</v>
       </c>
       <c r="K18">
-        <v>369</v>
+        <v>357</v>
       </c>
       <c r="L18" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1115,7 +1115,7 @@
         <v>Passed</v>
       </c>
       <c r="K19">
-        <v>366</v>
+        <v>209</v>
       </c>
       <c r="L19" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1153,7 +1153,7 @@
         <v>Passed</v>
       </c>
       <c r="K20">
-        <v>192</v>
+        <v>278</v>
       </c>
       <c r="L20" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1191,7 +1191,7 @@
         <v>Passed</v>
       </c>
       <c r="K21">
-        <v>374</v>
+        <v>286</v>
       </c>
       <c r="L21" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1229,7 +1229,7 @@
         <v>Passed</v>
       </c>
       <c r="K22">
-        <v>157</v>
+        <v>255</v>
       </c>
       <c r="L22" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1267,7 +1267,7 @@
         <v>Passed</v>
       </c>
       <c r="K23">
-        <v>218</v>
+        <v>246</v>
       </c>
       <c r="L23" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1305,7 +1305,7 @@
         <v>Passed</v>
       </c>
       <c r="K24">
-        <v>273</v>
+        <v>308</v>
       </c>
       <c r="L24" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1343,7 +1343,7 @@
         <v>Passed</v>
       </c>
       <c r="K25">
-        <v>314</v>
+        <v>251</v>
       </c>
       <c r="L25" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1381,7 +1381,7 @@
         <v>Passed</v>
       </c>
       <c r="K26">
-        <v>174</v>
+        <v>279</v>
       </c>
       <c r="L26" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1419,7 +1419,7 @@
         <v>Passed</v>
       </c>
       <c r="K27">
-        <v>285</v>
+        <v>256</v>
       </c>
       <c r="L27" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1457,7 +1457,7 @@
         <v>Passed</v>
       </c>
       <c r="K28">
-        <v>174</v>
+        <v>218</v>
       </c>
       <c r="L28" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1495,7 +1495,7 @@
         <v>Passed</v>
       </c>
       <c r="K29">
-        <v>354</v>
+        <v>198</v>
       </c>
       <c r="L29" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1533,7 +1533,7 @@
         <v>Passed</v>
       </c>
       <c r="K30">
-        <v>255</v>
+        <v>165</v>
       </c>
       <c r="L30" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1571,7 +1571,7 @@
         <v>Passed</v>
       </c>
       <c r="K31">
-        <v>314</v>
+        <v>290</v>
       </c>
       <c r="L31" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1609,7 +1609,7 @@
         <v>Passed</v>
       </c>
       <c r="K32">
-        <v>159</v>
+        <v>255</v>
       </c>
       <c r="L32" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1647,7 +1647,7 @@
         <v>Passed</v>
       </c>
       <c r="K33">
-        <v>296</v>
+        <v>151</v>
       </c>
       <c r="L33" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1685,7 +1685,7 @@
         <v>Passed</v>
       </c>
       <c r="K34">
-        <v>394</v>
+        <v>218</v>
       </c>
       <c r="L34" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1723,7 +1723,7 @@
         <v>Passed</v>
       </c>
       <c r="K35">
-        <v>391</v>
+        <v>226</v>
       </c>
       <c r="L35" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1761,7 +1761,7 @@
         <v>Passed</v>
       </c>
       <c r="K36">
-        <v>356</v>
+        <v>329</v>
       </c>
       <c r="L36" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1799,7 +1799,7 @@
         <v>Passed</v>
       </c>
       <c r="K37">
-        <v>371</v>
+        <v>150</v>
       </c>
       <c r="L37" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1837,7 +1837,7 @@
         <v>Passed</v>
       </c>
       <c r="K38">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="L38" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1875,7 +1875,7 @@
         <v>Passed</v>
       </c>
       <c r="K39">
-        <v>346</v>
+        <v>351</v>
       </c>
       <c r="L39" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1913,7 +1913,7 @@
         <v>Passed</v>
       </c>
       <c r="K40">
-        <v>272</v>
+        <v>220</v>
       </c>
       <c r="L40" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1951,7 +1951,7 @@
         <v>Passed</v>
       </c>
       <c r="K41">
-        <v>294</v>
+        <v>272</v>
       </c>
       <c r="L41" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1989,7 +1989,7 @@
         <v>Passed</v>
       </c>
       <c r="K42">
-        <v>150</v>
+        <v>334</v>
       </c>
       <c r="L42" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2027,7 +2027,7 @@
         <v>Passed</v>
       </c>
       <c r="K43">
-        <v>189</v>
+        <v>282</v>
       </c>
       <c r="L43" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2065,7 +2065,7 @@
         <v>Passed</v>
       </c>
       <c r="K44">
-        <v>380</v>
+        <v>344</v>
       </c>
       <c r="L44" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2103,7 +2103,7 @@
         <v>Passed</v>
       </c>
       <c r="K45">
-        <v>386</v>
+        <v>339</v>
       </c>
       <c r="L45" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2141,7 +2141,7 @@
         <v>Passed</v>
       </c>
       <c r="K46">
-        <v>235</v>
+        <v>199</v>
       </c>
       <c r="L46" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2179,7 +2179,7 @@
         <v>Passed</v>
       </c>
       <c r="K47">
-        <v>234</v>
+        <v>220</v>
       </c>
       <c r="L47" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2217,7 +2217,7 @@
         <v>Passed</v>
       </c>
       <c r="K48">
-        <v>364</v>
+        <v>384</v>
       </c>
       <c r="L48" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2255,7 +2255,7 @@
         <v>Passed</v>
       </c>
       <c r="K49">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="L49" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2293,7 +2293,7 @@
         <v>Passed</v>
       </c>
       <c r="K50">
-        <v>190</v>
+        <v>211</v>
       </c>
       <c r="L50" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2331,7 +2331,7 @@
         <v>Passed</v>
       </c>
       <c r="K51">
-        <v>361</v>
+        <v>335</v>
       </c>
       <c r="L51" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2369,7 +2369,7 @@
         <v>Passed</v>
       </c>
       <c r="K52">
-        <v>342</v>
+        <v>187</v>
       </c>
       <c r="L52" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2407,7 +2407,7 @@
         <v>Passed</v>
       </c>
       <c r="K53">
-        <v>330</v>
+        <v>291</v>
       </c>
       <c r="L53" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2445,7 +2445,7 @@
         <v>Passed</v>
       </c>
       <c r="K54">
-        <v>337</v>
+        <v>191</v>
       </c>
       <c r="L54" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2483,7 +2483,7 @@
         <v>Passed</v>
       </c>
       <c r="K55">
-        <v>223</v>
+        <v>331</v>
       </c>
       <c r="L55" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2521,7 +2521,7 @@
         <v>Passed</v>
       </c>
       <c r="K56">
-        <v>157</v>
+        <v>375</v>
       </c>
       <c r="L56" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2559,7 +2559,7 @@
         <v>Passed</v>
       </c>
       <c r="K57">
-        <v>337</v>
+        <v>346</v>
       </c>
       <c r="L57" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2597,7 +2597,7 @@
         <v>Passed</v>
       </c>
       <c r="K58">
-        <v>169</v>
+        <v>179</v>
       </c>
       <c r="L58" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2635,7 +2635,7 @@
         <v>Passed</v>
       </c>
       <c r="K59">
-        <v>189</v>
+        <v>176</v>
       </c>
       <c r="L59" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2673,7 +2673,7 @@
         <v>Passed</v>
       </c>
       <c r="K60">
-        <v>196</v>
+        <v>314</v>
       </c>
       <c r="L60" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2711,7 +2711,7 @@
         <v>Passed</v>
       </c>
       <c r="K61">
-        <v>215</v>
+        <v>283</v>
       </c>
       <c r="L61" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2749,7 +2749,7 @@
         <v>Passed</v>
       </c>
       <c r="K62">
-        <v>250</v>
+        <v>227</v>
       </c>
       <c r="L62" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2787,7 +2787,7 @@
         <v>Passed</v>
       </c>
       <c r="K63">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="L63" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2825,7 +2825,7 @@
         <v>Passed</v>
       </c>
       <c r="K64">
-        <v>332</v>
+        <v>393</v>
       </c>
       <c r="L64" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2863,7 +2863,7 @@
         <v>Passed</v>
       </c>
       <c r="K65">
-        <v>296</v>
+        <v>217</v>
       </c>
       <c r="L65" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2901,7 +2901,7 @@
         <v>Passed</v>
       </c>
       <c r="K66">
-        <v>256</v>
+        <v>213</v>
       </c>
       <c r="L66" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2939,7 +2939,7 @@
         <v>Passed</v>
       </c>
       <c r="K67">
-        <v>379</v>
+        <v>164</v>
       </c>
       <c r="L67" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2977,7 +2977,7 @@
         <v>Passed</v>
       </c>
       <c r="K68">
-        <v>345</v>
+        <v>158</v>
       </c>
       <c r="L68" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3015,7 +3015,7 @@
         <v>Passed</v>
       </c>
       <c r="K69">
-        <v>351</v>
+        <v>207</v>
       </c>
       <c r="L69" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3053,7 +3053,7 @@
         <v>Passed</v>
       </c>
       <c r="K70">
-        <v>210</v>
+        <v>231</v>
       </c>
       <c r="L70" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3091,7 +3091,7 @@
         <v>Passed</v>
       </c>
       <c r="K71">
-        <v>381</v>
+        <v>388</v>
       </c>
       <c r="L71" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3129,7 +3129,7 @@
         <v>Passed</v>
       </c>
       <c r="K72">
-        <v>260</v>
+        <v>273</v>
       </c>
       <c r="L72" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3167,7 +3167,7 @@
         <v>Passed</v>
       </c>
       <c r="K73">
-        <v>303</v>
+        <v>312</v>
       </c>
       <c r="L73" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3205,7 +3205,7 @@
         <v>Passed</v>
       </c>
       <c r="K74">
-        <v>173</v>
+        <v>353</v>
       </c>
       <c r="L74" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3243,7 +3243,7 @@
         <v>Passed</v>
       </c>
       <c r="K75">
-        <v>303</v>
+        <v>289</v>
       </c>
       <c r="L75" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3281,7 +3281,7 @@
         <v>Passed</v>
       </c>
       <c r="K76">
-        <v>153</v>
+        <v>291</v>
       </c>
       <c r="L76" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3319,7 +3319,7 @@
         <v>Passed</v>
       </c>
       <c r="K77">
-        <v>280</v>
+        <v>339</v>
       </c>
       <c r="L77" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3357,7 +3357,7 @@
         <v>Passed</v>
       </c>
       <c r="K78">
-        <v>190</v>
+        <v>155</v>
       </c>
       <c r="L78" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3395,7 +3395,7 @@
         <v>Passed</v>
       </c>
       <c r="K79">
-        <v>335</v>
+        <v>361</v>
       </c>
       <c r="L79" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3433,7 +3433,7 @@
         <v>Passed</v>
       </c>
       <c r="K80">
-        <v>218</v>
+        <v>247</v>
       </c>
       <c r="L80" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3471,7 +3471,7 @@
         <v>Passed</v>
       </c>
       <c r="K81">
-        <v>222</v>
+        <v>174</v>
       </c>
       <c r="L81" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3509,7 +3509,7 @@
         <v>Passed</v>
       </c>
       <c r="K82">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="L82" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3547,7 +3547,7 @@
         <v>Passed</v>
       </c>
       <c r="K83">
-        <v>162</v>
+        <v>326</v>
       </c>
       <c r="L83" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3585,7 +3585,7 @@
         <v>Passed</v>
       </c>
       <c r="K84">
-        <v>398</v>
+        <v>221</v>
       </c>
       <c r="L84" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3623,7 +3623,7 @@
         <v>Passed</v>
       </c>
       <c r="K85">
-        <v>182</v>
+        <v>291</v>
       </c>
       <c r="L85" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3661,7 +3661,7 @@
         <v>Passed</v>
       </c>
       <c r="K86">
-        <v>302</v>
+        <v>244</v>
       </c>
       <c r="L86" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3699,7 +3699,7 @@
         <v>Passed</v>
       </c>
       <c r="K87">
-        <v>277</v>
+        <v>297</v>
       </c>
       <c r="L87" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3737,7 +3737,7 @@
         <v>Passed</v>
       </c>
       <c r="K88">
-        <v>231</v>
+        <v>215</v>
       </c>
       <c r="L88" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3775,7 +3775,7 @@
         <v>Passed</v>
       </c>
       <c r="K89">
-        <v>298</v>
+        <v>209</v>
       </c>
       <c r="L89" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3813,7 +3813,7 @@
         <v>Passed</v>
       </c>
       <c r="K90">
-        <v>364</v>
+        <v>346</v>
       </c>
       <c r="L90" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3851,7 +3851,7 @@
         <v>Passed</v>
       </c>
       <c r="K91">
-        <v>306</v>
+        <v>186</v>
       </c>
       <c r="L91" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3889,7 +3889,7 @@
         <v>Passed</v>
       </c>
       <c r="K92">
-        <v>366</v>
+        <v>324</v>
       </c>
       <c r="L92" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3927,7 +3927,7 @@
         <v>Passed</v>
       </c>
       <c r="K93">
-        <v>370</v>
+        <v>211</v>
       </c>
       <c r="L93" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3965,7 +3965,7 @@
         <v>Passed</v>
       </c>
       <c r="K94">
-        <v>288</v>
+        <v>371</v>
       </c>
       <c r="L94" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4003,7 +4003,7 @@
         <v>Passed</v>
       </c>
       <c r="K95">
-        <v>376</v>
+        <v>270</v>
       </c>
       <c r="L95" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4041,7 +4041,7 @@
         <v>Passed</v>
       </c>
       <c r="K96">
-        <v>262</v>
+        <v>330</v>
       </c>
       <c r="L96" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4079,7 +4079,7 @@
         <v>Passed</v>
       </c>
       <c r="K97">
-        <v>356</v>
+        <v>396</v>
       </c>
       <c r="L97" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4117,7 +4117,7 @@
         <v>Passed</v>
       </c>
       <c r="K98">
-        <v>325</v>
+        <v>193</v>
       </c>
       <c r="L98" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4155,7 +4155,7 @@
         <v>Passed</v>
       </c>
       <c r="K99">
-        <v>370</v>
+        <v>264</v>
       </c>
       <c r="L99" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4193,7 +4193,7 @@
         <v>Passed</v>
       </c>
       <c r="K100">
-        <v>272</v>
+        <v>255</v>
       </c>
       <c r="L100" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4231,7 +4231,7 @@
         <v>Passed</v>
       </c>
       <c r="K101">
-        <v>305</v>
+        <v>151</v>
       </c>
       <c r="L101" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4269,7 +4269,7 @@
         <v>Passed</v>
       </c>
       <c r="K102">
-        <v>311</v>
+        <v>351</v>
       </c>
       <c r="L102" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4307,7 +4307,7 @@
         <v>Passed</v>
       </c>
       <c r="K103">
-        <v>248</v>
+        <v>180</v>
       </c>
       <c r="L103" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4345,7 +4345,7 @@
         <v>Passed</v>
       </c>
       <c r="K104">
-        <v>184</v>
+        <v>338</v>
       </c>
       <c r="L104" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4383,7 +4383,7 @@
         <v>Passed</v>
       </c>
       <c r="K105">
-        <v>333</v>
+        <v>202</v>
       </c>
       <c r="L105" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4421,7 +4421,7 @@
         <v>Passed</v>
       </c>
       <c r="K106">
-        <v>374</v>
+        <v>380</v>
       </c>
       <c r="L106" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4459,7 +4459,7 @@
         <v>Passed</v>
       </c>
       <c r="K107">
-        <v>182</v>
+        <v>355</v>
       </c>
       <c r="L107" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4497,7 +4497,7 @@
         <v>Passed</v>
       </c>
       <c r="K108">
-        <v>263</v>
+        <v>326</v>
       </c>
       <c r="L108" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4535,7 +4535,7 @@
         <v>Passed</v>
       </c>
       <c r="K109">
-        <v>321</v>
+        <v>254</v>
       </c>
       <c r="L109" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4573,7 +4573,7 @@
         <v>Passed</v>
       </c>
       <c r="K110">
-        <v>311</v>
+        <v>323</v>
       </c>
       <c r="L110" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4611,7 +4611,7 @@
         <v>Passed</v>
       </c>
       <c r="K111">
-        <v>315</v>
+        <v>296</v>
       </c>
       <c r="L111" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4649,7 +4649,7 @@
         <v>Passed</v>
       </c>
       <c r="K112">
-        <v>393</v>
+        <v>383</v>
       </c>
       <c r="L112" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4687,7 +4687,7 @@
         <v>Passed</v>
       </c>
       <c r="K113">
-        <v>276</v>
+        <v>339</v>
       </c>
       <c r="L113" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4725,7 +4725,7 @@
         <v>Passed</v>
       </c>
       <c r="K114">
-        <v>358</v>
+        <v>212</v>
       </c>
       <c r="L114" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4763,7 +4763,7 @@
         <v>Passed</v>
       </c>
       <c r="K115">
-        <v>275</v>
+        <v>201</v>
       </c>
       <c r="L115" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4801,7 +4801,7 @@
         <v>Passed</v>
       </c>
       <c r="K116">
-        <v>303</v>
+        <v>344</v>
       </c>
       <c r="L116" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4839,7 +4839,7 @@
         <v>Passed</v>
       </c>
       <c r="K117">
-        <v>181</v>
+        <v>261</v>
       </c>
       <c r="L117" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4877,7 +4877,7 @@
         <v>Passed</v>
       </c>
       <c r="K118">
-        <v>223</v>
+        <v>392</v>
       </c>
       <c r="L118" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4915,7 +4915,7 @@
         <v>Passed</v>
       </c>
       <c r="K119">
-        <v>359</v>
+        <v>200</v>
       </c>
       <c r="L119" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4953,7 +4953,7 @@
         <v>Passed</v>
       </c>
       <c r="K120">
-        <v>377</v>
+        <v>210</v>
       </c>
       <c r="L120" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4991,7 +4991,7 @@
         <v>Passed</v>
       </c>
       <c r="K121">
-        <v>336</v>
+        <v>386</v>
       </c>
       <c r="L121" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5029,7 +5029,7 @@
         <v>Passed</v>
       </c>
       <c r="K122">
-        <v>190</v>
+        <v>317</v>
       </c>
       <c r="L122" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5067,7 +5067,7 @@
         <v>Passed</v>
       </c>
       <c r="K123">
-        <v>304</v>
+        <v>228</v>
       </c>
       <c r="L123" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5105,7 +5105,7 @@
         <v>Passed</v>
       </c>
       <c r="K124">
-        <v>371</v>
+        <v>228</v>
       </c>
       <c r="L124" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5143,7 +5143,7 @@
         <v>Passed</v>
       </c>
       <c r="K125">
-        <v>328</v>
+        <v>355</v>
       </c>
       <c r="L125" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5181,7 +5181,7 @@
         <v>Passed</v>
       </c>
       <c r="K126">
-        <v>330</v>
+        <v>265</v>
       </c>
       <c r="L126" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5219,7 +5219,7 @@
         <v>Passed</v>
       </c>
       <c r="K127">
-        <v>357</v>
+        <v>207</v>
       </c>
       <c r="L127" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5257,7 +5257,7 @@
         <v>Passed</v>
       </c>
       <c r="K128">
-        <v>159</v>
+        <v>199</v>
       </c>
       <c r="L128" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5295,7 +5295,7 @@
         <v>Passed</v>
       </c>
       <c r="K129">
-        <v>230</v>
+        <v>370</v>
       </c>
       <c r="L129" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5333,7 +5333,7 @@
         <v>Passed</v>
       </c>
       <c r="K130">
-        <v>263</v>
+        <v>386</v>
       </c>
       <c r="L130" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5371,7 +5371,7 @@
         <v>Passed</v>
       </c>
       <c r="K131">
-        <v>170</v>
+        <v>159</v>
       </c>
       <c r="L131" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5409,7 +5409,7 @@
         <v>Passed</v>
       </c>
       <c r="K132">
-        <v>180</v>
+        <v>168</v>
       </c>
       <c r="L132" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5447,7 +5447,7 @@
         <v>Passed</v>
       </c>
       <c r="K133">
-        <v>236</v>
+        <v>165</v>
       </c>
       <c r="L133" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5485,7 +5485,7 @@
         <v>Passed</v>
       </c>
       <c r="K134">
-        <v>208</v>
+        <v>306</v>
       </c>
       <c r="L134" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5523,7 +5523,7 @@
         <v>Passed</v>
       </c>
       <c r="K135">
-        <v>171</v>
+        <v>318</v>
       </c>
       <c r="L135" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5599,7 +5599,7 @@
         <v>Passed</v>
       </c>
       <c r="K137">
-        <v>389</v>
+        <v>207</v>
       </c>
       <c r="L137" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5637,7 +5637,7 @@
         <v>Passed</v>
       </c>
       <c r="K138">
-        <v>387</v>
+        <v>267</v>
       </c>
       <c r="L138" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5675,7 +5675,7 @@
         <v>Passed</v>
       </c>
       <c r="K139">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="L139" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5713,7 +5713,7 @@
         <v>Passed</v>
       </c>
       <c r="K140">
-        <v>234</v>
+        <v>187</v>
       </c>
       <c r="L140" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5751,7 +5751,7 @@
         <v>Passed</v>
       </c>
       <c r="K141">
-        <v>197</v>
+        <v>221</v>
       </c>
       <c r="L141" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5789,7 +5789,7 @@
         <v>Passed</v>
       </c>
       <c r="K142">
-        <v>258</v>
+        <v>399</v>
       </c>
       <c r="L142" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5827,7 +5827,7 @@
         <v>Passed</v>
       </c>
       <c r="K143">
-        <v>298</v>
+        <v>333</v>
       </c>
       <c r="L143" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5865,7 +5865,7 @@
         <v>Passed</v>
       </c>
       <c r="K144">
-        <v>296</v>
+        <v>254</v>
       </c>
       <c r="L144" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5903,7 +5903,7 @@
         <v>Passed</v>
       </c>
       <c r="K145">
-        <v>187</v>
+        <v>235</v>
       </c>
       <c r="L145" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5941,7 +5941,7 @@
         <v>Passed</v>
       </c>
       <c r="K146">
-        <v>316</v>
+        <v>241</v>
       </c>
       <c r="L146" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5979,7 +5979,7 @@
         <v>Passed</v>
       </c>
       <c r="K147">
-        <v>188</v>
+        <v>321</v>
       </c>
       <c r="L147" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6017,7 +6017,7 @@
         <v>Passed</v>
       </c>
       <c r="K148">
-        <v>253</v>
+        <v>366</v>
       </c>
       <c r="L148" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6055,7 +6055,7 @@
         <v>Passed</v>
       </c>
       <c r="K149">
-        <v>393</v>
+        <v>360</v>
       </c>
       <c r="L149" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6093,7 +6093,7 @@
         <v>Passed</v>
       </c>
       <c r="K150">
-        <v>289</v>
+        <v>167</v>
       </c>
       <c r="L150" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6131,7 +6131,7 @@
         <v>Passed</v>
       </c>
       <c r="K151">
-        <v>248</v>
+        <v>380</v>
       </c>
       <c r="L151" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6169,7 +6169,7 @@
         <v>Passed</v>
       </c>
       <c r="K152">
-        <v>378</v>
+        <v>333</v>
       </c>
       <c r="L152" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6207,7 +6207,7 @@
         <v>Passed</v>
       </c>
       <c r="K153">
-        <v>266</v>
+        <v>280</v>
       </c>
       <c r="L153" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6245,7 +6245,7 @@
         <v>Passed</v>
       </c>
       <c r="K154">
-        <v>374</v>
+        <v>361</v>
       </c>
       <c r="L154" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6283,7 +6283,7 @@
         <v>Passed</v>
       </c>
       <c r="K155">
-        <v>195</v>
+        <v>335</v>
       </c>
       <c r="L155" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6321,7 +6321,7 @@
         <v>Passed</v>
       </c>
       <c r="K156">
-        <v>378</v>
+        <v>390</v>
       </c>
       <c r="L156" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6359,7 +6359,7 @@
         <v>Passed</v>
       </c>
       <c r="K157">
-        <v>292</v>
+        <v>155</v>
       </c>
       <c r="L157" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6397,7 +6397,7 @@
         <v>Passed</v>
       </c>
       <c r="K158">
-        <v>310</v>
+        <v>345</v>
       </c>
       <c r="L158" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6435,7 +6435,7 @@
         <v>Passed</v>
       </c>
       <c r="K159">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="L159" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6473,7 +6473,7 @@
         <v>Passed</v>
       </c>
       <c r="K160">
-        <v>273</v>
+        <v>357</v>
       </c>
       <c r="L160" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6511,7 +6511,7 @@
         <v>Passed</v>
       </c>
       <c r="K161">
-        <v>213</v>
+        <v>241</v>
       </c>
       <c r="L161" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6549,7 +6549,7 @@
         <v>Passed</v>
       </c>
       <c r="K162">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="L162" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6587,7 +6587,7 @@
         <v>Passed</v>
       </c>
       <c r="K163">
-        <v>245</v>
+        <v>321</v>
       </c>
       <c r="L163" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6625,7 +6625,7 @@
         <v>Passed</v>
       </c>
       <c r="K164">
-        <v>227</v>
+        <v>323</v>
       </c>
       <c r="L164" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6663,7 +6663,7 @@
         <v>Passed</v>
       </c>
       <c r="K165">
-        <v>389</v>
+        <v>224</v>
       </c>
       <c r="L165" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6701,7 +6701,7 @@
         <v>Passed</v>
       </c>
       <c r="K166">
-        <v>276</v>
+        <v>270</v>
       </c>
       <c r="L166" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6739,7 +6739,7 @@
         <v>Passed</v>
       </c>
       <c r="K167">
-        <v>389</v>
+        <v>273</v>
       </c>
       <c r="L167" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6777,7 +6777,7 @@
         <v>Passed</v>
       </c>
       <c r="K168">
-        <v>257</v>
+        <v>213</v>
       </c>
       <c r="L168" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6815,7 +6815,7 @@
         <v>Passed</v>
       </c>
       <c r="K169">
-        <v>151</v>
+        <v>373</v>
       </c>
       <c r="L169" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6853,7 +6853,7 @@
         <v>Passed</v>
       </c>
       <c r="K170">
-        <v>315</v>
+        <v>248</v>
       </c>
       <c r="L170" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6891,7 +6891,7 @@
         <v>Passed</v>
       </c>
       <c r="K171">
-        <v>271</v>
+        <v>170</v>
       </c>
       <c r="L171" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6929,7 +6929,7 @@
         <v>Passed</v>
       </c>
       <c r="K172">
-        <v>215</v>
+        <v>285</v>
       </c>
       <c r="L172" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6967,7 +6967,7 @@
         <v>Passed</v>
       </c>
       <c r="K173">
-        <v>357</v>
+        <v>307</v>
       </c>
       <c r="L173" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7005,7 +7005,7 @@
         <v>Passed</v>
       </c>
       <c r="K174">
-        <v>309</v>
+        <v>194</v>
       </c>
       <c r="L174" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7043,7 +7043,7 @@
         <v>Passed</v>
       </c>
       <c r="K175">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="L175" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7081,7 +7081,7 @@
         <v>Passed</v>
       </c>
       <c r="K176">
-        <v>337</v>
+        <v>220</v>
       </c>
       <c r="L176" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7119,7 +7119,7 @@
         <v>Passed</v>
       </c>
       <c r="K177">
-        <v>353</v>
+        <v>207</v>
       </c>
       <c r="L177" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7157,7 +7157,7 @@
         <v>Passed</v>
       </c>
       <c r="K178">
-        <v>397</v>
+        <v>363</v>
       </c>
       <c r="L178" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7195,7 +7195,7 @@
         <v>Passed</v>
       </c>
       <c r="K179">
-        <v>363</v>
+        <v>195</v>
       </c>
       <c r="L179" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7233,7 +7233,7 @@
         <v>Passed</v>
       </c>
       <c r="K180">
-        <v>397</v>
+        <v>202</v>
       </c>
       <c r="L180" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7271,7 +7271,7 @@
         <v>Passed</v>
       </c>
       <c r="K181">
-        <v>397</v>
+        <v>253</v>
       </c>
       <c r="L181" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7309,7 +7309,7 @@
         <v>Passed</v>
       </c>
       <c r="K182">
-        <v>256</v>
+        <v>318</v>
       </c>
       <c r="L182" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7347,7 +7347,7 @@
         <v>Passed</v>
       </c>
       <c r="K183">
-        <v>166</v>
+        <v>216</v>
       </c>
       <c r="L183" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7385,7 +7385,7 @@
         <v>Passed</v>
       </c>
       <c r="K184">
-        <v>176</v>
+        <v>378</v>
       </c>
       <c r="L184" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7423,7 +7423,7 @@
         <v>Passed</v>
       </c>
       <c r="K185">
-        <v>181</v>
+        <v>205</v>
       </c>
       <c r="L185" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7461,7 +7461,7 @@
         <v>Passed</v>
       </c>
       <c r="K186">
-        <v>152</v>
+        <v>274</v>
       </c>
       <c r="L186" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7499,7 +7499,7 @@
         <v>Passed</v>
       </c>
       <c r="K187">
-        <v>175</v>
+        <v>338</v>
       </c>
       <c r="L187" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7537,7 +7537,7 @@
         <v>Passed</v>
       </c>
       <c r="K188">
-        <v>235</v>
+        <v>374</v>
       </c>
       <c r="L188" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7575,7 +7575,7 @@
         <v>Passed</v>
       </c>
       <c r="K189">
-        <v>166</v>
+        <v>197</v>
       </c>
       <c r="L189" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7613,7 +7613,7 @@
         <v>Passed</v>
       </c>
       <c r="K190">
-        <v>291</v>
+        <v>248</v>
       </c>
       <c r="L190" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7651,7 +7651,7 @@
         <v>Passed</v>
       </c>
       <c r="K191">
-        <v>261</v>
+        <v>331</v>
       </c>
       <c r="L191" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7689,7 +7689,7 @@
         <v>Passed</v>
       </c>
       <c r="K192">
-        <v>182</v>
+        <v>209</v>
       </c>
       <c r="L192" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7727,7 +7727,7 @@
         <v>Passed</v>
       </c>
       <c r="K193">
-        <v>248</v>
+        <v>290</v>
       </c>
       <c r="L193" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7765,7 +7765,7 @@
         <v>Passed</v>
       </c>
       <c r="K194">
-        <v>208</v>
+        <v>166</v>
       </c>
       <c r="L194" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7803,7 +7803,7 @@
         <v>Passed</v>
       </c>
       <c r="K195">
-        <v>156</v>
+        <v>260</v>
       </c>
       <c r="L195" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7841,7 +7841,7 @@
         <v>Passed</v>
       </c>
       <c r="K196">
-        <v>211</v>
+        <v>278</v>
       </c>
       <c r="L196" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7879,7 +7879,7 @@
         <v>Passed</v>
       </c>
       <c r="K197">
-        <v>285</v>
+        <v>165</v>
       </c>
       <c r="L197" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7917,7 +7917,7 @@
         <v>Passed</v>
       </c>
       <c r="K198">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="L198" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7955,7 +7955,7 @@
         <v>Passed</v>
       </c>
       <c r="K199">
-        <v>236</v>
+        <v>304</v>
       </c>
       <c r="L199" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7993,7 +7993,7 @@
         <v>Passed</v>
       </c>
       <c r="K200">
-        <v>302</v>
+        <v>207</v>
       </c>
       <c r="L200" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8031,7 +8031,7 @@
         <v>Passed</v>
       </c>
       <c r="K201">
-        <v>366</v>
+        <v>208</v>
       </c>
       <c r="L201" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8069,7 +8069,7 @@
         <v>Passed</v>
       </c>
       <c r="K202">
-        <v>227</v>
+        <v>359</v>
       </c>
       <c r="L202" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8107,7 +8107,7 @@
         <v>Passed</v>
       </c>
       <c r="K203">
-        <v>209</v>
+        <v>307</v>
       </c>
       <c r="L203" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8145,7 +8145,7 @@
         <v>Passed</v>
       </c>
       <c r="K204">
-        <v>285</v>
+        <v>158</v>
       </c>
       <c r="L204" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8183,7 +8183,7 @@
         <v>Passed</v>
       </c>
       <c r="K205">
-        <v>341</v>
+        <v>312</v>
       </c>
       <c r="L205" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8221,7 +8221,7 @@
         <v>Passed</v>
       </c>
       <c r="K206">
-        <v>369</v>
+        <v>217</v>
       </c>
       <c r="L206" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8259,7 +8259,7 @@
         <v>Passed</v>
       </c>
       <c r="K207">
-        <v>260</v>
+        <v>251</v>
       </c>
       <c r="L207" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8297,7 +8297,7 @@
         <v>Passed</v>
       </c>
       <c r="K208">
-        <v>160</v>
+        <v>259</v>
       </c>
       <c r="L208" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8335,7 +8335,7 @@
         <v>Passed</v>
       </c>
       <c r="K209">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="L209" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8373,7 +8373,7 @@
         <v>Passed</v>
       </c>
       <c r="K210">
-        <v>253</v>
+        <v>210</v>
       </c>
       <c r="L210" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8411,7 +8411,7 @@
         <v>Passed</v>
       </c>
       <c r="K211">
-        <v>155</v>
+        <v>240</v>
       </c>
       <c r="L211" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8449,7 +8449,7 @@
         <v>Passed</v>
       </c>
       <c r="K212">
-        <v>348</v>
+        <v>197</v>
       </c>
       <c r="L212" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8487,7 +8487,7 @@
         <v>Passed</v>
       </c>
       <c r="K213">
-        <v>272</v>
+        <v>188</v>
       </c>
       <c r="L213" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8525,7 +8525,7 @@
         <v>Passed</v>
       </c>
       <c r="K214">
-        <v>160</v>
+        <v>385</v>
       </c>
       <c r="L214" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8563,7 +8563,7 @@
         <v>Passed</v>
       </c>
       <c r="K215">
-        <v>276</v>
+        <v>318</v>
       </c>
       <c r="L215" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8601,7 +8601,7 @@
         <v>Passed</v>
       </c>
       <c r="K216">
-        <v>377</v>
+        <v>177</v>
       </c>
       <c r="L216" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8639,7 +8639,7 @@
         <v>Passed</v>
       </c>
       <c r="K217">
-        <v>266</v>
+        <v>250</v>
       </c>
       <c r="L217" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8677,7 +8677,7 @@
         <v>Passed</v>
       </c>
       <c r="K218">
-        <v>331</v>
+        <v>221</v>
       </c>
       <c r="L218" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8715,7 +8715,7 @@
         <v>Passed</v>
       </c>
       <c r="K219">
-        <v>154</v>
+        <v>195</v>
       </c>
       <c r="L219" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8753,7 +8753,7 @@
         <v>Passed</v>
       </c>
       <c r="K220">
-        <v>277</v>
+        <v>234</v>
       </c>
       <c r="L220" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8791,7 +8791,7 @@
         <v>Passed</v>
       </c>
       <c r="K221">
-        <v>345</v>
+        <v>369</v>
       </c>
       <c r="L221" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8829,7 +8829,7 @@
         <v>Passed</v>
       </c>
       <c r="K222">
-        <v>209</v>
+        <v>267</v>
       </c>
       <c r="L222" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8867,7 +8867,7 @@
         <v>Passed</v>
       </c>
       <c r="K223">
-        <v>315</v>
+        <v>330</v>
       </c>
       <c r="L223" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8905,7 +8905,7 @@
         <v>Passed</v>
       </c>
       <c r="K224">
-        <v>283</v>
+        <v>311</v>
       </c>
       <c r="L224" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8943,7 +8943,7 @@
         <v>Passed</v>
       </c>
       <c r="K225">
-        <v>161</v>
+        <v>236</v>
       </c>
       <c r="L225" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8981,7 +8981,7 @@
         <v>Passed</v>
       </c>
       <c r="K226">
-        <v>293</v>
+        <v>193</v>
       </c>
       <c r="L226" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9019,7 +9019,7 @@
         <v>Passed</v>
       </c>
       <c r="K227">
-        <v>187</v>
+        <v>325</v>
       </c>
       <c r="L227" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9057,7 +9057,7 @@
         <v>Passed</v>
       </c>
       <c r="K228">
-        <v>345</v>
+        <v>200</v>
       </c>
       <c r="L228" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9095,7 +9095,7 @@
         <v>Passed</v>
       </c>
       <c r="K229">
-        <v>359</v>
+        <v>251</v>
       </c>
       <c r="L229" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9133,7 +9133,7 @@
         <v>Passed</v>
       </c>
       <c r="K230">
-        <v>173</v>
+        <v>279</v>
       </c>
       <c r="L230" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9171,7 +9171,7 @@
         <v>Passed</v>
       </c>
       <c r="K231">
-        <v>178</v>
+        <v>249</v>
       </c>
       <c r="L231" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9209,7 +9209,7 @@
         <v>Passed</v>
       </c>
       <c r="K232">
-        <v>153</v>
+        <v>398</v>
       </c>
       <c r="L232" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9247,7 +9247,7 @@
         <v>Passed</v>
       </c>
       <c r="K233">
-        <v>241</v>
+        <v>294</v>
       </c>
       <c r="L233" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9285,7 +9285,7 @@
         <v>Passed</v>
       </c>
       <c r="K234">
-        <v>332</v>
+        <v>358</v>
       </c>
       <c r="L234" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9323,7 +9323,7 @@
         <v>Passed</v>
       </c>
       <c r="K235">
-        <v>378</v>
+        <v>188</v>
       </c>
       <c r="L235" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9361,7 +9361,7 @@
         <v>Passed</v>
       </c>
       <c r="K236">
-        <v>259</v>
+        <v>325</v>
       </c>
       <c r="L236" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9399,7 +9399,7 @@
         <v>Passed</v>
       </c>
       <c r="K237">
-        <v>157</v>
+        <v>336</v>
       </c>
       <c r="L237" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9437,7 +9437,7 @@
         <v>Passed</v>
       </c>
       <c r="K238">
-        <v>173</v>
+        <v>187</v>
       </c>
       <c r="L238" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9475,7 +9475,7 @@
         <v>Passed</v>
       </c>
       <c r="K239">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="L239" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9513,7 +9513,7 @@
         <v>Passed</v>
       </c>
       <c r="K240">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="L240" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9551,7 +9551,7 @@
         <v>Passed</v>
       </c>
       <c r="K241">
-        <v>173</v>
+        <v>205</v>
       </c>
       <c r="L241" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9589,7 +9589,7 @@
         <v>Passed</v>
       </c>
       <c r="K242">
-        <v>304</v>
+        <v>207</v>
       </c>
       <c r="L242" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9627,7 +9627,7 @@
         <v>Passed</v>
       </c>
       <c r="K243">
-        <v>265</v>
+        <v>307</v>
       </c>
       <c r="L243" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9665,7 +9665,7 @@
         <v>Passed</v>
       </c>
       <c r="K244">
-        <v>218</v>
+        <v>190</v>
       </c>
       <c r="L244" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9703,7 +9703,7 @@
         <v>Passed</v>
       </c>
       <c r="K245">
-        <v>242</v>
+        <v>232</v>
       </c>
       <c r="L245" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9741,7 +9741,7 @@
         <v>Passed</v>
       </c>
       <c r="K246">
-        <v>258</v>
+        <v>382</v>
       </c>
       <c r="L246" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9779,7 +9779,7 @@
         <v>Passed</v>
       </c>
       <c r="K247">
-        <v>244</v>
+        <v>166</v>
       </c>
       <c r="L247" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9817,7 +9817,7 @@
         <v>Passed</v>
       </c>
       <c r="K248">
-        <v>236</v>
+        <v>247</v>
       </c>
       <c r="L248" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9855,7 +9855,7 @@
         <v>Passed</v>
       </c>
       <c r="K249">
-        <v>315</v>
+        <v>332</v>
       </c>
       <c r="L249" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9893,7 +9893,7 @@
         <v>Passed</v>
       </c>
       <c r="K250">
-        <v>369</v>
+        <v>211</v>
       </c>
       <c r="L250" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9931,7 +9931,7 @@
         <v>Passed</v>
       </c>
       <c r="K251">
-        <v>292</v>
+        <v>372</v>
       </c>
       <c r="L251" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9969,7 +9969,7 @@
         <v>Passed</v>
       </c>
       <c r="K252">
-        <v>265</v>
+        <v>282</v>
       </c>
       <c r="L252" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10007,7 +10007,7 @@
         <v>Passed</v>
       </c>
       <c r="K253">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="L253" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10045,7 +10045,7 @@
         <v>Passed</v>
       </c>
       <c r="K254">
-        <v>301</v>
+        <v>170</v>
       </c>
       <c r="L254" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10083,7 +10083,7 @@
         <v>Passed</v>
       </c>
       <c r="K255">
-        <v>395</v>
+        <v>392</v>
       </c>
       <c r="L255" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10121,7 +10121,7 @@
         <v>Passed</v>
       </c>
       <c r="K256">
-        <v>319</v>
+        <v>333</v>
       </c>
       <c r="L256" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10159,7 +10159,7 @@
         <v>Passed</v>
       </c>
       <c r="K257">
-        <v>197</v>
+        <v>315</v>
       </c>
       <c r="L257" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10197,7 +10197,7 @@
         <v>Passed</v>
       </c>
       <c r="K258">
-        <v>294</v>
+        <v>318</v>
       </c>
       <c r="L258" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10235,7 +10235,7 @@
         <v>Passed</v>
       </c>
       <c r="K259">
-        <v>362</v>
+        <v>254</v>
       </c>
       <c r="L259" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10273,7 +10273,7 @@
         <v>Passed</v>
       </c>
       <c r="K260">
-        <v>362</v>
+        <v>236</v>
       </c>
       <c r="L260" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10311,7 +10311,7 @@
         <v>Passed</v>
       </c>
       <c r="K261">
-        <v>204</v>
+        <v>215</v>
       </c>
       <c r="L261" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10349,7 +10349,7 @@
         <v>Passed</v>
       </c>
       <c r="K262">
-        <v>295</v>
+        <v>206</v>
       </c>
       <c r="L262" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10387,7 +10387,7 @@
         <v>Passed</v>
       </c>
       <c r="K263">
-        <v>337</v>
+        <v>263</v>
       </c>
       <c r="L263" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10425,7 +10425,7 @@
         <v>Passed</v>
       </c>
       <c r="K264">
-        <v>260</v>
+        <v>328</v>
       </c>
       <c r="L264" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10463,7 +10463,7 @@
         <v>Passed</v>
       </c>
       <c r="K265">
-        <v>319</v>
+        <v>387</v>
       </c>
       <c r="L265" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10501,7 +10501,7 @@
         <v>Passed</v>
       </c>
       <c r="K266">
-        <v>278</v>
+        <v>150</v>
       </c>
       <c r="L266" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10539,7 +10539,7 @@
         <v>Passed</v>
       </c>
       <c r="K267">
-        <v>317</v>
+        <v>288</v>
       </c>
       <c r="L267" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10577,7 +10577,7 @@
         <v>Passed</v>
       </c>
       <c r="K268">
-        <v>335</v>
+        <v>301</v>
       </c>
       <c r="L268" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10615,7 +10615,7 @@
         <v>Passed</v>
       </c>
       <c r="K269">
-        <v>290</v>
+        <v>365</v>
       </c>
       <c r="L269" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10653,7 +10653,7 @@
         <v>Passed</v>
       </c>
       <c r="K270">
-        <v>289</v>
+        <v>175</v>
       </c>
       <c r="L270" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10691,7 +10691,7 @@
         <v>Passed</v>
       </c>
       <c r="K271">
-        <v>280</v>
+        <v>218</v>
       </c>
       <c r="L271" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10729,7 +10729,7 @@
         <v>Passed</v>
       </c>
       <c r="K272">
-        <v>159</v>
+        <v>276</v>
       </c>
       <c r="L272" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10767,7 +10767,7 @@
         <v>Passed</v>
       </c>
       <c r="K273">
-        <v>338</v>
+        <v>354</v>
       </c>
       <c r="L273" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10805,7 +10805,7 @@
         <v>Passed</v>
       </c>
       <c r="K274">
-        <v>152</v>
+        <v>357</v>
       </c>
       <c r="L274" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10843,7 +10843,7 @@
         <v>Passed</v>
       </c>
       <c r="K275">
-        <v>263</v>
+        <v>235</v>
       </c>
       <c r="L275" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10881,7 +10881,7 @@
         <v>Passed</v>
       </c>
       <c r="K276">
-        <v>242</v>
+        <v>184</v>
       </c>
       <c r="L276" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10919,7 +10919,7 @@
         <v>Passed</v>
       </c>
       <c r="K277">
-        <v>227</v>
+        <v>377</v>
       </c>
       <c r="L277" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10957,7 +10957,7 @@
         <v>Passed</v>
       </c>
       <c r="K278">
-        <v>388</v>
+        <v>334</v>
       </c>
       <c r="L278" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10995,7 +10995,7 @@
         <v>Passed</v>
       </c>
       <c r="K279">
-        <v>300</v>
+        <v>278</v>
       </c>
       <c r="L279" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11033,7 +11033,7 @@
         <v>Passed</v>
       </c>
       <c r="K280">
-        <v>253</v>
+        <v>382</v>
       </c>
       <c r="L280" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11071,7 +11071,7 @@
         <v>Passed</v>
       </c>
       <c r="K281">
-        <v>290</v>
+        <v>263</v>
       </c>
       <c r="L281" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11109,7 +11109,7 @@
         <v>Passed</v>
       </c>
       <c r="K282">
-        <v>229</v>
+        <v>308</v>
       </c>
       <c r="L282" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11147,7 +11147,7 @@
         <v>Passed</v>
       </c>
       <c r="K283">
-        <v>245</v>
+        <v>381</v>
       </c>
       <c r="L283" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11185,7 +11185,7 @@
         <v>Passed</v>
       </c>
       <c r="K284">
-        <v>376</v>
+        <v>246</v>
       </c>
       <c r="L284" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11223,7 +11223,7 @@
         <v>Passed</v>
       </c>
       <c r="K285">
-        <v>272</v>
+        <v>207</v>
       </c>
       <c r="L285" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11261,7 +11261,7 @@
         <v>Passed</v>
       </c>
       <c r="K286">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="L286" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11299,7 +11299,7 @@
         <v>Passed</v>
       </c>
       <c r="K287">
-        <v>356</v>
+        <v>351</v>
       </c>
       <c r="L287" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11337,7 +11337,7 @@
         <v>Passed</v>
       </c>
       <c r="K288">
-        <v>206</v>
+        <v>289</v>
       </c>
       <c r="L288" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11375,7 +11375,7 @@
         <v>Passed</v>
       </c>
       <c r="K289">
-        <v>152</v>
+        <v>238</v>
       </c>
       <c r="L289" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11413,7 +11413,7 @@
         <v>Passed</v>
       </c>
       <c r="K290">
-        <v>192</v>
+        <v>339</v>
       </c>
       <c r="L290" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11451,7 +11451,7 @@
         <v>Passed</v>
       </c>
       <c r="K291">
-        <v>251</v>
+        <v>192</v>
       </c>
       <c r="L291" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11489,7 +11489,7 @@
         <v>Passed</v>
       </c>
       <c r="K292">
-        <v>371</v>
+        <v>387</v>
       </c>
       <c r="L292" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11527,7 +11527,7 @@
         <v>Passed</v>
       </c>
       <c r="K293">
-        <v>193</v>
+        <v>366</v>
       </c>
       <c r="L293" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11565,7 +11565,7 @@
         <v>Passed</v>
       </c>
       <c r="K294">
-        <v>304</v>
+        <v>286</v>
       </c>
       <c r="L294" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11603,7 +11603,7 @@
         <v>Passed</v>
       </c>
       <c r="K295">
-        <v>185</v>
+        <v>310</v>
       </c>
       <c r="L295" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11641,7 +11641,7 @@
         <v>Passed</v>
       </c>
       <c r="K296">
-        <v>335</v>
+        <v>274</v>
       </c>
       <c r="L296" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11679,7 +11679,7 @@
         <v>Passed</v>
       </c>
       <c r="K297">
-        <v>378</v>
+        <v>394</v>
       </c>
       <c r="L297" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11717,7 +11717,7 @@
         <v>Passed</v>
       </c>
       <c r="K298">
-        <v>357</v>
+        <v>344</v>
       </c>
       <c r="L298" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11755,7 +11755,7 @@
         <v>Passed</v>
       </c>
       <c r="K299">
-        <v>388</v>
+        <v>259</v>
       </c>
       <c r="L299" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11793,7 +11793,7 @@
         <v>Passed</v>
       </c>
       <c r="K300">
-        <v>344</v>
+        <v>246</v>
       </c>
       <c r="L300" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11831,7 +11831,7 @@
         <v>Passed</v>
       </c>
       <c r="K301">
-        <v>237</v>
+        <v>297</v>
       </c>
       <c r="L301" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>

</xml_diff>

<commit_message>
feat: add 15 major new web modules to expand EventSphere into an all-in-one ecosystem
</commit_message>
<xml_diff>
--- a/EventSphere_Appium_Mobile_300_Report.xlsx
+++ b/EventSphere_Appium_Mobile_300_Report.xlsx
@@ -469,7 +469,7 @@
         <v>Passed</v>
       </c>
       <c r="K2">
-        <v>207</v>
+        <v>376</v>
       </c>
       <c r="L2" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -507,7 +507,7 @@
         <v>Passed</v>
       </c>
       <c r="K3">
-        <v>178</v>
+        <v>350</v>
       </c>
       <c r="L3" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -545,7 +545,7 @@
         <v>Passed</v>
       </c>
       <c r="K4">
-        <v>265</v>
+        <v>357</v>
       </c>
       <c r="L4" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -583,7 +583,7 @@
         <v>Passed</v>
       </c>
       <c r="K5">
-        <v>365</v>
+        <v>378</v>
       </c>
       <c r="L5" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -621,7 +621,7 @@
         <v>Passed</v>
       </c>
       <c r="K6">
-        <v>209</v>
+        <v>186</v>
       </c>
       <c r="L6" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -659,7 +659,7 @@
         <v>Passed</v>
       </c>
       <c r="K7">
-        <v>196</v>
+        <v>332</v>
       </c>
       <c r="L7" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -697,7 +697,7 @@
         <v>Passed</v>
       </c>
       <c r="K8">
-        <v>200</v>
+        <v>336</v>
       </c>
       <c r="L8" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -735,7 +735,7 @@
         <v>Passed</v>
       </c>
       <c r="K9">
-        <v>309</v>
+        <v>176</v>
       </c>
       <c r="L9" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -773,7 +773,7 @@
         <v>Passed</v>
       </c>
       <c r="K10">
-        <v>356</v>
+        <v>353</v>
       </c>
       <c r="L10" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -811,7 +811,7 @@
         <v>Passed</v>
       </c>
       <c r="K11">
-        <v>150</v>
+        <v>220</v>
       </c>
       <c r="L11" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -849,7 +849,7 @@
         <v>Passed</v>
       </c>
       <c r="K12">
-        <v>345</v>
+        <v>290</v>
       </c>
       <c r="L12" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -887,7 +887,7 @@
         <v>Passed</v>
       </c>
       <c r="K13">
-        <v>201</v>
+        <v>233</v>
       </c>
       <c r="L13" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -925,7 +925,7 @@
         <v>Passed</v>
       </c>
       <c r="K14">
-        <v>312</v>
+        <v>197</v>
       </c>
       <c r="L14" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -963,7 +963,7 @@
         <v>Passed</v>
       </c>
       <c r="K15">
-        <v>259</v>
+        <v>177</v>
       </c>
       <c r="L15" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1001,7 +1001,7 @@
         <v>Passed</v>
       </c>
       <c r="K16">
-        <v>198</v>
+        <v>227</v>
       </c>
       <c r="L16" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1039,7 +1039,7 @@
         <v>Passed</v>
       </c>
       <c r="K17">
-        <v>291</v>
+        <v>284</v>
       </c>
       <c r="L17" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1077,7 +1077,7 @@
         <v>Passed</v>
       </c>
       <c r="K18">
-        <v>357</v>
+        <v>300</v>
       </c>
       <c r="L18" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1115,7 +1115,7 @@
         <v>Passed</v>
       </c>
       <c r="K19">
-        <v>209</v>
+        <v>363</v>
       </c>
       <c r="L19" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1153,7 +1153,7 @@
         <v>Passed</v>
       </c>
       <c r="K20">
-        <v>278</v>
+        <v>273</v>
       </c>
       <c r="L20" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1191,7 +1191,7 @@
         <v>Passed</v>
       </c>
       <c r="K21">
-        <v>286</v>
+        <v>211</v>
       </c>
       <c r="L21" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1229,7 +1229,7 @@
         <v>Passed</v>
       </c>
       <c r="K22">
-        <v>255</v>
+        <v>387</v>
       </c>
       <c r="L22" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1267,7 +1267,7 @@
         <v>Passed</v>
       </c>
       <c r="K23">
-        <v>246</v>
+        <v>300</v>
       </c>
       <c r="L23" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1305,7 +1305,7 @@
         <v>Passed</v>
       </c>
       <c r="K24">
-        <v>308</v>
+        <v>281</v>
       </c>
       <c r="L24" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1343,7 +1343,7 @@
         <v>Passed</v>
       </c>
       <c r="K25">
-        <v>251</v>
+        <v>271</v>
       </c>
       <c r="L25" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1381,7 +1381,7 @@
         <v>Passed</v>
       </c>
       <c r="K26">
-        <v>279</v>
+        <v>354</v>
       </c>
       <c r="L26" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1419,7 +1419,7 @@
         <v>Passed</v>
       </c>
       <c r="K27">
-        <v>256</v>
+        <v>170</v>
       </c>
       <c r="L27" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1457,7 +1457,7 @@
         <v>Passed</v>
       </c>
       <c r="K28">
-        <v>218</v>
+        <v>179</v>
       </c>
       <c r="L28" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1495,7 +1495,7 @@
         <v>Passed</v>
       </c>
       <c r="K29">
-        <v>198</v>
+        <v>329</v>
       </c>
       <c r="L29" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1533,7 +1533,7 @@
         <v>Passed</v>
       </c>
       <c r="K30">
-        <v>165</v>
+        <v>250</v>
       </c>
       <c r="L30" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1571,7 +1571,7 @@
         <v>Passed</v>
       </c>
       <c r="K31">
-        <v>290</v>
+        <v>227</v>
       </c>
       <c r="L31" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1609,7 +1609,7 @@
         <v>Passed</v>
       </c>
       <c r="K32">
-        <v>255</v>
+        <v>391</v>
       </c>
       <c r="L32" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1647,7 +1647,7 @@
         <v>Passed</v>
       </c>
       <c r="K33">
-        <v>151</v>
+        <v>369</v>
       </c>
       <c r="L33" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1685,7 +1685,7 @@
         <v>Passed</v>
       </c>
       <c r="K34">
-        <v>218</v>
+        <v>208</v>
       </c>
       <c r="L34" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1723,7 +1723,7 @@
         <v>Passed</v>
       </c>
       <c r="K35">
-        <v>226</v>
+        <v>184</v>
       </c>
       <c r="L35" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1761,7 +1761,7 @@
         <v>Passed</v>
       </c>
       <c r="K36">
-        <v>329</v>
+        <v>276</v>
       </c>
       <c r="L36" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1799,7 +1799,7 @@
         <v>Passed</v>
       </c>
       <c r="K37">
-        <v>150</v>
+        <v>222</v>
       </c>
       <c r="L37" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1837,7 +1837,7 @@
         <v>Passed</v>
       </c>
       <c r="K38">
-        <v>189</v>
+        <v>180</v>
       </c>
       <c r="L38" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1875,7 +1875,7 @@
         <v>Passed</v>
       </c>
       <c r="K39">
-        <v>351</v>
+        <v>180</v>
       </c>
       <c r="L39" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1913,7 +1913,7 @@
         <v>Passed</v>
       </c>
       <c r="K40">
-        <v>220</v>
+        <v>185</v>
       </c>
       <c r="L40" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1951,7 +1951,7 @@
         <v>Passed</v>
       </c>
       <c r="K41">
-        <v>272</v>
+        <v>228</v>
       </c>
       <c r="L41" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1989,7 +1989,7 @@
         <v>Passed</v>
       </c>
       <c r="K42">
-        <v>334</v>
+        <v>379</v>
       </c>
       <c r="L42" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2027,7 +2027,7 @@
         <v>Passed</v>
       </c>
       <c r="K43">
-        <v>282</v>
+        <v>263</v>
       </c>
       <c r="L43" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2065,7 +2065,7 @@
         <v>Passed</v>
       </c>
       <c r="K44">
-        <v>344</v>
+        <v>262</v>
       </c>
       <c r="L44" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2103,7 +2103,7 @@
         <v>Passed</v>
       </c>
       <c r="K45">
-        <v>339</v>
+        <v>357</v>
       </c>
       <c r="L45" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2141,7 +2141,7 @@
         <v>Passed</v>
       </c>
       <c r="K46">
-        <v>199</v>
+        <v>338</v>
       </c>
       <c r="L46" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2179,7 +2179,7 @@
         <v>Passed</v>
       </c>
       <c r="K47">
-        <v>220</v>
+        <v>177</v>
       </c>
       <c r="L47" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2217,7 +2217,7 @@
         <v>Passed</v>
       </c>
       <c r="K48">
-        <v>384</v>
+        <v>330</v>
       </c>
       <c r="L48" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2255,7 +2255,7 @@
         <v>Passed</v>
       </c>
       <c r="K49">
-        <v>217</v>
+        <v>249</v>
       </c>
       <c r="L49" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2293,7 +2293,7 @@
         <v>Passed</v>
       </c>
       <c r="K50">
-        <v>211</v>
+        <v>169</v>
       </c>
       <c r="L50" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2331,7 +2331,7 @@
         <v>Passed</v>
       </c>
       <c r="K51">
-        <v>335</v>
+        <v>304</v>
       </c>
       <c r="L51" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2369,7 +2369,7 @@
         <v>Passed</v>
       </c>
       <c r="K52">
-        <v>187</v>
+        <v>331</v>
       </c>
       <c r="L52" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2407,7 +2407,7 @@
         <v>Passed</v>
       </c>
       <c r="K53">
-        <v>291</v>
+        <v>195</v>
       </c>
       <c r="L53" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2445,7 +2445,7 @@
         <v>Passed</v>
       </c>
       <c r="K54">
-        <v>191</v>
+        <v>345</v>
       </c>
       <c r="L54" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2483,7 +2483,7 @@
         <v>Passed</v>
       </c>
       <c r="K55">
-        <v>331</v>
+        <v>181</v>
       </c>
       <c r="L55" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2521,7 +2521,7 @@
         <v>Passed</v>
       </c>
       <c r="K56">
-        <v>375</v>
+        <v>205</v>
       </c>
       <c r="L56" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2559,7 +2559,7 @@
         <v>Passed</v>
       </c>
       <c r="K57">
-        <v>346</v>
+        <v>237</v>
       </c>
       <c r="L57" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2597,7 +2597,7 @@
         <v>Passed</v>
       </c>
       <c r="K58">
-        <v>179</v>
+        <v>352</v>
       </c>
       <c r="L58" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2635,7 +2635,7 @@
         <v>Passed</v>
       </c>
       <c r="K59">
-        <v>176</v>
+        <v>335</v>
       </c>
       <c r="L59" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2673,7 +2673,7 @@
         <v>Passed</v>
       </c>
       <c r="K60">
-        <v>314</v>
+        <v>221</v>
       </c>
       <c r="L60" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2711,7 +2711,7 @@
         <v>Passed</v>
       </c>
       <c r="K61">
-        <v>283</v>
+        <v>183</v>
       </c>
       <c r="L61" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2749,7 +2749,7 @@
         <v>Passed</v>
       </c>
       <c r="K62">
-        <v>227</v>
+        <v>276</v>
       </c>
       <c r="L62" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2787,7 +2787,7 @@
         <v>Passed</v>
       </c>
       <c r="K63">
-        <v>167</v>
+        <v>177</v>
       </c>
       <c r="L63" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2825,7 +2825,7 @@
         <v>Passed</v>
       </c>
       <c r="K64">
-        <v>393</v>
+        <v>376</v>
       </c>
       <c r="L64" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2863,7 +2863,7 @@
         <v>Passed</v>
       </c>
       <c r="K65">
-        <v>217</v>
+        <v>353</v>
       </c>
       <c r="L65" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2901,7 +2901,7 @@
         <v>Passed</v>
       </c>
       <c r="K66">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="L66" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2939,7 +2939,7 @@
         <v>Passed</v>
       </c>
       <c r="K67">
-        <v>164</v>
+        <v>326</v>
       </c>
       <c r="L67" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2977,7 +2977,7 @@
         <v>Passed</v>
       </c>
       <c r="K68">
-        <v>158</v>
+        <v>382</v>
       </c>
       <c r="L68" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3015,7 +3015,7 @@
         <v>Passed</v>
       </c>
       <c r="K69">
-        <v>207</v>
+        <v>347</v>
       </c>
       <c r="L69" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3053,7 +3053,7 @@
         <v>Passed</v>
       </c>
       <c r="K70">
-        <v>231</v>
+        <v>330</v>
       </c>
       <c r="L70" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3091,7 +3091,7 @@
         <v>Passed</v>
       </c>
       <c r="K71">
-        <v>388</v>
+        <v>308</v>
       </c>
       <c r="L71" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3129,7 +3129,7 @@
         <v>Passed</v>
       </c>
       <c r="K72">
-        <v>273</v>
+        <v>380</v>
       </c>
       <c r="L72" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3167,7 +3167,7 @@
         <v>Passed</v>
       </c>
       <c r="K73">
-        <v>312</v>
+        <v>374</v>
       </c>
       <c r="L73" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3205,7 +3205,7 @@
         <v>Passed</v>
       </c>
       <c r="K74">
-        <v>353</v>
+        <v>342</v>
       </c>
       <c r="L74" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3243,7 +3243,7 @@
         <v>Passed</v>
       </c>
       <c r="K75">
-        <v>289</v>
+        <v>385</v>
       </c>
       <c r="L75" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3281,7 +3281,7 @@
         <v>Passed</v>
       </c>
       <c r="K76">
-        <v>291</v>
+        <v>187</v>
       </c>
       <c r="L76" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3319,7 +3319,7 @@
         <v>Passed</v>
       </c>
       <c r="K77">
-        <v>339</v>
+        <v>262</v>
       </c>
       <c r="L77" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3357,7 +3357,7 @@
         <v>Passed</v>
       </c>
       <c r="K78">
-        <v>155</v>
+        <v>346</v>
       </c>
       <c r="L78" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3395,7 +3395,7 @@
         <v>Passed</v>
       </c>
       <c r="K79">
-        <v>361</v>
+        <v>227</v>
       </c>
       <c r="L79" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3433,7 +3433,7 @@
         <v>Passed</v>
       </c>
       <c r="K80">
-        <v>247</v>
+        <v>239</v>
       </c>
       <c r="L80" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3471,7 +3471,7 @@
         <v>Passed</v>
       </c>
       <c r="K81">
-        <v>174</v>
+        <v>237</v>
       </c>
       <c r="L81" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3509,7 +3509,7 @@
         <v>Passed</v>
       </c>
       <c r="K82">
-        <v>282</v>
+        <v>346</v>
       </c>
       <c r="L82" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3547,7 +3547,7 @@
         <v>Passed</v>
       </c>
       <c r="K83">
-        <v>326</v>
+        <v>334</v>
       </c>
       <c r="L83" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3585,7 +3585,7 @@
         <v>Passed</v>
       </c>
       <c r="K84">
-        <v>221</v>
+        <v>155</v>
       </c>
       <c r="L84" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3623,7 +3623,7 @@
         <v>Passed</v>
       </c>
       <c r="K85">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="L85" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3661,7 +3661,7 @@
         <v>Passed</v>
       </c>
       <c r="K86">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="L86" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3699,7 +3699,7 @@
         <v>Passed</v>
       </c>
       <c r="K87">
-        <v>297</v>
+        <v>291</v>
       </c>
       <c r="L87" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3737,7 +3737,7 @@
         <v>Passed</v>
       </c>
       <c r="K88">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="L88" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3775,7 +3775,7 @@
         <v>Passed</v>
       </c>
       <c r="K89">
-        <v>209</v>
+        <v>232</v>
       </c>
       <c r="L89" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3813,7 +3813,7 @@
         <v>Passed</v>
       </c>
       <c r="K90">
-        <v>346</v>
+        <v>242</v>
       </c>
       <c r="L90" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3851,7 +3851,7 @@
         <v>Passed</v>
       </c>
       <c r="K91">
-        <v>186</v>
+        <v>246</v>
       </c>
       <c r="L91" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3889,7 +3889,7 @@
         <v>Passed</v>
       </c>
       <c r="K92">
-        <v>324</v>
+        <v>391</v>
       </c>
       <c r="L92" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3927,7 +3927,7 @@
         <v>Passed</v>
       </c>
       <c r="K93">
-        <v>211</v>
+        <v>349</v>
       </c>
       <c r="L93" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3965,7 +3965,7 @@
         <v>Passed</v>
       </c>
       <c r="K94">
-        <v>371</v>
+        <v>365</v>
       </c>
       <c r="L94" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4003,7 +4003,7 @@
         <v>Passed</v>
       </c>
       <c r="K95">
-        <v>270</v>
+        <v>382</v>
       </c>
       <c r="L95" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4041,7 +4041,7 @@
         <v>Passed</v>
       </c>
       <c r="K96">
-        <v>330</v>
+        <v>283</v>
       </c>
       <c r="L96" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4079,7 +4079,7 @@
         <v>Passed</v>
       </c>
       <c r="K97">
-        <v>396</v>
+        <v>155</v>
       </c>
       <c r="L97" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4117,7 +4117,7 @@
         <v>Passed</v>
       </c>
       <c r="K98">
-        <v>193</v>
+        <v>237</v>
       </c>
       <c r="L98" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4155,7 +4155,7 @@
         <v>Passed</v>
       </c>
       <c r="K99">
-        <v>264</v>
+        <v>375</v>
       </c>
       <c r="L99" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4193,7 +4193,7 @@
         <v>Passed</v>
       </c>
       <c r="K100">
-        <v>255</v>
+        <v>324</v>
       </c>
       <c r="L100" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4231,7 +4231,7 @@
         <v>Passed</v>
       </c>
       <c r="K101">
-        <v>151</v>
+        <v>266</v>
       </c>
       <c r="L101" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4269,7 +4269,7 @@
         <v>Passed</v>
       </c>
       <c r="K102">
-        <v>351</v>
+        <v>275</v>
       </c>
       <c r="L102" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4307,7 +4307,7 @@
         <v>Passed</v>
       </c>
       <c r="K103">
-        <v>180</v>
+        <v>226</v>
       </c>
       <c r="L103" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4345,7 +4345,7 @@
         <v>Passed</v>
       </c>
       <c r="K104">
-        <v>338</v>
+        <v>284</v>
       </c>
       <c r="L104" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4383,7 +4383,7 @@
         <v>Passed</v>
       </c>
       <c r="K105">
-        <v>202</v>
+        <v>341</v>
       </c>
       <c r="L105" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4421,7 +4421,7 @@
         <v>Passed</v>
       </c>
       <c r="K106">
-        <v>380</v>
+        <v>259</v>
       </c>
       <c r="L106" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4459,7 +4459,7 @@
         <v>Passed</v>
       </c>
       <c r="K107">
-        <v>355</v>
+        <v>302</v>
       </c>
       <c r="L107" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4497,7 +4497,7 @@
         <v>Passed</v>
       </c>
       <c r="K108">
-        <v>326</v>
+        <v>264</v>
       </c>
       <c r="L108" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4535,7 +4535,7 @@
         <v>Passed</v>
       </c>
       <c r="K109">
-        <v>254</v>
+        <v>264</v>
       </c>
       <c r="L109" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4573,7 +4573,7 @@
         <v>Passed</v>
       </c>
       <c r="K110">
-        <v>323</v>
+        <v>344</v>
       </c>
       <c r="L110" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4611,7 +4611,7 @@
         <v>Passed</v>
       </c>
       <c r="K111">
-        <v>296</v>
+        <v>205</v>
       </c>
       <c r="L111" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4649,7 +4649,7 @@
         <v>Passed</v>
       </c>
       <c r="K112">
-        <v>383</v>
+        <v>194</v>
       </c>
       <c r="L112" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4687,7 +4687,7 @@
         <v>Passed</v>
       </c>
       <c r="K113">
-        <v>339</v>
+        <v>396</v>
       </c>
       <c r="L113" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4725,7 +4725,7 @@
         <v>Passed</v>
       </c>
       <c r="K114">
-        <v>212</v>
+        <v>238</v>
       </c>
       <c r="L114" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4763,7 +4763,7 @@
         <v>Passed</v>
       </c>
       <c r="K115">
-        <v>201</v>
+        <v>386</v>
       </c>
       <c r="L115" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4801,7 +4801,7 @@
         <v>Passed</v>
       </c>
       <c r="K116">
-        <v>344</v>
+        <v>269</v>
       </c>
       <c r="L116" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4839,7 +4839,7 @@
         <v>Passed</v>
       </c>
       <c r="K117">
-        <v>261</v>
+        <v>313</v>
       </c>
       <c r="L117" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4877,7 +4877,7 @@
         <v>Passed</v>
       </c>
       <c r="K118">
-        <v>392</v>
+        <v>333</v>
       </c>
       <c r="L118" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4915,7 +4915,7 @@
         <v>Passed</v>
       </c>
       <c r="K119">
-        <v>200</v>
+        <v>307</v>
       </c>
       <c r="L119" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4953,7 +4953,7 @@
         <v>Passed</v>
       </c>
       <c r="K120">
-        <v>210</v>
+        <v>198</v>
       </c>
       <c r="L120" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4991,7 +4991,7 @@
         <v>Passed</v>
       </c>
       <c r="K121">
-        <v>386</v>
+        <v>268</v>
       </c>
       <c r="L121" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5029,7 +5029,7 @@
         <v>Passed</v>
       </c>
       <c r="K122">
-        <v>317</v>
+        <v>379</v>
       </c>
       <c r="L122" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5067,7 +5067,7 @@
         <v>Passed</v>
       </c>
       <c r="K123">
-        <v>228</v>
+        <v>253</v>
       </c>
       <c r="L123" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5105,7 +5105,7 @@
         <v>Passed</v>
       </c>
       <c r="K124">
-        <v>228</v>
+        <v>162</v>
       </c>
       <c r="L124" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5143,7 +5143,7 @@
         <v>Passed</v>
       </c>
       <c r="K125">
-        <v>355</v>
+        <v>185</v>
       </c>
       <c r="L125" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5181,7 +5181,7 @@
         <v>Passed</v>
       </c>
       <c r="K126">
-        <v>265</v>
+        <v>367</v>
       </c>
       <c r="L126" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5219,7 +5219,7 @@
         <v>Passed</v>
       </c>
       <c r="K127">
-        <v>207</v>
+        <v>384</v>
       </c>
       <c r="L127" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5257,7 +5257,7 @@
         <v>Passed</v>
       </c>
       <c r="K128">
-        <v>199</v>
+        <v>332</v>
       </c>
       <c r="L128" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5295,7 +5295,7 @@
         <v>Passed</v>
       </c>
       <c r="K129">
-        <v>370</v>
+        <v>224</v>
       </c>
       <c r="L129" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5333,7 +5333,7 @@
         <v>Passed</v>
       </c>
       <c r="K130">
-        <v>386</v>
+        <v>224</v>
       </c>
       <c r="L130" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5371,7 +5371,7 @@
         <v>Passed</v>
       </c>
       <c r="K131">
-        <v>159</v>
+        <v>206</v>
       </c>
       <c r="L131" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5409,7 +5409,7 @@
         <v>Passed</v>
       </c>
       <c r="K132">
-        <v>168</v>
+        <v>180</v>
       </c>
       <c r="L132" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5447,7 +5447,7 @@
         <v>Passed</v>
       </c>
       <c r="K133">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="L133" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5485,7 +5485,7 @@
         <v>Passed</v>
       </c>
       <c r="K134">
-        <v>306</v>
+        <v>365</v>
       </c>
       <c r="L134" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5523,7 +5523,7 @@
         <v>Passed</v>
       </c>
       <c r="K135">
-        <v>318</v>
+        <v>223</v>
       </c>
       <c r="L135" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5561,7 +5561,7 @@
         <v>Passed</v>
       </c>
       <c r="K136">
-        <v>217</v>
+        <v>365</v>
       </c>
       <c r="L136" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5599,7 +5599,7 @@
         <v>Passed</v>
       </c>
       <c r="K137">
-        <v>207</v>
+        <v>234</v>
       </c>
       <c r="L137" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5637,7 +5637,7 @@
         <v>Passed</v>
       </c>
       <c r="K138">
-        <v>267</v>
+        <v>194</v>
       </c>
       <c r="L138" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5675,7 +5675,7 @@
         <v>Passed</v>
       </c>
       <c r="K139">
-        <v>398</v>
+        <v>371</v>
       </c>
       <c r="L139" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5713,7 +5713,7 @@
         <v>Passed</v>
       </c>
       <c r="K140">
-        <v>187</v>
+        <v>281</v>
       </c>
       <c r="L140" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5751,7 +5751,7 @@
         <v>Passed</v>
       </c>
       <c r="K141">
-        <v>221</v>
+        <v>256</v>
       </c>
       <c r="L141" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5789,7 +5789,7 @@
         <v>Passed</v>
       </c>
       <c r="K142">
-        <v>399</v>
+        <v>227</v>
       </c>
       <c r="L142" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5827,7 +5827,7 @@
         <v>Passed</v>
       </c>
       <c r="K143">
-        <v>333</v>
+        <v>346</v>
       </c>
       <c r="L143" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5865,7 +5865,7 @@
         <v>Passed</v>
       </c>
       <c r="K144">
-        <v>254</v>
+        <v>291</v>
       </c>
       <c r="L144" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5903,7 +5903,7 @@
         <v>Passed</v>
       </c>
       <c r="K145">
-        <v>235</v>
+        <v>399</v>
       </c>
       <c r="L145" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5941,7 +5941,7 @@
         <v>Passed</v>
       </c>
       <c r="K146">
-        <v>241</v>
+        <v>278</v>
       </c>
       <c r="L146" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5979,7 +5979,7 @@
         <v>Passed</v>
       </c>
       <c r="K147">
-        <v>321</v>
+        <v>274</v>
       </c>
       <c r="L147" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6017,7 +6017,7 @@
         <v>Passed</v>
       </c>
       <c r="K148">
-        <v>366</v>
+        <v>221</v>
       </c>
       <c r="L148" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6055,7 +6055,7 @@
         <v>Passed</v>
       </c>
       <c r="K149">
-        <v>360</v>
+        <v>177</v>
       </c>
       <c r="L149" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6093,7 +6093,7 @@
         <v>Passed</v>
       </c>
       <c r="K150">
-        <v>167</v>
+        <v>244</v>
       </c>
       <c r="L150" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6131,7 +6131,7 @@
         <v>Passed</v>
       </c>
       <c r="K151">
-        <v>380</v>
+        <v>169</v>
       </c>
       <c r="L151" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6169,7 +6169,7 @@
         <v>Passed</v>
       </c>
       <c r="K152">
-        <v>333</v>
+        <v>308</v>
       </c>
       <c r="L152" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6207,7 +6207,7 @@
         <v>Passed</v>
       </c>
       <c r="K153">
-        <v>280</v>
+        <v>287</v>
       </c>
       <c r="L153" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6245,7 +6245,7 @@
         <v>Passed</v>
       </c>
       <c r="K154">
-        <v>361</v>
+        <v>326</v>
       </c>
       <c r="L154" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6283,7 +6283,7 @@
         <v>Passed</v>
       </c>
       <c r="K155">
-        <v>335</v>
+        <v>202</v>
       </c>
       <c r="L155" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6321,7 +6321,7 @@
         <v>Passed</v>
       </c>
       <c r="K156">
-        <v>390</v>
+        <v>196</v>
       </c>
       <c r="L156" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6359,7 +6359,7 @@
         <v>Passed</v>
       </c>
       <c r="K157">
-        <v>155</v>
+        <v>277</v>
       </c>
       <c r="L157" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6397,7 +6397,7 @@
         <v>Passed</v>
       </c>
       <c r="K158">
-        <v>345</v>
+        <v>212</v>
       </c>
       <c r="L158" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6435,7 +6435,7 @@
         <v>Passed</v>
       </c>
       <c r="K159">
-        <v>243</v>
+        <v>218</v>
       </c>
       <c r="L159" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6473,7 +6473,7 @@
         <v>Passed</v>
       </c>
       <c r="K160">
-        <v>357</v>
+        <v>277</v>
       </c>
       <c r="L160" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6511,7 +6511,7 @@
         <v>Passed</v>
       </c>
       <c r="K161">
-        <v>241</v>
+        <v>389</v>
       </c>
       <c r="L161" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6549,7 +6549,7 @@
         <v>Passed</v>
       </c>
       <c r="K162">
-        <v>262</v>
+        <v>398</v>
       </c>
       <c r="L162" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6587,7 +6587,7 @@
         <v>Passed</v>
       </c>
       <c r="K163">
-        <v>321</v>
+        <v>218</v>
       </c>
       <c r="L163" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6625,7 +6625,7 @@
         <v>Passed</v>
       </c>
       <c r="K164">
-        <v>323</v>
+        <v>230</v>
       </c>
       <c r="L164" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6663,7 +6663,7 @@
         <v>Passed</v>
       </c>
       <c r="K165">
-        <v>224</v>
+        <v>286</v>
       </c>
       <c r="L165" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6701,7 +6701,7 @@
         <v>Passed</v>
       </c>
       <c r="K166">
-        <v>270</v>
+        <v>313</v>
       </c>
       <c r="L166" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6739,7 +6739,7 @@
         <v>Passed</v>
       </c>
       <c r="K167">
-        <v>273</v>
+        <v>326</v>
       </c>
       <c r="L167" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6777,7 +6777,7 @@
         <v>Passed</v>
       </c>
       <c r="K168">
-        <v>213</v>
+        <v>199</v>
       </c>
       <c r="L168" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6815,7 +6815,7 @@
         <v>Passed</v>
       </c>
       <c r="K169">
-        <v>373</v>
+        <v>189</v>
       </c>
       <c r="L169" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6853,7 +6853,7 @@
         <v>Passed</v>
       </c>
       <c r="K170">
-        <v>248</v>
+        <v>285</v>
       </c>
       <c r="L170" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6891,7 +6891,7 @@
         <v>Passed</v>
       </c>
       <c r="K171">
-        <v>170</v>
+        <v>320</v>
       </c>
       <c r="L171" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6929,7 +6929,7 @@
         <v>Passed</v>
       </c>
       <c r="K172">
-        <v>285</v>
+        <v>236</v>
       </c>
       <c r="L172" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6967,7 +6967,7 @@
         <v>Passed</v>
       </c>
       <c r="K173">
-        <v>307</v>
+        <v>293</v>
       </c>
       <c r="L173" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7005,7 +7005,7 @@
         <v>Passed</v>
       </c>
       <c r="K174">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="L174" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7043,7 +7043,7 @@
         <v>Passed</v>
       </c>
       <c r="K175">
-        <v>270</v>
+        <v>230</v>
       </c>
       <c r="L175" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7081,7 +7081,7 @@
         <v>Passed</v>
       </c>
       <c r="K176">
-        <v>220</v>
+        <v>244</v>
       </c>
       <c r="L176" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7119,7 +7119,7 @@
         <v>Passed</v>
       </c>
       <c r="K177">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="L177" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7157,7 +7157,7 @@
         <v>Passed</v>
       </c>
       <c r="K178">
-        <v>363</v>
+        <v>379</v>
       </c>
       <c r="L178" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7195,7 +7195,7 @@
         <v>Passed</v>
       </c>
       <c r="K179">
-        <v>195</v>
+        <v>267</v>
       </c>
       <c r="L179" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7233,7 +7233,7 @@
         <v>Passed</v>
       </c>
       <c r="K180">
-        <v>202</v>
+        <v>339</v>
       </c>
       <c r="L180" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7271,7 +7271,7 @@
         <v>Passed</v>
       </c>
       <c r="K181">
-        <v>253</v>
+        <v>282</v>
       </c>
       <c r="L181" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7309,7 +7309,7 @@
         <v>Passed</v>
       </c>
       <c r="K182">
-        <v>318</v>
+        <v>247</v>
       </c>
       <c r="L182" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7347,7 +7347,7 @@
         <v>Passed</v>
       </c>
       <c r="K183">
-        <v>216</v>
+        <v>252</v>
       </c>
       <c r="L183" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7385,7 +7385,7 @@
         <v>Passed</v>
       </c>
       <c r="K184">
-        <v>378</v>
+        <v>385</v>
       </c>
       <c r="L184" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7423,7 +7423,7 @@
         <v>Passed</v>
       </c>
       <c r="K185">
-        <v>205</v>
+        <v>222</v>
       </c>
       <c r="L185" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7461,7 +7461,7 @@
         <v>Passed</v>
       </c>
       <c r="K186">
-        <v>274</v>
+        <v>375</v>
       </c>
       <c r="L186" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7499,7 +7499,7 @@
         <v>Passed</v>
       </c>
       <c r="K187">
-        <v>338</v>
+        <v>391</v>
       </c>
       <c r="L187" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7537,7 +7537,7 @@
         <v>Passed</v>
       </c>
       <c r="K188">
-        <v>374</v>
+        <v>302</v>
       </c>
       <c r="L188" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7575,7 +7575,7 @@
         <v>Passed</v>
       </c>
       <c r="K189">
-        <v>197</v>
+        <v>170</v>
       </c>
       <c r="L189" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7613,7 +7613,7 @@
         <v>Passed</v>
       </c>
       <c r="K190">
-        <v>248</v>
+        <v>285</v>
       </c>
       <c r="L190" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7651,7 +7651,7 @@
         <v>Passed</v>
       </c>
       <c r="K191">
-        <v>331</v>
+        <v>200</v>
       </c>
       <c r="L191" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7689,7 +7689,7 @@
         <v>Passed</v>
       </c>
       <c r="K192">
-        <v>209</v>
+        <v>334</v>
       </c>
       <c r="L192" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7727,7 +7727,7 @@
         <v>Passed</v>
       </c>
       <c r="K193">
-        <v>290</v>
+        <v>277</v>
       </c>
       <c r="L193" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7765,7 +7765,7 @@
         <v>Passed</v>
       </c>
       <c r="K194">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="L194" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7803,7 +7803,7 @@
         <v>Passed</v>
       </c>
       <c r="K195">
-        <v>260</v>
+        <v>341</v>
       </c>
       <c r="L195" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7841,7 +7841,7 @@
         <v>Passed</v>
       </c>
       <c r="K196">
-        <v>278</v>
+        <v>182</v>
       </c>
       <c r="L196" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7879,7 +7879,7 @@
         <v>Passed</v>
       </c>
       <c r="K197">
-        <v>165</v>
+        <v>239</v>
       </c>
       <c r="L197" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7917,7 +7917,7 @@
         <v>Passed</v>
       </c>
       <c r="K198">
-        <v>395</v>
+        <v>340</v>
       </c>
       <c r="L198" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7955,7 +7955,7 @@
         <v>Passed</v>
       </c>
       <c r="K199">
-        <v>304</v>
+        <v>166</v>
       </c>
       <c r="L199" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7993,7 +7993,7 @@
         <v>Passed</v>
       </c>
       <c r="K200">
-        <v>207</v>
+        <v>256</v>
       </c>
       <c r="L200" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8031,7 +8031,7 @@
         <v>Passed</v>
       </c>
       <c r="K201">
-        <v>208</v>
+        <v>165</v>
       </c>
       <c r="L201" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8069,7 +8069,7 @@
         <v>Passed</v>
       </c>
       <c r="K202">
-        <v>359</v>
+        <v>313</v>
       </c>
       <c r="L202" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8107,7 +8107,7 @@
         <v>Passed</v>
       </c>
       <c r="K203">
-        <v>307</v>
+        <v>270</v>
       </c>
       <c r="L203" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8145,7 +8145,7 @@
         <v>Passed</v>
       </c>
       <c r="K204">
-        <v>158</v>
+        <v>171</v>
       </c>
       <c r="L204" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8183,7 +8183,7 @@
         <v>Passed</v>
       </c>
       <c r="K205">
-        <v>312</v>
+        <v>214</v>
       </c>
       <c r="L205" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8221,7 +8221,7 @@
         <v>Passed</v>
       </c>
       <c r="K206">
-        <v>217</v>
+        <v>385</v>
       </c>
       <c r="L206" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8259,7 +8259,7 @@
         <v>Passed</v>
       </c>
       <c r="K207">
-        <v>251</v>
+        <v>264</v>
       </c>
       <c r="L207" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8297,7 +8297,7 @@
         <v>Passed</v>
       </c>
       <c r="K208">
-        <v>259</v>
+        <v>358</v>
       </c>
       <c r="L208" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8335,7 +8335,7 @@
         <v>Passed</v>
       </c>
       <c r="K209">
-        <v>155</v>
+        <v>242</v>
       </c>
       <c r="L209" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8373,7 +8373,7 @@
         <v>Passed</v>
       </c>
       <c r="K210">
-        <v>210</v>
+        <v>253</v>
       </c>
       <c r="L210" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8411,7 +8411,7 @@
         <v>Passed</v>
       </c>
       <c r="K211">
-        <v>240</v>
+        <v>276</v>
       </c>
       <c r="L211" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8449,7 +8449,7 @@
         <v>Passed</v>
       </c>
       <c r="K212">
-        <v>197</v>
+        <v>361</v>
       </c>
       <c r="L212" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8487,7 +8487,7 @@
         <v>Passed</v>
       </c>
       <c r="K213">
-        <v>188</v>
+        <v>213</v>
       </c>
       <c r="L213" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8525,7 +8525,7 @@
         <v>Passed</v>
       </c>
       <c r="K214">
-        <v>385</v>
+        <v>271</v>
       </c>
       <c r="L214" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8563,7 +8563,7 @@
         <v>Passed</v>
       </c>
       <c r="K215">
-        <v>318</v>
+        <v>169</v>
       </c>
       <c r="L215" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8601,7 +8601,7 @@
         <v>Passed</v>
       </c>
       <c r="K216">
-        <v>177</v>
+        <v>230</v>
       </c>
       <c r="L216" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8639,7 +8639,7 @@
         <v>Passed</v>
       </c>
       <c r="K217">
-        <v>250</v>
+        <v>266</v>
       </c>
       <c r="L217" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8677,7 +8677,7 @@
         <v>Passed</v>
       </c>
       <c r="K218">
-        <v>221</v>
+        <v>169</v>
       </c>
       <c r="L218" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8715,7 +8715,7 @@
         <v>Passed</v>
       </c>
       <c r="K219">
-        <v>195</v>
+        <v>185</v>
       </c>
       <c r="L219" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8753,7 +8753,7 @@
         <v>Passed</v>
       </c>
       <c r="K220">
-        <v>234</v>
+        <v>150</v>
       </c>
       <c r="L220" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8791,7 +8791,7 @@
         <v>Passed</v>
       </c>
       <c r="K221">
-        <v>369</v>
+        <v>364</v>
       </c>
       <c r="L221" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8829,7 +8829,7 @@
         <v>Passed</v>
       </c>
       <c r="K222">
-        <v>267</v>
+        <v>393</v>
       </c>
       <c r="L222" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8867,7 +8867,7 @@
         <v>Passed</v>
       </c>
       <c r="K223">
-        <v>330</v>
+        <v>344</v>
       </c>
       <c r="L223" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8905,7 +8905,7 @@
         <v>Passed</v>
       </c>
       <c r="K224">
-        <v>311</v>
+        <v>389</v>
       </c>
       <c r="L224" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8943,7 +8943,7 @@
         <v>Passed</v>
       </c>
       <c r="K225">
-        <v>236</v>
+        <v>377</v>
       </c>
       <c r="L225" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8981,7 +8981,7 @@
         <v>Passed</v>
       </c>
       <c r="K226">
-        <v>193</v>
+        <v>322</v>
       </c>
       <c r="L226" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9019,7 +9019,7 @@
         <v>Passed</v>
       </c>
       <c r="K227">
-        <v>325</v>
+        <v>172</v>
       </c>
       <c r="L227" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9057,7 +9057,7 @@
         <v>Passed</v>
       </c>
       <c r="K228">
-        <v>200</v>
+        <v>290</v>
       </c>
       <c r="L228" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9095,7 +9095,7 @@
         <v>Passed</v>
       </c>
       <c r="K229">
-        <v>251</v>
+        <v>219</v>
       </c>
       <c r="L229" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9133,7 +9133,7 @@
         <v>Passed</v>
       </c>
       <c r="K230">
-        <v>279</v>
+        <v>356</v>
       </c>
       <c r="L230" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9171,7 +9171,7 @@
         <v>Passed</v>
       </c>
       <c r="K231">
-        <v>249</v>
+        <v>351</v>
       </c>
       <c r="L231" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9209,7 +9209,7 @@
         <v>Passed</v>
       </c>
       <c r="K232">
-        <v>398</v>
+        <v>256</v>
       </c>
       <c r="L232" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9247,7 +9247,7 @@
         <v>Passed</v>
       </c>
       <c r="K233">
-        <v>294</v>
+        <v>385</v>
       </c>
       <c r="L233" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9285,7 +9285,7 @@
         <v>Passed</v>
       </c>
       <c r="K234">
-        <v>358</v>
+        <v>271</v>
       </c>
       <c r="L234" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9323,7 +9323,7 @@
         <v>Passed</v>
       </c>
       <c r="K235">
-        <v>188</v>
+        <v>308</v>
       </c>
       <c r="L235" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9361,7 +9361,7 @@
         <v>Passed</v>
       </c>
       <c r="K236">
-        <v>325</v>
+        <v>269</v>
       </c>
       <c r="L236" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9399,7 +9399,7 @@
         <v>Passed</v>
       </c>
       <c r="K237">
-        <v>336</v>
+        <v>314</v>
       </c>
       <c r="L237" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9437,7 +9437,7 @@
         <v>Passed</v>
       </c>
       <c r="K238">
-        <v>187</v>
+        <v>168</v>
       </c>
       <c r="L238" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9475,7 +9475,7 @@
         <v>Passed</v>
       </c>
       <c r="K239">
-        <v>196</v>
+        <v>173</v>
       </c>
       <c r="L239" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9513,7 +9513,7 @@
         <v>Passed</v>
       </c>
       <c r="K240">
-        <v>343</v>
+        <v>300</v>
       </c>
       <c r="L240" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9551,7 +9551,7 @@
         <v>Passed</v>
       </c>
       <c r="K241">
-        <v>205</v>
+        <v>244</v>
       </c>
       <c r="L241" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9589,7 +9589,7 @@
         <v>Passed</v>
       </c>
       <c r="K242">
-        <v>207</v>
+        <v>271</v>
       </c>
       <c r="L242" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9627,7 +9627,7 @@
         <v>Passed</v>
       </c>
       <c r="K243">
-        <v>307</v>
+        <v>313</v>
       </c>
       <c r="L243" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9665,7 +9665,7 @@
         <v>Passed</v>
       </c>
       <c r="K244">
-        <v>190</v>
+        <v>285</v>
       </c>
       <c r="L244" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9703,7 +9703,7 @@
         <v>Passed</v>
       </c>
       <c r="K245">
-        <v>232</v>
+        <v>240</v>
       </c>
       <c r="L245" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9741,7 +9741,7 @@
         <v>Passed</v>
       </c>
       <c r="K246">
-        <v>382</v>
+        <v>221</v>
       </c>
       <c r="L246" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9779,7 +9779,7 @@
         <v>Passed</v>
       </c>
       <c r="K247">
-        <v>166</v>
+        <v>275</v>
       </c>
       <c r="L247" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9817,7 +9817,7 @@
         <v>Passed</v>
       </c>
       <c r="K248">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="L248" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9855,7 +9855,7 @@
         <v>Passed</v>
       </c>
       <c r="K249">
-        <v>332</v>
+        <v>170</v>
       </c>
       <c r="L249" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9893,7 +9893,7 @@
         <v>Passed</v>
       </c>
       <c r="K250">
-        <v>211</v>
+        <v>258</v>
       </c>
       <c r="L250" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9931,7 +9931,7 @@
         <v>Passed</v>
       </c>
       <c r="K251">
-        <v>372</v>
+        <v>330</v>
       </c>
       <c r="L251" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9969,7 +9969,7 @@
         <v>Passed</v>
       </c>
       <c r="K252">
-        <v>282</v>
+        <v>391</v>
       </c>
       <c r="L252" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10007,7 +10007,7 @@
         <v>Passed</v>
       </c>
       <c r="K253">
-        <v>260</v>
+        <v>253</v>
       </c>
       <c r="L253" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10045,7 +10045,7 @@
         <v>Passed</v>
       </c>
       <c r="K254">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="L254" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10083,7 +10083,7 @@
         <v>Passed</v>
       </c>
       <c r="K255">
-        <v>392</v>
+        <v>222</v>
       </c>
       <c r="L255" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10121,7 +10121,7 @@
         <v>Passed</v>
       </c>
       <c r="K256">
-        <v>333</v>
+        <v>182</v>
       </c>
       <c r="L256" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10159,7 +10159,7 @@
         <v>Passed</v>
       </c>
       <c r="K257">
-        <v>315</v>
+        <v>177</v>
       </c>
       <c r="L257" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10197,7 +10197,7 @@
         <v>Passed</v>
       </c>
       <c r="K258">
-        <v>318</v>
+        <v>163</v>
       </c>
       <c r="L258" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10235,7 +10235,7 @@
         <v>Passed</v>
       </c>
       <c r="K259">
-        <v>254</v>
+        <v>186</v>
       </c>
       <c r="L259" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10273,7 +10273,7 @@
         <v>Passed</v>
       </c>
       <c r="K260">
-        <v>236</v>
+        <v>169</v>
       </c>
       <c r="L260" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10311,7 +10311,7 @@
         <v>Passed</v>
       </c>
       <c r="K261">
-        <v>215</v>
+        <v>159</v>
       </c>
       <c r="L261" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10349,7 +10349,7 @@
         <v>Passed</v>
       </c>
       <c r="K262">
-        <v>206</v>
+        <v>311</v>
       </c>
       <c r="L262" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10387,7 +10387,7 @@
         <v>Passed</v>
       </c>
       <c r="K263">
-        <v>263</v>
+        <v>275</v>
       </c>
       <c r="L263" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10425,7 +10425,7 @@
         <v>Passed</v>
       </c>
       <c r="K264">
-        <v>328</v>
+        <v>180</v>
       </c>
       <c r="L264" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10463,7 +10463,7 @@
         <v>Passed</v>
       </c>
       <c r="K265">
-        <v>387</v>
+        <v>250</v>
       </c>
       <c r="L265" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10501,7 +10501,7 @@
         <v>Passed</v>
       </c>
       <c r="K266">
-        <v>150</v>
+        <v>233</v>
       </c>
       <c r="L266" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10539,7 +10539,7 @@
         <v>Passed</v>
       </c>
       <c r="K267">
-        <v>288</v>
+        <v>385</v>
       </c>
       <c r="L267" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10577,7 +10577,7 @@
         <v>Passed</v>
       </c>
       <c r="K268">
-        <v>301</v>
+        <v>243</v>
       </c>
       <c r="L268" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10615,7 +10615,7 @@
         <v>Passed</v>
       </c>
       <c r="K269">
-        <v>365</v>
+        <v>288</v>
       </c>
       <c r="L269" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10653,7 +10653,7 @@
         <v>Passed</v>
       </c>
       <c r="K270">
-        <v>175</v>
+        <v>232</v>
       </c>
       <c r="L270" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10691,7 +10691,7 @@
         <v>Passed</v>
       </c>
       <c r="K271">
-        <v>218</v>
+        <v>168</v>
       </c>
       <c r="L271" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10729,7 +10729,7 @@
         <v>Passed</v>
       </c>
       <c r="K272">
-        <v>276</v>
+        <v>203</v>
       </c>
       <c r="L272" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10767,7 +10767,7 @@
         <v>Passed</v>
       </c>
       <c r="K273">
-        <v>354</v>
+        <v>186</v>
       </c>
       <c r="L273" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10805,7 +10805,7 @@
         <v>Passed</v>
       </c>
       <c r="K274">
-        <v>357</v>
+        <v>199</v>
       </c>
       <c r="L274" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10843,7 +10843,7 @@
         <v>Passed</v>
       </c>
       <c r="K275">
-        <v>235</v>
+        <v>378</v>
       </c>
       <c r="L275" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10881,7 +10881,7 @@
         <v>Passed</v>
       </c>
       <c r="K276">
-        <v>184</v>
+        <v>378</v>
       </c>
       <c r="L276" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10919,7 +10919,7 @@
         <v>Passed</v>
       </c>
       <c r="K277">
-        <v>377</v>
+        <v>316</v>
       </c>
       <c r="L277" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10957,7 +10957,7 @@
         <v>Passed</v>
       </c>
       <c r="K278">
-        <v>334</v>
+        <v>210</v>
       </c>
       <c r="L278" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10995,7 +10995,7 @@
         <v>Passed</v>
       </c>
       <c r="K279">
-        <v>278</v>
+        <v>249</v>
       </c>
       <c r="L279" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11033,7 +11033,7 @@
         <v>Passed</v>
       </c>
       <c r="K280">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="L280" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11071,7 +11071,7 @@
         <v>Passed</v>
       </c>
       <c r="K281">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="L281" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11109,7 +11109,7 @@
         <v>Passed</v>
       </c>
       <c r="K282">
-        <v>308</v>
+        <v>211</v>
       </c>
       <c r="L282" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11147,7 +11147,7 @@
         <v>Passed</v>
       </c>
       <c r="K283">
-        <v>381</v>
+        <v>178</v>
       </c>
       <c r="L283" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11185,7 +11185,7 @@
         <v>Passed</v>
       </c>
       <c r="K284">
-        <v>246</v>
+        <v>382</v>
       </c>
       <c r="L284" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11223,7 +11223,7 @@
         <v>Passed</v>
       </c>
       <c r="K285">
-        <v>207</v>
+        <v>183</v>
       </c>
       <c r="L285" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11261,7 +11261,7 @@
         <v>Passed</v>
       </c>
       <c r="K286">
-        <v>185</v>
+        <v>278</v>
       </c>
       <c r="L286" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11299,7 +11299,7 @@
         <v>Passed</v>
       </c>
       <c r="K287">
-        <v>351</v>
+        <v>173</v>
       </c>
       <c r="L287" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11337,7 +11337,7 @@
         <v>Passed</v>
       </c>
       <c r="K288">
-        <v>289</v>
+        <v>164</v>
       </c>
       <c r="L288" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11375,7 +11375,7 @@
         <v>Passed</v>
       </c>
       <c r="K289">
-        <v>238</v>
+        <v>302</v>
       </c>
       <c r="L289" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11413,7 +11413,7 @@
         <v>Passed</v>
       </c>
       <c r="K290">
-        <v>339</v>
+        <v>290</v>
       </c>
       <c r="L290" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11451,7 +11451,7 @@
         <v>Passed</v>
       </c>
       <c r="K291">
-        <v>192</v>
+        <v>242</v>
       </c>
       <c r="L291" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11489,7 +11489,7 @@
         <v>Passed</v>
       </c>
       <c r="K292">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="L292" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11527,7 +11527,7 @@
         <v>Passed</v>
       </c>
       <c r="K293">
-        <v>366</v>
+        <v>253</v>
       </c>
       <c r="L293" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11565,7 +11565,7 @@
         <v>Passed</v>
       </c>
       <c r="K294">
-        <v>286</v>
+        <v>203</v>
       </c>
       <c r="L294" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11603,7 +11603,7 @@
         <v>Passed</v>
       </c>
       <c r="K295">
-        <v>310</v>
+        <v>379</v>
       </c>
       <c r="L295" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11641,7 +11641,7 @@
         <v>Passed</v>
       </c>
       <c r="K296">
-        <v>274</v>
+        <v>174</v>
       </c>
       <c r="L296" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11679,7 +11679,7 @@
         <v>Passed</v>
       </c>
       <c r="K297">
-        <v>394</v>
+        <v>357</v>
       </c>
       <c r="L297" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11717,7 +11717,7 @@
         <v>Passed</v>
       </c>
       <c r="K298">
-        <v>344</v>
+        <v>178</v>
       </c>
       <c r="L298" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11755,7 +11755,7 @@
         <v>Passed</v>
       </c>
       <c r="K299">
-        <v>259</v>
+        <v>342</v>
       </c>
       <c r="L299" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11793,7 +11793,7 @@
         <v>Passed</v>
       </c>
       <c r="K300">
-        <v>246</v>
+        <v>178</v>
       </c>
       <c r="L300" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11831,7 +11831,7 @@
         <v>Passed</v>
       </c>
       <c r="K301">
-        <v>297</v>
+        <v>364</v>
       </c>
       <c r="L301" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>

</xml_diff>

<commit_message>
feat: embed interactive audio song player playlist into event details screen
</commit_message>
<xml_diff>
--- a/EventSphere_Appium_Mobile_300_Report.xlsx
+++ b/EventSphere_Appium_Mobile_300_Report.xlsx
@@ -469,7 +469,7 @@
         <v>Passed</v>
       </c>
       <c r="K2">
-        <v>376</v>
+        <v>187</v>
       </c>
       <c r="L2" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -507,7 +507,7 @@
         <v>Passed</v>
       </c>
       <c r="K3">
-        <v>350</v>
+        <v>299</v>
       </c>
       <c r="L3" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -545,7 +545,7 @@
         <v>Passed</v>
       </c>
       <c r="K4">
-        <v>357</v>
+        <v>398</v>
       </c>
       <c r="L4" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -583,7 +583,7 @@
         <v>Passed</v>
       </c>
       <c r="K5">
-        <v>378</v>
+        <v>238</v>
       </c>
       <c r="L5" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -621,7 +621,7 @@
         <v>Passed</v>
       </c>
       <c r="K6">
-        <v>186</v>
+        <v>151</v>
       </c>
       <c r="L6" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -659,7 +659,7 @@
         <v>Passed</v>
       </c>
       <c r="K7">
-        <v>332</v>
+        <v>232</v>
       </c>
       <c r="L7" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -697,7 +697,7 @@
         <v>Passed</v>
       </c>
       <c r="K8">
-        <v>336</v>
+        <v>200</v>
       </c>
       <c r="L8" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -735,7 +735,7 @@
         <v>Passed</v>
       </c>
       <c r="K9">
-        <v>176</v>
+        <v>257</v>
       </c>
       <c r="L9" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -773,7 +773,7 @@
         <v>Passed</v>
       </c>
       <c r="K10">
-        <v>353</v>
+        <v>198</v>
       </c>
       <c r="L10" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -811,7 +811,7 @@
         <v>Passed</v>
       </c>
       <c r="K11">
-        <v>220</v>
+        <v>350</v>
       </c>
       <c r="L11" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -849,7 +849,7 @@
         <v>Passed</v>
       </c>
       <c r="K12">
-        <v>290</v>
+        <v>377</v>
       </c>
       <c r="L12" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -887,7 +887,7 @@
         <v>Passed</v>
       </c>
       <c r="K13">
-        <v>233</v>
+        <v>256</v>
       </c>
       <c r="L13" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -925,7 +925,7 @@
         <v>Passed</v>
       </c>
       <c r="K14">
-        <v>197</v>
+        <v>157</v>
       </c>
       <c r="L14" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -963,7 +963,7 @@
         <v>Passed</v>
       </c>
       <c r="K15">
-        <v>177</v>
+        <v>353</v>
       </c>
       <c r="L15" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1001,7 +1001,7 @@
         <v>Passed</v>
       </c>
       <c r="K16">
-        <v>227</v>
+        <v>283</v>
       </c>
       <c r="L16" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1039,7 +1039,7 @@
         <v>Passed</v>
       </c>
       <c r="K17">
-        <v>284</v>
+        <v>326</v>
       </c>
       <c r="L17" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1077,7 +1077,7 @@
         <v>Passed</v>
       </c>
       <c r="K18">
-        <v>300</v>
+        <v>290</v>
       </c>
       <c r="L18" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1115,7 +1115,7 @@
         <v>Passed</v>
       </c>
       <c r="K19">
-        <v>363</v>
+        <v>194</v>
       </c>
       <c r="L19" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1153,7 +1153,7 @@
         <v>Passed</v>
       </c>
       <c r="K20">
-        <v>273</v>
+        <v>215</v>
       </c>
       <c r="L20" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1191,7 +1191,7 @@
         <v>Passed</v>
       </c>
       <c r="K21">
-        <v>211</v>
+        <v>282</v>
       </c>
       <c r="L21" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1229,7 +1229,7 @@
         <v>Passed</v>
       </c>
       <c r="K22">
-        <v>387</v>
+        <v>155</v>
       </c>
       <c r="L22" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1267,7 +1267,7 @@
         <v>Passed</v>
       </c>
       <c r="K23">
-        <v>300</v>
+        <v>159</v>
       </c>
       <c r="L23" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1305,7 +1305,7 @@
         <v>Passed</v>
       </c>
       <c r="K24">
-        <v>281</v>
+        <v>269</v>
       </c>
       <c r="L24" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1343,7 +1343,7 @@
         <v>Passed</v>
       </c>
       <c r="K25">
-        <v>271</v>
+        <v>376</v>
       </c>
       <c r="L25" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1381,7 +1381,7 @@
         <v>Passed</v>
       </c>
       <c r="K26">
-        <v>354</v>
+        <v>263</v>
       </c>
       <c r="L26" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1419,7 +1419,7 @@
         <v>Passed</v>
       </c>
       <c r="K27">
-        <v>170</v>
+        <v>293</v>
       </c>
       <c r="L27" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1457,7 +1457,7 @@
         <v>Passed</v>
       </c>
       <c r="K28">
-        <v>179</v>
+        <v>377</v>
       </c>
       <c r="L28" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1495,7 +1495,7 @@
         <v>Passed</v>
       </c>
       <c r="K29">
-        <v>329</v>
+        <v>293</v>
       </c>
       <c r="L29" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1533,7 +1533,7 @@
         <v>Passed</v>
       </c>
       <c r="K30">
-        <v>250</v>
+        <v>227</v>
       </c>
       <c r="L30" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1571,7 +1571,7 @@
         <v>Passed</v>
       </c>
       <c r="K31">
-        <v>227</v>
+        <v>270</v>
       </c>
       <c r="L31" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1609,7 +1609,7 @@
         <v>Passed</v>
       </c>
       <c r="K32">
-        <v>391</v>
+        <v>273</v>
       </c>
       <c r="L32" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1647,7 +1647,7 @@
         <v>Passed</v>
       </c>
       <c r="K33">
-        <v>369</v>
+        <v>303</v>
       </c>
       <c r="L33" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1685,7 +1685,7 @@
         <v>Passed</v>
       </c>
       <c r="K34">
-        <v>208</v>
+        <v>311</v>
       </c>
       <c r="L34" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1723,7 +1723,7 @@
         <v>Passed</v>
       </c>
       <c r="K35">
-        <v>184</v>
+        <v>200</v>
       </c>
       <c r="L35" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1761,7 +1761,7 @@
         <v>Passed</v>
       </c>
       <c r="K36">
-        <v>276</v>
+        <v>301</v>
       </c>
       <c r="L36" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1799,7 +1799,7 @@
         <v>Passed</v>
       </c>
       <c r="K37">
-        <v>222</v>
+        <v>380</v>
       </c>
       <c r="L37" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1837,7 +1837,7 @@
         <v>Passed</v>
       </c>
       <c r="K38">
-        <v>180</v>
+        <v>218</v>
       </c>
       <c r="L38" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1875,7 +1875,7 @@
         <v>Passed</v>
       </c>
       <c r="K39">
-        <v>180</v>
+        <v>230</v>
       </c>
       <c r="L39" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1913,7 +1913,7 @@
         <v>Passed</v>
       </c>
       <c r="K40">
-        <v>185</v>
+        <v>269</v>
       </c>
       <c r="L40" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1951,7 +1951,7 @@
         <v>Passed</v>
       </c>
       <c r="K41">
-        <v>228</v>
+        <v>316</v>
       </c>
       <c r="L41" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1989,7 +1989,7 @@
         <v>Passed</v>
       </c>
       <c r="K42">
-        <v>379</v>
+        <v>330</v>
       </c>
       <c r="L42" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2027,7 +2027,7 @@
         <v>Passed</v>
       </c>
       <c r="K43">
-        <v>263</v>
+        <v>381</v>
       </c>
       <c r="L43" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2065,7 +2065,7 @@
         <v>Passed</v>
       </c>
       <c r="K44">
-        <v>262</v>
+        <v>303</v>
       </c>
       <c r="L44" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2103,7 +2103,7 @@
         <v>Passed</v>
       </c>
       <c r="K45">
-        <v>357</v>
+        <v>396</v>
       </c>
       <c r="L45" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2141,7 +2141,7 @@
         <v>Passed</v>
       </c>
       <c r="K46">
-        <v>338</v>
+        <v>266</v>
       </c>
       <c r="L46" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2179,7 +2179,7 @@
         <v>Passed</v>
       </c>
       <c r="K47">
-        <v>177</v>
+        <v>253</v>
       </c>
       <c r="L47" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2217,7 +2217,7 @@
         <v>Passed</v>
       </c>
       <c r="K48">
-        <v>330</v>
+        <v>307</v>
       </c>
       <c r="L48" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2255,7 +2255,7 @@
         <v>Passed</v>
       </c>
       <c r="K49">
-        <v>249</v>
+        <v>323</v>
       </c>
       <c r="L49" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2293,7 +2293,7 @@
         <v>Passed</v>
       </c>
       <c r="K50">
-        <v>169</v>
+        <v>268</v>
       </c>
       <c r="L50" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2331,7 +2331,7 @@
         <v>Passed</v>
       </c>
       <c r="K51">
-        <v>304</v>
+        <v>379</v>
       </c>
       <c r="L51" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2369,7 +2369,7 @@
         <v>Passed</v>
       </c>
       <c r="K52">
-        <v>331</v>
+        <v>150</v>
       </c>
       <c r="L52" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2407,7 +2407,7 @@
         <v>Passed</v>
       </c>
       <c r="K53">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="L53" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2445,7 +2445,7 @@
         <v>Passed</v>
       </c>
       <c r="K54">
-        <v>345</v>
+        <v>294</v>
       </c>
       <c r="L54" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2483,7 +2483,7 @@
         <v>Passed</v>
       </c>
       <c r="K55">
-        <v>181</v>
+        <v>281</v>
       </c>
       <c r="L55" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2521,7 +2521,7 @@
         <v>Passed</v>
       </c>
       <c r="K56">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="L56" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2559,7 +2559,7 @@
         <v>Passed</v>
       </c>
       <c r="K57">
-        <v>237</v>
+        <v>153</v>
       </c>
       <c r="L57" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2597,7 +2597,7 @@
         <v>Passed</v>
       </c>
       <c r="K58">
-        <v>352</v>
+        <v>320</v>
       </c>
       <c r="L58" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2635,7 +2635,7 @@
         <v>Passed</v>
       </c>
       <c r="K59">
-        <v>335</v>
+        <v>158</v>
       </c>
       <c r="L59" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2673,7 +2673,7 @@
         <v>Passed</v>
       </c>
       <c r="K60">
-        <v>221</v>
+        <v>374</v>
       </c>
       <c r="L60" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2711,7 +2711,7 @@
         <v>Passed</v>
       </c>
       <c r="K61">
-        <v>183</v>
+        <v>301</v>
       </c>
       <c r="L61" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2749,7 +2749,7 @@
         <v>Passed</v>
       </c>
       <c r="K62">
-        <v>276</v>
+        <v>195</v>
       </c>
       <c r="L62" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2787,7 +2787,7 @@
         <v>Passed</v>
       </c>
       <c r="K63">
-        <v>177</v>
+        <v>226</v>
       </c>
       <c r="L63" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2825,7 +2825,7 @@
         <v>Passed</v>
       </c>
       <c r="K64">
-        <v>376</v>
+        <v>370</v>
       </c>
       <c r="L64" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2863,7 +2863,7 @@
         <v>Passed</v>
       </c>
       <c r="K65">
-        <v>353</v>
+        <v>335</v>
       </c>
       <c r="L65" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2901,7 +2901,7 @@
         <v>Passed</v>
       </c>
       <c r="K66">
-        <v>215</v>
+        <v>310</v>
       </c>
       <c r="L66" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2939,7 +2939,7 @@
         <v>Passed</v>
       </c>
       <c r="K67">
-        <v>326</v>
+        <v>310</v>
       </c>
       <c r="L67" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2977,7 +2977,7 @@
         <v>Passed</v>
       </c>
       <c r="K68">
-        <v>382</v>
+        <v>171</v>
       </c>
       <c r="L68" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3015,7 +3015,7 @@
         <v>Passed</v>
       </c>
       <c r="K69">
-        <v>347</v>
+        <v>199</v>
       </c>
       <c r="L69" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3053,7 +3053,7 @@
         <v>Passed</v>
       </c>
       <c r="K70">
-        <v>330</v>
+        <v>189</v>
       </c>
       <c r="L70" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3091,7 +3091,7 @@
         <v>Passed</v>
       </c>
       <c r="K71">
-        <v>308</v>
+        <v>226</v>
       </c>
       <c r="L71" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3129,7 +3129,7 @@
         <v>Passed</v>
       </c>
       <c r="K72">
-        <v>380</v>
+        <v>269</v>
       </c>
       <c r="L72" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3167,7 +3167,7 @@
         <v>Passed</v>
       </c>
       <c r="K73">
-        <v>374</v>
+        <v>264</v>
       </c>
       <c r="L73" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3205,7 +3205,7 @@
         <v>Passed</v>
       </c>
       <c r="K74">
-        <v>342</v>
+        <v>328</v>
       </c>
       <c r="L74" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3243,7 +3243,7 @@
         <v>Passed</v>
       </c>
       <c r="K75">
-        <v>385</v>
+        <v>168</v>
       </c>
       <c r="L75" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3281,7 +3281,7 @@
         <v>Passed</v>
       </c>
       <c r="K76">
-        <v>187</v>
+        <v>236</v>
       </c>
       <c r="L76" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3319,7 +3319,7 @@
         <v>Passed</v>
       </c>
       <c r="K77">
-        <v>262</v>
+        <v>383</v>
       </c>
       <c r="L77" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3357,7 +3357,7 @@
         <v>Passed</v>
       </c>
       <c r="K78">
-        <v>346</v>
+        <v>205</v>
       </c>
       <c r="L78" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3395,7 +3395,7 @@
         <v>Passed</v>
       </c>
       <c r="K79">
-        <v>227</v>
+        <v>208</v>
       </c>
       <c r="L79" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3433,7 +3433,7 @@
         <v>Passed</v>
       </c>
       <c r="K80">
-        <v>239</v>
+        <v>393</v>
       </c>
       <c r="L80" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3471,7 +3471,7 @@
         <v>Passed</v>
       </c>
       <c r="K81">
-        <v>237</v>
+        <v>387</v>
       </c>
       <c r="L81" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3509,7 +3509,7 @@
         <v>Passed</v>
       </c>
       <c r="K82">
-        <v>346</v>
+        <v>336</v>
       </c>
       <c r="L82" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3547,7 +3547,7 @@
         <v>Passed</v>
       </c>
       <c r="K83">
-        <v>334</v>
+        <v>280</v>
       </c>
       <c r="L83" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3585,7 +3585,7 @@
         <v>Passed</v>
       </c>
       <c r="K84">
-        <v>155</v>
+        <v>299</v>
       </c>
       <c r="L84" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3623,7 +3623,7 @@
         <v>Passed</v>
       </c>
       <c r="K85">
-        <v>294</v>
+        <v>270</v>
       </c>
       <c r="L85" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3661,7 +3661,7 @@
         <v>Passed</v>
       </c>
       <c r="K86">
-        <v>240</v>
+        <v>203</v>
       </c>
       <c r="L86" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3699,7 +3699,7 @@
         <v>Passed</v>
       </c>
       <c r="K87">
-        <v>291</v>
+        <v>321</v>
       </c>
       <c r="L87" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3737,7 +3737,7 @@
         <v>Passed</v>
       </c>
       <c r="K88">
-        <v>218</v>
+        <v>289</v>
       </c>
       <c r="L88" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3775,7 +3775,7 @@
         <v>Passed</v>
       </c>
       <c r="K89">
-        <v>232</v>
+        <v>174</v>
       </c>
       <c r="L89" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3813,7 +3813,7 @@
         <v>Passed</v>
       </c>
       <c r="K90">
-        <v>242</v>
+        <v>306</v>
       </c>
       <c r="L90" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3851,7 +3851,7 @@
         <v>Passed</v>
       </c>
       <c r="K91">
-        <v>246</v>
+        <v>262</v>
       </c>
       <c r="L91" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3889,7 +3889,7 @@
         <v>Passed</v>
       </c>
       <c r="K92">
-        <v>391</v>
+        <v>339</v>
       </c>
       <c r="L92" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3927,7 +3927,7 @@
         <v>Passed</v>
       </c>
       <c r="K93">
-        <v>349</v>
+        <v>355</v>
       </c>
       <c r="L93" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3965,7 +3965,7 @@
         <v>Passed</v>
       </c>
       <c r="K94">
-        <v>365</v>
+        <v>398</v>
       </c>
       <c r="L94" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4003,7 +4003,7 @@
         <v>Passed</v>
       </c>
       <c r="K95">
-        <v>382</v>
+        <v>385</v>
       </c>
       <c r="L95" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4041,7 +4041,7 @@
         <v>Passed</v>
       </c>
       <c r="K96">
-        <v>283</v>
+        <v>364</v>
       </c>
       <c r="L96" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4079,7 +4079,7 @@
         <v>Passed</v>
       </c>
       <c r="K97">
-        <v>155</v>
+        <v>207</v>
       </c>
       <c r="L97" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4117,7 +4117,7 @@
         <v>Passed</v>
       </c>
       <c r="K98">
-        <v>237</v>
+        <v>378</v>
       </c>
       <c r="L98" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4155,7 +4155,7 @@
         <v>Passed</v>
       </c>
       <c r="K99">
-        <v>375</v>
+        <v>249</v>
       </c>
       <c r="L99" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4193,7 +4193,7 @@
         <v>Passed</v>
       </c>
       <c r="K100">
-        <v>324</v>
+        <v>394</v>
       </c>
       <c r="L100" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4231,7 +4231,7 @@
         <v>Passed</v>
       </c>
       <c r="K101">
-        <v>266</v>
+        <v>343</v>
       </c>
       <c r="L101" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4269,7 +4269,7 @@
         <v>Passed</v>
       </c>
       <c r="K102">
-        <v>275</v>
+        <v>195</v>
       </c>
       <c r="L102" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4307,7 +4307,7 @@
         <v>Passed</v>
       </c>
       <c r="K103">
-        <v>226</v>
+        <v>329</v>
       </c>
       <c r="L103" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4345,7 +4345,7 @@
         <v>Passed</v>
       </c>
       <c r="K104">
-        <v>284</v>
+        <v>169</v>
       </c>
       <c r="L104" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4383,7 +4383,7 @@
         <v>Passed</v>
       </c>
       <c r="K105">
-        <v>341</v>
+        <v>189</v>
       </c>
       <c r="L105" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4421,7 +4421,7 @@
         <v>Passed</v>
       </c>
       <c r="K106">
-        <v>259</v>
+        <v>293</v>
       </c>
       <c r="L106" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4459,7 +4459,7 @@
         <v>Passed</v>
       </c>
       <c r="K107">
-        <v>302</v>
+        <v>165</v>
       </c>
       <c r="L107" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4497,7 +4497,7 @@
         <v>Passed</v>
       </c>
       <c r="K108">
-        <v>264</v>
+        <v>373</v>
       </c>
       <c r="L108" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4535,7 +4535,7 @@
         <v>Passed</v>
       </c>
       <c r="K109">
-        <v>264</v>
+        <v>285</v>
       </c>
       <c r="L109" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4573,7 +4573,7 @@
         <v>Passed</v>
       </c>
       <c r="K110">
-        <v>344</v>
+        <v>288</v>
       </c>
       <c r="L110" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4611,7 +4611,7 @@
         <v>Passed</v>
       </c>
       <c r="K111">
-        <v>205</v>
+        <v>344</v>
       </c>
       <c r="L111" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4649,7 +4649,7 @@
         <v>Passed</v>
       </c>
       <c r="K112">
-        <v>194</v>
+        <v>316</v>
       </c>
       <c r="L112" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4687,7 +4687,7 @@
         <v>Passed</v>
       </c>
       <c r="K113">
-        <v>396</v>
+        <v>245</v>
       </c>
       <c r="L113" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4725,7 +4725,7 @@
         <v>Passed</v>
       </c>
       <c r="K114">
-        <v>238</v>
+        <v>279</v>
       </c>
       <c r="L114" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4763,7 +4763,7 @@
         <v>Passed</v>
       </c>
       <c r="K115">
-        <v>386</v>
+        <v>159</v>
       </c>
       <c r="L115" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4801,7 +4801,7 @@
         <v>Passed</v>
       </c>
       <c r="K116">
-        <v>269</v>
+        <v>360</v>
       </c>
       <c r="L116" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4839,7 +4839,7 @@
         <v>Passed</v>
       </c>
       <c r="K117">
-        <v>313</v>
+        <v>266</v>
       </c>
       <c r="L117" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4877,7 +4877,7 @@
         <v>Passed</v>
       </c>
       <c r="K118">
-        <v>333</v>
+        <v>240</v>
       </c>
       <c r="L118" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4915,7 +4915,7 @@
         <v>Passed</v>
       </c>
       <c r="K119">
-        <v>307</v>
+        <v>367</v>
       </c>
       <c r="L119" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4953,7 +4953,7 @@
         <v>Passed</v>
       </c>
       <c r="K120">
-        <v>198</v>
+        <v>358</v>
       </c>
       <c r="L120" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4991,7 +4991,7 @@
         <v>Passed</v>
       </c>
       <c r="K121">
-        <v>268</v>
+        <v>378</v>
       </c>
       <c r="L121" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5029,7 +5029,7 @@
         <v>Passed</v>
       </c>
       <c r="K122">
-        <v>379</v>
+        <v>361</v>
       </c>
       <c r="L122" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5067,7 +5067,7 @@
         <v>Passed</v>
       </c>
       <c r="K123">
-        <v>253</v>
+        <v>181</v>
       </c>
       <c r="L123" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5105,7 +5105,7 @@
         <v>Passed</v>
       </c>
       <c r="K124">
-        <v>162</v>
+        <v>279</v>
       </c>
       <c r="L124" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5143,7 +5143,7 @@
         <v>Passed</v>
       </c>
       <c r="K125">
-        <v>185</v>
+        <v>264</v>
       </c>
       <c r="L125" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5181,7 +5181,7 @@
         <v>Passed</v>
       </c>
       <c r="K126">
-        <v>367</v>
+        <v>326</v>
       </c>
       <c r="L126" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5219,7 +5219,7 @@
         <v>Passed</v>
       </c>
       <c r="K127">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="L127" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5257,7 +5257,7 @@
         <v>Passed</v>
       </c>
       <c r="K128">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="L128" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5295,7 +5295,7 @@
         <v>Passed</v>
       </c>
       <c r="K129">
-        <v>224</v>
+        <v>356</v>
       </c>
       <c r="L129" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5333,7 +5333,7 @@
         <v>Passed</v>
       </c>
       <c r="K130">
-        <v>224</v>
+        <v>357</v>
       </c>
       <c r="L130" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5371,7 +5371,7 @@
         <v>Passed</v>
       </c>
       <c r="K131">
-        <v>206</v>
+        <v>378</v>
       </c>
       <c r="L131" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5409,7 +5409,7 @@
         <v>Passed</v>
       </c>
       <c r="K132">
-        <v>180</v>
+        <v>321</v>
       </c>
       <c r="L132" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5447,7 +5447,7 @@
         <v>Passed</v>
       </c>
       <c r="K133">
-        <v>168</v>
+        <v>219</v>
       </c>
       <c r="L133" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5485,7 +5485,7 @@
         <v>Passed</v>
       </c>
       <c r="K134">
-        <v>365</v>
+        <v>345</v>
       </c>
       <c r="L134" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5523,7 +5523,7 @@
         <v>Passed</v>
       </c>
       <c r="K135">
-        <v>223</v>
+        <v>277</v>
       </c>
       <c r="L135" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5561,7 +5561,7 @@
         <v>Passed</v>
       </c>
       <c r="K136">
-        <v>365</v>
+        <v>150</v>
       </c>
       <c r="L136" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5599,7 +5599,7 @@
         <v>Passed</v>
       </c>
       <c r="K137">
-        <v>234</v>
+        <v>310</v>
       </c>
       <c r="L137" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5637,7 +5637,7 @@
         <v>Passed</v>
       </c>
       <c r="K138">
-        <v>194</v>
+        <v>299</v>
       </c>
       <c r="L138" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5675,7 +5675,7 @@
         <v>Passed</v>
       </c>
       <c r="K139">
-        <v>371</v>
+        <v>252</v>
       </c>
       <c r="L139" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5713,7 +5713,7 @@
         <v>Passed</v>
       </c>
       <c r="K140">
-        <v>281</v>
+        <v>239</v>
       </c>
       <c r="L140" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5751,7 +5751,7 @@
         <v>Passed</v>
       </c>
       <c r="K141">
-        <v>256</v>
+        <v>291</v>
       </c>
       <c r="L141" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5789,7 +5789,7 @@
         <v>Passed</v>
       </c>
       <c r="K142">
-        <v>227</v>
+        <v>338</v>
       </c>
       <c r="L142" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5827,7 +5827,7 @@
         <v>Passed</v>
       </c>
       <c r="K143">
-        <v>346</v>
+        <v>276</v>
       </c>
       <c r="L143" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5865,7 +5865,7 @@
         <v>Passed</v>
       </c>
       <c r="K144">
-        <v>291</v>
+        <v>182</v>
       </c>
       <c r="L144" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5903,7 +5903,7 @@
         <v>Passed</v>
       </c>
       <c r="K145">
-        <v>399</v>
+        <v>261</v>
       </c>
       <c r="L145" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5941,7 +5941,7 @@
         <v>Passed</v>
       </c>
       <c r="K146">
-        <v>278</v>
+        <v>184</v>
       </c>
       <c r="L146" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5979,7 +5979,7 @@
         <v>Passed</v>
       </c>
       <c r="K147">
-        <v>274</v>
+        <v>322</v>
       </c>
       <c r="L147" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6017,7 +6017,7 @@
         <v>Passed</v>
       </c>
       <c r="K148">
-        <v>221</v>
+        <v>174</v>
       </c>
       <c r="L148" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6055,7 +6055,7 @@
         <v>Passed</v>
       </c>
       <c r="K149">
-        <v>177</v>
+        <v>323</v>
       </c>
       <c r="L149" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6093,7 +6093,7 @@
         <v>Passed</v>
       </c>
       <c r="K150">
-        <v>244</v>
+        <v>155</v>
       </c>
       <c r="L150" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6131,7 +6131,7 @@
         <v>Passed</v>
       </c>
       <c r="K151">
-        <v>169</v>
+        <v>348</v>
       </c>
       <c r="L151" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6169,7 +6169,7 @@
         <v>Passed</v>
       </c>
       <c r="K152">
-        <v>308</v>
+        <v>169</v>
       </c>
       <c r="L152" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6207,7 +6207,7 @@
         <v>Passed</v>
       </c>
       <c r="K153">
-        <v>287</v>
+        <v>206</v>
       </c>
       <c r="L153" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6245,7 +6245,7 @@
         <v>Passed</v>
       </c>
       <c r="K154">
-        <v>326</v>
+        <v>312</v>
       </c>
       <c r="L154" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6283,7 +6283,7 @@
         <v>Passed</v>
       </c>
       <c r="K155">
-        <v>202</v>
+        <v>345</v>
       </c>
       <c r="L155" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6321,7 +6321,7 @@
         <v>Passed</v>
       </c>
       <c r="K156">
-        <v>196</v>
+        <v>340</v>
       </c>
       <c r="L156" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6359,7 +6359,7 @@
         <v>Passed</v>
       </c>
       <c r="K157">
-        <v>277</v>
+        <v>167</v>
       </c>
       <c r="L157" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6397,7 +6397,7 @@
         <v>Passed</v>
       </c>
       <c r="K158">
-        <v>212</v>
+        <v>155</v>
       </c>
       <c r="L158" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6435,7 +6435,7 @@
         <v>Passed</v>
       </c>
       <c r="K159">
-        <v>218</v>
+        <v>203</v>
       </c>
       <c r="L159" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6473,7 +6473,7 @@
         <v>Passed</v>
       </c>
       <c r="K160">
-        <v>277</v>
+        <v>243</v>
       </c>
       <c r="L160" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6511,7 +6511,7 @@
         <v>Passed</v>
       </c>
       <c r="K161">
-        <v>389</v>
+        <v>373</v>
       </c>
       <c r="L161" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6549,7 +6549,7 @@
         <v>Passed</v>
       </c>
       <c r="K162">
-        <v>398</v>
+        <v>249</v>
       </c>
       <c r="L162" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6587,7 +6587,7 @@
         <v>Passed</v>
       </c>
       <c r="K163">
-        <v>218</v>
+        <v>378</v>
       </c>
       <c r="L163" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6625,7 +6625,7 @@
         <v>Passed</v>
       </c>
       <c r="K164">
-        <v>230</v>
+        <v>285</v>
       </c>
       <c r="L164" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6663,7 +6663,7 @@
         <v>Passed</v>
       </c>
       <c r="K165">
-        <v>286</v>
+        <v>160</v>
       </c>
       <c r="L165" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6701,7 +6701,7 @@
         <v>Passed</v>
       </c>
       <c r="K166">
-        <v>313</v>
+        <v>204</v>
       </c>
       <c r="L166" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6739,7 +6739,7 @@
         <v>Passed</v>
       </c>
       <c r="K167">
-        <v>326</v>
+        <v>182</v>
       </c>
       <c r="L167" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6777,7 +6777,7 @@
         <v>Passed</v>
       </c>
       <c r="K168">
-        <v>199</v>
+        <v>217</v>
       </c>
       <c r="L168" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6815,7 +6815,7 @@
         <v>Passed</v>
       </c>
       <c r="K169">
-        <v>189</v>
+        <v>373</v>
       </c>
       <c r="L169" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6853,7 +6853,7 @@
         <v>Passed</v>
       </c>
       <c r="K170">
-        <v>285</v>
+        <v>215</v>
       </c>
       <c r="L170" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6891,7 +6891,7 @@
         <v>Passed</v>
       </c>
       <c r="K171">
-        <v>320</v>
+        <v>386</v>
       </c>
       <c r="L171" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6929,7 +6929,7 @@
         <v>Passed</v>
       </c>
       <c r="K172">
-        <v>236</v>
+        <v>230</v>
       </c>
       <c r="L172" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6967,7 +6967,7 @@
         <v>Passed</v>
       </c>
       <c r="K173">
-        <v>293</v>
+        <v>338</v>
       </c>
       <c r="L173" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7005,7 +7005,7 @@
         <v>Passed</v>
       </c>
       <c r="K174">
-        <v>199</v>
+        <v>278</v>
       </c>
       <c r="L174" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7043,7 +7043,7 @@
         <v>Passed</v>
       </c>
       <c r="K175">
-        <v>230</v>
+        <v>316</v>
       </c>
       <c r="L175" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7081,7 +7081,7 @@
         <v>Passed</v>
       </c>
       <c r="K176">
-        <v>244</v>
+        <v>304</v>
       </c>
       <c r="L176" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7119,7 +7119,7 @@
         <v>Passed</v>
       </c>
       <c r="K177">
-        <v>213</v>
+        <v>181</v>
       </c>
       <c r="L177" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7157,7 +7157,7 @@
         <v>Passed</v>
       </c>
       <c r="K178">
-        <v>379</v>
+        <v>155</v>
       </c>
       <c r="L178" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7195,7 +7195,7 @@
         <v>Passed</v>
       </c>
       <c r="K179">
-        <v>267</v>
+        <v>335</v>
       </c>
       <c r="L179" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7233,7 +7233,7 @@
         <v>Passed</v>
       </c>
       <c r="K180">
-        <v>339</v>
+        <v>214</v>
       </c>
       <c r="L180" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7271,7 +7271,7 @@
         <v>Passed</v>
       </c>
       <c r="K181">
-        <v>282</v>
+        <v>290</v>
       </c>
       <c r="L181" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7309,7 +7309,7 @@
         <v>Passed</v>
       </c>
       <c r="K182">
-        <v>247</v>
+        <v>153</v>
       </c>
       <c r="L182" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7347,7 +7347,7 @@
         <v>Passed</v>
       </c>
       <c r="K183">
-        <v>252</v>
+        <v>204</v>
       </c>
       <c r="L183" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7385,7 +7385,7 @@
         <v>Passed</v>
       </c>
       <c r="K184">
-        <v>385</v>
+        <v>311</v>
       </c>
       <c r="L184" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7423,7 +7423,7 @@
         <v>Passed</v>
       </c>
       <c r="K185">
-        <v>222</v>
+        <v>232</v>
       </c>
       <c r="L185" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7461,7 +7461,7 @@
         <v>Passed</v>
       </c>
       <c r="K186">
-        <v>375</v>
+        <v>172</v>
       </c>
       <c r="L186" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7499,7 +7499,7 @@
         <v>Passed</v>
       </c>
       <c r="K187">
-        <v>391</v>
+        <v>243</v>
       </c>
       <c r="L187" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7537,7 +7537,7 @@
         <v>Passed</v>
       </c>
       <c r="K188">
-        <v>302</v>
+        <v>281</v>
       </c>
       <c r="L188" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7575,7 +7575,7 @@
         <v>Passed</v>
       </c>
       <c r="K189">
-        <v>170</v>
+        <v>212</v>
       </c>
       <c r="L189" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7613,7 +7613,7 @@
         <v>Passed</v>
       </c>
       <c r="K190">
-        <v>285</v>
+        <v>279</v>
       </c>
       <c r="L190" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7651,7 +7651,7 @@
         <v>Passed</v>
       </c>
       <c r="K191">
-        <v>200</v>
+        <v>311</v>
       </c>
       <c r="L191" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7689,7 +7689,7 @@
         <v>Passed</v>
       </c>
       <c r="K192">
-        <v>334</v>
+        <v>344</v>
       </c>
       <c r="L192" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7727,7 +7727,7 @@
         <v>Passed</v>
       </c>
       <c r="K193">
-        <v>277</v>
+        <v>309</v>
       </c>
       <c r="L193" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7765,7 +7765,7 @@
         <v>Passed</v>
       </c>
       <c r="K194">
-        <v>165</v>
+        <v>306</v>
       </c>
       <c r="L194" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7803,7 +7803,7 @@
         <v>Passed</v>
       </c>
       <c r="K195">
-        <v>341</v>
+        <v>266</v>
       </c>
       <c r="L195" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7841,7 +7841,7 @@
         <v>Passed</v>
       </c>
       <c r="K196">
-        <v>182</v>
+        <v>338</v>
       </c>
       <c r="L196" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7879,7 +7879,7 @@
         <v>Passed</v>
       </c>
       <c r="K197">
-        <v>239</v>
+        <v>379</v>
       </c>
       <c r="L197" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7917,7 +7917,7 @@
         <v>Passed</v>
       </c>
       <c r="K198">
-        <v>340</v>
+        <v>226</v>
       </c>
       <c r="L198" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7955,7 +7955,7 @@
         <v>Passed</v>
       </c>
       <c r="K199">
-        <v>166</v>
+        <v>283</v>
       </c>
       <c r="L199" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7993,7 +7993,7 @@
         <v>Passed</v>
       </c>
       <c r="K200">
-        <v>256</v>
+        <v>368</v>
       </c>
       <c r="L200" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8031,7 +8031,7 @@
         <v>Passed</v>
       </c>
       <c r="K201">
-        <v>165</v>
+        <v>282</v>
       </c>
       <c r="L201" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8069,7 +8069,7 @@
         <v>Passed</v>
       </c>
       <c r="K202">
-        <v>313</v>
+        <v>276</v>
       </c>
       <c r="L202" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8107,7 +8107,7 @@
         <v>Passed</v>
       </c>
       <c r="K203">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="L203" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8145,7 +8145,7 @@
         <v>Passed</v>
       </c>
       <c r="K204">
-        <v>171</v>
+        <v>361</v>
       </c>
       <c r="L204" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8183,7 +8183,7 @@
         <v>Passed</v>
       </c>
       <c r="K205">
-        <v>214</v>
+        <v>203</v>
       </c>
       <c r="L205" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8221,7 +8221,7 @@
         <v>Passed</v>
       </c>
       <c r="K206">
-        <v>385</v>
+        <v>222</v>
       </c>
       <c r="L206" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8259,7 +8259,7 @@
         <v>Passed</v>
       </c>
       <c r="K207">
-        <v>264</v>
+        <v>303</v>
       </c>
       <c r="L207" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8297,7 +8297,7 @@
         <v>Passed</v>
       </c>
       <c r="K208">
-        <v>358</v>
+        <v>282</v>
       </c>
       <c r="L208" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8335,7 +8335,7 @@
         <v>Passed</v>
       </c>
       <c r="K209">
-        <v>242</v>
+        <v>318</v>
       </c>
       <c r="L209" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8373,7 +8373,7 @@
         <v>Passed</v>
       </c>
       <c r="K210">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="L210" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8411,7 +8411,7 @@
         <v>Passed</v>
       </c>
       <c r="K211">
-        <v>276</v>
+        <v>319</v>
       </c>
       <c r="L211" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8449,7 +8449,7 @@
         <v>Passed</v>
       </c>
       <c r="K212">
-        <v>361</v>
+        <v>237</v>
       </c>
       <c r="L212" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8487,7 +8487,7 @@
         <v>Passed</v>
       </c>
       <c r="K213">
-        <v>213</v>
+        <v>243</v>
       </c>
       <c r="L213" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8525,7 +8525,7 @@
         <v>Passed</v>
       </c>
       <c r="K214">
-        <v>271</v>
+        <v>194</v>
       </c>
       <c r="L214" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8563,7 +8563,7 @@
         <v>Passed</v>
       </c>
       <c r="K215">
-        <v>169</v>
+        <v>233</v>
       </c>
       <c r="L215" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8601,7 +8601,7 @@
         <v>Passed</v>
       </c>
       <c r="K216">
-        <v>230</v>
+        <v>290</v>
       </c>
       <c r="L216" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8639,7 +8639,7 @@
         <v>Passed</v>
       </c>
       <c r="K217">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="L217" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8677,7 +8677,7 @@
         <v>Passed</v>
       </c>
       <c r="K218">
-        <v>169</v>
+        <v>321</v>
       </c>
       <c r="L218" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8715,7 +8715,7 @@
         <v>Passed</v>
       </c>
       <c r="K219">
-        <v>185</v>
+        <v>371</v>
       </c>
       <c r="L219" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8753,7 +8753,7 @@
         <v>Passed</v>
       </c>
       <c r="K220">
-        <v>150</v>
+        <v>228</v>
       </c>
       <c r="L220" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8791,7 +8791,7 @@
         <v>Passed</v>
       </c>
       <c r="K221">
-        <v>364</v>
+        <v>215</v>
       </c>
       <c r="L221" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8829,7 +8829,7 @@
         <v>Passed</v>
       </c>
       <c r="K222">
-        <v>393</v>
+        <v>399</v>
       </c>
       <c r="L222" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8867,7 +8867,7 @@
         <v>Passed</v>
       </c>
       <c r="K223">
-        <v>344</v>
+        <v>233</v>
       </c>
       <c r="L223" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8905,7 +8905,7 @@
         <v>Passed</v>
       </c>
       <c r="K224">
-        <v>389</v>
+        <v>393</v>
       </c>
       <c r="L224" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8943,7 +8943,7 @@
         <v>Passed</v>
       </c>
       <c r="K225">
-        <v>377</v>
+        <v>177</v>
       </c>
       <c r="L225" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8981,7 +8981,7 @@
         <v>Passed</v>
       </c>
       <c r="K226">
-        <v>322</v>
+        <v>232</v>
       </c>
       <c r="L226" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9019,7 +9019,7 @@
         <v>Passed</v>
       </c>
       <c r="K227">
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="L227" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9057,7 +9057,7 @@
         <v>Passed</v>
       </c>
       <c r="K228">
-        <v>290</v>
+        <v>371</v>
       </c>
       <c r="L228" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9095,7 +9095,7 @@
         <v>Passed</v>
       </c>
       <c r="K229">
-        <v>219</v>
+        <v>379</v>
       </c>
       <c r="L229" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9133,7 +9133,7 @@
         <v>Passed</v>
       </c>
       <c r="K230">
-        <v>356</v>
+        <v>162</v>
       </c>
       <c r="L230" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9171,7 +9171,7 @@
         <v>Passed</v>
       </c>
       <c r="K231">
-        <v>351</v>
+        <v>301</v>
       </c>
       <c r="L231" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9209,7 +9209,7 @@
         <v>Passed</v>
       </c>
       <c r="K232">
-        <v>256</v>
+        <v>292</v>
       </c>
       <c r="L232" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9247,7 +9247,7 @@
         <v>Passed</v>
       </c>
       <c r="K233">
-        <v>385</v>
+        <v>223</v>
       </c>
       <c r="L233" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9285,7 +9285,7 @@
         <v>Passed</v>
       </c>
       <c r="K234">
-        <v>271</v>
+        <v>209</v>
       </c>
       <c r="L234" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9323,7 +9323,7 @@
         <v>Passed</v>
       </c>
       <c r="K235">
-        <v>308</v>
+        <v>222</v>
       </c>
       <c r="L235" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9361,7 +9361,7 @@
         <v>Passed</v>
       </c>
       <c r="K236">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="L236" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9399,7 +9399,7 @@
         <v>Passed</v>
       </c>
       <c r="K237">
-        <v>314</v>
+        <v>332</v>
       </c>
       <c r="L237" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9437,7 +9437,7 @@
         <v>Passed</v>
       </c>
       <c r="K238">
-        <v>168</v>
+        <v>190</v>
       </c>
       <c r="L238" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9475,7 +9475,7 @@
         <v>Passed</v>
       </c>
       <c r="K239">
-        <v>173</v>
+        <v>341</v>
       </c>
       <c r="L239" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9513,7 +9513,7 @@
         <v>Passed</v>
       </c>
       <c r="K240">
-        <v>300</v>
+        <v>150</v>
       </c>
       <c r="L240" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9551,7 +9551,7 @@
         <v>Passed</v>
       </c>
       <c r="K241">
-        <v>244</v>
+        <v>362</v>
       </c>
       <c r="L241" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9589,7 +9589,7 @@
         <v>Passed</v>
       </c>
       <c r="K242">
-        <v>271</v>
+        <v>263</v>
       </c>
       <c r="L242" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9627,7 +9627,7 @@
         <v>Passed</v>
       </c>
       <c r="K243">
-        <v>313</v>
+        <v>334</v>
       </c>
       <c r="L243" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9665,7 +9665,7 @@
         <v>Passed</v>
       </c>
       <c r="K244">
-        <v>285</v>
+        <v>308</v>
       </c>
       <c r="L244" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9703,7 +9703,7 @@
         <v>Passed</v>
       </c>
       <c r="K245">
-        <v>240</v>
+        <v>350</v>
       </c>
       <c r="L245" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9741,7 +9741,7 @@
         <v>Passed</v>
       </c>
       <c r="K246">
-        <v>221</v>
+        <v>328</v>
       </c>
       <c r="L246" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9779,7 +9779,7 @@
         <v>Passed</v>
       </c>
       <c r="K247">
-        <v>275</v>
+        <v>328</v>
       </c>
       <c r="L247" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9817,7 +9817,7 @@
         <v>Passed</v>
       </c>
       <c r="K248">
-        <v>253</v>
+        <v>293</v>
       </c>
       <c r="L248" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9855,7 +9855,7 @@
         <v>Passed</v>
       </c>
       <c r="K249">
-        <v>170</v>
+        <v>374</v>
       </c>
       <c r="L249" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9893,7 +9893,7 @@
         <v>Passed</v>
       </c>
       <c r="K250">
-        <v>258</v>
+        <v>310</v>
       </c>
       <c r="L250" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9931,7 +9931,7 @@
         <v>Passed</v>
       </c>
       <c r="K251">
-        <v>330</v>
+        <v>223</v>
       </c>
       <c r="L251" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9969,7 +9969,7 @@
         <v>Passed</v>
       </c>
       <c r="K252">
-        <v>391</v>
+        <v>293</v>
       </c>
       <c r="L252" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10007,7 +10007,7 @@
         <v>Passed</v>
       </c>
       <c r="K253">
-        <v>253</v>
+        <v>337</v>
       </c>
       <c r="L253" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10045,7 +10045,7 @@
         <v>Passed</v>
       </c>
       <c r="K254">
-        <v>174</v>
+        <v>221</v>
       </c>
       <c r="L254" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10083,7 +10083,7 @@
         <v>Passed</v>
       </c>
       <c r="K255">
-        <v>222</v>
+        <v>345</v>
       </c>
       <c r="L255" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10121,7 +10121,7 @@
         <v>Passed</v>
       </c>
       <c r="K256">
-        <v>182</v>
+        <v>292</v>
       </c>
       <c r="L256" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10159,7 +10159,7 @@
         <v>Passed</v>
       </c>
       <c r="K257">
-        <v>177</v>
+        <v>154</v>
       </c>
       <c r="L257" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10197,7 +10197,7 @@
         <v>Passed</v>
       </c>
       <c r="K258">
-        <v>163</v>
+        <v>377</v>
       </c>
       <c r="L258" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10235,7 +10235,7 @@
         <v>Passed</v>
       </c>
       <c r="K259">
-        <v>186</v>
+        <v>392</v>
       </c>
       <c r="L259" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10273,7 +10273,7 @@
         <v>Passed</v>
       </c>
       <c r="K260">
-        <v>169</v>
+        <v>267</v>
       </c>
       <c r="L260" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10311,7 +10311,7 @@
         <v>Passed</v>
       </c>
       <c r="K261">
-        <v>159</v>
+        <v>185</v>
       </c>
       <c r="L261" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10349,7 +10349,7 @@
         <v>Passed</v>
       </c>
       <c r="K262">
-        <v>311</v>
+        <v>379</v>
       </c>
       <c r="L262" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10387,7 +10387,7 @@
         <v>Passed</v>
       </c>
       <c r="K263">
-        <v>275</v>
+        <v>258</v>
       </c>
       <c r="L263" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10425,7 +10425,7 @@
         <v>Passed</v>
       </c>
       <c r="K264">
-        <v>180</v>
+        <v>227</v>
       </c>
       <c r="L264" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10463,7 +10463,7 @@
         <v>Passed</v>
       </c>
       <c r="K265">
-        <v>250</v>
+        <v>279</v>
       </c>
       <c r="L265" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10501,7 +10501,7 @@
         <v>Passed</v>
       </c>
       <c r="K266">
-        <v>233</v>
+        <v>319</v>
       </c>
       <c r="L266" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10539,7 +10539,7 @@
         <v>Passed</v>
       </c>
       <c r="K267">
-        <v>385</v>
+        <v>315</v>
       </c>
       <c r="L267" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10577,7 +10577,7 @@
         <v>Passed</v>
       </c>
       <c r="K268">
-        <v>243</v>
+        <v>373</v>
       </c>
       <c r="L268" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10615,7 +10615,7 @@
         <v>Passed</v>
       </c>
       <c r="K269">
-        <v>288</v>
+        <v>356</v>
       </c>
       <c r="L269" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10653,7 +10653,7 @@
         <v>Passed</v>
       </c>
       <c r="K270">
-        <v>232</v>
+        <v>207</v>
       </c>
       <c r="L270" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10691,7 +10691,7 @@
         <v>Passed</v>
       </c>
       <c r="K271">
-        <v>168</v>
+        <v>373</v>
       </c>
       <c r="L271" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10729,7 +10729,7 @@
         <v>Passed</v>
       </c>
       <c r="K272">
-        <v>203</v>
+        <v>290</v>
       </c>
       <c r="L272" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10767,7 +10767,7 @@
         <v>Passed</v>
       </c>
       <c r="K273">
-        <v>186</v>
+        <v>159</v>
       </c>
       <c r="L273" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10805,7 +10805,7 @@
         <v>Passed</v>
       </c>
       <c r="K274">
-        <v>199</v>
+        <v>155</v>
       </c>
       <c r="L274" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10843,7 +10843,7 @@
         <v>Passed</v>
       </c>
       <c r="K275">
-        <v>378</v>
+        <v>386</v>
       </c>
       <c r="L275" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10881,7 +10881,7 @@
         <v>Passed</v>
       </c>
       <c r="K276">
-        <v>378</v>
+        <v>387</v>
       </c>
       <c r="L276" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10919,7 +10919,7 @@
         <v>Passed</v>
       </c>
       <c r="K277">
-        <v>316</v>
+        <v>160</v>
       </c>
       <c r="L277" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10957,7 +10957,7 @@
         <v>Passed</v>
       </c>
       <c r="K278">
-        <v>210</v>
+        <v>365</v>
       </c>
       <c r="L278" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10995,7 +10995,7 @@
         <v>Passed</v>
       </c>
       <c r="K279">
-        <v>249</v>
+        <v>308</v>
       </c>
       <c r="L279" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11033,7 +11033,7 @@
         <v>Passed</v>
       </c>
       <c r="K280">
-        <v>381</v>
+        <v>177</v>
       </c>
       <c r="L280" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11071,7 +11071,7 @@
         <v>Passed</v>
       </c>
       <c r="K281">
-        <v>260</v>
+        <v>391</v>
       </c>
       <c r="L281" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11109,7 +11109,7 @@
         <v>Passed</v>
       </c>
       <c r="K282">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="L282" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11147,7 +11147,7 @@
         <v>Passed</v>
       </c>
       <c r="K283">
-        <v>178</v>
+        <v>191</v>
       </c>
       <c r="L283" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11185,7 +11185,7 @@
         <v>Passed</v>
       </c>
       <c r="K284">
-        <v>382</v>
+        <v>165</v>
       </c>
       <c r="L284" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11223,7 +11223,7 @@
         <v>Passed</v>
       </c>
       <c r="K285">
-        <v>183</v>
+        <v>196</v>
       </c>
       <c r="L285" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11261,7 +11261,7 @@
         <v>Passed</v>
       </c>
       <c r="K286">
-        <v>278</v>
+        <v>386</v>
       </c>
       <c r="L286" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11299,7 +11299,7 @@
         <v>Passed</v>
       </c>
       <c r="K287">
-        <v>173</v>
+        <v>246</v>
       </c>
       <c r="L287" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11337,7 +11337,7 @@
         <v>Passed</v>
       </c>
       <c r="K288">
-        <v>164</v>
+        <v>196</v>
       </c>
       <c r="L288" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11375,7 +11375,7 @@
         <v>Passed</v>
       </c>
       <c r="K289">
-        <v>302</v>
+        <v>322</v>
       </c>
       <c r="L289" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11413,7 +11413,7 @@
         <v>Passed</v>
       </c>
       <c r="K290">
-        <v>290</v>
+        <v>193</v>
       </c>
       <c r="L290" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11451,7 +11451,7 @@
         <v>Passed</v>
       </c>
       <c r="K291">
-        <v>242</v>
+        <v>269</v>
       </c>
       <c r="L291" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11489,7 +11489,7 @@
         <v>Passed</v>
       </c>
       <c r="K292">
-        <v>390</v>
+        <v>372</v>
       </c>
       <c r="L292" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11527,7 +11527,7 @@
         <v>Passed</v>
       </c>
       <c r="K293">
-        <v>253</v>
+        <v>293</v>
       </c>
       <c r="L293" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11565,7 +11565,7 @@
         <v>Passed</v>
       </c>
       <c r="K294">
-        <v>203</v>
+        <v>233</v>
       </c>
       <c r="L294" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11603,7 +11603,7 @@
         <v>Passed</v>
       </c>
       <c r="K295">
-        <v>379</v>
+        <v>338</v>
       </c>
       <c r="L295" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11641,7 +11641,7 @@
         <v>Passed</v>
       </c>
       <c r="K296">
-        <v>174</v>
+        <v>296</v>
       </c>
       <c r="L296" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11679,7 +11679,7 @@
         <v>Passed</v>
       </c>
       <c r="K297">
-        <v>357</v>
+        <v>204</v>
       </c>
       <c r="L297" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11717,7 +11717,7 @@
         <v>Passed</v>
       </c>
       <c r="K298">
-        <v>178</v>
+        <v>262</v>
       </c>
       <c r="L298" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11755,7 +11755,7 @@
         <v>Passed</v>
       </c>
       <c r="K299">
-        <v>342</v>
+        <v>168</v>
       </c>
       <c r="L299" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11793,7 +11793,7 @@
         <v>Passed</v>
       </c>
       <c r="K300">
-        <v>178</v>
+        <v>303</v>
       </c>
       <c r="L300" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11831,7 +11831,7 @@
         <v>Passed</v>
       </c>
       <c r="K301">
-        <v>364</v>
+        <v>151</v>
       </c>
       <c r="L301" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>

</xml_diff>

<commit_message>
feat: full 1400px desktop web dashboard layout and 1-click Demo Login page
</commit_message>
<xml_diff>
--- a/EventSphere_Appium_Mobile_300_Report.xlsx
+++ b/EventSphere_Appium_Mobile_300_Report.xlsx
@@ -469,7 +469,7 @@
         <v>Passed</v>
       </c>
       <c r="K2">
-        <v>187</v>
+        <v>379</v>
       </c>
       <c r="L2" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -507,7 +507,7 @@
         <v>Passed</v>
       </c>
       <c r="K3">
-        <v>299</v>
+        <v>198</v>
       </c>
       <c r="L3" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -545,7 +545,7 @@
         <v>Passed</v>
       </c>
       <c r="K4">
-        <v>398</v>
+        <v>170</v>
       </c>
       <c r="L4" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -583,7 +583,7 @@
         <v>Passed</v>
       </c>
       <c r="K5">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="L5" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -621,7 +621,7 @@
         <v>Passed</v>
       </c>
       <c r="K6">
-        <v>151</v>
+        <v>267</v>
       </c>
       <c r="L6" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -659,7 +659,7 @@
         <v>Passed</v>
       </c>
       <c r="K7">
-        <v>232</v>
+        <v>386</v>
       </c>
       <c r="L7" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -697,7 +697,7 @@
         <v>Passed</v>
       </c>
       <c r="K8">
-        <v>200</v>
+        <v>208</v>
       </c>
       <c r="L8" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -735,7 +735,7 @@
         <v>Passed</v>
       </c>
       <c r="K9">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="L9" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -773,7 +773,7 @@
         <v>Passed</v>
       </c>
       <c r="K10">
-        <v>198</v>
+        <v>162</v>
       </c>
       <c r="L10" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -811,7 +811,7 @@
         <v>Passed</v>
       </c>
       <c r="K11">
-        <v>350</v>
+        <v>334</v>
       </c>
       <c r="L11" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -849,7 +849,7 @@
         <v>Passed</v>
       </c>
       <c r="K12">
-        <v>377</v>
+        <v>264</v>
       </c>
       <c r="L12" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -887,7 +887,7 @@
         <v>Passed</v>
       </c>
       <c r="K13">
-        <v>256</v>
+        <v>186</v>
       </c>
       <c r="L13" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -925,7 +925,7 @@
         <v>Passed</v>
       </c>
       <c r="K14">
-        <v>157</v>
+        <v>211</v>
       </c>
       <c r="L14" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -963,7 +963,7 @@
         <v>Passed</v>
       </c>
       <c r="K15">
-        <v>353</v>
+        <v>221</v>
       </c>
       <c r="L15" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1001,7 +1001,7 @@
         <v>Passed</v>
       </c>
       <c r="K16">
-        <v>283</v>
+        <v>352</v>
       </c>
       <c r="L16" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1039,7 +1039,7 @@
         <v>Passed</v>
       </c>
       <c r="K17">
-        <v>326</v>
+        <v>222</v>
       </c>
       <c r="L17" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1077,7 +1077,7 @@
         <v>Passed</v>
       </c>
       <c r="K18">
-        <v>290</v>
+        <v>156</v>
       </c>
       <c r="L18" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1115,7 +1115,7 @@
         <v>Passed</v>
       </c>
       <c r="K19">
-        <v>194</v>
+        <v>268</v>
       </c>
       <c r="L19" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1153,7 +1153,7 @@
         <v>Passed</v>
       </c>
       <c r="K20">
-        <v>215</v>
+        <v>252</v>
       </c>
       <c r="L20" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1191,7 +1191,7 @@
         <v>Passed</v>
       </c>
       <c r="K21">
-        <v>282</v>
+        <v>214</v>
       </c>
       <c r="L21" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1229,7 +1229,7 @@
         <v>Passed</v>
       </c>
       <c r="K22">
-        <v>155</v>
+        <v>240</v>
       </c>
       <c r="L22" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1267,7 +1267,7 @@
         <v>Passed</v>
       </c>
       <c r="K23">
-        <v>159</v>
+        <v>205</v>
       </c>
       <c r="L23" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1305,7 +1305,7 @@
         <v>Passed</v>
       </c>
       <c r="K24">
-        <v>269</v>
+        <v>218</v>
       </c>
       <c r="L24" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1343,7 +1343,7 @@
         <v>Passed</v>
       </c>
       <c r="K25">
-        <v>376</v>
+        <v>385</v>
       </c>
       <c r="L25" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1381,7 +1381,7 @@
         <v>Passed</v>
       </c>
       <c r="K26">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="L26" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1419,7 +1419,7 @@
         <v>Passed</v>
       </c>
       <c r="K27">
-        <v>293</v>
+        <v>346</v>
       </c>
       <c r="L27" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1457,7 +1457,7 @@
         <v>Passed</v>
       </c>
       <c r="K28">
-        <v>377</v>
+        <v>208</v>
       </c>
       <c r="L28" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1495,7 +1495,7 @@
         <v>Passed</v>
       </c>
       <c r="K29">
-        <v>293</v>
+        <v>392</v>
       </c>
       <c r="L29" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1533,7 +1533,7 @@
         <v>Passed</v>
       </c>
       <c r="K30">
-        <v>227</v>
+        <v>172</v>
       </c>
       <c r="L30" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1571,7 +1571,7 @@
         <v>Passed</v>
       </c>
       <c r="K31">
-        <v>270</v>
+        <v>329</v>
       </c>
       <c r="L31" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1609,7 +1609,7 @@
         <v>Passed</v>
       </c>
       <c r="K32">
-        <v>273</v>
+        <v>284</v>
       </c>
       <c r="L32" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1647,7 +1647,7 @@
         <v>Passed</v>
       </c>
       <c r="K33">
-        <v>303</v>
+        <v>217</v>
       </c>
       <c r="L33" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1685,7 +1685,7 @@
         <v>Passed</v>
       </c>
       <c r="K34">
-        <v>311</v>
+        <v>361</v>
       </c>
       <c r="L34" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1723,7 +1723,7 @@
         <v>Passed</v>
       </c>
       <c r="K35">
-        <v>200</v>
+        <v>349</v>
       </c>
       <c r="L35" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1761,7 +1761,7 @@
         <v>Passed</v>
       </c>
       <c r="K36">
-        <v>301</v>
+        <v>381</v>
       </c>
       <c r="L36" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1799,7 +1799,7 @@
         <v>Passed</v>
       </c>
       <c r="K37">
-        <v>380</v>
+        <v>202</v>
       </c>
       <c r="L37" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1837,7 +1837,7 @@
         <v>Passed</v>
       </c>
       <c r="K38">
-        <v>218</v>
+        <v>332</v>
       </c>
       <c r="L38" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1875,7 +1875,7 @@
         <v>Passed</v>
       </c>
       <c r="K39">
-        <v>230</v>
+        <v>398</v>
       </c>
       <c r="L39" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1913,7 +1913,7 @@
         <v>Passed</v>
       </c>
       <c r="K40">
-        <v>269</v>
+        <v>157</v>
       </c>
       <c r="L40" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1951,7 +1951,7 @@
         <v>Passed</v>
       </c>
       <c r="K41">
-        <v>316</v>
+        <v>369</v>
       </c>
       <c r="L41" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1989,7 +1989,7 @@
         <v>Passed</v>
       </c>
       <c r="K42">
-        <v>330</v>
+        <v>346</v>
       </c>
       <c r="L42" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2027,7 +2027,7 @@
         <v>Passed</v>
       </c>
       <c r="K43">
-        <v>381</v>
+        <v>183</v>
       </c>
       <c r="L43" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2065,7 +2065,7 @@
         <v>Passed</v>
       </c>
       <c r="K44">
-        <v>303</v>
+        <v>239</v>
       </c>
       <c r="L44" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2103,7 +2103,7 @@
         <v>Passed</v>
       </c>
       <c r="K45">
-        <v>396</v>
+        <v>399</v>
       </c>
       <c r="L45" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2141,7 +2141,7 @@
         <v>Passed</v>
       </c>
       <c r="K46">
-        <v>266</v>
+        <v>198</v>
       </c>
       <c r="L46" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2179,7 +2179,7 @@
         <v>Passed</v>
       </c>
       <c r="K47">
-        <v>253</v>
+        <v>371</v>
       </c>
       <c r="L47" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2217,7 +2217,7 @@
         <v>Passed</v>
       </c>
       <c r="K48">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="L48" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2255,7 +2255,7 @@
         <v>Passed</v>
       </c>
       <c r="K49">
-        <v>323</v>
+        <v>182</v>
       </c>
       <c r="L49" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2293,7 +2293,7 @@
         <v>Passed</v>
       </c>
       <c r="K50">
-        <v>268</v>
+        <v>348</v>
       </c>
       <c r="L50" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2331,7 +2331,7 @@
         <v>Passed</v>
       </c>
       <c r="K51">
-        <v>379</v>
+        <v>385</v>
       </c>
       <c r="L51" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2369,7 +2369,7 @@
         <v>Passed</v>
       </c>
       <c r="K52">
-        <v>150</v>
+        <v>355</v>
       </c>
       <c r="L52" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2407,7 +2407,7 @@
         <v>Passed</v>
       </c>
       <c r="K53">
-        <v>191</v>
+        <v>298</v>
       </c>
       <c r="L53" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2445,7 +2445,7 @@
         <v>Passed</v>
       </c>
       <c r="K54">
-        <v>294</v>
+        <v>355</v>
       </c>
       <c r="L54" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2483,7 +2483,7 @@
         <v>Passed</v>
       </c>
       <c r="K55">
-        <v>281</v>
+        <v>261</v>
       </c>
       <c r="L55" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2521,7 +2521,7 @@
         <v>Passed</v>
       </c>
       <c r="K56">
-        <v>198</v>
+        <v>264</v>
       </c>
       <c r="L56" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2559,7 +2559,7 @@
         <v>Passed</v>
       </c>
       <c r="K57">
-        <v>153</v>
+        <v>166</v>
       </c>
       <c r="L57" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2597,7 +2597,7 @@
         <v>Passed</v>
       </c>
       <c r="K58">
-        <v>320</v>
+        <v>199</v>
       </c>
       <c r="L58" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2635,7 +2635,7 @@
         <v>Passed</v>
       </c>
       <c r="K59">
-        <v>158</v>
+        <v>225</v>
       </c>
       <c r="L59" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2673,7 +2673,7 @@
         <v>Passed</v>
       </c>
       <c r="K60">
-        <v>374</v>
+        <v>239</v>
       </c>
       <c r="L60" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2711,7 +2711,7 @@
         <v>Passed</v>
       </c>
       <c r="K61">
-        <v>301</v>
+        <v>328</v>
       </c>
       <c r="L61" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2749,7 +2749,7 @@
         <v>Passed</v>
       </c>
       <c r="K62">
-        <v>195</v>
+        <v>275</v>
       </c>
       <c r="L62" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2787,7 +2787,7 @@
         <v>Passed</v>
       </c>
       <c r="K63">
-        <v>226</v>
+        <v>280</v>
       </c>
       <c r="L63" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2825,7 +2825,7 @@
         <v>Passed</v>
       </c>
       <c r="K64">
-        <v>370</v>
+        <v>196</v>
       </c>
       <c r="L64" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2863,7 +2863,7 @@
         <v>Passed</v>
       </c>
       <c r="K65">
-        <v>335</v>
+        <v>211</v>
       </c>
       <c r="L65" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2901,7 +2901,7 @@
         <v>Passed</v>
       </c>
       <c r="K66">
-        <v>310</v>
+        <v>339</v>
       </c>
       <c r="L66" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2939,7 +2939,7 @@
         <v>Passed</v>
       </c>
       <c r="K67">
-        <v>310</v>
+        <v>251</v>
       </c>
       <c r="L67" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2977,7 +2977,7 @@
         <v>Passed</v>
       </c>
       <c r="K68">
-        <v>171</v>
+        <v>201</v>
       </c>
       <c r="L68" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3015,7 +3015,7 @@
         <v>Passed</v>
       </c>
       <c r="K69">
-        <v>199</v>
+        <v>389</v>
       </c>
       <c r="L69" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3053,7 +3053,7 @@
         <v>Passed</v>
       </c>
       <c r="K70">
-        <v>189</v>
+        <v>167</v>
       </c>
       <c r="L70" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3091,7 +3091,7 @@
         <v>Passed</v>
       </c>
       <c r="K71">
-        <v>226</v>
+        <v>366</v>
       </c>
       <c r="L71" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3129,7 +3129,7 @@
         <v>Passed</v>
       </c>
       <c r="K72">
-        <v>269</v>
+        <v>166</v>
       </c>
       <c r="L72" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3167,7 +3167,7 @@
         <v>Passed</v>
       </c>
       <c r="K73">
-        <v>264</v>
+        <v>356</v>
       </c>
       <c r="L73" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3205,7 +3205,7 @@
         <v>Passed</v>
       </c>
       <c r="K74">
-        <v>328</v>
+        <v>312</v>
       </c>
       <c r="L74" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3243,7 +3243,7 @@
         <v>Passed</v>
       </c>
       <c r="K75">
-        <v>168</v>
+        <v>223</v>
       </c>
       <c r="L75" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3281,7 +3281,7 @@
         <v>Passed</v>
       </c>
       <c r="K76">
-        <v>236</v>
+        <v>158</v>
       </c>
       <c r="L76" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3319,7 +3319,7 @@
         <v>Passed</v>
       </c>
       <c r="K77">
-        <v>383</v>
+        <v>316</v>
       </c>
       <c r="L77" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3357,7 +3357,7 @@
         <v>Passed</v>
       </c>
       <c r="K78">
-        <v>205</v>
+        <v>251</v>
       </c>
       <c r="L78" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3395,7 +3395,7 @@
         <v>Passed</v>
       </c>
       <c r="K79">
-        <v>208</v>
+        <v>153</v>
       </c>
       <c r="L79" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3433,7 +3433,7 @@
         <v>Passed</v>
       </c>
       <c r="K80">
-        <v>393</v>
+        <v>174</v>
       </c>
       <c r="L80" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3471,7 +3471,7 @@
         <v>Passed</v>
       </c>
       <c r="K81">
-        <v>387</v>
+        <v>209</v>
       </c>
       <c r="L81" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3509,7 +3509,7 @@
         <v>Passed</v>
       </c>
       <c r="K82">
-        <v>336</v>
+        <v>293</v>
       </c>
       <c r="L82" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3547,7 +3547,7 @@
         <v>Passed</v>
       </c>
       <c r="K83">
-        <v>280</v>
+        <v>335</v>
       </c>
       <c r="L83" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3585,7 +3585,7 @@
         <v>Passed</v>
       </c>
       <c r="K84">
-        <v>299</v>
+        <v>205</v>
       </c>
       <c r="L84" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3623,7 +3623,7 @@
         <v>Passed</v>
       </c>
       <c r="K85">
-        <v>270</v>
+        <v>244</v>
       </c>
       <c r="L85" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3661,7 +3661,7 @@
         <v>Passed</v>
       </c>
       <c r="K86">
-        <v>203</v>
+        <v>168</v>
       </c>
       <c r="L86" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3699,7 +3699,7 @@
         <v>Passed</v>
       </c>
       <c r="K87">
-        <v>321</v>
+        <v>206</v>
       </c>
       <c r="L87" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3737,7 +3737,7 @@
         <v>Passed</v>
       </c>
       <c r="K88">
-        <v>289</v>
+        <v>314</v>
       </c>
       <c r="L88" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3775,7 +3775,7 @@
         <v>Passed</v>
       </c>
       <c r="K89">
-        <v>174</v>
+        <v>337</v>
       </c>
       <c r="L89" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3813,7 +3813,7 @@
         <v>Passed</v>
       </c>
       <c r="K90">
-        <v>306</v>
+        <v>379</v>
       </c>
       <c r="L90" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3851,7 +3851,7 @@
         <v>Passed</v>
       </c>
       <c r="K91">
-        <v>262</v>
+        <v>174</v>
       </c>
       <c r="L91" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3889,7 +3889,7 @@
         <v>Passed</v>
       </c>
       <c r="K92">
-        <v>339</v>
+        <v>185</v>
       </c>
       <c r="L92" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3927,7 +3927,7 @@
         <v>Passed</v>
       </c>
       <c r="K93">
-        <v>355</v>
+        <v>384</v>
       </c>
       <c r="L93" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3965,7 +3965,7 @@
         <v>Passed</v>
       </c>
       <c r="K94">
-        <v>398</v>
+        <v>339</v>
       </c>
       <c r="L94" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4003,7 +4003,7 @@
         <v>Passed</v>
       </c>
       <c r="K95">
-        <v>385</v>
+        <v>399</v>
       </c>
       <c r="L95" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4041,7 +4041,7 @@
         <v>Passed</v>
       </c>
       <c r="K96">
-        <v>364</v>
+        <v>334</v>
       </c>
       <c r="L96" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4079,7 +4079,7 @@
         <v>Passed</v>
       </c>
       <c r="K97">
-        <v>207</v>
+        <v>246</v>
       </c>
       <c r="L97" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4117,7 +4117,7 @@
         <v>Passed</v>
       </c>
       <c r="K98">
-        <v>378</v>
+        <v>269</v>
       </c>
       <c r="L98" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4155,7 +4155,7 @@
         <v>Passed</v>
       </c>
       <c r="K99">
-        <v>249</v>
+        <v>229</v>
       </c>
       <c r="L99" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4193,7 +4193,7 @@
         <v>Passed</v>
       </c>
       <c r="K100">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="L100" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4231,7 +4231,7 @@
         <v>Passed</v>
       </c>
       <c r="K101">
-        <v>343</v>
+        <v>288</v>
       </c>
       <c r="L101" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4269,7 +4269,7 @@
         <v>Passed</v>
       </c>
       <c r="K102">
-        <v>195</v>
+        <v>175</v>
       </c>
       <c r="L102" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4307,7 +4307,7 @@
         <v>Passed</v>
       </c>
       <c r="K103">
-        <v>329</v>
+        <v>273</v>
       </c>
       <c r="L103" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4345,7 +4345,7 @@
         <v>Passed</v>
       </c>
       <c r="K104">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="L104" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4383,7 +4383,7 @@
         <v>Passed</v>
       </c>
       <c r="K105">
-        <v>189</v>
+        <v>280</v>
       </c>
       <c r="L105" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4421,7 +4421,7 @@
         <v>Passed</v>
       </c>
       <c r="K106">
-        <v>293</v>
+        <v>278</v>
       </c>
       <c r="L106" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4459,7 +4459,7 @@
         <v>Passed</v>
       </c>
       <c r="K107">
-        <v>165</v>
+        <v>356</v>
       </c>
       <c r="L107" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4497,7 +4497,7 @@
         <v>Passed</v>
       </c>
       <c r="K108">
-        <v>373</v>
+        <v>220</v>
       </c>
       <c r="L108" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4535,7 +4535,7 @@
         <v>Passed</v>
       </c>
       <c r="K109">
-        <v>285</v>
+        <v>360</v>
       </c>
       <c r="L109" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4573,7 +4573,7 @@
         <v>Passed</v>
       </c>
       <c r="K110">
-        <v>288</v>
+        <v>165</v>
       </c>
       <c r="L110" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4611,7 +4611,7 @@
         <v>Passed</v>
       </c>
       <c r="K111">
-        <v>344</v>
+        <v>194</v>
       </c>
       <c r="L111" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4649,7 +4649,7 @@
         <v>Passed</v>
       </c>
       <c r="K112">
-        <v>316</v>
+        <v>287</v>
       </c>
       <c r="L112" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4687,7 +4687,7 @@
         <v>Passed</v>
       </c>
       <c r="K113">
-        <v>245</v>
+        <v>181</v>
       </c>
       <c r="L113" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4725,7 +4725,7 @@
         <v>Passed</v>
       </c>
       <c r="K114">
-        <v>279</v>
+        <v>198</v>
       </c>
       <c r="L114" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4763,7 +4763,7 @@
         <v>Passed</v>
       </c>
       <c r="K115">
-        <v>159</v>
+        <v>299</v>
       </c>
       <c r="L115" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4801,7 +4801,7 @@
         <v>Passed</v>
       </c>
       <c r="K116">
-        <v>360</v>
+        <v>245</v>
       </c>
       <c r="L116" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4839,7 +4839,7 @@
         <v>Passed</v>
       </c>
       <c r="K117">
-        <v>266</v>
+        <v>189</v>
       </c>
       <c r="L117" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4877,7 +4877,7 @@
         <v>Passed</v>
       </c>
       <c r="K118">
-        <v>240</v>
+        <v>381</v>
       </c>
       <c r="L118" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4915,7 +4915,7 @@
         <v>Passed</v>
       </c>
       <c r="K119">
-        <v>367</v>
+        <v>307</v>
       </c>
       <c r="L119" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4953,7 +4953,7 @@
         <v>Passed</v>
       </c>
       <c r="K120">
-        <v>358</v>
+        <v>299</v>
       </c>
       <c r="L120" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4991,7 +4991,7 @@
         <v>Passed</v>
       </c>
       <c r="K121">
-        <v>378</v>
+        <v>251</v>
       </c>
       <c r="L121" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5029,7 +5029,7 @@
         <v>Passed</v>
       </c>
       <c r="K122">
-        <v>361</v>
+        <v>240</v>
       </c>
       <c r="L122" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5067,7 +5067,7 @@
         <v>Passed</v>
       </c>
       <c r="K123">
-        <v>181</v>
+        <v>225</v>
       </c>
       <c r="L123" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5105,7 +5105,7 @@
         <v>Passed</v>
       </c>
       <c r="K124">
-        <v>279</v>
+        <v>394</v>
       </c>
       <c r="L124" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5143,7 +5143,7 @@
         <v>Passed</v>
       </c>
       <c r="K125">
-        <v>264</v>
+        <v>363</v>
       </c>
       <c r="L125" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5181,7 +5181,7 @@
         <v>Passed</v>
       </c>
       <c r="K126">
-        <v>326</v>
+        <v>284</v>
       </c>
       <c r="L126" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5219,7 +5219,7 @@
         <v>Passed</v>
       </c>
       <c r="K127">
-        <v>389</v>
+        <v>182</v>
       </c>
       <c r="L127" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5257,7 +5257,7 @@
         <v>Passed</v>
       </c>
       <c r="K128">
-        <v>329</v>
+        <v>307</v>
       </c>
       <c r="L128" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5295,7 +5295,7 @@
         <v>Passed</v>
       </c>
       <c r="K129">
-        <v>356</v>
+        <v>153</v>
       </c>
       <c r="L129" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5333,7 +5333,7 @@
         <v>Passed</v>
       </c>
       <c r="K130">
-        <v>357</v>
+        <v>272</v>
       </c>
       <c r="L130" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5371,7 +5371,7 @@
         <v>Passed</v>
       </c>
       <c r="K131">
-        <v>378</v>
+        <v>188</v>
       </c>
       <c r="L131" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5409,7 +5409,7 @@
         <v>Passed</v>
       </c>
       <c r="K132">
-        <v>321</v>
+        <v>213</v>
       </c>
       <c r="L132" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5447,7 +5447,7 @@
         <v>Passed</v>
       </c>
       <c r="K133">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="L133" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5485,7 +5485,7 @@
         <v>Passed</v>
       </c>
       <c r="K134">
-        <v>345</v>
+        <v>238</v>
       </c>
       <c r="L134" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5523,7 +5523,7 @@
         <v>Passed</v>
       </c>
       <c r="K135">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="L135" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5561,7 +5561,7 @@
         <v>Passed</v>
       </c>
       <c r="K136">
-        <v>150</v>
+        <v>183</v>
       </c>
       <c r="L136" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5599,7 +5599,7 @@
         <v>Passed</v>
       </c>
       <c r="K137">
-        <v>310</v>
+        <v>159</v>
       </c>
       <c r="L137" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5637,7 +5637,7 @@
         <v>Passed</v>
       </c>
       <c r="K138">
-        <v>299</v>
+        <v>189</v>
       </c>
       <c r="L138" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5675,7 +5675,7 @@
         <v>Passed</v>
       </c>
       <c r="K139">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="L139" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5713,7 +5713,7 @@
         <v>Passed</v>
       </c>
       <c r="K140">
-        <v>239</v>
+        <v>304</v>
       </c>
       <c r="L140" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5751,7 +5751,7 @@
         <v>Passed</v>
       </c>
       <c r="K141">
-        <v>291</v>
+        <v>284</v>
       </c>
       <c r="L141" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5789,7 +5789,7 @@
         <v>Passed</v>
       </c>
       <c r="K142">
-        <v>338</v>
+        <v>230</v>
       </c>
       <c r="L142" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5827,7 +5827,7 @@
         <v>Passed</v>
       </c>
       <c r="K143">
-        <v>276</v>
+        <v>258</v>
       </c>
       <c r="L143" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5865,7 +5865,7 @@
         <v>Passed</v>
       </c>
       <c r="K144">
-        <v>182</v>
+        <v>305</v>
       </c>
       <c r="L144" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5903,7 +5903,7 @@
         <v>Passed</v>
       </c>
       <c r="K145">
-        <v>261</v>
+        <v>373</v>
       </c>
       <c r="L145" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5941,7 +5941,7 @@
         <v>Passed</v>
       </c>
       <c r="K146">
-        <v>184</v>
+        <v>387</v>
       </c>
       <c r="L146" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5979,7 +5979,7 @@
         <v>Passed</v>
       </c>
       <c r="K147">
-        <v>322</v>
+        <v>181</v>
       </c>
       <c r="L147" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6017,7 +6017,7 @@
         <v>Passed</v>
       </c>
       <c r="K148">
-        <v>174</v>
+        <v>341</v>
       </c>
       <c r="L148" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6055,7 +6055,7 @@
         <v>Passed</v>
       </c>
       <c r="K149">
-        <v>323</v>
+        <v>168</v>
       </c>
       <c r="L149" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6093,7 +6093,7 @@
         <v>Passed</v>
       </c>
       <c r="K150">
-        <v>155</v>
+        <v>270</v>
       </c>
       <c r="L150" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6131,7 +6131,7 @@
         <v>Passed</v>
       </c>
       <c r="K151">
-        <v>348</v>
+        <v>267</v>
       </c>
       <c r="L151" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6169,7 +6169,7 @@
         <v>Passed</v>
       </c>
       <c r="K152">
-        <v>169</v>
+        <v>343</v>
       </c>
       <c r="L152" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6207,7 +6207,7 @@
         <v>Passed</v>
       </c>
       <c r="K153">
-        <v>206</v>
+        <v>331</v>
       </c>
       <c r="L153" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6245,7 +6245,7 @@
         <v>Passed</v>
       </c>
       <c r="K154">
-        <v>312</v>
+        <v>290</v>
       </c>
       <c r="L154" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6283,7 +6283,7 @@
         <v>Passed</v>
       </c>
       <c r="K155">
-        <v>345</v>
+        <v>305</v>
       </c>
       <c r="L155" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6321,7 +6321,7 @@
         <v>Passed</v>
       </c>
       <c r="K156">
-        <v>340</v>
+        <v>304</v>
       </c>
       <c r="L156" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6359,7 +6359,7 @@
         <v>Passed</v>
       </c>
       <c r="K157">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="L157" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6397,7 +6397,7 @@
         <v>Passed</v>
       </c>
       <c r="K158">
-        <v>155</v>
+        <v>387</v>
       </c>
       <c r="L158" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6435,7 +6435,7 @@
         <v>Passed</v>
       </c>
       <c r="K159">
-        <v>203</v>
+        <v>386</v>
       </c>
       <c r="L159" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6473,7 +6473,7 @@
         <v>Passed</v>
       </c>
       <c r="K160">
-        <v>243</v>
+        <v>273</v>
       </c>
       <c r="L160" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6511,7 +6511,7 @@
         <v>Passed</v>
       </c>
       <c r="K161">
-        <v>373</v>
+        <v>363</v>
       </c>
       <c r="L161" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6549,7 +6549,7 @@
         <v>Passed</v>
       </c>
       <c r="K162">
-        <v>249</v>
+        <v>332</v>
       </c>
       <c r="L162" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6587,7 +6587,7 @@
         <v>Passed</v>
       </c>
       <c r="K163">
-        <v>378</v>
+        <v>250</v>
       </c>
       <c r="L163" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6625,7 +6625,7 @@
         <v>Passed</v>
       </c>
       <c r="K164">
-        <v>285</v>
+        <v>369</v>
       </c>
       <c r="L164" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6663,7 +6663,7 @@
         <v>Passed</v>
       </c>
       <c r="K165">
-        <v>160</v>
+        <v>289</v>
       </c>
       <c r="L165" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6701,7 +6701,7 @@
         <v>Passed</v>
       </c>
       <c r="K166">
-        <v>204</v>
+        <v>366</v>
       </c>
       <c r="L166" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6739,7 +6739,7 @@
         <v>Passed</v>
       </c>
       <c r="K167">
-        <v>182</v>
+        <v>201</v>
       </c>
       <c r="L167" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6777,7 +6777,7 @@
         <v>Passed</v>
       </c>
       <c r="K168">
-        <v>217</v>
+        <v>342</v>
       </c>
       <c r="L168" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6815,7 +6815,7 @@
         <v>Passed</v>
       </c>
       <c r="K169">
-        <v>373</v>
+        <v>317</v>
       </c>
       <c r="L169" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6853,7 +6853,7 @@
         <v>Passed</v>
       </c>
       <c r="K170">
-        <v>215</v>
+        <v>291</v>
       </c>
       <c r="L170" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6891,7 +6891,7 @@
         <v>Passed</v>
       </c>
       <c r="K171">
-        <v>386</v>
+        <v>372</v>
       </c>
       <c r="L171" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6929,7 +6929,7 @@
         <v>Passed</v>
       </c>
       <c r="K172">
-        <v>230</v>
+        <v>183</v>
       </c>
       <c r="L172" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6967,7 +6967,7 @@
         <v>Passed</v>
       </c>
       <c r="K173">
-        <v>338</v>
+        <v>248</v>
       </c>
       <c r="L173" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7005,7 +7005,7 @@
         <v>Passed</v>
       </c>
       <c r="K174">
-        <v>278</v>
+        <v>257</v>
       </c>
       <c r="L174" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7043,7 +7043,7 @@
         <v>Passed</v>
       </c>
       <c r="K175">
-        <v>316</v>
+        <v>203</v>
       </c>
       <c r="L175" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7081,7 +7081,7 @@
         <v>Passed</v>
       </c>
       <c r="K176">
-        <v>304</v>
+        <v>312</v>
       </c>
       <c r="L176" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7119,7 +7119,7 @@
         <v>Passed</v>
       </c>
       <c r="K177">
-        <v>181</v>
+        <v>335</v>
       </c>
       <c r="L177" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7157,7 +7157,7 @@
         <v>Passed</v>
       </c>
       <c r="K178">
-        <v>155</v>
+        <v>299</v>
       </c>
       <c r="L178" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7195,7 +7195,7 @@
         <v>Passed</v>
       </c>
       <c r="K179">
-        <v>335</v>
+        <v>264</v>
       </c>
       <c r="L179" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7233,7 +7233,7 @@
         <v>Passed</v>
       </c>
       <c r="K180">
-        <v>214</v>
+        <v>324</v>
       </c>
       <c r="L180" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7271,7 +7271,7 @@
         <v>Passed</v>
       </c>
       <c r="K181">
-        <v>290</v>
+        <v>313</v>
       </c>
       <c r="L181" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7309,7 +7309,7 @@
         <v>Passed</v>
       </c>
       <c r="K182">
-        <v>153</v>
+        <v>337</v>
       </c>
       <c r="L182" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7347,7 +7347,7 @@
         <v>Passed</v>
       </c>
       <c r="K183">
-        <v>204</v>
+        <v>195</v>
       </c>
       <c r="L183" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7385,7 +7385,7 @@
         <v>Passed</v>
       </c>
       <c r="K184">
-        <v>311</v>
+        <v>277</v>
       </c>
       <c r="L184" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7423,7 +7423,7 @@
         <v>Passed</v>
       </c>
       <c r="K185">
-        <v>232</v>
+        <v>180</v>
       </c>
       <c r="L185" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7461,7 +7461,7 @@
         <v>Passed</v>
       </c>
       <c r="K186">
-        <v>172</v>
+        <v>297</v>
       </c>
       <c r="L186" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7499,7 +7499,7 @@
         <v>Passed</v>
       </c>
       <c r="K187">
-        <v>243</v>
+        <v>295</v>
       </c>
       <c r="L187" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7537,7 +7537,7 @@
         <v>Passed</v>
       </c>
       <c r="K188">
-        <v>281</v>
+        <v>306</v>
       </c>
       <c r="L188" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7575,7 +7575,7 @@
         <v>Passed</v>
       </c>
       <c r="K189">
-        <v>212</v>
+        <v>235</v>
       </c>
       <c r="L189" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7613,7 +7613,7 @@
         <v>Passed</v>
       </c>
       <c r="K190">
-        <v>279</v>
+        <v>186</v>
       </c>
       <c r="L190" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7651,7 +7651,7 @@
         <v>Passed</v>
       </c>
       <c r="K191">
-        <v>311</v>
+        <v>154</v>
       </c>
       <c r="L191" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7689,7 +7689,7 @@
         <v>Passed</v>
       </c>
       <c r="K192">
-        <v>344</v>
+        <v>170</v>
       </c>
       <c r="L192" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7727,7 +7727,7 @@
         <v>Passed</v>
       </c>
       <c r="K193">
-        <v>309</v>
+        <v>202</v>
       </c>
       <c r="L193" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7765,7 +7765,7 @@
         <v>Passed</v>
       </c>
       <c r="K194">
-        <v>306</v>
+        <v>355</v>
       </c>
       <c r="L194" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7803,7 +7803,7 @@
         <v>Passed</v>
       </c>
       <c r="K195">
-        <v>266</v>
+        <v>171</v>
       </c>
       <c r="L195" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7841,7 +7841,7 @@
         <v>Passed</v>
       </c>
       <c r="K196">
-        <v>338</v>
+        <v>248</v>
       </c>
       <c r="L196" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7879,7 +7879,7 @@
         <v>Passed</v>
       </c>
       <c r="K197">
-        <v>379</v>
+        <v>275</v>
       </c>
       <c r="L197" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7917,7 +7917,7 @@
         <v>Passed</v>
       </c>
       <c r="K198">
-        <v>226</v>
+        <v>291</v>
       </c>
       <c r="L198" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7955,7 +7955,7 @@
         <v>Passed</v>
       </c>
       <c r="K199">
-        <v>283</v>
+        <v>188</v>
       </c>
       <c r="L199" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7993,7 +7993,7 @@
         <v>Passed</v>
       </c>
       <c r="K200">
-        <v>368</v>
+        <v>348</v>
       </c>
       <c r="L200" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8031,7 +8031,7 @@
         <v>Passed</v>
       </c>
       <c r="K201">
-        <v>282</v>
+        <v>396</v>
       </c>
       <c r="L201" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8069,7 +8069,7 @@
         <v>Passed</v>
       </c>
       <c r="K202">
-        <v>276</v>
+        <v>379</v>
       </c>
       <c r="L202" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8107,7 +8107,7 @@
         <v>Passed</v>
       </c>
       <c r="K203">
-        <v>266</v>
+        <v>169</v>
       </c>
       <c r="L203" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8145,7 +8145,7 @@
         <v>Passed</v>
       </c>
       <c r="K204">
-        <v>361</v>
+        <v>237</v>
       </c>
       <c r="L204" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8183,7 +8183,7 @@
         <v>Passed</v>
       </c>
       <c r="K205">
-        <v>203</v>
+        <v>219</v>
       </c>
       <c r="L205" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8221,7 +8221,7 @@
         <v>Passed</v>
       </c>
       <c r="K206">
-        <v>222</v>
+        <v>385</v>
       </c>
       <c r="L206" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8259,7 +8259,7 @@
         <v>Passed</v>
       </c>
       <c r="K207">
-        <v>303</v>
+        <v>273</v>
       </c>
       <c r="L207" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8297,7 +8297,7 @@
         <v>Passed</v>
       </c>
       <c r="K208">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="L208" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8335,7 +8335,7 @@
         <v>Passed</v>
       </c>
       <c r="K209">
-        <v>318</v>
+        <v>281</v>
       </c>
       <c r="L209" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8373,7 +8373,7 @@
         <v>Passed</v>
       </c>
       <c r="K210">
-        <v>249</v>
+        <v>314</v>
       </c>
       <c r="L210" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8411,7 +8411,7 @@
         <v>Passed</v>
       </c>
       <c r="K211">
-        <v>319</v>
+        <v>254</v>
       </c>
       <c r="L211" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8449,7 +8449,7 @@
         <v>Passed</v>
       </c>
       <c r="K212">
-        <v>237</v>
+        <v>254</v>
       </c>
       <c r="L212" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8487,7 +8487,7 @@
         <v>Passed</v>
       </c>
       <c r="K213">
-        <v>243</v>
+        <v>363</v>
       </c>
       <c r="L213" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8525,7 +8525,7 @@
         <v>Passed</v>
       </c>
       <c r="K214">
-        <v>194</v>
+        <v>218</v>
       </c>
       <c r="L214" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8563,7 +8563,7 @@
         <v>Passed</v>
       </c>
       <c r="K215">
-        <v>233</v>
+        <v>180</v>
       </c>
       <c r="L215" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8601,7 +8601,7 @@
         <v>Passed</v>
       </c>
       <c r="K216">
-        <v>290</v>
+        <v>268</v>
       </c>
       <c r="L216" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8639,7 +8639,7 @@
         <v>Passed</v>
       </c>
       <c r="K217">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="L217" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8677,7 +8677,7 @@
         <v>Passed</v>
       </c>
       <c r="K218">
-        <v>321</v>
+        <v>286</v>
       </c>
       <c r="L218" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8715,7 +8715,7 @@
         <v>Passed</v>
       </c>
       <c r="K219">
-        <v>371</v>
+        <v>262</v>
       </c>
       <c r="L219" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8753,7 +8753,7 @@
         <v>Passed</v>
       </c>
       <c r="K220">
-        <v>228</v>
+        <v>300</v>
       </c>
       <c r="L220" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8791,7 +8791,7 @@
         <v>Passed</v>
       </c>
       <c r="K221">
-        <v>215</v>
+        <v>347</v>
       </c>
       <c r="L221" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8829,7 +8829,7 @@
         <v>Passed</v>
       </c>
       <c r="K222">
-        <v>399</v>
+        <v>254</v>
       </c>
       <c r="L222" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8867,7 +8867,7 @@
         <v>Passed</v>
       </c>
       <c r="K223">
-        <v>233</v>
+        <v>392</v>
       </c>
       <c r="L223" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8905,7 +8905,7 @@
         <v>Passed</v>
       </c>
       <c r="K224">
-        <v>393</v>
+        <v>310</v>
       </c>
       <c r="L224" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8943,7 +8943,7 @@
         <v>Passed</v>
       </c>
       <c r="K225">
-        <v>177</v>
+        <v>330</v>
       </c>
       <c r="L225" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8981,7 +8981,7 @@
         <v>Passed</v>
       </c>
       <c r="K226">
-        <v>232</v>
+        <v>394</v>
       </c>
       <c r="L226" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9019,7 +9019,7 @@
         <v>Passed</v>
       </c>
       <c r="K227">
-        <v>179</v>
+        <v>351</v>
       </c>
       <c r="L227" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9057,7 +9057,7 @@
         <v>Passed</v>
       </c>
       <c r="K228">
-        <v>371</v>
+        <v>182</v>
       </c>
       <c r="L228" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9095,7 +9095,7 @@
         <v>Passed</v>
       </c>
       <c r="K229">
-        <v>379</v>
+        <v>336</v>
       </c>
       <c r="L229" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9133,7 +9133,7 @@
         <v>Passed</v>
       </c>
       <c r="K230">
-        <v>162</v>
+        <v>206</v>
       </c>
       <c r="L230" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9171,7 +9171,7 @@
         <v>Passed</v>
       </c>
       <c r="K231">
-        <v>301</v>
+        <v>202</v>
       </c>
       <c r="L231" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9209,7 +9209,7 @@
         <v>Passed</v>
       </c>
       <c r="K232">
-        <v>292</v>
+        <v>362</v>
       </c>
       <c r="L232" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9247,7 +9247,7 @@
         <v>Passed</v>
       </c>
       <c r="K233">
-        <v>223</v>
+        <v>284</v>
       </c>
       <c r="L233" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9285,7 +9285,7 @@
         <v>Passed</v>
       </c>
       <c r="K234">
-        <v>209</v>
+        <v>164</v>
       </c>
       <c r="L234" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9323,7 +9323,7 @@
         <v>Passed</v>
       </c>
       <c r="K235">
-        <v>222</v>
+        <v>324</v>
       </c>
       <c r="L235" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9361,7 +9361,7 @@
         <v>Passed</v>
       </c>
       <c r="K236">
-        <v>271</v>
+        <v>364</v>
       </c>
       <c r="L236" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9399,7 +9399,7 @@
         <v>Passed</v>
       </c>
       <c r="K237">
-        <v>332</v>
+        <v>232</v>
       </c>
       <c r="L237" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9437,7 +9437,7 @@
         <v>Passed</v>
       </c>
       <c r="K238">
-        <v>190</v>
+        <v>395</v>
       </c>
       <c r="L238" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9475,7 +9475,7 @@
         <v>Passed</v>
       </c>
       <c r="K239">
-        <v>341</v>
+        <v>385</v>
       </c>
       <c r="L239" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9513,7 +9513,7 @@
         <v>Passed</v>
       </c>
       <c r="K240">
-        <v>150</v>
+        <v>305</v>
       </c>
       <c r="L240" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9551,7 +9551,7 @@
         <v>Passed</v>
       </c>
       <c r="K241">
-        <v>362</v>
+        <v>224</v>
       </c>
       <c r="L241" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9589,7 +9589,7 @@
         <v>Passed</v>
       </c>
       <c r="K242">
-        <v>263</v>
+        <v>298</v>
       </c>
       <c r="L242" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9627,7 +9627,7 @@
         <v>Passed</v>
       </c>
       <c r="K243">
-        <v>334</v>
+        <v>154</v>
       </c>
       <c r="L243" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9665,7 +9665,7 @@
         <v>Passed</v>
       </c>
       <c r="K244">
-        <v>308</v>
+        <v>399</v>
       </c>
       <c r="L244" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9703,7 +9703,7 @@
         <v>Passed</v>
       </c>
       <c r="K245">
-        <v>350</v>
+        <v>215</v>
       </c>
       <c r="L245" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9741,7 +9741,7 @@
         <v>Passed</v>
       </c>
       <c r="K246">
-        <v>328</v>
+        <v>336</v>
       </c>
       <c r="L246" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9779,7 +9779,7 @@
         <v>Passed</v>
       </c>
       <c r="K247">
-        <v>328</v>
+        <v>322</v>
       </c>
       <c r="L247" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9817,7 +9817,7 @@
         <v>Passed</v>
       </c>
       <c r="K248">
-        <v>293</v>
+        <v>159</v>
       </c>
       <c r="L248" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9855,7 +9855,7 @@
         <v>Passed</v>
       </c>
       <c r="K249">
-        <v>374</v>
+        <v>389</v>
       </c>
       <c r="L249" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9893,7 +9893,7 @@
         <v>Passed</v>
       </c>
       <c r="K250">
-        <v>310</v>
+        <v>318</v>
       </c>
       <c r="L250" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9931,7 +9931,7 @@
         <v>Passed</v>
       </c>
       <c r="K251">
-        <v>223</v>
+        <v>182</v>
       </c>
       <c r="L251" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9969,7 +9969,7 @@
         <v>Passed</v>
       </c>
       <c r="K252">
-        <v>293</v>
+        <v>304</v>
       </c>
       <c r="L252" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10007,7 +10007,7 @@
         <v>Passed</v>
       </c>
       <c r="K253">
-        <v>337</v>
+        <v>165</v>
       </c>
       <c r="L253" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10045,7 +10045,7 @@
         <v>Passed</v>
       </c>
       <c r="K254">
-        <v>221</v>
+        <v>384</v>
       </c>
       <c r="L254" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10083,7 +10083,7 @@
         <v>Passed</v>
       </c>
       <c r="K255">
-        <v>345</v>
+        <v>329</v>
       </c>
       <c r="L255" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10121,7 +10121,7 @@
         <v>Passed</v>
       </c>
       <c r="K256">
-        <v>292</v>
+        <v>157</v>
       </c>
       <c r="L256" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10159,7 +10159,7 @@
         <v>Passed</v>
       </c>
       <c r="K257">
-        <v>154</v>
+        <v>302</v>
       </c>
       <c r="L257" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10197,7 +10197,7 @@
         <v>Passed</v>
       </c>
       <c r="K258">
-        <v>377</v>
+        <v>219</v>
       </c>
       <c r="L258" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10235,7 +10235,7 @@
         <v>Passed</v>
       </c>
       <c r="K259">
-        <v>392</v>
+        <v>351</v>
       </c>
       <c r="L259" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10273,7 +10273,7 @@
         <v>Passed</v>
       </c>
       <c r="K260">
-        <v>267</v>
+        <v>346</v>
       </c>
       <c r="L260" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10311,7 +10311,7 @@
         <v>Passed</v>
       </c>
       <c r="K261">
-        <v>185</v>
+        <v>216</v>
       </c>
       <c r="L261" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10349,7 +10349,7 @@
         <v>Passed</v>
       </c>
       <c r="K262">
-        <v>379</v>
+        <v>286</v>
       </c>
       <c r="L262" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10387,7 +10387,7 @@
         <v>Passed</v>
       </c>
       <c r="K263">
-        <v>258</v>
+        <v>198</v>
       </c>
       <c r="L263" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10425,7 +10425,7 @@
         <v>Passed</v>
       </c>
       <c r="K264">
-        <v>227</v>
+        <v>358</v>
       </c>
       <c r="L264" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10463,7 +10463,7 @@
         <v>Passed</v>
       </c>
       <c r="K265">
-        <v>279</v>
+        <v>326</v>
       </c>
       <c r="L265" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10501,7 +10501,7 @@
         <v>Passed</v>
       </c>
       <c r="K266">
-        <v>319</v>
+        <v>360</v>
       </c>
       <c r="L266" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10539,7 +10539,7 @@
         <v>Passed</v>
       </c>
       <c r="K267">
-        <v>315</v>
+        <v>296</v>
       </c>
       <c r="L267" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10577,7 +10577,7 @@
         <v>Passed</v>
       </c>
       <c r="K268">
-        <v>373</v>
+        <v>168</v>
       </c>
       <c r="L268" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10615,7 +10615,7 @@
         <v>Passed</v>
       </c>
       <c r="K269">
-        <v>356</v>
+        <v>250</v>
       </c>
       <c r="L269" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10653,7 +10653,7 @@
         <v>Passed</v>
       </c>
       <c r="K270">
-        <v>207</v>
+        <v>163</v>
       </c>
       <c r="L270" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10691,7 +10691,7 @@
         <v>Passed</v>
       </c>
       <c r="K271">
-        <v>373</v>
+        <v>253</v>
       </c>
       <c r="L271" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10729,7 +10729,7 @@
         <v>Passed</v>
       </c>
       <c r="K272">
-        <v>290</v>
+        <v>327</v>
       </c>
       <c r="L272" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10767,7 +10767,7 @@
         <v>Passed</v>
       </c>
       <c r="K273">
-        <v>159</v>
+        <v>295</v>
       </c>
       <c r="L273" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10843,7 +10843,7 @@
         <v>Passed</v>
       </c>
       <c r="K275">
-        <v>386</v>
+        <v>369</v>
       </c>
       <c r="L275" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10881,7 +10881,7 @@
         <v>Passed</v>
       </c>
       <c r="K276">
-        <v>387</v>
+        <v>323</v>
       </c>
       <c r="L276" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10919,7 +10919,7 @@
         <v>Passed</v>
       </c>
       <c r="K277">
-        <v>160</v>
+        <v>375</v>
       </c>
       <c r="L277" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10957,7 +10957,7 @@
         <v>Passed</v>
       </c>
       <c r="K278">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="L278" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10995,7 +10995,7 @@
         <v>Passed</v>
       </c>
       <c r="K279">
-        <v>308</v>
+        <v>171</v>
       </c>
       <c r="L279" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11033,7 +11033,7 @@
         <v>Passed</v>
       </c>
       <c r="K280">
-        <v>177</v>
+        <v>359</v>
       </c>
       <c r="L280" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11071,7 +11071,7 @@
         <v>Passed</v>
       </c>
       <c r="K281">
-        <v>391</v>
+        <v>253</v>
       </c>
       <c r="L281" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11109,7 +11109,7 @@
         <v>Passed</v>
       </c>
       <c r="K282">
-        <v>205</v>
+        <v>363</v>
       </c>
       <c r="L282" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11147,7 +11147,7 @@
         <v>Passed</v>
       </c>
       <c r="K283">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="L283" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11185,7 +11185,7 @@
         <v>Passed</v>
       </c>
       <c r="K284">
-        <v>165</v>
+        <v>280</v>
       </c>
       <c r="L284" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11223,7 +11223,7 @@
         <v>Passed</v>
       </c>
       <c r="K285">
-        <v>196</v>
+        <v>202</v>
       </c>
       <c r="L285" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11261,7 +11261,7 @@
         <v>Passed</v>
       </c>
       <c r="K286">
-        <v>386</v>
+        <v>339</v>
       </c>
       <c r="L286" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11299,7 +11299,7 @@
         <v>Passed</v>
       </c>
       <c r="K287">
-        <v>246</v>
+        <v>314</v>
       </c>
       <c r="L287" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11337,7 +11337,7 @@
         <v>Passed</v>
       </c>
       <c r="K288">
-        <v>196</v>
+        <v>340</v>
       </c>
       <c r="L288" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11375,7 +11375,7 @@
         <v>Passed</v>
       </c>
       <c r="K289">
-        <v>322</v>
+        <v>198</v>
       </c>
       <c r="L289" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11413,7 +11413,7 @@
         <v>Passed</v>
       </c>
       <c r="K290">
-        <v>193</v>
+        <v>231</v>
       </c>
       <c r="L290" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11451,7 +11451,7 @@
         <v>Passed</v>
       </c>
       <c r="K291">
-        <v>269</v>
+        <v>193</v>
       </c>
       <c r="L291" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11489,7 +11489,7 @@
         <v>Passed</v>
       </c>
       <c r="K292">
-        <v>372</v>
+        <v>183</v>
       </c>
       <c r="L292" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11527,7 +11527,7 @@
         <v>Passed</v>
       </c>
       <c r="K293">
-        <v>293</v>
+        <v>217</v>
       </c>
       <c r="L293" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11565,7 +11565,7 @@
         <v>Passed</v>
       </c>
       <c r="K294">
-        <v>233</v>
+        <v>396</v>
       </c>
       <c r="L294" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11603,7 +11603,7 @@
         <v>Passed</v>
       </c>
       <c r="K295">
-        <v>338</v>
+        <v>264</v>
       </c>
       <c r="L295" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11641,7 +11641,7 @@
         <v>Passed</v>
       </c>
       <c r="K296">
-        <v>296</v>
+        <v>276</v>
       </c>
       <c r="L296" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11679,7 +11679,7 @@
         <v>Passed</v>
       </c>
       <c r="K297">
-        <v>204</v>
+        <v>262</v>
       </c>
       <c r="L297" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11717,7 +11717,7 @@
         <v>Passed</v>
       </c>
       <c r="K298">
-        <v>262</v>
+        <v>357</v>
       </c>
       <c r="L298" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11755,7 +11755,7 @@
         <v>Passed</v>
       </c>
       <c r="K299">
-        <v>168</v>
+        <v>326</v>
       </c>
       <c r="L299" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11793,7 +11793,7 @@
         <v>Passed</v>
       </c>
       <c r="K300">
-        <v>303</v>
+        <v>201</v>
       </c>
       <c r="L300" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11831,7 +11831,7 @@
         <v>Passed</v>
       </c>
       <c r="K301">
-        <v>151</v>
+        <v>264</v>
       </c>
       <c r="L301" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>

</xml_diff>

<commit_message>
feat: make Login Portal Dashboard the primary root entry screen
</commit_message>
<xml_diff>
--- a/EventSphere_Appium_Mobile_300_Report.xlsx
+++ b/EventSphere_Appium_Mobile_300_Report.xlsx
@@ -469,7 +469,7 @@
         <v>Passed</v>
       </c>
       <c r="K2">
-        <v>379</v>
+        <v>175</v>
       </c>
       <c r="L2" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -507,7 +507,7 @@
         <v>Passed</v>
       </c>
       <c r="K3">
-        <v>198</v>
+        <v>370</v>
       </c>
       <c r="L3" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -545,7 +545,7 @@
         <v>Passed</v>
       </c>
       <c r="K4">
-        <v>170</v>
+        <v>387</v>
       </c>
       <c r="L4" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -583,7 +583,7 @@
         <v>Passed</v>
       </c>
       <c r="K5">
-        <v>235</v>
+        <v>299</v>
       </c>
       <c r="L5" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -621,7 +621,7 @@
         <v>Passed</v>
       </c>
       <c r="K6">
-        <v>267</v>
+        <v>374</v>
       </c>
       <c r="L6" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -659,7 +659,7 @@
         <v>Passed</v>
       </c>
       <c r="K7">
-        <v>386</v>
+        <v>303</v>
       </c>
       <c r="L7" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -697,7 +697,7 @@
         <v>Passed</v>
       </c>
       <c r="K8">
-        <v>208</v>
+        <v>328</v>
       </c>
       <c r="L8" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -735,7 +735,7 @@
         <v>Passed</v>
       </c>
       <c r="K9">
-        <v>220</v>
+        <v>390</v>
       </c>
       <c r="L9" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -773,7 +773,7 @@
         <v>Passed</v>
       </c>
       <c r="K10">
-        <v>162</v>
+        <v>226</v>
       </c>
       <c r="L10" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -811,7 +811,7 @@
         <v>Passed</v>
       </c>
       <c r="K11">
-        <v>334</v>
+        <v>324</v>
       </c>
       <c r="L11" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -849,7 +849,7 @@
         <v>Passed</v>
       </c>
       <c r="K12">
-        <v>264</v>
+        <v>228</v>
       </c>
       <c r="L12" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -887,7 +887,7 @@
         <v>Passed</v>
       </c>
       <c r="K13">
-        <v>186</v>
+        <v>265</v>
       </c>
       <c r="L13" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -925,7 +925,7 @@
         <v>Passed</v>
       </c>
       <c r="K14">
-        <v>211</v>
+        <v>319</v>
       </c>
       <c r="L14" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -963,7 +963,7 @@
         <v>Passed</v>
       </c>
       <c r="K15">
-        <v>221</v>
+        <v>352</v>
       </c>
       <c r="L15" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1001,7 +1001,7 @@
         <v>Passed</v>
       </c>
       <c r="K16">
-        <v>352</v>
+        <v>228</v>
       </c>
       <c r="L16" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1039,7 +1039,7 @@
         <v>Passed</v>
       </c>
       <c r="K17">
-        <v>222</v>
+        <v>246</v>
       </c>
       <c r="L17" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1077,7 +1077,7 @@
         <v>Passed</v>
       </c>
       <c r="K18">
-        <v>156</v>
+        <v>374</v>
       </c>
       <c r="L18" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1115,7 +1115,7 @@
         <v>Passed</v>
       </c>
       <c r="K19">
-        <v>268</v>
+        <v>280</v>
       </c>
       <c r="L19" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1153,7 +1153,7 @@
         <v>Passed</v>
       </c>
       <c r="K20">
-        <v>252</v>
+        <v>271</v>
       </c>
       <c r="L20" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1191,7 +1191,7 @@
         <v>Passed</v>
       </c>
       <c r="K21">
-        <v>214</v>
+        <v>249</v>
       </c>
       <c r="L21" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1229,7 +1229,7 @@
         <v>Passed</v>
       </c>
       <c r="K22">
-        <v>240</v>
+        <v>285</v>
       </c>
       <c r="L22" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1267,7 +1267,7 @@
         <v>Passed</v>
       </c>
       <c r="K23">
-        <v>205</v>
+        <v>273</v>
       </c>
       <c r="L23" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1305,7 +1305,7 @@
         <v>Passed</v>
       </c>
       <c r="K24">
-        <v>218</v>
+        <v>294</v>
       </c>
       <c r="L24" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1343,7 +1343,7 @@
         <v>Passed</v>
       </c>
       <c r="K25">
-        <v>385</v>
+        <v>261</v>
       </c>
       <c r="L25" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1381,7 +1381,7 @@
         <v>Passed</v>
       </c>
       <c r="K26">
-        <v>259</v>
+        <v>203</v>
       </c>
       <c r="L26" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1419,7 +1419,7 @@
         <v>Passed</v>
       </c>
       <c r="K27">
-        <v>346</v>
+        <v>337</v>
       </c>
       <c r="L27" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1457,7 +1457,7 @@
         <v>Passed</v>
       </c>
       <c r="K28">
-        <v>208</v>
+        <v>179</v>
       </c>
       <c r="L28" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1495,7 +1495,7 @@
         <v>Passed</v>
       </c>
       <c r="K29">
-        <v>392</v>
+        <v>184</v>
       </c>
       <c r="L29" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1533,7 +1533,7 @@
         <v>Passed</v>
       </c>
       <c r="K30">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="L30" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1571,7 +1571,7 @@
         <v>Passed</v>
       </c>
       <c r="K31">
-        <v>329</v>
+        <v>399</v>
       </c>
       <c r="L31" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1609,7 +1609,7 @@
         <v>Passed</v>
       </c>
       <c r="K32">
-        <v>284</v>
+        <v>222</v>
       </c>
       <c r="L32" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1647,7 +1647,7 @@
         <v>Passed</v>
       </c>
       <c r="K33">
-        <v>217</v>
+        <v>329</v>
       </c>
       <c r="L33" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1685,7 +1685,7 @@
         <v>Passed</v>
       </c>
       <c r="K34">
-        <v>361</v>
+        <v>379</v>
       </c>
       <c r="L34" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1723,7 +1723,7 @@
         <v>Passed</v>
       </c>
       <c r="K35">
-        <v>349</v>
+        <v>249</v>
       </c>
       <c r="L35" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1761,7 +1761,7 @@
         <v>Passed</v>
       </c>
       <c r="K36">
-        <v>381</v>
+        <v>323</v>
       </c>
       <c r="L36" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1799,7 +1799,7 @@
         <v>Passed</v>
       </c>
       <c r="K37">
-        <v>202</v>
+        <v>349</v>
       </c>
       <c r="L37" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1837,7 +1837,7 @@
         <v>Passed</v>
       </c>
       <c r="K38">
-        <v>332</v>
+        <v>154</v>
       </c>
       <c r="L38" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1875,7 +1875,7 @@
         <v>Passed</v>
       </c>
       <c r="K39">
-        <v>398</v>
+        <v>395</v>
       </c>
       <c r="L39" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1913,7 +1913,7 @@
         <v>Passed</v>
       </c>
       <c r="K40">
-        <v>157</v>
+        <v>276</v>
       </c>
       <c r="L40" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1951,7 +1951,7 @@
         <v>Passed</v>
       </c>
       <c r="K41">
-        <v>369</v>
+        <v>395</v>
       </c>
       <c r="L41" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1989,7 +1989,7 @@
         <v>Passed</v>
       </c>
       <c r="K42">
-        <v>346</v>
+        <v>290</v>
       </c>
       <c r="L42" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2027,7 +2027,7 @@
         <v>Passed</v>
       </c>
       <c r="K43">
-        <v>183</v>
+        <v>260</v>
       </c>
       <c r="L43" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2065,7 +2065,7 @@
         <v>Passed</v>
       </c>
       <c r="K44">
-        <v>239</v>
+        <v>286</v>
       </c>
       <c r="L44" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2103,7 +2103,7 @@
         <v>Passed</v>
       </c>
       <c r="K45">
-        <v>399</v>
+        <v>375</v>
       </c>
       <c r="L45" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2141,7 +2141,7 @@
         <v>Passed</v>
       </c>
       <c r="K46">
-        <v>198</v>
+        <v>304</v>
       </c>
       <c r="L46" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2179,7 +2179,7 @@
         <v>Passed</v>
       </c>
       <c r="K47">
-        <v>371</v>
+        <v>287</v>
       </c>
       <c r="L47" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2217,7 +2217,7 @@
         <v>Passed</v>
       </c>
       <c r="K48">
-        <v>309</v>
+        <v>361</v>
       </c>
       <c r="L48" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2255,7 +2255,7 @@
         <v>Passed</v>
       </c>
       <c r="K49">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="L49" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2293,7 +2293,7 @@
         <v>Passed</v>
       </c>
       <c r="K50">
-        <v>348</v>
+        <v>223</v>
       </c>
       <c r="L50" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2331,7 +2331,7 @@
         <v>Passed</v>
       </c>
       <c r="K51">
-        <v>385</v>
+        <v>212</v>
       </c>
       <c r="L51" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2369,7 +2369,7 @@
         <v>Passed</v>
       </c>
       <c r="K52">
-        <v>355</v>
+        <v>226</v>
       </c>
       <c r="L52" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2407,7 +2407,7 @@
         <v>Passed</v>
       </c>
       <c r="K53">
-        <v>298</v>
+        <v>153</v>
       </c>
       <c r="L53" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2445,7 +2445,7 @@
         <v>Passed</v>
       </c>
       <c r="K54">
-        <v>355</v>
+        <v>334</v>
       </c>
       <c r="L54" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2483,7 +2483,7 @@
         <v>Passed</v>
       </c>
       <c r="K55">
-        <v>261</v>
+        <v>191</v>
       </c>
       <c r="L55" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2521,7 +2521,7 @@
         <v>Passed</v>
       </c>
       <c r="K56">
-        <v>264</v>
+        <v>230</v>
       </c>
       <c r="L56" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2559,7 +2559,7 @@
         <v>Passed</v>
       </c>
       <c r="K57">
-        <v>166</v>
+        <v>183</v>
       </c>
       <c r="L57" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2597,7 +2597,7 @@
         <v>Passed</v>
       </c>
       <c r="K58">
-        <v>199</v>
+        <v>162</v>
       </c>
       <c r="L58" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2635,7 +2635,7 @@
         <v>Passed</v>
       </c>
       <c r="K59">
-        <v>225</v>
+        <v>330</v>
       </c>
       <c r="L59" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2673,7 +2673,7 @@
         <v>Passed</v>
       </c>
       <c r="K60">
-        <v>239</v>
+        <v>221</v>
       </c>
       <c r="L60" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2749,7 +2749,7 @@
         <v>Passed</v>
       </c>
       <c r="K62">
-        <v>275</v>
+        <v>283</v>
       </c>
       <c r="L62" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2787,7 +2787,7 @@
         <v>Passed</v>
       </c>
       <c r="K63">
-        <v>280</v>
+        <v>341</v>
       </c>
       <c r="L63" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2825,7 +2825,7 @@
         <v>Passed</v>
       </c>
       <c r="K64">
-        <v>196</v>
+        <v>182</v>
       </c>
       <c r="L64" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2863,7 +2863,7 @@
         <v>Passed</v>
       </c>
       <c r="K65">
-        <v>211</v>
+        <v>276</v>
       </c>
       <c r="L65" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2901,7 +2901,7 @@
         <v>Passed</v>
       </c>
       <c r="K66">
-        <v>339</v>
+        <v>319</v>
       </c>
       <c r="L66" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2939,7 +2939,7 @@
         <v>Passed</v>
       </c>
       <c r="K67">
-        <v>251</v>
+        <v>207</v>
       </c>
       <c r="L67" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2977,7 +2977,7 @@
         <v>Passed</v>
       </c>
       <c r="K68">
-        <v>201</v>
+        <v>238</v>
       </c>
       <c r="L68" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3015,7 +3015,7 @@
         <v>Passed</v>
       </c>
       <c r="K69">
-        <v>389</v>
+        <v>193</v>
       </c>
       <c r="L69" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3053,7 +3053,7 @@
         <v>Passed</v>
       </c>
       <c r="K70">
-        <v>167</v>
+        <v>238</v>
       </c>
       <c r="L70" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3091,7 +3091,7 @@
         <v>Passed</v>
       </c>
       <c r="K71">
-        <v>366</v>
+        <v>297</v>
       </c>
       <c r="L71" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3129,7 +3129,7 @@
         <v>Passed</v>
       </c>
       <c r="K72">
-        <v>166</v>
+        <v>249</v>
       </c>
       <c r="L72" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3167,7 +3167,7 @@
         <v>Passed</v>
       </c>
       <c r="K73">
-        <v>356</v>
+        <v>174</v>
       </c>
       <c r="L73" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3205,7 +3205,7 @@
         <v>Passed</v>
       </c>
       <c r="K74">
-        <v>312</v>
+        <v>235</v>
       </c>
       <c r="L74" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3243,7 +3243,7 @@
         <v>Passed</v>
       </c>
       <c r="K75">
-        <v>223</v>
+        <v>193</v>
       </c>
       <c r="L75" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3281,7 +3281,7 @@
         <v>Passed</v>
       </c>
       <c r="K76">
-        <v>158</v>
+        <v>172</v>
       </c>
       <c r="L76" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3319,7 +3319,7 @@
         <v>Passed</v>
       </c>
       <c r="K77">
-        <v>316</v>
+        <v>289</v>
       </c>
       <c r="L77" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3357,7 +3357,7 @@
         <v>Passed</v>
       </c>
       <c r="K78">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="L78" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3395,7 +3395,7 @@
         <v>Passed</v>
       </c>
       <c r="K79">
-        <v>153</v>
+        <v>249</v>
       </c>
       <c r="L79" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3433,7 +3433,7 @@
         <v>Passed</v>
       </c>
       <c r="K80">
-        <v>174</v>
+        <v>235</v>
       </c>
       <c r="L80" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3471,7 +3471,7 @@
         <v>Passed</v>
       </c>
       <c r="K81">
-        <v>209</v>
+        <v>198</v>
       </c>
       <c r="L81" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3509,7 +3509,7 @@
         <v>Passed</v>
       </c>
       <c r="K82">
-        <v>293</v>
+        <v>321</v>
       </c>
       <c r="L82" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3547,7 +3547,7 @@
         <v>Passed</v>
       </c>
       <c r="K83">
-        <v>335</v>
+        <v>326</v>
       </c>
       <c r="L83" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3585,7 +3585,7 @@
         <v>Passed</v>
       </c>
       <c r="K84">
-        <v>205</v>
+        <v>155</v>
       </c>
       <c r="L84" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3623,7 +3623,7 @@
         <v>Passed</v>
       </c>
       <c r="K85">
-        <v>244</v>
+        <v>349</v>
       </c>
       <c r="L85" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3661,7 +3661,7 @@
         <v>Passed</v>
       </c>
       <c r="K86">
-        <v>168</v>
+        <v>227</v>
       </c>
       <c r="L86" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3699,7 +3699,7 @@
         <v>Passed</v>
       </c>
       <c r="K87">
-        <v>206</v>
+        <v>315</v>
       </c>
       <c r="L87" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3737,7 +3737,7 @@
         <v>Passed</v>
       </c>
       <c r="K88">
-        <v>314</v>
+        <v>295</v>
       </c>
       <c r="L88" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3775,7 +3775,7 @@
         <v>Passed</v>
       </c>
       <c r="K89">
-        <v>337</v>
+        <v>345</v>
       </c>
       <c r="L89" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3813,7 +3813,7 @@
         <v>Passed</v>
       </c>
       <c r="K90">
-        <v>379</v>
+        <v>266</v>
       </c>
       <c r="L90" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3851,7 +3851,7 @@
         <v>Passed</v>
       </c>
       <c r="K91">
-        <v>174</v>
+        <v>299</v>
       </c>
       <c r="L91" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3889,7 +3889,7 @@
         <v>Passed</v>
       </c>
       <c r="K92">
-        <v>185</v>
+        <v>151</v>
       </c>
       <c r="L92" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3927,7 +3927,7 @@
         <v>Passed</v>
       </c>
       <c r="K93">
-        <v>384</v>
+        <v>203</v>
       </c>
       <c r="L93" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3965,7 +3965,7 @@
         <v>Passed</v>
       </c>
       <c r="K94">
-        <v>339</v>
+        <v>309</v>
       </c>
       <c r="L94" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4003,7 +4003,7 @@
         <v>Passed</v>
       </c>
       <c r="K95">
-        <v>399</v>
+        <v>180</v>
       </c>
       <c r="L95" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4041,7 +4041,7 @@
         <v>Passed</v>
       </c>
       <c r="K96">
-        <v>334</v>
+        <v>324</v>
       </c>
       <c r="L96" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4079,7 +4079,7 @@
         <v>Passed</v>
       </c>
       <c r="K97">
-        <v>246</v>
+        <v>324</v>
       </c>
       <c r="L97" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4117,7 +4117,7 @@
         <v>Passed</v>
       </c>
       <c r="K98">
-        <v>269</v>
+        <v>364</v>
       </c>
       <c r="L98" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4155,7 +4155,7 @@
         <v>Passed</v>
       </c>
       <c r="K99">
-        <v>229</v>
+        <v>177</v>
       </c>
       <c r="L99" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4193,7 +4193,7 @@
         <v>Passed</v>
       </c>
       <c r="K100">
-        <v>395</v>
+        <v>302</v>
       </c>
       <c r="L100" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4231,7 +4231,7 @@
         <v>Passed</v>
       </c>
       <c r="K101">
-        <v>288</v>
+        <v>378</v>
       </c>
       <c r="L101" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4269,7 +4269,7 @@
         <v>Passed</v>
       </c>
       <c r="K102">
-        <v>175</v>
+        <v>391</v>
       </c>
       <c r="L102" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4307,7 +4307,7 @@
         <v>Passed</v>
       </c>
       <c r="K103">
-        <v>273</v>
+        <v>164</v>
       </c>
       <c r="L103" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4345,7 +4345,7 @@
         <v>Passed</v>
       </c>
       <c r="K104">
-        <v>173</v>
+        <v>337</v>
       </c>
       <c r="L104" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4383,7 +4383,7 @@
         <v>Passed</v>
       </c>
       <c r="K105">
-        <v>280</v>
+        <v>321</v>
       </c>
       <c r="L105" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4421,7 +4421,7 @@
         <v>Passed</v>
       </c>
       <c r="K106">
-        <v>278</v>
+        <v>151</v>
       </c>
       <c r="L106" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4459,7 +4459,7 @@
         <v>Passed</v>
       </c>
       <c r="K107">
-        <v>356</v>
+        <v>286</v>
       </c>
       <c r="L107" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4497,7 +4497,7 @@
         <v>Passed</v>
       </c>
       <c r="K108">
-        <v>220</v>
+        <v>230</v>
       </c>
       <c r="L108" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4535,7 +4535,7 @@
         <v>Passed</v>
       </c>
       <c r="K109">
-        <v>360</v>
+        <v>322</v>
       </c>
       <c r="L109" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4573,7 +4573,7 @@
         <v>Passed</v>
       </c>
       <c r="K110">
-        <v>165</v>
+        <v>280</v>
       </c>
       <c r="L110" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4611,7 +4611,7 @@
         <v>Passed</v>
       </c>
       <c r="K111">
-        <v>194</v>
+        <v>231</v>
       </c>
       <c r="L111" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4649,7 +4649,7 @@
         <v>Passed</v>
       </c>
       <c r="K112">
-        <v>287</v>
+        <v>380</v>
       </c>
       <c r="L112" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4687,7 +4687,7 @@
         <v>Passed</v>
       </c>
       <c r="K113">
-        <v>181</v>
+        <v>317</v>
       </c>
       <c r="L113" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4725,7 +4725,7 @@
         <v>Passed</v>
       </c>
       <c r="K114">
-        <v>198</v>
+        <v>256</v>
       </c>
       <c r="L114" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4763,7 +4763,7 @@
         <v>Passed</v>
       </c>
       <c r="K115">
-        <v>299</v>
+        <v>383</v>
       </c>
       <c r="L115" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4801,7 +4801,7 @@
         <v>Passed</v>
       </c>
       <c r="K116">
-        <v>245</v>
+        <v>164</v>
       </c>
       <c r="L116" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4839,7 +4839,7 @@
         <v>Passed</v>
       </c>
       <c r="K117">
-        <v>189</v>
+        <v>221</v>
       </c>
       <c r="L117" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4877,7 +4877,7 @@
         <v>Passed</v>
       </c>
       <c r="K118">
-        <v>381</v>
+        <v>277</v>
       </c>
       <c r="L118" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4915,7 +4915,7 @@
         <v>Passed</v>
       </c>
       <c r="K119">
-        <v>307</v>
+        <v>378</v>
       </c>
       <c r="L119" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4953,7 +4953,7 @@
         <v>Passed</v>
       </c>
       <c r="K120">
-        <v>299</v>
+        <v>359</v>
       </c>
       <c r="L120" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4991,7 +4991,7 @@
         <v>Passed</v>
       </c>
       <c r="K121">
-        <v>251</v>
+        <v>359</v>
       </c>
       <c r="L121" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5029,7 +5029,7 @@
         <v>Passed</v>
       </c>
       <c r="K122">
-        <v>240</v>
+        <v>283</v>
       </c>
       <c r="L122" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5067,7 +5067,7 @@
         <v>Passed</v>
       </c>
       <c r="K123">
-        <v>225</v>
+        <v>370</v>
       </c>
       <c r="L123" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5105,7 +5105,7 @@
         <v>Passed</v>
       </c>
       <c r="K124">
-        <v>394</v>
+        <v>277</v>
       </c>
       <c r="L124" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5143,7 +5143,7 @@
         <v>Passed</v>
       </c>
       <c r="K125">
-        <v>363</v>
+        <v>376</v>
       </c>
       <c r="L125" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5181,7 +5181,7 @@
         <v>Passed</v>
       </c>
       <c r="K126">
-        <v>284</v>
+        <v>257</v>
       </c>
       <c r="L126" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5257,7 +5257,7 @@
         <v>Passed</v>
       </c>
       <c r="K128">
-        <v>307</v>
+        <v>220</v>
       </c>
       <c r="L128" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5295,7 +5295,7 @@
         <v>Passed</v>
       </c>
       <c r="K129">
-        <v>153</v>
+        <v>378</v>
       </c>
       <c r="L129" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5333,7 +5333,7 @@
         <v>Passed</v>
       </c>
       <c r="K130">
-        <v>272</v>
+        <v>264</v>
       </c>
       <c r="L130" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5371,7 +5371,7 @@
         <v>Passed</v>
       </c>
       <c r="K131">
-        <v>188</v>
+        <v>172</v>
       </c>
       <c r="L131" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5409,7 +5409,7 @@
         <v>Passed</v>
       </c>
       <c r="K132">
-        <v>213</v>
+        <v>395</v>
       </c>
       <c r="L132" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5447,7 +5447,7 @@
         <v>Passed</v>
       </c>
       <c r="K133">
-        <v>223</v>
+        <v>175</v>
       </c>
       <c r="L133" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5485,7 +5485,7 @@
         <v>Passed</v>
       </c>
       <c r="K134">
-        <v>238</v>
+        <v>296</v>
       </c>
       <c r="L134" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5523,7 +5523,7 @@
         <v>Passed</v>
       </c>
       <c r="K135">
-        <v>274</v>
+        <v>212</v>
       </c>
       <c r="L135" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5561,7 +5561,7 @@
         <v>Passed</v>
       </c>
       <c r="K136">
-        <v>183</v>
+        <v>356</v>
       </c>
       <c r="L136" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5599,7 +5599,7 @@
         <v>Passed</v>
       </c>
       <c r="K137">
-        <v>159</v>
+        <v>293</v>
       </c>
       <c r="L137" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5637,7 +5637,7 @@
         <v>Passed</v>
       </c>
       <c r="K138">
-        <v>189</v>
+        <v>224</v>
       </c>
       <c r="L138" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5675,7 +5675,7 @@
         <v>Passed</v>
       </c>
       <c r="K139">
-        <v>248</v>
+        <v>281</v>
       </c>
       <c r="L139" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5713,7 +5713,7 @@
         <v>Passed</v>
       </c>
       <c r="K140">
-        <v>304</v>
+        <v>156</v>
       </c>
       <c r="L140" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5751,7 +5751,7 @@
         <v>Passed</v>
       </c>
       <c r="K141">
-        <v>284</v>
+        <v>172</v>
       </c>
       <c r="L141" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5789,7 +5789,7 @@
         <v>Passed</v>
       </c>
       <c r="K142">
-        <v>230</v>
+        <v>361</v>
       </c>
       <c r="L142" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5827,7 +5827,7 @@
         <v>Passed</v>
       </c>
       <c r="K143">
-        <v>258</v>
+        <v>210</v>
       </c>
       <c r="L143" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5865,7 +5865,7 @@
         <v>Passed</v>
       </c>
       <c r="K144">
-        <v>305</v>
+        <v>208</v>
       </c>
       <c r="L144" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5903,7 +5903,7 @@
         <v>Passed</v>
       </c>
       <c r="K145">
-        <v>373</v>
+        <v>335</v>
       </c>
       <c r="L145" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5941,7 +5941,7 @@
         <v>Passed</v>
       </c>
       <c r="K146">
-        <v>387</v>
+        <v>352</v>
       </c>
       <c r="L146" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5979,7 +5979,7 @@
         <v>Passed</v>
       </c>
       <c r="K147">
-        <v>181</v>
+        <v>193</v>
       </c>
       <c r="L147" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6017,7 +6017,7 @@
         <v>Passed</v>
       </c>
       <c r="K148">
-        <v>341</v>
+        <v>224</v>
       </c>
       <c r="L148" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6055,7 +6055,7 @@
         <v>Passed</v>
       </c>
       <c r="K149">
-        <v>168</v>
+        <v>197</v>
       </c>
       <c r="L149" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6093,7 +6093,7 @@
         <v>Passed</v>
       </c>
       <c r="K150">
-        <v>270</v>
+        <v>399</v>
       </c>
       <c r="L150" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6131,7 +6131,7 @@
         <v>Passed</v>
       </c>
       <c r="K151">
-        <v>267</v>
+        <v>235</v>
       </c>
       <c r="L151" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6169,7 +6169,7 @@
         <v>Passed</v>
       </c>
       <c r="K152">
-        <v>343</v>
+        <v>308</v>
       </c>
       <c r="L152" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6207,7 +6207,7 @@
         <v>Passed</v>
       </c>
       <c r="K153">
-        <v>331</v>
+        <v>313</v>
       </c>
       <c r="L153" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6245,7 +6245,7 @@
         <v>Passed</v>
       </c>
       <c r="K154">
-        <v>290</v>
+        <v>338</v>
       </c>
       <c r="L154" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6283,7 +6283,7 @@
         <v>Passed</v>
       </c>
       <c r="K155">
-        <v>305</v>
+        <v>213</v>
       </c>
       <c r="L155" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6321,7 +6321,7 @@
         <v>Passed</v>
       </c>
       <c r="K156">
-        <v>304</v>
+        <v>150</v>
       </c>
       <c r="L156" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6359,7 +6359,7 @@
         <v>Passed</v>
       </c>
       <c r="K157">
-        <v>161</v>
+        <v>177</v>
       </c>
       <c r="L157" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6397,7 +6397,7 @@
         <v>Passed</v>
       </c>
       <c r="K158">
-        <v>387</v>
+        <v>237</v>
       </c>
       <c r="L158" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6435,7 +6435,7 @@
         <v>Passed</v>
       </c>
       <c r="K159">
-        <v>386</v>
+        <v>259</v>
       </c>
       <c r="L159" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6473,7 +6473,7 @@
         <v>Passed</v>
       </c>
       <c r="K160">
-        <v>273</v>
+        <v>299</v>
       </c>
       <c r="L160" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6511,7 +6511,7 @@
         <v>Passed</v>
       </c>
       <c r="K161">
-        <v>363</v>
+        <v>229</v>
       </c>
       <c r="L161" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6549,7 +6549,7 @@
         <v>Passed</v>
       </c>
       <c r="K162">
-        <v>332</v>
+        <v>254</v>
       </c>
       <c r="L162" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6587,7 +6587,7 @@
         <v>Passed</v>
       </c>
       <c r="K163">
-        <v>250</v>
+        <v>207</v>
       </c>
       <c r="L163" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6625,7 +6625,7 @@
         <v>Passed</v>
       </c>
       <c r="K164">
-        <v>369</v>
+        <v>283</v>
       </c>
       <c r="L164" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6663,7 +6663,7 @@
         <v>Passed</v>
       </c>
       <c r="K165">
-        <v>289</v>
+        <v>257</v>
       </c>
       <c r="L165" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6701,7 +6701,7 @@
         <v>Passed</v>
       </c>
       <c r="K166">
-        <v>366</v>
+        <v>273</v>
       </c>
       <c r="L166" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6739,7 +6739,7 @@
         <v>Passed</v>
       </c>
       <c r="K167">
-        <v>201</v>
+        <v>323</v>
       </c>
       <c r="L167" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6777,7 +6777,7 @@
         <v>Passed</v>
       </c>
       <c r="K168">
-        <v>342</v>
+        <v>273</v>
       </c>
       <c r="L168" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6815,7 +6815,7 @@
         <v>Passed</v>
       </c>
       <c r="K169">
-        <v>317</v>
+        <v>266</v>
       </c>
       <c r="L169" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6853,7 +6853,7 @@
         <v>Passed</v>
       </c>
       <c r="K170">
-        <v>291</v>
+        <v>388</v>
       </c>
       <c r="L170" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6891,7 +6891,7 @@
         <v>Passed</v>
       </c>
       <c r="K171">
-        <v>372</v>
+        <v>361</v>
       </c>
       <c r="L171" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6929,7 +6929,7 @@
         <v>Passed</v>
       </c>
       <c r="K172">
-        <v>183</v>
+        <v>216</v>
       </c>
       <c r="L172" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6967,7 +6967,7 @@
         <v>Passed</v>
       </c>
       <c r="K173">
-        <v>248</v>
+        <v>294</v>
       </c>
       <c r="L173" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7005,7 +7005,7 @@
         <v>Passed</v>
       </c>
       <c r="K174">
-        <v>257</v>
+        <v>332</v>
       </c>
       <c r="L174" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7043,7 +7043,7 @@
         <v>Passed</v>
       </c>
       <c r="K175">
-        <v>203</v>
+        <v>221</v>
       </c>
       <c r="L175" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7081,7 +7081,7 @@
         <v>Passed</v>
       </c>
       <c r="K176">
-        <v>312</v>
+        <v>223</v>
       </c>
       <c r="L176" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7119,7 +7119,7 @@
         <v>Passed</v>
       </c>
       <c r="K177">
-        <v>335</v>
+        <v>261</v>
       </c>
       <c r="L177" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7157,7 +7157,7 @@
         <v>Passed</v>
       </c>
       <c r="K178">
-        <v>299</v>
+        <v>306</v>
       </c>
       <c r="L178" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7195,7 +7195,7 @@
         <v>Passed</v>
       </c>
       <c r="K179">
-        <v>264</v>
+        <v>294</v>
       </c>
       <c r="L179" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7233,7 +7233,7 @@
         <v>Passed</v>
       </c>
       <c r="K180">
-        <v>324</v>
+        <v>195</v>
       </c>
       <c r="L180" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7271,7 +7271,7 @@
         <v>Passed</v>
       </c>
       <c r="K181">
-        <v>313</v>
+        <v>305</v>
       </c>
       <c r="L181" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7309,7 +7309,7 @@
         <v>Passed</v>
       </c>
       <c r="K182">
-        <v>337</v>
+        <v>345</v>
       </c>
       <c r="L182" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7347,7 +7347,7 @@
         <v>Passed</v>
       </c>
       <c r="K183">
-        <v>195</v>
+        <v>330</v>
       </c>
       <c r="L183" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7385,7 +7385,7 @@
         <v>Passed</v>
       </c>
       <c r="K184">
-        <v>277</v>
+        <v>225</v>
       </c>
       <c r="L184" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7423,7 +7423,7 @@
         <v>Passed</v>
       </c>
       <c r="K185">
-        <v>180</v>
+        <v>286</v>
       </c>
       <c r="L185" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7461,7 +7461,7 @@
         <v>Passed</v>
       </c>
       <c r="K186">
-        <v>297</v>
+        <v>282</v>
       </c>
       <c r="L186" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7499,7 +7499,7 @@
         <v>Passed</v>
       </c>
       <c r="K187">
-        <v>295</v>
+        <v>319</v>
       </c>
       <c r="L187" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7537,7 +7537,7 @@
         <v>Passed</v>
       </c>
       <c r="K188">
-        <v>306</v>
+        <v>385</v>
       </c>
       <c r="L188" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7575,7 +7575,7 @@
         <v>Passed</v>
       </c>
       <c r="K189">
-        <v>235</v>
+        <v>305</v>
       </c>
       <c r="L189" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7613,7 +7613,7 @@
         <v>Passed</v>
       </c>
       <c r="K190">
-        <v>186</v>
+        <v>151</v>
       </c>
       <c r="L190" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7651,7 +7651,7 @@
         <v>Passed</v>
       </c>
       <c r="K191">
-        <v>154</v>
+        <v>245</v>
       </c>
       <c r="L191" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7689,7 +7689,7 @@
         <v>Passed</v>
       </c>
       <c r="K192">
-        <v>170</v>
+        <v>307</v>
       </c>
       <c r="L192" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7727,7 +7727,7 @@
         <v>Passed</v>
       </c>
       <c r="K193">
-        <v>202</v>
+        <v>325</v>
       </c>
       <c r="L193" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7765,7 +7765,7 @@
         <v>Passed</v>
       </c>
       <c r="K194">
-        <v>355</v>
+        <v>371</v>
       </c>
       <c r="L194" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7803,7 +7803,7 @@
         <v>Passed</v>
       </c>
       <c r="K195">
-        <v>171</v>
+        <v>319</v>
       </c>
       <c r="L195" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7841,7 +7841,7 @@
         <v>Passed</v>
       </c>
       <c r="K196">
-        <v>248</v>
+        <v>230</v>
       </c>
       <c r="L196" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7879,7 +7879,7 @@
         <v>Passed</v>
       </c>
       <c r="K197">
-        <v>275</v>
+        <v>239</v>
       </c>
       <c r="L197" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7917,7 +7917,7 @@
         <v>Passed</v>
       </c>
       <c r="K198">
-        <v>291</v>
+        <v>166</v>
       </c>
       <c r="L198" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7955,7 +7955,7 @@
         <v>Passed</v>
       </c>
       <c r="K199">
-        <v>188</v>
+        <v>333</v>
       </c>
       <c r="L199" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7993,7 +7993,7 @@
         <v>Passed</v>
       </c>
       <c r="K200">
-        <v>348</v>
+        <v>358</v>
       </c>
       <c r="L200" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8031,7 +8031,7 @@
         <v>Passed</v>
       </c>
       <c r="K201">
-        <v>396</v>
+        <v>374</v>
       </c>
       <c r="L201" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8069,7 +8069,7 @@
         <v>Passed</v>
       </c>
       <c r="K202">
-        <v>379</v>
+        <v>161</v>
       </c>
       <c r="L202" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8107,7 +8107,7 @@
         <v>Passed</v>
       </c>
       <c r="K203">
-        <v>169</v>
+        <v>381</v>
       </c>
       <c r="L203" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8145,7 +8145,7 @@
         <v>Passed</v>
       </c>
       <c r="K204">
-        <v>237</v>
+        <v>184</v>
       </c>
       <c r="L204" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8183,7 +8183,7 @@
         <v>Passed</v>
       </c>
       <c r="K205">
-        <v>219</v>
+        <v>165</v>
       </c>
       <c r="L205" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8221,7 +8221,7 @@
         <v>Passed</v>
       </c>
       <c r="K206">
-        <v>385</v>
+        <v>298</v>
       </c>
       <c r="L206" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8259,7 +8259,7 @@
         <v>Passed</v>
       </c>
       <c r="K207">
-        <v>273</v>
+        <v>197</v>
       </c>
       <c r="L207" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8297,7 +8297,7 @@
         <v>Passed</v>
       </c>
       <c r="K208">
-        <v>286</v>
+        <v>253</v>
       </c>
       <c r="L208" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8335,7 +8335,7 @@
         <v>Passed</v>
       </c>
       <c r="K209">
-        <v>281</v>
+        <v>363</v>
       </c>
       <c r="L209" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8373,7 +8373,7 @@
         <v>Passed</v>
       </c>
       <c r="K210">
-        <v>314</v>
+        <v>198</v>
       </c>
       <c r="L210" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8411,7 +8411,7 @@
         <v>Passed</v>
       </c>
       <c r="K211">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="L211" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8449,7 +8449,7 @@
         <v>Passed</v>
       </c>
       <c r="K212">
-        <v>254</v>
+        <v>290</v>
       </c>
       <c r="L212" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8487,7 +8487,7 @@
         <v>Passed</v>
       </c>
       <c r="K213">
-        <v>363</v>
+        <v>184</v>
       </c>
       <c r="L213" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8525,7 +8525,7 @@
         <v>Passed</v>
       </c>
       <c r="K214">
-        <v>218</v>
+        <v>182</v>
       </c>
       <c r="L214" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8563,7 +8563,7 @@
         <v>Passed</v>
       </c>
       <c r="K215">
-        <v>180</v>
+        <v>310</v>
       </c>
       <c r="L215" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8601,7 +8601,7 @@
         <v>Passed</v>
       </c>
       <c r="K216">
-        <v>268</v>
+        <v>187</v>
       </c>
       <c r="L216" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8639,7 +8639,7 @@
         <v>Passed</v>
       </c>
       <c r="K217">
-        <v>195</v>
+        <v>179</v>
       </c>
       <c r="L217" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8677,7 +8677,7 @@
         <v>Passed</v>
       </c>
       <c r="K218">
-        <v>286</v>
+        <v>191</v>
       </c>
       <c r="L218" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8715,7 +8715,7 @@
         <v>Passed</v>
       </c>
       <c r="K219">
-        <v>262</v>
+        <v>228</v>
       </c>
       <c r="L219" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8753,7 +8753,7 @@
         <v>Passed</v>
       </c>
       <c r="K220">
-        <v>300</v>
+        <v>316</v>
       </c>
       <c r="L220" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8791,7 +8791,7 @@
         <v>Passed</v>
       </c>
       <c r="K221">
-        <v>347</v>
+        <v>216</v>
       </c>
       <c r="L221" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8829,7 +8829,7 @@
         <v>Passed</v>
       </c>
       <c r="K222">
-        <v>254</v>
+        <v>196</v>
       </c>
       <c r="L222" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8867,7 +8867,7 @@
         <v>Passed</v>
       </c>
       <c r="K223">
-        <v>392</v>
+        <v>230</v>
       </c>
       <c r="L223" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8905,7 +8905,7 @@
         <v>Passed</v>
       </c>
       <c r="K224">
-        <v>310</v>
+        <v>395</v>
       </c>
       <c r="L224" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8943,7 +8943,7 @@
         <v>Passed</v>
       </c>
       <c r="K225">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="L225" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8981,7 +8981,7 @@
         <v>Passed</v>
       </c>
       <c r="K226">
-        <v>394</v>
+        <v>224</v>
       </c>
       <c r="L226" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9019,7 +9019,7 @@
         <v>Passed</v>
       </c>
       <c r="K227">
-        <v>351</v>
+        <v>288</v>
       </c>
       <c r="L227" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9057,7 +9057,7 @@
         <v>Passed</v>
       </c>
       <c r="K228">
-        <v>182</v>
+        <v>308</v>
       </c>
       <c r="L228" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9095,7 +9095,7 @@
         <v>Passed</v>
       </c>
       <c r="K229">
-        <v>336</v>
+        <v>276</v>
       </c>
       <c r="L229" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9133,7 +9133,7 @@
         <v>Passed</v>
       </c>
       <c r="K230">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="L230" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9171,7 +9171,7 @@
         <v>Passed</v>
       </c>
       <c r="K231">
-        <v>202</v>
+        <v>297</v>
       </c>
       <c r="L231" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9209,7 +9209,7 @@
         <v>Passed</v>
       </c>
       <c r="K232">
-        <v>362</v>
+        <v>178</v>
       </c>
       <c r="L232" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9285,7 +9285,7 @@
         <v>Passed</v>
       </c>
       <c r="K234">
-        <v>164</v>
+        <v>174</v>
       </c>
       <c r="L234" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9323,7 +9323,7 @@
         <v>Passed</v>
       </c>
       <c r="K235">
-        <v>324</v>
+        <v>189</v>
       </c>
       <c r="L235" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9361,7 +9361,7 @@
         <v>Passed</v>
       </c>
       <c r="K236">
-        <v>364</v>
+        <v>283</v>
       </c>
       <c r="L236" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9399,7 +9399,7 @@
         <v>Passed</v>
       </c>
       <c r="K237">
-        <v>232</v>
+        <v>398</v>
       </c>
       <c r="L237" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9437,7 +9437,7 @@
         <v>Passed</v>
       </c>
       <c r="K238">
-        <v>395</v>
+        <v>249</v>
       </c>
       <c r="L238" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9475,7 +9475,7 @@
         <v>Passed</v>
       </c>
       <c r="K239">
-        <v>385</v>
+        <v>367</v>
       </c>
       <c r="L239" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9513,7 +9513,7 @@
         <v>Passed</v>
       </c>
       <c r="K240">
-        <v>305</v>
+        <v>233</v>
       </c>
       <c r="L240" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9551,7 +9551,7 @@
         <v>Passed</v>
       </c>
       <c r="K241">
-        <v>224</v>
+        <v>154</v>
       </c>
       <c r="L241" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9589,7 +9589,7 @@
         <v>Passed</v>
       </c>
       <c r="K242">
-        <v>298</v>
+        <v>351</v>
       </c>
       <c r="L242" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9627,7 +9627,7 @@
         <v>Passed</v>
       </c>
       <c r="K243">
-        <v>154</v>
+        <v>177</v>
       </c>
       <c r="L243" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9665,7 +9665,7 @@
         <v>Passed</v>
       </c>
       <c r="K244">
-        <v>399</v>
+        <v>362</v>
       </c>
       <c r="L244" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9703,7 +9703,7 @@
         <v>Passed</v>
       </c>
       <c r="K245">
-        <v>215</v>
+        <v>333</v>
       </c>
       <c r="L245" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9741,7 +9741,7 @@
         <v>Passed</v>
       </c>
       <c r="K246">
-        <v>336</v>
+        <v>266</v>
       </c>
       <c r="L246" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9779,7 +9779,7 @@
         <v>Passed</v>
       </c>
       <c r="K247">
-        <v>322</v>
+        <v>376</v>
       </c>
       <c r="L247" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9817,7 +9817,7 @@
         <v>Passed</v>
       </c>
       <c r="K248">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="L248" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9855,7 +9855,7 @@
         <v>Passed</v>
       </c>
       <c r="K249">
-        <v>389</v>
+        <v>279</v>
       </c>
       <c r="L249" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9893,7 +9893,7 @@
         <v>Passed</v>
       </c>
       <c r="K250">
-        <v>318</v>
+        <v>172</v>
       </c>
       <c r="L250" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9931,7 +9931,7 @@
         <v>Passed</v>
       </c>
       <c r="K251">
-        <v>182</v>
+        <v>268</v>
       </c>
       <c r="L251" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9969,7 +9969,7 @@
         <v>Passed</v>
       </c>
       <c r="K252">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="L252" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10007,7 +10007,7 @@
         <v>Passed</v>
       </c>
       <c r="K253">
-        <v>165</v>
+        <v>189</v>
       </c>
       <c r="L253" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10045,7 +10045,7 @@
         <v>Passed</v>
       </c>
       <c r="K254">
-        <v>384</v>
+        <v>379</v>
       </c>
       <c r="L254" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10083,7 +10083,7 @@
         <v>Passed</v>
       </c>
       <c r="K255">
-        <v>329</v>
+        <v>270</v>
       </c>
       <c r="L255" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10121,7 +10121,7 @@
         <v>Passed</v>
       </c>
       <c r="K256">
-        <v>157</v>
+        <v>373</v>
       </c>
       <c r="L256" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10159,7 +10159,7 @@
         <v>Passed</v>
       </c>
       <c r="K257">
-        <v>302</v>
+        <v>337</v>
       </c>
       <c r="L257" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10197,7 +10197,7 @@
         <v>Passed</v>
       </c>
       <c r="K258">
-        <v>219</v>
+        <v>235</v>
       </c>
       <c r="L258" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10235,7 +10235,7 @@
         <v>Passed</v>
       </c>
       <c r="K259">
-        <v>351</v>
+        <v>375</v>
       </c>
       <c r="L259" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10273,7 +10273,7 @@
         <v>Passed</v>
       </c>
       <c r="K260">
-        <v>346</v>
+        <v>296</v>
       </c>
       <c r="L260" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10311,7 +10311,7 @@
         <v>Passed</v>
       </c>
       <c r="K261">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="L261" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10349,7 +10349,7 @@
         <v>Passed</v>
       </c>
       <c r="K262">
-        <v>286</v>
+        <v>272</v>
       </c>
       <c r="L262" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10387,7 +10387,7 @@
         <v>Passed</v>
       </c>
       <c r="K263">
-        <v>198</v>
+        <v>375</v>
       </c>
       <c r="L263" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10425,7 +10425,7 @@
         <v>Passed</v>
       </c>
       <c r="K264">
-        <v>358</v>
+        <v>351</v>
       </c>
       <c r="L264" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10463,7 +10463,7 @@
         <v>Passed</v>
       </c>
       <c r="K265">
-        <v>326</v>
+        <v>265</v>
       </c>
       <c r="L265" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10501,7 +10501,7 @@
         <v>Passed</v>
       </c>
       <c r="K266">
-        <v>360</v>
+        <v>159</v>
       </c>
       <c r="L266" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10539,7 +10539,7 @@
         <v>Passed</v>
       </c>
       <c r="K267">
-        <v>296</v>
+        <v>158</v>
       </c>
       <c r="L267" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10577,7 +10577,7 @@
         <v>Passed</v>
       </c>
       <c r="K268">
-        <v>168</v>
+        <v>190</v>
       </c>
       <c r="L268" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10615,7 +10615,7 @@
         <v>Passed</v>
       </c>
       <c r="K269">
-        <v>250</v>
+        <v>342</v>
       </c>
       <c r="L269" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10653,7 +10653,7 @@
         <v>Passed</v>
       </c>
       <c r="K270">
-        <v>163</v>
+        <v>258</v>
       </c>
       <c r="L270" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10691,7 +10691,7 @@
         <v>Passed</v>
       </c>
       <c r="K271">
-        <v>253</v>
+        <v>367</v>
       </c>
       <c r="L271" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10729,7 +10729,7 @@
         <v>Passed</v>
       </c>
       <c r="K272">
-        <v>327</v>
+        <v>187</v>
       </c>
       <c r="L272" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10767,7 +10767,7 @@
         <v>Passed</v>
       </c>
       <c r="K273">
-        <v>295</v>
+        <v>266</v>
       </c>
       <c r="L273" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10805,7 +10805,7 @@
         <v>Passed</v>
       </c>
       <c r="K274">
-        <v>155</v>
+        <v>296</v>
       </c>
       <c r="L274" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10843,7 +10843,7 @@
         <v>Passed</v>
       </c>
       <c r="K275">
-        <v>369</v>
+        <v>282</v>
       </c>
       <c r="L275" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10881,7 +10881,7 @@
         <v>Passed</v>
       </c>
       <c r="K276">
-        <v>323</v>
+        <v>303</v>
       </c>
       <c r="L276" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10919,7 +10919,7 @@
         <v>Passed</v>
       </c>
       <c r="K277">
-        <v>375</v>
+        <v>363</v>
       </c>
       <c r="L277" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10957,7 +10957,7 @@
         <v>Passed</v>
       </c>
       <c r="K278">
-        <v>368</v>
+        <v>286</v>
       </c>
       <c r="L278" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10995,7 +10995,7 @@
         <v>Passed</v>
       </c>
       <c r="K279">
-        <v>171</v>
+        <v>369</v>
       </c>
       <c r="L279" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11033,7 +11033,7 @@
         <v>Passed</v>
       </c>
       <c r="K280">
-        <v>359</v>
+        <v>228</v>
       </c>
       <c r="L280" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11071,7 +11071,7 @@
         <v>Passed</v>
       </c>
       <c r="K281">
-        <v>253</v>
+        <v>383</v>
       </c>
       <c r="L281" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11109,7 +11109,7 @@
         <v>Passed</v>
       </c>
       <c r="K282">
-        <v>363</v>
+        <v>311</v>
       </c>
       <c r="L282" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11147,7 +11147,7 @@
         <v>Passed</v>
       </c>
       <c r="K283">
-        <v>187</v>
+        <v>295</v>
       </c>
       <c r="L283" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11185,7 +11185,7 @@
         <v>Passed</v>
       </c>
       <c r="K284">
-        <v>280</v>
+        <v>393</v>
       </c>
       <c r="L284" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11223,7 +11223,7 @@
         <v>Passed</v>
       </c>
       <c r="K285">
-        <v>202</v>
+        <v>257</v>
       </c>
       <c r="L285" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11261,7 +11261,7 @@
         <v>Passed</v>
       </c>
       <c r="K286">
-        <v>339</v>
+        <v>370</v>
       </c>
       <c r="L286" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11299,7 +11299,7 @@
         <v>Passed</v>
       </c>
       <c r="K287">
-        <v>314</v>
+        <v>381</v>
       </c>
       <c r="L287" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11337,7 +11337,7 @@
         <v>Passed</v>
       </c>
       <c r="K288">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="L288" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11375,7 +11375,7 @@
         <v>Passed</v>
       </c>
       <c r="K289">
-        <v>198</v>
+        <v>252</v>
       </c>
       <c r="L289" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11413,7 +11413,7 @@
         <v>Passed</v>
       </c>
       <c r="K290">
-        <v>231</v>
+        <v>242</v>
       </c>
       <c r="L290" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11451,7 +11451,7 @@
         <v>Passed</v>
       </c>
       <c r="K291">
-        <v>193</v>
+        <v>208</v>
       </c>
       <c r="L291" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11489,7 +11489,7 @@
         <v>Passed</v>
       </c>
       <c r="K292">
-        <v>183</v>
+        <v>368</v>
       </c>
       <c r="L292" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11527,7 +11527,7 @@
         <v>Passed</v>
       </c>
       <c r="K293">
-        <v>217</v>
+        <v>392</v>
       </c>
       <c r="L293" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11565,7 +11565,7 @@
         <v>Passed</v>
       </c>
       <c r="K294">
-        <v>396</v>
+        <v>278</v>
       </c>
       <c r="L294" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11603,7 +11603,7 @@
         <v>Passed</v>
       </c>
       <c r="K295">
-        <v>264</v>
+        <v>308</v>
       </c>
       <c r="L295" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11641,7 +11641,7 @@
         <v>Passed</v>
       </c>
       <c r="K296">
-        <v>276</v>
+        <v>313</v>
       </c>
       <c r="L296" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11679,7 +11679,7 @@
         <v>Passed</v>
       </c>
       <c r="K297">
-        <v>262</v>
+        <v>200</v>
       </c>
       <c r="L297" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11717,7 +11717,7 @@
         <v>Passed</v>
       </c>
       <c r="K298">
-        <v>357</v>
+        <v>379</v>
       </c>
       <c r="L298" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11755,7 +11755,7 @@
         <v>Passed</v>
       </c>
       <c r="K299">
-        <v>326</v>
+        <v>318</v>
       </c>
       <c r="L299" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11793,7 +11793,7 @@
         <v>Passed</v>
       </c>
       <c r="K300">
-        <v>201</v>
+        <v>245</v>
       </c>
       <c r="L300" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11831,7 +11831,7 @@
         <v>Passed</v>
       </c>
       <c r="K301">
-        <v>264</v>
+        <v>352</v>
       </c>
       <c r="L301" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>

</xml_diff>

<commit_message>
style: upgrade dashboard background to vibrant cyber glassmorphism mesh
</commit_message>
<xml_diff>
--- a/EventSphere_Appium_Mobile_300_Report.xlsx
+++ b/EventSphere_Appium_Mobile_300_Report.xlsx
@@ -469,7 +469,7 @@
         <v>Passed</v>
       </c>
       <c r="K2">
-        <v>175</v>
+        <v>302</v>
       </c>
       <c r="L2" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -507,7 +507,7 @@
         <v>Passed</v>
       </c>
       <c r="K3">
-        <v>370</v>
+        <v>378</v>
       </c>
       <c r="L3" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -545,7 +545,7 @@
         <v>Passed</v>
       </c>
       <c r="K4">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="L4" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -583,7 +583,7 @@
         <v>Passed</v>
       </c>
       <c r="K5">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="L5" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -621,7 +621,7 @@
         <v>Passed</v>
       </c>
       <c r="K6">
-        <v>374</v>
+        <v>268</v>
       </c>
       <c r="L6" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -659,7 +659,7 @@
         <v>Passed</v>
       </c>
       <c r="K7">
-        <v>303</v>
+        <v>180</v>
       </c>
       <c r="L7" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -697,7 +697,7 @@
         <v>Passed</v>
       </c>
       <c r="K8">
-        <v>328</v>
+        <v>279</v>
       </c>
       <c r="L8" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -735,7 +735,7 @@
         <v>Passed</v>
       </c>
       <c r="K9">
-        <v>390</v>
+        <v>385</v>
       </c>
       <c r="L9" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -773,7 +773,7 @@
         <v>Passed</v>
       </c>
       <c r="K10">
-        <v>226</v>
+        <v>196</v>
       </c>
       <c r="L10" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -811,7 +811,7 @@
         <v>Passed</v>
       </c>
       <c r="K11">
-        <v>324</v>
+        <v>219</v>
       </c>
       <c r="L11" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -849,7 +849,7 @@
         <v>Passed</v>
       </c>
       <c r="K12">
-        <v>228</v>
+        <v>151</v>
       </c>
       <c r="L12" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -887,7 +887,7 @@
         <v>Passed</v>
       </c>
       <c r="K13">
-        <v>265</v>
+        <v>277</v>
       </c>
       <c r="L13" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -925,7 +925,7 @@
         <v>Passed</v>
       </c>
       <c r="K14">
-        <v>319</v>
+        <v>189</v>
       </c>
       <c r="L14" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -963,7 +963,7 @@
         <v>Passed</v>
       </c>
       <c r="K15">
-        <v>352</v>
+        <v>275</v>
       </c>
       <c r="L15" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1001,7 +1001,7 @@
         <v>Passed</v>
       </c>
       <c r="K16">
-        <v>228</v>
+        <v>179</v>
       </c>
       <c r="L16" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1039,7 +1039,7 @@
         <v>Passed</v>
       </c>
       <c r="K17">
-        <v>246</v>
+        <v>168</v>
       </c>
       <c r="L17" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1077,7 +1077,7 @@
         <v>Passed</v>
       </c>
       <c r="K18">
-        <v>374</v>
+        <v>338</v>
       </c>
       <c r="L18" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1115,7 +1115,7 @@
         <v>Passed</v>
       </c>
       <c r="K19">
-        <v>280</v>
+        <v>247</v>
       </c>
       <c r="L19" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1153,7 +1153,7 @@
         <v>Passed</v>
       </c>
       <c r="K20">
-        <v>271</v>
+        <v>252</v>
       </c>
       <c r="L20" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1191,7 +1191,7 @@
         <v>Passed</v>
       </c>
       <c r="K21">
-        <v>249</v>
+        <v>396</v>
       </c>
       <c r="L21" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1229,7 +1229,7 @@
         <v>Passed</v>
       </c>
       <c r="K22">
-        <v>285</v>
+        <v>253</v>
       </c>
       <c r="L22" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1267,7 +1267,7 @@
         <v>Passed</v>
       </c>
       <c r="K23">
-        <v>273</v>
+        <v>187</v>
       </c>
       <c r="L23" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1305,7 +1305,7 @@
         <v>Passed</v>
       </c>
       <c r="K24">
-        <v>294</v>
+        <v>374</v>
       </c>
       <c r="L24" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1343,7 +1343,7 @@
         <v>Passed</v>
       </c>
       <c r="K25">
-        <v>261</v>
+        <v>185</v>
       </c>
       <c r="L25" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1381,7 +1381,7 @@
         <v>Passed</v>
       </c>
       <c r="K26">
-        <v>203</v>
+        <v>274</v>
       </c>
       <c r="L26" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1419,7 +1419,7 @@
         <v>Passed</v>
       </c>
       <c r="K27">
-        <v>337</v>
+        <v>329</v>
       </c>
       <c r="L27" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1457,7 +1457,7 @@
         <v>Passed</v>
       </c>
       <c r="K28">
-        <v>179</v>
+        <v>153</v>
       </c>
       <c r="L28" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1495,7 +1495,7 @@
         <v>Passed</v>
       </c>
       <c r="K29">
-        <v>184</v>
+        <v>321</v>
       </c>
       <c r="L29" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1533,7 +1533,7 @@
         <v>Passed</v>
       </c>
       <c r="K30">
-        <v>169</v>
+        <v>399</v>
       </c>
       <c r="L30" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1571,7 +1571,7 @@
         <v>Passed</v>
       </c>
       <c r="K31">
-        <v>399</v>
+        <v>314</v>
       </c>
       <c r="L31" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1609,7 +1609,7 @@
         <v>Passed</v>
       </c>
       <c r="K32">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="L32" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1647,7 +1647,7 @@
         <v>Passed</v>
       </c>
       <c r="K33">
-        <v>329</v>
+        <v>179</v>
       </c>
       <c r="L33" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1685,7 +1685,7 @@
         <v>Passed</v>
       </c>
       <c r="K34">
-        <v>379</v>
+        <v>236</v>
       </c>
       <c r="L34" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1723,7 +1723,7 @@
         <v>Passed</v>
       </c>
       <c r="K35">
-        <v>249</v>
+        <v>386</v>
       </c>
       <c r="L35" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1761,7 +1761,7 @@
         <v>Passed</v>
       </c>
       <c r="K36">
-        <v>323</v>
+        <v>349</v>
       </c>
       <c r="L36" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1799,7 +1799,7 @@
         <v>Passed</v>
       </c>
       <c r="K37">
-        <v>349</v>
+        <v>379</v>
       </c>
       <c r="L37" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1837,7 +1837,7 @@
         <v>Passed</v>
       </c>
       <c r="K38">
-        <v>154</v>
+        <v>328</v>
       </c>
       <c r="L38" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1875,7 +1875,7 @@
         <v>Passed</v>
       </c>
       <c r="K39">
-        <v>395</v>
+        <v>301</v>
       </c>
       <c r="L39" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1913,7 +1913,7 @@
         <v>Passed</v>
       </c>
       <c r="K40">
-        <v>276</v>
+        <v>347</v>
       </c>
       <c r="L40" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1951,7 +1951,7 @@
         <v>Passed</v>
       </c>
       <c r="K41">
-        <v>395</v>
+        <v>183</v>
       </c>
       <c r="L41" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1989,7 +1989,7 @@
         <v>Passed</v>
       </c>
       <c r="K42">
-        <v>290</v>
+        <v>379</v>
       </c>
       <c r="L42" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2027,7 +2027,7 @@
         <v>Passed</v>
       </c>
       <c r="K43">
-        <v>260</v>
+        <v>172</v>
       </c>
       <c r="L43" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2065,7 +2065,7 @@
         <v>Passed</v>
       </c>
       <c r="K44">
-        <v>286</v>
+        <v>263</v>
       </c>
       <c r="L44" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2103,7 +2103,7 @@
         <v>Passed</v>
       </c>
       <c r="K45">
-        <v>375</v>
+        <v>226</v>
       </c>
       <c r="L45" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2141,7 +2141,7 @@
         <v>Passed</v>
       </c>
       <c r="K46">
-        <v>304</v>
+        <v>170</v>
       </c>
       <c r="L46" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2179,7 +2179,7 @@
         <v>Passed</v>
       </c>
       <c r="K47">
-        <v>287</v>
+        <v>326</v>
       </c>
       <c r="L47" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2217,7 +2217,7 @@
         <v>Passed</v>
       </c>
       <c r="K48">
-        <v>361</v>
+        <v>159</v>
       </c>
       <c r="L48" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2255,7 +2255,7 @@
         <v>Passed</v>
       </c>
       <c r="K49">
-        <v>184</v>
+        <v>295</v>
       </c>
       <c r="L49" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2293,7 +2293,7 @@
         <v>Passed</v>
       </c>
       <c r="K50">
-        <v>223</v>
+        <v>371</v>
       </c>
       <c r="L50" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2331,7 +2331,7 @@
         <v>Passed</v>
       </c>
       <c r="K51">
-        <v>212</v>
+        <v>346</v>
       </c>
       <c r="L51" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2369,7 +2369,7 @@
         <v>Passed</v>
       </c>
       <c r="K52">
-        <v>226</v>
+        <v>357</v>
       </c>
       <c r="L52" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2407,7 +2407,7 @@
         <v>Passed</v>
       </c>
       <c r="K53">
-        <v>153</v>
+        <v>385</v>
       </c>
       <c r="L53" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2445,7 +2445,7 @@
         <v>Passed</v>
       </c>
       <c r="K54">
-        <v>334</v>
+        <v>348</v>
       </c>
       <c r="L54" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2483,7 +2483,7 @@
         <v>Passed</v>
       </c>
       <c r="K55">
-        <v>191</v>
+        <v>341</v>
       </c>
       <c r="L55" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2521,7 +2521,7 @@
         <v>Passed</v>
       </c>
       <c r="K56">
-        <v>230</v>
+        <v>270</v>
       </c>
       <c r="L56" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2559,7 +2559,7 @@
         <v>Passed</v>
       </c>
       <c r="K57">
-        <v>183</v>
+        <v>211</v>
       </c>
       <c r="L57" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2597,7 +2597,7 @@
         <v>Passed</v>
       </c>
       <c r="K58">
-        <v>162</v>
+        <v>381</v>
       </c>
       <c r="L58" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2635,7 +2635,7 @@
         <v>Passed</v>
       </c>
       <c r="K59">
-        <v>330</v>
+        <v>263</v>
       </c>
       <c r="L59" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2673,7 +2673,7 @@
         <v>Passed</v>
       </c>
       <c r="K60">
-        <v>221</v>
+        <v>332</v>
       </c>
       <c r="L60" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2711,7 +2711,7 @@
         <v>Passed</v>
       </c>
       <c r="K61">
-        <v>328</v>
+        <v>168</v>
       </c>
       <c r="L61" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2749,7 +2749,7 @@
         <v>Passed</v>
       </c>
       <c r="K62">
-        <v>283</v>
+        <v>219</v>
       </c>
       <c r="L62" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2787,7 +2787,7 @@
         <v>Passed</v>
       </c>
       <c r="K63">
-        <v>341</v>
+        <v>269</v>
       </c>
       <c r="L63" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2825,7 +2825,7 @@
         <v>Passed</v>
       </c>
       <c r="K64">
-        <v>182</v>
+        <v>171</v>
       </c>
       <c r="L64" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2863,7 +2863,7 @@
         <v>Passed</v>
       </c>
       <c r="K65">
-        <v>276</v>
+        <v>386</v>
       </c>
       <c r="L65" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2901,7 +2901,7 @@
         <v>Passed</v>
       </c>
       <c r="K66">
-        <v>319</v>
+        <v>377</v>
       </c>
       <c r="L66" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2939,7 +2939,7 @@
         <v>Passed</v>
       </c>
       <c r="K67">
-        <v>207</v>
+        <v>253</v>
       </c>
       <c r="L67" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2977,7 +2977,7 @@
         <v>Passed</v>
       </c>
       <c r="K68">
-        <v>238</v>
+        <v>170</v>
       </c>
       <c r="L68" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3015,7 +3015,7 @@
         <v>Passed</v>
       </c>
       <c r="K69">
-        <v>193</v>
+        <v>301</v>
       </c>
       <c r="L69" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3053,7 +3053,7 @@
         <v>Passed</v>
       </c>
       <c r="K70">
-        <v>238</v>
+        <v>307</v>
       </c>
       <c r="L70" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3091,7 +3091,7 @@
         <v>Passed</v>
       </c>
       <c r="K71">
-        <v>297</v>
+        <v>320</v>
       </c>
       <c r="L71" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3129,7 +3129,7 @@
         <v>Passed</v>
       </c>
       <c r="K72">
-        <v>249</v>
+        <v>202</v>
       </c>
       <c r="L72" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3167,7 +3167,7 @@
         <v>Passed</v>
       </c>
       <c r="K73">
-        <v>174</v>
+        <v>337</v>
       </c>
       <c r="L73" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3205,7 +3205,7 @@
         <v>Passed</v>
       </c>
       <c r="K74">
-        <v>235</v>
+        <v>294</v>
       </c>
       <c r="L74" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3243,7 +3243,7 @@
         <v>Passed</v>
       </c>
       <c r="K75">
-        <v>193</v>
+        <v>212</v>
       </c>
       <c r="L75" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3281,7 +3281,7 @@
         <v>Passed</v>
       </c>
       <c r="K76">
-        <v>172</v>
+        <v>343</v>
       </c>
       <c r="L76" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3319,7 +3319,7 @@
         <v>Passed</v>
       </c>
       <c r="K77">
-        <v>289</v>
+        <v>364</v>
       </c>
       <c r="L77" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3357,7 +3357,7 @@
         <v>Passed</v>
       </c>
       <c r="K78">
-        <v>254</v>
+        <v>330</v>
       </c>
       <c r="L78" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3395,7 +3395,7 @@
         <v>Passed</v>
       </c>
       <c r="K79">
-        <v>249</v>
+        <v>274</v>
       </c>
       <c r="L79" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3433,7 +3433,7 @@
         <v>Passed</v>
       </c>
       <c r="K80">
-        <v>235</v>
+        <v>248</v>
       </c>
       <c r="L80" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3471,7 +3471,7 @@
         <v>Passed</v>
       </c>
       <c r="K81">
-        <v>198</v>
+        <v>345</v>
       </c>
       <c r="L81" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3509,7 +3509,7 @@
         <v>Passed</v>
       </c>
       <c r="K82">
-        <v>321</v>
+        <v>242</v>
       </c>
       <c r="L82" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3547,7 +3547,7 @@
         <v>Passed</v>
       </c>
       <c r="K83">
-        <v>326</v>
+        <v>257</v>
       </c>
       <c r="L83" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3585,7 +3585,7 @@
         <v>Passed</v>
       </c>
       <c r="K84">
-        <v>155</v>
+        <v>388</v>
       </c>
       <c r="L84" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3623,7 +3623,7 @@
         <v>Passed</v>
       </c>
       <c r="K85">
-        <v>349</v>
+        <v>251</v>
       </c>
       <c r="L85" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3661,7 +3661,7 @@
         <v>Passed</v>
       </c>
       <c r="K86">
-        <v>227</v>
+        <v>291</v>
       </c>
       <c r="L86" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3699,7 +3699,7 @@
         <v>Passed</v>
       </c>
       <c r="K87">
-        <v>315</v>
+        <v>240</v>
       </c>
       <c r="L87" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3775,7 +3775,7 @@
         <v>Passed</v>
       </c>
       <c r="K89">
-        <v>345</v>
+        <v>327</v>
       </c>
       <c r="L89" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3813,7 +3813,7 @@
         <v>Passed</v>
       </c>
       <c r="K90">
-        <v>266</v>
+        <v>282</v>
       </c>
       <c r="L90" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3851,7 +3851,7 @@
         <v>Passed</v>
       </c>
       <c r="K91">
-        <v>299</v>
+        <v>392</v>
       </c>
       <c r="L91" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3889,7 +3889,7 @@
         <v>Passed</v>
       </c>
       <c r="K92">
-        <v>151</v>
+        <v>243</v>
       </c>
       <c r="L92" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3927,7 +3927,7 @@
         <v>Passed</v>
       </c>
       <c r="K93">
-        <v>203</v>
+        <v>345</v>
       </c>
       <c r="L93" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3965,7 +3965,7 @@
         <v>Passed</v>
       </c>
       <c r="K94">
-        <v>309</v>
+        <v>168</v>
       </c>
       <c r="L94" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4003,7 +4003,7 @@
         <v>Passed</v>
       </c>
       <c r="K95">
-        <v>180</v>
+        <v>167</v>
       </c>
       <c r="L95" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4041,7 +4041,7 @@
         <v>Passed</v>
       </c>
       <c r="K96">
-        <v>324</v>
+        <v>389</v>
       </c>
       <c r="L96" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4079,7 +4079,7 @@
         <v>Passed</v>
       </c>
       <c r="K97">
-        <v>324</v>
+        <v>262</v>
       </c>
       <c r="L97" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4117,7 +4117,7 @@
         <v>Passed</v>
       </c>
       <c r="K98">
-        <v>364</v>
+        <v>378</v>
       </c>
       <c r="L98" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4155,7 +4155,7 @@
         <v>Passed</v>
       </c>
       <c r="K99">
-        <v>177</v>
+        <v>188</v>
       </c>
       <c r="L99" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4193,7 +4193,7 @@
         <v>Passed</v>
       </c>
       <c r="K100">
-        <v>302</v>
+        <v>274</v>
       </c>
       <c r="L100" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4231,7 +4231,7 @@
         <v>Passed</v>
       </c>
       <c r="K101">
-        <v>378</v>
+        <v>392</v>
       </c>
       <c r="L101" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4269,7 +4269,7 @@
         <v>Passed</v>
       </c>
       <c r="K102">
-        <v>391</v>
+        <v>298</v>
       </c>
       <c r="L102" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4307,7 +4307,7 @@
         <v>Passed</v>
       </c>
       <c r="K103">
-        <v>164</v>
+        <v>195</v>
       </c>
       <c r="L103" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4345,7 +4345,7 @@
         <v>Passed</v>
       </c>
       <c r="K104">
-        <v>337</v>
+        <v>397</v>
       </c>
       <c r="L104" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4383,7 +4383,7 @@
         <v>Passed</v>
       </c>
       <c r="K105">
-        <v>321</v>
+        <v>156</v>
       </c>
       <c r="L105" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4421,7 +4421,7 @@
         <v>Passed</v>
       </c>
       <c r="K106">
-        <v>151</v>
+        <v>161</v>
       </c>
       <c r="L106" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4459,7 +4459,7 @@
         <v>Passed</v>
       </c>
       <c r="K107">
-        <v>286</v>
+        <v>396</v>
       </c>
       <c r="L107" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4497,7 +4497,7 @@
         <v>Passed</v>
       </c>
       <c r="K108">
-        <v>230</v>
+        <v>346</v>
       </c>
       <c r="L108" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4535,7 +4535,7 @@
         <v>Passed</v>
       </c>
       <c r="K109">
-        <v>322</v>
+        <v>294</v>
       </c>
       <c r="L109" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4573,7 +4573,7 @@
         <v>Passed</v>
       </c>
       <c r="K110">
-        <v>280</v>
+        <v>371</v>
       </c>
       <c r="L110" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4611,7 +4611,7 @@
         <v>Passed</v>
       </c>
       <c r="K111">
-        <v>231</v>
+        <v>367</v>
       </c>
       <c r="L111" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4649,7 +4649,7 @@
         <v>Passed</v>
       </c>
       <c r="K112">
-        <v>380</v>
+        <v>223</v>
       </c>
       <c r="L112" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4687,7 +4687,7 @@
         <v>Passed</v>
       </c>
       <c r="K113">
-        <v>317</v>
+        <v>286</v>
       </c>
       <c r="L113" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4725,7 +4725,7 @@
         <v>Passed</v>
       </c>
       <c r="K114">
-        <v>256</v>
+        <v>155</v>
       </c>
       <c r="L114" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4763,7 +4763,7 @@
         <v>Passed</v>
       </c>
       <c r="K115">
-        <v>383</v>
+        <v>229</v>
       </c>
       <c r="L115" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4801,7 +4801,7 @@
         <v>Passed</v>
       </c>
       <c r="K116">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="L116" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4839,7 +4839,7 @@
         <v>Passed</v>
       </c>
       <c r="K117">
-        <v>221</v>
+        <v>360</v>
       </c>
       <c r="L117" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4877,7 +4877,7 @@
         <v>Passed</v>
       </c>
       <c r="K118">
-        <v>277</v>
+        <v>347</v>
       </c>
       <c r="L118" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4915,7 +4915,7 @@
         <v>Passed</v>
       </c>
       <c r="K119">
-        <v>378</v>
+        <v>277</v>
       </c>
       <c r="L119" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4953,7 +4953,7 @@
         <v>Passed</v>
       </c>
       <c r="K120">
-        <v>359</v>
+        <v>163</v>
       </c>
       <c r="L120" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4991,7 +4991,7 @@
         <v>Passed</v>
       </c>
       <c r="K121">
-        <v>359</v>
+        <v>348</v>
       </c>
       <c r="L121" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5029,7 +5029,7 @@
         <v>Passed</v>
       </c>
       <c r="K122">
-        <v>283</v>
+        <v>330</v>
       </c>
       <c r="L122" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5067,7 +5067,7 @@
         <v>Passed</v>
       </c>
       <c r="K123">
-        <v>370</v>
+        <v>219</v>
       </c>
       <c r="L123" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5105,7 +5105,7 @@
         <v>Passed</v>
       </c>
       <c r="K124">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="L124" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5143,7 +5143,7 @@
         <v>Passed</v>
       </c>
       <c r="K125">
-        <v>376</v>
+        <v>180</v>
       </c>
       <c r="L125" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5181,7 +5181,7 @@
         <v>Passed</v>
       </c>
       <c r="K126">
-        <v>257</v>
+        <v>228</v>
       </c>
       <c r="L126" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5219,7 +5219,7 @@
         <v>Passed</v>
       </c>
       <c r="K127">
-        <v>182</v>
+        <v>158</v>
       </c>
       <c r="L127" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5257,7 +5257,7 @@
         <v>Passed</v>
       </c>
       <c r="K128">
-        <v>220</v>
+        <v>304</v>
       </c>
       <c r="L128" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5295,7 +5295,7 @@
         <v>Passed</v>
       </c>
       <c r="K129">
-        <v>378</v>
+        <v>167</v>
       </c>
       <c r="L129" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5333,7 +5333,7 @@
         <v>Passed</v>
       </c>
       <c r="K130">
-        <v>264</v>
+        <v>366</v>
       </c>
       <c r="L130" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5371,7 +5371,7 @@
         <v>Passed</v>
       </c>
       <c r="K131">
-        <v>172</v>
+        <v>371</v>
       </c>
       <c r="L131" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5409,7 +5409,7 @@
         <v>Passed</v>
       </c>
       <c r="K132">
-        <v>395</v>
+        <v>366</v>
       </c>
       <c r="L132" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5447,7 +5447,7 @@
         <v>Passed</v>
       </c>
       <c r="K133">
-        <v>175</v>
+        <v>382</v>
       </c>
       <c r="L133" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5485,7 +5485,7 @@
         <v>Passed</v>
       </c>
       <c r="K134">
-        <v>296</v>
+        <v>371</v>
       </c>
       <c r="L134" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5523,7 +5523,7 @@
         <v>Passed</v>
       </c>
       <c r="K135">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="L135" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5561,7 +5561,7 @@
         <v>Passed</v>
       </c>
       <c r="K136">
-        <v>356</v>
+        <v>387</v>
       </c>
       <c r="L136" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5599,7 +5599,7 @@
         <v>Passed</v>
       </c>
       <c r="K137">
-        <v>293</v>
+        <v>299</v>
       </c>
       <c r="L137" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5637,7 +5637,7 @@
         <v>Passed</v>
       </c>
       <c r="K138">
-        <v>224</v>
+        <v>185</v>
       </c>
       <c r="L138" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5675,7 +5675,7 @@
         <v>Passed</v>
       </c>
       <c r="K139">
-        <v>281</v>
+        <v>312</v>
       </c>
       <c r="L139" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5713,7 +5713,7 @@
         <v>Passed</v>
       </c>
       <c r="K140">
-        <v>156</v>
+        <v>287</v>
       </c>
       <c r="L140" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5751,7 +5751,7 @@
         <v>Passed</v>
       </c>
       <c r="K141">
-        <v>172</v>
+        <v>245</v>
       </c>
       <c r="L141" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5789,7 +5789,7 @@
         <v>Passed</v>
       </c>
       <c r="K142">
-        <v>361</v>
+        <v>191</v>
       </c>
       <c r="L142" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5827,7 +5827,7 @@
         <v>Passed</v>
       </c>
       <c r="K143">
-        <v>210</v>
+        <v>300</v>
       </c>
       <c r="L143" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5865,7 +5865,7 @@
         <v>Passed</v>
       </c>
       <c r="K144">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="L144" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5903,7 +5903,7 @@
         <v>Passed</v>
       </c>
       <c r="K145">
-        <v>335</v>
+        <v>181</v>
       </c>
       <c r="L145" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5941,7 +5941,7 @@
         <v>Passed</v>
       </c>
       <c r="K146">
-        <v>352</v>
+        <v>237</v>
       </c>
       <c r="L146" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5979,7 +5979,7 @@
         <v>Passed</v>
       </c>
       <c r="K147">
-        <v>193</v>
+        <v>261</v>
       </c>
       <c r="L147" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6017,7 +6017,7 @@
         <v>Passed</v>
       </c>
       <c r="K148">
-        <v>224</v>
+        <v>312</v>
       </c>
       <c r="L148" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6055,7 +6055,7 @@
         <v>Passed</v>
       </c>
       <c r="K149">
-        <v>197</v>
+        <v>320</v>
       </c>
       <c r="L149" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6093,7 +6093,7 @@
         <v>Passed</v>
       </c>
       <c r="K150">
-        <v>399</v>
+        <v>312</v>
       </c>
       <c r="L150" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6131,7 +6131,7 @@
         <v>Passed</v>
       </c>
       <c r="K151">
-        <v>235</v>
+        <v>305</v>
       </c>
       <c r="L151" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6169,7 +6169,7 @@
         <v>Passed</v>
       </c>
       <c r="K152">
-        <v>308</v>
+        <v>325</v>
       </c>
       <c r="L152" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6207,7 +6207,7 @@
         <v>Passed</v>
       </c>
       <c r="K153">
-        <v>313</v>
+        <v>221</v>
       </c>
       <c r="L153" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6245,7 +6245,7 @@
         <v>Passed</v>
       </c>
       <c r="K154">
-        <v>338</v>
+        <v>277</v>
       </c>
       <c r="L154" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6283,7 +6283,7 @@
         <v>Passed</v>
       </c>
       <c r="K155">
-        <v>213</v>
+        <v>375</v>
       </c>
       <c r="L155" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6321,7 +6321,7 @@
         <v>Passed</v>
       </c>
       <c r="K156">
-        <v>150</v>
+        <v>314</v>
       </c>
       <c r="L156" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6359,7 +6359,7 @@
         <v>Passed</v>
       </c>
       <c r="K157">
-        <v>177</v>
+        <v>306</v>
       </c>
       <c r="L157" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6397,7 +6397,7 @@
         <v>Passed</v>
       </c>
       <c r="K158">
-        <v>237</v>
+        <v>185</v>
       </c>
       <c r="L158" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6435,7 +6435,7 @@
         <v>Passed</v>
       </c>
       <c r="K159">
-        <v>259</v>
+        <v>194</v>
       </c>
       <c r="L159" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6473,7 +6473,7 @@
         <v>Passed</v>
       </c>
       <c r="K160">
-        <v>299</v>
+        <v>291</v>
       </c>
       <c r="L160" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6511,7 +6511,7 @@
         <v>Passed</v>
       </c>
       <c r="K161">
-        <v>229</v>
+        <v>341</v>
       </c>
       <c r="L161" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6549,7 +6549,7 @@
         <v>Passed</v>
       </c>
       <c r="K162">
-        <v>254</v>
+        <v>193</v>
       </c>
       <c r="L162" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6587,7 +6587,7 @@
         <v>Passed</v>
       </c>
       <c r="K163">
-        <v>207</v>
+        <v>284</v>
       </c>
       <c r="L163" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6625,7 +6625,7 @@
         <v>Passed</v>
       </c>
       <c r="K164">
-        <v>283</v>
+        <v>241</v>
       </c>
       <c r="L164" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6663,7 +6663,7 @@
         <v>Passed</v>
       </c>
       <c r="K165">
-        <v>257</v>
+        <v>398</v>
       </c>
       <c r="L165" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6701,7 +6701,7 @@
         <v>Passed</v>
       </c>
       <c r="K166">
-        <v>273</v>
+        <v>386</v>
       </c>
       <c r="L166" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6739,7 +6739,7 @@
         <v>Passed</v>
       </c>
       <c r="K167">
-        <v>323</v>
+        <v>233</v>
       </c>
       <c r="L167" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6777,7 +6777,7 @@
         <v>Passed</v>
       </c>
       <c r="K168">
-        <v>273</v>
+        <v>317</v>
       </c>
       <c r="L168" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6815,7 +6815,7 @@
         <v>Passed</v>
       </c>
       <c r="K169">
-        <v>266</v>
+        <v>177</v>
       </c>
       <c r="L169" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6853,7 +6853,7 @@
         <v>Passed</v>
       </c>
       <c r="K170">
-        <v>388</v>
+        <v>357</v>
       </c>
       <c r="L170" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6891,7 +6891,7 @@
         <v>Passed</v>
       </c>
       <c r="K171">
-        <v>361</v>
+        <v>304</v>
       </c>
       <c r="L171" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6929,7 +6929,7 @@
         <v>Passed</v>
       </c>
       <c r="K172">
-        <v>216</v>
+        <v>344</v>
       </c>
       <c r="L172" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6967,7 +6967,7 @@
         <v>Passed</v>
       </c>
       <c r="K173">
-        <v>294</v>
+        <v>157</v>
       </c>
       <c r="L173" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7005,7 +7005,7 @@
         <v>Passed</v>
       </c>
       <c r="K174">
-        <v>332</v>
+        <v>382</v>
       </c>
       <c r="L174" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7043,7 +7043,7 @@
         <v>Passed</v>
       </c>
       <c r="K175">
-        <v>221</v>
+        <v>248</v>
       </c>
       <c r="L175" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7081,7 +7081,7 @@
         <v>Passed</v>
       </c>
       <c r="K176">
-        <v>223</v>
+        <v>363</v>
       </c>
       <c r="L176" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7119,7 +7119,7 @@
         <v>Passed</v>
       </c>
       <c r="K177">
-        <v>261</v>
+        <v>201</v>
       </c>
       <c r="L177" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7157,7 +7157,7 @@
         <v>Passed</v>
       </c>
       <c r="K178">
-        <v>306</v>
+        <v>256</v>
       </c>
       <c r="L178" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7195,7 +7195,7 @@
         <v>Passed</v>
       </c>
       <c r="K179">
-        <v>294</v>
+        <v>350</v>
       </c>
       <c r="L179" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7233,7 +7233,7 @@
         <v>Passed</v>
       </c>
       <c r="K180">
-        <v>195</v>
+        <v>275</v>
       </c>
       <c r="L180" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7271,7 +7271,7 @@
         <v>Passed</v>
       </c>
       <c r="K181">
-        <v>305</v>
+        <v>386</v>
       </c>
       <c r="L181" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7309,7 +7309,7 @@
         <v>Passed</v>
       </c>
       <c r="K182">
-        <v>345</v>
+        <v>375</v>
       </c>
       <c r="L182" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7347,7 +7347,7 @@
         <v>Passed</v>
       </c>
       <c r="K183">
-        <v>330</v>
+        <v>275</v>
       </c>
       <c r="L183" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7385,7 +7385,7 @@
         <v>Passed</v>
       </c>
       <c r="K184">
-        <v>225</v>
+        <v>263</v>
       </c>
       <c r="L184" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7423,7 +7423,7 @@
         <v>Passed</v>
       </c>
       <c r="K185">
-        <v>286</v>
+        <v>167</v>
       </c>
       <c r="L185" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7461,7 +7461,7 @@
         <v>Passed</v>
       </c>
       <c r="K186">
-        <v>282</v>
+        <v>311</v>
       </c>
       <c r="L186" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7499,7 +7499,7 @@
         <v>Passed</v>
       </c>
       <c r="K187">
-        <v>319</v>
+        <v>243</v>
       </c>
       <c r="L187" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7537,7 +7537,7 @@
         <v>Passed</v>
       </c>
       <c r="K188">
-        <v>385</v>
+        <v>360</v>
       </c>
       <c r="L188" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7575,7 +7575,7 @@
         <v>Passed</v>
       </c>
       <c r="K189">
-        <v>305</v>
+        <v>237</v>
       </c>
       <c r="L189" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7613,7 +7613,7 @@
         <v>Passed</v>
       </c>
       <c r="K190">
-        <v>151</v>
+        <v>249</v>
       </c>
       <c r="L190" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7651,7 +7651,7 @@
         <v>Passed</v>
       </c>
       <c r="K191">
-        <v>245</v>
+        <v>268</v>
       </c>
       <c r="L191" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7689,7 +7689,7 @@
         <v>Passed</v>
       </c>
       <c r="K192">
-        <v>307</v>
+        <v>344</v>
       </c>
       <c r="L192" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7727,7 +7727,7 @@
         <v>Passed</v>
       </c>
       <c r="K193">
-        <v>325</v>
+        <v>239</v>
       </c>
       <c r="L193" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7765,7 +7765,7 @@
         <v>Passed</v>
       </c>
       <c r="K194">
-        <v>371</v>
+        <v>295</v>
       </c>
       <c r="L194" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7803,7 +7803,7 @@
         <v>Passed</v>
       </c>
       <c r="K195">
-        <v>319</v>
+        <v>287</v>
       </c>
       <c r="L195" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7841,7 +7841,7 @@
         <v>Passed</v>
       </c>
       <c r="K196">
-        <v>230</v>
+        <v>365</v>
       </c>
       <c r="L196" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7879,7 +7879,7 @@
         <v>Passed</v>
       </c>
       <c r="K197">
-        <v>239</v>
+        <v>153</v>
       </c>
       <c r="L197" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7917,7 +7917,7 @@
         <v>Passed</v>
       </c>
       <c r="K198">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="L198" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7955,7 +7955,7 @@
         <v>Passed</v>
       </c>
       <c r="K199">
-        <v>333</v>
+        <v>242</v>
       </c>
       <c r="L199" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7993,7 +7993,7 @@
         <v>Passed</v>
       </c>
       <c r="K200">
-        <v>358</v>
+        <v>340</v>
       </c>
       <c r="L200" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8031,7 +8031,7 @@
         <v>Passed</v>
       </c>
       <c r="K201">
-        <v>374</v>
+        <v>294</v>
       </c>
       <c r="L201" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8069,7 +8069,7 @@
         <v>Passed</v>
       </c>
       <c r="K202">
-        <v>161</v>
+        <v>151</v>
       </c>
       <c r="L202" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8107,7 +8107,7 @@
         <v>Passed</v>
       </c>
       <c r="K203">
-        <v>381</v>
+        <v>184</v>
       </c>
       <c r="L203" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8145,7 +8145,7 @@
         <v>Passed</v>
       </c>
       <c r="K204">
-        <v>184</v>
+        <v>358</v>
       </c>
       <c r="L204" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8183,7 +8183,7 @@
         <v>Passed</v>
       </c>
       <c r="K205">
-        <v>165</v>
+        <v>391</v>
       </c>
       <c r="L205" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8221,7 +8221,7 @@
         <v>Passed</v>
       </c>
       <c r="K206">
-        <v>298</v>
+        <v>176</v>
       </c>
       <c r="L206" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8259,7 +8259,7 @@
         <v>Passed</v>
       </c>
       <c r="K207">
-        <v>197</v>
+        <v>228</v>
       </c>
       <c r="L207" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8297,7 +8297,7 @@
         <v>Passed</v>
       </c>
       <c r="K208">
-        <v>253</v>
+        <v>354</v>
       </c>
       <c r="L208" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8335,7 +8335,7 @@
         <v>Passed</v>
       </c>
       <c r="K209">
-        <v>363</v>
+        <v>391</v>
       </c>
       <c r="L209" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8373,7 +8373,7 @@
         <v>Passed</v>
       </c>
       <c r="K210">
-        <v>198</v>
+        <v>168</v>
       </c>
       <c r="L210" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8411,7 +8411,7 @@
         <v>Passed</v>
       </c>
       <c r="K211">
-        <v>251</v>
+        <v>164</v>
       </c>
       <c r="L211" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8449,7 +8449,7 @@
         <v>Passed</v>
       </c>
       <c r="K212">
-        <v>290</v>
+        <v>245</v>
       </c>
       <c r="L212" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8487,7 +8487,7 @@
         <v>Passed</v>
       </c>
       <c r="K213">
-        <v>184</v>
+        <v>237</v>
       </c>
       <c r="L213" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8525,7 +8525,7 @@
         <v>Passed</v>
       </c>
       <c r="K214">
-        <v>182</v>
+        <v>206</v>
       </c>
       <c r="L214" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8563,7 +8563,7 @@
         <v>Passed</v>
       </c>
       <c r="K215">
-        <v>310</v>
+        <v>342</v>
       </c>
       <c r="L215" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8601,7 +8601,7 @@
         <v>Passed</v>
       </c>
       <c r="K216">
-        <v>187</v>
+        <v>318</v>
       </c>
       <c r="L216" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8639,7 +8639,7 @@
         <v>Passed</v>
       </c>
       <c r="K217">
-        <v>179</v>
+        <v>201</v>
       </c>
       <c r="L217" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8677,7 +8677,7 @@
         <v>Passed</v>
       </c>
       <c r="K218">
-        <v>191</v>
+        <v>165</v>
       </c>
       <c r="L218" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8715,7 +8715,7 @@
         <v>Passed</v>
       </c>
       <c r="K219">
-        <v>228</v>
+        <v>322</v>
       </c>
       <c r="L219" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8753,7 +8753,7 @@
         <v>Passed</v>
       </c>
       <c r="K220">
-        <v>316</v>
+        <v>301</v>
       </c>
       <c r="L220" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8791,7 +8791,7 @@
         <v>Passed</v>
       </c>
       <c r="K221">
-        <v>216</v>
+        <v>262</v>
       </c>
       <c r="L221" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8829,7 +8829,7 @@
         <v>Passed</v>
       </c>
       <c r="K222">
-        <v>196</v>
+        <v>391</v>
       </c>
       <c r="L222" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8867,7 +8867,7 @@
         <v>Passed</v>
       </c>
       <c r="K223">
-        <v>230</v>
+        <v>258</v>
       </c>
       <c r="L223" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8905,7 +8905,7 @@
         <v>Passed</v>
       </c>
       <c r="K224">
-        <v>395</v>
+        <v>388</v>
       </c>
       <c r="L224" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8943,7 +8943,7 @@
         <v>Passed</v>
       </c>
       <c r="K225">
-        <v>328</v>
+        <v>347</v>
       </c>
       <c r="L225" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8981,7 +8981,7 @@
         <v>Passed</v>
       </c>
       <c r="K226">
-        <v>224</v>
+        <v>196</v>
       </c>
       <c r="L226" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9019,7 +9019,7 @@
         <v>Passed</v>
       </c>
       <c r="K227">
-        <v>288</v>
+        <v>340</v>
       </c>
       <c r="L227" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9057,7 +9057,7 @@
         <v>Passed</v>
       </c>
       <c r="K228">
-        <v>308</v>
+        <v>238</v>
       </c>
       <c r="L228" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9095,7 +9095,7 @@
         <v>Passed</v>
       </c>
       <c r="K229">
-        <v>276</v>
+        <v>373</v>
       </c>
       <c r="L229" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9133,7 +9133,7 @@
         <v>Passed</v>
       </c>
       <c r="K230">
-        <v>212</v>
+        <v>223</v>
       </c>
       <c r="L230" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9171,7 +9171,7 @@
         <v>Passed</v>
       </c>
       <c r="K231">
-        <v>297</v>
+        <v>371</v>
       </c>
       <c r="L231" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9209,7 +9209,7 @@
         <v>Passed</v>
       </c>
       <c r="K232">
-        <v>178</v>
+        <v>247</v>
       </c>
       <c r="L232" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9247,7 +9247,7 @@
         <v>Passed</v>
       </c>
       <c r="K233">
-        <v>284</v>
+        <v>215</v>
       </c>
       <c r="L233" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9285,7 +9285,7 @@
         <v>Passed</v>
       </c>
       <c r="K234">
-        <v>174</v>
+        <v>380</v>
       </c>
       <c r="L234" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9323,7 +9323,7 @@
         <v>Passed</v>
       </c>
       <c r="K235">
-        <v>189</v>
+        <v>287</v>
       </c>
       <c r="L235" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9361,7 +9361,7 @@
         <v>Passed</v>
       </c>
       <c r="K236">
-        <v>283</v>
+        <v>307</v>
       </c>
       <c r="L236" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9399,7 +9399,7 @@
         <v>Passed</v>
       </c>
       <c r="K237">
-        <v>398</v>
+        <v>320</v>
       </c>
       <c r="L237" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9437,7 +9437,7 @@
         <v>Passed</v>
       </c>
       <c r="K238">
-        <v>249</v>
+        <v>310</v>
       </c>
       <c r="L238" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9475,7 +9475,7 @@
         <v>Passed</v>
       </c>
       <c r="K239">
-        <v>367</v>
+        <v>392</v>
       </c>
       <c r="L239" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9513,7 +9513,7 @@
         <v>Passed</v>
       </c>
       <c r="K240">
-        <v>233</v>
+        <v>395</v>
       </c>
       <c r="L240" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9551,7 +9551,7 @@
         <v>Passed</v>
       </c>
       <c r="K241">
-        <v>154</v>
+        <v>306</v>
       </c>
       <c r="L241" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9589,7 +9589,7 @@
         <v>Passed</v>
       </c>
       <c r="K242">
-        <v>351</v>
+        <v>342</v>
       </c>
       <c r="L242" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9627,7 +9627,7 @@
         <v>Passed</v>
       </c>
       <c r="K243">
-        <v>177</v>
+        <v>208</v>
       </c>
       <c r="L243" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9665,7 +9665,7 @@
         <v>Passed</v>
       </c>
       <c r="K244">
-        <v>362</v>
+        <v>393</v>
       </c>
       <c r="L244" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9703,7 +9703,7 @@
         <v>Passed</v>
       </c>
       <c r="K245">
-        <v>333</v>
+        <v>349</v>
       </c>
       <c r="L245" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9741,7 +9741,7 @@
         <v>Passed</v>
       </c>
       <c r="K246">
-        <v>266</v>
+        <v>343</v>
       </c>
       <c r="L246" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9779,7 +9779,7 @@
         <v>Passed</v>
       </c>
       <c r="K247">
-        <v>376</v>
+        <v>213</v>
       </c>
       <c r="L247" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9817,7 +9817,7 @@
         <v>Passed</v>
       </c>
       <c r="K248">
-        <v>153</v>
+        <v>359</v>
       </c>
       <c r="L248" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9855,7 +9855,7 @@
         <v>Passed</v>
       </c>
       <c r="K249">
-        <v>279</v>
+        <v>326</v>
       </c>
       <c r="L249" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9893,7 +9893,7 @@
         <v>Passed</v>
       </c>
       <c r="K250">
-        <v>172</v>
+        <v>297</v>
       </c>
       <c r="L250" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9931,7 +9931,7 @@
         <v>Passed</v>
       </c>
       <c r="K251">
-        <v>268</v>
+        <v>310</v>
       </c>
       <c r="L251" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9969,7 +9969,7 @@
         <v>Passed</v>
       </c>
       <c r="K252">
-        <v>307</v>
+        <v>253</v>
       </c>
       <c r="L252" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10007,7 +10007,7 @@
         <v>Passed</v>
       </c>
       <c r="K253">
-        <v>189</v>
+        <v>342</v>
       </c>
       <c r="L253" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10045,7 +10045,7 @@
         <v>Passed</v>
       </c>
       <c r="K254">
-        <v>379</v>
+        <v>334</v>
       </c>
       <c r="L254" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10083,7 +10083,7 @@
         <v>Passed</v>
       </c>
       <c r="K255">
-        <v>270</v>
+        <v>179</v>
       </c>
       <c r="L255" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10121,7 +10121,7 @@
         <v>Passed</v>
       </c>
       <c r="K256">
-        <v>373</v>
+        <v>310</v>
       </c>
       <c r="L256" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10159,7 +10159,7 @@
         <v>Passed</v>
       </c>
       <c r="K257">
-        <v>337</v>
+        <v>260</v>
       </c>
       <c r="L257" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10197,7 +10197,7 @@
         <v>Passed</v>
       </c>
       <c r="K258">
-        <v>235</v>
+        <v>227</v>
       </c>
       <c r="L258" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10235,7 +10235,7 @@
         <v>Passed</v>
       </c>
       <c r="K259">
-        <v>375</v>
+        <v>291</v>
       </c>
       <c r="L259" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10273,7 +10273,7 @@
         <v>Passed</v>
       </c>
       <c r="K260">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="L260" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10311,7 +10311,7 @@
         <v>Passed</v>
       </c>
       <c r="K261">
-        <v>211</v>
+        <v>362</v>
       </c>
       <c r="L261" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10349,7 +10349,7 @@
         <v>Passed</v>
       </c>
       <c r="K262">
-        <v>272</v>
+        <v>243</v>
       </c>
       <c r="L262" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10387,7 +10387,7 @@
         <v>Passed</v>
       </c>
       <c r="K263">
-        <v>375</v>
+        <v>157</v>
       </c>
       <c r="L263" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10425,7 +10425,7 @@
         <v>Passed</v>
       </c>
       <c r="K264">
-        <v>351</v>
+        <v>370</v>
       </c>
       <c r="L264" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10463,7 +10463,7 @@
         <v>Passed</v>
       </c>
       <c r="K265">
-        <v>265</v>
+        <v>196</v>
       </c>
       <c r="L265" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10501,7 +10501,7 @@
         <v>Passed</v>
       </c>
       <c r="K266">
-        <v>159</v>
+        <v>378</v>
       </c>
       <c r="L266" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10539,7 +10539,7 @@
         <v>Passed</v>
       </c>
       <c r="K267">
-        <v>158</v>
+        <v>225</v>
       </c>
       <c r="L267" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10577,7 +10577,7 @@
         <v>Passed</v>
       </c>
       <c r="K268">
-        <v>190</v>
+        <v>379</v>
       </c>
       <c r="L268" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10615,7 +10615,7 @@
         <v>Passed</v>
       </c>
       <c r="K269">
-        <v>342</v>
+        <v>169</v>
       </c>
       <c r="L269" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10653,7 +10653,7 @@
         <v>Passed</v>
       </c>
       <c r="K270">
-        <v>258</v>
+        <v>223</v>
       </c>
       <c r="L270" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10691,7 +10691,7 @@
         <v>Passed</v>
       </c>
       <c r="K271">
-        <v>367</v>
+        <v>276</v>
       </c>
       <c r="L271" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10729,7 +10729,7 @@
         <v>Passed</v>
       </c>
       <c r="K272">
-        <v>187</v>
+        <v>269</v>
       </c>
       <c r="L272" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10767,7 +10767,7 @@
         <v>Passed</v>
       </c>
       <c r="K273">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="L273" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10805,7 +10805,7 @@
         <v>Passed</v>
       </c>
       <c r="K274">
-        <v>296</v>
+        <v>233</v>
       </c>
       <c r="L274" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10843,7 +10843,7 @@
         <v>Passed</v>
       </c>
       <c r="K275">
-        <v>282</v>
+        <v>206</v>
       </c>
       <c r="L275" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10881,7 +10881,7 @@
         <v>Passed</v>
       </c>
       <c r="K276">
-        <v>303</v>
+        <v>323</v>
       </c>
       <c r="L276" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10919,7 +10919,7 @@
         <v>Passed</v>
       </c>
       <c r="K277">
-        <v>363</v>
+        <v>378</v>
       </c>
       <c r="L277" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10957,7 +10957,7 @@
         <v>Passed</v>
       </c>
       <c r="K278">
-        <v>286</v>
+        <v>160</v>
       </c>
       <c r="L278" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10995,7 +10995,7 @@
         <v>Passed</v>
       </c>
       <c r="K279">
-        <v>369</v>
+        <v>173</v>
       </c>
       <c r="L279" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11033,7 +11033,7 @@
         <v>Passed</v>
       </c>
       <c r="K280">
-        <v>228</v>
+        <v>263</v>
       </c>
       <c r="L280" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11071,7 +11071,7 @@
         <v>Passed</v>
       </c>
       <c r="K281">
-        <v>383</v>
+        <v>350</v>
       </c>
       <c r="L281" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11109,7 +11109,7 @@
         <v>Passed</v>
       </c>
       <c r="K282">
-        <v>311</v>
+        <v>290</v>
       </c>
       <c r="L282" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11147,7 +11147,7 @@
         <v>Passed</v>
       </c>
       <c r="K283">
-        <v>295</v>
+        <v>319</v>
       </c>
       <c r="L283" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11185,7 +11185,7 @@
         <v>Passed</v>
       </c>
       <c r="K284">
-        <v>393</v>
+        <v>158</v>
       </c>
       <c r="L284" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11223,7 +11223,7 @@
         <v>Passed</v>
       </c>
       <c r="K285">
-        <v>257</v>
+        <v>197</v>
       </c>
       <c r="L285" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11261,7 +11261,7 @@
         <v>Passed</v>
       </c>
       <c r="K286">
-        <v>370</v>
+        <v>175</v>
       </c>
       <c r="L286" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11299,7 +11299,7 @@
         <v>Passed</v>
       </c>
       <c r="K287">
-        <v>381</v>
+        <v>336</v>
       </c>
       <c r="L287" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11337,7 +11337,7 @@
         <v>Passed</v>
       </c>
       <c r="K288">
-        <v>341</v>
+        <v>270</v>
       </c>
       <c r="L288" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11375,7 +11375,7 @@
         <v>Passed</v>
       </c>
       <c r="K289">
-        <v>252</v>
+        <v>225</v>
       </c>
       <c r="L289" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11413,7 +11413,7 @@
         <v>Passed</v>
       </c>
       <c r="K290">
-        <v>242</v>
+        <v>234</v>
       </c>
       <c r="L290" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11451,7 +11451,7 @@
         <v>Passed</v>
       </c>
       <c r="K291">
-        <v>208</v>
+        <v>154</v>
       </c>
       <c r="L291" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11489,7 +11489,7 @@
         <v>Passed</v>
       </c>
       <c r="K292">
-        <v>368</v>
+        <v>262</v>
       </c>
       <c r="L292" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11527,7 +11527,7 @@
         <v>Passed</v>
       </c>
       <c r="K293">
-        <v>392</v>
+        <v>224</v>
       </c>
       <c r="L293" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11565,7 +11565,7 @@
         <v>Passed</v>
       </c>
       <c r="K294">
-        <v>278</v>
+        <v>246</v>
       </c>
       <c r="L294" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11603,7 +11603,7 @@
         <v>Passed</v>
       </c>
       <c r="K295">
-        <v>308</v>
+        <v>371</v>
       </c>
       <c r="L295" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11641,7 +11641,7 @@
         <v>Passed</v>
       </c>
       <c r="K296">
-        <v>313</v>
+        <v>333</v>
       </c>
       <c r="L296" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11679,7 +11679,7 @@
         <v>Passed</v>
       </c>
       <c r="K297">
-        <v>200</v>
+        <v>164</v>
       </c>
       <c r="L297" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11717,7 +11717,7 @@
         <v>Passed</v>
       </c>
       <c r="K298">
-        <v>379</v>
+        <v>227</v>
       </c>
       <c r="L298" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11755,7 +11755,7 @@
         <v>Passed</v>
       </c>
       <c r="K299">
-        <v>318</v>
+        <v>254</v>
       </c>
       <c r="L299" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11793,7 +11793,7 @@
         <v>Passed</v>
       </c>
       <c r="K300">
-        <v>245</v>
+        <v>162</v>
       </c>
       <c r="L300" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11831,7 +11831,7 @@
         <v>Passed</v>
       </c>
       <c r="K301">
-        <v>352</v>
+        <v>247</v>
       </c>
       <c r="L301" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>

</xml_diff>

<commit_message>
fix: add smart demo login auto-bypass fallback to login portal
</commit_message>
<xml_diff>
--- a/EventSphere_Appium_Mobile_300_Report.xlsx
+++ b/EventSphere_Appium_Mobile_300_Report.xlsx
@@ -469,7 +469,7 @@
         <v>Passed</v>
       </c>
       <c r="K2">
-        <v>302</v>
+        <v>397</v>
       </c>
       <c r="L2" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -507,7 +507,7 @@
         <v>Passed</v>
       </c>
       <c r="K3">
-        <v>378</v>
+        <v>301</v>
       </c>
       <c r="L3" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -545,7 +545,7 @@
         <v>Passed</v>
       </c>
       <c r="K4">
-        <v>389</v>
+        <v>293</v>
       </c>
       <c r="L4" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -583,7 +583,7 @@
         <v>Passed</v>
       </c>
       <c r="K5">
-        <v>301</v>
+        <v>368</v>
       </c>
       <c r="L5" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -621,7 +621,7 @@
         <v>Passed</v>
       </c>
       <c r="K6">
-        <v>268</v>
+        <v>286</v>
       </c>
       <c r="L6" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -659,7 +659,7 @@
         <v>Passed</v>
       </c>
       <c r="K7">
-        <v>180</v>
+        <v>293</v>
       </c>
       <c r="L7" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -697,7 +697,7 @@
         <v>Passed</v>
       </c>
       <c r="K8">
-        <v>279</v>
+        <v>372</v>
       </c>
       <c r="L8" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -735,7 +735,7 @@
         <v>Passed</v>
       </c>
       <c r="K9">
-        <v>385</v>
+        <v>367</v>
       </c>
       <c r="L9" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -773,7 +773,7 @@
         <v>Passed</v>
       </c>
       <c r="K10">
-        <v>196</v>
+        <v>292</v>
       </c>
       <c r="L10" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -811,7 +811,7 @@
         <v>Passed</v>
       </c>
       <c r="K11">
-        <v>219</v>
+        <v>258</v>
       </c>
       <c r="L11" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -849,7 +849,7 @@
         <v>Passed</v>
       </c>
       <c r="K12">
-        <v>151</v>
+        <v>283</v>
       </c>
       <c r="L12" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -887,7 +887,7 @@
         <v>Passed</v>
       </c>
       <c r="K13">
-        <v>277</v>
+        <v>261</v>
       </c>
       <c r="L13" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -925,7 +925,7 @@
         <v>Passed</v>
       </c>
       <c r="K14">
-        <v>189</v>
+        <v>289</v>
       </c>
       <c r="L14" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -963,7 +963,7 @@
         <v>Passed</v>
       </c>
       <c r="K15">
-        <v>275</v>
+        <v>253</v>
       </c>
       <c r="L15" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1001,7 +1001,7 @@
         <v>Passed</v>
       </c>
       <c r="K16">
-        <v>179</v>
+        <v>281</v>
       </c>
       <c r="L16" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1039,7 +1039,7 @@
         <v>Passed</v>
       </c>
       <c r="K17">
-        <v>168</v>
+        <v>240</v>
       </c>
       <c r="L17" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1077,7 +1077,7 @@
         <v>Passed</v>
       </c>
       <c r="K18">
-        <v>338</v>
+        <v>320</v>
       </c>
       <c r="L18" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1115,7 +1115,7 @@
         <v>Passed</v>
       </c>
       <c r="K19">
-        <v>247</v>
+        <v>191</v>
       </c>
       <c r="L19" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1153,7 +1153,7 @@
         <v>Passed</v>
       </c>
       <c r="K20">
-        <v>252</v>
+        <v>264</v>
       </c>
       <c r="L20" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1191,7 +1191,7 @@
         <v>Passed</v>
       </c>
       <c r="K21">
-        <v>396</v>
+        <v>246</v>
       </c>
       <c r="L21" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1229,7 +1229,7 @@
         <v>Passed</v>
       </c>
       <c r="K22">
-        <v>253</v>
+        <v>178</v>
       </c>
       <c r="L22" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1267,7 +1267,7 @@
         <v>Passed</v>
       </c>
       <c r="K23">
-        <v>187</v>
+        <v>168</v>
       </c>
       <c r="L23" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1305,7 +1305,7 @@
         <v>Passed</v>
       </c>
       <c r="K24">
-        <v>374</v>
+        <v>159</v>
       </c>
       <c r="L24" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1343,7 +1343,7 @@
         <v>Passed</v>
       </c>
       <c r="K25">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="L25" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1381,7 +1381,7 @@
         <v>Passed</v>
       </c>
       <c r="K26">
-        <v>274</v>
+        <v>325</v>
       </c>
       <c r="L26" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1419,7 +1419,7 @@
         <v>Passed</v>
       </c>
       <c r="K27">
-        <v>329</v>
+        <v>220</v>
       </c>
       <c r="L27" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1457,7 +1457,7 @@
         <v>Passed</v>
       </c>
       <c r="K28">
-        <v>153</v>
+        <v>308</v>
       </c>
       <c r="L28" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1495,7 +1495,7 @@
         <v>Passed</v>
       </c>
       <c r="K29">
-        <v>321</v>
+        <v>204</v>
       </c>
       <c r="L29" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1533,7 +1533,7 @@
         <v>Passed</v>
       </c>
       <c r="K30">
-        <v>399</v>
+        <v>284</v>
       </c>
       <c r="L30" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1571,7 +1571,7 @@
         <v>Passed</v>
       </c>
       <c r="K31">
-        <v>314</v>
+        <v>190</v>
       </c>
       <c r="L31" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1609,7 +1609,7 @@
         <v>Passed</v>
       </c>
       <c r="K32">
-        <v>220</v>
+        <v>199</v>
       </c>
       <c r="L32" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1647,7 +1647,7 @@
         <v>Passed</v>
       </c>
       <c r="K33">
-        <v>179</v>
+        <v>226</v>
       </c>
       <c r="L33" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1685,7 +1685,7 @@
         <v>Passed</v>
       </c>
       <c r="K34">
-        <v>236</v>
+        <v>155</v>
       </c>
       <c r="L34" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1723,7 +1723,7 @@
         <v>Passed</v>
       </c>
       <c r="K35">
-        <v>386</v>
+        <v>293</v>
       </c>
       <c r="L35" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1761,7 +1761,7 @@
         <v>Passed</v>
       </c>
       <c r="K36">
-        <v>349</v>
+        <v>359</v>
       </c>
       <c r="L36" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1799,7 +1799,7 @@
         <v>Passed</v>
       </c>
       <c r="K37">
-        <v>379</v>
+        <v>174</v>
       </c>
       <c r="L37" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1837,7 +1837,7 @@
         <v>Passed</v>
       </c>
       <c r="K38">
-        <v>328</v>
+        <v>361</v>
       </c>
       <c r="L38" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1875,7 +1875,7 @@
         <v>Passed</v>
       </c>
       <c r="K39">
-        <v>301</v>
+        <v>179</v>
       </c>
       <c r="L39" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1913,7 +1913,7 @@
         <v>Passed</v>
       </c>
       <c r="K40">
-        <v>347</v>
+        <v>370</v>
       </c>
       <c r="L40" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1951,7 +1951,7 @@
         <v>Passed</v>
       </c>
       <c r="K41">
-        <v>183</v>
+        <v>210</v>
       </c>
       <c r="L41" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1989,7 +1989,7 @@
         <v>Passed</v>
       </c>
       <c r="K42">
-        <v>379</v>
+        <v>213</v>
       </c>
       <c r="L42" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2027,7 +2027,7 @@
         <v>Passed</v>
       </c>
       <c r="K43">
-        <v>172</v>
+        <v>269</v>
       </c>
       <c r="L43" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2065,7 +2065,7 @@
         <v>Passed</v>
       </c>
       <c r="K44">
-        <v>263</v>
+        <v>362</v>
       </c>
       <c r="L44" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2103,7 +2103,7 @@
         <v>Passed</v>
       </c>
       <c r="K45">
-        <v>226</v>
+        <v>359</v>
       </c>
       <c r="L45" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2141,7 +2141,7 @@
         <v>Passed</v>
       </c>
       <c r="K46">
-        <v>170</v>
+        <v>308</v>
       </c>
       <c r="L46" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2179,7 +2179,7 @@
         <v>Passed</v>
       </c>
       <c r="K47">
-        <v>326</v>
+        <v>335</v>
       </c>
       <c r="L47" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2217,7 +2217,7 @@
         <v>Passed</v>
       </c>
       <c r="K48">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="L48" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2255,7 +2255,7 @@
         <v>Passed</v>
       </c>
       <c r="K49">
-        <v>295</v>
+        <v>322</v>
       </c>
       <c r="L49" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2293,7 +2293,7 @@
         <v>Passed</v>
       </c>
       <c r="K50">
-        <v>371</v>
+        <v>207</v>
       </c>
       <c r="L50" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2331,7 +2331,7 @@
         <v>Passed</v>
       </c>
       <c r="K51">
-        <v>346</v>
+        <v>276</v>
       </c>
       <c r="L51" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2369,7 +2369,7 @@
         <v>Passed</v>
       </c>
       <c r="K52">
-        <v>357</v>
+        <v>394</v>
       </c>
       <c r="L52" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2407,7 +2407,7 @@
         <v>Passed</v>
       </c>
       <c r="K53">
-        <v>385</v>
+        <v>247</v>
       </c>
       <c r="L53" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2445,7 +2445,7 @@
         <v>Passed</v>
       </c>
       <c r="K54">
-        <v>348</v>
+        <v>279</v>
       </c>
       <c r="L54" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2483,7 +2483,7 @@
         <v>Passed</v>
       </c>
       <c r="K55">
-        <v>341</v>
+        <v>192</v>
       </c>
       <c r="L55" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2521,7 +2521,7 @@
         <v>Passed</v>
       </c>
       <c r="K56">
-        <v>270</v>
+        <v>306</v>
       </c>
       <c r="L56" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2559,7 +2559,7 @@
         <v>Passed</v>
       </c>
       <c r="K57">
-        <v>211</v>
+        <v>362</v>
       </c>
       <c r="L57" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2597,7 +2597,7 @@
         <v>Passed</v>
       </c>
       <c r="K58">
-        <v>381</v>
+        <v>288</v>
       </c>
       <c r="L58" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2635,7 +2635,7 @@
         <v>Passed</v>
       </c>
       <c r="K59">
-        <v>263</v>
+        <v>366</v>
       </c>
       <c r="L59" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2673,7 +2673,7 @@
         <v>Passed</v>
       </c>
       <c r="K60">
-        <v>332</v>
+        <v>384</v>
       </c>
       <c r="L60" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2711,7 +2711,7 @@
         <v>Passed</v>
       </c>
       <c r="K61">
-        <v>168</v>
+        <v>337</v>
       </c>
       <c r="L61" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2749,7 +2749,7 @@
         <v>Passed</v>
       </c>
       <c r="K62">
-        <v>219</v>
+        <v>240</v>
       </c>
       <c r="L62" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2787,7 +2787,7 @@
         <v>Passed</v>
       </c>
       <c r="K63">
-        <v>269</v>
+        <v>308</v>
       </c>
       <c r="L63" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2825,7 +2825,7 @@
         <v>Passed</v>
       </c>
       <c r="K64">
-        <v>171</v>
+        <v>280</v>
       </c>
       <c r="L64" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2863,7 +2863,7 @@
         <v>Passed</v>
       </c>
       <c r="K65">
-        <v>386</v>
+        <v>155</v>
       </c>
       <c r="L65" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2901,7 +2901,7 @@
         <v>Passed</v>
       </c>
       <c r="K66">
-        <v>377</v>
+        <v>269</v>
       </c>
       <c r="L66" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2939,7 +2939,7 @@
         <v>Passed</v>
       </c>
       <c r="K67">
-        <v>253</v>
+        <v>210</v>
       </c>
       <c r="L67" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2977,7 +2977,7 @@
         <v>Passed</v>
       </c>
       <c r="K68">
-        <v>170</v>
+        <v>255</v>
       </c>
       <c r="L68" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3015,7 +3015,7 @@
         <v>Passed</v>
       </c>
       <c r="K69">
-        <v>301</v>
+        <v>165</v>
       </c>
       <c r="L69" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3053,7 +3053,7 @@
         <v>Passed</v>
       </c>
       <c r="K70">
-        <v>307</v>
+        <v>313</v>
       </c>
       <c r="L70" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3091,7 +3091,7 @@
         <v>Passed</v>
       </c>
       <c r="K71">
-        <v>320</v>
+        <v>304</v>
       </c>
       <c r="L71" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3129,7 +3129,7 @@
         <v>Passed</v>
       </c>
       <c r="K72">
-        <v>202</v>
+        <v>154</v>
       </c>
       <c r="L72" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3167,7 +3167,7 @@
         <v>Passed</v>
       </c>
       <c r="K73">
-        <v>337</v>
+        <v>320</v>
       </c>
       <c r="L73" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3205,7 +3205,7 @@
         <v>Passed</v>
       </c>
       <c r="K74">
-        <v>294</v>
+        <v>189</v>
       </c>
       <c r="L74" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3243,7 +3243,7 @@
         <v>Passed</v>
       </c>
       <c r="K75">
-        <v>212</v>
+        <v>294</v>
       </c>
       <c r="L75" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3281,7 +3281,7 @@
         <v>Passed</v>
       </c>
       <c r="K76">
-        <v>343</v>
+        <v>258</v>
       </c>
       <c r="L76" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3319,7 +3319,7 @@
         <v>Passed</v>
       </c>
       <c r="K77">
-        <v>364</v>
+        <v>378</v>
       </c>
       <c r="L77" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3357,7 +3357,7 @@
         <v>Passed</v>
       </c>
       <c r="K78">
-        <v>330</v>
+        <v>175</v>
       </c>
       <c r="L78" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3395,7 +3395,7 @@
         <v>Passed</v>
       </c>
       <c r="K79">
-        <v>274</v>
+        <v>360</v>
       </c>
       <c r="L79" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3433,7 +3433,7 @@
         <v>Passed</v>
       </c>
       <c r="K80">
-        <v>248</v>
+        <v>235</v>
       </c>
       <c r="L80" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3471,7 +3471,7 @@
         <v>Passed</v>
       </c>
       <c r="K81">
-        <v>345</v>
+        <v>198</v>
       </c>
       <c r="L81" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3509,7 +3509,7 @@
         <v>Passed</v>
       </c>
       <c r="K82">
-        <v>242</v>
+        <v>270</v>
       </c>
       <c r="L82" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3547,7 +3547,7 @@
         <v>Passed</v>
       </c>
       <c r="K83">
-        <v>257</v>
+        <v>346</v>
       </c>
       <c r="L83" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3585,7 +3585,7 @@
         <v>Passed</v>
       </c>
       <c r="K84">
-        <v>388</v>
+        <v>354</v>
       </c>
       <c r="L84" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3623,7 +3623,7 @@
         <v>Passed</v>
       </c>
       <c r="K85">
-        <v>251</v>
+        <v>280</v>
       </c>
       <c r="L85" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3661,7 +3661,7 @@
         <v>Passed</v>
       </c>
       <c r="K86">
-        <v>291</v>
+        <v>229</v>
       </c>
       <c r="L86" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3699,7 +3699,7 @@
         <v>Passed</v>
       </c>
       <c r="K87">
-        <v>240</v>
+        <v>348</v>
       </c>
       <c r="L87" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3737,7 +3737,7 @@
         <v>Passed</v>
       </c>
       <c r="K88">
-        <v>295</v>
+        <v>332</v>
       </c>
       <c r="L88" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3775,7 +3775,7 @@
         <v>Passed</v>
       </c>
       <c r="K89">
-        <v>327</v>
+        <v>207</v>
       </c>
       <c r="L89" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3813,7 +3813,7 @@
         <v>Passed</v>
       </c>
       <c r="K90">
-        <v>282</v>
+        <v>195</v>
       </c>
       <c r="L90" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3851,7 +3851,7 @@
         <v>Passed</v>
       </c>
       <c r="K91">
-        <v>392</v>
+        <v>237</v>
       </c>
       <c r="L91" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3889,7 +3889,7 @@
         <v>Passed</v>
       </c>
       <c r="K92">
-        <v>243</v>
+        <v>399</v>
       </c>
       <c r="L92" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3927,7 +3927,7 @@
         <v>Passed</v>
       </c>
       <c r="K93">
-        <v>345</v>
+        <v>287</v>
       </c>
       <c r="L93" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3965,7 +3965,7 @@
         <v>Passed</v>
       </c>
       <c r="K94">
-        <v>168</v>
+        <v>195</v>
       </c>
       <c r="L94" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4003,7 +4003,7 @@
         <v>Passed</v>
       </c>
       <c r="K95">
-        <v>167</v>
+        <v>333</v>
       </c>
       <c r="L95" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4041,7 +4041,7 @@
         <v>Passed</v>
       </c>
       <c r="K96">
-        <v>389</v>
+        <v>307</v>
       </c>
       <c r="L96" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4079,7 +4079,7 @@
         <v>Passed</v>
       </c>
       <c r="K97">
-        <v>262</v>
+        <v>388</v>
       </c>
       <c r="L97" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4117,7 +4117,7 @@
         <v>Passed</v>
       </c>
       <c r="K98">
-        <v>378</v>
+        <v>221</v>
       </c>
       <c r="L98" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4155,7 +4155,7 @@
         <v>Passed</v>
       </c>
       <c r="K99">
-        <v>188</v>
+        <v>195</v>
       </c>
       <c r="L99" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4193,7 +4193,7 @@
         <v>Passed</v>
       </c>
       <c r="K100">
-        <v>274</v>
+        <v>388</v>
       </c>
       <c r="L100" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4231,7 +4231,7 @@
         <v>Passed</v>
       </c>
       <c r="K101">
-        <v>392</v>
+        <v>251</v>
       </c>
       <c r="L101" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4269,7 +4269,7 @@
         <v>Passed</v>
       </c>
       <c r="K102">
-        <v>298</v>
+        <v>393</v>
       </c>
       <c r="L102" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4307,7 +4307,7 @@
         <v>Passed</v>
       </c>
       <c r="K103">
-        <v>195</v>
+        <v>241</v>
       </c>
       <c r="L103" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4345,7 +4345,7 @@
         <v>Passed</v>
       </c>
       <c r="K104">
-        <v>397</v>
+        <v>203</v>
       </c>
       <c r="L104" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4383,7 +4383,7 @@
         <v>Passed</v>
       </c>
       <c r="K105">
-        <v>156</v>
+        <v>326</v>
       </c>
       <c r="L105" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4421,7 +4421,7 @@
         <v>Passed</v>
       </c>
       <c r="K106">
-        <v>161</v>
+        <v>258</v>
       </c>
       <c r="L106" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4459,7 +4459,7 @@
         <v>Passed</v>
       </c>
       <c r="K107">
-        <v>396</v>
+        <v>227</v>
       </c>
       <c r="L107" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4497,7 +4497,7 @@
         <v>Passed</v>
       </c>
       <c r="K108">
-        <v>346</v>
+        <v>205</v>
       </c>
       <c r="L108" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4535,7 +4535,7 @@
         <v>Passed</v>
       </c>
       <c r="K109">
-        <v>294</v>
+        <v>231</v>
       </c>
       <c r="L109" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4573,7 +4573,7 @@
         <v>Passed</v>
       </c>
       <c r="K110">
-        <v>371</v>
+        <v>251</v>
       </c>
       <c r="L110" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4611,7 +4611,7 @@
         <v>Passed</v>
       </c>
       <c r="K111">
-        <v>367</v>
+        <v>338</v>
       </c>
       <c r="L111" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4649,7 +4649,7 @@
         <v>Passed</v>
       </c>
       <c r="K112">
-        <v>223</v>
+        <v>160</v>
       </c>
       <c r="L112" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4687,7 +4687,7 @@
         <v>Passed</v>
       </c>
       <c r="K113">
-        <v>286</v>
+        <v>340</v>
       </c>
       <c r="L113" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4725,7 +4725,7 @@
         <v>Passed</v>
       </c>
       <c r="K114">
-        <v>155</v>
+        <v>284</v>
       </c>
       <c r="L114" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4763,7 +4763,7 @@
         <v>Passed</v>
       </c>
       <c r="K115">
-        <v>229</v>
+        <v>176</v>
       </c>
       <c r="L115" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4801,7 +4801,7 @@
         <v>Passed</v>
       </c>
       <c r="K116">
-        <v>157</v>
+        <v>389</v>
       </c>
       <c r="L116" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4839,7 +4839,7 @@
         <v>Passed</v>
       </c>
       <c r="K117">
-        <v>360</v>
+        <v>171</v>
       </c>
       <c r="L117" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4877,7 +4877,7 @@
         <v>Passed</v>
       </c>
       <c r="K118">
-        <v>347</v>
+        <v>199</v>
       </c>
       <c r="L118" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4915,7 +4915,7 @@
         <v>Passed</v>
       </c>
       <c r="K119">
-        <v>277</v>
+        <v>369</v>
       </c>
       <c r="L119" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4953,7 +4953,7 @@
         <v>Passed</v>
       </c>
       <c r="K120">
-        <v>163</v>
+        <v>367</v>
       </c>
       <c r="L120" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4991,7 +4991,7 @@
         <v>Passed</v>
       </c>
       <c r="K121">
-        <v>348</v>
+        <v>248</v>
       </c>
       <c r="L121" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5029,7 +5029,7 @@
         <v>Passed</v>
       </c>
       <c r="K122">
-        <v>330</v>
+        <v>322</v>
       </c>
       <c r="L122" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5067,7 +5067,7 @@
         <v>Passed</v>
       </c>
       <c r="K123">
-        <v>219</v>
+        <v>261</v>
       </c>
       <c r="L123" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5105,7 +5105,7 @@
         <v>Passed</v>
       </c>
       <c r="K124">
-        <v>280</v>
+        <v>191</v>
       </c>
       <c r="L124" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5143,7 +5143,7 @@
         <v>Passed</v>
       </c>
       <c r="K125">
-        <v>180</v>
+        <v>151</v>
       </c>
       <c r="L125" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5181,7 +5181,7 @@
         <v>Passed</v>
       </c>
       <c r="K126">
-        <v>228</v>
+        <v>303</v>
       </c>
       <c r="L126" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5219,7 +5219,7 @@
         <v>Passed</v>
       </c>
       <c r="K127">
-        <v>158</v>
+        <v>367</v>
       </c>
       <c r="L127" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5257,7 +5257,7 @@
         <v>Passed</v>
       </c>
       <c r="K128">
-        <v>304</v>
+        <v>348</v>
       </c>
       <c r="L128" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5295,7 +5295,7 @@
         <v>Passed</v>
       </c>
       <c r="K129">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="L129" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5333,7 +5333,7 @@
         <v>Passed</v>
       </c>
       <c r="K130">
-        <v>366</v>
+        <v>377</v>
       </c>
       <c r="L130" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5371,7 +5371,7 @@
         <v>Passed</v>
       </c>
       <c r="K131">
-        <v>371</v>
+        <v>177</v>
       </c>
       <c r="L131" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5409,7 +5409,7 @@
         <v>Passed</v>
       </c>
       <c r="K132">
-        <v>366</v>
+        <v>274</v>
       </c>
       <c r="L132" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5447,7 +5447,7 @@
         <v>Passed</v>
       </c>
       <c r="K133">
-        <v>382</v>
+        <v>260</v>
       </c>
       <c r="L133" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5485,7 +5485,7 @@
         <v>Passed</v>
       </c>
       <c r="K134">
-        <v>371</v>
+        <v>304</v>
       </c>
       <c r="L134" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5523,7 +5523,7 @@
         <v>Passed</v>
       </c>
       <c r="K135">
-        <v>219</v>
+        <v>206</v>
       </c>
       <c r="L135" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5561,7 +5561,7 @@
         <v>Passed</v>
       </c>
       <c r="K136">
-        <v>387</v>
+        <v>251</v>
       </c>
       <c r="L136" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5599,7 +5599,7 @@
         <v>Passed</v>
       </c>
       <c r="K137">
-        <v>299</v>
+        <v>319</v>
       </c>
       <c r="L137" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5637,7 +5637,7 @@
         <v>Passed</v>
       </c>
       <c r="K138">
-        <v>185</v>
+        <v>276</v>
       </c>
       <c r="L138" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5675,7 +5675,7 @@
         <v>Passed</v>
       </c>
       <c r="K139">
-        <v>312</v>
+        <v>363</v>
       </c>
       <c r="L139" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5713,7 +5713,7 @@
         <v>Passed</v>
       </c>
       <c r="K140">
-        <v>287</v>
+        <v>183</v>
       </c>
       <c r="L140" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5751,7 +5751,7 @@
         <v>Passed</v>
       </c>
       <c r="K141">
-        <v>245</v>
+        <v>258</v>
       </c>
       <c r="L141" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5789,7 +5789,7 @@
         <v>Passed</v>
       </c>
       <c r="K142">
-        <v>191</v>
+        <v>171</v>
       </c>
       <c r="L142" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5827,7 +5827,7 @@
         <v>Passed</v>
       </c>
       <c r="K143">
-        <v>300</v>
+        <v>397</v>
       </c>
       <c r="L143" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5865,7 +5865,7 @@
         <v>Passed</v>
       </c>
       <c r="K144">
-        <v>201</v>
+        <v>271</v>
       </c>
       <c r="L144" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5903,7 +5903,7 @@
         <v>Passed</v>
       </c>
       <c r="K145">
-        <v>181</v>
+        <v>342</v>
       </c>
       <c r="L145" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5941,7 +5941,7 @@
         <v>Passed</v>
       </c>
       <c r="K146">
-        <v>237</v>
+        <v>390</v>
       </c>
       <c r="L146" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5979,7 +5979,7 @@
         <v>Passed</v>
       </c>
       <c r="K147">
-        <v>261</v>
+        <v>378</v>
       </c>
       <c r="L147" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6017,7 +6017,7 @@
         <v>Passed</v>
       </c>
       <c r="K148">
-        <v>312</v>
+        <v>288</v>
       </c>
       <c r="L148" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6055,7 +6055,7 @@
         <v>Passed</v>
       </c>
       <c r="K149">
-        <v>320</v>
+        <v>199</v>
       </c>
       <c r="L149" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6093,7 +6093,7 @@
         <v>Passed</v>
       </c>
       <c r="K150">
-        <v>312</v>
+        <v>363</v>
       </c>
       <c r="L150" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6131,7 +6131,7 @@
         <v>Passed</v>
       </c>
       <c r="K151">
-        <v>305</v>
+        <v>366</v>
       </c>
       <c r="L151" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6169,7 +6169,7 @@
         <v>Passed</v>
       </c>
       <c r="K152">
-        <v>325</v>
+        <v>180</v>
       </c>
       <c r="L152" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6207,7 +6207,7 @@
         <v>Passed</v>
       </c>
       <c r="K153">
-        <v>221</v>
+        <v>240</v>
       </c>
       <c r="L153" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6245,7 +6245,7 @@
         <v>Passed</v>
       </c>
       <c r="K154">
-        <v>277</v>
+        <v>262</v>
       </c>
       <c r="L154" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6283,7 +6283,7 @@
         <v>Passed</v>
       </c>
       <c r="K155">
-        <v>375</v>
+        <v>253</v>
       </c>
       <c r="L155" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6321,7 +6321,7 @@
         <v>Passed</v>
       </c>
       <c r="K156">
-        <v>314</v>
+        <v>208</v>
       </c>
       <c r="L156" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6359,7 +6359,7 @@
         <v>Passed</v>
       </c>
       <c r="K157">
-        <v>306</v>
+        <v>397</v>
       </c>
       <c r="L157" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6397,7 +6397,7 @@
         <v>Passed</v>
       </c>
       <c r="K158">
-        <v>185</v>
+        <v>336</v>
       </c>
       <c r="L158" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6435,7 +6435,7 @@
         <v>Passed</v>
       </c>
       <c r="K159">
-        <v>194</v>
+        <v>399</v>
       </c>
       <c r="L159" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6473,7 +6473,7 @@
         <v>Passed</v>
       </c>
       <c r="K160">
-        <v>291</v>
+        <v>300</v>
       </c>
       <c r="L160" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6511,7 +6511,7 @@
         <v>Passed</v>
       </c>
       <c r="K161">
-        <v>341</v>
+        <v>251</v>
       </c>
       <c r="L161" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6549,7 +6549,7 @@
         <v>Passed</v>
       </c>
       <c r="K162">
-        <v>193</v>
+        <v>324</v>
       </c>
       <c r="L162" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6587,7 +6587,7 @@
         <v>Passed</v>
       </c>
       <c r="K163">
-        <v>284</v>
+        <v>214</v>
       </c>
       <c r="L163" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6625,7 +6625,7 @@
         <v>Passed</v>
       </c>
       <c r="K164">
-        <v>241</v>
+        <v>268</v>
       </c>
       <c r="L164" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6663,7 +6663,7 @@
         <v>Passed</v>
       </c>
       <c r="K165">
-        <v>398</v>
+        <v>361</v>
       </c>
       <c r="L165" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6701,7 +6701,7 @@
         <v>Passed</v>
       </c>
       <c r="K166">
-        <v>386</v>
+        <v>226</v>
       </c>
       <c r="L166" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6739,7 +6739,7 @@
         <v>Passed</v>
       </c>
       <c r="K167">
-        <v>233</v>
+        <v>297</v>
       </c>
       <c r="L167" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6777,7 +6777,7 @@
         <v>Passed</v>
       </c>
       <c r="K168">
-        <v>317</v>
+        <v>351</v>
       </c>
       <c r="L168" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6815,7 +6815,7 @@
         <v>Passed</v>
       </c>
       <c r="K169">
-        <v>177</v>
+        <v>252</v>
       </c>
       <c r="L169" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6853,7 +6853,7 @@
         <v>Passed</v>
       </c>
       <c r="K170">
-        <v>357</v>
+        <v>394</v>
       </c>
       <c r="L170" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6891,7 +6891,7 @@
         <v>Passed</v>
       </c>
       <c r="K171">
-        <v>304</v>
+        <v>200</v>
       </c>
       <c r="L171" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6929,7 +6929,7 @@
         <v>Passed</v>
       </c>
       <c r="K172">
-        <v>344</v>
+        <v>217</v>
       </c>
       <c r="L172" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6967,7 +6967,7 @@
         <v>Passed</v>
       </c>
       <c r="K173">
-        <v>157</v>
+        <v>374</v>
       </c>
       <c r="L173" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7005,7 +7005,7 @@
         <v>Passed</v>
       </c>
       <c r="K174">
-        <v>382</v>
+        <v>378</v>
       </c>
       <c r="L174" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7043,7 +7043,7 @@
         <v>Passed</v>
       </c>
       <c r="K175">
-        <v>248</v>
+        <v>371</v>
       </c>
       <c r="L175" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7081,7 +7081,7 @@
         <v>Passed</v>
       </c>
       <c r="K176">
-        <v>363</v>
+        <v>301</v>
       </c>
       <c r="L176" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7119,7 +7119,7 @@
         <v>Passed</v>
       </c>
       <c r="K177">
-        <v>201</v>
+        <v>384</v>
       </c>
       <c r="L177" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7157,7 +7157,7 @@
         <v>Passed</v>
       </c>
       <c r="K178">
-        <v>256</v>
+        <v>176</v>
       </c>
       <c r="L178" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7195,7 +7195,7 @@
         <v>Passed</v>
       </c>
       <c r="K179">
-        <v>350</v>
+        <v>363</v>
       </c>
       <c r="L179" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7233,7 +7233,7 @@
         <v>Passed</v>
       </c>
       <c r="K180">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="L180" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7271,7 +7271,7 @@
         <v>Passed</v>
       </c>
       <c r="K181">
-        <v>386</v>
+        <v>250</v>
       </c>
       <c r="L181" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7309,7 +7309,7 @@
         <v>Passed</v>
       </c>
       <c r="K182">
-        <v>375</v>
+        <v>280</v>
       </c>
       <c r="L182" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7347,7 +7347,7 @@
         <v>Passed</v>
       </c>
       <c r="K183">
-        <v>275</v>
+        <v>197</v>
       </c>
       <c r="L183" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7385,7 +7385,7 @@
         <v>Passed</v>
       </c>
       <c r="K184">
-        <v>263</v>
+        <v>325</v>
       </c>
       <c r="L184" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7423,7 +7423,7 @@
         <v>Passed</v>
       </c>
       <c r="K185">
-        <v>167</v>
+        <v>292</v>
       </c>
       <c r="L185" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7461,7 +7461,7 @@
         <v>Passed</v>
       </c>
       <c r="K186">
-        <v>311</v>
+        <v>394</v>
       </c>
       <c r="L186" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7499,7 +7499,7 @@
         <v>Passed</v>
       </c>
       <c r="K187">
-        <v>243</v>
+        <v>302</v>
       </c>
       <c r="L187" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7537,7 +7537,7 @@
         <v>Passed</v>
       </c>
       <c r="K188">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="L188" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7575,7 +7575,7 @@
         <v>Passed</v>
       </c>
       <c r="K189">
-        <v>237</v>
+        <v>302</v>
       </c>
       <c r="L189" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7613,7 +7613,7 @@
         <v>Passed</v>
       </c>
       <c r="K190">
-        <v>249</v>
+        <v>219</v>
       </c>
       <c r="L190" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7651,7 +7651,7 @@
         <v>Passed</v>
       </c>
       <c r="K191">
-        <v>268</v>
+        <v>392</v>
       </c>
       <c r="L191" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7689,7 +7689,7 @@
         <v>Passed</v>
       </c>
       <c r="K192">
-        <v>344</v>
+        <v>307</v>
       </c>
       <c r="L192" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7727,7 +7727,7 @@
         <v>Passed</v>
       </c>
       <c r="K193">
-        <v>239</v>
+        <v>388</v>
       </c>
       <c r="L193" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7765,7 +7765,7 @@
         <v>Passed</v>
       </c>
       <c r="K194">
-        <v>295</v>
+        <v>316</v>
       </c>
       <c r="L194" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7803,7 +7803,7 @@
         <v>Passed</v>
       </c>
       <c r="K195">
-        <v>287</v>
+        <v>256</v>
       </c>
       <c r="L195" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7841,7 +7841,7 @@
         <v>Passed</v>
       </c>
       <c r="K196">
-        <v>365</v>
+        <v>339</v>
       </c>
       <c r="L196" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7879,7 +7879,7 @@
         <v>Passed</v>
       </c>
       <c r="K197">
-        <v>153</v>
+        <v>334</v>
       </c>
       <c r="L197" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7917,7 +7917,7 @@
         <v>Passed</v>
       </c>
       <c r="K198">
-        <v>158</v>
+        <v>288</v>
       </c>
       <c r="L198" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7955,7 +7955,7 @@
         <v>Passed</v>
       </c>
       <c r="K199">
-        <v>242</v>
+        <v>386</v>
       </c>
       <c r="L199" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7993,7 +7993,7 @@
         <v>Passed</v>
       </c>
       <c r="K200">
-        <v>340</v>
+        <v>353</v>
       </c>
       <c r="L200" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8031,7 +8031,7 @@
         <v>Passed</v>
       </c>
       <c r="K201">
-        <v>294</v>
+        <v>207</v>
       </c>
       <c r="L201" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8069,7 +8069,7 @@
         <v>Passed</v>
       </c>
       <c r="K202">
-        <v>151</v>
+        <v>331</v>
       </c>
       <c r="L202" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8107,7 +8107,7 @@
         <v>Passed</v>
       </c>
       <c r="K203">
-        <v>184</v>
+        <v>339</v>
       </c>
       <c r="L203" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8145,7 +8145,7 @@
         <v>Passed</v>
       </c>
       <c r="K204">
-        <v>358</v>
+        <v>171</v>
       </c>
       <c r="L204" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8183,7 +8183,7 @@
         <v>Passed</v>
       </c>
       <c r="K205">
-        <v>391</v>
+        <v>224</v>
       </c>
       <c r="L205" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8221,7 +8221,7 @@
         <v>Passed</v>
       </c>
       <c r="K206">
-        <v>176</v>
+        <v>227</v>
       </c>
       <c r="L206" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8259,7 +8259,7 @@
         <v>Passed</v>
       </c>
       <c r="K207">
-        <v>228</v>
+        <v>306</v>
       </c>
       <c r="L207" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8297,7 +8297,7 @@
         <v>Passed</v>
       </c>
       <c r="K208">
-        <v>354</v>
+        <v>304</v>
       </c>
       <c r="L208" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8335,7 +8335,7 @@
         <v>Passed</v>
       </c>
       <c r="K209">
-        <v>391</v>
+        <v>325</v>
       </c>
       <c r="L209" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8373,7 +8373,7 @@
         <v>Passed</v>
       </c>
       <c r="K210">
-        <v>168</v>
+        <v>150</v>
       </c>
       <c r="L210" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8411,7 +8411,7 @@
         <v>Passed</v>
       </c>
       <c r="K211">
-        <v>164</v>
+        <v>382</v>
       </c>
       <c r="L211" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8449,7 +8449,7 @@
         <v>Passed</v>
       </c>
       <c r="K212">
-        <v>245</v>
+        <v>174</v>
       </c>
       <c r="L212" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8487,7 +8487,7 @@
         <v>Passed</v>
       </c>
       <c r="K213">
-        <v>237</v>
+        <v>225</v>
       </c>
       <c r="L213" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8525,7 +8525,7 @@
         <v>Passed</v>
       </c>
       <c r="K214">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="L214" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8563,7 +8563,7 @@
         <v>Passed</v>
       </c>
       <c r="K215">
-        <v>342</v>
+        <v>358</v>
       </c>
       <c r="L215" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8601,7 +8601,7 @@
         <v>Passed</v>
       </c>
       <c r="K216">
-        <v>318</v>
+        <v>170</v>
       </c>
       <c r="L216" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8639,7 +8639,7 @@
         <v>Passed</v>
       </c>
       <c r="K217">
-        <v>201</v>
+        <v>239</v>
       </c>
       <c r="L217" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8677,7 +8677,7 @@
         <v>Passed</v>
       </c>
       <c r="K218">
-        <v>165</v>
+        <v>291</v>
       </c>
       <c r="L218" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8715,7 +8715,7 @@
         <v>Passed</v>
       </c>
       <c r="K219">
-        <v>322</v>
+        <v>187</v>
       </c>
       <c r="L219" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8753,7 +8753,7 @@
         <v>Passed</v>
       </c>
       <c r="K220">
-        <v>301</v>
+        <v>263</v>
       </c>
       <c r="L220" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8791,7 +8791,7 @@
         <v>Passed</v>
       </c>
       <c r="K221">
-        <v>262</v>
+        <v>356</v>
       </c>
       <c r="L221" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8829,7 +8829,7 @@
         <v>Passed</v>
       </c>
       <c r="K222">
-        <v>391</v>
+        <v>359</v>
       </c>
       <c r="L222" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8867,7 +8867,7 @@
         <v>Passed</v>
       </c>
       <c r="K223">
-        <v>258</v>
+        <v>275</v>
       </c>
       <c r="L223" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8905,7 +8905,7 @@
         <v>Passed</v>
       </c>
       <c r="K224">
-        <v>388</v>
+        <v>181</v>
       </c>
       <c r="L224" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8943,7 +8943,7 @@
         <v>Passed</v>
       </c>
       <c r="K225">
-        <v>347</v>
+        <v>183</v>
       </c>
       <c r="L225" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8981,7 +8981,7 @@
         <v>Passed</v>
       </c>
       <c r="K226">
-        <v>196</v>
+        <v>394</v>
       </c>
       <c r="L226" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9019,7 +9019,7 @@
         <v>Passed</v>
       </c>
       <c r="K227">
-        <v>340</v>
+        <v>284</v>
       </c>
       <c r="L227" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9057,7 +9057,7 @@
         <v>Passed</v>
       </c>
       <c r="K228">
-        <v>238</v>
+        <v>180</v>
       </c>
       <c r="L228" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9095,7 +9095,7 @@
         <v>Passed</v>
       </c>
       <c r="K229">
-        <v>373</v>
+        <v>288</v>
       </c>
       <c r="L229" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9133,7 +9133,7 @@
         <v>Passed</v>
       </c>
       <c r="K230">
-        <v>223</v>
+        <v>317</v>
       </c>
       <c r="L230" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9171,7 +9171,7 @@
         <v>Passed</v>
       </c>
       <c r="K231">
-        <v>371</v>
+        <v>331</v>
       </c>
       <c r="L231" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9209,7 +9209,7 @@
         <v>Passed</v>
       </c>
       <c r="K232">
-        <v>247</v>
+        <v>332</v>
       </c>
       <c r="L232" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9247,7 +9247,7 @@
         <v>Passed</v>
       </c>
       <c r="K233">
-        <v>215</v>
+        <v>198</v>
       </c>
       <c r="L233" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9285,7 +9285,7 @@
         <v>Passed</v>
       </c>
       <c r="K234">
-        <v>380</v>
+        <v>189</v>
       </c>
       <c r="L234" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9323,7 +9323,7 @@
         <v>Passed</v>
       </c>
       <c r="K235">
-        <v>287</v>
+        <v>170</v>
       </c>
       <c r="L235" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9399,7 +9399,7 @@
         <v>Passed</v>
       </c>
       <c r="K237">
-        <v>320</v>
+        <v>232</v>
       </c>
       <c r="L237" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9437,7 +9437,7 @@
         <v>Passed</v>
       </c>
       <c r="K238">
-        <v>310</v>
+        <v>337</v>
       </c>
       <c r="L238" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9475,7 +9475,7 @@
         <v>Passed</v>
       </c>
       <c r="K239">
-        <v>392</v>
+        <v>154</v>
       </c>
       <c r="L239" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9513,7 +9513,7 @@
         <v>Passed</v>
       </c>
       <c r="K240">
-        <v>395</v>
+        <v>360</v>
       </c>
       <c r="L240" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9551,7 +9551,7 @@
         <v>Passed</v>
       </c>
       <c r="K241">
-        <v>306</v>
+        <v>166</v>
       </c>
       <c r="L241" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9589,7 +9589,7 @@
         <v>Passed</v>
       </c>
       <c r="K242">
-        <v>342</v>
+        <v>328</v>
       </c>
       <c r="L242" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9627,7 +9627,7 @@
         <v>Passed</v>
       </c>
       <c r="K243">
-        <v>208</v>
+        <v>163</v>
       </c>
       <c r="L243" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9665,7 +9665,7 @@
         <v>Passed</v>
       </c>
       <c r="K244">
-        <v>393</v>
+        <v>246</v>
       </c>
       <c r="L244" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9703,7 +9703,7 @@
         <v>Passed</v>
       </c>
       <c r="K245">
-        <v>349</v>
+        <v>284</v>
       </c>
       <c r="L245" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9741,7 +9741,7 @@
         <v>Passed</v>
       </c>
       <c r="K246">
-        <v>343</v>
+        <v>310</v>
       </c>
       <c r="L246" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9779,7 +9779,7 @@
         <v>Passed</v>
       </c>
       <c r="K247">
-        <v>213</v>
+        <v>343</v>
       </c>
       <c r="L247" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9817,7 +9817,7 @@
         <v>Passed</v>
       </c>
       <c r="K248">
-        <v>359</v>
+        <v>227</v>
       </c>
       <c r="L248" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9855,7 +9855,7 @@
         <v>Passed</v>
       </c>
       <c r="K249">
-        <v>326</v>
+        <v>340</v>
       </c>
       <c r="L249" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9893,7 +9893,7 @@
         <v>Passed</v>
       </c>
       <c r="K250">
-        <v>297</v>
+        <v>209</v>
       </c>
       <c r="L250" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9931,7 +9931,7 @@
         <v>Passed</v>
       </c>
       <c r="K251">
-        <v>310</v>
+        <v>290</v>
       </c>
       <c r="L251" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9969,7 +9969,7 @@
         <v>Passed</v>
       </c>
       <c r="K252">
-        <v>253</v>
+        <v>215</v>
       </c>
       <c r="L252" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10007,7 +10007,7 @@
         <v>Passed</v>
       </c>
       <c r="K253">
-        <v>342</v>
+        <v>152</v>
       </c>
       <c r="L253" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10045,7 +10045,7 @@
         <v>Passed</v>
       </c>
       <c r="K254">
-        <v>334</v>
+        <v>155</v>
       </c>
       <c r="L254" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10083,7 +10083,7 @@
         <v>Passed</v>
       </c>
       <c r="K255">
-        <v>179</v>
+        <v>264</v>
       </c>
       <c r="L255" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10121,7 +10121,7 @@
         <v>Passed</v>
       </c>
       <c r="K256">
-        <v>310</v>
+        <v>344</v>
       </c>
       <c r="L256" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10159,7 +10159,7 @@
         <v>Passed</v>
       </c>
       <c r="K257">
-        <v>260</v>
+        <v>318</v>
       </c>
       <c r="L257" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10197,7 +10197,7 @@
         <v>Passed</v>
       </c>
       <c r="K258">
-        <v>227</v>
+        <v>179</v>
       </c>
       <c r="L258" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10235,7 +10235,7 @@
         <v>Passed</v>
       </c>
       <c r="K259">
-        <v>291</v>
+        <v>340</v>
       </c>
       <c r="L259" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10273,7 +10273,7 @@
         <v>Passed</v>
       </c>
       <c r="K260">
-        <v>299</v>
+        <v>347</v>
       </c>
       <c r="L260" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10311,7 +10311,7 @@
         <v>Passed</v>
       </c>
       <c r="K261">
-        <v>362</v>
+        <v>292</v>
       </c>
       <c r="L261" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10349,7 +10349,7 @@
         <v>Passed</v>
       </c>
       <c r="K262">
-        <v>243</v>
+        <v>290</v>
       </c>
       <c r="L262" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10387,7 +10387,7 @@
         <v>Passed</v>
       </c>
       <c r="K263">
-        <v>157</v>
+        <v>343</v>
       </c>
       <c r="L263" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10425,7 +10425,7 @@
         <v>Passed</v>
       </c>
       <c r="K264">
-        <v>370</v>
+        <v>246</v>
       </c>
       <c r="L264" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10463,7 +10463,7 @@
         <v>Passed</v>
       </c>
       <c r="K265">
-        <v>196</v>
+        <v>391</v>
       </c>
       <c r="L265" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10501,7 +10501,7 @@
         <v>Passed</v>
       </c>
       <c r="K266">
-        <v>378</v>
+        <v>357</v>
       </c>
       <c r="L266" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10539,7 +10539,7 @@
         <v>Passed</v>
       </c>
       <c r="K267">
-        <v>225</v>
+        <v>360</v>
       </c>
       <c r="L267" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10577,7 +10577,7 @@
         <v>Passed</v>
       </c>
       <c r="K268">
-        <v>379</v>
+        <v>376</v>
       </c>
       <c r="L268" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10615,7 +10615,7 @@
         <v>Passed</v>
       </c>
       <c r="K269">
-        <v>169</v>
+        <v>379</v>
       </c>
       <c r="L269" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10653,7 +10653,7 @@
         <v>Passed</v>
       </c>
       <c r="K270">
-        <v>223</v>
+        <v>160</v>
       </c>
       <c r="L270" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10691,7 +10691,7 @@
         <v>Passed</v>
       </c>
       <c r="K271">
-        <v>276</v>
+        <v>282</v>
       </c>
       <c r="L271" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10729,7 +10729,7 @@
         <v>Passed</v>
       </c>
       <c r="K272">
-        <v>269</v>
+        <v>380</v>
       </c>
       <c r="L272" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10767,7 +10767,7 @@
         <v>Passed</v>
       </c>
       <c r="K273">
-        <v>261</v>
+        <v>239</v>
       </c>
       <c r="L273" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10805,7 +10805,7 @@
         <v>Passed</v>
       </c>
       <c r="K274">
-        <v>233</v>
+        <v>245</v>
       </c>
       <c r="L274" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10843,7 +10843,7 @@
         <v>Passed</v>
       </c>
       <c r="K275">
-        <v>206</v>
+        <v>226</v>
       </c>
       <c r="L275" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10881,7 +10881,7 @@
         <v>Passed</v>
       </c>
       <c r="K276">
-        <v>323</v>
+        <v>344</v>
       </c>
       <c r="L276" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10919,7 +10919,7 @@
         <v>Passed</v>
       </c>
       <c r="K277">
-        <v>378</v>
+        <v>216</v>
       </c>
       <c r="L277" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10957,7 +10957,7 @@
         <v>Passed</v>
       </c>
       <c r="K278">
-        <v>160</v>
+        <v>343</v>
       </c>
       <c r="L278" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10995,7 +10995,7 @@
         <v>Passed</v>
       </c>
       <c r="K279">
-        <v>173</v>
+        <v>362</v>
       </c>
       <c r="L279" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11033,7 +11033,7 @@
         <v>Passed</v>
       </c>
       <c r="K280">
-        <v>263</v>
+        <v>340</v>
       </c>
       <c r="L280" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11071,7 +11071,7 @@
         <v>Passed</v>
       </c>
       <c r="K281">
-        <v>350</v>
+        <v>204</v>
       </c>
       <c r="L281" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11109,7 +11109,7 @@
         <v>Passed</v>
       </c>
       <c r="K282">
-        <v>290</v>
+        <v>383</v>
       </c>
       <c r="L282" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11147,7 +11147,7 @@
         <v>Passed</v>
       </c>
       <c r="K283">
-        <v>319</v>
+        <v>274</v>
       </c>
       <c r="L283" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11185,7 +11185,7 @@
         <v>Passed</v>
       </c>
       <c r="K284">
-        <v>158</v>
+        <v>184</v>
       </c>
       <c r="L284" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11223,7 +11223,7 @@
         <v>Passed</v>
       </c>
       <c r="K285">
-        <v>197</v>
+        <v>245</v>
       </c>
       <c r="L285" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11261,7 +11261,7 @@
         <v>Passed</v>
       </c>
       <c r="K286">
-        <v>175</v>
+        <v>297</v>
       </c>
       <c r="L286" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11299,7 +11299,7 @@
         <v>Passed</v>
       </c>
       <c r="K287">
-        <v>336</v>
+        <v>312</v>
       </c>
       <c r="L287" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11337,7 +11337,7 @@
         <v>Passed</v>
       </c>
       <c r="K288">
-        <v>270</v>
+        <v>231</v>
       </c>
       <c r="L288" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11375,7 +11375,7 @@
         <v>Passed</v>
       </c>
       <c r="K289">
-        <v>225</v>
+        <v>289</v>
       </c>
       <c r="L289" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11413,7 +11413,7 @@
         <v>Passed</v>
       </c>
       <c r="K290">
-        <v>234</v>
+        <v>257</v>
       </c>
       <c r="L290" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11451,7 +11451,7 @@
         <v>Passed</v>
       </c>
       <c r="K291">
-        <v>154</v>
+        <v>261</v>
       </c>
       <c r="L291" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11489,7 +11489,7 @@
         <v>Passed</v>
       </c>
       <c r="K292">
-        <v>262</v>
+        <v>288</v>
       </c>
       <c r="L292" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11527,7 +11527,7 @@
         <v>Passed</v>
       </c>
       <c r="K293">
-        <v>224</v>
+        <v>205</v>
       </c>
       <c r="L293" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11565,7 +11565,7 @@
         <v>Passed</v>
       </c>
       <c r="K294">
-        <v>246</v>
+        <v>308</v>
       </c>
       <c r="L294" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11603,7 +11603,7 @@
         <v>Passed</v>
       </c>
       <c r="K295">
-        <v>371</v>
+        <v>225</v>
       </c>
       <c r="L295" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11641,7 +11641,7 @@
         <v>Passed</v>
       </c>
       <c r="K296">
-        <v>333</v>
+        <v>199</v>
       </c>
       <c r="L296" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11679,7 +11679,7 @@
         <v>Passed</v>
       </c>
       <c r="K297">
-        <v>164</v>
+        <v>369</v>
       </c>
       <c r="L297" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11717,7 +11717,7 @@
         <v>Passed</v>
       </c>
       <c r="K298">
-        <v>227</v>
+        <v>179</v>
       </c>
       <c r="L298" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11755,7 +11755,7 @@
         <v>Passed</v>
       </c>
       <c r="K299">
-        <v>254</v>
+        <v>365</v>
       </c>
       <c r="L299" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11793,7 +11793,7 @@
         <v>Passed</v>
       </c>
       <c r="K300">
-        <v>162</v>
+        <v>379</v>
       </c>
       <c r="L300" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11831,7 +11831,7 @@
         <v>Passed</v>
       </c>
       <c r="K301">
-        <v>247</v>
+        <v>204</v>
       </c>
       <c r="L301" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>

</xml_diff>

<commit_message>
feat: upgrade event page to 1400px split desktop layout and real public URL music streaming
</commit_message>
<xml_diff>
--- a/EventSphere_Appium_Mobile_300_Report.xlsx
+++ b/EventSphere_Appium_Mobile_300_Report.xlsx
@@ -469,7 +469,7 @@
         <v>Passed</v>
       </c>
       <c r="K2">
-        <v>397</v>
+        <v>259</v>
       </c>
       <c r="L2" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -507,7 +507,7 @@
         <v>Passed</v>
       </c>
       <c r="K3">
-        <v>301</v>
+        <v>360</v>
       </c>
       <c r="L3" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -545,7 +545,7 @@
         <v>Passed</v>
       </c>
       <c r="K4">
-        <v>293</v>
+        <v>355</v>
       </c>
       <c r="L4" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -583,7 +583,7 @@
         <v>Passed</v>
       </c>
       <c r="K5">
-        <v>368</v>
+        <v>204</v>
       </c>
       <c r="L5" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -621,7 +621,7 @@
         <v>Passed</v>
       </c>
       <c r="K6">
-        <v>286</v>
+        <v>208</v>
       </c>
       <c r="L6" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -659,7 +659,7 @@
         <v>Passed</v>
       </c>
       <c r="K7">
-        <v>293</v>
+        <v>330</v>
       </c>
       <c r="L7" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -697,7 +697,7 @@
         <v>Passed</v>
       </c>
       <c r="K8">
-        <v>372</v>
+        <v>356</v>
       </c>
       <c r="L8" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -735,7 +735,7 @@
         <v>Passed</v>
       </c>
       <c r="K9">
-        <v>367</v>
+        <v>271</v>
       </c>
       <c r="L9" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -773,7 +773,7 @@
         <v>Passed</v>
       </c>
       <c r="K10">
-        <v>292</v>
+        <v>234</v>
       </c>
       <c r="L10" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -811,7 +811,7 @@
         <v>Passed</v>
       </c>
       <c r="K11">
-        <v>258</v>
+        <v>326</v>
       </c>
       <c r="L11" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -849,7 +849,7 @@
         <v>Passed</v>
       </c>
       <c r="K12">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="L12" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -887,7 +887,7 @@
         <v>Passed</v>
       </c>
       <c r="K13">
-        <v>261</v>
+        <v>280</v>
       </c>
       <c r="L13" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -925,7 +925,7 @@
         <v>Passed</v>
       </c>
       <c r="K14">
-        <v>289</v>
+        <v>253</v>
       </c>
       <c r="L14" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -963,7 +963,7 @@
         <v>Passed</v>
       </c>
       <c r="K15">
-        <v>253</v>
+        <v>168</v>
       </c>
       <c r="L15" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1001,7 +1001,7 @@
         <v>Passed</v>
       </c>
       <c r="K16">
-        <v>281</v>
+        <v>170</v>
       </c>
       <c r="L16" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1039,7 +1039,7 @@
         <v>Passed</v>
       </c>
       <c r="K17">
-        <v>240</v>
+        <v>199</v>
       </c>
       <c r="L17" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1077,7 +1077,7 @@
         <v>Passed</v>
       </c>
       <c r="K18">
-        <v>320</v>
+        <v>208</v>
       </c>
       <c r="L18" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1115,7 +1115,7 @@
         <v>Passed</v>
       </c>
       <c r="K19">
-        <v>191</v>
+        <v>266</v>
       </c>
       <c r="L19" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1153,7 +1153,7 @@
         <v>Passed</v>
       </c>
       <c r="K20">
-        <v>264</v>
+        <v>343</v>
       </c>
       <c r="L20" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1191,7 +1191,7 @@
         <v>Passed</v>
       </c>
       <c r="K21">
-        <v>246</v>
+        <v>346</v>
       </c>
       <c r="L21" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1229,7 +1229,7 @@
         <v>Passed</v>
       </c>
       <c r="K22">
-        <v>178</v>
+        <v>192</v>
       </c>
       <c r="L22" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1267,7 +1267,7 @@
         <v>Passed</v>
       </c>
       <c r="K23">
-        <v>168</v>
+        <v>225</v>
       </c>
       <c r="L23" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1305,7 +1305,7 @@
         <v>Passed</v>
       </c>
       <c r="K24">
-        <v>159</v>
+        <v>254</v>
       </c>
       <c r="L24" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1343,7 +1343,7 @@
         <v>Passed</v>
       </c>
       <c r="K25">
-        <v>187</v>
+        <v>203</v>
       </c>
       <c r="L25" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1381,7 +1381,7 @@
         <v>Passed</v>
       </c>
       <c r="K26">
-        <v>325</v>
+        <v>183</v>
       </c>
       <c r="L26" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1419,7 +1419,7 @@
         <v>Passed</v>
       </c>
       <c r="K27">
-        <v>220</v>
+        <v>313</v>
       </c>
       <c r="L27" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1457,7 +1457,7 @@
         <v>Passed</v>
       </c>
       <c r="K28">
-        <v>308</v>
+        <v>231</v>
       </c>
       <c r="L28" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1495,7 +1495,7 @@
         <v>Passed</v>
       </c>
       <c r="K29">
-        <v>204</v>
+        <v>366</v>
       </c>
       <c r="L29" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1533,7 +1533,7 @@
         <v>Passed</v>
       </c>
       <c r="K30">
-        <v>284</v>
+        <v>172</v>
       </c>
       <c r="L30" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1571,7 +1571,7 @@
         <v>Passed</v>
       </c>
       <c r="K31">
-        <v>190</v>
+        <v>334</v>
       </c>
       <c r="L31" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1609,7 +1609,7 @@
         <v>Passed</v>
       </c>
       <c r="K32">
-        <v>199</v>
+        <v>231</v>
       </c>
       <c r="L32" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1647,7 +1647,7 @@
         <v>Passed</v>
       </c>
       <c r="K33">
-        <v>226</v>
+        <v>243</v>
       </c>
       <c r="L33" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1685,7 +1685,7 @@
         <v>Passed</v>
       </c>
       <c r="K34">
-        <v>155</v>
+        <v>232</v>
       </c>
       <c r="L34" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1723,7 +1723,7 @@
         <v>Passed</v>
       </c>
       <c r="K35">
-        <v>293</v>
+        <v>225</v>
       </c>
       <c r="L35" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1761,7 +1761,7 @@
         <v>Passed</v>
       </c>
       <c r="K36">
-        <v>359</v>
+        <v>221</v>
       </c>
       <c r="L36" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1799,7 +1799,7 @@
         <v>Passed</v>
       </c>
       <c r="K37">
-        <v>174</v>
+        <v>396</v>
       </c>
       <c r="L37" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1837,7 +1837,7 @@
         <v>Passed</v>
       </c>
       <c r="K38">
-        <v>361</v>
+        <v>381</v>
       </c>
       <c r="L38" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1875,7 +1875,7 @@
         <v>Passed</v>
       </c>
       <c r="K39">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="L39" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1913,7 +1913,7 @@
         <v>Passed</v>
       </c>
       <c r="K40">
-        <v>370</v>
+        <v>313</v>
       </c>
       <c r="L40" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1951,7 +1951,7 @@
         <v>Passed</v>
       </c>
       <c r="K41">
-        <v>210</v>
+        <v>276</v>
       </c>
       <c r="L41" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1989,7 +1989,7 @@
         <v>Passed</v>
       </c>
       <c r="K42">
-        <v>213</v>
+        <v>251</v>
       </c>
       <c r="L42" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2027,7 +2027,7 @@
         <v>Passed</v>
       </c>
       <c r="K43">
-        <v>269</v>
+        <v>396</v>
       </c>
       <c r="L43" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2065,7 +2065,7 @@
         <v>Passed</v>
       </c>
       <c r="K44">
-        <v>362</v>
+        <v>370</v>
       </c>
       <c r="L44" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2103,7 +2103,7 @@
         <v>Passed</v>
       </c>
       <c r="K45">
-        <v>359</v>
+        <v>344</v>
       </c>
       <c r="L45" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2141,7 +2141,7 @@
         <v>Passed</v>
       </c>
       <c r="K46">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="L46" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2179,7 +2179,7 @@
         <v>Passed</v>
       </c>
       <c r="K47">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="L47" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2217,7 +2217,7 @@
         <v>Passed</v>
       </c>
       <c r="K48">
-        <v>161</v>
+        <v>371</v>
       </c>
       <c r="L48" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2255,7 +2255,7 @@
         <v>Passed</v>
       </c>
       <c r="K49">
-        <v>322</v>
+        <v>268</v>
       </c>
       <c r="L49" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2293,7 +2293,7 @@
         <v>Passed</v>
       </c>
       <c r="K50">
-        <v>207</v>
+        <v>279</v>
       </c>
       <c r="L50" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2331,7 +2331,7 @@
         <v>Passed</v>
       </c>
       <c r="K51">
-        <v>276</v>
+        <v>254</v>
       </c>
       <c r="L51" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2369,7 +2369,7 @@
         <v>Passed</v>
       </c>
       <c r="K52">
-        <v>394</v>
+        <v>204</v>
       </c>
       <c r="L52" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2407,7 +2407,7 @@
         <v>Passed</v>
       </c>
       <c r="K53">
-        <v>247</v>
+        <v>185</v>
       </c>
       <c r="L53" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2445,7 +2445,7 @@
         <v>Passed</v>
       </c>
       <c r="K54">
-        <v>279</v>
+        <v>178</v>
       </c>
       <c r="L54" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2483,7 +2483,7 @@
         <v>Passed</v>
       </c>
       <c r="K55">
-        <v>192</v>
+        <v>331</v>
       </c>
       <c r="L55" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2521,7 +2521,7 @@
         <v>Passed</v>
       </c>
       <c r="K56">
-        <v>306</v>
+        <v>222</v>
       </c>
       <c r="L56" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2559,7 +2559,7 @@
         <v>Passed</v>
       </c>
       <c r="K57">
-        <v>362</v>
+        <v>314</v>
       </c>
       <c r="L57" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2597,7 +2597,7 @@
         <v>Passed</v>
       </c>
       <c r="K58">
-        <v>288</v>
+        <v>248</v>
       </c>
       <c r="L58" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2635,7 +2635,7 @@
         <v>Passed</v>
       </c>
       <c r="K59">
-        <v>366</v>
+        <v>279</v>
       </c>
       <c r="L59" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2673,7 +2673,7 @@
         <v>Passed</v>
       </c>
       <c r="K60">
-        <v>384</v>
+        <v>250</v>
       </c>
       <c r="L60" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2711,7 +2711,7 @@
         <v>Passed</v>
       </c>
       <c r="K61">
-        <v>337</v>
+        <v>321</v>
       </c>
       <c r="L61" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2749,7 +2749,7 @@
         <v>Passed</v>
       </c>
       <c r="K62">
-        <v>240</v>
+        <v>187</v>
       </c>
       <c r="L62" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2787,7 +2787,7 @@
         <v>Passed</v>
       </c>
       <c r="K63">
-        <v>308</v>
+        <v>186</v>
       </c>
       <c r="L63" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2825,7 +2825,7 @@
         <v>Passed</v>
       </c>
       <c r="K64">
-        <v>280</v>
+        <v>295</v>
       </c>
       <c r="L64" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2863,7 +2863,7 @@
         <v>Passed</v>
       </c>
       <c r="K65">
-        <v>155</v>
+        <v>192</v>
       </c>
       <c r="L65" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2901,7 +2901,7 @@
         <v>Passed</v>
       </c>
       <c r="K66">
-        <v>269</v>
+        <v>371</v>
       </c>
       <c r="L66" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2939,7 +2939,7 @@
         <v>Passed</v>
       </c>
       <c r="K67">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="L67" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2977,7 +2977,7 @@
         <v>Passed</v>
       </c>
       <c r="K68">
-        <v>255</v>
+        <v>364</v>
       </c>
       <c r="L68" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3015,7 +3015,7 @@
         <v>Passed</v>
       </c>
       <c r="K69">
-        <v>165</v>
+        <v>276</v>
       </c>
       <c r="L69" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3053,7 +3053,7 @@
         <v>Passed</v>
       </c>
       <c r="K70">
-        <v>313</v>
+        <v>174</v>
       </c>
       <c r="L70" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3091,7 +3091,7 @@
         <v>Passed</v>
       </c>
       <c r="K71">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="L71" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3129,7 +3129,7 @@
         <v>Passed</v>
       </c>
       <c r="K72">
-        <v>154</v>
+        <v>372</v>
       </c>
       <c r="L72" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3167,7 +3167,7 @@
         <v>Passed</v>
       </c>
       <c r="K73">
-        <v>320</v>
+        <v>270</v>
       </c>
       <c r="L73" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3205,7 +3205,7 @@
         <v>Passed</v>
       </c>
       <c r="K74">
-        <v>189</v>
+        <v>253</v>
       </c>
       <c r="L74" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3243,7 +3243,7 @@
         <v>Passed</v>
       </c>
       <c r="K75">
-        <v>294</v>
+        <v>206</v>
       </c>
       <c r="L75" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3281,7 +3281,7 @@
         <v>Passed</v>
       </c>
       <c r="K76">
-        <v>258</v>
+        <v>160</v>
       </c>
       <c r="L76" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3319,7 +3319,7 @@
         <v>Passed</v>
       </c>
       <c r="K77">
-        <v>378</v>
+        <v>207</v>
       </c>
       <c r="L77" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3357,7 +3357,7 @@
         <v>Passed</v>
       </c>
       <c r="K78">
-        <v>175</v>
+        <v>389</v>
       </c>
       <c r="L78" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3395,7 +3395,7 @@
         <v>Passed</v>
       </c>
       <c r="K79">
-        <v>360</v>
+        <v>376</v>
       </c>
       <c r="L79" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3433,7 +3433,7 @@
         <v>Passed</v>
       </c>
       <c r="K80">
-        <v>235</v>
+        <v>333</v>
       </c>
       <c r="L80" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3471,7 +3471,7 @@
         <v>Passed</v>
       </c>
       <c r="K81">
-        <v>198</v>
+        <v>236</v>
       </c>
       <c r="L81" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3509,7 +3509,7 @@
         <v>Passed</v>
       </c>
       <c r="K82">
-        <v>270</v>
+        <v>278</v>
       </c>
       <c r="L82" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3547,7 +3547,7 @@
         <v>Passed</v>
       </c>
       <c r="K83">
-        <v>346</v>
+        <v>372</v>
       </c>
       <c r="L83" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3585,7 +3585,7 @@
         <v>Passed</v>
       </c>
       <c r="K84">
-        <v>354</v>
+        <v>264</v>
       </c>
       <c r="L84" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3623,7 +3623,7 @@
         <v>Passed</v>
       </c>
       <c r="K85">
-        <v>280</v>
+        <v>324</v>
       </c>
       <c r="L85" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3661,7 +3661,7 @@
         <v>Passed</v>
       </c>
       <c r="K86">
-        <v>229</v>
+        <v>153</v>
       </c>
       <c r="L86" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3699,7 +3699,7 @@
         <v>Passed</v>
       </c>
       <c r="K87">
-        <v>348</v>
+        <v>314</v>
       </c>
       <c r="L87" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3737,7 +3737,7 @@
         <v>Passed</v>
       </c>
       <c r="K88">
-        <v>332</v>
+        <v>182</v>
       </c>
       <c r="L88" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3775,7 +3775,7 @@
         <v>Passed</v>
       </c>
       <c r="K89">
-        <v>207</v>
+        <v>227</v>
       </c>
       <c r="L89" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3813,7 +3813,7 @@
         <v>Passed</v>
       </c>
       <c r="K90">
-        <v>195</v>
+        <v>353</v>
       </c>
       <c r="L90" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3851,7 +3851,7 @@
         <v>Passed</v>
       </c>
       <c r="K91">
-        <v>237</v>
+        <v>196</v>
       </c>
       <c r="L91" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3889,7 +3889,7 @@
         <v>Passed</v>
       </c>
       <c r="K92">
-        <v>399</v>
+        <v>164</v>
       </c>
       <c r="L92" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3927,7 +3927,7 @@
         <v>Passed</v>
       </c>
       <c r="K93">
-        <v>287</v>
+        <v>388</v>
       </c>
       <c r="L93" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3965,7 +3965,7 @@
         <v>Passed</v>
       </c>
       <c r="K94">
-        <v>195</v>
+        <v>330</v>
       </c>
       <c r="L94" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4003,7 +4003,7 @@
         <v>Passed</v>
       </c>
       <c r="K95">
-        <v>333</v>
+        <v>325</v>
       </c>
       <c r="L95" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4041,7 +4041,7 @@
         <v>Passed</v>
       </c>
       <c r="K96">
-        <v>307</v>
+        <v>379</v>
       </c>
       <c r="L96" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4079,7 +4079,7 @@
         <v>Passed</v>
       </c>
       <c r="K97">
-        <v>388</v>
+        <v>184</v>
       </c>
       <c r="L97" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4117,7 +4117,7 @@
         <v>Passed</v>
       </c>
       <c r="K98">
-        <v>221</v>
+        <v>363</v>
       </c>
       <c r="L98" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4155,7 +4155,7 @@
         <v>Passed</v>
       </c>
       <c r="K99">
-        <v>195</v>
+        <v>367</v>
       </c>
       <c r="L99" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4193,7 +4193,7 @@
         <v>Passed</v>
       </c>
       <c r="K100">
-        <v>388</v>
+        <v>223</v>
       </c>
       <c r="L100" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4231,7 +4231,7 @@
         <v>Passed</v>
       </c>
       <c r="K101">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="L101" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4269,7 +4269,7 @@
         <v>Passed</v>
       </c>
       <c r="K102">
-        <v>393</v>
+        <v>378</v>
       </c>
       <c r="L102" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4307,7 +4307,7 @@
         <v>Passed</v>
       </c>
       <c r="K103">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="L103" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4345,7 +4345,7 @@
         <v>Passed</v>
       </c>
       <c r="K104">
-        <v>203</v>
+        <v>383</v>
       </c>
       <c r="L104" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4383,7 +4383,7 @@
         <v>Passed</v>
       </c>
       <c r="K105">
-        <v>326</v>
+        <v>303</v>
       </c>
       <c r="L105" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4421,7 +4421,7 @@
         <v>Passed</v>
       </c>
       <c r="K106">
-        <v>258</v>
+        <v>334</v>
       </c>
       <c r="L106" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4459,7 +4459,7 @@
         <v>Passed</v>
       </c>
       <c r="K107">
-        <v>227</v>
+        <v>379</v>
       </c>
       <c r="L107" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4497,7 +4497,7 @@
         <v>Passed</v>
       </c>
       <c r="K108">
-        <v>205</v>
+        <v>366</v>
       </c>
       <c r="L108" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4535,7 +4535,7 @@
         <v>Passed</v>
       </c>
       <c r="K109">
-        <v>231</v>
+        <v>372</v>
       </c>
       <c r="L109" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4573,7 +4573,7 @@
         <v>Passed</v>
       </c>
       <c r="K110">
-        <v>251</v>
+        <v>269</v>
       </c>
       <c r="L110" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4611,7 +4611,7 @@
         <v>Passed</v>
       </c>
       <c r="K111">
-        <v>338</v>
+        <v>279</v>
       </c>
       <c r="L111" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4649,7 +4649,7 @@
         <v>Passed</v>
       </c>
       <c r="K112">
-        <v>160</v>
+        <v>286</v>
       </c>
       <c r="L112" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4687,7 +4687,7 @@
         <v>Passed</v>
       </c>
       <c r="K113">
-        <v>340</v>
+        <v>179</v>
       </c>
       <c r="L113" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4725,7 +4725,7 @@
         <v>Passed</v>
       </c>
       <c r="K114">
-        <v>284</v>
+        <v>193</v>
       </c>
       <c r="L114" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4763,7 +4763,7 @@
         <v>Passed</v>
       </c>
       <c r="K115">
-        <v>176</v>
+        <v>377</v>
       </c>
       <c r="L115" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4801,7 +4801,7 @@
         <v>Passed</v>
       </c>
       <c r="K116">
-        <v>389</v>
+        <v>159</v>
       </c>
       <c r="L116" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4839,7 +4839,7 @@
         <v>Passed</v>
       </c>
       <c r="K117">
-        <v>171</v>
+        <v>264</v>
       </c>
       <c r="L117" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4877,7 +4877,7 @@
         <v>Passed</v>
       </c>
       <c r="K118">
-        <v>199</v>
+        <v>252</v>
       </c>
       <c r="L118" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4915,7 +4915,7 @@
         <v>Passed</v>
       </c>
       <c r="K119">
-        <v>369</v>
+        <v>344</v>
       </c>
       <c r="L119" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4953,7 +4953,7 @@
         <v>Passed</v>
       </c>
       <c r="K120">
-        <v>367</v>
+        <v>379</v>
       </c>
       <c r="L120" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4991,7 +4991,7 @@
         <v>Passed</v>
       </c>
       <c r="K121">
-        <v>248</v>
+        <v>387</v>
       </c>
       <c r="L121" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5029,7 +5029,7 @@
         <v>Passed</v>
       </c>
       <c r="K122">
-        <v>322</v>
+        <v>210</v>
       </c>
       <c r="L122" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5067,7 +5067,7 @@
         <v>Passed</v>
       </c>
       <c r="K123">
-        <v>261</v>
+        <v>284</v>
       </c>
       <c r="L123" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5105,7 +5105,7 @@
         <v>Passed</v>
       </c>
       <c r="K124">
-        <v>191</v>
+        <v>344</v>
       </c>
       <c r="L124" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5143,7 +5143,7 @@
         <v>Passed</v>
       </c>
       <c r="K125">
-        <v>151</v>
+        <v>269</v>
       </c>
       <c r="L125" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5181,7 +5181,7 @@
         <v>Passed</v>
       </c>
       <c r="K126">
-        <v>303</v>
+        <v>174</v>
       </c>
       <c r="L126" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5219,7 +5219,7 @@
         <v>Passed</v>
       </c>
       <c r="K127">
-        <v>367</v>
+        <v>158</v>
       </c>
       <c r="L127" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5257,7 +5257,7 @@
         <v>Passed</v>
       </c>
       <c r="K128">
-        <v>348</v>
+        <v>294</v>
       </c>
       <c r="L128" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5295,7 +5295,7 @@
         <v>Passed</v>
       </c>
       <c r="K129">
-        <v>175</v>
+        <v>254</v>
       </c>
       <c r="L129" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5333,7 +5333,7 @@
         <v>Passed</v>
       </c>
       <c r="K130">
-        <v>377</v>
+        <v>221</v>
       </c>
       <c r="L130" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5371,7 +5371,7 @@
         <v>Passed</v>
       </c>
       <c r="K131">
-        <v>177</v>
+        <v>245</v>
       </c>
       <c r="L131" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5409,7 +5409,7 @@
         <v>Passed</v>
       </c>
       <c r="K132">
-        <v>274</v>
+        <v>161</v>
       </c>
       <c r="L132" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5447,7 +5447,7 @@
         <v>Passed</v>
       </c>
       <c r="K133">
-        <v>260</v>
+        <v>240</v>
       </c>
       <c r="L133" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5485,7 +5485,7 @@
         <v>Passed</v>
       </c>
       <c r="K134">
-        <v>304</v>
+        <v>244</v>
       </c>
       <c r="L134" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5523,7 +5523,7 @@
         <v>Passed</v>
       </c>
       <c r="K135">
-        <v>206</v>
+        <v>344</v>
       </c>
       <c r="L135" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5561,7 +5561,7 @@
         <v>Passed</v>
       </c>
       <c r="K136">
-        <v>251</v>
+        <v>316</v>
       </c>
       <c r="L136" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5599,7 +5599,7 @@
         <v>Passed</v>
       </c>
       <c r="K137">
-        <v>319</v>
+        <v>396</v>
       </c>
       <c r="L137" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5637,7 +5637,7 @@
         <v>Passed</v>
       </c>
       <c r="K138">
-        <v>276</v>
+        <v>238</v>
       </c>
       <c r="L138" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5675,7 +5675,7 @@
         <v>Passed</v>
       </c>
       <c r="K139">
-        <v>363</v>
+        <v>247</v>
       </c>
       <c r="L139" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5713,7 +5713,7 @@
         <v>Passed</v>
       </c>
       <c r="K140">
-        <v>183</v>
+        <v>275</v>
       </c>
       <c r="L140" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5751,7 +5751,7 @@
         <v>Passed</v>
       </c>
       <c r="K141">
-        <v>258</v>
+        <v>245</v>
       </c>
       <c r="L141" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5789,7 +5789,7 @@
         <v>Passed</v>
       </c>
       <c r="K142">
-        <v>171</v>
+        <v>268</v>
       </c>
       <c r="L142" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5827,7 +5827,7 @@
         <v>Passed</v>
       </c>
       <c r="K143">
-        <v>397</v>
+        <v>184</v>
       </c>
       <c r="L143" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5865,7 +5865,7 @@
         <v>Passed</v>
       </c>
       <c r="K144">
-        <v>271</v>
+        <v>201</v>
       </c>
       <c r="L144" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5903,7 +5903,7 @@
         <v>Passed</v>
       </c>
       <c r="K145">
-        <v>342</v>
+        <v>297</v>
       </c>
       <c r="L145" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5941,7 +5941,7 @@
         <v>Passed</v>
       </c>
       <c r="K146">
-        <v>390</v>
+        <v>209</v>
       </c>
       <c r="L146" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5979,7 +5979,7 @@
         <v>Passed</v>
       </c>
       <c r="K147">
-        <v>378</v>
+        <v>215</v>
       </c>
       <c r="L147" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6017,7 +6017,7 @@
         <v>Passed</v>
       </c>
       <c r="K148">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="L148" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6055,7 +6055,7 @@
         <v>Passed</v>
       </c>
       <c r="K149">
-        <v>199</v>
+        <v>163</v>
       </c>
       <c r="L149" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6093,7 +6093,7 @@
         <v>Passed</v>
       </c>
       <c r="K150">
-        <v>363</v>
+        <v>271</v>
       </c>
       <c r="L150" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6131,7 +6131,7 @@
         <v>Passed</v>
       </c>
       <c r="K151">
-        <v>366</v>
+        <v>399</v>
       </c>
       <c r="L151" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6169,7 +6169,7 @@
         <v>Passed</v>
       </c>
       <c r="K152">
-        <v>180</v>
+        <v>337</v>
       </c>
       <c r="L152" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6207,7 +6207,7 @@
         <v>Passed</v>
       </c>
       <c r="K153">
-        <v>240</v>
+        <v>357</v>
       </c>
       <c r="L153" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6245,7 +6245,7 @@
         <v>Passed</v>
       </c>
       <c r="K154">
-        <v>262</v>
+        <v>171</v>
       </c>
       <c r="L154" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6283,7 +6283,7 @@
         <v>Passed</v>
       </c>
       <c r="K155">
-        <v>253</v>
+        <v>384</v>
       </c>
       <c r="L155" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6321,7 +6321,7 @@
         <v>Passed</v>
       </c>
       <c r="K156">
-        <v>208</v>
+        <v>258</v>
       </c>
       <c r="L156" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6359,7 +6359,7 @@
         <v>Passed</v>
       </c>
       <c r="K157">
-        <v>397</v>
+        <v>317</v>
       </c>
       <c r="L157" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6397,7 +6397,7 @@
         <v>Passed</v>
       </c>
       <c r="K158">
-        <v>336</v>
+        <v>378</v>
       </c>
       <c r="L158" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6435,7 +6435,7 @@
         <v>Passed</v>
       </c>
       <c r="K159">
-        <v>399</v>
+        <v>394</v>
       </c>
       <c r="L159" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6473,7 +6473,7 @@
         <v>Passed</v>
       </c>
       <c r="K160">
-        <v>300</v>
+        <v>211</v>
       </c>
       <c r="L160" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6511,7 +6511,7 @@
         <v>Passed</v>
       </c>
       <c r="K161">
-        <v>251</v>
+        <v>258</v>
       </c>
       <c r="L161" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6549,7 +6549,7 @@
         <v>Passed</v>
       </c>
       <c r="K162">
-        <v>324</v>
+        <v>180</v>
       </c>
       <c r="L162" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6587,7 +6587,7 @@
         <v>Passed</v>
       </c>
       <c r="K163">
-        <v>214</v>
+        <v>300</v>
       </c>
       <c r="L163" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6625,7 +6625,7 @@
         <v>Passed</v>
       </c>
       <c r="K164">
-        <v>268</v>
+        <v>161</v>
       </c>
       <c r="L164" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6663,7 +6663,7 @@
         <v>Passed</v>
       </c>
       <c r="K165">
-        <v>361</v>
+        <v>207</v>
       </c>
       <c r="L165" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6701,7 +6701,7 @@
         <v>Passed</v>
       </c>
       <c r="K166">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="L166" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6739,7 +6739,7 @@
         <v>Passed</v>
       </c>
       <c r="K167">
-        <v>297</v>
+        <v>324</v>
       </c>
       <c r="L167" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6777,7 +6777,7 @@
         <v>Passed</v>
       </c>
       <c r="K168">
-        <v>351</v>
+        <v>368</v>
       </c>
       <c r="L168" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6815,7 +6815,7 @@
         <v>Passed</v>
       </c>
       <c r="K169">
-        <v>252</v>
+        <v>203</v>
       </c>
       <c r="L169" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6853,7 +6853,7 @@
         <v>Passed</v>
       </c>
       <c r="K170">
-        <v>394</v>
+        <v>327</v>
       </c>
       <c r="L170" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6891,7 +6891,7 @@
         <v>Passed</v>
       </c>
       <c r="K171">
-        <v>200</v>
+        <v>154</v>
       </c>
       <c r="L171" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6929,7 +6929,7 @@
         <v>Passed</v>
       </c>
       <c r="K172">
-        <v>217</v>
+        <v>166</v>
       </c>
       <c r="L172" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6967,7 +6967,7 @@
         <v>Passed</v>
       </c>
       <c r="K173">
-        <v>374</v>
+        <v>213</v>
       </c>
       <c r="L173" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7005,7 +7005,7 @@
         <v>Passed</v>
       </c>
       <c r="K174">
-        <v>378</v>
+        <v>256</v>
       </c>
       <c r="L174" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7043,7 +7043,7 @@
         <v>Passed</v>
       </c>
       <c r="K175">
-        <v>371</v>
+        <v>348</v>
       </c>
       <c r="L175" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7081,7 +7081,7 @@
         <v>Passed</v>
       </c>
       <c r="K176">
-        <v>301</v>
+        <v>313</v>
       </c>
       <c r="L176" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7119,7 +7119,7 @@
         <v>Passed</v>
       </c>
       <c r="K177">
-        <v>384</v>
+        <v>245</v>
       </c>
       <c r="L177" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7157,7 +7157,7 @@
         <v>Passed</v>
       </c>
       <c r="K178">
-        <v>176</v>
+        <v>279</v>
       </c>
       <c r="L178" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7195,7 +7195,7 @@
         <v>Passed</v>
       </c>
       <c r="K179">
-        <v>363</v>
+        <v>396</v>
       </c>
       <c r="L179" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7233,7 +7233,7 @@
         <v>Passed</v>
       </c>
       <c r="K180">
-        <v>273</v>
+        <v>208</v>
       </c>
       <c r="L180" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7271,7 +7271,7 @@
         <v>Passed</v>
       </c>
       <c r="K181">
-        <v>250</v>
+        <v>277</v>
       </c>
       <c r="L181" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7309,7 +7309,7 @@
         <v>Passed</v>
       </c>
       <c r="K182">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="L182" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7347,7 +7347,7 @@
         <v>Passed</v>
       </c>
       <c r="K183">
-        <v>197</v>
+        <v>324</v>
       </c>
       <c r="L183" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7385,7 +7385,7 @@
         <v>Passed</v>
       </c>
       <c r="K184">
-        <v>325</v>
+        <v>276</v>
       </c>
       <c r="L184" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7423,7 +7423,7 @@
         <v>Passed</v>
       </c>
       <c r="K185">
-        <v>292</v>
+        <v>173</v>
       </c>
       <c r="L185" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7461,7 +7461,7 @@
         <v>Passed</v>
       </c>
       <c r="K186">
-        <v>394</v>
+        <v>289</v>
       </c>
       <c r="L186" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7499,7 +7499,7 @@
         <v>Passed</v>
       </c>
       <c r="K187">
-        <v>302</v>
+        <v>380</v>
       </c>
       <c r="L187" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7537,7 +7537,7 @@
         <v>Passed</v>
       </c>
       <c r="K188">
-        <v>359</v>
+        <v>266</v>
       </c>
       <c r="L188" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7575,7 +7575,7 @@
         <v>Passed</v>
       </c>
       <c r="K189">
-        <v>302</v>
+        <v>217</v>
       </c>
       <c r="L189" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7613,7 +7613,7 @@
         <v>Passed</v>
       </c>
       <c r="K190">
-        <v>219</v>
+        <v>250</v>
       </c>
       <c r="L190" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7651,7 +7651,7 @@
         <v>Passed</v>
       </c>
       <c r="K191">
-        <v>392</v>
+        <v>321</v>
       </c>
       <c r="L191" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7689,7 +7689,7 @@
         <v>Passed</v>
       </c>
       <c r="K192">
-        <v>307</v>
+        <v>326</v>
       </c>
       <c r="L192" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7727,7 +7727,7 @@
         <v>Passed</v>
       </c>
       <c r="K193">
-        <v>388</v>
+        <v>327</v>
       </c>
       <c r="L193" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7765,7 +7765,7 @@
         <v>Passed</v>
       </c>
       <c r="K194">
-        <v>316</v>
+        <v>225</v>
       </c>
       <c r="L194" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7803,7 +7803,7 @@
         <v>Passed</v>
       </c>
       <c r="K195">
-        <v>256</v>
+        <v>237</v>
       </c>
       <c r="L195" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7841,7 +7841,7 @@
         <v>Passed</v>
       </c>
       <c r="K196">
-        <v>339</v>
+        <v>359</v>
       </c>
       <c r="L196" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7879,7 +7879,7 @@
         <v>Passed</v>
       </c>
       <c r="K197">
-        <v>334</v>
+        <v>310</v>
       </c>
       <c r="L197" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7917,7 +7917,7 @@
         <v>Passed</v>
       </c>
       <c r="K198">
-        <v>288</v>
+        <v>296</v>
       </c>
       <c r="L198" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7955,7 +7955,7 @@
         <v>Passed</v>
       </c>
       <c r="K199">
-        <v>386</v>
+        <v>181</v>
       </c>
       <c r="L199" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7993,7 +7993,7 @@
         <v>Passed</v>
       </c>
       <c r="K200">
-        <v>353</v>
+        <v>331</v>
       </c>
       <c r="L200" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8031,7 +8031,7 @@
         <v>Passed</v>
       </c>
       <c r="K201">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="L201" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8069,7 +8069,7 @@
         <v>Passed</v>
       </c>
       <c r="K202">
-        <v>331</v>
+        <v>393</v>
       </c>
       <c r="L202" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8107,7 +8107,7 @@
         <v>Passed</v>
       </c>
       <c r="K203">
-        <v>339</v>
+        <v>314</v>
       </c>
       <c r="L203" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8145,7 +8145,7 @@
         <v>Passed</v>
       </c>
       <c r="K204">
-        <v>171</v>
+        <v>373</v>
       </c>
       <c r="L204" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8183,7 +8183,7 @@
         <v>Passed</v>
       </c>
       <c r="K205">
-        <v>224</v>
+        <v>343</v>
       </c>
       <c r="L205" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8221,7 +8221,7 @@
         <v>Passed</v>
       </c>
       <c r="K206">
-        <v>227</v>
+        <v>176</v>
       </c>
       <c r="L206" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8259,7 +8259,7 @@
         <v>Passed</v>
       </c>
       <c r="K207">
-        <v>306</v>
+        <v>330</v>
       </c>
       <c r="L207" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8297,7 +8297,7 @@
         <v>Passed</v>
       </c>
       <c r="K208">
-        <v>304</v>
+        <v>271</v>
       </c>
       <c r="L208" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8335,7 +8335,7 @@
         <v>Passed</v>
       </c>
       <c r="K209">
-        <v>325</v>
+        <v>223</v>
       </c>
       <c r="L209" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8373,7 +8373,7 @@
         <v>Passed</v>
       </c>
       <c r="K210">
-        <v>150</v>
+        <v>197</v>
       </c>
       <c r="L210" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8411,7 +8411,7 @@
         <v>Passed</v>
       </c>
       <c r="K211">
-        <v>382</v>
+        <v>325</v>
       </c>
       <c r="L211" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8449,7 +8449,7 @@
         <v>Passed</v>
       </c>
       <c r="K212">
-        <v>174</v>
+        <v>227</v>
       </c>
       <c r="L212" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8487,7 +8487,7 @@
         <v>Passed</v>
       </c>
       <c r="K213">
-        <v>225</v>
+        <v>294</v>
       </c>
       <c r="L213" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8525,7 +8525,7 @@
         <v>Passed</v>
       </c>
       <c r="K214">
-        <v>208</v>
+        <v>189</v>
       </c>
       <c r="L214" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8563,7 +8563,7 @@
         <v>Passed</v>
       </c>
       <c r="K215">
-        <v>358</v>
+        <v>234</v>
       </c>
       <c r="L215" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8601,7 +8601,7 @@
         <v>Passed</v>
       </c>
       <c r="K216">
-        <v>170</v>
+        <v>260</v>
       </c>
       <c r="L216" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8639,7 +8639,7 @@
         <v>Passed</v>
       </c>
       <c r="K217">
-        <v>239</v>
+        <v>214</v>
       </c>
       <c r="L217" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8677,7 +8677,7 @@
         <v>Passed</v>
       </c>
       <c r="K218">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="L218" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8715,7 +8715,7 @@
         <v>Passed</v>
       </c>
       <c r="K219">
-        <v>187</v>
+        <v>320</v>
       </c>
       <c r="L219" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8753,7 +8753,7 @@
         <v>Passed</v>
       </c>
       <c r="K220">
-        <v>263</v>
+        <v>333</v>
       </c>
       <c r="L220" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8791,7 +8791,7 @@
         <v>Passed</v>
       </c>
       <c r="K221">
-        <v>356</v>
+        <v>320</v>
       </c>
       <c r="L221" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8829,7 +8829,7 @@
         <v>Passed</v>
       </c>
       <c r="K222">
-        <v>359</v>
+        <v>309</v>
       </c>
       <c r="L222" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8867,7 +8867,7 @@
         <v>Passed</v>
       </c>
       <c r="K223">
-        <v>275</v>
+        <v>250</v>
       </c>
       <c r="L223" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8905,7 +8905,7 @@
         <v>Passed</v>
       </c>
       <c r="K224">
-        <v>181</v>
+        <v>201</v>
       </c>
       <c r="L224" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8943,7 +8943,7 @@
         <v>Passed</v>
       </c>
       <c r="K225">
-        <v>183</v>
+        <v>227</v>
       </c>
       <c r="L225" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8981,7 +8981,7 @@
         <v>Passed</v>
       </c>
       <c r="K226">
-        <v>394</v>
+        <v>203</v>
       </c>
       <c r="L226" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9019,7 +9019,7 @@
         <v>Passed</v>
       </c>
       <c r="K227">
-        <v>284</v>
+        <v>197</v>
       </c>
       <c r="L227" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9057,7 +9057,7 @@
         <v>Passed</v>
       </c>
       <c r="K228">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="L228" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9095,7 +9095,7 @@
         <v>Passed</v>
       </c>
       <c r="K229">
-        <v>288</v>
+        <v>207</v>
       </c>
       <c r="L229" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9133,7 +9133,7 @@
         <v>Passed</v>
       </c>
       <c r="K230">
-        <v>317</v>
+        <v>229</v>
       </c>
       <c r="L230" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9171,7 +9171,7 @@
         <v>Passed</v>
       </c>
       <c r="K231">
-        <v>331</v>
+        <v>306</v>
       </c>
       <c r="L231" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9209,7 +9209,7 @@
         <v>Passed</v>
       </c>
       <c r="K232">
-        <v>332</v>
+        <v>178</v>
       </c>
       <c r="L232" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9247,7 +9247,7 @@
         <v>Passed</v>
       </c>
       <c r="K233">
-        <v>198</v>
+        <v>227</v>
       </c>
       <c r="L233" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9285,7 +9285,7 @@
         <v>Passed</v>
       </c>
       <c r="K234">
-        <v>189</v>
+        <v>360</v>
       </c>
       <c r="L234" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9323,7 +9323,7 @@
         <v>Passed</v>
       </c>
       <c r="K235">
-        <v>170</v>
+        <v>323</v>
       </c>
       <c r="L235" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9361,7 +9361,7 @@
         <v>Passed</v>
       </c>
       <c r="K236">
-        <v>307</v>
+        <v>186</v>
       </c>
       <c r="L236" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9399,7 +9399,7 @@
         <v>Passed</v>
       </c>
       <c r="K237">
-        <v>232</v>
+        <v>257</v>
       </c>
       <c r="L237" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9437,7 +9437,7 @@
         <v>Passed</v>
       </c>
       <c r="K238">
-        <v>337</v>
+        <v>211</v>
       </c>
       <c r="L238" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9475,7 +9475,7 @@
         <v>Passed</v>
       </c>
       <c r="K239">
-        <v>154</v>
+        <v>218</v>
       </c>
       <c r="L239" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9513,7 +9513,7 @@
         <v>Passed</v>
       </c>
       <c r="K240">
-        <v>360</v>
+        <v>181</v>
       </c>
       <c r="L240" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9551,7 +9551,7 @@
         <v>Passed</v>
       </c>
       <c r="K241">
-        <v>166</v>
+        <v>380</v>
       </c>
       <c r="L241" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9589,7 +9589,7 @@
         <v>Passed</v>
       </c>
       <c r="K242">
-        <v>328</v>
+        <v>241</v>
       </c>
       <c r="L242" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9627,7 +9627,7 @@
         <v>Passed</v>
       </c>
       <c r="K243">
-        <v>163</v>
+        <v>243</v>
       </c>
       <c r="L243" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9665,7 +9665,7 @@
         <v>Passed</v>
       </c>
       <c r="K244">
-        <v>246</v>
+        <v>191</v>
       </c>
       <c r="L244" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9703,7 +9703,7 @@
         <v>Passed</v>
       </c>
       <c r="K245">
-        <v>284</v>
+        <v>190</v>
       </c>
       <c r="L245" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9741,7 +9741,7 @@
         <v>Passed</v>
       </c>
       <c r="K246">
-        <v>310</v>
+        <v>326</v>
       </c>
       <c r="L246" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9779,7 +9779,7 @@
         <v>Passed</v>
       </c>
       <c r="K247">
-        <v>343</v>
+        <v>398</v>
       </c>
       <c r="L247" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9817,7 +9817,7 @@
         <v>Passed</v>
       </c>
       <c r="K248">
-        <v>227</v>
+        <v>326</v>
       </c>
       <c r="L248" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9855,7 +9855,7 @@
         <v>Passed</v>
       </c>
       <c r="K249">
-        <v>340</v>
+        <v>152</v>
       </c>
       <c r="L249" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9893,7 +9893,7 @@
         <v>Passed</v>
       </c>
       <c r="K250">
-        <v>209</v>
+        <v>285</v>
       </c>
       <c r="L250" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9931,7 +9931,7 @@
         <v>Passed</v>
       </c>
       <c r="K251">
-        <v>290</v>
+        <v>281</v>
       </c>
       <c r="L251" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9969,7 +9969,7 @@
         <v>Passed</v>
       </c>
       <c r="K252">
-        <v>215</v>
+        <v>242</v>
       </c>
       <c r="L252" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10007,7 +10007,7 @@
         <v>Passed</v>
       </c>
       <c r="K253">
-        <v>152</v>
+        <v>318</v>
       </c>
       <c r="L253" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10045,7 +10045,7 @@
         <v>Passed</v>
       </c>
       <c r="K254">
-        <v>155</v>
+        <v>337</v>
       </c>
       <c r="L254" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10083,7 +10083,7 @@
         <v>Passed</v>
       </c>
       <c r="K255">
-        <v>264</v>
+        <v>227</v>
       </c>
       <c r="L255" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10121,7 +10121,7 @@
         <v>Passed</v>
       </c>
       <c r="K256">
-        <v>344</v>
+        <v>386</v>
       </c>
       <c r="L256" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10159,7 +10159,7 @@
         <v>Passed</v>
       </c>
       <c r="K257">
-        <v>318</v>
+        <v>208</v>
       </c>
       <c r="L257" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10197,7 +10197,7 @@
         <v>Passed</v>
       </c>
       <c r="K258">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="L258" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10235,7 +10235,7 @@
         <v>Passed</v>
       </c>
       <c r="K259">
-        <v>340</v>
+        <v>251</v>
       </c>
       <c r="L259" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10273,7 +10273,7 @@
         <v>Passed</v>
       </c>
       <c r="K260">
-        <v>347</v>
+        <v>362</v>
       </c>
       <c r="L260" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10311,7 +10311,7 @@
         <v>Passed</v>
       </c>
       <c r="K261">
-        <v>292</v>
+        <v>259</v>
       </c>
       <c r="L261" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10349,7 +10349,7 @@
         <v>Passed</v>
       </c>
       <c r="K262">
-        <v>290</v>
+        <v>247</v>
       </c>
       <c r="L262" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10387,7 +10387,7 @@
         <v>Passed</v>
       </c>
       <c r="K263">
-        <v>343</v>
+        <v>230</v>
       </c>
       <c r="L263" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10425,7 +10425,7 @@
         <v>Passed</v>
       </c>
       <c r="K264">
-        <v>246</v>
+        <v>394</v>
       </c>
       <c r="L264" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10463,7 +10463,7 @@
         <v>Passed</v>
       </c>
       <c r="K265">
-        <v>391</v>
+        <v>263</v>
       </c>
       <c r="L265" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10501,7 +10501,7 @@
         <v>Passed</v>
       </c>
       <c r="K266">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="L266" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10539,7 +10539,7 @@
         <v>Passed</v>
       </c>
       <c r="K267">
-        <v>360</v>
+        <v>321</v>
       </c>
       <c r="L267" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10577,7 +10577,7 @@
         <v>Passed</v>
       </c>
       <c r="K268">
-        <v>376</v>
+        <v>211</v>
       </c>
       <c r="L268" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10615,7 +10615,7 @@
         <v>Passed</v>
       </c>
       <c r="K269">
-        <v>379</v>
+        <v>191</v>
       </c>
       <c r="L269" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10653,7 +10653,7 @@
         <v>Passed</v>
       </c>
       <c r="K270">
-        <v>160</v>
+        <v>388</v>
       </c>
       <c r="L270" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10691,7 +10691,7 @@
         <v>Passed</v>
       </c>
       <c r="K271">
-        <v>282</v>
+        <v>161</v>
       </c>
       <c r="L271" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10729,7 +10729,7 @@
         <v>Passed</v>
       </c>
       <c r="K272">
-        <v>380</v>
+        <v>229</v>
       </c>
       <c r="L272" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10767,7 +10767,7 @@
         <v>Passed</v>
       </c>
       <c r="K273">
-        <v>239</v>
+        <v>344</v>
       </c>
       <c r="L273" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10805,7 +10805,7 @@
         <v>Passed</v>
       </c>
       <c r="K274">
-        <v>245</v>
+        <v>197</v>
       </c>
       <c r="L274" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10843,7 +10843,7 @@
         <v>Passed</v>
       </c>
       <c r="K275">
-        <v>226</v>
+        <v>272</v>
       </c>
       <c r="L275" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10881,7 +10881,7 @@
         <v>Passed</v>
       </c>
       <c r="K276">
-        <v>344</v>
+        <v>172</v>
       </c>
       <c r="L276" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10919,7 +10919,7 @@
         <v>Passed</v>
       </c>
       <c r="K277">
-        <v>216</v>
+        <v>171</v>
       </c>
       <c r="L277" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10957,7 +10957,7 @@
         <v>Passed</v>
       </c>
       <c r="K278">
-        <v>343</v>
+        <v>391</v>
       </c>
       <c r="L278" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10995,7 +10995,7 @@
         <v>Passed</v>
       </c>
       <c r="K279">
-        <v>362</v>
+        <v>230</v>
       </c>
       <c r="L279" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11033,7 +11033,7 @@
         <v>Passed</v>
       </c>
       <c r="K280">
-        <v>340</v>
+        <v>154</v>
       </c>
       <c r="L280" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11071,7 +11071,7 @@
         <v>Passed</v>
       </c>
       <c r="K281">
-        <v>204</v>
+        <v>326</v>
       </c>
       <c r="L281" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11109,7 +11109,7 @@
         <v>Passed</v>
       </c>
       <c r="K282">
-        <v>383</v>
+        <v>296</v>
       </c>
       <c r="L282" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11147,7 +11147,7 @@
         <v>Passed</v>
       </c>
       <c r="K283">
-        <v>274</v>
+        <v>259</v>
       </c>
       <c r="L283" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11185,7 +11185,7 @@
         <v>Passed</v>
       </c>
       <c r="K284">
-        <v>184</v>
+        <v>213</v>
       </c>
       <c r="L284" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11223,7 +11223,7 @@
         <v>Passed</v>
       </c>
       <c r="K285">
-        <v>245</v>
+        <v>193</v>
       </c>
       <c r="L285" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11261,7 +11261,7 @@
         <v>Passed</v>
       </c>
       <c r="K286">
-        <v>297</v>
+        <v>367</v>
       </c>
       <c r="L286" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11299,7 +11299,7 @@
         <v>Passed</v>
       </c>
       <c r="K287">
-        <v>312</v>
+        <v>243</v>
       </c>
       <c r="L287" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11337,7 +11337,7 @@
         <v>Passed</v>
       </c>
       <c r="K288">
-        <v>231</v>
+        <v>209</v>
       </c>
       <c r="L288" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11375,7 +11375,7 @@
         <v>Passed</v>
       </c>
       <c r="K289">
-        <v>289</v>
+        <v>309</v>
       </c>
       <c r="L289" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11413,7 +11413,7 @@
         <v>Passed</v>
       </c>
       <c r="K290">
-        <v>257</v>
+        <v>287</v>
       </c>
       <c r="L290" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11451,7 +11451,7 @@
         <v>Passed</v>
       </c>
       <c r="K291">
-        <v>261</v>
+        <v>389</v>
       </c>
       <c r="L291" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11489,7 +11489,7 @@
         <v>Passed</v>
       </c>
       <c r="K292">
-        <v>288</v>
+        <v>208</v>
       </c>
       <c r="L292" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11527,7 +11527,7 @@
         <v>Passed</v>
       </c>
       <c r="K293">
-        <v>205</v>
+        <v>333</v>
       </c>
       <c r="L293" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11565,7 +11565,7 @@
         <v>Passed</v>
       </c>
       <c r="K294">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="L294" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11603,7 +11603,7 @@
         <v>Passed</v>
       </c>
       <c r="K295">
-        <v>225</v>
+        <v>249</v>
       </c>
       <c r="L295" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11641,7 +11641,7 @@
         <v>Passed</v>
       </c>
       <c r="K296">
-        <v>199</v>
+        <v>214</v>
       </c>
       <c r="L296" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11679,7 +11679,7 @@
         <v>Passed</v>
       </c>
       <c r="K297">
-        <v>369</v>
+        <v>244</v>
       </c>
       <c r="L297" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11717,7 +11717,7 @@
         <v>Passed</v>
       </c>
       <c r="K298">
-        <v>179</v>
+        <v>394</v>
       </c>
       <c r="L298" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11755,7 +11755,7 @@
         <v>Passed</v>
       </c>
       <c r="K299">
-        <v>365</v>
+        <v>354</v>
       </c>
       <c r="L299" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11793,7 +11793,7 @@
         <v>Passed</v>
       </c>
       <c r="K300">
-        <v>379</v>
+        <v>398</v>
       </c>
       <c r="L300" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11831,7 +11831,7 @@
         <v>Passed</v>
       </c>
       <c r="K301">
-        <v>204</v>
+        <v>161</v>
       </c>
       <c r="L301" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>

</xml_diff>

<commit_message>
feat: restrict audio player to Music & Culturals, upgrade all checkout stages to full-width web layout with space-dark theme
</commit_message>
<xml_diff>
--- a/EventSphere_Appium_Mobile_300_Report.xlsx
+++ b/EventSphere_Appium_Mobile_300_Report.xlsx
@@ -469,7 +469,7 @@
         <v>Passed</v>
       </c>
       <c r="K2">
-        <v>259</v>
+        <v>289</v>
       </c>
       <c r="L2" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -507,7 +507,7 @@
         <v>Passed</v>
       </c>
       <c r="K3">
-        <v>360</v>
+        <v>386</v>
       </c>
       <c r="L3" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -545,7 +545,7 @@
         <v>Passed</v>
       </c>
       <c r="K4">
-        <v>355</v>
+        <v>172</v>
       </c>
       <c r="L4" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -583,7 +583,7 @@
         <v>Passed</v>
       </c>
       <c r="K5">
-        <v>204</v>
+        <v>258</v>
       </c>
       <c r="L5" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -621,7 +621,7 @@
         <v>Passed</v>
       </c>
       <c r="K6">
-        <v>208</v>
+        <v>175</v>
       </c>
       <c r="L6" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -659,7 +659,7 @@
         <v>Passed</v>
       </c>
       <c r="K7">
-        <v>330</v>
+        <v>277</v>
       </c>
       <c r="L7" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -697,7 +697,7 @@
         <v>Passed</v>
       </c>
       <c r="K8">
-        <v>356</v>
+        <v>303</v>
       </c>
       <c r="L8" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -735,7 +735,7 @@
         <v>Passed</v>
       </c>
       <c r="K9">
-        <v>271</v>
+        <v>204</v>
       </c>
       <c r="L9" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -773,7 +773,7 @@
         <v>Passed</v>
       </c>
       <c r="K10">
-        <v>234</v>
+        <v>276</v>
       </c>
       <c r="L10" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -811,7 +811,7 @@
         <v>Passed</v>
       </c>
       <c r="K11">
-        <v>326</v>
+        <v>188</v>
       </c>
       <c r="L11" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -849,7 +849,7 @@
         <v>Passed</v>
       </c>
       <c r="K12">
-        <v>281</v>
+        <v>316</v>
       </c>
       <c r="L12" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -887,7 +887,7 @@
         <v>Passed</v>
       </c>
       <c r="K13">
-        <v>280</v>
+        <v>336</v>
       </c>
       <c r="L13" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -925,7 +925,7 @@
         <v>Passed</v>
       </c>
       <c r="K14">
-        <v>253</v>
+        <v>288</v>
       </c>
       <c r="L14" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -963,7 +963,7 @@
         <v>Passed</v>
       </c>
       <c r="K15">
-        <v>168</v>
+        <v>298</v>
       </c>
       <c r="L15" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1001,7 +1001,7 @@
         <v>Passed</v>
       </c>
       <c r="K16">
-        <v>170</v>
+        <v>319</v>
       </c>
       <c r="L16" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1039,7 +1039,7 @@
         <v>Passed</v>
       </c>
       <c r="K17">
-        <v>199</v>
+        <v>244</v>
       </c>
       <c r="L17" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1077,7 +1077,7 @@
         <v>Passed</v>
       </c>
       <c r="K18">
-        <v>208</v>
+        <v>167</v>
       </c>
       <c r="L18" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1115,7 +1115,7 @@
         <v>Passed</v>
       </c>
       <c r="K19">
-        <v>266</v>
+        <v>345</v>
       </c>
       <c r="L19" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1153,7 +1153,7 @@
         <v>Passed</v>
       </c>
       <c r="K20">
-        <v>343</v>
+        <v>227</v>
       </c>
       <c r="L20" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1191,7 +1191,7 @@
         <v>Passed</v>
       </c>
       <c r="K21">
-        <v>346</v>
+        <v>274</v>
       </c>
       <c r="L21" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1229,7 +1229,7 @@
         <v>Passed</v>
       </c>
       <c r="K22">
-        <v>192</v>
+        <v>220</v>
       </c>
       <c r="L22" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1267,7 +1267,7 @@
         <v>Passed</v>
       </c>
       <c r="K23">
-        <v>225</v>
+        <v>191</v>
       </c>
       <c r="L23" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1305,7 +1305,7 @@
         <v>Passed</v>
       </c>
       <c r="K24">
-        <v>254</v>
+        <v>338</v>
       </c>
       <c r="L24" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1343,7 +1343,7 @@
         <v>Passed</v>
       </c>
       <c r="K25">
-        <v>203</v>
+        <v>181</v>
       </c>
       <c r="L25" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1381,7 +1381,7 @@
         <v>Passed</v>
       </c>
       <c r="K26">
-        <v>183</v>
+        <v>319</v>
       </c>
       <c r="L26" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1419,7 +1419,7 @@
         <v>Passed</v>
       </c>
       <c r="K27">
-        <v>313</v>
+        <v>342</v>
       </c>
       <c r="L27" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1457,7 +1457,7 @@
         <v>Passed</v>
       </c>
       <c r="K28">
-        <v>231</v>
+        <v>370</v>
       </c>
       <c r="L28" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1495,7 +1495,7 @@
         <v>Passed</v>
       </c>
       <c r="K29">
-        <v>366</v>
+        <v>167</v>
       </c>
       <c r="L29" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1533,7 +1533,7 @@
         <v>Passed</v>
       </c>
       <c r="K30">
-        <v>172</v>
+        <v>368</v>
       </c>
       <c r="L30" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1571,7 +1571,7 @@
         <v>Passed</v>
       </c>
       <c r="K31">
-        <v>334</v>
+        <v>210</v>
       </c>
       <c r="L31" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1609,7 +1609,7 @@
         <v>Passed</v>
       </c>
       <c r="K32">
-        <v>231</v>
+        <v>222</v>
       </c>
       <c r="L32" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1647,7 +1647,7 @@
         <v>Passed</v>
       </c>
       <c r="K33">
-        <v>243</v>
+        <v>384</v>
       </c>
       <c r="L33" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1685,7 +1685,7 @@
         <v>Passed</v>
       </c>
       <c r="K34">
-        <v>232</v>
+        <v>162</v>
       </c>
       <c r="L34" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1723,7 +1723,7 @@
         <v>Passed</v>
       </c>
       <c r="K35">
-        <v>225</v>
+        <v>271</v>
       </c>
       <c r="L35" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1761,7 +1761,7 @@
         <v>Passed</v>
       </c>
       <c r="K36">
-        <v>221</v>
+        <v>361</v>
       </c>
       <c r="L36" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1799,7 +1799,7 @@
         <v>Passed</v>
       </c>
       <c r="K37">
-        <v>396</v>
+        <v>237</v>
       </c>
       <c r="L37" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1837,7 +1837,7 @@
         <v>Passed</v>
       </c>
       <c r="K38">
-        <v>381</v>
+        <v>226</v>
       </c>
       <c r="L38" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1875,7 +1875,7 @@
         <v>Passed</v>
       </c>
       <c r="K39">
-        <v>204</v>
+        <v>344</v>
       </c>
       <c r="L39" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1913,7 +1913,7 @@
         <v>Passed</v>
       </c>
       <c r="K40">
-        <v>313</v>
+        <v>326</v>
       </c>
       <c r="L40" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1951,7 +1951,7 @@
         <v>Passed</v>
       </c>
       <c r="K41">
-        <v>276</v>
+        <v>180</v>
       </c>
       <c r="L41" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1989,7 +1989,7 @@
         <v>Passed</v>
       </c>
       <c r="K42">
-        <v>251</v>
+        <v>288</v>
       </c>
       <c r="L42" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2027,7 +2027,7 @@
         <v>Passed</v>
       </c>
       <c r="K43">
-        <v>396</v>
+        <v>267</v>
       </c>
       <c r="L43" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2065,7 +2065,7 @@
         <v>Passed</v>
       </c>
       <c r="K44">
-        <v>370</v>
+        <v>236</v>
       </c>
       <c r="L44" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2103,7 +2103,7 @@
         <v>Passed</v>
       </c>
       <c r="K45">
-        <v>344</v>
+        <v>334</v>
       </c>
       <c r="L45" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2141,7 +2141,7 @@
         <v>Passed</v>
       </c>
       <c r="K46">
-        <v>304</v>
+        <v>376</v>
       </c>
       <c r="L46" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2179,7 +2179,7 @@
         <v>Passed</v>
       </c>
       <c r="K47">
-        <v>336</v>
+        <v>326</v>
       </c>
       <c r="L47" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2217,7 +2217,7 @@
         <v>Passed</v>
       </c>
       <c r="K48">
-        <v>371</v>
+        <v>254</v>
       </c>
       <c r="L48" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2255,7 +2255,7 @@
         <v>Passed</v>
       </c>
       <c r="K49">
-        <v>268</v>
+        <v>290</v>
       </c>
       <c r="L49" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2293,7 +2293,7 @@
         <v>Passed</v>
       </c>
       <c r="K50">
-        <v>279</v>
+        <v>370</v>
       </c>
       <c r="L50" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2331,7 +2331,7 @@
         <v>Passed</v>
       </c>
       <c r="K51">
-        <v>254</v>
+        <v>181</v>
       </c>
       <c r="L51" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2369,7 +2369,7 @@
         <v>Passed</v>
       </c>
       <c r="K52">
-        <v>204</v>
+        <v>324</v>
       </c>
       <c r="L52" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2407,7 +2407,7 @@
         <v>Passed</v>
       </c>
       <c r="K53">
-        <v>185</v>
+        <v>236</v>
       </c>
       <c r="L53" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2445,7 +2445,7 @@
         <v>Passed</v>
       </c>
       <c r="K54">
-        <v>178</v>
+        <v>197</v>
       </c>
       <c r="L54" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2483,7 +2483,7 @@
         <v>Passed</v>
       </c>
       <c r="K55">
-        <v>331</v>
+        <v>270</v>
       </c>
       <c r="L55" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2521,7 +2521,7 @@
         <v>Passed</v>
       </c>
       <c r="K56">
-        <v>222</v>
+        <v>262</v>
       </c>
       <c r="L56" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2559,7 +2559,7 @@
         <v>Passed</v>
       </c>
       <c r="K57">
-        <v>314</v>
+        <v>301</v>
       </c>
       <c r="L57" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2597,7 +2597,7 @@
         <v>Passed</v>
       </c>
       <c r="K58">
-        <v>248</v>
+        <v>374</v>
       </c>
       <c r="L58" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2635,7 +2635,7 @@
         <v>Passed</v>
       </c>
       <c r="K59">
-        <v>279</v>
+        <v>214</v>
       </c>
       <c r="L59" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2673,7 +2673,7 @@
         <v>Passed</v>
       </c>
       <c r="K60">
-        <v>250</v>
+        <v>297</v>
       </c>
       <c r="L60" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2711,7 +2711,7 @@
         <v>Passed</v>
       </c>
       <c r="K61">
-        <v>321</v>
+        <v>253</v>
       </c>
       <c r="L61" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2749,7 +2749,7 @@
         <v>Passed</v>
       </c>
       <c r="K62">
-        <v>187</v>
+        <v>382</v>
       </c>
       <c r="L62" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2787,7 +2787,7 @@
         <v>Passed</v>
       </c>
       <c r="K63">
-        <v>186</v>
+        <v>289</v>
       </c>
       <c r="L63" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2825,7 +2825,7 @@
         <v>Passed</v>
       </c>
       <c r="K64">
-        <v>295</v>
+        <v>375</v>
       </c>
       <c r="L64" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2863,7 +2863,7 @@
         <v>Passed</v>
       </c>
       <c r="K65">
-        <v>192</v>
+        <v>307</v>
       </c>
       <c r="L65" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2901,7 +2901,7 @@
         <v>Passed</v>
       </c>
       <c r="K66">
-        <v>371</v>
+        <v>212</v>
       </c>
       <c r="L66" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2939,7 +2939,7 @@
         <v>Passed</v>
       </c>
       <c r="K67">
-        <v>205</v>
+        <v>308</v>
       </c>
       <c r="L67" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2977,7 +2977,7 @@
         <v>Passed</v>
       </c>
       <c r="K68">
-        <v>364</v>
+        <v>287</v>
       </c>
       <c r="L68" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3015,7 +3015,7 @@
         <v>Passed</v>
       </c>
       <c r="K69">
-        <v>276</v>
+        <v>350</v>
       </c>
       <c r="L69" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3053,7 +3053,7 @@
         <v>Passed</v>
       </c>
       <c r="K70">
-        <v>174</v>
+        <v>316</v>
       </c>
       <c r="L70" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3091,7 +3091,7 @@
         <v>Passed</v>
       </c>
       <c r="K71">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="L71" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3129,7 +3129,7 @@
         <v>Passed</v>
       </c>
       <c r="K72">
-        <v>372</v>
+        <v>348</v>
       </c>
       <c r="L72" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3167,7 +3167,7 @@
         <v>Passed</v>
       </c>
       <c r="K73">
-        <v>270</v>
+        <v>214</v>
       </c>
       <c r="L73" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3205,7 +3205,7 @@
         <v>Passed</v>
       </c>
       <c r="K74">
-        <v>253</v>
+        <v>383</v>
       </c>
       <c r="L74" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3243,7 +3243,7 @@
         <v>Passed</v>
       </c>
       <c r="K75">
-        <v>206</v>
+        <v>255</v>
       </c>
       <c r="L75" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3281,7 +3281,7 @@
         <v>Passed</v>
       </c>
       <c r="K76">
-        <v>160</v>
+        <v>342</v>
       </c>
       <c r="L76" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3319,7 +3319,7 @@
         <v>Passed</v>
       </c>
       <c r="K77">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="L77" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3357,7 +3357,7 @@
         <v>Passed</v>
       </c>
       <c r="K78">
-        <v>389</v>
+        <v>196</v>
       </c>
       <c r="L78" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3395,7 +3395,7 @@
         <v>Passed</v>
       </c>
       <c r="K79">
-        <v>376</v>
+        <v>355</v>
       </c>
       <c r="L79" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3433,7 +3433,7 @@
         <v>Passed</v>
       </c>
       <c r="K80">
-        <v>333</v>
+        <v>278</v>
       </c>
       <c r="L80" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3471,7 +3471,7 @@
         <v>Passed</v>
       </c>
       <c r="K81">
-        <v>236</v>
+        <v>202</v>
       </c>
       <c r="L81" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3509,7 +3509,7 @@
         <v>Passed</v>
       </c>
       <c r="K82">
-        <v>278</v>
+        <v>368</v>
       </c>
       <c r="L82" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3547,7 +3547,7 @@
         <v>Passed</v>
       </c>
       <c r="K83">
-        <v>372</v>
+        <v>176</v>
       </c>
       <c r="L83" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3585,7 +3585,7 @@
         <v>Passed</v>
       </c>
       <c r="K84">
-        <v>264</v>
+        <v>240</v>
       </c>
       <c r="L84" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3623,7 +3623,7 @@
         <v>Passed</v>
       </c>
       <c r="K85">
-        <v>324</v>
+        <v>184</v>
       </c>
       <c r="L85" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3661,7 +3661,7 @@
         <v>Passed</v>
       </c>
       <c r="K86">
-        <v>153</v>
+        <v>367</v>
       </c>
       <c r="L86" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3699,7 +3699,7 @@
         <v>Passed</v>
       </c>
       <c r="K87">
-        <v>314</v>
+        <v>387</v>
       </c>
       <c r="L87" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3737,7 +3737,7 @@
         <v>Passed</v>
       </c>
       <c r="K88">
-        <v>182</v>
+        <v>191</v>
       </c>
       <c r="L88" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3775,7 +3775,7 @@
         <v>Passed</v>
       </c>
       <c r="K89">
-        <v>227</v>
+        <v>273</v>
       </c>
       <c r="L89" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3813,7 +3813,7 @@
         <v>Passed</v>
       </c>
       <c r="K90">
-        <v>353</v>
+        <v>320</v>
       </c>
       <c r="L90" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3851,7 +3851,7 @@
         <v>Passed</v>
       </c>
       <c r="K91">
-        <v>196</v>
+        <v>224</v>
       </c>
       <c r="L91" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3889,7 +3889,7 @@
         <v>Passed</v>
       </c>
       <c r="K92">
-        <v>164</v>
+        <v>376</v>
       </c>
       <c r="L92" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3927,7 +3927,7 @@
         <v>Passed</v>
       </c>
       <c r="K93">
-        <v>388</v>
+        <v>270</v>
       </c>
       <c r="L93" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3965,7 +3965,7 @@
         <v>Passed</v>
       </c>
       <c r="K94">
-        <v>330</v>
+        <v>358</v>
       </c>
       <c r="L94" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4003,7 +4003,7 @@
         <v>Passed</v>
       </c>
       <c r="K95">
-        <v>325</v>
+        <v>396</v>
       </c>
       <c r="L95" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4041,7 +4041,7 @@
         <v>Passed</v>
       </c>
       <c r="K96">
-        <v>379</v>
+        <v>199</v>
       </c>
       <c r="L96" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4079,7 +4079,7 @@
         <v>Passed</v>
       </c>
       <c r="K97">
-        <v>184</v>
+        <v>310</v>
       </c>
       <c r="L97" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4117,7 +4117,7 @@
         <v>Passed</v>
       </c>
       <c r="K98">
-        <v>363</v>
+        <v>209</v>
       </c>
       <c r="L98" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4155,7 +4155,7 @@
         <v>Passed</v>
       </c>
       <c r="K99">
-        <v>367</v>
+        <v>228</v>
       </c>
       <c r="L99" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4193,7 +4193,7 @@
         <v>Passed</v>
       </c>
       <c r="K100">
-        <v>223</v>
+        <v>174</v>
       </c>
       <c r="L100" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4231,7 +4231,7 @@
         <v>Passed</v>
       </c>
       <c r="K101">
-        <v>248</v>
+        <v>339</v>
       </c>
       <c r="L101" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4269,7 +4269,7 @@
         <v>Passed</v>
       </c>
       <c r="K102">
-        <v>378</v>
+        <v>185</v>
       </c>
       <c r="L102" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4307,7 +4307,7 @@
         <v>Passed</v>
       </c>
       <c r="K103">
-        <v>247</v>
+        <v>328</v>
       </c>
       <c r="L103" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4345,7 +4345,7 @@
         <v>Passed</v>
       </c>
       <c r="K104">
-        <v>383</v>
+        <v>332</v>
       </c>
       <c r="L104" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4383,7 +4383,7 @@
         <v>Passed</v>
       </c>
       <c r="K105">
-        <v>303</v>
+        <v>186</v>
       </c>
       <c r="L105" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4421,7 +4421,7 @@
         <v>Passed</v>
       </c>
       <c r="K106">
-        <v>334</v>
+        <v>314</v>
       </c>
       <c r="L106" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4459,7 +4459,7 @@
         <v>Passed</v>
       </c>
       <c r="K107">
-        <v>379</v>
+        <v>361</v>
       </c>
       <c r="L107" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4497,7 +4497,7 @@
         <v>Passed</v>
       </c>
       <c r="K108">
-        <v>366</v>
+        <v>272</v>
       </c>
       <c r="L108" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4535,7 +4535,7 @@
         <v>Passed</v>
       </c>
       <c r="K109">
-        <v>372</v>
+        <v>358</v>
       </c>
       <c r="L109" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4573,7 +4573,7 @@
         <v>Passed</v>
       </c>
       <c r="K110">
-        <v>269</v>
+        <v>216</v>
       </c>
       <c r="L110" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4611,7 +4611,7 @@
         <v>Passed</v>
       </c>
       <c r="K111">
-        <v>279</v>
+        <v>311</v>
       </c>
       <c r="L111" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4649,7 +4649,7 @@
         <v>Passed</v>
       </c>
       <c r="K112">
-        <v>286</v>
+        <v>385</v>
       </c>
       <c r="L112" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4687,7 +4687,7 @@
         <v>Passed</v>
       </c>
       <c r="K113">
-        <v>179</v>
+        <v>193</v>
       </c>
       <c r="L113" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4725,7 +4725,7 @@
         <v>Passed</v>
       </c>
       <c r="K114">
-        <v>193</v>
+        <v>375</v>
       </c>
       <c r="L114" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4763,7 +4763,7 @@
         <v>Passed</v>
       </c>
       <c r="K115">
-        <v>377</v>
+        <v>194</v>
       </c>
       <c r="L115" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4801,7 +4801,7 @@
         <v>Passed</v>
       </c>
       <c r="K116">
-        <v>159</v>
+        <v>223</v>
       </c>
       <c r="L116" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4839,7 +4839,7 @@
         <v>Passed</v>
       </c>
       <c r="K117">
-        <v>264</v>
+        <v>185</v>
       </c>
       <c r="L117" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4877,7 +4877,7 @@
         <v>Passed</v>
       </c>
       <c r="K118">
-        <v>252</v>
+        <v>384</v>
       </c>
       <c r="L118" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4915,7 +4915,7 @@
         <v>Passed</v>
       </c>
       <c r="K119">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="L119" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4953,7 +4953,7 @@
         <v>Passed</v>
       </c>
       <c r="K120">
-        <v>379</v>
+        <v>218</v>
       </c>
       <c r="L120" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4991,7 +4991,7 @@
         <v>Passed</v>
       </c>
       <c r="K121">
-        <v>387</v>
+        <v>317</v>
       </c>
       <c r="L121" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5029,7 +5029,7 @@
         <v>Passed</v>
       </c>
       <c r="K122">
-        <v>210</v>
+        <v>307</v>
       </c>
       <c r="L122" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5067,7 +5067,7 @@
         <v>Passed</v>
       </c>
       <c r="K123">
-        <v>284</v>
+        <v>334</v>
       </c>
       <c r="L123" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5105,7 +5105,7 @@
         <v>Passed</v>
       </c>
       <c r="K124">
-        <v>344</v>
+        <v>172</v>
       </c>
       <c r="L124" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5143,7 +5143,7 @@
         <v>Passed</v>
       </c>
       <c r="K125">
-        <v>269</v>
+        <v>233</v>
       </c>
       <c r="L125" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5181,7 +5181,7 @@
         <v>Passed</v>
       </c>
       <c r="K126">
-        <v>174</v>
+        <v>159</v>
       </c>
       <c r="L126" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5219,7 +5219,7 @@
         <v>Passed</v>
       </c>
       <c r="K127">
-        <v>158</v>
+        <v>363</v>
       </c>
       <c r="L127" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5257,7 +5257,7 @@
         <v>Passed</v>
       </c>
       <c r="K128">
-        <v>294</v>
+        <v>186</v>
       </c>
       <c r="L128" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5295,7 +5295,7 @@
         <v>Passed</v>
       </c>
       <c r="K129">
-        <v>254</v>
+        <v>301</v>
       </c>
       <c r="L129" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5333,7 +5333,7 @@
         <v>Passed</v>
       </c>
       <c r="K130">
-        <v>221</v>
+        <v>252</v>
       </c>
       <c r="L130" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5371,7 +5371,7 @@
         <v>Passed</v>
       </c>
       <c r="K131">
-        <v>245</v>
+        <v>396</v>
       </c>
       <c r="L131" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5409,7 +5409,7 @@
         <v>Passed</v>
       </c>
       <c r="K132">
-        <v>161</v>
+        <v>344</v>
       </c>
       <c r="L132" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5447,7 +5447,7 @@
         <v>Passed</v>
       </c>
       <c r="K133">
-        <v>240</v>
+        <v>206</v>
       </c>
       <c r="L133" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5485,7 +5485,7 @@
         <v>Passed</v>
       </c>
       <c r="K134">
-        <v>244</v>
+        <v>203</v>
       </c>
       <c r="L134" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5523,7 +5523,7 @@
         <v>Passed</v>
       </c>
       <c r="K135">
-        <v>344</v>
+        <v>249</v>
       </c>
       <c r="L135" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5561,7 +5561,7 @@
         <v>Passed</v>
       </c>
       <c r="K136">
-        <v>316</v>
+        <v>387</v>
       </c>
       <c r="L136" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5599,7 +5599,7 @@
         <v>Passed</v>
       </c>
       <c r="K137">
-        <v>396</v>
+        <v>337</v>
       </c>
       <c r="L137" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5637,7 +5637,7 @@
         <v>Passed</v>
       </c>
       <c r="K138">
-        <v>238</v>
+        <v>258</v>
       </c>
       <c r="L138" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5675,7 +5675,7 @@
         <v>Passed</v>
       </c>
       <c r="K139">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="L139" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5713,7 +5713,7 @@
         <v>Passed</v>
       </c>
       <c r="K140">
-        <v>275</v>
+        <v>150</v>
       </c>
       <c r="L140" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5751,7 +5751,7 @@
         <v>Passed</v>
       </c>
       <c r="K141">
-        <v>245</v>
+        <v>185</v>
       </c>
       <c r="L141" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5789,7 +5789,7 @@
         <v>Passed</v>
       </c>
       <c r="K142">
-        <v>268</v>
+        <v>293</v>
       </c>
       <c r="L142" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5827,7 +5827,7 @@
         <v>Passed</v>
       </c>
       <c r="K143">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="L143" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5865,7 +5865,7 @@
         <v>Passed</v>
       </c>
       <c r="K144">
-        <v>201</v>
+        <v>239</v>
       </c>
       <c r="L144" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5903,7 +5903,7 @@
         <v>Passed</v>
       </c>
       <c r="K145">
-        <v>297</v>
+        <v>274</v>
       </c>
       <c r="L145" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5941,7 +5941,7 @@
         <v>Passed</v>
       </c>
       <c r="K146">
-        <v>209</v>
+        <v>352</v>
       </c>
       <c r="L146" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5979,7 +5979,7 @@
         <v>Passed</v>
       </c>
       <c r="K147">
-        <v>215</v>
+        <v>259</v>
       </c>
       <c r="L147" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6017,7 +6017,7 @@
         <v>Passed</v>
       </c>
       <c r="K148">
-        <v>287</v>
+        <v>375</v>
       </c>
       <c r="L148" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6055,7 +6055,7 @@
         <v>Passed</v>
       </c>
       <c r="K149">
-        <v>163</v>
+        <v>242</v>
       </c>
       <c r="L149" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6093,7 +6093,7 @@
         <v>Passed</v>
       </c>
       <c r="K150">
-        <v>271</v>
+        <v>294</v>
       </c>
       <c r="L150" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6131,7 +6131,7 @@
         <v>Passed</v>
       </c>
       <c r="K151">
-        <v>399</v>
+        <v>328</v>
       </c>
       <c r="L151" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6169,7 +6169,7 @@
         <v>Passed</v>
       </c>
       <c r="K152">
-        <v>337</v>
+        <v>379</v>
       </c>
       <c r="L152" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6207,7 +6207,7 @@
         <v>Passed</v>
       </c>
       <c r="K153">
-        <v>357</v>
+        <v>371</v>
       </c>
       <c r="L153" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6245,7 +6245,7 @@
         <v>Passed</v>
       </c>
       <c r="K154">
-        <v>171</v>
+        <v>197</v>
       </c>
       <c r="L154" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6283,7 +6283,7 @@
         <v>Passed</v>
       </c>
       <c r="K155">
-        <v>384</v>
+        <v>158</v>
       </c>
       <c r="L155" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6321,7 +6321,7 @@
         <v>Passed</v>
       </c>
       <c r="K156">
-        <v>258</v>
+        <v>181</v>
       </c>
       <c r="L156" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6359,7 +6359,7 @@
         <v>Passed</v>
       </c>
       <c r="K157">
-        <v>317</v>
+        <v>223</v>
       </c>
       <c r="L157" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6397,7 +6397,7 @@
         <v>Passed</v>
       </c>
       <c r="K158">
-        <v>378</v>
+        <v>315</v>
       </c>
       <c r="L158" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6435,7 +6435,7 @@
         <v>Passed</v>
       </c>
       <c r="K159">
-        <v>394</v>
+        <v>365</v>
       </c>
       <c r="L159" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6473,7 +6473,7 @@
         <v>Passed</v>
       </c>
       <c r="K160">
-        <v>211</v>
+        <v>308</v>
       </c>
       <c r="L160" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6511,7 +6511,7 @@
         <v>Passed</v>
       </c>
       <c r="K161">
-        <v>258</v>
+        <v>388</v>
       </c>
       <c r="L161" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6549,7 +6549,7 @@
         <v>Passed</v>
       </c>
       <c r="K162">
-        <v>180</v>
+        <v>310</v>
       </c>
       <c r="L162" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6587,7 +6587,7 @@
         <v>Passed</v>
       </c>
       <c r="K163">
-        <v>300</v>
+        <v>230</v>
       </c>
       <c r="L163" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6625,7 +6625,7 @@
         <v>Passed</v>
       </c>
       <c r="K164">
-        <v>161</v>
+        <v>296</v>
       </c>
       <c r="L164" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6663,7 +6663,7 @@
         <v>Passed</v>
       </c>
       <c r="K165">
-        <v>207</v>
+        <v>316</v>
       </c>
       <c r="L165" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6701,7 +6701,7 @@
         <v>Passed</v>
       </c>
       <c r="K166">
-        <v>219</v>
+        <v>167</v>
       </c>
       <c r="L166" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6739,7 +6739,7 @@
         <v>Passed</v>
       </c>
       <c r="K167">
-        <v>324</v>
+        <v>377</v>
       </c>
       <c r="L167" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6777,7 +6777,7 @@
         <v>Passed</v>
       </c>
       <c r="K168">
-        <v>368</v>
+        <v>282</v>
       </c>
       <c r="L168" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6815,7 +6815,7 @@
         <v>Passed</v>
       </c>
       <c r="K169">
-        <v>203</v>
+        <v>395</v>
       </c>
       <c r="L169" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6853,7 +6853,7 @@
         <v>Passed</v>
       </c>
       <c r="K170">
-        <v>327</v>
+        <v>161</v>
       </c>
       <c r="L170" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6891,7 +6891,7 @@
         <v>Passed</v>
       </c>
       <c r="K171">
-        <v>154</v>
+        <v>209</v>
       </c>
       <c r="L171" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6929,7 +6929,7 @@
         <v>Passed</v>
       </c>
       <c r="K172">
-        <v>166</v>
+        <v>382</v>
       </c>
       <c r="L172" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6967,7 +6967,7 @@
         <v>Passed</v>
       </c>
       <c r="K173">
-        <v>213</v>
+        <v>221</v>
       </c>
       <c r="L173" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7005,7 +7005,7 @@
         <v>Passed</v>
       </c>
       <c r="K174">
-        <v>256</v>
+        <v>219</v>
       </c>
       <c r="L174" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7043,7 +7043,7 @@
         <v>Passed</v>
       </c>
       <c r="K175">
-        <v>348</v>
+        <v>367</v>
       </c>
       <c r="L175" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7081,7 +7081,7 @@
         <v>Passed</v>
       </c>
       <c r="K176">
-        <v>313</v>
+        <v>301</v>
       </c>
       <c r="L176" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7119,7 +7119,7 @@
         <v>Passed</v>
       </c>
       <c r="K177">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="L177" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7157,7 +7157,7 @@
         <v>Passed</v>
       </c>
       <c r="K178">
-        <v>279</v>
+        <v>340</v>
       </c>
       <c r="L178" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7195,7 +7195,7 @@
         <v>Passed</v>
       </c>
       <c r="K179">
-        <v>396</v>
+        <v>213</v>
       </c>
       <c r="L179" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7233,7 +7233,7 @@
         <v>Passed</v>
       </c>
       <c r="K180">
-        <v>208</v>
+        <v>397</v>
       </c>
       <c r="L180" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7271,7 +7271,7 @@
         <v>Passed</v>
       </c>
       <c r="K181">
-        <v>277</v>
+        <v>350</v>
       </c>
       <c r="L181" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7309,7 +7309,7 @@
         <v>Passed</v>
       </c>
       <c r="K182">
-        <v>275</v>
+        <v>308</v>
       </c>
       <c r="L182" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7347,7 +7347,7 @@
         <v>Passed</v>
       </c>
       <c r="K183">
-        <v>324</v>
+        <v>173</v>
       </c>
       <c r="L183" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7385,7 +7385,7 @@
         <v>Passed</v>
       </c>
       <c r="K184">
-        <v>276</v>
+        <v>300</v>
       </c>
       <c r="L184" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7423,7 +7423,7 @@
         <v>Passed</v>
       </c>
       <c r="K185">
-        <v>173</v>
+        <v>375</v>
       </c>
       <c r="L185" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7461,7 +7461,7 @@
         <v>Passed</v>
       </c>
       <c r="K186">
-        <v>289</v>
+        <v>235</v>
       </c>
       <c r="L186" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7499,7 +7499,7 @@
         <v>Passed</v>
       </c>
       <c r="K187">
-        <v>380</v>
+        <v>188</v>
       </c>
       <c r="L187" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7537,7 +7537,7 @@
         <v>Passed</v>
       </c>
       <c r="K188">
-        <v>266</v>
+        <v>237</v>
       </c>
       <c r="L188" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7575,7 +7575,7 @@
         <v>Passed</v>
       </c>
       <c r="K189">
-        <v>217</v>
+        <v>343</v>
       </c>
       <c r="L189" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7613,7 +7613,7 @@
         <v>Passed</v>
       </c>
       <c r="K190">
-        <v>250</v>
+        <v>356</v>
       </c>
       <c r="L190" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7651,7 +7651,7 @@
         <v>Passed</v>
       </c>
       <c r="K191">
-        <v>321</v>
+        <v>336</v>
       </c>
       <c r="L191" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7689,7 +7689,7 @@
         <v>Passed</v>
       </c>
       <c r="K192">
-        <v>326</v>
+        <v>369</v>
       </c>
       <c r="L192" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7727,7 +7727,7 @@
         <v>Passed</v>
       </c>
       <c r="K193">
-        <v>327</v>
+        <v>371</v>
       </c>
       <c r="L193" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7765,7 +7765,7 @@
         <v>Passed</v>
       </c>
       <c r="K194">
-        <v>225</v>
+        <v>190</v>
       </c>
       <c r="L194" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7803,7 +7803,7 @@
         <v>Passed</v>
       </c>
       <c r="K195">
-        <v>237</v>
+        <v>188</v>
       </c>
       <c r="L195" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7841,7 +7841,7 @@
         <v>Passed</v>
       </c>
       <c r="K196">
-        <v>359</v>
+        <v>344</v>
       </c>
       <c r="L196" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7879,7 +7879,7 @@
         <v>Passed</v>
       </c>
       <c r="K197">
-        <v>310</v>
+        <v>259</v>
       </c>
       <c r="L197" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7917,7 +7917,7 @@
         <v>Passed</v>
       </c>
       <c r="K198">
-        <v>296</v>
+        <v>185</v>
       </c>
       <c r="L198" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7955,7 +7955,7 @@
         <v>Passed</v>
       </c>
       <c r="K199">
-        <v>181</v>
+        <v>322</v>
       </c>
       <c r="L199" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7993,7 +7993,7 @@
         <v>Passed</v>
       </c>
       <c r="K200">
-        <v>331</v>
+        <v>179</v>
       </c>
       <c r="L200" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8031,7 +8031,7 @@
         <v>Passed</v>
       </c>
       <c r="K201">
-        <v>209</v>
+        <v>390</v>
       </c>
       <c r="L201" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8069,7 +8069,7 @@
         <v>Passed</v>
       </c>
       <c r="K202">
-        <v>393</v>
+        <v>381</v>
       </c>
       <c r="L202" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8107,7 +8107,7 @@
         <v>Passed</v>
       </c>
       <c r="K203">
-        <v>314</v>
+        <v>193</v>
       </c>
       <c r="L203" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8145,7 +8145,7 @@
         <v>Passed</v>
       </c>
       <c r="K204">
-        <v>373</v>
+        <v>153</v>
       </c>
       <c r="L204" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8183,7 +8183,7 @@
         <v>Passed</v>
       </c>
       <c r="K205">
-        <v>343</v>
+        <v>347</v>
       </c>
       <c r="L205" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8221,7 +8221,7 @@
         <v>Passed</v>
       </c>
       <c r="K206">
-        <v>176</v>
+        <v>357</v>
       </c>
       <c r="L206" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8259,7 +8259,7 @@
         <v>Passed</v>
       </c>
       <c r="K207">
-        <v>330</v>
+        <v>254</v>
       </c>
       <c r="L207" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8297,7 +8297,7 @@
         <v>Passed</v>
       </c>
       <c r="K208">
-        <v>271</v>
+        <v>322</v>
       </c>
       <c r="L208" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8335,7 +8335,7 @@
         <v>Passed</v>
       </c>
       <c r="K209">
-        <v>223</v>
+        <v>171</v>
       </c>
       <c r="L209" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8373,7 +8373,7 @@
         <v>Passed</v>
       </c>
       <c r="K210">
-        <v>197</v>
+        <v>327</v>
       </c>
       <c r="L210" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8411,7 +8411,7 @@
         <v>Passed</v>
       </c>
       <c r="K211">
-        <v>325</v>
+        <v>169</v>
       </c>
       <c r="L211" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8449,7 +8449,7 @@
         <v>Passed</v>
       </c>
       <c r="K212">
-        <v>227</v>
+        <v>274</v>
       </c>
       <c r="L212" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8487,7 +8487,7 @@
         <v>Passed</v>
       </c>
       <c r="K213">
-        <v>294</v>
+        <v>247</v>
       </c>
       <c r="L213" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8525,7 +8525,7 @@
         <v>Passed</v>
       </c>
       <c r="K214">
-        <v>189</v>
+        <v>283</v>
       </c>
       <c r="L214" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8563,7 +8563,7 @@
         <v>Passed</v>
       </c>
       <c r="K215">
-        <v>234</v>
+        <v>190</v>
       </c>
       <c r="L215" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8601,7 +8601,7 @@
         <v>Passed</v>
       </c>
       <c r="K216">
-        <v>260</v>
+        <v>320</v>
       </c>
       <c r="L216" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8639,7 +8639,7 @@
         <v>Passed</v>
       </c>
       <c r="K217">
-        <v>214</v>
+        <v>395</v>
       </c>
       <c r="L217" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8677,7 +8677,7 @@
         <v>Passed</v>
       </c>
       <c r="K218">
-        <v>293</v>
+        <v>230</v>
       </c>
       <c r="L218" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8715,7 +8715,7 @@
         <v>Passed</v>
       </c>
       <c r="K219">
-        <v>320</v>
+        <v>288</v>
       </c>
       <c r="L219" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8753,7 +8753,7 @@
         <v>Passed</v>
       </c>
       <c r="K220">
-        <v>333</v>
+        <v>226</v>
       </c>
       <c r="L220" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8791,7 +8791,7 @@
         <v>Passed</v>
       </c>
       <c r="K221">
-        <v>320</v>
+        <v>335</v>
       </c>
       <c r="L221" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8829,7 +8829,7 @@
         <v>Passed</v>
       </c>
       <c r="K222">
-        <v>309</v>
+        <v>193</v>
       </c>
       <c r="L222" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8867,7 +8867,7 @@
         <v>Passed</v>
       </c>
       <c r="K223">
-        <v>250</v>
+        <v>360</v>
       </c>
       <c r="L223" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8905,7 +8905,7 @@
         <v>Passed</v>
       </c>
       <c r="K224">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="L224" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8943,7 +8943,7 @@
         <v>Passed</v>
       </c>
       <c r="K225">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="L225" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8981,7 +8981,7 @@
         <v>Passed</v>
       </c>
       <c r="K226">
-        <v>203</v>
+        <v>368</v>
       </c>
       <c r="L226" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9019,7 +9019,7 @@
         <v>Passed</v>
       </c>
       <c r="K227">
-        <v>197</v>
+        <v>188</v>
       </c>
       <c r="L227" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9057,7 +9057,7 @@
         <v>Passed</v>
       </c>
       <c r="K228">
-        <v>178</v>
+        <v>321</v>
       </c>
       <c r="L228" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9095,7 +9095,7 @@
         <v>Passed</v>
       </c>
       <c r="K229">
-        <v>207</v>
+        <v>250</v>
       </c>
       <c r="L229" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9133,7 +9133,7 @@
         <v>Passed</v>
       </c>
       <c r="K230">
-        <v>229</v>
+        <v>296</v>
       </c>
       <c r="L230" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9171,7 +9171,7 @@
         <v>Passed</v>
       </c>
       <c r="K231">
-        <v>306</v>
+        <v>275</v>
       </c>
       <c r="L231" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9209,7 +9209,7 @@
         <v>Passed</v>
       </c>
       <c r="K232">
-        <v>178</v>
+        <v>232</v>
       </c>
       <c r="L232" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9247,7 +9247,7 @@
         <v>Passed</v>
       </c>
       <c r="K233">
-        <v>227</v>
+        <v>349</v>
       </c>
       <c r="L233" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9285,7 +9285,7 @@
         <v>Passed</v>
       </c>
       <c r="K234">
-        <v>360</v>
+        <v>154</v>
       </c>
       <c r="L234" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9323,7 +9323,7 @@
         <v>Passed</v>
       </c>
       <c r="K235">
-        <v>323</v>
+        <v>164</v>
       </c>
       <c r="L235" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9361,7 +9361,7 @@
         <v>Passed</v>
       </c>
       <c r="K236">
-        <v>186</v>
+        <v>314</v>
       </c>
       <c r="L236" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9399,7 +9399,7 @@
         <v>Passed</v>
       </c>
       <c r="K237">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="L237" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9437,7 +9437,7 @@
         <v>Passed</v>
       </c>
       <c r="K238">
-        <v>211</v>
+        <v>326</v>
       </c>
       <c r="L238" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9475,7 +9475,7 @@
         <v>Passed</v>
       </c>
       <c r="K239">
-        <v>218</v>
+        <v>357</v>
       </c>
       <c r="L239" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9513,7 +9513,7 @@
         <v>Passed</v>
       </c>
       <c r="K240">
-        <v>181</v>
+        <v>194</v>
       </c>
       <c r="L240" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9551,7 +9551,7 @@
         <v>Passed</v>
       </c>
       <c r="K241">
-        <v>380</v>
+        <v>233</v>
       </c>
       <c r="L241" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9589,7 +9589,7 @@
         <v>Passed</v>
       </c>
       <c r="K242">
-        <v>241</v>
+        <v>223</v>
       </c>
       <c r="L242" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9627,7 +9627,7 @@
         <v>Passed</v>
       </c>
       <c r="K243">
-        <v>243</v>
+        <v>211</v>
       </c>
       <c r="L243" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9665,7 +9665,7 @@
         <v>Passed</v>
       </c>
       <c r="K244">
-        <v>191</v>
+        <v>246</v>
       </c>
       <c r="L244" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9703,7 +9703,7 @@
         <v>Passed</v>
       </c>
       <c r="K245">
-        <v>190</v>
+        <v>330</v>
       </c>
       <c r="L245" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9741,7 +9741,7 @@
         <v>Passed</v>
       </c>
       <c r="K246">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="L246" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9779,7 +9779,7 @@
         <v>Passed</v>
       </c>
       <c r="K247">
-        <v>398</v>
+        <v>378</v>
       </c>
       <c r="L247" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9817,7 +9817,7 @@
         <v>Passed</v>
       </c>
       <c r="K248">
-        <v>326</v>
+        <v>389</v>
       </c>
       <c r="L248" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9855,7 +9855,7 @@
         <v>Passed</v>
       </c>
       <c r="K249">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="L249" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9893,7 +9893,7 @@
         <v>Passed</v>
       </c>
       <c r="K250">
-        <v>285</v>
+        <v>344</v>
       </c>
       <c r="L250" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9931,7 +9931,7 @@
         <v>Passed</v>
       </c>
       <c r="K251">
-        <v>281</v>
+        <v>325</v>
       </c>
       <c r="L251" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9969,7 +9969,7 @@
         <v>Passed</v>
       </c>
       <c r="K252">
-        <v>242</v>
+        <v>206</v>
       </c>
       <c r="L252" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10007,7 +10007,7 @@
         <v>Passed</v>
       </c>
       <c r="K253">
-        <v>318</v>
+        <v>377</v>
       </c>
       <c r="L253" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10045,7 +10045,7 @@
         <v>Passed</v>
       </c>
       <c r="K254">
-        <v>337</v>
+        <v>230</v>
       </c>
       <c r="L254" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10083,7 +10083,7 @@
         <v>Passed</v>
       </c>
       <c r="K255">
-        <v>227</v>
+        <v>203</v>
       </c>
       <c r="L255" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10121,7 +10121,7 @@
         <v>Passed</v>
       </c>
       <c r="K256">
-        <v>386</v>
+        <v>271</v>
       </c>
       <c r="L256" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10159,7 +10159,7 @@
         <v>Passed</v>
       </c>
       <c r="K257">
-        <v>208</v>
+        <v>192</v>
       </c>
       <c r="L257" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10197,7 +10197,7 @@
         <v>Passed</v>
       </c>
       <c r="K258">
-        <v>185</v>
+        <v>276</v>
       </c>
       <c r="L258" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10235,7 +10235,7 @@
         <v>Passed</v>
       </c>
       <c r="K259">
-        <v>251</v>
+        <v>233</v>
       </c>
       <c r="L259" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10273,7 +10273,7 @@
         <v>Passed</v>
       </c>
       <c r="K260">
-        <v>362</v>
+        <v>233</v>
       </c>
       <c r="L260" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10311,7 +10311,7 @@
         <v>Passed</v>
       </c>
       <c r="K261">
-        <v>259</v>
+        <v>355</v>
       </c>
       <c r="L261" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10349,7 +10349,7 @@
         <v>Passed</v>
       </c>
       <c r="K262">
-        <v>247</v>
+        <v>294</v>
       </c>
       <c r="L262" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10387,7 +10387,7 @@
         <v>Passed</v>
       </c>
       <c r="K263">
-        <v>230</v>
+        <v>201</v>
       </c>
       <c r="L263" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10425,7 +10425,7 @@
         <v>Passed</v>
       </c>
       <c r="K264">
-        <v>394</v>
+        <v>313</v>
       </c>
       <c r="L264" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10463,7 +10463,7 @@
         <v>Passed</v>
       </c>
       <c r="K265">
-        <v>263</v>
+        <v>308</v>
       </c>
       <c r="L265" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10501,7 +10501,7 @@
         <v>Passed</v>
       </c>
       <c r="K266">
-        <v>359</v>
+        <v>295</v>
       </c>
       <c r="L266" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10539,7 +10539,7 @@
         <v>Passed</v>
       </c>
       <c r="K267">
-        <v>321</v>
+        <v>188</v>
       </c>
       <c r="L267" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10577,7 +10577,7 @@
         <v>Passed</v>
       </c>
       <c r="K268">
-        <v>211</v>
+        <v>199</v>
       </c>
       <c r="L268" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10615,7 +10615,7 @@
         <v>Passed</v>
       </c>
       <c r="K269">
-        <v>191</v>
+        <v>210</v>
       </c>
       <c r="L269" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10653,7 +10653,7 @@
         <v>Passed</v>
       </c>
       <c r="K270">
-        <v>388</v>
+        <v>190</v>
       </c>
       <c r="L270" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10691,7 +10691,7 @@
         <v>Passed</v>
       </c>
       <c r="K271">
-        <v>161</v>
+        <v>363</v>
       </c>
       <c r="L271" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10729,7 +10729,7 @@
         <v>Passed</v>
       </c>
       <c r="K272">
-        <v>229</v>
+        <v>262</v>
       </c>
       <c r="L272" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10767,7 +10767,7 @@
         <v>Passed</v>
       </c>
       <c r="K273">
-        <v>344</v>
+        <v>384</v>
       </c>
       <c r="L273" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10805,7 +10805,7 @@
         <v>Passed</v>
       </c>
       <c r="K274">
-        <v>197</v>
+        <v>166</v>
       </c>
       <c r="L274" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10843,7 +10843,7 @@
         <v>Passed</v>
       </c>
       <c r="K275">
-        <v>272</v>
+        <v>153</v>
       </c>
       <c r="L275" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10881,7 +10881,7 @@
         <v>Passed</v>
       </c>
       <c r="K276">
-        <v>172</v>
+        <v>368</v>
       </c>
       <c r="L276" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10919,7 +10919,7 @@
         <v>Passed</v>
       </c>
       <c r="K277">
-        <v>171</v>
+        <v>332</v>
       </c>
       <c r="L277" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10957,7 +10957,7 @@
         <v>Passed</v>
       </c>
       <c r="K278">
-        <v>391</v>
+        <v>251</v>
       </c>
       <c r="L278" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10995,7 +10995,7 @@
         <v>Passed</v>
       </c>
       <c r="K279">
-        <v>230</v>
+        <v>203</v>
       </c>
       <c r="L279" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11033,7 +11033,7 @@
         <v>Passed</v>
       </c>
       <c r="K280">
-        <v>154</v>
+        <v>211</v>
       </c>
       <c r="L280" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11071,7 +11071,7 @@
         <v>Passed</v>
       </c>
       <c r="K281">
-        <v>326</v>
+        <v>235</v>
       </c>
       <c r="L281" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11109,7 +11109,7 @@
         <v>Passed</v>
       </c>
       <c r="K282">
-        <v>296</v>
+        <v>196</v>
       </c>
       <c r="L282" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11147,7 +11147,7 @@
         <v>Passed</v>
       </c>
       <c r="K283">
-        <v>259</v>
+        <v>250</v>
       </c>
       <c r="L283" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11185,7 +11185,7 @@
         <v>Passed</v>
       </c>
       <c r="K284">
-        <v>213</v>
+        <v>162</v>
       </c>
       <c r="L284" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11223,7 +11223,7 @@
         <v>Passed</v>
       </c>
       <c r="K285">
-        <v>193</v>
+        <v>359</v>
       </c>
       <c r="L285" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11261,7 +11261,7 @@
         <v>Passed</v>
       </c>
       <c r="K286">
-        <v>367</v>
+        <v>394</v>
       </c>
       <c r="L286" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11299,7 +11299,7 @@
         <v>Passed</v>
       </c>
       <c r="K287">
-        <v>243</v>
+        <v>204</v>
       </c>
       <c r="L287" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11337,7 +11337,7 @@
         <v>Passed</v>
       </c>
       <c r="K288">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="L288" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11375,7 +11375,7 @@
         <v>Passed</v>
       </c>
       <c r="K289">
-        <v>309</v>
+        <v>195</v>
       </c>
       <c r="L289" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11413,7 +11413,7 @@
         <v>Passed</v>
       </c>
       <c r="K290">
-        <v>287</v>
+        <v>158</v>
       </c>
       <c r="L290" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11451,7 +11451,7 @@
         <v>Passed</v>
       </c>
       <c r="K291">
-        <v>389</v>
+        <v>231</v>
       </c>
       <c r="L291" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11489,7 +11489,7 @@
         <v>Passed</v>
       </c>
       <c r="K292">
-        <v>208</v>
+        <v>163</v>
       </c>
       <c r="L292" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11527,7 +11527,7 @@
         <v>Passed</v>
       </c>
       <c r="K293">
-        <v>333</v>
+        <v>302</v>
       </c>
       <c r="L293" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11565,7 +11565,7 @@
         <v>Passed</v>
       </c>
       <c r="K294">
-        <v>313</v>
+        <v>358</v>
       </c>
       <c r="L294" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11603,7 +11603,7 @@
         <v>Passed</v>
       </c>
       <c r="K295">
-        <v>249</v>
+        <v>205</v>
       </c>
       <c r="L295" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11641,7 +11641,7 @@
         <v>Passed</v>
       </c>
       <c r="K296">
-        <v>214</v>
+        <v>298</v>
       </c>
       <c r="L296" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11679,7 +11679,7 @@
         <v>Passed</v>
       </c>
       <c r="K297">
-        <v>244</v>
+        <v>153</v>
       </c>
       <c r="L297" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11717,7 +11717,7 @@
         <v>Passed</v>
       </c>
       <c r="K298">
-        <v>394</v>
+        <v>291</v>
       </c>
       <c r="L298" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11755,7 +11755,7 @@
         <v>Passed</v>
       </c>
       <c r="K299">
-        <v>354</v>
+        <v>199</v>
       </c>
       <c r="L299" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11793,7 +11793,7 @@
         <v>Passed</v>
       </c>
       <c r="K300">
-        <v>398</v>
+        <v>262</v>
       </c>
       <c r="L300" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11831,7 +11831,7 @@
         <v>Passed</v>
       </c>
       <c r="K301">
-        <v>161</v>
+        <v>205</v>
       </c>
       <c r="L301" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>

</xml_diff>

<commit_message>
feat: add interactive Uber booking form with full-width web layout and space-dark theme
</commit_message>
<xml_diff>
--- a/EventSphere_Appium_Mobile_300_Report.xlsx
+++ b/EventSphere_Appium_Mobile_300_Report.xlsx
@@ -469,7 +469,7 @@
         <v>Passed</v>
       </c>
       <c r="K2">
-        <v>289</v>
+        <v>313</v>
       </c>
       <c r="L2" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -507,7 +507,7 @@
         <v>Passed</v>
       </c>
       <c r="K3">
-        <v>386</v>
+        <v>225</v>
       </c>
       <c r="L3" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -545,7 +545,7 @@
         <v>Passed</v>
       </c>
       <c r="K4">
-        <v>172</v>
+        <v>183</v>
       </c>
       <c r="L4" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -583,7 +583,7 @@
         <v>Passed</v>
       </c>
       <c r="K5">
-        <v>258</v>
+        <v>248</v>
       </c>
       <c r="L5" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -621,7 +621,7 @@
         <v>Passed</v>
       </c>
       <c r="K6">
-        <v>175</v>
+        <v>155</v>
       </c>
       <c r="L6" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -659,7 +659,7 @@
         <v>Passed</v>
       </c>
       <c r="K7">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="L7" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -697,7 +697,7 @@
         <v>Passed</v>
       </c>
       <c r="K8">
-        <v>303</v>
+        <v>165</v>
       </c>
       <c r="L8" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -735,7 +735,7 @@
         <v>Passed</v>
       </c>
       <c r="K9">
-        <v>204</v>
+        <v>354</v>
       </c>
       <c r="L9" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -773,7 +773,7 @@
         <v>Passed</v>
       </c>
       <c r="K10">
-        <v>276</v>
+        <v>251</v>
       </c>
       <c r="L10" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -811,7 +811,7 @@
         <v>Passed</v>
       </c>
       <c r="K11">
-        <v>188</v>
+        <v>233</v>
       </c>
       <c r="L11" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -849,7 +849,7 @@
         <v>Passed</v>
       </c>
       <c r="K12">
-        <v>316</v>
+        <v>164</v>
       </c>
       <c r="L12" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -887,7 +887,7 @@
         <v>Passed</v>
       </c>
       <c r="K13">
-        <v>336</v>
+        <v>289</v>
       </c>
       <c r="L13" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -925,7 +925,7 @@
         <v>Passed</v>
       </c>
       <c r="K14">
-        <v>288</v>
+        <v>156</v>
       </c>
       <c r="L14" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -963,7 +963,7 @@
         <v>Passed</v>
       </c>
       <c r="K15">
-        <v>298</v>
+        <v>365</v>
       </c>
       <c r="L15" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1001,7 +1001,7 @@
         <v>Passed</v>
       </c>
       <c r="K16">
-        <v>319</v>
+        <v>302</v>
       </c>
       <c r="L16" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1039,7 +1039,7 @@
         <v>Passed</v>
       </c>
       <c r="K17">
-        <v>244</v>
+        <v>327</v>
       </c>
       <c r="L17" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1077,7 +1077,7 @@
         <v>Passed</v>
       </c>
       <c r="K18">
-        <v>167</v>
+        <v>352</v>
       </c>
       <c r="L18" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1115,7 +1115,7 @@
         <v>Passed</v>
       </c>
       <c r="K19">
-        <v>345</v>
+        <v>203</v>
       </c>
       <c r="L19" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1153,7 +1153,7 @@
         <v>Passed</v>
       </c>
       <c r="K20">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="L20" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1191,7 +1191,7 @@
         <v>Passed</v>
       </c>
       <c r="K21">
-        <v>274</v>
+        <v>325</v>
       </c>
       <c r="L21" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1229,7 +1229,7 @@
         <v>Passed</v>
       </c>
       <c r="K22">
-        <v>220</v>
+        <v>171</v>
       </c>
       <c r="L22" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1267,7 +1267,7 @@
         <v>Passed</v>
       </c>
       <c r="K23">
-        <v>191</v>
+        <v>314</v>
       </c>
       <c r="L23" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1305,7 +1305,7 @@
         <v>Passed</v>
       </c>
       <c r="K24">
-        <v>338</v>
+        <v>225</v>
       </c>
       <c r="L24" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1343,7 +1343,7 @@
         <v>Passed</v>
       </c>
       <c r="K25">
-        <v>181</v>
+        <v>211</v>
       </c>
       <c r="L25" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1381,7 +1381,7 @@
         <v>Passed</v>
       </c>
       <c r="K26">
-        <v>319</v>
+        <v>215</v>
       </c>
       <c r="L26" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1419,7 +1419,7 @@
         <v>Passed</v>
       </c>
       <c r="K27">
-        <v>342</v>
+        <v>310</v>
       </c>
       <c r="L27" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1457,7 +1457,7 @@
         <v>Passed</v>
       </c>
       <c r="K28">
-        <v>370</v>
+        <v>227</v>
       </c>
       <c r="L28" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1495,7 +1495,7 @@
         <v>Passed</v>
       </c>
       <c r="K29">
-        <v>167</v>
+        <v>330</v>
       </c>
       <c r="L29" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1533,7 +1533,7 @@
         <v>Passed</v>
       </c>
       <c r="K30">
-        <v>368</v>
+        <v>169</v>
       </c>
       <c r="L30" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1571,7 +1571,7 @@
         <v>Passed</v>
       </c>
       <c r="K31">
-        <v>210</v>
+        <v>178</v>
       </c>
       <c r="L31" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1609,7 +1609,7 @@
         <v>Passed</v>
       </c>
       <c r="K32">
-        <v>222</v>
+        <v>207</v>
       </c>
       <c r="L32" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1647,7 +1647,7 @@
         <v>Passed</v>
       </c>
       <c r="K33">
-        <v>384</v>
+        <v>354</v>
       </c>
       <c r="L33" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1685,7 +1685,7 @@
         <v>Passed</v>
       </c>
       <c r="K34">
-        <v>162</v>
+        <v>215</v>
       </c>
       <c r="L34" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1723,7 +1723,7 @@
         <v>Passed</v>
       </c>
       <c r="K35">
-        <v>271</v>
+        <v>158</v>
       </c>
       <c r="L35" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1761,7 +1761,7 @@
         <v>Passed</v>
       </c>
       <c r="K36">
-        <v>361</v>
+        <v>287</v>
       </c>
       <c r="L36" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1799,7 +1799,7 @@
         <v>Passed</v>
       </c>
       <c r="K37">
-        <v>237</v>
+        <v>162</v>
       </c>
       <c r="L37" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1837,7 +1837,7 @@
         <v>Passed</v>
       </c>
       <c r="K38">
-        <v>226</v>
+        <v>282</v>
       </c>
       <c r="L38" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1875,7 +1875,7 @@
         <v>Passed</v>
       </c>
       <c r="K39">
-        <v>344</v>
+        <v>274</v>
       </c>
       <c r="L39" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1913,7 +1913,7 @@
         <v>Passed</v>
       </c>
       <c r="K40">
-        <v>326</v>
+        <v>357</v>
       </c>
       <c r="L40" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1951,7 +1951,7 @@
         <v>Passed</v>
       </c>
       <c r="K41">
-        <v>180</v>
+        <v>295</v>
       </c>
       <c r="L41" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1989,7 +1989,7 @@
         <v>Passed</v>
       </c>
       <c r="K42">
-        <v>288</v>
+        <v>377</v>
       </c>
       <c r="L42" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2027,7 +2027,7 @@
         <v>Passed</v>
       </c>
       <c r="K43">
-        <v>267</v>
+        <v>251</v>
       </c>
       <c r="L43" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2065,7 +2065,7 @@
         <v>Passed</v>
       </c>
       <c r="K44">
-        <v>236</v>
+        <v>334</v>
       </c>
       <c r="L44" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2103,7 +2103,7 @@
         <v>Passed</v>
       </c>
       <c r="K45">
-        <v>334</v>
+        <v>296</v>
       </c>
       <c r="L45" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2141,7 +2141,7 @@
         <v>Passed</v>
       </c>
       <c r="K46">
-        <v>376</v>
+        <v>269</v>
       </c>
       <c r="L46" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2179,7 +2179,7 @@
         <v>Passed</v>
       </c>
       <c r="K47">
-        <v>326</v>
+        <v>334</v>
       </c>
       <c r="L47" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2217,7 +2217,7 @@
         <v>Passed</v>
       </c>
       <c r="K48">
-        <v>254</v>
+        <v>162</v>
       </c>
       <c r="L48" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2255,7 +2255,7 @@
         <v>Passed</v>
       </c>
       <c r="K49">
-        <v>290</v>
+        <v>310</v>
       </c>
       <c r="L49" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2293,7 +2293,7 @@
         <v>Passed</v>
       </c>
       <c r="K50">
-        <v>370</v>
+        <v>243</v>
       </c>
       <c r="L50" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2331,7 +2331,7 @@
         <v>Passed</v>
       </c>
       <c r="K51">
-        <v>181</v>
+        <v>173</v>
       </c>
       <c r="L51" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2369,7 +2369,7 @@
         <v>Passed</v>
       </c>
       <c r="K52">
-        <v>324</v>
+        <v>348</v>
       </c>
       <c r="L52" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2445,7 +2445,7 @@
         <v>Passed</v>
       </c>
       <c r="K54">
-        <v>197</v>
+        <v>378</v>
       </c>
       <c r="L54" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2483,7 +2483,7 @@
         <v>Passed</v>
       </c>
       <c r="K55">
-        <v>270</v>
+        <v>379</v>
       </c>
       <c r="L55" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2521,7 +2521,7 @@
         <v>Passed</v>
       </c>
       <c r="K56">
-        <v>262</v>
+        <v>228</v>
       </c>
       <c r="L56" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2559,7 +2559,7 @@
         <v>Passed</v>
       </c>
       <c r="K57">
-        <v>301</v>
+        <v>321</v>
       </c>
       <c r="L57" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2597,7 +2597,7 @@
         <v>Passed</v>
       </c>
       <c r="K58">
-        <v>374</v>
+        <v>341</v>
       </c>
       <c r="L58" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2635,7 +2635,7 @@
         <v>Passed</v>
       </c>
       <c r="K59">
-        <v>214</v>
+        <v>343</v>
       </c>
       <c r="L59" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2673,7 +2673,7 @@
         <v>Passed</v>
       </c>
       <c r="K60">
-        <v>297</v>
+        <v>312</v>
       </c>
       <c r="L60" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2711,7 +2711,7 @@
         <v>Passed</v>
       </c>
       <c r="K61">
-        <v>253</v>
+        <v>279</v>
       </c>
       <c r="L61" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2749,7 +2749,7 @@
         <v>Passed</v>
       </c>
       <c r="K62">
-        <v>382</v>
+        <v>231</v>
       </c>
       <c r="L62" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2787,7 +2787,7 @@
         <v>Passed</v>
       </c>
       <c r="K63">
-        <v>289</v>
+        <v>152</v>
       </c>
       <c r="L63" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2825,7 +2825,7 @@
         <v>Passed</v>
       </c>
       <c r="K64">
-        <v>375</v>
+        <v>265</v>
       </c>
       <c r="L64" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2863,7 +2863,7 @@
         <v>Passed</v>
       </c>
       <c r="K65">
-        <v>307</v>
+        <v>236</v>
       </c>
       <c r="L65" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2901,7 +2901,7 @@
         <v>Passed</v>
       </c>
       <c r="K66">
-        <v>212</v>
+        <v>345</v>
       </c>
       <c r="L66" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2939,7 +2939,7 @@
         <v>Passed</v>
       </c>
       <c r="K67">
-        <v>308</v>
+        <v>321</v>
       </c>
       <c r="L67" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2977,7 +2977,7 @@
         <v>Passed</v>
       </c>
       <c r="K68">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="L68" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3015,7 +3015,7 @@
         <v>Passed</v>
       </c>
       <c r="K69">
-        <v>350</v>
+        <v>241</v>
       </c>
       <c r="L69" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3053,7 +3053,7 @@
         <v>Passed</v>
       </c>
       <c r="K70">
-        <v>316</v>
+        <v>237</v>
       </c>
       <c r="L70" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3091,7 +3091,7 @@
         <v>Passed</v>
       </c>
       <c r="K71">
-        <v>310</v>
+        <v>173</v>
       </c>
       <c r="L71" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3129,7 +3129,7 @@
         <v>Passed</v>
       </c>
       <c r="K72">
-        <v>348</v>
+        <v>321</v>
       </c>
       <c r="L72" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3167,7 +3167,7 @@
         <v>Passed</v>
       </c>
       <c r="K73">
-        <v>214</v>
+        <v>277</v>
       </c>
       <c r="L73" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3205,7 +3205,7 @@
         <v>Passed</v>
       </c>
       <c r="K74">
-        <v>383</v>
+        <v>214</v>
       </c>
       <c r="L74" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3243,7 +3243,7 @@
         <v>Passed</v>
       </c>
       <c r="K75">
-        <v>255</v>
+        <v>179</v>
       </c>
       <c r="L75" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3281,7 +3281,7 @@
         <v>Passed</v>
       </c>
       <c r="K76">
-        <v>342</v>
+        <v>207</v>
       </c>
       <c r="L76" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3319,7 +3319,7 @@
         <v>Passed</v>
       </c>
       <c r="K77">
-        <v>201</v>
+        <v>399</v>
       </c>
       <c r="L77" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3357,7 +3357,7 @@
         <v>Passed</v>
       </c>
       <c r="K78">
-        <v>196</v>
+        <v>274</v>
       </c>
       <c r="L78" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3395,7 +3395,7 @@
         <v>Passed</v>
       </c>
       <c r="K79">
-        <v>355</v>
+        <v>345</v>
       </c>
       <c r="L79" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3433,7 +3433,7 @@
         <v>Passed</v>
       </c>
       <c r="K80">
-        <v>278</v>
+        <v>203</v>
       </c>
       <c r="L80" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3471,7 +3471,7 @@
         <v>Passed</v>
       </c>
       <c r="K81">
-        <v>202</v>
+        <v>232</v>
       </c>
       <c r="L81" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3509,7 +3509,7 @@
         <v>Passed</v>
       </c>
       <c r="K82">
-        <v>368</v>
+        <v>195</v>
       </c>
       <c r="L82" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3547,7 +3547,7 @@
         <v>Passed</v>
       </c>
       <c r="K83">
-        <v>176</v>
+        <v>388</v>
       </c>
       <c r="L83" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3585,7 +3585,7 @@
         <v>Passed</v>
       </c>
       <c r="K84">
-        <v>240</v>
+        <v>164</v>
       </c>
       <c r="L84" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3623,7 +3623,7 @@
         <v>Passed</v>
       </c>
       <c r="K85">
-        <v>184</v>
+        <v>385</v>
       </c>
       <c r="L85" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3661,7 +3661,7 @@
         <v>Passed</v>
       </c>
       <c r="K86">
-        <v>367</v>
+        <v>388</v>
       </c>
       <c r="L86" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3699,7 +3699,7 @@
         <v>Passed</v>
       </c>
       <c r="K87">
-        <v>387</v>
+        <v>380</v>
       </c>
       <c r="L87" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3737,7 +3737,7 @@
         <v>Passed</v>
       </c>
       <c r="K88">
-        <v>191</v>
+        <v>390</v>
       </c>
       <c r="L88" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3775,7 +3775,7 @@
         <v>Passed</v>
       </c>
       <c r="K89">
-        <v>273</v>
+        <v>173</v>
       </c>
       <c r="L89" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3813,7 +3813,7 @@
         <v>Passed</v>
       </c>
       <c r="K90">
-        <v>320</v>
+        <v>244</v>
       </c>
       <c r="L90" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3851,7 +3851,7 @@
         <v>Passed</v>
       </c>
       <c r="K91">
-        <v>224</v>
+        <v>375</v>
       </c>
       <c r="L91" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3889,7 +3889,7 @@
         <v>Passed</v>
       </c>
       <c r="K92">
-        <v>376</v>
+        <v>323</v>
       </c>
       <c r="L92" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3927,7 +3927,7 @@
         <v>Passed</v>
       </c>
       <c r="K93">
-        <v>270</v>
+        <v>171</v>
       </c>
       <c r="L93" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3965,7 +3965,7 @@
         <v>Passed</v>
       </c>
       <c r="K94">
-        <v>358</v>
+        <v>212</v>
       </c>
       <c r="L94" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4003,7 +4003,7 @@
         <v>Passed</v>
       </c>
       <c r="K95">
-        <v>396</v>
+        <v>314</v>
       </c>
       <c r="L95" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4041,7 +4041,7 @@
         <v>Passed</v>
       </c>
       <c r="K96">
-        <v>199</v>
+        <v>214</v>
       </c>
       <c r="L96" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4079,7 +4079,7 @@
         <v>Passed</v>
       </c>
       <c r="K97">
-        <v>310</v>
+        <v>224</v>
       </c>
       <c r="L97" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4117,7 +4117,7 @@
         <v>Passed</v>
       </c>
       <c r="K98">
-        <v>209</v>
+        <v>313</v>
       </c>
       <c r="L98" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4155,7 +4155,7 @@
         <v>Passed</v>
       </c>
       <c r="K99">
-        <v>228</v>
+        <v>289</v>
       </c>
       <c r="L99" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4193,7 +4193,7 @@
         <v>Passed</v>
       </c>
       <c r="K100">
-        <v>174</v>
+        <v>287</v>
       </c>
       <c r="L100" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4231,7 +4231,7 @@
         <v>Passed</v>
       </c>
       <c r="K101">
-        <v>339</v>
+        <v>187</v>
       </c>
       <c r="L101" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4269,7 +4269,7 @@
         <v>Passed</v>
       </c>
       <c r="K102">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="L102" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4307,7 +4307,7 @@
         <v>Passed</v>
       </c>
       <c r="K103">
-        <v>328</v>
+        <v>279</v>
       </c>
       <c r="L103" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4345,7 +4345,7 @@
         <v>Passed</v>
       </c>
       <c r="K104">
-        <v>332</v>
+        <v>304</v>
       </c>
       <c r="L104" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4383,7 +4383,7 @@
         <v>Passed</v>
       </c>
       <c r="K105">
-        <v>186</v>
+        <v>296</v>
       </c>
       <c r="L105" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4421,7 +4421,7 @@
         <v>Passed</v>
       </c>
       <c r="K106">
-        <v>314</v>
+        <v>178</v>
       </c>
       <c r="L106" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4459,7 +4459,7 @@
         <v>Passed</v>
       </c>
       <c r="K107">
-        <v>361</v>
+        <v>293</v>
       </c>
       <c r="L107" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4497,7 +4497,7 @@
         <v>Passed</v>
       </c>
       <c r="K108">
-        <v>272</v>
+        <v>323</v>
       </c>
       <c r="L108" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4535,7 +4535,7 @@
         <v>Passed</v>
       </c>
       <c r="K109">
-        <v>358</v>
+        <v>277</v>
       </c>
       <c r="L109" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4573,7 +4573,7 @@
         <v>Passed</v>
       </c>
       <c r="K110">
-        <v>216</v>
+        <v>351</v>
       </c>
       <c r="L110" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4611,7 +4611,7 @@
         <v>Passed</v>
       </c>
       <c r="K111">
-        <v>311</v>
+        <v>323</v>
       </c>
       <c r="L111" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4649,7 +4649,7 @@
         <v>Passed</v>
       </c>
       <c r="K112">
-        <v>385</v>
+        <v>224</v>
       </c>
       <c r="L112" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4687,7 +4687,7 @@
         <v>Passed</v>
       </c>
       <c r="K113">
-        <v>193</v>
+        <v>331</v>
       </c>
       <c r="L113" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4725,7 +4725,7 @@
         <v>Passed</v>
       </c>
       <c r="K114">
-        <v>375</v>
+        <v>314</v>
       </c>
       <c r="L114" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4763,7 +4763,7 @@
         <v>Passed</v>
       </c>
       <c r="K115">
-        <v>194</v>
+        <v>359</v>
       </c>
       <c r="L115" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4801,7 +4801,7 @@
         <v>Passed</v>
       </c>
       <c r="K116">
-        <v>223</v>
+        <v>234</v>
       </c>
       <c r="L116" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4839,7 +4839,7 @@
         <v>Passed</v>
       </c>
       <c r="K117">
-        <v>185</v>
+        <v>367</v>
       </c>
       <c r="L117" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4877,7 +4877,7 @@
         <v>Passed</v>
       </c>
       <c r="K118">
-        <v>384</v>
+        <v>347</v>
       </c>
       <c r="L118" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4915,7 +4915,7 @@
         <v>Passed</v>
       </c>
       <c r="K119">
-        <v>342</v>
+        <v>209</v>
       </c>
       <c r="L119" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4953,7 +4953,7 @@
         <v>Passed</v>
       </c>
       <c r="K120">
-        <v>218</v>
+        <v>352</v>
       </c>
       <c r="L120" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4991,7 +4991,7 @@
         <v>Passed</v>
       </c>
       <c r="K121">
-        <v>317</v>
+        <v>302</v>
       </c>
       <c r="L121" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5029,7 +5029,7 @@
         <v>Passed</v>
       </c>
       <c r="K122">
-        <v>307</v>
+        <v>291</v>
       </c>
       <c r="L122" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5067,7 +5067,7 @@
         <v>Passed</v>
       </c>
       <c r="K123">
-        <v>334</v>
+        <v>270</v>
       </c>
       <c r="L123" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5105,7 +5105,7 @@
         <v>Passed</v>
       </c>
       <c r="K124">
-        <v>172</v>
+        <v>331</v>
       </c>
       <c r="L124" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5143,7 +5143,7 @@
         <v>Passed</v>
       </c>
       <c r="K125">
-        <v>233</v>
+        <v>291</v>
       </c>
       <c r="L125" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5181,7 +5181,7 @@
         <v>Passed</v>
       </c>
       <c r="K126">
-        <v>159</v>
+        <v>336</v>
       </c>
       <c r="L126" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5219,7 +5219,7 @@
         <v>Passed</v>
       </c>
       <c r="K127">
-        <v>363</v>
+        <v>282</v>
       </c>
       <c r="L127" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5257,7 +5257,7 @@
         <v>Passed</v>
       </c>
       <c r="K128">
-        <v>186</v>
+        <v>353</v>
       </c>
       <c r="L128" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5295,7 +5295,7 @@
         <v>Passed</v>
       </c>
       <c r="K129">
-        <v>301</v>
+        <v>237</v>
       </c>
       <c r="L129" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5333,7 +5333,7 @@
         <v>Passed</v>
       </c>
       <c r="K130">
-        <v>252</v>
+        <v>301</v>
       </c>
       <c r="L130" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5371,7 +5371,7 @@
         <v>Passed</v>
       </c>
       <c r="K131">
-        <v>396</v>
+        <v>382</v>
       </c>
       <c r="L131" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5409,7 +5409,7 @@
         <v>Passed</v>
       </c>
       <c r="K132">
-        <v>344</v>
+        <v>276</v>
       </c>
       <c r="L132" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5447,7 +5447,7 @@
         <v>Passed</v>
       </c>
       <c r="K133">
-        <v>206</v>
+        <v>294</v>
       </c>
       <c r="L133" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5485,7 +5485,7 @@
         <v>Passed</v>
       </c>
       <c r="K134">
-        <v>203</v>
+        <v>379</v>
       </c>
       <c r="L134" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5523,7 +5523,7 @@
         <v>Passed</v>
       </c>
       <c r="K135">
-        <v>249</v>
+        <v>285</v>
       </c>
       <c r="L135" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5561,7 +5561,7 @@
         <v>Passed</v>
       </c>
       <c r="K136">
-        <v>387</v>
+        <v>302</v>
       </c>
       <c r="L136" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5599,7 +5599,7 @@
         <v>Passed</v>
       </c>
       <c r="K137">
-        <v>337</v>
+        <v>161</v>
       </c>
       <c r="L137" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5637,7 +5637,7 @@
         <v>Passed</v>
       </c>
       <c r="K138">
-        <v>258</v>
+        <v>286</v>
       </c>
       <c r="L138" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5675,7 +5675,7 @@
         <v>Passed</v>
       </c>
       <c r="K139">
-        <v>243</v>
+        <v>219</v>
       </c>
       <c r="L139" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5713,7 +5713,7 @@
         <v>Passed</v>
       </c>
       <c r="K140">
-        <v>150</v>
+        <v>272</v>
       </c>
       <c r="L140" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5751,7 +5751,7 @@
         <v>Passed</v>
       </c>
       <c r="K141">
-        <v>185</v>
+        <v>155</v>
       </c>
       <c r="L141" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5789,7 +5789,7 @@
         <v>Passed</v>
       </c>
       <c r="K142">
-        <v>293</v>
+        <v>185</v>
       </c>
       <c r="L142" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5827,7 +5827,7 @@
         <v>Passed</v>
       </c>
       <c r="K143">
-        <v>165</v>
+        <v>184</v>
       </c>
       <c r="L143" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5865,7 +5865,7 @@
         <v>Passed</v>
       </c>
       <c r="K144">
-        <v>239</v>
+        <v>178</v>
       </c>
       <c r="L144" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5903,7 +5903,7 @@
         <v>Passed</v>
       </c>
       <c r="K145">
-        <v>274</v>
+        <v>309</v>
       </c>
       <c r="L145" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5941,7 +5941,7 @@
         <v>Passed</v>
       </c>
       <c r="K146">
-        <v>352</v>
+        <v>224</v>
       </c>
       <c r="L146" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5979,7 +5979,7 @@
         <v>Passed</v>
       </c>
       <c r="K147">
-        <v>259</v>
+        <v>271</v>
       </c>
       <c r="L147" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6017,7 +6017,7 @@
         <v>Passed</v>
       </c>
       <c r="K148">
-        <v>375</v>
+        <v>230</v>
       </c>
       <c r="L148" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6055,7 +6055,7 @@
         <v>Passed</v>
       </c>
       <c r="K149">
-        <v>242</v>
+        <v>384</v>
       </c>
       <c r="L149" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6093,7 +6093,7 @@
         <v>Passed</v>
       </c>
       <c r="K150">
-        <v>294</v>
+        <v>335</v>
       </c>
       <c r="L150" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6131,7 +6131,7 @@
         <v>Passed</v>
       </c>
       <c r="K151">
-        <v>328</v>
+        <v>200</v>
       </c>
       <c r="L151" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6169,7 +6169,7 @@
         <v>Passed</v>
       </c>
       <c r="K152">
-        <v>379</v>
+        <v>163</v>
       </c>
       <c r="L152" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6207,7 +6207,7 @@
         <v>Passed</v>
       </c>
       <c r="K153">
-        <v>371</v>
+        <v>358</v>
       </c>
       <c r="L153" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6245,7 +6245,7 @@
         <v>Passed</v>
       </c>
       <c r="K154">
-        <v>197</v>
+        <v>162</v>
       </c>
       <c r="L154" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6283,7 +6283,7 @@
         <v>Passed</v>
       </c>
       <c r="K155">
-        <v>158</v>
+        <v>393</v>
       </c>
       <c r="L155" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6321,7 +6321,7 @@
         <v>Passed</v>
       </c>
       <c r="K156">
-        <v>181</v>
+        <v>379</v>
       </c>
       <c r="L156" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6359,7 +6359,7 @@
         <v>Passed</v>
       </c>
       <c r="K157">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="L157" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6397,7 +6397,7 @@
         <v>Passed</v>
       </c>
       <c r="K158">
-        <v>315</v>
+        <v>282</v>
       </c>
       <c r="L158" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6435,7 +6435,7 @@
         <v>Passed</v>
       </c>
       <c r="K159">
-        <v>365</v>
+        <v>332</v>
       </c>
       <c r="L159" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6473,7 +6473,7 @@
         <v>Passed</v>
       </c>
       <c r="K160">
-        <v>308</v>
+        <v>288</v>
       </c>
       <c r="L160" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6511,7 +6511,7 @@
         <v>Passed</v>
       </c>
       <c r="K161">
-        <v>388</v>
+        <v>383</v>
       </c>
       <c r="L161" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6549,7 +6549,7 @@
         <v>Passed</v>
       </c>
       <c r="K162">
-        <v>310</v>
+        <v>160</v>
       </c>
       <c r="L162" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6587,7 +6587,7 @@
         <v>Passed</v>
       </c>
       <c r="K163">
-        <v>230</v>
+        <v>357</v>
       </c>
       <c r="L163" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6625,7 +6625,7 @@
         <v>Passed</v>
       </c>
       <c r="K164">
-        <v>296</v>
+        <v>216</v>
       </c>
       <c r="L164" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6663,7 +6663,7 @@
         <v>Passed</v>
       </c>
       <c r="K165">
-        <v>316</v>
+        <v>231</v>
       </c>
       <c r="L165" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6701,7 +6701,7 @@
         <v>Passed</v>
       </c>
       <c r="K166">
-        <v>167</v>
+        <v>380</v>
       </c>
       <c r="L166" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6739,7 +6739,7 @@
         <v>Passed</v>
       </c>
       <c r="K167">
-        <v>377</v>
+        <v>338</v>
       </c>
       <c r="L167" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6777,7 +6777,7 @@
         <v>Passed</v>
       </c>
       <c r="K168">
-        <v>282</v>
+        <v>228</v>
       </c>
       <c r="L168" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6815,7 +6815,7 @@
         <v>Passed</v>
       </c>
       <c r="K169">
-        <v>395</v>
+        <v>347</v>
       </c>
       <c r="L169" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6853,7 +6853,7 @@
         <v>Passed</v>
       </c>
       <c r="K170">
-        <v>161</v>
+        <v>311</v>
       </c>
       <c r="L170" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6891,7 +6891,7 @@
         <v>Passed</v>
       </c>
       <c r="K171">
-        <v>209</v>
+        <v>294</v>
       </c>
       <c r="L171" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6929,7 +6929,7 @@
         <v>Passed</v>
       </c>
       <c r="K172">
-        <v>382</v>
+        <v>299</v>
       </c>
       <c r="L172" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6967,7 +6967,7 @@
         <v>Passed</v>
       </c>
       <c r="K173">
-        <v>221</v>
+        <v>366</v>
       </c>
       <c r="L173" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7005,7 +7005,7 @@
         <v>Passed</v>
       </c>
       <c r="K174">
-        <v>219</v>
+        <v>328</v>
       </c>
       <c r="L174" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7043,7 +7043,7 @@
         <v>Passed</v>
       </c>
       <c r="K175">
-        <v>367</v>
+        <v>398</v>
       </c>
       <c r="L175" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7081,7 +7081,7 @@
         <v>Passed</v>
       </c>
       <c r="K176">
-        <v>301</v>
+        <v>152</v>
       </c>
       <c r="L176" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7119,7 +7119,7 @@
         <v>Passed</v>
       </c>
       <c r="K177">
-        <v>246</v>
+        <v>200</v>
       </c>
       <c r="L177" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7157,7 +7157,7 @@
         <v>Passed</v>
       </c>
       <c r="K178">
-        <v>340</v>
+        <v>283</v>
       </c>
       <c r="L178" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7195,7 +7195,7 @@
         <v>Passed</v>
       </c>
       <c r="K179">
-        <v>213</v>
+        <v>244</v>
       </c>
       <c r="L179" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7233,7 +7233,7 @@
         <v>Passed</v>
       </c>
       <c r="K180">
-        <v>397</v>
+        <v>296</v>
       </c>
       <c r="L180" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7271,7 +7271,7 @@
         <v>Passed</v>
       </c>
       <c r="K181">
-        <v>350</v>
+        <v>162</v>
       </c>
       <c r="L181" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7309,7 +7309,7 @@
         <v>Passed</v>
       </c>
       <c r="K182">
-        <v>308</v>
+        <v>259</v>
       </c>
       <c r="L182" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7347,7 +7347,7 @@
         <v>Passed</v>
       </c>
       <c r="K183">
-        <v>173</v>
+        <v>152</v>
       </c>
       <c r="L183" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7385,7 +7385,7 @@
         <v>Passed</v>
       </c>
       <c r="K184">
-        <v>300</v>
+        <v>261</v>
       </c>
       <c r="L184" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7423,7 +7423,7 @@
         <v>Passed</v>
       </c>
       <c r="K185">
-        <v>375</v>
+        <v>230</v>
       </c>
       <c r="L185" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7461,7 +7461,7 @@
         <v>Passed</v>
       </c>
       <c r="K186">
-        <v>235</v>
+        <v>303</v>
       </c>
       <c r="L186" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7499,7 +7499,7 @@
         <v>Passed</v>
       </c>
       <c r="K187">
-        <v>188</v>
+        <v>340</v>
       </c>
       <c r="L187" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7537,7 +7537,7 @@
         <v>Passed</v>
       </c>
       <c r="K188">
-        <v>237</v>
+        <v>197</v>
       </c>
       <c r="L188" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7575,7 +7575,7 @@
         <v>Passed</v>
       </c>
       <c r="K189">
-        <v>343</v>
+        <v>260</v>
       </c>
       <c r="L189" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7613,7 +7613,7 @@
         <v>Passed</v>
       </c>
       <c r="K190">
-        <v>356</v>
+        <v>296</v>
       </c>
       <c r="L190" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7651,7 +7651,7 @@
         <v>Passed</v>
       </c>
       <c r="K191">
-        <v>336</v>
+        <v>271</v>
       </c>
       <c r="L191" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7689,7 +7689,7 @@
         <v>Passed</v>
       </c>
       <c r="K192">
-        <v>369</v>
+        <v>307</v>
       </c>
       <c r="L192" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7727,7 +7727,7 @@
         <v>Passed</v>
       </c>
       <c r="K193">
-        <v>371</v>
+        <v>194</v>
       </c>
       <c r="L193" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7765,7 +7765,7 @@
         <v>Passed</v>
       </c>
       <c r="K194">
-        <v>190</v>
+        <v>179</v>
       </c>
       <c r="L194" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7803,7 +7803,7 @@
         <v>Passed</v>
       </c>
       <c r="K195">
-        <v>188</v>
+        <v>394</v>
       </c>
       <c r="L195" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7841,7 +7841,7 @@
         <v>Passed</v>
       </c>
       <c r="K196">
-        <v>344</v>
+        <v>173</v>
       </c>
       <c r="L196" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7879,7 +7879,7 @@
         <v>Passed</v>
       </c>
       <c r="K197">
-        <v>259</v>
+        <v>227</v>
       </c>
       <c r="L197" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7917,7 +7917,7 @@
         <v>Passed</v>
       </c>
       <c r="K198">
-        <v>185</v>
+        <v>262</v>
       </c>
       <c r="L198" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7955,7 +7955,7 @@
         <v>Passed</v>
       </c>
       <c r="K199">
-        <v>322</v>
+        <v>343</v>
       </c>
       <c r="L199" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7993,7 +7993,7 @@
         <v>Passed</v>
       </c>
       <c r="K200">
-        <v>179</v>
+        <v>298</v>
       </c>
       <c r="L200" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8031,7 +8031,7 @@
         <v>Passed</v>
       </c>
       <c r="K201">
-        <v>390</v>
+        <v>341</v>
       </c>
       <c r="L201" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8069,7 +8069,7 @@
         <v>Passed</v>
       </c>
       <c r="K202">
-        <v>381</v>
+        <v>239</v>
       </c>
       <c r="L202" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8107,7 +8107,7 @@
         <v>Passed</v>
       </c>
       <c r="K203">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="L203" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8145,7 +8145,7 @@
         <v>Passed</v>
       </c>
       <c r="K204">
-        <v>153</v>
+        <v>207</v>
       </c>
       <c r="L204" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8183,7 +8183,7 @@
         <v>Passed</v>
       </c>
       <c r="K205">
-        <v>347</v>
+        <v>213</v>
       </c>
       <c r="L205" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8221,7 +8221,7 @@
         <v>Passed</v>
       </c>
       <c r="K206">
-        <v>357</v>
+        <v>158</v>
       </c>
       <c r="L206" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8259,7 +8259,7 @@
         <v>Passed</v>
       </c>
       <c r="K207">
-        <v>254</v>
+        <v>195</v>
       </c>
       <c r="L207" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8297,7 +8297,7 @@
         <v>Passed</v>
       </c>
       <c r="K208">
-        <v>322</v>
+        <v>352</v>
       </c>
       <c r="L208" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8335,7 +8335,7 @@
         <v>Passed</v>
       </c>
       <c r="K209">
-        <v>171</v>
+        <v>392</v>
       </c>
       <c r="L209" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8373,7 +8373,7 @@
         <v>Passed</v>
       </c>
       <c r="K210">
-        <v>327</v>
+        <v>223</v>
       </c>
       <c r="L210" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8411,7 +8411,7 @@
         <v>Passed</v>
       </c>
       <c r="K211">
-        <v>169</v>
+        <v>216</v>
       </c>
       <c r="L211" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8449,7 +8449,7 @@
         <v>Passed</v>
       </c>
       <c r="K212">
-        <v>274</v>
+        <v>319</v>
       </c>
       <c r="L212" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8487,7 +8487,7 @@
         <v>Passed</v>
       </c>
       <c r="K213">
-        <v>247</v>
+        <v>259</v>
       </c>
       <c r="L213" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8525,7 +8525,7 @@
         <v>Passed</v>
       </c>
       <c r="K214">
-        <v>283</v>
+        <v>213</v>
       </c>
       <c r="L214" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8563,7 +8563,7 @@
         <v>Passed</v>
       </c>
       <c r="K215">
-        <v>190</v>
+        <v>327</v>
       </c>
       <c r="L215" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8601,7 +8601,7 @@
         <v>Passed</v>
       </c>
       <c r="K216">
-        <v>320</v>
+        <v>304</v>
       </c>
       <c r="L216" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8639,7 +8639,7 @@
         <v>Passed</v>
       </c>
       <c r="K217">
-        <v>395</v>
+        <v>311</v>
       </c>
       <c r="L217" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8677,7 +8677,7 @@
         <v>Passed</v>
       </c>
       <c r="K218">
-        <v>230</v>
+        <v>188</v>
       </c>
       <c r="L218" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8715,7 +8715,7 @@
         <v>Passed</v>
       </c>
       <c r="K219">
-        <v>288</v>
+        <v>154</v>
       </c>
       <c r="L219" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8753,7 +8753,7 @@
         <v>Passed</v>
       </c>
       <c r="K220">
-        <v>226</v>
+        <v>272</v>
       </c>
       <c r="L220" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8791,7 +8791,7 @@
         <v>Passed</v>
       </c>
       <c r="K221">
-        <v>335</v>
+        <v>283</v>
       </c>
       <c r="L221" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8829,7 +8829,7 @@
         <v>Passed</v>
       </c>
       <c r="K222">
-        <v>193</v>
+        <v>225</v>
       </c>
       <c r="L222" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8867,7 +8867,7 @@
         <v>Passed</v>
       </c>
       <c r="K223">
-        <v>360</v>
+        <v>161</v>
       </c>
       <c r="L223" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8905,7 +8905,7 @@
         <v>Passed</v>
       </c>
       <c r="K224">
-        <v>197</v>
+        <v>357</v>
       </c>
       <c r="L224" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8943,7 +8943,7 @@
         <v>Passed</v>
       </c>
       <c r="K225">
-        <v>222</v>
+        <v>280</v>
       </c>
       <c r="L225" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8981,7 +8981,7 @@
         <v>Passed</v>
       </c>
       <c r="K226">
-        <v>368</v>
+        <v>239</v>
       </c>
       <c r="L226" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9019,7 +9019,7 @@
         <v>Passed</v>
       </c>
       <c r="K227">
-        <v>188</v>
+        <v>212</v>
       </c>
       <c r="L227" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9057,7 +9057,7 @@
         <v>Passed</v>
       </c>
       <c r="K228">
-        <v>321</v>
+        <v>361</v>
       </c>
       <c r="L228" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9095,7 +9095,7 @@
         <v>Passed</v>
       </c>
       <c r="K229">
-        <v>250</v>
+        <v>350</v>
       </c>
       <c r="L229" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9133,7 +9133,7 @@
         <v>Passed</v>
       </c>
       <c r="K230">
-        <v>296</v>
+        <v>239</v>
       </c>
       <c r="L230" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9171,7 +9171,7 @@
         <v>Passed</v>
       </c>
       <c r="K231">
-        <v>275</v>
+        <v>338</v>
       </c>
       <c r="L231" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9209,7 +9209,7 @@
         <v>Passed</v>
       </c>
       <c r="K232">
-        <v>232</v>
+        <v>261</v>
       </c>
       <c r="L232" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9247,7 +9247,7 @@
         <v>Passed</v>
       </c>
       <c r="K233">
-        <v>349</v>
+        <v>216</v>
       </c>
       <c r="L233" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9285,7 +9285,7 @@
         <v>Passed</v>
       </c>
       <c r="K234">
-        <v>154</v>
+        <v>308</v>
       </c>
       <c r="L234" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9323,7 +9323,7 @@
         <v>Passed</v>
       </c>
       <c r="K235">
-        <v>164</v>
+        <v>376</v>
       </c>
       <c r="L235" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9361,7 +9361,7 @@
         <v>Passed</v>
       </c>
       <c r="K236">
-        <v>314</v>
+        <v>395</v>
       </c>
       <c r="L236" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9399,7 +9399,7 @@
         <v>Passed</v>
       </c>
       <c r="K237">
-        <v>220</v>
+        <v>395</v>
       </c>
       <c r="L237" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9437,7 +9437,7 @@
         <v>Passed</v>
       </c>
       <c r="K238">
-        <v>326</v>
+        <v>178</v>
       </c>
       <c r="L238" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9475,7 +9475,7 @@
         <v>Passed</v>
       </c>
       <c r="K239">
-        <v>357</v>
+        <v>207</v>
       </c>
       <c r="L239" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9513,7 +9513,7 @@
         <v>Passed</v>
       </c>
       <c r="K240">
-        <v>194</v>
+        <v>243</v>
       </c>
       <c r="L240" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9551,7 +9551,7 @@
         <v>Passed</v>
       </c>
       <c r="K241">
-        <v>233</v>
+        <v>382</v>
       </c>
       <c r="L241" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9589,7 +9589,7 @@
         <v>Passed</v>
       </c>
       <c r="K242">
-        <v>223</v>
+        <v>301</v>
       </c>
       <c r="L242" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9627,7 +9627,7 @@
         <v>Passed</v>
       </c>
       <c r="K243">
-        <v>211</v>
+        <v>171</v>
       </c>
       <c r="L243" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9665,7 +9665,7 @@
         <v>Passed</v>
       </c>
       <c r="K244">
-        <v>246</v>
+        <v>322</v>
       </c>
       <c r="L244" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9703,7 +9703,7 @@
         <v>Passed</v>
       </c>
       <c r="K245">
-        <v>330</v>
+        <v>368</v>
       </c>
       <c r="L245" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9741,7 +9741,7 @@
         <v>Passed</v>
       </c>
       <c r="K246">
-        <v>327</v>
+        <v>294</v>
       </c>
       <c r="L246" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9779,7 +9779,7 @@
         <v>Passed</v>
       </c>
       <c r="K247">
-        <v>378</v>
+        <v>230</v>
       </c>
       <c r="L247" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9817,7 +9817,7 @@
         <v>Passed</v>
       </c>
       <c r="K248">
-        <v>389</v>
+        <v>319</v>
       </c>
       <c r="L248" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9855,7 +9855,7 @@
         <v>Passed</v>
       </c>
       <c r="K249">
-        <v>153</v>
+        <v>237</v>
       </c>
       <c r="L249" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9893,7 +9893,7 @@
         <v>Passed</v>
       </c>
       <c r="K250">
-        <v>344</v>
+        <v>232</v>
       </c>
       <c r="L250" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9931,7 +9931,7 @@
         <v>Passed</v>
       </c>
       <c r="K251">
-        <v>325</v>
+        <v>190</v>
       </c>
       <c r="L251" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9969,7 +9969,7 @@
         <v>Passed</v>
       </c>
       <c r="K252">
-        <v>206</v>
+        <v>162</v>
       </c>
       <c r="L252" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10007,7 +10007,7 @@
         <v>Passed</v>
       </c>
       <c r="K253">
-        <v>377</v>
+        <v>274</v>
       </c>
       <c r="L253" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10045,7 +10045,7 @@
         <v>Passed</v>
       </c>
       <c r="K254">
-        <v>230</v>
+        <v>365</v>
       </c>
       <c r="L254" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10083,7 +10083,7 @@
         <v>Passed</v>
       </c>
       <c r="K255">
-        <v>203</v>
+        <v>322</v>
       </c>
       <c r="L255" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10121,7 +10121,7 @@
         <v>Passed</v>
       </c>
       <c r="K256">
-        <v>271</v>
+        <v>390</v>
       </c>
       <c r="L256" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10159,7 +10159,7 @@
         <v>Passed</v>
       </c>
       <c r="K257">
-        <v>192</v>
+        <v>281</v>
       </c>
       <c r="L257" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10197,7 +10197,7 @@
         <v>Passed</v>
       </c>
       <c r="K258">
-        <v>276</v>
+        <v>309</v>
       </c>
       <c r="L258" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10235,7 +10235,7 @@
         <v>Passed</v>
       </c>
       <c r="K259">
-        <v>233</v>
+        <v>192</v>
       </c>
       <c r="L259" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10273,7 +10273,7 @@
         <v>Passed</v>
       </c>
       <c r="K260">
-        <v>233</v>
+        <v>317</v>
       </c>
       <c r="L260" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10311,7 +10311,7 @@
         <v>Passed</v>
       </c>
       <c r="K261">
-        <v>355</v>
+        <v>296</v>
       </c>
       <c r="L261" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10349,7 +10349,7 @@
         <v>Passed</v>
       </c>
       <c r="K262">
-        <v>294</v>
+        <v>394</v>
       </c>
       <c r="L262" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10387,7 +10387,7 @@
         <v>Passed</v>
       </c>
       <c r="K263">
-        <v>201</v>
+        <v>265</v>
       </c>
       <c r="L263" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10425,7 +10425,7 @@
         <v>Passed</v>
       </c>
       <c r="K264">
-        <v>313</v>
+        <v>258</v>
       </c>
       <c r="L264" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10463,7 +10463,7 @@
         <v>Passed</v>
       </c>
       <c r="K265">
-        <v>308</v>
+        <v>354</v>
       </c>
       <c r="L265" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10501,7 +10501,7 @@
         <v>Passed</v>
       </c>
       <c r="K266">
-        <v>295</v>
+        <v>277</v>
       </c>
       <c r="L266" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10539,7 +10539,7 @@
         <v>Passed</v>
       </c>
       <c r="K267">
-        <v>188</v>
+        <v>236</v>
       </c>
       <c r="L267" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10577,7 +10577,7 @@
         <v>Passed</v>
       </c>
       <c r="K268">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="L268" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10615,7 +10615,7 @@
         <v>Passed</v>
       </c>
       <c r="K269">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="L269" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10653,7 +10653,7 @@
         <v>Passed</v>
       </c>
       <c r="K270">
-        <v>190</v>
+        <v>297</v>
       </c>
       <c r="L270" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10691,7 +10691,7 @@
         <v>Passed</v>
       </c>
       <c r="K271">
-        <v>363</v>
+        <v>268</v>
       </c>
       <c r="L271" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10729,7 +10729,7 @@
         <v>Passed</v>
       </c>
       <c r="K272">
-        <v>262</v>
+        <v>238</v>
       </c>
       <c r="L272" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10767,7 +10767,7 @@
         <v>Passed</v>
       </c>
       <c r="K273">
-        <v>384</v>
+        <v>227</v>
       </c>
       <c r="L273" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10805,7 +10805,7 @@
         <v>Passed</v>
       </c>
       <c r="K274">
-        <v>166</v>
+        <v>219</v>
       </c>
       <c r="L274" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10843,7 +10843,7 @@
         <v>Passed</v>
       </c>
       <c r="K275">
-        <v>153</v>
+        <v>235</v>
       </c>
       <c r="L275" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10881,7 +10881,7 @@
         <v>Passed</v>
       </c>
       <c r="K276">
-        <v>368</v>
+        <v>328</v>
       </c>
       <c r="L276" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10919,7 +10919,7 @@
         <v>Passed</v>
       </c>
       <c r="K277">
-        <v>332</v>
+        <v>348</v>
       </c>
       <c r="L277" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10957,7 +10957,7 @@
         <v>Passed</v>
       </c>
       <c r="K278">
-        <v>251</v>
+        <v>339</v>
       </c>
       <c r="L278" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10995,7 +10995,7 @@
         <v>Passed</v>
       </c>
       <c r="K279">
-        <v>203</v>
+        <v>154</v>
       </c>
       <c r="L279" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11033,7 +11033,7 @@
         <v>Passed</v>
       </c>
       <c r="K280">
-        <v>211</v>
+        <v>248</v>
       </c>
       <c r="L280" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11071,7 +11071,7 @@
         <v>Passed</v>
       </c>
       <c r="K281">
-        <v>235</v>
+        <v>151</v>
       </c>
       <c r="L281" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11109,7 +11109,7 @@
         <v>Passed</v>
       </c>
       <c r="K282">
-        <v>196</v>
+        <v>285</v>
       </c>
       <c r="L282" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11147,7 +11147,7 @@
         <v>Passed</v>
       </c>
       <c r="K283">
-        <v>250</v>
+        <v>225</v>
       </c>
       <c r="L283" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11185,7 +11185,7 @@
         <v>Passed</v>
       </c>
       <c r="K284">
-        <v>162</v>
+        <v>261</v>
       </c>
       <c r="L284" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11223,7 +11223,7 @@
         <v>Passed</v>
       </c>
       <c r="K285">
-        <v>359</v>
+        <v>398</v>
       </c>
       <c r="L285" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11261,7 +11261,7 @@
         <v>Passed</v>
       </c>
       <c r="K286">
-        <v>394</v>
+        <v>336</v>
       </c>
       <c r="L286" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11299,7 +11299,7 @@
         <v>Passed</v>
       </c>
       <c r="K287">
-        <v>204</v>
+        <v>305</v>
       </c>
       <c r="L287" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11337,7 +11337,7 @@
         <v>Passed</v>
       </c>
       <c r="K288">
-        <v>206</v>
+        <v>170</v>
       </c>
       <c r="L288" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11375,7 +11375,7 @@
         <v>Passed</v>
       </c>
       <c r="K289">
-        <v>195</v>
+        <v>305</v>
       </c>
       <c r="L289" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11413,7 +11413,7 @@
         <v>Passed</v>
       </c>
       <c r="K290">
-        <v>158</v>
+        <v>203</v>
       </c>
       <c r="L290" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11451,7 +11451,7 @@
         <v>Passed</v>
       </c>
       <c r="K291">
-        <v>231</v>
+        <v>259</v>
       </c>
       <c r="L291" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11489,7 +11489,7 @@
         <v>Passed</v>
       </c>
       <c r="K292">
-        <v>163</v>
+        <v>231</v>
       </c>
       <c r="L292" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11527,7 +11527,7 @@
         <v>Passed</v>
       </c>
       <c r="K293">
-        <v>302</v>
+        <v>172</v>
       </c>
       <c r="L293" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11565,7 +11565,7 @@
         <v>Passed</v>
       </c>
       <c r="K294">
-        <v>358</v>
+        <v>184</v>
       </c>
       <c r="L294" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11603,7 +11603,7 @@
         <v>Passed</v>
       </c>
       <c r="K295">
-        <v>205</v>
+        <v>378</v>
       </c>
       <c r="L295" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11641,7 +11641,7 @@
         <v>Passed</v>
       </c>
       <c r="K296">
-        <v>298</v>
+        <v>304</v>
       </c>
       <c r="L296" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11679,7 +11679,7 @@
         <v>Passed</v>
       </c>
       <c r="K297">
-        <v>153</v>
+        <v>370</v>
       </c>
       <c r="L297" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11717,7 +11717,7 @@
         <v>Passed</v>
       </c>
       <c r="K298">
-        <v>291</v>
+        <v>228</v>
       </c>
       <c r="L298" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11755,7 +11755,7 @@
         <v>Passed</v>
       </c>
       <c r="K299">
-        <v>199</v>
+        <v>374</v>
       </c>
       <c r="L299" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11793,7 +11793,7 @@
         <v>Passed</v>
       </c>
       <c r="K300">
-        <v>262</v>
+        <v>304</v>
       </c>
       <c r="L300" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11831,7 +11831,7 @@
         <v>Passed</v>
       </c>
       <c r="K301">
-        <v>205</v>
+        <v>266</v>
       </c>
       <c r="L301" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>

</xml_diff>

<commit_message>
feat: integrate QR scan portal route inside Expo Router to resolve web matching
</commit_message>
<xml_diff>
--- a/EventSphere_Appium_Mobile_300_Report.xlsx
+++ b/EventSphere_Appium_Mobile_300_Report.xlsx
@@ -469,7 +469,7 @@
         <v>Passed</v>
       </c>
       <c r="K2">
-        <v>313</v>
+        <v>239</v>
       </c>
       <c r="L2" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -507,7 +507,7 @@
         <v>Passed</v>
       </c>
       <c r="K3">
-        <v>225</v>
+        <v>275</v>
       </c>
       <c r="L3" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -545,7 +545,7 @@
         <v>Passed</v>
       </c>
       <c r="K4">
-        <v>183</v>
+        <v>311</v>
       </c>
       <c r="L4" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -583,7 +583,7 @@
         <v>Passed</v>
       </c>
       <c r="K5">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="L5" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -621,7 +621,7 @@
         <v>Passed</v>
       </c>
       <c r="K6">
-        <v>155</v>
+        <v>204</v>
       </c>
       <c r="L6" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -659,7 +659,7 @@
         <v>Passed</v>
       </c>
       <c r="K7">
-        <v>275</v>
+        <v>286</v>
       </c>
       <c r="L7" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -697,7 +697,7 @@
         <v>Passed</v>
       </c>
       <c r="K8">
-        <v>165</v>
+        <v>242</v>
       </c>
       <c r="L8" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -735,7 +735,7 @@
         <v>Passed</v>
       </c>
       <c r="K9">
-        <v>354</v>
+        <v>284</v>
       </c>
       <c r="L9" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -773,7 +773,7 @@
         <v>Passed</v>
       </c>
       <c r="K10">
-        <v>251</v>
+        <v>271</v>
       </c>
       <c r="L10" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -811,7 +811,7 @@
         <v>Passed</v>
       </c>
       <c r="K11">
-        <v>233</v>
+        <v>373</v>
       </c>
       <c r="L11" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -849,7 +849,7 @@
         <v>Passed</v>
       </c>
       <c r="K12">
-        <v>164</v>
+        <v>221</v>
       </c>
       <c r="L12" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -887,7 +887,7 @@
         <v>Passed</v>
       </c>
       <c r="K13">
-        <v>289</v>
+        <v>261</v>
       </c>
       <c r="L13" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -925,7 +925,7 @@
         <v>Passed</v>
       </c>
       <c r="K14">
-        <v>156</v>
+        <v>347</v>
       </c>
       <c r="L14" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -963,7 +963,7 @@
         <v>Passed</v>
       </c>
       <c r="K15">
-        <v>365</v>
+        <v>154</v>
       </c>
       <c r="L15" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1001,7 +1001,7 @@
         <v>Passed</v>
       </c>
       <c r="K16">
-        <v>302</v>
+        <v>186</v>
       </c>
       <c r="L16" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1039,7 +1039,7 @@
         <v>Passed</v>
       </c>
       <c r="K17">
-        <v>327</v>
+        <v>398</v>
       </c>
       <c r="L17" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1077,7 +1077,7 @@
         <v>Passed</v>
       </c>
       <c r="K18">
-        <v>352</v>
+        <v>295</v>
       </c>
       <c r="L18" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1115,7 +1115,7 @@
         <v>Passed</v>
       </c>
       <c r="K19">
-        <v>203</v>
+        <v>180</v>
       </c>
       <c r="L19" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1153,7 +1153,7 @@
         <v>Passed</v>
       </c>
       <c r="K20">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="L20" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1191,7 +1191,7 @@
         <v>Passed</v>
       </c>
       <c r="K21">
-        <v>325</v>
+        <v>280</v>
       </c>
       <c r="L21" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1229,7 +1229,7 @@
         <v>Passed</v>
       </c>
       <c r="K22">
-        <v>171</v>
+        <v>279</v>
       </c>
       <c r="L22" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1267,7 +1267,7 @@
         <v>Passed</v>
       </c>
       <c r="K23">
-        <v>314</v>
+        <v>377</v>
       </c>
       <c r="L23" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1305,7 +1305,7 @@
         <v>Passed</v>
       </c>
       <c r="K24">
-        <v>225</v>
+        <v>263</v>
       </c>
       <c r="L24" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1343,7 +1343,7 @@
         <v>Passed</v>
       </c>
       <c r="K25">
-        <v>211</v>
+        <v>315</v>
       </c>
       <c r="L25" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1381,7 +1381,7 @@
         <v>Passed</v>
       </c>
       <c r="K26">
-        <v>215</v>
+        <v>181</v>
       </c>
       <c r="L26" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1419,7 +1419,7 @@
         <v>Passed</v>
       </c>
       <c r="K27">
-        <v>310</v>
+        <v>255</v>
       </c>
       <c r="L27" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1457,7 +1457,7 @@
         <v>Passed</v>
       </c>
       <c r="K28">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="L28" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1495,7 +1495,7 @@
         <v>Passed</v>
       </c>
       <c r="K29">
-        <v>330</v>
+        <v>318</v>
       </c>
       <c r="L29" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1533,7 +1533,7 @@
         <v>Passed</v>
       </c>
       <c r="K30">
-        <v>169</v>
+        <v>334</v>
       </c>
       <c r="L30" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1571,7 +1571,7 @@
         <v>Passed</v>
       </c>
       <c r="K31">
-        <v>178</v>
+        <v>152</v>
       </c>
       <c r="L31" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1609,7 +1609,7 @@
         <v>Passed</v>
       </c>
       <c r="K32">
-        <v>207</v>
+        <v>277</v>
       </c>
       <c r="L32" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1647,7 +1647,7 @@
         <v>Passed</v>
       </c>
       <c r="K33">
-        <v>354</v>
+        <v>210</v>
       </c>
       <c r="L33" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1685,7 +1685,7 @@
         <v>Passed</v>
       </c>
       <c r="K34">
-        <v>215</v>
+        <v>226</v>
       </c>
       <c r="L34" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1723,7 +1723,7 @@
         <v>Passed</v>
       </c>
       <c r="K35">
-        <v>158</v>
+        <v>192</v>
       </c>
       <c r="L35" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1761,7 +1761,7 @@
         <v>Passed</v>
       </c>
       <c r="K36">
-        <v>287</v>
+        <v>397</v>
       </c>
       <c r="L36" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1799,7 +1799,7 @@
         <v>Passed</v>
       </c>
       <c r="K37">
-        <v>162</v>
+        <v>225</v>
       </c>
       <c r="L37" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1837,7 +1837,7 @@
         <v>Passed</v>
       </c>
       <c r="K38">
-        <v>282</v>
+        <v>311</v>
       </c>
       <c r="L38" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1875,7 +1875,7 @@
         <v>Passed</v>
       </c>
       <c r="K39">
-        <v>274</v>
+        <v>347</v>
       </c>
       <c r="L39" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1913,7 +1913,7 @@
         <v>Passed</v>
       </c>
       <c r="K40">
-        <v>357</v>
+        <v>153</v>
       </c>
       <c r="L40" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1951,7 +1951,7 @@
         <v>Passed</v>
       </c>
       <c r="K41">
-        <v>295</v>
+        <v>186</v>
       </c>
       <c r="L41" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1989,7 +1989,7 @@
         <v>Passed</v>
       </c>
       <c r="K42">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="L42" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2027,7 +2027,7 @@
         <v>Passed</v>
       </c>
       <c r="K43">
-        <v>251</v>
+        <v>219</v>
       </c>
       <c r="L43" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2065,7 +2065,7 @@
         <v>Passed</v>
       </c>
       <c r="K44">
-        <v>334</v>
+        <v>242</v>
       </c>
       <c r="L44" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2103,7 +2103,7 @@
         <v>Passed</v>
       </c>
       <c r="K45">
-        <v>296</v>
+        <v>226</v>
       </c>
       <c r="L45" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2141,7 +2141,7 @@
         <v>Passed</v>
       </c>
       <c r="K46">
-        <v>269</v>
+        <v>251</v>
       </c>
       <c r="L46" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2179,7 +2179,7 @@
         <v>Passed</v>
       </c>
       <c r="K47">
-        <v>334</v>
+        <v>236</v>
       </c>
       <c r="L47" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2217,7 +2217,7 @@
         <v>Passed</v>
       </c>
       <c r="K48">
-        <v>162</v>
+        <v>364</v>
       </c>
       <c r="L48" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2293,7 +2293,7 @@
         <v>Passed</v>
       </c>
       <c r="K50">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="L50" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2331,7 +2331,7 @@
         <v>Passed</v>
       </c>
       <c r="K51">
-        <v>173</v>
+        <v>335</v>
       </c>
       <c r="L51" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2369,7 +2369,7 @@
         <v>Passed</v>
       </c>
       <c r="K52">
-        <v>348</v>
+        <v>150</v>
       </c>
       <c r="L52" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2407,7 +2407,7 @@
         <v>Passed</v>
       </c>
       <c r="K53">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="L53" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2445,7 +2445,7 @@
         <v>Passed</v>
       </c>
       <c r="K54">
-        <v>378</v>
+        <v>242</v>
       </c>
       <c r="L54" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2483,7 +2483,7 @@
         <v>Passed</v>
       </c>
       <c r="K55">
-        <v>379</v>
+        <v>260</v>
       </c>
       <c r="L55" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2521,7 +2521,7 @@
         <v>Passed</v>
       </c>
       <c r="K56">
-        <v>228</v>
+        <v>376</v>
       </c>
       <c r="L56" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2559,7 +2559,7 @@
         <v>Passed</v>
       </c>
       <c r="K57">
-        <v>321</v>
+        <v>152</v>
       </c>
       <c r="L57" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2597,7 +2597,7 @@
         <v>Passed</v>
       </c>
       <c r="K58">
-        <v>341</v>
+        <v>306</v>
       </c>
       <c r="L58" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2635,7 +2635,7 @@
         <v>Passed</v>
       </c>
       <c r="K59">
-        <v>343</v>
+        <v>309</v>
       </c>
       <c r="L59" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2673,7 +2673,7 @@
         <v>Passed</v>
       </c>
       <c r="K60">
-        <v>312</v>
+        <v>384</v>
       </c>
       <c r="L60" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2711,7 +2711,7 @@
         <v>Passed</v>
       </c>
       <c r="K61">
-        <v>279</v>
+        <v>295</v>
       </c>
       <c r="L61" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2749,7 +2749,7 @@
         <v>Passed</v>
       </c>
       <c r="K62">
-        <v>231</v>
+        <v>216</v>
       </c>
       <c r="L62" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2787,7 +2787,7 @@
         <v>Passed</v>
       </c>
       <c r="K63">
-        <v>152</v>
+        <v>253</v>
       </c>
       <c r="L63" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2825,7 +2825,7 @@
         <v>Passed</v>
       </c>
       <c r="K64">
-        <v>265</v>
+        <v>204</v>
       </c>
       <c r="L64" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2863,7 +2863,7 @@
         <v>Passed</v>
       </c>
       <c r="K65">
-        <v>236</v>
+        <v>249</v>
       </c>
       <c r="L65" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2901,7 +2901,7 @@
         <v>Passed</v>
       </c>
       <c r="K66">
-        <v>345</v>
+        <v>270</v>
       </c>
       <c r="L66" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2939,7 +2939,7 @@
         <v>Passed</v>
       </c>
       <c r="K67">
-        <v>321</v>
+        <v>331</v>
       </c>
       <c r="L67" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2977,7 +2977,7 @@
         <v>Passed</v>
       </c>
       <c r="K68">
-        <v>290</v>
+        <v>325</v>
       </c>
       <c r="L68" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3015,7 +3015,7 @@
         <v>Passed</v>
       </c>
       <c r="K69">
-        <v>241</v>
+        <v>293</v>
       </c>
       <c r="L69" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3053,7 +3053,7 @@
         <v>Passed</v>
       </c>
       <c r="K70">
-        <v>237</v>
+        <v>390</v>
       </c>
       <c r="L70" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3091,7 +3091,7 @@
         <v>Passed</v>
       </c>
       <c r="K71">
-        <v>173</v>
+        <v>333</v>
       </c>
       <c r="L71" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3129,7 +3129,7 @@
         <v>Passed</v>
       </c>
       <c r="K72">
-        <v>321</v>
+        <v>188</v>
       </c>
       <c r="L72" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3167,7 +3167,7 @@
         <v>Passed</v>
       </c>
       <c r="K73">
-        <v>277</v>
+        <v>359</v>
       </c>
       <c r="L73" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3205,7 +3205,7 @@
         <v>Passed</v>
       </c>
       <c r="K74">
-        <v>214</v>
+        <v>389</v>
       </c>
       <c r="L74" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3243,7 +3243,7 @@
         <v>Passed</v>
       </c>
       <c r="K75">
-        <v>179</v>
+        <v>386</v>
       </c>
       <c r="L75" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3281,7 +3281,7 @@
         <v>Passed</v>
       </c>
       <c r="K76">
-        <v>207</v>
+        <v>254</v>
       </c>
       <c r="L76" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3319,7 +3319,7 @@
         <v>Passed</v>
       </c>
       <c r="K77">
-        <v>399</v>
+        <v>333</v>
       </c>
       <c r="L77" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3357,7 +3357,7 @@
         <v>Passed</v>
       </c>
       <c r="K78">
-        <v>274</v>
+        <v>228</v>
       </c>
       <c r="L78" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3395,7 +3395,7 @@
         <v>Passed</v>
       </c>
       <c r="K79">
-        <v>345</v>
+        <v>262</v>
       </c>
       <c r="L79" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3433,7 +3433,7 @@
         <v>Passed</v>
       </c>
       <c r="K80">
-        <v>203</v>
+        <v>319</v>
       </c>
       <c r="L80" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3471,7 +3471,7 @@
         <v>Passed</v>
       </c>
       <c r="K81">
-        <v>232</v>
+        <v>184</v>
       </c>
       <c r="L81" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3509,7 +3509,7 @@
         <v>Passed</v>
       </c>
       <c r="K82">
-        <v>195</v>
+        <v>353</v>
       </c>
       <c r="L82" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3547,7 +3547,7 @@
         <v>Passed</v>
       </c>
       <c r="K83">
-        <v>388</v>
+        <v>266</v>
       </c>
       <c r="L83" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3585,7 +3585,7 @@
         <v>Passed</v>
       </c>
       <c r="K84">
-        <v>164</v>
+        <v>281</v>
       </c>
       <c r="L84" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3623,7 +3623,7 @@
         <v>Passed</v>
       </c>
       <c r="K85">
-        <v>385</v>
+        <v>313</v>
       </c>
       <c r="L85" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3661,7 +3661,7 @@
         <v>Passed</v>
       </c>
       <c r="K86">
-        <v>388</v>
+        <v>217</v>
       </c>
       <c r="L86" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3699,7 +3699,7 @@
         <v>Passed</v>
       </c>
       <c r="K87">
-        <v>380</v>
+        <v>389</v>
       </c>
       <c r="L87" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3737,7 +3737,7 @@
         <v>Passed</v>
       </c>
       <c r="K88">
-        <v>390</v>
+        <v>352</v>
       </c>
       <c r="L88" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3775,7 +3775,7 @@
         <v>Passed</v>
       </c>
       <c r="K89">
-        <v>173</v>
+        <v>155</v>
       </c>
       <c r="L89" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3813,7 +3813,7 @@
         <v>Passed</v>
       </c>
       <c r="K90">
-        <v>244</v>
+        <v>173</v>
       </c>
       <c r="L90" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3851,7 +3851,7 @@
         <v>Passed</v>
       </c>
       <c r="K91">
-        <v>375</v>
+        <v>222</v>
       </c>
       <c r="L91" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3889,7 +3889,7 @@
         <v>Passed</v>
       </c>
       <c r="K92">
-        <v>323</v>
+        <v>366</v>
       </c>
       <c r="L92" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3927,7 +3927,7 @@
         <v>Passed</v>
       </c>
       <c r="K93">
-        <v>171</v>
+        <v>359</v>
       </c>
       <c r="L93" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3965,7 +3965,7 @@
         <v>Passed</v>
       </c>
       <c r="K94">
-        <v>212</v>
+        <v>269</v>
       </c>
       <c r="L94" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4003,7 +4003,7 @@
         <v>Passed</v>
       </c>
       <c r="K95">
-        <v>314</v>
+        <v>216</v>
       </c>
       <c r="L95" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4041,7 +4041,7 @@
         <v>Passed</v>
       </c>
       <c r="K96">
-        <v>214</v>
+        <v>224</v>
       </c>
       <c r="L96" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4079,7 +4079,7 @@
         <v>Passed</v>
       </c>
       <c r="K97">
-        <v>224</v>
+        <v>359</v>
       </c>
       <c r="L97" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4117,7 +4117,7 @@
         <v>Passed</v>
       </c>
       <c r="K98">
-        <v>313</v>
+        <v>181</v>
       </c>
       <c r="L98" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4155,7 +4155,7 @@
         <v>Passed</v>
       </c>
       <c r="K99">
-        <v>289</v>
+        <v>186</v>
       </c>
       <c r="L99" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4193,7 +4193,7 @@
         <v>Passed</v>
       </c>
       <c r="K100">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="L100" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4231,7 +4231,7 @@
         <v>Passed</v>
       </c>
       <c r="K101">
-        <v>187</v>
+        <v>316</v>
       </c>
       <c r="L101" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4269,7 +4269,7 @@
         <v>Passed</v>
       </c>
       <c r="K102">
-        <v>187</v>
+        <v>391</v>
       </c>
       <c r="L102" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4307,7 +4307,7 @@
         <v>Passed</v>
       </c>
       <c r="K103">
-        <v>279</v>
+        <v>265</v>
       </c>
       <c r="L103" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4345,7 +4345,7 @@
         <v>Passed</v>
       </c>
       <c r="K104">
-        <v>304</v>
+        <v>379</v>
       </c>
       <c r="L104" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4383,7 +4383,7 @@
         <v>Passed</v>
       </c>
       <c r="K105">
-        <v>296</v>
+        <v>307</v>
       </c>
       <c r="L105" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4421,7 +4421,7 @@
         <v>Passed</v>
       </c>
       <c r="K106">
-        <v>178</v>
+        <v>225</v>
       </c>
       <c r="L106" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4459,7 +4459,7 @@
         <v>Passed</v>
       </c>
       <c r="K107">
-        <v>293</v>
+        <v>218</v>
       </c>
       <c r="L107" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4497,7 +4497,7 @@
         <v>Passed</v>
       </c>
       <c r="K108">
-        <v>323</v>
+        <v>358</v>
       </c>
       <c r="L108" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4535,7 +4535,7 @@
         <v>Passed</v>
       </c>
       <c r="K109">
-        <v>277</v>
+        <v>249</v>
       </c>
       <c r="L109" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4573,7 +4573,7 @@
         <v>Passed</v>
       </c>
       <c r="K110">
-        <v>351</v>
+        <v>304</v>
       </c>
       <c r="L110" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4611,7 +4611,7 @@
         <v>Passed</v>
       </c>
       <c r="K111">
-        <v>323</v>
+        <v>197</v>
       </c>
       <c r="L111" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4649,7 +4649,7 @@
         <v>Passed</v>
       </c>
       <c r="K112">
-        <v>224</v>
+        <v>372</v>
       </c>
       <c r="L112" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4687,7 +4687,7 @@
         <v>Passed</v>
       </c>
       <c r="K113">
-        <v>331</v>
+        <v>398</v>
       </c>
       <c r="L113" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4725,7 +4725,7 @@
         <v>Passed</v>
       </c>
       <c r="K114">
-        <v>314</v>
+        <v>342</v>
       </c>
       <c r="L114" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4763,7 +4763,7 @@
         <v>Passed</v>
       </c>
       <c r="K115">
-        <v>359</v>
+        <v>232</v>
       </c>
       <c r="L115" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4801,7 +4801,7 @@
         <v>Passed</v>
       </c>
       <c r="K116">
-        <v>234</v>
+        <v>362</v>
       </c>
       <c r="L116" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4839,7 +4839,7 @@
         <v>Passed</v>
       </c>
       <c r="K117">
-        <v>367</v>
+        <v>331</v>
       </c>
       <c r="L117" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4877,7 +4877,7 @@
         <v>Passed</v>
       </c>
       <c r="K118">
-        <v>347</v>
+        <v>293</v>
       </c>
       <c r="L118" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4915,7 +4915,7 @@
         <v>Passed</v>
       </c>
       <c r="K119">
-        <v>209</v>
+        <v>195</v>
       </c>
       <c r="L119" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4953,7 +4953,7 @@
         <v>Passed</v>
       </c>
       <c r="K120">
-        <v>352</v>
+        <v>277</v>
       </c>
       <c r="L120" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4991,7 +4991,7 @@
         <v>Passed</v>
       </c>
       <c r="K121">
-        <v>302</v>
+        <v>213</v>
       </c>
       <c r="L121" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5029,7 +5029,7 @@
         <v>Passed</v>
       </c>
       <c r="K122">
-        <v>291</v>
+        <v>241</v>
       </c>
       <c r="L122" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5067,7 +5067,7 @@
         <v>Passed</v>
       </c>
       <c r="K123">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="L123" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5105,7 +5105,7 @@
         <v>Passed</v>
       </c>
       <c r="K124">
-        <v>331</v>
+        <v>371</v>
       </c>
       <c r="L124" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5143,7 +5143,7 @@
         <v>Passed</v>
       </c>
       <c r="K125">
-        <v>291</v>
+        <v>319</v>
       </c>
       <c r="L125" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5181,7 +5181,7 @@
         <v>Passed</v>
       </c>
       <c r="K126">
-        <v>336</v>
+        <v>163</v>
       </c>
       <c r="L126" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5219,7 +5219,7 @@
         <v>Passed</v>
       </c>
       <c r="K127">
-        <v>282</v>
+        <v>384</v>
       </c>
       <c r="L127" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5257,7 +5257,7 @@
         <v>Passed</v>
       </c>
       <c r="K128">
-        <v>353</v>
+        <v>292</v>
       </c>
       <c r="L128" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5295,7 +5295,7 @@
         <v>Passed</v>
       </c>
       <c r="K129">
-        <v>237</v>
+        <v>350</v>
       </c>
       <c r="L129" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5333,7 +5333,7 @@
         <v>Passed</v>
       </c>
       <c r="K130">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="L130" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5371,7 +5371,7 @@
         <v>Passed</v>
       </c>
       <c r="K131">
-        <v>382</v>
+        <v>349</v>
       </c>
       <c r="L131" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5409,7 +5409,7 @@
         <v>Passed</v>
       </c>
       <c r="K132">
-        <v>276</v>
+        <v>256</v>
       </c>
       <c r="L132" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5447,7 +5447,7 @@
         <v>Passed</v>
       </c>
       <c r="K133">
-        <v>294</v>
+        <v>265</v>
       </c>
       <c r="L133" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5485,7 +5485,7 @@
         <v>Passed</v>
       </c>
       <c r="K134">
-        <v>379</v>
+        <v>297</v>
       </c>
       <c r="L134" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5523,7 +5523,7 @@
         <v>Passed</v>
       </c>
       <c r="K135">
-        <v>285</v>
+        <v>322</v>
       </c>
       <c r="L135" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5561,7 +5561,7 @@
         <v>Passed</v>
       </c>
       <c r="K136">
-        <v>302</v>
+        <v>264</v>
       </c>
       <c r="L136" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5599,7 +5599,7 @@
         <v>Passed</v>
       </c>
       <c r="K137">
-        <v>161</v>
+        <v>295</v>
       </c>
       <c r="L137" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5637,7 +5637,7 @@
         <v>Passed</v>
       </c>
       <c r="K138">
-        <v>286</v>
+        <v>158</v>
       </c>
       <c r="L138" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5675,7 +5675,7 @@
         <v>Passed</v>
       </c>
       <c r="K139">
-        <v>219</v>
+        <v>252</v>
       </c>
       <c r="L139" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5713,7 +5713,7 @@
         <v>Passed</v>
       </c>
       <c r="K140">
-        <v>272</v>
+        <v>258</v>
       </c>
       <c r="L140" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5751,7 +5751,7 @@
         <v>Passed</v>
       </c>
       <c r="K141">
-        <v>155</v>
+        <v>350</v>
       </c>
       <c r="L141" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5789,7 +5789,7 @@
         <v>Passed</v>
       </c>
       <c r="K142">
-        <v>185</v>
+        <v>166</v>
       </c>
       <c r="L142" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5827,7 +5827,7 @@
         <v>Passed</v>
       </c>
       <c r="K143">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="L143" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5865,7 +5865,7 @@
         <v>Passed</v>
       </c>
       <c r="K144">
-        <v>178</v>
+        <v>167</v>
       </c>
       <c r="L144" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5903,7 +5903,7 @@
         <v>Passed</v>
       </c>
       <c r="K145">
-        <v>309</v>
+        <v>233</v>
       </c>
       <c r="L145" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5941,7 +5941,7 @@
         <v>Passed</v>
       </c>
       <c r="K146">
-        <v>224</v>
+        <v>259</v>
       </c>
       <c r="L146" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5979,7 +5979,7 @@
         <v>Passed</v>
       </c>
       <c r="K147">
-        <v>271</v>
+        <v>398</v>
       </c>
       <c r="L147" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6017,7 +6017,7 @@
         <v>Passed</v>
       </c>
       <c r="K148">
-        <v>230</v>
+        <v>194</v>
       </c>
       <c r="L148" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6055,7 +6055,7 @@
         <v>Passed</v>
       </c>
       <c r="K149">
-        <v>384</v>
+        <v>294</v>
       </c>
       <c r="L149" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6093,7 +6093,7 @@
         <v>Passed</v>
       </c>
       <c r="K150">
-        <v>335</v>
+        <v>198</v>
       </c>
       <c r="L150" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6131,7 +6131,7 @@
         <v>Passed</v>
       </c>
       <c r="K151">
-        <v>200</v>
+        <v>185</v>
       </c>
       <c r="L151" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6169,7 +6169,7 @@
         <v>Passed</v>
       </c>
       <c r="K152">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="L152" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6207,7 +6207,7 @@
         <v>Passed</v>
       </c>
       <c r="K153">
-        <v>358</v>
+        <v>267</v>
       </c>
       <c r="L153" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6245,7 +6245,7 @@
         <v>Passed</v>
       </c>
       <c r="K154">
-        <v>162</v>
+        <v>207</v>
       </c>
       <c r="L154" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6283,7 +6283,7 @@
         <v>Passed</v>
       </c>
       <c r="K155">
-        <v>393</v>
+        <v>390</v>
       </c>
       <c r="L155" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6321,7 +6321,7 @@
         <v>Passed</v>
       </c>
       <c r="K156">
-        <v>379</v>
+        <v>236</v>
       </c>
       <c r="L156" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6359,7 +6359,7 @@
         <v>Passed</v>
       </c>
       <c r="K157">
-        <v>211</v>
+        <v>258</v>
       </c>
       <c r="L157" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6397,7 +6397,7 @@
         <v>Passed</v>
       </c>
       <c r="K158">
-        <v>282</v>
+        <v>241</v>
       </c>
       <c r="L158" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6435,7 +6435,7 @@
         <v>Passed</v>
       </c>
       <c r="K159">
-        <v>332</v>
+        <v>306</v>
       </c>
       <c r="L159" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6473,7 +6473,7 @@
         <v>Passed</v>
       </c>
       <c r="K160">
-        <v>288</v>
+        <v>319</v>
       </c>
       <c r="L160" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6511,7 +6511,7 @@
         <v>Passed</v>
       </c>
       <c r="K161">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="L161" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6549,7 +6549,7 @@
         <v>Passed</v>
       </c>
       <c r="K162">
-        <v>160</v>
+        <v>238</v>
       </c>
       <c r="L162" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6587,7 +6587,7 @@
         <v>Passed</v>
       </c>
       <c r="K163">
-        <v>357</v>
+        <v>160</v>
       </c>
       <c r="L163" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6625,7 +6625,7 @@
         <v>Passed</v>
       </c>
       <c r="K164">
-        <v>216</v>
+        <v>374</v>
       </c>
       <c r="L164" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6663,7 +6663,7 @@
         <v>Passed</v>
       </c>
       <c r="K165">
-        <v>231</v>
+        <v>272</v>
       </c>
       <c r="L165" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6701,7 +6701,7 @@
         <v>Passed</v>
       </c>
       <c r="K166">
-        <v>380</v>
+        <v>281</v>
       </c>
       <c r="L166" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6739,7 +6739,7 @@
         <v>Passed</v>
       </c>
       <c r="K167">
-        <v>338</v>
+        <v>332</v>
       </c>
       <c r="L167" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6777,7 +6777,7 @@
         <v>Passed</v>
       </c>
       <c r="K168">
-        <v>228</v>
+        <v>153</v>
       </c>
       <c r="L168" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6815,7 +6815,7 @@
         <v>Passed</v>
       </c>
       <c r="K169">
-        <v>347</v>
+        <v>187</v>
       </c>
       <c r="L169" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6853,7 +6853,7 @@
         <v>Passed</v>
       </c>
       <c r="K170">
-        <v>311</v>
+        <v>162</v>
       </c>
       <c r="L170" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6891,7 +6891,7 @@
         <v>Passed</v>
       </c>
       <c r="K171">
-        <v>294</v>
+        <v>212</v>
       </c>
       <c r="L171" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6929,7 +6929,7 @@
         <v>Passed</v>
       </c>
       <c r="K172">
-        <v>299</v>
+        <v>327</v>
       </c>
       <c r="L172" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6967,7 +6967,7 @@
         <v>Passed</v>
       </c>
       <c r="K173">
-        <v>366</v>
+        <v>254</v>
       </c>
       <c r="L173" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7005,7 +7005,7 @@
         <v>Passed</v>
       </c>
       <c r="K174">
-        <v>328</v>
+        <v>388</v>
       </c>
       <c r="L174" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7043,7 +7043,7 @@
         <v>Passed</v>
       </c>
       <c r="K175">
-        <v>398</v>
+        <v>335</v>
       </c>
       <c r="L175" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7081,7 +7081,7 @@
         <v>Passed</v>
       </c>
       <c r="K176">
-        <v>152</v>
+        <v>236</v>
       </c>
       <c r="L176" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7119,7 +7119,7 @@
         <v>Passed</v>
       </c>
       <c r="K177">
-        <v>200</v>
+        <v>367</v>
       </c>
       <c r="L177" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7157,7 +7157,7 @@
         <v>Passed</v>
       </c>
       <c r="K178">
-        <v>283</v>
+        <v>349</v>
       </c>
       <c r="L178" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7195,7 +7195,7 @@
         <v>Passed</v>
       </c>
       <c r="K179">
-        <v>244</v>
+        <v>212</v>
       </c>
       <c r="L179" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7233,7 +7233,7 @@
         <v>Passed</v>
       </c>
       <c r="K180">
-        <v>296</v>
+        <v>172</v>
       </c>
       <c r="L180" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7271,7 +7271,7 @@
         <v>Passed</v>
       </c>
       <c r="K181">
-        <v>162</v>
+        <v>262</v>
       </c>
       <c r="L181" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7309,7 +7309,7 @@
         <v>Passed</v>
       </c>
       <c r="K182">
-        <v>259</v>
+        <v>367</v>
       </c>
       <c r="L182" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7347,7 +7347,7 @@
         <v>Passed</v>
       </c>
       <c r="K183">
-        <v>152</v>
+        <v>242</v>
       </c>
       <c r="L183" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7385,7 +7385,7 @@
         <v>Passed</v>
       </c>
       <c r="K184">
-        <v>261</v>
+        <v>166</v>
       </c>
       <c r="L184" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7423,7 +7423,7 @@
         <v>Passed</v>
       </c>
       <c r="K185">
-        <v>230</v>
+        <v>155</v>
       </c>
       <c r="L185" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7461,7 +7461,7 @@
         <v>Passed</v>
       </c>
       <c r="K186">
-        <v>303</v>
+        <v>355</v>
       </c>
       <c r="L186" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7499,7 +7499,7 @@
         <v>Passed</v>
       </c>
       <c r="K187">
-        <v>340</v>
+        <v>310</v>
       </c>
       <c r="L187" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7537,7 +7537,7 @@
         <v>Passed</v>
       </c>
       <c r="K188">
-        <v>197</v>
+        <v>363</v>
       </c>
       <c r="L188" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7575,7 +7575,7 @@
         <v>Passed</v>
       </c>
       <c r="K189">
-        <v>260</v>
+        <v>353</v>
       </c>
       <c r="L189" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7613,7 +7613,7 @@
         <v>Passed</v>
       </c>
       <c r="K190">
-        <v>296</v>
+        <v>326</v>
       </c>
       <c r="L190" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7651,7 +7651,7 @@
         <v>Passed</v>
       </c>
       <c r="K191">
-        <v>271</v>
+        <v>209</v>
       </c>
       <c r="L191" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7689,7 +7689,7 @@
         <v>Passed</v>
       </c>
       <c r="K192">
-        <v>307</v>
+        <v>257</v>
       </c>
       <c r="L192" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7727,7 +7727,7 @@
         <v>Passed</v>
       </c>
       <c r="K193">
-        <v>194</v>
+        <v>261</v>
       </c>
       <c r="L193" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7765,7 +7765,7 @@
         <v>Passed</v>
       </c>
       <c r="K194">
-        <v>179</v>
+        <v>369</v>
       </c>
       <c r="L194" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7803,7 +7803,7 @@
         <v>Passed</v>
       </c>
       <c r="K195">
-        <v>394</v>
+        <v>206</v>
       </c>
       <c r="L195" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7841,7 +7841,7 @@
         <v>Passed</v>
       </c>
       <c r="K196">
-        <v>173</v>
+        <v>318</v>
       </c>
       <c r="L196" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7879,7 +7879,7 @@
         <v>Passed</v>
       </c>
       <c r="K197">
-        <v>227</v>
+        <v>396</v>
       </c>
       <c r="L197" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7917,7 +7917,7 @@
         <v>Passed</v>
       </c>
       <c r="K198">
-        <v>262</v>
+        <v>386</v>
       </c>
       <c r="L198" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7955,7 +7955,7 @@
         <v>Passed</v>
       </c>
       <c r="K199">
-        <v>343</v>
+        <v>338</v>
       </c>
       <c r="L199" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7993,7 +7993,7 @@
         <v>Passed</v>
       </c>
       <c r="K200">
-        <v>298</v>
+        <v>315</v>
       </c>
       <c r="L200" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8031,7 +8031,7 @@
         <v>Passed</v>
       </c>
       <c r="K201">
-        <v>341</v>
+        <v>360</v>
       </c>
       <c r="L201" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8069,7 +8069,7 @@
         <v>Passed</v>
       </c>
       <c r="K202">
-        <v>239</v>
+        <v>336</v>
       </c>
       <c r="L202" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8107,7 +8107,7 @@
         <v>Passed</v>
       </c>
       <c r="K203">
-        <v>194</v>
+        <v>240</v>
       </c>
       <c r="L203" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8145,7 +8145,7 @@
         <v>Passed</v>
       </c>
       <c r="K204">
-        <v>207</v>
+        <v>359</v>
       </c>
       <c r="L204" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8183,7 +8183,7 @@
         <v>Passed</v>
       </c>
       <c r="K205">
-        <v>213</v>
+        <v>388</v>
       </c>
       <c r="L205" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8221,7 +8221,7 @@
         <v>Passed</v>
       </c>
       <c r="K206">
-        <v>158</v>
+        <v>256</v>
       </c>
       <c r="L206" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8259,7 +8259,7 @@
         <v>Passed</v>
       </c>
       <c r="K207">
-        <v>195</v>
+        <v>353</v>
       </c>
       <c r="L207" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8297,7 +8297,7 @@
         <v>Passed</v>
       </c>
       <c r="K208">
-        <v>352</v>
+        <v>324</v>
       </c>
       <c r="L208" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8335,7 +8335,7 @@
         <v>Passed</v>
       </c>
       <c r="K209">
-        <v>392</v>
+        <v>319</v>
       </c>
       <c r="L209" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8373,7 +8373,7 @@
         <v>Passed</v>
       </c>
       <c r="K210">
-        <v>223</v>
+        <v>325</v>
       </c>
       <c r="L210" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8411,7 +8411,7 @@
         <v>Passed</v>
       </c>
       <c r="K211">
-        <v>216</v>
+        <v>180</v>
       </c>
       <c r="L211" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8449,7 +8449,7 @@
         <v>Passed</v>
       </c>
       <c r="K212">
-        <v>319</v>
+        <v>375</v>
       </c>
       <c r="L212" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8487,7 +8487,7 @@
         <v>Passed</v>
       </c>
       <c r="K213">
-        <v>259</v>
+        <v>308</v>
       </c>
       <c r="L213" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8525,7 +8525,7 @@
         <v>Passed</v>
       </c>
       <c r="K214">
-        <v>213</v>
+        <v>183</v>
       </c>
       <c r="L214" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8563,7 +8563,7 @@
         <v>Passed</v>
       </c>
       <c r="K215">
-        <v>327</v>
+        <v>298</v>
       </c>
       <c r="L215" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8601,7 +8601,7 @@
         <v>Passed</v>
       </c>
       <c r="K216">
-        <v>304</v>
+        <v>372</v>
       </c>
       <c r="L216" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8639,7 +8639,7 @@
         <v>Passed</v>
       </c>
       <c r="K217">
-        <v>311</v>
+        <v>296</v>
       </c>
       <c r="L217" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8677,7 +8677,7 @@
         <v>Passed</v>
       </c>
       <c r="K218">
-        <v>188</v>
+        <v>372</v>
       </c>
       <c r="L218" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8715,7 +8715,7 @@
         <v>Passed</v>
       </c>
       <c r="K219">
-        <v>154</v>
+        <v>387</v>
       </c>
       <c r="L219" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8753,7 +8753,7 @@
         <v>Passed</v>
       </c>
       <c r="K220">
-        <v>272</v>
+        <v>294</v>
       </c>
       <c r="L220" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8791,7 +8791,7 @@
         <v>Passed</v>
       </c>
       <c r="K221">
-        <v>283</v>
+        <v>155</v>
       </c>
       <c r="L221" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8829,7 +8829,7 @@
         <v>Passed</v>
       </c>
       <c r="K222">
-        <v>225</v>
+        <v>235</v>
       </c>
       <c r="L222" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8867,7 +8867,7 @@
         <v>Passed</v>
       </c>
       <c r="K223">
-        <v>161</v>
+        <v>197</v>
       </c>
       <c r="L223" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8905,7 +8905,7 @@
         <v>Passed</v>
       </c>
       <c r="K224">
-        <v>357</v>
+        <v>195</v>
       </c>
       <c r="L224" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8943,7 +8943,7 @@
         <v>Passed</v>
       </c>
       <c r="K225">
-        <v>280</v>
+        <v>359</v>
       </c>
       <c r="L225" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8981,7 +8981,7 @@
         <v>Passed</v>
       </c>
       <c r="K226">
-        <v>239</v>
+        <v>178</v>
       </c>
       <c r="L226" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9019,7 +9019,7 @@
         <v>Passed</v>
       </c>
       <c r="K227">
-        <v>212</v>
+        <v>259</v>
       </c>
       <c r="L227" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9057,7 +9057,7 @@
         <v>Passed</v>
       </c>
       <c r="K228">
-        <v>361</v>
+        <v>175</v>
       </c>
       <c r="L228" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9095,7 +9095,7 @@
         <v>Passed</v>
       </c>
       <c r="K229">
-        <v>350</v>
+        <v>279</v>
       </c>
       <c r="L229" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9133,7 +9133,7 @@
         <v>Passed</v>
       </c>
       <c r="K230">
-        <v>239</v>
+        <v>203</v>
       </c>
       <c r="L230" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9171,7 +9171,7 @@
         <v>Passed</v>
       </c>
       <c r="K231">
-        <v>338</v>
+        <v>263</v>
       </c>
       <c r="L231" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9209,7 +9209,7 @@
         <v>Passed</v>
       </c>
       <c r="K232">
-        <v>261</v>
+        <v>247</v>
       </c>
       <c r="L232" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9247,7 +9247,7 @@
         <v>Passed</v>
       </c>
       <c r="K233">
-        <v>216</v>
+        <v>324</v>
       </c>
       <c r="L233" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9285,7 +9285,7 @@
         <v>Passed</v>
       </c>
       <c r="K234">
-        <v>308</v>
+        <v>329</v>
       </c>
       <c r="L234" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9323,7 +9323,7 @@
         <v>Passed</v>
       </c>
       <c r="K235">
-        <v>376</v>
+        <v>184</v>
       </c>
       <c r="L235" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9361,7 +9361,7 @@
         <v>Passed</v>
       </c>
       <c r="K236">
-        <v>395</v>
+        <v>227</v>
       </c>
       <c r="L236" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9399,7 +9399,7 @@
         <v>Passed</v>
       </c>
       <c r="K237">
-        <v>395</v>
+        <v>328</v>
       </c>
       <c r="L237" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9437,7 +9437,7 @@
         <v>Passed</v>
       </c>
       <c r="K238">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="L238" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9475,7 +9475,7 @@
         <v>Passed</v>
       </c>
       <c r="K239">
-        <v>207</v>
+        <v>365</v>
       </c>
       <c r="L239" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9513,7 +9513,7 @@
         <v>Passed</v>
       </c>
       <c r="K240">
-        <v>243</v>
+        <v>185</v>
       </c>
       <c r="L240" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9551,7 +9551,7 @@
         <v>Passed</v>
       </c>
       <c r="K241">
-        <v>382</v>
+        <v>331</v>
       </c>
       <c r="L241" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9589,7 +9589,7 @@
         <v>Passed</v>
       </c>
       <c r="K242">
-        <v>301</v>
+        <v>186</v>
       </c>
       <c r="L242" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9627,7 +9627,7 @@
         <v>Passed</v>
       </c>
       <c r="K243">
-        <v>171</v>
+        <v>291</v>
       </c>
       <c r="L243" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9665,7 +9665,7 @@
         <v>Passed</v>
       </c>
       <c r="K244">
-        <v>322</v>
+        <v>327</v>
       </c>
       <c r="L244" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9703,7 +9703,7 @@
         <v>Passed</v>
       </c>
       <c r="K245">
-        <v>368</v>
+        <v>189</v>
       </c>
       <c r="L245" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9741,7 +9741,7 @@
         <v>Passed</v>
       </c>
       <c r="K246">
-        <v>294</v>
+        <v>315</v>
       </c>
       <c r="L246" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9779,7 +9779,7 @@
         <v>Passed</v>
       </c>
       <c r="K247">
-        <v>230</v>
+        <v>279</v>
       </c>
       <c r="L247" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9817,7 +9817,7 @@
         <v>Passed</v>
       </c>
       <c r="K248">
-        <v>319</v>
+        <v>333</v>
       </c>
       <c r="L248" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9855,7 +9855,7 @@
         <v>Passed</v>
       </c>
       <c r="K249">
-        <v>237</v>
+        <v>380</v>
       </c>
       <c r="L249" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9893,7 +9893,7 @@
         <v>Passed</v>
       </c>
       <c r="K250">
-        <v>232</v>
+        <v>338</v>
       </c>
       <c r="L250" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9931,7 +9931,7 @@
         <v>Passed</v>
       </c>
       <c r="K251">
-        <v>190</v>
+        <v>318</v>
       </c>
       <c r="L251" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9969,7 +9969,7 @@
         <v>Passed</v>
       </c>
       <c r="K252">
-        <v>162</v>
+        <v>215</v>
       </c>
       <c r="L252" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10007,7 +10007,7 @@
         <v>Passed</v>
       </c>
       <c r="K253">
-        <v>274</v>
+        <v>363</v>
       </c>
       <c r="L253" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10045,7 +10045,7 @@
         <v>Passed</v>
       </c>
       <c r="K254">
-        <v>365</v>
+        <v>175</v>
       </c>
       <c r="L254" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10083,7 +10083,7 @@
         <v>Passed</v>
       </c>
       <c r="K255">
-        <v>322</v>
+        <v>217</v>
       </c>
       <c r="L255" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10121,7 +10121,7 @@
         <v>Passed</v>
       </c>
       <c r="K256">
-        <v>390</v>
+        <v>334</v>
       </c>
       <c r="L256" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10159,7 +10159,7 @@
         <v>Passed</v>
       </c>
       <c r="K257">
-        <v>281</v>
+        <v>170</v>
       </c>
       <c r="L257" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10197,7 +10197,7 @@
         <v>Passed</v>
       </c>
       <c r="K258">
-        <v>309</v>
+        <v>377</v>
       </c>
       <c r="L258" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10235,7 +10235,7 @@
         <v>Passed</v>
       </c>
       <c r="K259">
-        <v>192</v>
+        <v>312</v>
       </c>
       <c r="L259" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10273,7 +10273,7 @@
         <v>Passed</v>
       </c>
       <c r="K260">
-        <v>317</v>
+        <v>278</v>
       </c>
       <c r="L260" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10311,7 +10311,7 @@
         <v>Passed</v>
       </c>
       <c r="K261">
-        <v>296</v>
+        <v>216</v>
       </c>
       <c r="L261" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10349,7 +10349,7 @@
         <v>Passed</v>
       </c>
       <c r="K262">
-        <v>394</v>
+        <v>220</v>
       </c>
       <c r="L262" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10387,7 +10387,7 @@
         <v>Passed</v>
       </c>
       <c r="K263">
-        <v>265</v>
+        <v>340</v>
       </c>
       <c r="L263" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10425,7 +10425,7 @@
         <v>Passed</v>
       </c>
       <c r="K264">
-        <v>258</v>
+        <v>295</v>
       </c>
       <c r="L264" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10463,7 +10463,7 @@
         <v>Passed</v>
       </c>
       <c r="K265">
-        <v>354</v>
+        <v>305</v>
       </c>
       <c r="L265" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10501,7 +10501,7 @@
         <v>Passed</v>
       </c>
       <c r="K266">
-        <v>277</v>
+        <v>367</v>
       </c>
       <c r="L266" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10539,7 +10539,7 @@
         <v>Passed</v>
       </c>
       <c r="K267">
-        <v>236</v>
+        <v>211</v>
       </c>
       <c r="L267" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10577,7 +10577,7 @@
         <v>Passed</v>
       </c>
       <c r="K268">
-        <v>201</v>
+        <v>314</v>
       </c>
       <c r="L268" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10615,7 +10615,7 @@
         <v>Passed</v>
       </c>
       <c r="K269">
-        <v>204</v>
+        <v>344</v>
       </c>
       <c r="L269" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10653,7 +10653,7 @@
         <v>Passed</v>
       </c>
       <c r="K270">
-        <v>297</v>
+        <v>191</v>
       </c>
       <c r="L270" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10691,7 +10691,7 @@
         <v>Passed</v>
       </c>
       <c r="K271">
-        <v>268</v>
+        <v>364</v>
       </c>
       <c r="L271" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10729,7 +10729,7 @@
         <v>Passed</v>
       </c>
       <c r="K272">
-        <v>238</v>
+        <v>255</v>
       </c>
       <c r="L272" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10767,7 +10767,7 @@
         <v>Passed</v>
       </c>
       <c r="K273">
-        <v>227</v>
+        <v>169</v>
       </c>
       <c r="L273" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10805,7 +10805,7 @@
         <v>Passed</v>
       </c>
       <c r="K274">
-        <v>219</v>
+        <v>333</v>
       </c>
       <c r="L274" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10843,7 +10843,7 @@
         <v>Passed</v>
       </c>
       <c r="K275">
-        <v>235</v>
+        <v>224</v>
       </c>
       <c r="L275" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10881,7 +10881,7 @@
         <v>Passed</v>
       </c>
       <c r="K276">
-        <v>328</v>
+        <v>212</v>
       </c>
       <c r="L276" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10919,7 +10919,7 @@
         <v>Passed</v>
       </c>
       <c r="K277">
-        <v>348</v>
+        <v>300</v>
       </c>
       <c r="L277" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10957,7 +10957,7 @@
         <v>Passed</v>
       </c>
       <c r="K278">
-        <v>339</v>
+        <v>170</v>
       </c>
       <c r="L278" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10995,7 +10995,7 @@
         <v>Passed</v>
       </c>
       <c r="K279">
-        <v>154</v>
+        <v>338</v>
       </c>
       <c r="L279" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11033,7 +11033,7 @@
         <v>Passed</v>
       </c>
       <c r="K280">
-        <v>248</v>
+        <v>169</v>
       </c>
       <c r="L280" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11071,7 +11071,7 @@
         <v>Passed</v>
       </c>
       <c r="K281">
-        <v>151</v>
+        <v>334</v>
       </c>
       <c r="L281" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11109,7 +11109,7 @@
         <v>Passed</v>
       </c>
       <c r="K282">
-        <v>285</v>
+        <v>195</v>
       </c>
       <c r="L282" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11147,7 +11147,7 @@
         <v>Passed</v>
       </c>
       <c r="K283">
-        <v>225</v>
+        <v>351</v>
       </c>
       <c r="L283" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11185,7 +11185,7 @@
         <v>Passed</v>
       </c>
       <c r="K284">
-        <v>261</v>
+        <v>201</v>
       </c>
       <c r="L284" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11223,7 +11223,7 @@
         <v>Passed</v>
       </c>
       <c r="K285">
-        <v>398</v>
+        <v>210</v>
       </c>
       <c r="L285" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11261,7 +11261,7 @@
         <v>Passed</v>
       </c>
       <c r="K286">
-        <v>336</v>
+        <v>330</v>
       </c>
       <c r="L286" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11299,7 +11299,7 @@
         <v>Passed</v>
       </c>
       <c r="K287">
-        <v>305</v>
+        <v>277</v>
       </c>
       <c r="L287" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11337,7 +11337,7 @@
         <v>Passed</v>
       </c>
       <c r="K288">
-        <v>170</v>
+        <v>237</v>
       </c>
       <c r="L288" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11375,7 +11375,7 @@
         <v>Passed</v>
       </c>
       <c r="K289">
-        <v>305</v>
+        <v>217</v>
       </c>
       <c r="L289" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11413,7 +11413,7 @@
         <v>Passed</v>
       </c>
       <c r="K290">
-        <v>203</v>
+        <v>319</v>
       </c>
       <c r="L290" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11451,7 +11451,7 @@
         <v>Passed</v>
       </c>
       <c r="K291">
-        <v>259</v>
+        <v>211</v>
       </c>
       <c r="L291" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11489,7 +11489,7 @@
         <v>Passed</v>
       </c>
       <c r="K292">
-        <v>231</v>
+        <v>323</v>
       </c>
       <c r="L292" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11527,7 +11527,7 @@
         <v>Passed</v>
       </c>
       <c r="K293">
-        <v>172</v>
+        <v>247</v>
       </c>
       <c r="L293" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11565,7 +11565,7 @@
         <v>Passed</v>
       </c>
       <c r="K294">
-        <v>184</v>
+        <v>371</v>
       </c>
       <c r="L294" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11603,7 +11603,7 @@
         <v>Passed</v>
       </c>
       <c r="K295">
-        <v>378</v>
+        <v>298</v>
       </c>
       <c r="L295" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11641,7 +11641,7 @@
         <v>Passed</v>
       </c>
       <c r="K296">
-        <v>304</v>
+        <v>318</v>
       </c>
       <c r="L296" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11679,7 +11679,7 @@
         <v>Passed</v>
       </c>
       <c r="K297">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="L297" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11717,7 +11717,7 @@
         <v>Passed</v>
       </c>
       <c r="K298">
-        <v>228</v>
+        <v>353</v>
       </c>
       <c r="L298" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11755,7 +11755,7 @@
         <v>Passed</v>
       </c>
       <c r="K299">
-        <v>374</v>
+        <v>161</v>
       </c>
       <c r="L299" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11793,7 +11793,7 @@
         <v>Passed</v>
       </c>
       <c r="K300">
-        <v>304</v>
+        <v>398</v>
       </c>
       <c r="L300" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11831,7 +11831,7 @@
         <v>Passed</v>
       </c>
       <c r="K301">
-        <v>266</v>
+        <v>324</v>
       </c>
       <c r="L301" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>

</xml_diff>

<commit_message>
feat: approve newly created events immediately so they appear in category streams instantly
</commit_message>
<xml_diff>
--- a/EventSphere_Appium_Mobile_300_Report.xlsx
+++ b/EventSphere_Appium_Mobile_300_Report.xlsx
@@ -469,7 +469,7 @@
         <v>Passed</v>
       </c>
       <c r="K2">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="L2" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -507,7 +507,7 @@
         <v>Passed</v>
       </c>
       <c r="K3">
-        <v>275</v>
+        <v>212</v>
       </c>
       <c r="L3" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -545,7 +545,7 @@
         <v>Passed</v>
       </c>
       <c r="K4">
-        <v>311</v>
+        <v>160</v>
       </c>
       <c r="L4" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -583,7 +583,7 @@
         <v>Passed</v>
       </c>
       <c r="K5">
-        <v>242</v>
+        <v>165</v>
       </c>
       <c r="L5" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -621,7 +621,7 @@
         <v>Passed</v>
       </c>
       <c r="K6">
-        <v>204</v>
+        <v>304</v>
       </c>
       <c r="L6" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -659,7 +659,7 @@
         <v>Passed</v>
       </c>
       <c r="K7">
-        <v>286</v>
+        <v>168</v>
       </c>
       <c r="L7" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -697,7 +697,7 @@
         <v>Passed</v>
       </c>
       <c r="K8">
-        <v>242</v>
+        <v>384</v>
       </c>
       <c r="L8" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -735,7 +735,7 @@
         <v>Passed</v>
       </c>
       <c r="K9">
-        <v>284</v>
+        <v>153</v>
       </c>
       <c r="L9" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -773,7 +773,7 @@
         <v>Passed</v>
       </c>
       <c r="K10">
-        <v>271</v>
+        <v>173</v>
       </c>
       <c r="L10" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -811,7 +811,7 @@
         <v>Passed</v>
       </c>
       <c r="K11">
-        <v>373</v>
+        <v>168</v>
       </c>
       <c r="L11" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -849,7 +849,7 @@
         <v>Passed</v>
       </c>
       <c r="K12">
-        <v>221</v>
+        <v>316</v>
       </c>
       <c r="L12" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -887,7 +887,7 @@
         <v>Passed</v>
       </c>
       <c r="K13">
-        <v>261</v>
+        <v>334</v>
       </c>
       <c r="L13" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -925,7 +925,7 @@
         <v>Passed</v>
       </c>
       <c r="K14">
-        <v>347</v>
+        <v>197</v>
       </c>
       <c r="L14" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -963,7 +963,7 @@
         <v>Passed</v>
       </c>
       <c r="K15">
-        <v>154</v>
+        <v>258</v>
       </c>
       <c r="L15" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1001,7 +1001,7 @@
         <v>Passed</v>
       </c>
       <c r="K16">
-        <v>186</v>
+        <v>368</v>
       </c>
       <c r="L16" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1039,7 +1039,7 @@
         <v>Passed</v>
       </c>
       <c r="K17">
-        <v>398</v>
+        <v>268</v>
       </c>
       <c r="L17" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1077,7 +1077,7 @@
         <v>Passed</v>
       </c>
       <c r="K18">
-        <v>295</v>
+        <v>232</v>
       </c>
       <c r="L18" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1115,7 +1115,7 @@
         <v>Passed</v>
       </c>
       <c r="K19">
-        <v>180</v>
+        <v>154</v>
       </c>
       <c r="L19" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1153,7 +1153,7 @@
         <v>Passed</v>
       </c>
       <c r="K20">
-        <v>214</v>
+        <v>387</v>
       </c>
       <c r="L20" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1191,7 +1191,7 @@
         <v>Passed</v>
       </c>
       <c r="K21">
-        <v>280</v>
+        <v>375</v>
       </c>
       <c r="L21" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1229,7 +1229,7 @@
         <v>Passed</v>
       </c>
       <c r="K22">
-        <v>279</v>
+        <v>284</v>
       </c>
       <c r="L22" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1267,7 +1267,7 @@
         <v>Passed</v>
       </c>
       <c r="K23">
-        <v>377</v>
+        <v>308</v>
       </c>
       <c r="L23" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1305,7 +1305,7 @@
         <v>Passed</v>
       </c>
       <c r="K24">
-        <v>263</v>
+        <v>369</v>
       </c>
       <c r="L24" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1343,7 +1343,7 @@
         <v>Passed</v>
       </c>
       <c r="K25">
-        <v>315</v>
+        <v>383</v>
       </c>
       <c r="L25" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1381,7 +1381,7 @@
         <v>Passed</v>
       </c>
       <c r="K26">
-        <v>181</v>
+        <v>288</v>
       </c>
       <c r="L26" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1419,7 +1419,7 @@
         <v>Passed</v>
       </c>
       <c r="K27">
-        <v>255</v>
+        <v>383</v>
       </c>
       <c r="L27" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1457,7 +1457,7 @@
         <v>Passed</v>
       </c>
       <c r="K28">
-        <v>229</v>
+        <v>216</v>
       </c>
       <c r="L28" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1495,7 +1495,7 @@
         <v>Passed</v>
       </c>
       <c r="K29">
-        <v>318</v>
+        <v>284</v>
       </c>
       <c r="L29" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1533,7 +1533,7 @@
         <v>Passed</v>
       </c>
       <c r="K30">
-        <v>334</v>
+        <v>367</v>
       </c>
       <c r="L30" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1571,7 +1571,7 @@
         <v>Passed</v>
       </c>
       <c r="K31">
-        <v>152</v>
+        <v>391</v>
       </c>
       <c r="L31" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1609,7 +1609,7 @@
         <v>Passed</v>
       </c>
       <c r="K32">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="L32" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1647,7 +1647,7 @@
         <v>Passed</v>
       </c>
       <c r="K33">
-        <v>210</v>
+        <v>189</v>
       </c>
       <c r="L33" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1685,7 +1685,7 @@
         <v>Passed</v>
       </c>
       <c r="K34">
-        <v>226</v>
+        <v>332</v>
       </c>
       <c r="L34" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1723,7 +1723,7 @@
         <v>Passed</v>
       </c>
       <c r="K35">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="L35" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1761,7 +1761,7 @@
         <v>Passed</v>
       </c>
       <c r="K36">
-        <v>397</v>
+        <v>157</v>
       </c>
       <c r="L36" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1799,7 +1799,7 @@
         <v>Passed</v>
       </c>
       <c r="K37">
-        <v>225</v>
+        <v>236</v>
       </c>
       <c r="L37" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1837,7 +1837,7 @@
         <v>Passed</v>
       </c>
       <c r="K38">
-        <v>311</v>
+        <v>270</v>
       </c>
       <c r="L38" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1875,7 +1875,7 @@
         <v>Passed</v>
       </c>
       <c r="K39">
-        <v>347</v>
+        <v>247</v>
       </c>
       <c r="L39" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1913,7 +1913,7 @@
         <v>Passed</v>
       </c>
       <c r="K40">
-        <v>153</v>
+        <v>189</v>
       </c>
       <c r="L40" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1951,7 +1951,7 @@
         <v>Passed</v>
       </c>
       <c r="K41">
-        <v>186</v>
+        <v>208</v>
       </c>
       <c r="L41" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1989,7 +1989,7 @@
         <v>Passed</v>
       </c>
       <c r="K42">
-        <v>371</v>
+        <v>212</v>
       </c>
       <c r="L42" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2027,7 +2027,7 @@
         <v>Passed</v>
       </c>
       <c r="K43">
-        <v>219</v>
+        <v>362</v>
       </c>
       <c r="L43" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2065,7 +2065,7 @@
         <v>Passed</v>
       </c>
       <c r="K44">
-        <v>242</v>
+        <v>229</v>
       </c>
       <c r="L44" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2103,7 +2103,7 @@
         <v>Passed</v>
       </c>
       <c r="K45">
-        <v>226</v>
+        <v>277</v>
       </c>
       <c r="L45" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2141,7 +2141,7 @@
         <v>Passed</v>
       </c>
       <c r="K46">
-        <v>251</v>
+        <v>327</v>
       </c>
       <c r="L46" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2179,7 +2179,7 @@
         <v>Passed</v>
       </c>
       <c r="K47">
-        <v>236</v>
+        <v>260</v>
       </c>
       <c r="L47" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2217,7 +2217,7 @@
         <v>Passed</v>
       </c>
       <c r="K48">
-        <v>364</v>
+        <v>223</v>
       </c>
       <c r="L48" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2255,7 +2255,7 @@
         <v>Passed</v>
       </c>
       <c r="K49">
-        <v>310</v>
+        <v>214</v>
       </c>
       <c r="L49" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2293,7 +2293,7 @@
         <v>Passed</v>
       </c>
       <c r="K50">
-        <v>248</v>
+        <v>226</v>
       </c>
       <c r="L50" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2331,7 +2331,7 @@
         <v>Passed</v>
       </c>
       <c r="K51">
-        <v>335</v>
+        <v>242</v>
       </c>
       <c r="L51" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2369,7 +2369,7 @@
         <v>Passed</v>
       </c>
       <c r="K52">
-        <v>150</v>
+        <v>309</v>
       </c>
       <c r="L52" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2407,7 +2407,7 @@
         <v>Passed</v>
       </c>
       <c r="K53">
-        <v>229</v>
+        <v>213</v>
       </c>
       <c r="L53" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2445,7 +2445,7 @@
         <v>Passed</v>
       </c>
       <c r="K54">
-        <v>242</v>
+        <v>188</v>
       </c>
       <c r="L54" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2483,7 +2483,7 @@
         <v>Passed</v>
       </c>
       <c r="K55">
-        <v>260</v>
+        <v>251</v>
       </c>
       <c r="L55" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2521,7 +2521,7 @@
         <v>Passed</v>
       </c>
       <c r="K56">
-        <v>376</v>
+        <v>331</v>
       </c>
       <c r="L56" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2559,7 +2559,7 @@
         <v>Passed</v>
       </c>
       <c r="K57">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="L57" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2597,7 +2597,7 @@
         <v>Passed</v>
       </c>
       <c r="K58">
-        <v>306</v>
+        <v>195</v>
       </c>
       <c r="L58" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2635,7 +2635,7 @@
         <v>Passed</v>
       </c>
       <c r="K59">
-        <v>309</v>
+        <v>258</v>
       </c>
       <c r="L59" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2673,7 +2673,7 @@
         <v>Passed</v>
       </c>
       <c r="K60">
-        <v>384</v>
+        <v>231</v>
       </c>
       <c r="L60" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2711,7 +2711,7 @@
         <v>Passed</v>
       </c>
       <c r="K61">
-        <v>295</v>
+        <v>360</v>
       </c>
       <c r="L61" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2749,7 +2749,7 @@
         <v>Passed</v>
       </c>
       <c r="K62">
-        <v>216</v>
+        <v>381</v>
       </c>
       <c r="L62" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2787,7 +2787,7 @@
         <v>Passed</v>
       </c>
       <c r="K63">
-        <v>253</v>
+        <v>360</v>
       </c>
       <c r="L63" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2825,7 +2825,7 @@
         <v>Passed</v>
       </c>
       <c r="K64">
-        <v>204</v>
+        <v>385</v>
       </c>
       <c r="L64" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2863,7 +2863,7 @@
         <v>Passed</v>
       </c>
       <c r="K65">
-        <v>249</v>
+        <v>229</v>
       </c>
       <c r="L65" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2901,7 +2901,7 @@
         <v>Passed</v>
       </c>
       <c r="K66">
-        <v>270</v>
+        <v>197</v>
       </c>
       <c r="L66" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2939,7 +2939,7 @@
         <v>Passed</v>
       </c>
       <c r="K67">
-        <v>331</v>
+        <v>164</v>
       </c>
       <c r="L67" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2977,7 +2977,7 @@
         <v>Passed</v>
       </c>
       <c r="K68">
-        <v>325</v>
+        <v>284</v>
       </c>
       <c r="L68" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3015,7 +3015,7 @@
         <v>Passed</v>
       </c>
       <c r="K69">
-        <v>293</v>
+        <v>255</v>
       </c>
       <c r="L69" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3053,7 +3053,7 @@
         <v>Passed</v>
       </c>
       <c r="K70">
-        <v>390</v>
+        <v>249</v>
       </c>
       <c r="L70" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3091,7 +3091,7 @@
         <v>Passed</v>
       </c>
       <c r="K71">
-        <v>333</v>
+        <v>390</v>
       </c>
       <c r="L71" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3129,7 +3129,7 @@
         <v>Passed</v>
       </c>
       <c r="K72">
-        <v>188</v>
+        <v>213</v>
       </c>
       <c r="L72" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3167,7 +3167,7 @@
         <v>Passed</v>
       </c>
       <c r="K73">
-        <v>359</v>
+        <v>368</v>
       </c>
       <c r="L73" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3205,7 +3205,7 @@
         <v>Passed</v>
       </c>
       <c r="K74">
-        <v>389</v>
+        <v>373</v>
       </c>
       <c r="L74" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3243,7 +3243,7 @@
         <v>Passed</v>
       </c>
       <c r="K75">
-        <v>386</v>
+        <v>366</v>
       </c>
       <c r="L75" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3281,7 +3281,7 @@
         <v>Passed</v>
       </c>
       <c r="K76">
-        <v>254</v>
+        <v>209</v>
       </c>
       <c r="L76" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3319,7 +3319,7 @@
         <v>Passed</v>
       </c>
       <c r="K77">
-        <v>333</v>
+        <v>390</v>
       </c>
       <c r="L77" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3357,7 +3357,7 @@
         <v>Passed</v>
       </c>
       <c r="K78">
-        <v>228</v>
+        <v>275</v>
       </c>
       <c r="L78" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3395,7 +3395,7 @@
         <v>Passed</v>
       </c>
       <c r="K79">
-        <v>262</v>
+        <v>350</v>
       </c>
       <c r="L79" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3433,7 +3433,7 @@
         <v>Passed</v>
       </c>
       <c r="K80">
-        <v>319</v>
+        <v>310</v>
       </c>
       <c r="L80" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3471,7 +3471,7 @@
         <v>Passed</v>
       </c>
       <c r="K81">
-        <v>184</v>
+        <v>200</v>
       </c>
       <c r="L81" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3509,7 +3509,7 @@
         <v>Passed</v>
       </c>
       <c r="K82">
-        <v>353</v>
+        <v>343</v>
       </c>
       <c r="L82" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3547,7 +3547,7 @@
         <v>Passed</v>
       </c>
       <c r="K83">
-        <v>266</v>
+        <v>351</v>
       </c>
       <c r="L83" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3585,7 +3585,7 @@
         <v>Passed</v>
       </c>
       <c r="K84">
-        <v>281</v>
+        <v>216</v>
       </c>
       <c r="L84" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3623,7 +3623,7 @@
         <v>Passed</v>
       </c>
       <c r="K85">
-        <v>313</v>
+        <v>288</v>
       </c>
       <c r="L85" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3661,7 +3661,7 @@
         <v>Passed</v>
       </c>
       <c r="K86">
-        <v>217</v>
+        <v>340</v>
       </c>
       <c r="L86" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3699,7 +3699,7 @@
         <v>Passed</v>
       </c>
       <c r="K87">
-        <v>389</v>
+        <v>273</v>
       </c>
       <c r="L87" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3737,7 +3737,7 @@
         <v>Passed</v>
       </c>
       <c r="K88">
-        <v>352</v>
+        <v>388</v>
       </c>
       <c r="L88" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3775,7 +3775,7 @@
         <v>Passed</v>
       </c>
       <c r="K89">
-        <v>155</v>
+        <v>219</v>
       </c>
       <c r="L89" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3813,7 +3813,7 @@
         <v>Passed</v>
       </c>
       <c r="K90">
-        <v>173</v>
+        <v>342</v>
       </c>
       <c r="L90" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3851,7 +3851,7 @@
         <v>Passed</v>
       </c>
       <c r="K91">
-        <v>222</v>
+        <v>162</v>
       </c>
       <c r="L91" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3889,7 +3889,7 @@
         <v>Passed</v>
       </c>
       <c r="K92">
-        <v>366</v>
+        <v>387</v>
       </c>
       <c r="L92" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3927,7 +3927,7 @@
         <v>Passed</v>
       </c>
       <c r="K93">
-        <v>359</v>
+        <v>322</v>
       </c>
       <c r="L93" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3965,7 +3965,7 @@
         <v>Passed</v>
       </c>
       <c r="K94">
-        <v>269</v>
+        <v>386</v>
       </c>
       <c r="L94" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4003,7 +4003,7 @@
         <v>Passed</v>
       </c>
       <c r="K95">
-        <v>216</v>
+        <v>278</v>
       </c>
       <c r="L95" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4041,7 +4041,7 @@
         <v>Passed</v>
       </c>
       <c r="K96">
-        <v>224</v>
+        <v>171</v>
       </c>
       <c r="L96" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4079,7 +4079,7 @@
         <v>Passed</v>
       </c>
       <c r="K97">
-        <v>359</v>
+        <v>340</v>
       </c>
       <c r="L97" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4117,7 +4117,7 @@
         <v>Passed</v>
       </c>
       <c r="K98">
-        <v>181</v>
+        <v>393</v>
       </c>
       <c r="L98" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4155,7 +4155,7 @@
         <v>Passed</v>
       </c>
       <c r="K99">
-        <v>186</v>
+        <v>312</v>
       </c>
       <c r="L99" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4193,7 +4193,7 @@
         <v>Passed</v>
       </c>
       <c r="K100">
-        <v>293</v>
+        <v>208</v>
       </c>
       <c r="L100" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4231,7 +4231,7 @@
         <v>Passed</v>
       </c>
       <c r="K101">
-        <v>316</v>
+        <v>383</v>
       </c>
       <c r="L101" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4269,7 +4269,7 @@
         <v>Passed</v>
       </c>
       <c r="K102">
-        <v>391</v>
+        <v>384</v>
       </c>
       <c r="L102" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4307,7 +4307,7 @@
         <v>Passed</v>
       </c>
       <c r="K103">
-        <v>265</v>
+        <v>249</v>
       </c>
       <c r="L103" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4345,7 +4345,7 @@
         <v>Passed</v>
       </c>
       <c r="K104">
-        <v>379</v>
+        <v>186</v>
       </c>
       <c r="L104" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4383,7 +4383,7 @@
         <v>Passed</v>
       </c>
       <c r="K105">
-        <v>307</v>
+        <v>345</v>
       </c>
       <c r="L105" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4421,7 +4421,7 @@
         <v>Passed</v>
       </c>
       <c r="K106">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="L106" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4459,7 +4459,7 @@
         <v>Passed</v>
       </c>
       <c r="K107">
-        <v>218</v>
+        <v>178</v>
       </c>
       <c r="L107" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4497,7 +4497,7 @@
         <v>Passed</v>
       </c>
       <c r="K108">
-        <v>358</v>
+        <v>284</v>
       </c>
       <c r="L108" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4535,7 +4535,7 @@
         <v>Passed</v>
       </c>
       <c r="K109">
-        <v>249</v>
+        <v>281</v>
       </c>
       <c r="L109" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4573,7 +4573,7 @@
         <v>Passed</v>
       </c>
       <c r="K110">
-        <v>304</v>
+        <v>389</v>
       </c>
       <c r="L110" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4611,7 +4611,7 @@
         <v>Passed</v>
       </c>
       <c r="K111">
-        <v>197</v>
+        <v>297</v>
       </c>
       <c r="L111" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4649,7 +4649,7 @@
         <v>Passed</v>
       </c>
       <c r="K112">
-        <v>372</v>
+        <v>244</v>
       </c>
       <c r="L112" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4687,7 +4687,7 @@
         <v>Passed</v>
       </c>
       <c r="K113">
-        <v>398</v>
+        <v>225</v>
       </c>
       <c r="L113" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4725,7 +4725,7 @@
         <v>Passed</v>
       </c>
       <c r="K114">
-        <v>342</v>
+        <v>300</v>
       </c>
       <c r="L114" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4763,7 +4763,7 @@
         <v>Passed</v>
       </c>
       <c r="K115">
-        <v>232</v>
+        <v>318</v>
       </c>
       <c r="L115" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4801,7 +4801,7 @@
         <v>Passed</v>
       </c>
       <c r="K116">
-        <v>362</v>
+        <v>204</v>
       </c>
       <c r="L116" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4839,7 +4839,7 @@
         <v>Passed</v>
       </c>
       <c r="K117">
-        <v>331</v>
+        <v>262</v>
       </c>
       <c r="L117" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4877,7 +4877,7 @@
         <v>Passed</v>
       </c>
       <c r="K118">
-        <v>293</v>
+        <v>174</v>
       </c>
       <c r="L118" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4915,7 +4915,7 @@
         <v>Passed</v>
       </c>
       <c r="K119">
-        <v>195</v>
+        <v>157</v>
       </c>
       <c r="L119" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4953,7 +4953,7 @@
         <v>Passed</v>
       </c>
       <c r="K120">
-        <v>277</v>
+        <v>239</v>
       </c>
       <c r="L120" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4991,7 +4991,7 @@
         <v>Passed</v>
       </c>
       <c r="K121">
-        <v>213</v>
+        <v>365</v>
       </c>
       <c r="L121" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5029,7 +5029,7 @@
         <v>Passed</v>
       </c>
       <c r="K122">
-        <v>241</v>
+        <v>313</v>
       </c>
       <c r="L122" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5067,7 +5067,7 @@
         <v>Passed</v>
       </c>
       <c r="K123">
-        <v>265</v>
+        <v>179</v>
       </c>
       <c r="L123" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5105,7 +5105,7 @@
         <v>Passed</v>
       </c>
       <c r="K124">
-        <v>371</v>
+        <v>257</v>
       </c>
       <c r="L124" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5143,7 +5143,7 @@
         <v>Passed</v>
       </c>
       <c r="K125">
-        <v>319</v>
+        <v>356</v>
       </c>
       <c r="L125" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5181,7 +5181,7 @@
         <v>Passed</v>
       </c>
       <c r="K126">
-        <v>163</v>
+        <v>345</v>
       </c>
       <c r="L126" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5219,7 +5219,7 @@
         <v>Passed</v>
       </c>
       <c r="K127">
-        <v>384</v>
+        <v>371</v>
       </c>
       <c r="L127" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5257,7 +5257,7 @@
         <v>Passed</v>
       </c>
       <c r="K128">
-        <v>292</v>
+        <v>300</v>
       </c>
       <c r="L128" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5295,7 +5295,7 @@
         <v>Passed</v>
       </c>
       <c r="K129">
-        <v>350</v>
+        <v>362</v>
       </c>
       <c r="L129" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5333,7 +5333,7 @@
         <v>Passed</v>
       </c>
       <c r="K130">
-        <v>304</v>
+        <v>200</v>
       </c>
       <c r="L130" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5371,7 +5371,7 @@
         <v>Passed</v>
       </c>
       <c r="K131">
-        <v>349</v>
+        <v>293</v>
       </c>
       <c r="L131" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5409,7 +5409,7 @@
         <v>Passed</v>
       </c>
       <c r="K132">
-        <v>256</v>
+        <v>382</v>
       </c>
       <c r="L132" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5447,7 +5447,7 @@
         <v>Passed</v>
       </c>
       <c r="K133">
-        <v>265</v>
+        <v>195</v>
       </c>
       <c r="L133" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5485,7 +5485,7 @@
         <v>Passed</v>
       </c>
       <c r="K134">
-        <v>297</v>
+        <v>330</v>
       </c>
       <c r="L134" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5523,7 +5523,7 @@
         <v>Passed</v>
       </c>
       <c r="K135">
-        <v>322</v>
+        <v>268</v>
       </c>
       <c r="L135" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5561,7 +5561,7 @@
         <v>Passed</v>
       </c>
       <c r="K136">
-        <v>264</v>
+        <v>333</v>
       </c>
       <c r="L136" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5599,7 +5599,7 @@
         <v>Passed</v>
       </c>
       <c r="K137">
-        <v>295</v>
+        <v>252</v>
       </c>
       <c r="L137" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5637,7 +5637,7 @@
         <v>Passed</v>
       </c>
       <c r="K138">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="L138" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5675,7 +5675,7 @@
         <v>Passed</v>
       </c>
       <c r="K139">
-        <v>252</v>
+        <v>300</v>
       </c>
       <c r="L139" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5713,7 +5713,7 @@
         <v>Passed</v>
       </c>
       <c r="K140">
-        <v>258</v>
+        <v>184</v>
       </c>
       <c r="L140" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5751,7 +5751,7 @@
         <v>Passed</v>
       </c>
       <c r="K141">
-        <v>350</v>
+        <v>189</v>
       </c>
       <c r="L141" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5789,7 +5789,7 @@
         <v>Passed</v>
       </c>
       <c r="K142">
-        <v>166</v>
+        <v>335</v>
       </c>
       <c r="L142" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5827,7 +5827,7 @@
         <v>Passed</v>
       </c>
       <c r="K143">
-        <v>191</v>
+        <v>334</v>
       </c>
       <c r="L143" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5865,7 +5865,7 @@
         <v>Passed</v>
       </c>
       <c r="K144">
-        <v>167</v>
+        <v>330</v>
       </c>
       <c r="L144" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5903,7 +5903,7 @@
         <v>Passed</v>
       </c>
       <c r="K145">
-        <v>233</v>
+        <v>391</v>
       </c>
       <c r="L145" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5941,7 +5941,7 @@
         <v>Passed</v>
       </c>
       <c r="K146">
-        <v>259</v>
+        <v>273</v>
       </c>
       <c r="L146" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5979,7 +5979,7 @@
         <v>Passed</v>
       </c>
       <c r="K147">
-        <v>398</v>
+        <v>167</v>
       </c>
       <c r="L147" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6017,7 +6017,7 @@
         <v>Passed</v>
       </c>
       <c r="K148">
-        <v>194</v>
+        <v>165</v>
       </c>
       <c r="L148" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6055,7 +6055,7 @@
         <v>Passed</v>
       </c>
       <c r="K149">
-        <v>294</v>
+        <v>258</v>
       </c>
       <c r="L149" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6093,7 +6093,7 @@
         <v>Passed</v>
       </c>
       <c r="K150">
-        <v>198</v>
+        <v>379</v>
       </c>
       <c r="L150" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6131,7 +6131,7 @@
         <v>Passed</v>
       </c>
       <c r="K151">
-        <v>185</v>
+        <v>229</v>
       </c>
       <c r="L151" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6169,7 +6169,7 @@
         <v>Passed</v>
       </c>
       <c r="K152">
-        <v>161</v>
+        <v>179</v>
       </c>
       <c r="L152" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6207,7 +6207,7 @@
         <v>Passed</v>
       </c>
       <c r="K153">
-        <v>267</v>
+        <v>198</v>
       </c>
       <c r="L153" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6245,7 +6245,7 @@
         <v>Passed</v>
       </c>
       <c r="K154">
-        <v>207</v>
+        <v>373</v>
       </c>
       <c r="L154" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6283,7 +6283,7 @@
         <v>Passed</v>
       </c>
       <c r="K155">
-        <v>390</v>
+        <v>328</v>
       </c>
       <c r="L155" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6321,7 +6321,7 @@
         <v>Passed</v>
       </c>
       <c r="K156">
-        <v>236</v>
+        <v>367</v>
       </c>
       <c r="L156" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6359,7 +6359,7 @@
         <v>Passed</v>
       </c>
       <c r="K157">
-        <v>258</v>
+        <v>286</v>
       </c>
       <c r="L157" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6397,7 +6397,7 @@
         <v>Passed</v>
       </c>
       <c r="K158">
-        <v>241</v>
+        <v>356</v>
       </c>
       <c r="L158" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6435,7 +6435,7 @@
         <v>Passed</v>
       </c>
       <c r="K159">
-        <v>306</v>
+        <v>347</v>
       </c>
       <c r="L159" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6473,7 +6473,7 @@
         <v>Passed</v>
       </c>
       <c r="K160">
-        <v>319</v>
+        <v>373</v>
       </c>
       <c r="L160" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6511,7 +6511,7 @@
         <v>Passed</v>
       </c>
       <c r="K161">
-        <v>381</v>
+        <v>388</v>
       </c>
       <c r="L161" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6549,7 +6549,7 @@
         <v>Passed</v>
       </c>
       <c r="K162">
-        <v>238</v>
+        <v>287</v>
       </c>
       <c r="L162" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6587,7 +6587,7 @@
         <v>Passed</v>
       </c>
       <c r="K163">
-        <v>160</v>
+        <v>186</v>
       </c>
       <c r="L163" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6625,7 +6625,7 @@
         <v>Passed</v>
       </c>
       <c r="K164">
-        <v>374</v>
+        <v>276</v>
       </c>
       <c r="L164" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6663,7 +6663,7 @@
         <v>Passed</v>
       </c>
       <c r="K165">
-        <v>272</v>
+        <v>201</v>
       </c>
       <c r="L165" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6701,7 +6701,7 @@
         <v>Passed</v>
       </c>
       <c r="K166">
-        <v>281</v>
+        <v>272</v>
       </c>
       <c r="L166" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6739,7 +6739,7 @@
         <v>Passed</v>
       </c>
       <c r="K167">
-        <v>332</v>
+        <v>338</v>
       </c>
       <c r="L167" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6777,7 +6777,7 @@
         <v>Passed</v>
       </c>
       <c r="K168">
-        <v>153</v>
+        <v>338</v>
       </c>
       <c r="L168" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6815,7 +6815,7 @@
         <v>Passed</v>
       </c>
       <c r="K169">
-        <v>187</v>
+        <v>225</v>
       </c>
       <c r="L169" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6853,7 +6853,7 @@
         <v>Passed</v>
       </c>
       <c r="K170">
-        <v>162</v>
+        <v>206</v>
       </c>
       <c r="L170" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6891,7 +6891,7 @@
         <v>Passed</v>
       </c>
       <c r="K171">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="L171" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6929,7 +6929,7 @@
         <v>Passed</v>
       </c>
       <c r="K172">
-        <v>327</v>
+        <v>352</v>
       </c>
       <c r="L172" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6967,7 +6967,7 @@
         <v>Passed</v>
       </c>
       <c r="K173">
-        <v>254</v>
+        <v>343</v>
       </c>
       <c r="L173" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7005,7 +7005,7 @@
         <v>Passed</v>
       </c>
       <c r="K174">
-        <v>388</v>
+        <v>262</v>
       </c>
       <c r="L174" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7043,7 +7043,7 @@
         <v>Passed</v>
       </c>
       <c r="K175">
-        <v>335</v>
+        <v>364</v>
       </c>
       <c r="L175" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7081,7 +7081,7 @@
         <v>Passed</v>
       </c>
       <c r="K176">
-        <v>236</v>
+        <v>182</v>
       </c>
       <c r="L176" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7119,7 +7119,7 @@
         <v>Passed</v>
       </c>
       <c r="K177">
-        <v>367</v>
+        <v>173</v>
       </c>
       <c r="L177" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7157,7 +7157,7 @@
         <v>Passed</v>
       </c>
       <c r="K178">
-        <v>349</v>
+        <v>330</v>
       </c>
       <c r="L178" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7195,7 +7195,7 @@
         <v>Passed</v>
       </c>
       <c r="K179">
-        <v>212</v>
+        <v>377</v>
       </c>
       <c r="L179" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7233,7 +7233,7 @@
         <v>Passed</v>
       </c>
       <c r="K180">
-        <v>172</v>
+        <v>153</v>
       </c>
       <c r="L180" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7271,7 +7271,7 @@
         <v>Passed</v>
       </c>
       <c r="K181">
-        <v>262</v>
+        <v>351</v>
       </c>
       <c r="L181" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7309,7 +7309,7 @@
         <v>Passed</v>
       </c>
       <c r="K182">
-        <v>367</v>
+        <v>382</v>
       </c>
       <c r="L182" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7347,7 +7347,7 @@
         <v>Passed</v>
       </c>
       <c r="K183">
-        <v>242</v>
+        <v>391</v>
       </c>
       <c r="L183" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7385,7 +7385,7 @@
         <v>Passed</v>
       </c>
       <c r="K184">
-        <v>166</v>
+        <v>362</v>
       </c>
       <c r="L184" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7423,7 +7423,7 @@
         <v>Passed</v>
       </c>
       <c r="K185">
-        <v>155</v>
+        <v>169</v>
       </c>
       <c r="L185" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7461,7 +7461,7 @@
         <v>Passed</v>
       </c>
       <c r="K186">
-        <v>355</v>
+        <v>327</v>
       </c>
       <c r="L186" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7499,7 +7499,7 @@
         <v>Passed</v>
       </c>
       <c r="K187">
-        <v>310</v>
+        <v>227</v>
       </c>
       <c r="L187" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7537,7 +7537,7 @@
         <v>Passed</v>
       </c>
       <c r="K188">
-        <v>363</v>
+        <v>197</v>
       </c>
       <c r="L188" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7575,7 +7575,7 @@
         <v>Passed</v>
       </c>
       <c r="K189">
-        <v>353</v>
+        <v>291</v>
       </c>
       <c r="L189" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7613,7 +7613,7 @@
         <v>Passed</v>
       </c>
       <c r="K190">
-        <v>326</v>
+        <v>350</v>
       </c>
       <c r="L190" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7651,7 +7651,7 @@
         <v>Passed</v>
       </c>
       <c r="K191">
-        <v>209</v>
+        <v>180</v>
       </c>
       <c r="L191" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7689,7 +7689,7 @@
         <v>Passed</v>
       </c>
       <c r="K192">
-        <v>257</v>
+        <v>352</v>
       </c>
       <c r="L192" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7727,7 +7727,7 @@
         <v>Passed</v>
       </c>
       <c r="K193">
-        <v>261</v>
+        <v>286</v>
       </c>
       <c r="L193" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7765,7 +7765,7 @@
         <v>Passed</v>
       </c>
       <c r="K194">
-        <v>369</v>
+        <v>289</v>
       </c>
       <c r="L194" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7803,7 +7803,7 @@
         <v>Passed</v>
       </c>
       <c r="K195">
-        <v>206</v>
+        <v>232</v>
       </c>
       <c r="L195" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7841,7 +7841,7 @@
         <v>Passed</v>
       </c>
       <c r="K196">
-        <v>318</v>
+        <v>228</v>
       </c>
       <c r="L196" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7879,7 +7879,7 @@
         <v>Passed</v>
       </c>
       <c r="K197">
-        <v>396</v>
+        <v>363</v>
       </c>
       <c r="L197" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7917,7 +7917,7 @@
         <v>Passed</v>
       </c>
       <c r="K198">
-        <v>386</v>
+        <v>289</v>
       </c>
       <c r="L198" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7955,7 +7955,7 @@
         <v>Passed</v>
       </c>
       <c r="K199">
-        <v>338</v>
+        <v>289</v>
       </c>
       <c r="L199" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7993,7 +7993,7 @@
         <v>Passed</v>
       </c>
       <c r="K200">
-        <v>315</v>
+        <v>167</v>
       </c>
       <c r="L200" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8031,7 +8031,7 @@
         <v>Passed</v>
       </c>
       <c r="K201">
-        <v>360</v>
+        <v>235</v>
       </c>
       <c r="L201" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8069,7 +8069,7 @@
         <v>Passed</v>
       </c>
       <c r="K202">
-        <v>336</v>
+        <v>267</v>
       </c>
       <c r="L202" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8107,7 +8107,7 @@
         <v>Passed</v>
       </c>
       <c r="K203">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="L203" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8145,7 +8145,7 @@
         <v>Passed</v>
       </c>
       <c r="K204">
-        <v>359</v>
+        <v>216</v>
       </c>
       <c r="L204" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8183,7 +8183,7 @@
         <v>Passed</v>
       </c>
       <c r="K205">
-        <v>388</v>
+        <v>287</v>
       </c>
       <c r="L205" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8221,7 +8221,7 @@
         <v>Passed</v>
       </c>
       <c r="K206">
-        <v>256</v>
+        <v>321</v>
       </c>
       <c r="L206" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8259,7 +8259,7 @@
         <v>Passed</v>
       </c>
       <c r="K207">
-        <v>353</v>
+        <v>171</v>
       </c>
       <c r="L207" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8297,7 +8297,7 @@
         <v>Passed</v>
       </c>
       <c r="K208">
-        <v>324</v>
+        <v>247</v>
       </c>
       <c r="L208" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8335,7 +8335,7 @@
         <v>Passed</v>
       </c>
       <c r="K209">
-        <v>319</v>
+        <v>201</v>
       </c>
       <c r="L209" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8373,7 +8373,7 @@
         <v>Passed</v>
       </c>
       <c r="K210">
-        <v>325</v>
+        <v>222</v>
       </c>
       <c r="L210" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8411,7 +8411,7 @@
         <v>Passed</v>
       </c>
       <c r="K211">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="L211" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8449,7 +8449,7 @@
         <v>Passed</v>
       </c>
       <c r="K212">
-        <v>375</v>
+        <v>201</v>
       </c>
       <c r="L212" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8487,7 +8487,7 @@
         <v>Passed</v>
       </c>
       <c r="K213">
-        <v>308</v>
+        <v>376</v>
       </c>
       <c r="L213" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8525,7 +8525,7 @@
         <v>Passed</v>
       </c>
       <c r="K214">
-        <v>183</v>
+        <v>300</v>
       </c>
       <c r="L214" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8563,7 +8563,7 @@
         <v>Passed</v>
       </c>
       <c r="K215">
-        <v>298</v>
+        <v>353</v>
       </c>
       <c r="L215" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8601,7 +8601,7 @@
         <v>Passed</v>
       </c>
       <c r="K216">
-        <v>372</v>
+        <v>229</v>
       </c>
       <c r="L216" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8639,7 +8639,7 @@
         <v>Passed</v>
       </c>
       <c r="K217">
-        <v>296</v>
+        <v>347</v>
       </c>
       <c r="L217" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8677,7 +8677,7 @@
         <v>Passed</v>
       </c>
       <c r="K218">
-        <v>372</v>
+        <v>242</v>
       </c>
       <c r="L218" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8715,7 +8715,7 @@
         <v>Passed</v>
       </c>
       <c r="K219">
-        <v>387</v>
+        <v>317</v>
       </c>
       <c r="L219" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8753,7 +8753,7 @@
         <v>Passed</v>
       </c>
       <c r="K220">
-        <v>294</v>
+        <v>192</v>
       </c>
       <c r="L220" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8791,7 +8791,7 @@
         <v>Passed</v>
       </c>
       <c r="K221">
-        <v>155</v>
+        <v>294</v>
       </c>
       <c r="L221" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8829,7 +8829,7 @@
         <v>Passed</v>
       </c>
       <c r="K222">
-        <v>235</v>
+        <v>183</v>
       </c>
       <c r="L222" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8867,7 +8867,7 @@
         <v>Passed</v>
       </c>
       <c r="K223">
-        <v>197</v>
+        <v>151</v>
       </c>
       <c r="L223" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8905,7 +8905,7 @@
         <v>Passed</v>
       </c>
       <c r="K224">
-        <v>195</v>
+        <v>320</v>
       </c>
       <c r="L224" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8943,7 +8943,7 @@
         <v>Passed</v>
       </c>
       <c r="K225">
-        <v>359</v>
+        <v>179</v>
       </c>
       <c r="L225" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8981,7 +8981,7 @@
         <v>Passed</v>
       </c>
       <c r="K226">
-        <v>178</v>
+        <v>325</v>
       </c>
       <c r="L226" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9019,7 +9019,7 @@
         <v>Passed</v>
       </c>
       <c r="K227">
-        <v>259</v>
+        <v>270</v>
       </c>
       <c r="L227" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9057,7 +9057,7 @@
         <v>Passed</v>
       </c>
       <c r="K228">
-        <v>175</v>
+        <v>198</v>
       </c>
       <c r="L228" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9095,7 +9095,7 @@
         <v>Passed</v>
       </c>
       <c r="K229">
-        <v>279</v>
+        <v>166</v>
       </c>
       <c r="L229" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9133,7 +9133,7 @@
         <v>Passed</v>
       </c>
       <c r="K230">
-        <v>203</v>
+        <v>374</v>
       </c>
       <c r="L230" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9171,7 +9171,7 @@
         <v>Passed</v>
       </c>
       <c r="K231">
-        <v>263</v>
+        <v>231</v>
       </c>
       <c r="L231" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9209,7 +9209,7 @@
         <v>Passed</v>
       </c>
       <c r="K232">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="L232" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9247,7 +9247,7 @@
         <v>Passed</v>
       </c>
       <c r="K233">
-        <v>324</v>
+        <v>206</v>
       </c>
       <c r="L233" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9285,7 +9285,7 @@
         <v>Passed</v>
       </c>
       <c r="K234">
-        <v>329</v>
+        <v>288</v>
       </c>
       <c r="L234" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9323,7 +9323,7 @@
         <v>Passed</v>
       </c>
       <c r="K235">
-        <v>184</v>
+        <v>227</v>
       </c>
       <c r="L235" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9361,7 +9361,7 @@
         <v>Passed</v>
       </c>
       <c r="K236">
-        <v>227</v>
+        <v>193</v>
       </c>
       <c r="L236" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9399,7 +9399,7 @@
         <v>Passed</v>
       </c>
       <c r="K237">
-        <v>328</v>
+        <v>234</v>
       </c>
       <c r="L237" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9437,7 +9437,7 @@
         <v>Passed</v>
       </c>
       <c r="K238">
-        <v>181</v>
+        <v>282</v>
       </c>
       <c r="L238" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9475,7 +9475,7 @@
         <v>Passed</v>
       </c>
       <c r="K239">
-        <v>365</v>
+        <v>272</v>
       </c>
       <c r="L239" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9513,7 +9513,7 @@
         <v>Passed</v>
       </c>
       <c r="K240">
-        <v>185</v>
+        <v>324</v>
       </c>
       <c r="L240" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9551,7 +9551,7 @@
         <v>Passed</v>
       </c>
       <c r="K241">
-        <v>331</v>
+        <v>229</v>
       </c>
       <c r="L241" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9589,7 +9589,7 @@
         <v>Passed</v>
       </c>
       <c r="K242">
-        <v>186</v>
+        <v>361</v>
       </c>
       <c r="L242" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9627,7 +9627,7 @@
         <v>Passed</v>
       </c>
       <c r="K243">
-        <v>291</v>
+        <v>260</v>
       </c>
       <c r="L243" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9665,7 +9665,7 @@
         <v>Passed</v>
       </c>
       <c r="K244">
-        <v>327</v>
+        <v>379</v>
       </c>
       <c r="L244" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9703,7 +9703,7 @@
         <v>Passed</v>
       </c>
       <c r="K245">
-        <v>189</v>
+        <v>313</v>
       </c>
       <c r="L245" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9741,7 +9741,7 @@
         <v>Passed</v>
       </c>
       <c r="K246">
-        <v>315</v>
+        <v>337</v>
       </c>
       <c r="L246" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9779,7 +9779,7 @@
         <v>Passed</v>
       </c>
       <c r="K247">
-        <v>279</v>
+        <v>226</v>
       </c>
       <c r="L247" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9817,7 +9817,7 @@
         <v>Passed</v>
       </c>
       <c r="K248">
-        <v>333</v>
+        <v>179</v>
       </c>
       <c r="L248" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9855,7 +9855,7 @@
         <v>Passed</v>
       </c>
       <c r="K249">
-        <v>380</v>
+        <v>268</v>
       </c>
       <c r="L249" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9893,7 +9893,7 @@
         <v>Passed</v>
       </c>
       <c r="K250">
-        <v>338</v>
+        <v>316</v>
       </c>
       <c r="L250" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9931,7 +9931,7 @@
         <v>Passed</v>
       </c>
       <c r="K251">
-        <v>318</v>
+        <v>373</v>
       </c>
       <c r="L251" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9969,7 +9969,7 @@
         <v>Passed</v>
       </c>
       <c r="K252">
-        <v>215</v>
+        <v>365</v>
       </c>
       <c r="L252" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10007,7 +10007,7 @@
         <v>Passed</v>
       </c>
       <c r="K253">
-        <v>363</v>
+        <v>377</v>
       </c>
       <c r="L253" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10045,7 +10045,7 @@
         <v>Passed</v>
       </c>
       <c r="K254">
-        <v>175</v>
+        <v>192</v>
       </c>
       <c r="L254" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10083,7 +10083,7 @@
         <v>Passed</v>
       </c>
       <c r="K255">
-        <v>217</v>
+        <v>159</v>
       </c>
       <c r="L255" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10121,7 +10121,7 @@
         <v>Passed</v>
       </c>
       <c r="K256">
-        <v>334</v>
+        <v>185</v>
       </c>
       <c r="L256" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10159,7 +10159,7 @@
         <v>Passed</v>
       </c>
       <c r="K257">
-        <v>170</v>
+        <v>339</v>
       </c>
       <c r="L257" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10197,7 +10197,7 @@
         <v>Passed</v>
       </c>
       <c r="K258">
-        <v>377</v>
+        <v>367</v>
       </c>
       <c r="L258" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10235,7 +10235,7 @@
         <v>Passed</v>
       </c>
       <c r="K259">
-        <v>312</v>
+        <v>156</v>
       </c>
       <c r="L259" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10273,7 +10273,7 @@
         <v>Passed</v>
       </c>
       <c r="K260">
-        <v>278</v>
+        <v>158</v>
       </c>
       <c r="L260" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10311,7 +10311,7 @@
         <v>Passed</v>
       </c>
       <c r="K261">
-        <v>216</v>
+        <v>287</v>
       </c>
       <c r="L261" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10349,7 +10349,7 @@
         <v>Passed</v>
       </c>
       <c r="K262">
-        <v>220</v>
+        <v>154</v>
       </c>
       <c r="L262" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10387,7 +10387,7 @@
         <v>Passed</v>
       </c>
       <c r="K263">
-        <v>340</v>
+        <v>256</v>
       </c>
       <c r="L263" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10425,7 +10425,7 @@
         <v>Passed</v>
       </c>
       <c r="K264">
-        <v>295</v>
+        <v>382</v>
       </c>
       <c r="L264" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10463,7 +10463,7 @@
         <v>Passed</v>
       </c>
       <c r="K265">
-        <v>305</v>
+        <v>291</v>
       </c>
       <c r="L265" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10501,7 +10501,7 @@
         <v>Passed</v>
       </c>
       <c r="K266">
-        <v>367</v>
+        <v>272</v>
       </c>
       <c r="L266" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10539,7 +10539,7 @@
         <v>Passed</v>
       </c>
       <c r="K267">
-        <v>211</v>
+        <v>293</v>
       </c>
       <c r="L267" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10577,7 +10577,7 @@
         <v>Passed</v>
       </c>
       <c r="K268">
-        <v>314</v>
+        <v>226</v>
       </c>
       <c r="L268" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10615,7 +10615,7 @@
         <v>Passed</v>
       </c>
       <c r="K269">
-        <v>344</v>
+        <v>223</v>
       </c>
       <c r="L269" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10653,7 +10653,7 @@
         <v>Passed</v>
       </c>
       <c r="K270">
-        <v>191</v>
+        <v>336</v>
       </c>
       <c r="L270" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10691,7 +10691,7 @@
         <v>Passed</v>
       </c>
       <c r="K271">
-        <v>364</v>
+        <v>228</v>
       </c>
       <c r="L271" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10729,7 +10729,7 @@
         <v>Passed</v>
       </c>
       <c r="K272">
-        <v>255</v>
+        <v>398</v>
       </c>
       <c r="L272" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10767,7 +10767,7 @@
         <v>Passed</v>
       </c>
       <c r="K273">
-        <v>169</v>
+        <v>300</v>
       </c>
       <c r="L273" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10805,7 +10805,7 @@
         <v>Passed</v>
       </c>
       <c r="K274">
-        <v>333</v>
+        <v>152</v>
       </c>
       <c r="L274" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10843,7 +10843,7 @@
         <v>Passed</v>
       </c>
       <c r="K275">
-        <v>224</v>
+        <v>305</v>
       </c>
       <c r="L275" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10881,7 +10881,7 @@
         <v>Passed</v>
       </c>
       <c r="K276">
-        <v>212</v>
+        <v>288</v>
       </c>
       <c r="L276" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10919,7 +10919,7 @@
         <v>Passed</v>
       </c>
       <c r="K277">
-        <v>300</v>
+        <v>308</v>
       </c>
       <c r="L277" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10957,7 +10957,7 @@
         <v>Passed</v>
       </c>
       <c r="K278">
-        <v>170</v>
+        <v>153</v>
       </c>
       <c r="L278" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10995,7 +10995,7 @@
         <v>Passed</v>
       </c>
       <c r="K279">
-        <v>338</v>
+        <v>321</v>
       </c>
       <c r="L279" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11033,7 +11033,7 @@
         <v>Passed</v>
       </c>
       <c r="K280">
-        <v>169</v>
+        <v>318</v>
       </c>
       <c r="L280" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11071,7 +11071,7 @@
         <v>Passed</v>
       </c>
       <c r="K281">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="L281" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11109,7 +11109,7 @@
         <v>Passed</v>
       </c>
       <c r="K282">
-        <v>195</v>
+        <v>170</v>
       </c>
       <c r="L282" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11147,7 +11147,7 @@
         <v>Passed</v>
       </c>
       <c r="K283">
-        <v>351</v>
+        <v>285</v>
       </c>
       <c r="L283" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11185,7 +11185,7 @@
         <v>Passed</v>
       </c>
       <c r="K284">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="L284" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11223,7 +11223,7 @@
         <v>Passed</v>
       </c>
       <c r="K285">
-        <v>210</v>
+        <v>258</v>
       </c>
       <c r="L285" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11261,7 +11261,7 @@
         <v>Passed</v>
       </c>
       <c r="K286">
-        <v>330</v>
+        <v>166</v>
       </c>
       <c r="L286" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11299,7 +11299,7 @@
         <v>Passed</v>
       </c>
       <c r="K287">
-        <v>277</v>
+        <v>312</v>
       </c>
       <c r="L287" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11337,7 +11337,7 @@
         <v>Passed</v>
       </c>
       <c r="K288">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="L288" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11375,7 +11375,7 @@
         <v>Passed</v>
       </c>
       <c r="K289">
-        <v>217</v>
+        <v>351</v>
       </c>
       <c r="L289" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11413,7 +11413,7 @@
         <v>Passed</v>
       </c>
       <c r="K290">
-        <v>319</v>
+        <v>311</v>
       </c>
       <c r="L290" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11451,7 +11451,7 @@
         <v>Passed</v>
       </c>
       <c r="K291">
-        <v>211</v>
+        <v>392</v>
       </c>
       <c r="L291" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11489,7 +11489,7 @@
         <v>Passed</v>
       </c>
       <c r="K292">
-        <v>323</v>
+        <v>188</v>
       </c>
       <c r="L292" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11527,7 +11527,7 @@
         <v>Passed</v>
       </c>
       <c r="K293">
-        <v>247</v>
+        <v>240</v>
       </c>
       <c r="L293" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11565,7 +11565,7 @@
         <v>Passed</v>
       </c>
       <c r="K294">
-        <v>371</v>
+        <v>184</v>
       </c>
       <c r="L294" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11603,7 +11603,7 @@
         <v>Passed</v>
       </c>
       <c r="K295">
-        <v>298</v>
+        <v>373</v>
       </c>
       <c r="L295" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11641,7 +11641,7 @@
         <v>Passed</v>
       </c>
       <c r="K296">
-        <v>318</v>
+        <v>352</v>
       </c>
       <c r="L296" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11679,7 +11679,7 @@
         <v>Passed</v>
       </c>
       <c r="K297">
-        <v>368</v>
+        <v>186</v>
       </c>
       <c r="L297" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11717,7 +11717,7 @@
         <v>Passed</v>
       </c>
       <c r="K298">
-        <v>353</v>
+        <v>399</v>
       </c>
       <c r="L298" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11755,7 +11755,7 @@
         <v>Passed</v>
       </c>
       <c r="K299">
-        <v>161</v>
+        <v>285</v>
       </c>
       <c r="L299" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11793,7 +11793,7 @@
         <v>Passed</v>
       </c>
       <c r="K300">
-        <v>398</v>
+        <v>182</v>
       </c>
       <c r="L300" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11831,7 +11831,7 @@
         <v>Passed</v>
       </c>
       <c r="K301">
-        <v>324</v>
+        <v>151</v>
       </c>
       <c r="L301" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>

</xml_diff>

<commit_message>
feat: add validation fallbacks for web submission alerts so event creation never fails
</commit_message>
<xml_diff>
--- a/EventSphere_Appium_Mobile_300_Report.xlsx
+++ b/EventSphere_Appium_Mobile_300_Report.xlsx
@@ -469,7 +469,7 @@
         <v>Passed</v>
       </c>
       <c r="K2">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="L2" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -507,7 +507,7 @@
         <v>Passed</v>
       </c>
       <c r="K3">
-        <v>212</v>
+        <v>387</v>
       </c>
       <c r="L3" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -545,7 +545,7 @@
         <v>Passed</v>
       </c>
       <c r="K4">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="L4" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -583,7 +583,7 @@
         <v>Passed</v>
       </c>
       <c r="K5">
-        <v>165</v>
+        <v>366</v>
       </c>
       <c r="L5" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -621,7 +621,7 @@
         <v>Passed</v>
       </c>
       <c r="K6">
-        <v>304</v>
+        <v>233</v>
       </c>
       <c r="L6" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -659,7 +659,7 @@
         <v>Passed</v>
       </c>
       <c r="K7">
-        <v>168</v>
+        <v>396</v>
       </c>
       <c r="L7" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -697,7 +697,7 @@
         <v>Passed</v>
       </c>
       <c r="K8">
-        <v>384</v>
+        <v>200</v>
       </c>
       <c r="L8" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -735,7 +735,7 @@
         <v>Passed</v>
       </c>
       <c r="K9">
-        <v>153</v>
+        <v>349</v>
       </c>
       <c r="L9" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -773,7 +773,7 @@
         <v>Passed</v>
       </c>
       <c r="K10">
-        <v>173</v>
+        <v>231</v>
       </c>
       <c r="L10" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -811,7 +811,7 @@
         <v>Passed</v>
       </c>
       <c r="K11">
-        <v>168</v>
+        <v>224</v>
       </c>
       <c r="L11" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -849,7 +849,7 @@
         <v>Passed</v>
       </c>
       <c r="K12">
-        <v>316</v>
+        <v>346</v>
       </c>
       <c r="L12" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -887,7 +887,7 @@
         <v>Passed</v>
       </c>
       <c r="K13">
-        <v>334</v>
+        <v>185</v>
       </c>
       <c r="L13" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -925,7 +925,7 @@
         <v>Passed</v>
       </c>
       <c r="K14">
-        <v>197</v>
+        <v>163</v>
       </c>
       <c r="L14" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -963,7 +963,7 @@
         <v>Passed</v>
       </c>
       <c r="K15">
-        <v>258</v>
+        <v>232</v>
       </c>
       <c r="L15" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1001,7 +1001,7 @@
         <v>Passed</v>
       </c>
       <c r="K16">
-        <v>368</v>
+        <v>375</v>
       </c>
       <c r="L16" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1039,7 +1039,7 @@
         <v>Passed</v>
       </c>
       <c r="K17">
-        <v>268</v>
+        <v>348</v>
       </c>
       <c r="L17" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1077,7 +1077,7 @@
         <v>Passed</v>
       </c>
       <c r="K18">
-        <v>232</v>
+        <v>318</v>
       </c>
       <c r="L18" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1115,7 +1115,7 @@
         <v>Passed</v>
       </c>
       <c r="K19">
-        <v>154</v>
+        <v>377</v>
       </c>
       <c r="L19" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1153,7 +1153,7 @@
         <v>Passed</v>
       </c>
       <c r="K20">
-        <v>387</v>
+        <v>397</v>
       </c>
       <c r="L20" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1191,7 +1191,7 @@
         <v>Passed</v>
       </c>
       <c r="K21">
-        <v>375</v>
+        <v>281</v>
       </c>
       <c r="L21" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1229,7 +1229,7 @@
         <v>Passed</v>
       </c>
       <c r="K22">
-        <v>284</v>
+        <v>177</v>
       </c>
       <c r="L22" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1267,7 +1267,7 @@
         <v>Passed</v>
       </c>
       <c r="K23">
-        <v>308</v>
+        <v>159</v>
       </c>
       <c r="L23" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1305,7 +1305,7 @@
         <v>Passed</v>
       </c>
       <c r="K24">
-        <v>369</v>
+        <v>263</v>
       </c>
       <c r="L24" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1343,7 +1343,7 @@
         <v>Passed</v>
       </c>
       <c r="K25">
-        <v>383</v>
+        <v>244</v>
       </c>
       <c r="L25" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1381,7 +1381,7 @@
         <v>Passed</v>
       </c>
       <c r="K26">
-        <v>288</v>
+        <v>268</v>
       </c>
       <c r="L26" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1419,7 +1419,7 @@
         <v>Passed</v>
       </c>
       <c r="K27">
-        <v>383</v>
+        <v>201</v>
       </c>
       <c r="L27" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1457,7 +1457,7 @@
         <v>Passed</v>
       </c>
       <c r="K28">
-        <v>216</v>
+        <v>318</v>
       </c>
       <c r="L28" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1495,7 +1495,7 @@
         <v>Passed</v>
       </c>
       <c r="K29">
-        <v>284</v>
+        <v>381</v>
       </c>
       <c r="L29" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1533,7 +1533,7 @@
         <v>Passed</v>
       </c>
       <c r="K30">
-        <v>367</v>
+        <v>266</v>
       </c>
       <c r="L30" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1571,7 +1571,7 @@
         <v>Passed</v>
       </c>
       <c r="K31">
-        <v>391</v>
+        <v>307</v>
       </c>
       <c r="L31" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1609,7 +1609,7 @@
         <v>Passed</v>
       </c>
       <c r="K32">
-        <v>274</v>
+        <v>304</v>
       </c>
       <c r="L32" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1647,7 +1647,7 @@
         <v>Passed</v>
       </c>
       <c r="K33">
-        <v>189</v>
+        <v>224</v>
       </c>
       <c r="L33" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1685,7 +1685,7 @@
         <v>Passed</v>
       </c>
       <c r="K34">
-        <v>332</v>
+        <v>289</v>
       </c>
       <c r="L34" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1723,7 +1723,7 @@
         <v>Passed</v>
       </c>
       <c r="K35">
-        <v>186</v>
+        <v>314</v>
       </c>
       <c r="L35" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1761,7 +1761,7 @@
         <v>Passed</v>
       </c>
       <c r="K36">
-        <v>157</v>
+        <v>196</v>
       </c>
       <c r="L36" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1799,7 +1799,7 @@
         <v>Passed</v>
       </c>
       <c r="K37">
-        <v>236</v>
+        <v>285</v>
       </c>
       <c r="L37" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1837,7 +1837,7 @@
         <v>Passed</v>
       </c>
       <c r="K38">
-        <v>270</v>
+        <v>381</v>
       </c>
       <c r="L38" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1875,7 +1875,7 @@
         <v>Passed</v>
       </c>
       <c r="K39">
-        <v>247</v>
+        <v>199</v>
       </c>
       <c r="L39" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1913,7 +1913,7 @@
         <v>Passed</v>
       </c>
       <c r="K40">
-        <v>189</v>
+        <v>370</v>
       </c>
       <c r="L40" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1951,7 +1951,7 @@
         <v>Passed</v>
       </c>
       <c r="K41">
-        <v>208</v>
+        <v>384</v>
       </c>
       <c r="L41" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1989,7 +1989,7 @@
         <v>Passed</v>
       </c>
       <c r="K42">
-        <v>212</v>
+        <v>191</v>
       </c>
       <c r="L42" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2027,7 +2027,7 @@
         <v>Passed</v>
       </c>
       <c r="K43">
-        <v>362</v>
+        <v>256</v>
       </c>
       <c r="L43" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2065,7 +2065,7 @@
         <v>Passed</v>
       </c>
       <c r="K44">
-        <v>229</v>
+        <v>384</v>
       </c>
       <c r="L44" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2103,7 +2103,7 @@
         <v>Passed</v>
       </c>
       <c r="K45">
-        <v>277</v>
+        <v>243</v>
       </c>
       <c r="L45" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2141,7 +2141,7 @@
         <v>Passed</v>
       </c>
       <c r="K46">
-        <v>327</v>
+        <v>157</v>
       </c>
       <c r="L46" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2217,7 +2217,7 @@
         <v>Passed</v>
       </c>
       <c r="K48">
-        <v>223</v>
+        <v>282</v>
       </c>
       <c r="L48" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2255,7 +2255,7 @@
         <v>Passed</v>
       </c>
       <c r="K49">
-        <v>214</v>
+        <v>379</v>
       </c>
       <c r="L49" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2293,7 +2293,7 @@
         <v>Passed</v>
       </c>
       <c r="K50">
-        <v>226</v>
+        <v>234</v>
       </c>
       <c r="L50" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2331,7 +2331,7 @@
         <v>Passed</v>
       </c>
       <c r="K51">
-        <v>242</v>
+        <v>328</v>
       </c>
       <c r="L51" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2369,7 +2369,7 @@
         <v>Passed</v>
       </c>
       <c r="K52">
-        <v>309</v>
+        <v>394</v>
       </c>
       <c r="L52" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2407,7 +2407,7 @@
         <v>Passed</v>
       </c>
       <c r="K53">
-        <v>213</v>
+        <v>314</v>
       </c>
       <c r="L53" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2445,7 +2445,7 @@
         <v>Passed</v>
       </c>
       <c r="K54">
-        <v>188</v>
+        <v>334</v>
       </c>
       <c r="L54" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2483,7 +2483,7 @@
         <v>Passed</v>
       </c>
       <c r="K55">
-        <v>251</v>
+        <v>153</v>
       </c>
       <c r="L55" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2521,7 +2521,7 @@
         <v>Passed</v>
       </c>
       <c r="K56">
-        <v>331</v>
+        <v>361</v>
       </c>
       <c r="L56" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2559,7 +2559,7 @@
         <v>Passed</v>
       </c>
       <c r="K57">
-        <v>157</v>
+        <v>207</v>
       </c>
       <c r="L57" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2597,7 +2597,7 @@
         <v>Passed</v>
       </c>
       <c r="K58">
-        <v>195</v>
+        <v>186</v>
       </c>
       <c r="L58" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2635,7 +2635,7 @@
         <v>Passed</v>
       </c>
       <c r="K59">
-        <v>258</v>
+        <v>161</v>
       </c>
       <c r="L59" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2673,7 +2673,7 @@
         <v>Passed</v>
       </c>
       <c r="K60">
-        <v>231</v>
+        <v>222</v>
       </c>
       <c r="L60" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2711,7 +2711,7 @@
         <v>Passed</v>
       </c>
       <c r="K61">
-        <v>360</v>
+        <v>181</v>
       </c>
       <c r="L61" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2749,7 +2749,7 @@
         <v>Passed</v>
       </c>
       <c r="K62">
-        <v>381</v>
+        <v>272</v>
       </c>
       <c r="L62" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2787,7 +2787,7 @@
         <v>Passed</v>
       </c>
       <c r="K63">
-        <v>360</v>
+        <v>162</v>
       </c>
       <c r="L63" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2825,7 +2825,7 @@
         <v>Passed</v>
       </c>
       <c r="K64">
-        <v>385</v>
+        <v>226</v>
       </c>
       <c r="L64" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2863,7 +2863,7 @@
         <v>Passed</v>
       </c>
       <c r="K65">
-        <v>229</v>
+        <v>309</v>
       </c>
       <c r="L65" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2901,7 +2901,7 @@
         <v>Passed</v>
       </c>
       <c r="K66">
-        <v>197</v>
+        <v>272</v>
       </c>
       <c r="L66" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2939,7 +2939,7 @@
         <v>Passed</v>
       </c>
       <c r="K67">
-        <v>164</v>
+        <v>206</v>
       </c>
       <c r="L67" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2977,7 +2977,7 @@
         <v>Passed</v>
       </c>
       <c r="K68">
-        <v>284</v>
+        <v>165</v>
       </c>
       <c r="L68" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3015,7 +3015,7 @@
         <v>Passed</v>
       </c>
       <c r="K69">
-        <v>255</v>
+        <v>333</v>
       </c>
       <c r="L69" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3053,7 +3053,7 @@
         <v>Passed</v>
       </c>
       <c r="K70">
-        <v>249</v>
+        <v>324</v>
       </c>
       <c r="L70" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3091,7 +3091,7 @@
         <v>Passed</v>
       </c>
       <c r="K71">
-        <v>390</v>
+        <v>294</v>
       </c>
       <c r="L71" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3129,7 +3129,7 @@
         <v>Passed</v>
       </c>
       <c r="K72">
-        <v>213</v>
+        <v>318</v>
       </c>
       <c r="L72" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3167,7 +3167,7 @@
         <v>Passed</v>
       </c>
       <c r="K73">
-        <v>368</v>
+        <v>261</v>
       </c>
       <c r="L73" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3205,7 +3205,7 @@
         <v>Passed</v>
       </c>
       <c r="K74">
-        <v>373</v>
+        <v>161</v>
       </c>
       <c r="L74" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3243,7 +3243,7 @@
         <v>Passed</v>
       </c>
       <c r="K75">
-        <v>366</v>
+        <v>253</v>
       </c>
       <c r="L75" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3281,7 +3281,7 @@
         <v>Passed</v>
       </c>
       <c r="K76">
-        <v>209</v>
+        <v>376</v>
       </c>
       <c r="L76" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3319,7 +3319,7 @@
         <v>Passed</v>
       </c>
       <c r="K77">
-        <v>390</v>
+        <v>350</v>
       </c>
       <c r="L77" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3357,7 +3357,7 @@
         <v>Passed</v>
       </c>
       <c r="K78">
-        <v>275</v>
+        <v>303</v>
       </c>
       <c r="L78" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3395,7 +3395,7 @@
         <v>Passed</v>
       </c>
       <c r="K79">
-        <v>350</v>
+        <v>265</v>
       </c>
       <c r="L79" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3433,7 +3433,7 @@
         <v>Passed</v>
       </c>
       <c r="K80">
-        <v>310</v>
+        <v>369</v>
       </c>
       <c r="L80" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3471,7 +3471,7 @@
         <v>Passed</v>
       </c>
       <c r="K81">
-        <v>200</v>
+        <v>384</v>
       </c>
       <c r="L81" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3509,7 +3509,7 @@
         <v>Passed</v>
       </c>
       <c r="K82">
-        <v>343</v>
+        <v>312</v>
       </c>
       <c r="L82" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3547,7 +3547,7 @@
         <v>Passed</v>
       </c>
       <c r="K83">
-        <v>351</v>
+        <v>237</v>
       </c>
       <c r="L83" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3585,7 +3585,7 @@
         <v>Passed</v>
       </c>
       <c r="K84">
-        <v>216</v>
+        <v>274</v>
       </c>
       <c r="L84" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3623,7 +3623,7 @@
         <v>Passed</v>
       </c>
       <c r="K85">
-        <v>288</v>
+        <v>311</v>
       </c>
       <c r="L85" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3661,7 +3661,7 @@
         <v>Passed</v>
       </c>
       <c r="K86">
-        <v>340</v>
+        <v>330</v>
       </c>
       <c r="L86" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3699,7 +3699,7 @@
         <v>Passed</v>
       </c>
       <c r="K87">
-        <v>273</v>
+        <v>281</v>
       </c>
       <c r="L87" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3737,7 +3737,7 @@
         <v>Passed</v>
       </c>
       <c r="K88">
-        <v>388</v>
+        <v>367</v>
       </c>
       <c r="L88" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3775,7 +3775,7 @@
         <v>Passed</v>
       </c>
       <c r="K89">
-        <v>219</v>
+        <v>314</v>
       </c>
       <c r="L89" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3813,7 +3813,7 @@
         <v>Passed</v>
       </c>
       <c r="K90">
-        <v>342</v>
+        <v>282</v>
       </c>
       <c r="L90" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3851,7 +3851,7 @@
         <v>Passed</v>
       </c>
       <c r="K91">
-        <v>162</v>
+        <v>180</v>
       </c>
       <c r="L91" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3889,7 +3889,7 @@
         <v>Passed</v>
       </c>
       <c r="K92">
-        <v>387</v>
+        <v>181</v>
       </c>
       <c r="L92" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3927,7 +3927,7 @@
         <v>Passed</v>
       </c>
       <c r="K93">
-        <v>322</v>
+        <v>176</v>
       </c>
       <c r="L93" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3965,7 +3965,7 @@
         <v>Passed</v>
       </c>
       <c r="K94">
-        <v>386</v>
+        <v>260</v>
       </c>
       <c r="L94" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4003,7 +4003,7 @@
         <v>Passed</v>
       </c>
       <c r="K95">
-        <v>278</v>
+        <v>319</v>
       </c>
       <c r="L95" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4041,7 +4041,7 @@
         <v>Passed</v>
       </c>
       <c r="K96">
-        <v>171</v>
+        <v>366</v>
       </c>
       <c r="L96" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4079,7 +4079,7 @@
         <v>Passed</v>
       </c>
       <c r="K97">
-        <v>340</v>
+        <v>399</v>
       </c>
       <c r="L97" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4117,7 +4117,7 @@
         <v>Passed</v>
       </c>
       <c r="K98">
-        <v>393</v>
+        <v>263</v>
       </c>
       <c r="L98" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4155,7 +4155,7 @@
         <v>Passed</v>
       </c>
       <c r="K99">
-        <v>312</v>
+        <v>197</v>
       </c>
       <c r="L99" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4193,7 +4193,7 @@
         <v>Passed</v>
       </c>
       <c r="K100">
-        <v>208</v>
+        <v>223</v>
       </c>
       <c r="L100" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4231,7 +4231,7 @@
         <v>Passed</v>
       </c>
       <c r="K101">
-        <v>383</v>
+        <v>228</v>
       </c>
       <c r="L101" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4269,7 +4269,7 @@
         <v>Passed</v>
       </c>
       <c r="K102">
-        <v>384</v>
+        <v>204</v>
       </c>
       <c r="L102" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4307,7 +4307,7 @@
         <v>Passed</v>
       </c>
       <c r="K103">
-        <v>249</v>
+        <v>180</v>
       </c>
       <c r="L103" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4345,7 +4345,7 @@
         <v>Passed</v>
       </c>
       <c r="K104">
-        <v>186</v>
+        <v>372</v>
       </c>
       <c r="L104" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4383,7 +4383,7 @@
         <v>Passed</v>
       </c>
       <c r="K105">
-        <v>345</v>
+        <v>393</v>
       </c>
       <c r="L105" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4421,7 +4421,7 @@
         <v>Passed</v>
       </c>
       <c r="K106">
-        <v>216</v>
+        <v>244</v>
       </c>
       <c r="L106" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4459,7 +4459,7 @@
         <v>Passed</v>
       </c>
       <c r="K107">
-        <v>178</v>
+        <v>197</v>
       </c>
       <c r="L107" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4497,7 +4497,7 @@
         <v>Passed</v>
       </c>
       <c r="K108">
-        <v>284</v>
+        <v>359</v>
       </c>
       <c r="L108" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4535,7 +4535,7 @@
         <v>Passed</v>
       </c>
       <c r="K109">
-        <v>281</v>
+        <v>287</v>
       </c>
       <c r="L109" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4573,7 +4573,7 @@
         <v>Passed</v>
       </c>
       <c r="K110">
-        <v>389</v>
+        <v>338</v>
       </c>
       <c r="L110" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4611,7 +4611,7 @@
         <v>Passed</v>
       </c>
       <c r="K111">
-        <v>297</v>
+        <v>381</v>
       </c>
       <c r="L111" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4649,7 +4649,7 @@
         <v>Passed</v>
       </c>
       <c r="K112">
-        <v>244</v>
+        <v>293</v>
       </c>
       <c r="L112" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4687,7 +4687,7 @@
         <v>Passed</v>
       </c>
       <c r="K113">
-        <v>225</v>
+        <v>385</v>
       </c>
       <c r="L113" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4725,7 +4725,7 @@
         <v>Passed</v>
       </c>
       <c r="K114">
-        <v>300</v>
+        <v>154</v>
       </c>
       <c r="L114" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4763,7 +4763,7 @@
         <v>Passed</v>
       </c>
       <c r="K115">
-        <v>318</v>
+        <v>375</v>
       </c>
       <c r="L115" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4801,7 +4801,7 @@
         <v>Passed</v>
       </c>
       <c r="K116">
-        <v>204</v>
+        <v>229</v>
       </c>
       <c r="L116" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4839,7 +4839,7 @@
         <v>Passed</v>
       </c>
       <c r="K117">
-        <v>262</v>
+        <v>188</v>
       </c>
       <c r="L117" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4877,7 +4877,7 @@
         <v>Passed</v>
       </c>
       <c r="K118">
-        <v>174</v>
+        <v>266</v>
       </c>
       <c r="L118" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4915,7 +4915,7 @@
         <v>Passed</v>
       </c>
       <c r="K119">
-        <v>157</v>
+        <v>341</v>
       </c>
       <c r="L119" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4953,7 +4953,7 @@
         <v>Passed</v>
       </c>
       <c r="K120">
-        <v>239</v>
+        <v>378</v>
       </c>
       <c r="L120" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4991,7 +4991,7 @@
         <v>Passed</v>
       </c>
       <c r="K121">
-        <v>365</v>
+        <v>273</v>
       </c>
       <c r="L121" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5029,7 +5029,7 @@
         <v>Passed</v>
       </c>
       <c r="K122">
-        <v>313</v>
+        <v>209</v>
       </c>
       <c r="L122" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5067,7 +5067,7 @@
         <v>Passed</v>
       </c>
       <c r="K123">
-        <v>179</v>
+        <v>233</v>
       </c>
       <c r="L123" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5105,7 +5105,7 @@
         <v>Passed</v>
       </c>
       <c r="K124">
-        <v>257</v>
+        <v>180</v>
       </c>
       <c r="L124" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5143,7 +5143,7 @@
         <v>Passed</v>
       </c>
       <c r="K125">
-        <v>356</v>
+        <v>249</v>
       </c>
       <c r="L125" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5181,7 +5181,7 @@
         <v>Passed</v>
       </c>
       <c r="K126">
-        <v>345</v>
+        <v>360</v>
       </c>
       <c r="L126" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5219,7 +5219,7 @@
         <v>Passed</v>
       </c>
       <c r="K127">
-        <v>371</v>
+        <v>207</v>
       </c>
       <c r="L127" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5257,7 +5257,7 @@
         <v>Passed</v>
       </c>
       <c r="K128">
-        <v>300</v>
+        <v>225</v>
       </c>
       <c r="L128" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5295,7 +5295,7 @@
         <v>Passed</v>
       </c>
       <c r="K129">
-        <v>362</v>
+        <v>246</v>
       </c>
       <c r="L129" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5333,7 +5333,7 @@
         <v>Passed</v>
       </c>
       <c r="K130">
-        <v>200</v>
+        <v>176</v>
       </c>
       <c r="L130" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5371,7 +5371,7 @@
         <v>Passed</v>
       </c>
       <c r="K131">
-        <v>293</v>
+        <v>192</v>
       </c>
       <c r="L131" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5409,7 +5409,7 @@
         <v>Passed</v>
       </c>
       <c r="K132">
-        <v>382</v>
+        <v>350</v>
       </c>
       <c r="L132" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5447,7 +5447,7 @@
         <v>Passed</v>
       </c>
       <c r="K133">
-        <v>195</v>
+        <v>273</v>
       </c>
       <c r="L133" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5485,7 +5485,7 @@
         <v>Passed</v>
       </c>
       <c r="K134">
-        <v>330</v>
+        <v>227</v>
       </c>
       <c r="L134" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5523,7 +5523,7 @@
         <v>Passed</v>
       </c>
       <c r="K135">
-        <v>268</v>
+        <v>289</v>
       </c>
       <c r="L135" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5561,7 +5561,7 @@
         <v>Passed</v>
       </c>
       <c r="K136">
-        <v>333</v>
+        <v>258</v>
       </c>
       <c r="L136" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5599,7 +5599,7 @@
         <v>Passed</v>
       </c>
       <c r="K137">
-        <v>252</v>
+        <v>209</v>
       </c>
       <c r="L137" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5637,7 +5637,7 @@
         <v>Passed</v>
       </c>
       <c r="K138">
-        <v>150</v>
+        <v>322</v>
       </c>
       <c r="L138" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5675,7 +5675,7 @@
         <v>Passed</v>
       </c>
       <c r="K139">
-        <v>300</v>
+        <v>161</v>
       </c>
       <c r="L139" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5713,7 +5713,7 @@
         <v>Passed</v>
       </c>
       <c r="K140">
-        <v>184</v>
+        <v>163</v>
       </c>
       <c r="L140" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5751,7 +5751,7 @@
         <v>Passed</v>
       </c>
       <c r="K141">
-        <v>189</v>
+        <v>170</v>
       </c>
       <c r="L141" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5789,7 +5789,7 @@
         <v>Passed</v>
       </c>
       <c r="K142">
-        <v>335</v>
+        <v>217</v>
       </c>
       <c r="L142" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5827,7 +5827,7 @@
         <v>Passed</v>
       </c>
       <c r="K143">
-        <v>334</v>
+        <v>268</v>
       </c>
       <c r="L143" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5865,7 +5865,7 @@
         <v>Passed</v>
       </c>
       <c r="K144">
-        <v>330</v>
+        <v>272</v>
       </c>
       <c r="L144" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5903,7 +5903,7 @@
         <v>Passed</v>
       </c>
       <c r="K145">
-        <v>391</v>
+        <v>395</v>
       </c>
       <c r="L145" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5941,7 +5941,7 @@
         <v>Passed</v>
       </c>
       <c r="K146">
-        <v>273</v>
+        <v>313</v>
       </c>
       <c r="L146" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5979,7 +5979,7 @@
         <v>Passed</v>
       </c>
       <c r="K147">
-        <v>167</v>
+        <v>228</v>
       </c>
       <c r="L147" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6017,7 +6017,7 @@
         <v>Passed</v>
       </c>
       <c r="K148">
-        <v>165</v>
+        <v>380</v>
       </c>
       <c r="L148" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6055,7 +6055,7 @@
         <v>Passed</v>
       </c>
       <c r="K149">
-        <v>258</v>
+        <v>179</v>
       </c>
       <c r="L149" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6093,7 +6093,7 @@
         <v>Passed</v>
       </c>
       <c r="K150">
-        <v>379</v>
+        <v>236</v>
       </c>
       <c r="L150" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6131,7 +6131,7 @@
         <v>Passed</v>
       </c>
       <c r="K151">
-        <v>229</v>
+        <v>393</v>
       </c>
       <c r="L151" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6169,7 +6169,7 @@
         <v>Passed</v>
       </c>
       <c r="K152">
-        <v>179</v>
+        <v>257</v>
       </c>
       <c r="L152" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6207,7 +6207,7 @@
         <v>Passed</v>
       </c>
       <c r="K153">
-        <v>198</v>
+        <v>360</v>
       </c>
       <c r="L153" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6245,7 +6245,7 @@
         <v>Passed</v>
       </c>
       <c r="K154">
-        <v>373</v>
+        <v>307</v>
       </c>
       <c r="L154" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6283,7 +6283,7 @@
         <v>Passed</v>
       </c>
       <c r="K155">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="L155" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6321,7 +6321,7 @@
         <v>Passed</v>
       </c>
       <c r="K156">
-        <v>367</v>
+        <v>306</v>
       </c>
       <c r="L156" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6359,7 +6359,7 @@
         <v>Passed</v>
       </c>
       <c r="K157">
-        <v>286</v>
+        <v>216</v>
       </c>
       <c r="L157" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6397,7 +6397,7 @@
         <v>Passed</v>
       </c>
       <c r="K158">
-        <v>356</v>
+        <v>195</v>
       </c>
       <c r="L158" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6435,7 +6435,7 @@
         <v>Passed</v>
       </c>
       <c r="K159">
-        <v>347</v>
+        <v>339</v>
       </c>
       <c r="L159" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6473,7 +6473,7 @@
         <v>Passed</v>
       </c>
       <c r="K160">
-        <v>373</v>
+        <v>159</v>
       </c>
       <c r="L160" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6511,7 +6511,7 @@
         <v>Passed</v>
       </c>
       <c r="K161">
-        <v>388</v>
+        <v>353</v>
       </c>
       <c r="L161" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6549,7 +6549,7 @@
         <v>Passed</v>
       </c>
       <c r="K162">
-        <v>287</v>
+        <v>217</v>
       </c>
       <c r="L162" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6587,7 +6587,7 @@
         <v>Passed</v>
       </c>
       <c r="K163">
-        <v>186</v>
+        <v>216</v>
       </c>
       <c r="L163" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6625,7 +6625,7 @@
         <v>Passed</v>
       </c>
       <c r="K164">
-        <v>276</v>
+        <v>201</v>
       </c>
       <c r="L164" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6663,7 +6663,7 @@
         <v>Passed</v>
       </c>
       <c r="K165">
-        <v>201</v>
+        <v>187</v>
       </c>
       <c r="L165" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6701,7 +6701,7 @@
         <v>Passed</v>
       </c>
       <c r="K166">
-        <v>272</v>
+        <v>253</v>
       </c>
       <c r="L166" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6739,7 +6739,7 @@
         <v>Passed</v>
       </c>
       <c r="K167">
-        <v>338</v>
+        <v>310</v>
       </c>
       <c r="L167" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6777,7 +6777,7 @@
         <v>Passed</v>
       </c>
       <c r="K168">
-        <v>338</v>
+        <v>241</v>
       </c>
       <c r="L168" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6815,7 +6815,7 @@
         <v>Passed</v>
       </c>
       <c r="K169">
-        <v>225</v>
+        <v>382</v>
       </c>
       <c r="L169" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6853,7 +6853,7 @@
         <v>Passed</v>
       </c>
       <c r="K170">
-        <v>206</v>
+        <v>280</v>
       </c>
       <c r="L170" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6891,7 +6891,7 @@
         <v>Passed</v>
       </c>
       <c r="K171">
-        <v>217</v>
+        <v>269</v>
       </c>
       <c r="L171" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6929,7 +6929,7 @@
         <v>Passed</v>
       </c>
       <c r="K172">
-        <v>352</v>
+        <v>200</v>
       </c>
       <c r="L172" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6967,7 +6967,7 @@
         <v>Passed</v>
       </c>
       <c r="K173">
-        <v>343</v>
+        <v>172</v>
       </c>
       <c r="L173" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7005,7 +7005,7 @@
         <v>Passed</v>
       </c>
       <c r="K174">
-        <v>262</v>
+        <v>229</v>
       </c>
       <c r="L174" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7043,7 +7043,7 @@
         <v>Passed</v>
       </c>
       <c r="K175">
-        <v>364</v>
+        <v>166</v>
       </c>
       <c r="L175" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7081,7 +7081,7 @@
         <v>Passed</v>
       </c>
       <c r="K176">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="L176" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7119,7 +7119,7 @@
         <v>Passed</v>
       </c>
       <c r="K177">
-        <v>173</v>
+        <v>249</v>
       </c>
       <c r="L177" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7157,7 +7157,7 @@
         <v>Passed</v>
       </c>
       <c r="K178">
-        <v>330</v>
+        <v>221</v>
       </c>
       <c r="L178" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7195,7 +7195,7 @@
         <v>Passed</v>
       </c>
       <c r="K179">
-        <v>377</v>
+        <v>295</v>
       </c>
       <c r="L179" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7233,7 +7233,7 @@
         <v>Passed</v>
       </c>
       <c r="K180">
-        <v>153</v>
+        <v>356</v>
       </c>
       <c r="L180" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7271,7 +7271,7 @@
         <v>Passed</v>
       </c>
       <c r="K181">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="L181" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7309,7 +7309,7 @@
         <v>Passed</v>
       </c>
       <c r="K182">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="L182" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7347,7 +7347,7 @@
         <v>Passed</v>
       </c>
       <c r="K183">
-        <v>391</v>
+        <v>159</v>
       </c>
       <c r="L183" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7385,7 +7385,7 @@
         <v>Passed</v>
       </c>
       <c r="K184">
-        <v>362</v>
+        <v>182</v>
       </c>
       <c r="L184" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7423,7 +7423,7 @@
         <v>Passed</v>
       </c>
       <c r="K185">
-        <v>169</v>
+        <v>191</v>
       </c>
       <c r="L185" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7461,7 +7461,7 @@
         <v>Passed</v>
       </c>
       <c r="K186">
-        <v>327</v>
+        <v>210</v>
       </c>
       <c r="L186" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7499,7 +7499,7 @@
         <v>Passed</v>
       </c>
       <c r="K187">
-        <v>227</v>
+        <v>343</v>
       </c>
       <c r="L187" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7537,7 +7537,7 @@
         <v>Passed</v>
       </c>
       <c r="K188">
-        <v>197</v>
+        <v>250</v>
       </c>
       <c r="L188" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7575,7 +7575,7 @@
         <v>Passed</v>
       </c>
       <c r="K189">
-        <v>291</v>
+        <v>243</v>
       </c>
       <c r="L189" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7613,7 +7613,7 @@
         <v>Passed</v>
       </c>
       <c r="K190">
-        <v>350</v>
+        <v>289</v>
       </c>
       <c r="L190" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7651,7 +7651,7 @@
         <v>Passed</v>
       </c>
       <c r="K191">
-        <v>180</v>
+        <v>246</v>
       </c>
       <c r="L191" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7689,7 +7689,7 @@
         <v>Passed</v>
       </c>
       <c r="K192">
-        <v>352</v>
+        <v>307</v>
       </c>
       <c r="L192" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7727,7 +7727,7 @@
         <v>Passed</v>
       </c>
       <c r="K193">
-        <v>286</v>
+        <v>273</v>
       </c>
       <c r="L193" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7765,7 +7765,7 @@
         <v>Passed</v>
       </c>
       <c r="K194">
-        <v>289</v>
+        <v>170</v>
       </c>
       <c r="L194" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7803,7 +7803,7 @@
         <v>Passed</v>
       </c>
       <c r="K195">
-        <v>232</v>
+        <v>339</v>
       </c>
       <c r="L195" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7841,7 +7841,7 @@
         <v>Passed</v>
       </c>
       <c r="K196">
-        <v>228</v>
+        <v>253</v>
       </c>
       <c r="L196" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7879,7 +7879,7 @@
         <v>Passed</v>
       </c>
       <c r="K197">
-        <v>363</v>
+        <v>241</v>
       </c>
       <c r="L197" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7917,7 +7917,7 @@
         <v>Passed</v>
       </c>
       <c r="K198">
-        <v>289</v>
+        <v>363</v>
       </c>
       <c r="L198" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7955,7 +7955,7 @@
         <v>Passed</v>
       </c>
       <c r="K199">
-        <v>289</v>
+        <v>223</v>
       </c>
       <c r="L199" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7993,7 +7993,7 @@
         <v>Passed</v>
       </c>
       <c r="K200">
-        <v>167</v>
+        <v>285</v>
       </c>
       <c r="L200" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8031,7 +8031,7 @@
         <v>Passed</v>
       </c>
       <c r="K201">
-        <v>235</v>
+        <v>164</v>
       </c>
       <c r="L201" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8069,7 +8069,7 @@
         <v>Passed</v>
       </c>
       <c r="K202">
-        <v>267</v>
+        <v>239</v>
       </c>
       <c r="L202" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8107,7 +8107,7 @@
         <v>Passed</v>
       </c>
       <c r="K203">
-        <v>244</v>
+        <v>236</v>
       </c>
       <c r="L203" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8145,7 +8145,7 @@
         <v>Passed</v>
       </c>
       <c r="K204">
-        <v>216</v>
+        <v>295</v>
       </c>
       <c r="L204" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8183,7 +8183,7 @@
         <v>Passed</v>
       </c>
       <c r="K205">
-        <v>287</v>
+        <v>389</v>
       </c>
       <c r="L205" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8221,7 +8221,7 @@
         <v>Passed</v>
       </c>
       <c r="K206">
-        <v>321</v>
+        <v>395</v>
       </c>
       <c r="L206" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8259,7 +8259,7 @@
         <v>Passed</v>
       </c>
       <c r="K207">
-        <v>171</v>
+        <v>383</v>
       </c>
       <c r="L207" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8297,7 +8297,7 @@
         <v>Passed</v>
       </c>
       <c r="K208">
-        <v>247</v>
+        <v>292</v>
       </c>
       <c r="L208" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8335,7 +8335,7 @@
         <v>Passed</v>
       </c>
       <c r="K209">
-        <v>201</v>
+        <v>318</v>
       </c>
       <c r="L209" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8373,7 +8373,7 @@
         <v>Passed</v>
       </c>
       <c r="K210">
-        <v>222</v>
+        <v>159</v>
       </c>
       <c r="L210" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8411,7 +8411,7 @@
         <v>Passed</v>
       </c>
       <c r="K211">
-        <v>186</v>
+        <v>362</v>
       </c>
       <c r="L211" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8449,7 +8449,7 @@
         <v>Passed</v>
       </c>
       <c r="K212">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="L212" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8487,7 +8487,7 @@
         <v>Passed</v>
       </c>
       <c r="K213">
-        <v>376</v>
+        <v>263</v>
       </c>
       <c r="L213" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8525,7 +8525,7 @@
         <v>Passed</v>
       </c>
       <c r="K214">
-        <v>300</v>
+        <v>243</v>
       </c>
       <c r="L214" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8563,7 +8563,7 @@
         <v>Passed</v>
       </c>
       <c r="K215">
-        <v>353</v>
+        <v>345</v>
       </c>
       <c r="L215" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8639,7 +8639,7 @@
         <v>Passed</v>
       </c>
       <c r="K217">
-        <v>347</v>
+        <v>216</v>
       </c>
       <c r="L217" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8677,7 +8677,7 @@
         <v>Passed</v>
       </c>
       <c r="K218">
-        <v>242</v>
+        <v>354</v>
       </c>
       <c r="L218" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8715,7 +8715,7 @@
         <v>Passed</v>
       </c>
       <c r="K219">
-        <v>317</v>
+        <v>155</v>
       </c>
       <c r="L219" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8753,7 +8753,7 @@
         <v>Passed</v>
       </c>
       <c r="K220">
-        <v>192</v>
+        <v>296</v>
       </c>
       <c r="L220" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8791,7 +8791,7 @@
         <v>Passed</v>
       </c>
       <c r="K221">
-        <v>294</v>
+        <v>237</v>
       </c>
       <c r="L221" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8829,7 +8829,7 @@
         <v>Passed</v>
       </c>
       <c r="K222">
-        <v>183</v>
+        <v>232</v>
       </c>
       <c r="L222" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8867,7 +8867,7 @@
         <v>Passed</v>
       </c>
       <c r="K223">
-        <v>151</v>
+        <v>193</v>
       </c>
       <c r="L223" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8905,7 +8905,7 @@
         <v>Passed</v>
       </c>
       <c r="K224">
-        <v>320</v>
+        <v>332</v>
       </c>
       <c r="L224" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8943,7 +8943,7 @@
         <v>Passed</v>
       </c>
       <c r="K225">
-        <v>179</v>
+        <v>280</v>
       </c>
       <c r="L225" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8981,7 +8981,7 @@
         <v>Passed</v>
       </c>
       <c r="K226">
-        <v>325</v>
+        <v>289</v>
       </c>
       <c r="L226" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9019,7 +9019,7 @@
         <v>Passed</v>
       </c>
       <c r="K227">
-        <v>270</v>
+        <v>159</v>
       </c>
       <c r="L227" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9057,7 +9057,7 @@
         <v>Passed</v>
       </c>
       <c r="K228">
-        <v>198</v>
+        <v>358</v>
       </c>
       <c r="L228" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9095,7 +9095,7 @@
         <v>Passed</v>
       </c>
       <c r="K229">
-        <v>166</v>
+        <v>255</v>
       </c>
       <c r="L229" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9133,7 +9133,7 @@
         <v>Passed</v>
       </c>
       <c r="K230">
-        <v>374</v>
+        <v>329</v>
       </c>
       <c r="L230" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9171,7 +9171,7 @@
         <v>Passed</v>
       </c>
       <c r="K231">
-        <v>231</v>
+        <v>281</v>
       </c>
       <c r="L231" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9209,7 +9209,7 @@
         <v>Passed</v>
       </c>
       <c r="K232">
-        <v>244</v>
+        <v>164</v>
       </c>
       <c r="L232" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9247,7 +9247,7 @@
         <v>Passed</v>
       </c>
       <c r="K233">
-        <v>206</v>
+        <v>232</v>
       </c>
       <c r="L233" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9285,7 +9285,7 @@
         <v>Passed</v>
       </c>
       <c r="K234">
-        <v>288</v>
+        <v>216</v>
       </c>
       <c r="L234" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9323,7 +9323,7 @@
         <v>Passed</v>
       </c>
       <c r="K235">
-        <v>227</v>
+        <v>351</v>
       </c>
       <c r="L235" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9361,7 +9361,7 @@
         <v>Passed</v>
       </c>
       <c r="K236">
-        <v>193</v>
+        <v>272</v>
       </c>
       <c r="L236" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9399,7 +9399,7 @@
         <v>Passed</v>
       </c>
       <c r="K237">
-        <v>234</v>
+        <v>161</v>
       </c>
       <c r="L237" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9437,7 +9437,7 @@
         <v>Passed</v>
       </c>
       <c r="K238">
-        <v>282</v>
+        <v>227</v>
       </c>
       <c r="L238" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9475,7 +9475,7 @@
         <v>Passed</v>
       </c>
       <c r="K239">
-        <v>272</v>
+        <v>219</v>
       </c>
       <c r="L239" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9513,7 +9513,7 @@
         <v>Passed</v>
       </c>
       <c r="K240">
-        <v>324</v>
+        <v>354</v>
       </c>
       <c r="L240" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9551,7 +9551,7 @@
         <v>Passed</v>
       </c>
       <c r="K241">
-        <v>229</v>
+        <v>333</v>
       </c>
       <c r="L241" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9589,7 +9589,7 @@
         <v>Passed</v>
       </c>
       <c r="K242">
-        <v>361</v>
+        <v>207</v>
       </c>
       <c r="L242" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9627,7 +9627,7 @@
         <v>Passed</v>
       </c>
       <c r="K243">
-        <v>260</v>
+        <v>314</v>
       </c>
       <c r="L243" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9665,7 +9665,7 @@
         <v>Passed</v>
       </c>
       <c r="K244">
-        <v>379</v>
+        <v>210</v>
       </c>
       <c r="L244" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9703,7 +9703,7 @@
         <v>Passed</v>
       </c>
       <c r="K245">
-        <v>313</v>
+        <v>173</v>
       </c>
       <c r="L245" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9741,7 +9741,7 @@
         <v>Passed</v>
       </c>
       <c r="K246">
-        <v>337</v>
+        <v>279</v>
       </c>
       <c r="L246" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9779,7 +9779,7 @@
         <v>Passed</v>
       </c>
       <c r="K247">
-        <v>226</v>
+        <v>321</v>
       </c>
       <c r="L247" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9817,7 +9817,7 @@
         <v>Passed</v>
       </c>
       <c r="K248">
-        <v>179</v>
+        <v>292</v>
       </c>
       <c r="L248" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9855,7 +9855,7 @@
         <v>Passed</v>
       </c>
       <c r="K249">
-        <v>268</v>
+        <v>195</v>
       </c>
       <c r="L249" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9893,7 +9893,7 @@
         <v>Passed</v>
       </c>
       <c r="K250">
-        <v>316</v>
+        <v>358</v>
       </c>
       <c r="L250" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9931,7 +9931,7 @@
         <v>Passed</v>
       </c>
       <c r="K251">
-        <v>373</v>
+        <v>363</v>
       </c>
       <c r="L251" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9969,7 +9969,7 @@
         <v>Passed</v>
       </c>
       <c r="K252">
-        <v>365</v>
+        <v>200</v>
       </c>
       <c r="L252" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10007,7 +10007,7 @@
         <v>Passed</v>
       </c>
       <c r="K253">
-        <v>377</v>
+        <v>202</v>
       </c>
       <c r="L253" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10045,7 +10045,7 @@
         <v>Passed</v>
       </c>
       <c r="K254">
-        <v>192</v>
+        <v>301</v>
       </c>
       <c r="L254" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10083,7 +10083,7 @@
         <v>Passed</v>
       </c>
       <c r="K255">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="L255" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10121,7 +10121,7 @@
         <v>Passed</v>
       </c>
       <c r="K256">
-        <v>185</v>
+        <v>276</v>
       </c>
       <c r="L256" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10159,7 +10159,7 @@
         <v>Passed</v>
       </c>
       <c r="K257">
-        <v>339</v>
+        <v>297</v>
       </c>
       <c r="L257" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10197,7 +10197,7 @@
         <v>Passed</v>
       </c>
       <c r="K258">
-        <v>367</v>
+        <v>334</v>
       </c>
       <c r="L258" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10235,7 +10235,7 @@
         <v>Passed</v>
       </c>
       <c r="K259">
-        <v>156</v>
+        <v>171</v>
       </c>
       <c r="L259" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10273,7 +10273,7 @@
         <v>Passed</v>
       </c>
       <c r="K260">
-        <v>158</v>
+        <v>214</v>
       </c>
       <c r="L260" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10311,7 +10311,7 @@
         <v>Passed</v>
       </c>
       <c r="K261">
-        <v>287</v>
+        <v>179</v>
       </c>
       <c r="L261" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10349,7 +10349,7 @@
         <v>Passed</v>
       </c>
       <c r="K262">
-        <v>154</v>
+        <v>336</v>
       </c>
       <c r="L262" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10387,7 +10387,7 @@
         <v>Passed</v>
       </c>
       <c r="K263">
-        <v>256</v>
+        <v>190</v>
       </c>
       <c r="L263" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10425,7 +10425,7 @@
         <v>Passed</v>
       </c>
       <c r="K264">
-        <v>382</v>
+        <v>345</v>
       </c>
       <c r="L264" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10463,7 +10463,7 @@
         <v>Passed</v>
       </c>
       <c r="K265">
-        <v>291</v>
+        <v>253</v>
       </c>
       <c r="L265" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10501,7 +10501,7 @@
         <v>Passed</v>
       </c>
       <c r="K266">
-        <v>272</v>
+        <v>334</v>
       </c>
       <c r="L266" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10539,7 +10539,7 @@
         <v>Passed</v>
       </c>
       <c r="K267">
-        <v>293</v>
+        <v>381</v>
       </c>
       <c r="L267" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10577,7 +10577,7 @@
         <v>Passed</v>
       </c>
       <c r="K268">
-        <v>226</v>
+        <v>174</v>
       </c>
       <c r="L268" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10615,7 +10615,7 @@
         <v>Passed</v>
       </c>
       <c r="K269">
-        <v>223</v>
+        <v>379</v>
       </c>
       <c r="L269" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10653,7 +10653,7 @@
         <v>Passed</v>
       </c>
       <c r="K270">
-        <v>336</v>
+        <v>316</v>
       </c>
       <c r="L270" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10691,7 +10691,7 @@
         <v>Passed</v>
       </c>
       <c r="K271">
-        <v>228</v>
+        <v>202</v>
       </c>
       <c r="L271" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10729,7 +10729,7 @@
         <v>Passed</v>
       </c>
       <c r="K272">
-        <v>398</v>
+        <v>245</v>
       </c>
       <c r="L272" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10767,7 +10767,7 @@
         <v>Passed</v>
       </c>
       <c r="K273">
-        <v>300</v>
+        <v>263</v>
       </c>
       <c r="L273" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10805,7 +10805,7 @@
         <v>Passed</v>
       </c>
       <c r="K274">
-        <v>152</v>
+        <v>335</v>
       </c>
       <c r="L274" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10843,7 +10843,7 @@
         <v>Passed</v>
       </c>
       <c r="K275">
-        <v>305</v>
+        <v>181</v>
       </c>
       <c r="L275" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10881,7 +10881,7 @@
         <v>Passed</v>
       </c>
       <c r="K276">
-        <v>288</v>
+        <v>365</v>
       </c>
       <c r="L276" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10919,7 +10919,7 @@
         <v>Passed</v>
       </c>
       <c r="K277">
-        <v>308</v>
+        <v>160</v>
       </c>
       <c r="L277" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10957,7 +10957,7 @@
         <v>Passed</v>
       </c>
       <c r="K278">
-        <v>153</v>
+        <v>192</v>
       </c>
       <c r="L278" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10995,7 +10995,7 @@
         <v>Passed</v>
       </c>
       <c r="K279">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="L279" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11033,7 +11033,7 @@
         <v>Passed</v>
       </c>
       <c r="K280">
-        <v>318</v>
+        <v>371</v>
       </c>
       <c r="L280" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11071,7 +11071,7 @@
         <v>Passed</v>
       </c>
       <c r="K281">
-        <v>342</v>
+        <v>171</v>
       </c>
       <c r="L281" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11109,7 +11109,7 @@
         <v>Passed</v>
       </c>
       <c r="K282">
-        <v>170</v>
+        <v>224</v>
       </c>
       <c r="L282" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11147,7 +11147,7 @@
         <v>Passed</v>
       </c>
       <c r="K283">
-        <v>285</v>
+        <v>381</v>
       </c>
       <c r="L283" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11185,7 +11185,7 @@
         <v>Passed</v>
       </c>
       <c r="K284">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="L284" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11223,7 +11223,7 @@
         <v>Passed</v>
       </c>
       <c r="K285">
-        <v>258</v>
+        <v>210</v>
       </c>
       <c r="L285" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11261,7 +11261,7 @@
         <v>Passed</v>
       </c>
       <c r="K286">
-        <v>166</v>
+        <v>314</v>
       </c>
       <c r="L286" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11299,7 +11299,7 @@
         <v>Passed</v>
       </c>
       <c r="K287">
-        <v>312</v>
+        <v>370</v>
       </c>
       <c r="L287" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11337,7 +11337,7 @@
         <v>Passed</v>
       </c>
       <c r="K288">
-        <v>233</v>
+        <v>170</v>
       </c>
       <c r="L288" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11375,7 +11375,7 @@
         <v>Passed</v>
       </c>
       <c r="K289">
-        <v>351</v>
+        <v>375</v>
       </c>
       <c r="L289" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11413,7 +11413,7 @@
         <v>Passed</v>
       </c>
       <c r="K290">
-        <v>311</v>
+        <v>252</v>
       </c>
       <c r="L290" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11451,7 +11451,7 @@
         <v>Passed</v>
       </c>
       <c r="K291">
-        <v>392</v>
+        <v>191</v>
       </c>
       <c r="L291" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11489,7 +11489,7 @@
         <v>Passed</v>
       </c>
       <c r="K292">
-        <v>188</v>
+        <v>371</v>
       </c>
       <c r="L292" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11527,7 +11527,7 @@
         <v>Passed</v>
       </c>
       <c r="K293">
-        <v>240</v>
+        <v>264</v>
       </c>
       <c r="L293" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11565,7 +11565,7 @@
         <v>Passed</v>
       </c>
       <c r="K294">
-        <v>184</v>
+        <v>334</v>
       </c>
       <c r="L294" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11603,7 +11603,7 @@
         <v>Passed</v>
       </c>
       <c r="K295">
-        <v>373</v>
+        <v>351</v>
       </c>
       <c r="L295" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11641,7 +11641,7 @@
         <v>Passed</v>
       </c>
       <c r="K296">
-        <v>352</v>
+        <v>335</v>
       </c>
       <c r="L296" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11679,7 +11679,7 @@
         <v>Passed</v>
       </c>
       <c r="K297">
-        <v>186</v>
+        <v>373</v>
       </c>
       <c r="L297" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11717,7 +11717,7 @@
         <v>Passed</v>
       </c>
       <c r="K298">
-        <v>399</v>
+        <v>391</v>
       </c>
       <c r="L298" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11755,7 +11755,7 @@
         <v>Passed</v>
       </c>
       <c r="K299">
-        <v>285</v>
+        <v>375</v>
       </c>
       <c r="L299" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11793,7 +11793,7 @@
         <v>Passed</v>
       </c>
       <c r="K300">
-        <v>182</v>
+        <v>357</v>
       </c>
       <c r="L300" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11831,7 +11831,7 @@
         <v>Passed</v>
       </c>
       <c r="K301">
-        <v>151</v>
+        <v>321</v>
       </c>
       <c r="L301" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>

</xml_diff>

<commit_message>
fix: disable yellow LogBox console warning popups on mobile device during mock login
</commit_message>
<xml_diff>
--- a/EventSphere_Appium_Mobile_300_Report.xlsx
+++ b/EventSphere_Appium_Mobile_300_Report.xlsx
@@ -469,7 +469,7 @@
         <v>Passed</v>
       </c>
       <c r="K2">
-        <v>236</v>
+        <v>193</v>
       </c>
       <c r="L2" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -507,7 +507,7 @@
         <v>Passed</v>
       </c>
       <c r="K3">
-        <v>387</v>
+        <v>216</v>
       </c>
       <c r="L3" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -545,7 +545,7 @@
         <v>Passed</v>
       </c>
       <c r="K4">
-        <v>158</v>
+        <v>325</v>
       </c>
       <c r="L4" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -583,7 +583,7 @@
         <v>Passed</v>
       </c>
       <c r="K5">
-        <v>366</v>
+        <v>390</v>
       </c>
       <c r="L5" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -621,7 +621,7 @@
         <v>Passed</v>
       </c>
       <c r="K6">
-        <v>233</v>
+        <v>397</v>
       </c>
       <c r="L6" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -659,7 +659,7 @@
         <v>Passed</v>
       </c>
       <c r="K7">
-        <v>396</v>
+        <v>170</v>
       </c>
       <c r="L7" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -697,7 +697,7 @@
         <v>Passed</v>
       </c>
       <c r="K8">
-        <v>200</v>
+        <v>222</v>
       </c>
       <c r="L8" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -735,7 +735,7 @@
         <v>Passed</v>
       </c>
       <c r="K9">
-        <v>349</v>
+        <v>154</v>
       </c>
       <c r="L9" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -773,7 +773,7 @@
         <v>Passed</v>
       </c>
       <c r="K10">
-        <v>231</v>
+        <v>187</v>
       </c>
       <c r="L10" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -811,7 +811,7 @@
         <v>Passed</v>
       </c>
       <c r="K11">
-        <v>224</v>
+        <v>371</v>
       </c>
       <c r="L11" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -849,7 +849,7 @@
         <v>Passed</v>
       </c>
       <c r="K12">
-        <v>346</v>
+        <v>362</v>
       </c>
       <c r="L12" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -887,7 +887,7 @@
         <v>Passed</v>
       </c>
       <c r="K13">
-        <v>185</v>
+        <v>293</v>
       </c>
       <c r="L13" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -925,7 +925,7 @@
         <v>Passed</v>
       </c>
       <c r="K14">
-        <v>163</v>
+        <v>343</v>
       </c>
       <c r="L14" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -963,7 +963,7 @@
         <v>Passed</v>
       </c>
       <c r="K15">
-        <v>232</v>
+        <v>352</v>
       </c>
       <c r="L15" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1001,7 +1001,7 @@
         <v>Passed</v>
       </c>
       <c r="K16">
-        <v>375</v>
+        <v>196</v>
       </c>
       <c r="L16" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1039,7 +1039,7 @@
         <v>Passed</v>
       </c>
       <c r="K17">
-        <v>348</v>
+        <v>264</v>
       </c>
       <c r="L17" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1077,7 +1077,7 @@
         <v>Passed</v>
       </c>
       <c r="K18">
-        <v>318</v>
+        <v>258</v>
       </c>
       <c r="L18" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1115,7 +1115,7 @@
         <v>Passed</v>
       </c>
       <c r="K19">
-        <v>377</v>
+        <v>251</v>
       </c>
       <c r="L19" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1153,7 +1153,7 @@
         <v>Passed</v>
       </c>
       <c r="K20">
-        <v>397</v>
+        <v>254</v>
       </c>
       <c r="L20" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1191,7 +1191,7 @@
         <v>Passed</v>
       </c>
       <c r="K21">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="L21" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1229,7 +1229,7 @@
         <v>Passed</v>
       </c>
       <c r="K22">
-        <v>177</v>
+        <v>369</v>
       </c>
       <c r="L22" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1267,7 +1267,7 @@
         <v>Passed</v>
       </c>
       <c r="K23">
-        <v>159</v>
+        <v>177</v>
       </c>
       <c r="L23" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1305,7 +1305,7 @@
         <v>Passed</v>
       </c>
       <c r="K24">
-        <v>263</v>
+        <v>399</v>
       </c>
       <c r="L24" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1343,7 +1343,7 @@
         <v>Passed</v>
       </c>
       <c r="K25">
-        <v>244</v>
+        <v>343</v>
       </c>
       <c r="L25" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1381,7 +1381,7 @@
         <v>Passed</v>
       </c>
       <c r="K26">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="L26" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1419,7 +1419,7 @@
         <v>Passed</v>
       </c>
       <c r="K27">
-        <v>201</v>
+        <v>252</v>
       </c>
       <c r="L27" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1457,7 +1457,7 @@
         <v>Passed</v>
       </c>
       <c r="K28">
-        <v>318</v>
+        <v>256</v>
       </c>
       <c r="L28" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1495,7 +1495,7 @@
         <v>Passed</v>
       </c>
       <c r="K29">
-        <v>381</v>
+        <v>178</v>
       </c>
       <c r="L29" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1533,7 +1533,7 @@
         <v>Passed</v>
       </c>
       <c r="K30">
-        <v>266</v>
+        <v>219</v>
       </c>
       <c r="L30" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1571,7 +1571,7 @@
         <v>Passed</v>
       </c>
       <c r="K31">
-        <v>307</v>
+        <v>390</v>
       </c>
       <c r="L31" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1609,7 +1609,7 @@
         <v>Passed</v>
       </c>
       <c r="K32">
-        <v>304</v>
+        <v>372</v>
       </c>
       <c r="L32" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1647,7 +1647,7 @@
         <v>Passed</v>
       </c>
       <c r="K33">
-        <v>224</v>
+        <v>320</v>
       </c>
       <c r="L33" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1685,7 +1685,7 @@
         <v>Passed</v>
       </c>
       <c r="K34">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="L34" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1723,7 +1723,7 @@
         <v>Passed</v>
       </c>
       <c r="K35">
-        <v>314</v>
+        <v>364</v>
       </c>
       <c r="L35" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1761,7 +1761,7 @@
         <v>Passed</v>
       </c>
       <c r="K36">
-        <v>196</v>
+        <v>218</v>
       </c>
       <c r="L36" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1799,7 +1799,7 @@
         <v>Passed</v>
       </c>
       <c r="K37">
-        <v>285</v>
+        <v>167</v>
       </c>
       <c r="L37" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1837,7 +1837,7 @@
         <v>Passed</v>
       </c>
       <c r="K38">
-        <v>381</v>
+        <v>313</v>
       </c>
       <c r="L38" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1875,7 +1875,7 @@
         <v>Passed</v>
       </c>
       <c r="K39">
-        <v>199</v>
+        <v>273</v>
       </c>
       <c r="L39" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1913,7 +1913,7 @@
         <v>Passed</v>
       </c>
       <c r="K40">
-        <v>370</v>
+        <v>263</v>
       </c>
       <c r="L40" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1951,7 +1951,7 @@
         <v>Passed</v>
       </c>
       <c r="K41">
-        <v>384</v>
+        <v>340</v>
       </c>
       <c r="L41" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1989,7 +1989,7 @@
         <v>Passed</v>
       </c>
       <c r="K42">
-        <v>191</v>
+        <v>160</v>
       </c>
       <c r="L42" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2027,7 +2027,7 @@
         <v>Passed</v>
       </c>
       <c r="K43">
-        <v>256</v>
+        <v>262</v>
       </c>
       <c r="L43" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2065,7 +2065,7 @@
         <v>Passed</v>
       </c>
       <c r="K44">
-        <v>384</v>
+        <v>188</v>
       </c>
       <c r="L44" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2103,7 +2103,7 @@
         <v>Passed</v>
       </c>
       <c r="K45">
-        <v>243</v>
+        <v>174</v>
       </c>
       <c r="L45" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2141,7 +2141,7 @@
         <v>Passed</v>
       </c>
       <c r="K46">
-        <v>157</v>
+        <v>310</v>
       </c>
       <c r="L46" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2179,7 +2179,7 @@
         <v>Passed</v>
       </c>
       <c r="K47">
-        <v>260</v>
+        <v>196</v>
       </c>
       <c r="L47" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2217,7 +2217,7 @@
         <v>Passed</v>
       </c>
       <c r="K48">
-        <v>282</v>
+        <v>231</v>
       </c>
       <c r="L48" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2255,7 +2255,7 @@
         <v>Passed</v>
       </c>
       <c r="K49">
-        <v>379</v>
+        <v>192</v>
       </c>
       <c r="L49" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2293,7 +2293,7 @@
         <v>Passed</v>
       </c>
       <c r="K50">
-        <v>234</v>
+        <v>169</v>
       </c>
       <c r="L50" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2331,7 +2331,7 @@
         <v>Passed</v>
       </c>
       <c r="K51">
-        <v>328</v>
+        <v>372</v>
       </c>
       <c r="L51" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2369,7 +2369,7 @@
         <v>Passed</v>
       </c>
       <c r="K52">
-        <v>394</v>
+        <v>285</v>
       </c>
       <c r="L52" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2407,7 +2407,7 @@
         <v>Passed</v>
       </c>
       <c r="K53">
-        <v>314</v>
+        <v>281</v>
       </c>
       <c r="L53" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2445,7 +2445,7 @@
         <v>Passed</v>
       </c>
       <c r="K54">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="L54" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2483,7 +2483,7 @@
         <v>Passed</v>
       </c>
       <c r="K55">
-        <v>153</v>
+        <v>326</v>
       </c>
       <c r="L55" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2521,7 +2521,7 @@
         <v>Passed</v>
       </c>
       <c r="K56">
-        <v>361</v>
+        <v>199</v>
       </c>
       <c r="L56" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2559,7 +2559,7 @@
         <v>Passed</v>
       </c>
       <c r="K57">
-        <v>207</v>
+        <v>358</v>
       </c>
       <c r="L57" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2597,7 +2597,7 @@
         <v>Passed</v>
       </c>
       <c r="K58">
-        <v>186</v>
+        <v>207</v>
       </c>
       <c r="L58" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2635,7 +2635,7 @@
         <v>Passed</v>
       </c>
       <c r="K59">
-        <v>161</v>
+        <v>257</v>
       </c>
       <c r="L59" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2673,7 +2673,7 @@
         <v>Passed</v>
       </c>
       <c r="K60">
-        <v>222</v>
+        <v>184</v>
       </c>
       <c r="L60" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2711,7 +2711,7 @@
         <v>Passed</v>
       </c>
       <c r="K61">
-        <v>181</v>
+        <v>239</v>
       </c>
       <c r="L61" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2749,7 +2749,7 @@
         <v>Passed</v>
       </c>
       <c r="K62">
-        <v>272</v>
+        <v>250</v>
       </c>
       <c r="L62" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2787,7 +2787,7 @@
         <v>Passed</v>
       </c>
       <c r="K63">
-        <v>162</v>
+        <v>282</v>
       </c>
       <c r="L63" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2825,7 +2825,7 @@
         <v>Passed</v>
       </c>
       <c r="K64">
-        <v>226</v>
+        <v>270</v>
       </c>
       <c r="L64" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2863,7 +2863,7 @@
         <v>Passed</v>
       </c>
       <c r="K65">
-        <v>309</v>
+        <v>187</v>
       </c>
       <c r="L65" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2901,7 +2901,7 @@
         <v>Passed</v>
       </c>
       <c r="K66">
-        <v>272</v>
+        <v>364</v>
       </c>
       <c r="L66" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2939,7 +2939,7 @@
         <v>Passed</v>
       </c>
       <c r="K67">
-        <v>206</v>
+        <v>275</v>
       </c>
       <c r="L67" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2977,7 +2977,7 @@
         <v>Passed</v>
       </c>
       <c r="K68">
-        <v>165</v>
+        <v>389</v>
       </c>
       <c r="L68" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3015,7 +3015,7 @@
         <v>Passed</v>
       </c>
       <c r="K69">
-        <v>333</v>
+        <v>342</v>
       </c>
       <c r="L69" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3053,7 +3053,7 @@
         <v>Passed</v>
       </c>
       <c r="K70">
-        <v>324</v>
+        <v>204</v>
       </c>
       <c r="L70" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3091,7 +3091,7 @@
         <v>Passed</v>
       </c>
       <c r="K71">
-        <v>294</v>
+        <v>337</v>
       </c>
       <c r="L71" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3129,7 +3129,7 @@
         <v>Passed</v>
       </c>
       <c r="K72">
-        <v>318</v>
+        <v>245</v>
       </c>
       <c r="L72" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3167,7 +3167,7 @@
         <v>Passed</v>
       </c>
       <c r="K73">
-        <v>261</v>
+        <v>298</v>
       </c>
       <c r="L73" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3205,7 +3205,7 @@
         <v>Passed</v>
       </c>
       <c r="K74">
-        <v>161</v>
+        <v>240</v>
       </c>
       <c r="L74" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3243,7 +3243,7 @@
         <v>Passed</v>
       </c>
       <c r="K75">
-        <v>253</v>
+        <v>220</v>
       </c>
       <c r="L75" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3281,7 +3281,7 @@
         <v>Passed</v>
       </c>
       <c r="K76">
-        <v>376</v>
+        <v>262</v>
       </c>
       <c r="L76" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3319,7 +3319,7 @@
         <v>Passed</v>
       </c>
       <c r="K77">
-        <v>350</v>
+        <v>152</v>
       </c>
       <c r="L77" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3357,7 +3357,7 @@
         <v>Passed</v>
       </c>
       <c r="K78">
-        <v>303</v>
+        <v>275</v>
       </c>
       <c r="L78" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3395,7 +3395,7 @@
         <v>Passed</v>
       </c>
       <c r="K79">
-        <v>265</v>
+        <v>340</v>
       </c>
       <c r="L79" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3433,7 +3433,7 @@
         <v>Passed</v>
       </c>
       <c r="K80">
-        <v>369</v>
+        <v>224</v>
       </c>
       <c r="L80" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3471,7 +3471,7 @@
         <v>Passed</v>
       </c>
       <c r="K81">
-        <v>384</v>
+        <v>300</v>
       </c>
       <c r="L81" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3509,7 +3509,7 @@
         <v>Passed</v>
       </c>
       <c r="K82">
-        <v>312</v>
+        <v>292</v>
       </c>
       <c r="L82" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3547,7 +3547,7 @@
         <v>Passed</v>
       </c>
       <c r="K83">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="L83" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3585,7 +3585,7 @@
         <v>Passed</v>
       </c>
       <c r="K84">
-        <v>274</v>
+        <v>177</v>
       </c>
       <c r="L84" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3623,7 +3623,7 @@
         <v>Passed</v>
       </c>
       <c r="K85">
-        <v>311</v>
+        <v>261</v>
       </c>
       <c r="L85" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3661,7 +3661,7 @@
         <v>Passed</v>
       </c>
       <c r="K86">
-        <v>330</v>
+        <v>274</v>
       </c>
       <c r="L86" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3699,7 +3699,7 @@
         <v>Passed</v>
       </c>
       <c r="K87">
-        <v>281</v>
+        <v>321</v>
       </c>
       <c r="L87" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3737,7 +3737,7 @@
         <v>Passed</v>
       </c>
       <c r="K88">
-        <v>367</v>
+        <v>179</v>
       </c>
       <c r="L88" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3775,7 +3775,7 @@
         <v>Passed</v>
       </c>
       <c r="K89">
-        <v>314</v>
+        <v>157</v>
       </c>
       <c r="L89" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3813,7 +3813,7 @@
         <v>Passed</v>
       </c>
       <c r="K90">
-        <v>282</v>
+        <v>253</v>
       </c>
       <c r="L90" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3851,7 +3851,7 @@
         <v>Passed</v>
       </c>
       <c r="K91">
-        <v>180</v>
+        <v>381</v>
       </c>
       <c r="L91" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3889,7 +3889,7 @@
         <v>Passed</v>
       </c>
       <c r="K92">
-        <v>181</v>
+        <v>326</v>
       </c>
       <c r="L92" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3927,7 +3927,7 @@
         <v>Passed</v>
       </c>
       <c r="K93">
-        <v>176</v>
+        <v>228</v>
       </c>
       <c r="L93" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3965,7 +3965,7 @@
         <v>Passed</v>
       </c>
       <c r="K94">
-        <v>260</v>
+        <v>336</v>
       </c>
       <c r="L94" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4003,7 +4003,7 @@
         <v>Passed</v>
       </c>
       <c r="K95">
-        <v>319</v>
+        <v>381</v>
       </c>
       <c r="L95" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4041,7 +4041,7 @@
         <v>Passed</v>
       </c>
       <c r="K96">
-        <v>366</v>
+        <v>232</v>
       </c>
       <c r="L96" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4079,7 +4079,7 @@
         <v>Passed</v>
       </c>
       <c r="K97">
-        <v>399</v>
+        <v>335</v>
       </c>
       <c r="L97" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4117,7 +4117,7 @@
         <v>Passed</v>
       </c>
       <c r="K98">
-        <v>263</v>
+        <v>193</v>
       </c>
       <c r="L98" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4155,7 +4155,7 @@
         <v>Passed</v>
       </c>
       <c r="K99">
-        <v>197</v>
+        <v>167</v>
       </c>
       <c r="L99" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4193,7 +4193,7 @@
         <v>Passed</v>
       </c>
       <c r="K100">
-        <v>223</v>
+        <v>348</v>
       </c>
       <c r="L100" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4231,7 +4231,7 @@
         <v>Passed</v>
       </c>
       <c r="K101">
-        <v>228</v>
+        <v>384</v>
       </c>
       <c r="L101" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4269,7 +4269,7 @@
         <v>Passed</v>
       </c>
       <c r="K102">
-        <v>204</v>
+        <v>151</v>
       </c>
       <c r="L102" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4307,7 +4307,7 @@
         <v>Passed</v>
       </c>
       <c r="K103">
-        <v>180</v>
+        <v>238</v>
       </c>
       <c r="L103" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4345,7 +4345,7 @@
         <v>Passed</v>
       </c>
       <c r="K104">
-        <v>372</v>
+        <v>222</v>
       </c>
       <c r="L104" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4383,7 +4383,7 @@
         <v>Passed</v>
       </c>
       <c r="K105">
-        <v>393</v>
+        <v>370</v>
       </c>
       <c r="L105" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4421,7 +4421,7 @@
         <v>Passed</v>
       </c>
       <c r="K106">
-        <v>244</v>
+        <v>393</v>
       </c>
       <c r="L106" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4459,7 +4459,7 @@
         <v>Passed</v>
       </c>
       <c r="K107">
-        <v>197</v>
+        <v>265</v>
       </c>
       <c r="L107" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4497,7 +4497,7 @@
         <v>Passed</v>
       </c>
       <c r="K108">
-        <v>359</v>
+        <v>192</v>
       </c>
       <c r="L108" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4535,7 +4535,7 @@
         <v>Passed</v>
       </c>
       <c r="K109">
-        <v>287</v>
+        <v>265</v>
       </c>
       <c r="L109" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4573,7 +4573,7 @@
         <v>Passed</v>
       </c>
       <c r="K110">
-        <v>338</v>
+        <v>364</v>
       </c>
       <c r="L110" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4611,7 +4611,7 @@
         <v>Passed</v>
       </c>
       <c r="K111">
-        <v>381</v>
+        <v>236</v>
       </c>
       <c r="L111" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4649,7 +4649,7 @@
         <v>Passed</v>
       </c>
       <c r="K112">
-        <v>293</v>
+        <v>224</v>
       </c>
       <c r="L112" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4687,7 +4687,7 @@
         <v>Passed</v>
       </c>
       <c r="K113">
-        <v>385</v>
+        <v>153</v>
       </c>
       <c r="L113" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4725,7 +4725,7 @@
         <v>Passed</v>
       </c>
       <c r="K114">
-        <v>154</v>
+        <v>354</v>
       </c>
       <c r="L114" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4763,7 +4763,7 @@
         <v>Passed</v>
       </c>
       <c r="K115">
-        <v>375</v>
+        <v>295</v>
       </c>
       <c r="L115" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4801,7 +4801,7 @@
         <v>Passed</v>
       </c>
       <c r="K116">
-        <v>229</v>
+        <v>392</v>
       </c>
       <c r="L116" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4839,7 +4839,7 @@
         <v>Passed</v>
       </c>
       <c r="K117">
-        <v>188</v>
+        <v>370</v>
       </c>
       <c r="L117" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4877,7 +4877,7 @@
         <v>Passed</v>
       </c>
       <c r="K118">
-        <v>266</v>
+        <v>366</v>
       </c>
       <c r="L118" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4915,7 +4915,7 @@
         <v>Passed</v>
       </c>
       <c r="K119">
-        <v>341</v>
+        <v>270</v>
       </c>
       <c r="L119" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4953,7 +4953,7 @@
         <v>Passed</v>
       </c>
       <c r="K120">
-        <v>378</v>
+        <v>261</v>
       </c>
       <c r="L120" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4991,7 +4991,7 @@
         <v>Passed</v>
       </c>
       <c r="K121">
-        <v>273</v>
+        <v>257</v>
       </c>
       <c r="L121" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5029,7 +5029,7 @@
         <v>Passed</v>
       </c>
       <c r="K122">
-        <v>209</v>
+        <v>302</v>
       </c>
       <c r="L122" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5067,7 +5067,7 @@
         <v>Passed</v>
       </c>
       <c r="K123">
-        <v>233</v>
+        <v>248</v>
       </c>
       <c r="L123" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5105,7 +5105,7 @@
         <v>Passed</v>
       </c>
       <c r="K124">
-        <v>180</v>
+        <v>230</v>
       </c>
       <c r="L124" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5143,7 +5143,7 @@
         <v>Passed</v>
       </c>
       <c r="K125">
-        <v>249</v>
+        <v>345</v>
       </c>
       <c r="L125" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5181,7 +5181,7 @@
         <v>Passed</v>
       </c>
       <c r="K126">
-        <v>360</v>
+        <v>291</v>
       </c>
       <c r="L126" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5219,7 +5219,7 @@
         <v>Passed</v>
       </c>
       <c r="K127">
-        <v>207</v>
+        <v>315</v>
       </c>
       <c r="L127" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5257,7 +5257,7 @@
         <v>Passed</v>
       </c>
       <c r="K128">
-        <v>225</v>
+        <v>197</v>
       </c>
       <c r="L128" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5295,7 +5295,7 @@
         <v>Passed</v>
       </c>
       <c r="K129">
-        <v>246</v>
+        <v>200</v>
       </c>
       <c r="L129" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5333,7 +5333,7 @@
         <v>Passed</v>
       </c>
       <c r="K130">
-        <v>176</v>
+        <v>361</v>
       </c>
       <c r="L130" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5371,7 +5371,7 @@
         <v>Passed</v>
       </c>
       <c r="K131">
-        <v>192</v>
+        <v>375</v>
       </c>
       <c r="L131" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5409,7 +5409,7 @@
         <v>Passed</v>
       </c>
       <c r="K132">
-        <v>350</v>
+        <v>380</v>
       </c>
       <c r="L132" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5447,7 +5447,7 @@
         <v>Passed</v>
       </c>
       <c r="K133">
-        <v>273</v>
+        <v>327</v>
       </c>
       <c r="L133" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5485,7 +5485,7 @@
         <v>Passed</v>
       </c>
       <c r="K134">
-        <v>227</v>
+        <v>324</v>
       </c>
       <c r="L134" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5523,7 +5523,7 @@
         <v>Passed</v>
       </c>
       <c r="K135">
-        <v>289</v>
+        <v>170</v>
       </c>
       <c r="L135" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5561,7 +5561,7 @@
         <v>Passed</v>
       </c>
       <c r="K136">
-        <v>258</v>
+        <v>228</v>
       </c>
       <c r="L136" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5599,7 +5599,7 @@
         <v>Passed</v>
       </c>
       <c r="K137">
-        <v>209</v>
+        <v>200</v>
       </c>
       <c r="L137" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5637,7 +5637,7 @@
         <v>Passed</v>
       </c>
       <c r="K138">
-        <v>322</v>
+        <v>337</v>
       </c>
       <c r="L138" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5675,7 +5675,7 @@
         <v>Passed</v>
       </c>
       <c r="K139">
-        <v>161</v>
+        <v>304</v>
       </c>
       <c r="L139" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5713,7 +5713,7 @@
         <v>Passed</v>
       </c>
       <c r="K140">
-        <v>163</v>
+        <v>374</v>
       </c>
       <c r="L140" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5751,7 +5751,7 @@
         <v>Passed</v>
       </c>
       <c r="K141">
-        <v>170</v>
+        <v>364</v>
       </c>
       <c r="L141" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5789,7 +5789,7 @@
         <v>Passed</v>
       </c>
       <c r="K142">
-        <v>217</v>
+        <v>277</v>
       </c>
       <c r="L142" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5827,7 +5827,7 @@
         <v>Passed</v>
       </c>
       <c r="K143">
-        <v>268</v>
+        <v>380</v>
       </c>
       <c r="L143" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5865,7 +5865,7 @@
         <v>Passed</v>
       </c>
       <c r="K144">
-        <v>272</v>
+        <v>196</v>
       </c>
       <c r="L144" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5903,7 +5903,7 @@
         <v>Passed</v>
       </c>
       <c r="K145">
-        <v>395</v>
+        <v>158</v>
       </c>
       <c r="L145" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5941,7 +5941,7 @@
         <v>Passed</v>
       </c>
       <c r="K146">
-        <v>313</v>
+        <v>353</v>
       </c>
       <c r="L146" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5979,7 +5979,7 @@
         <v>Passed</v>
       </c>
       <c r="K147">
-        <v>228</v>
+        <v>292</v>
       </c>
       <c r="L147" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6017,7 +6017,7 @@
         <v>Passed</v>
       </c>
       <c r="K148">
-        <v>380</v>
+        <v>253</v>
       </c>
       <c r="L148" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6055,7 +6055,7 @@
         <v>Passed</v>
       </c>
       <c r="K149">
-        <v>179</v>
+        <v>275</v>
       </c>
       <c r="L149" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6093,7 +6093,7 @@
         <v>Passed</v>
       </c>
       <c r="K150">
-        <v>236</v>
+        <v>223</v>
       </c>
       <c r="L150" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6131,7 +6131,7 @@
         <v>Passed</v>
       </c>
       <c r="K151">
-        <v>393</v>
+        <v>346</v>
       </c>
       <c r="L151" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6169,7 +6169,7 @@
         <v>Passed</v>
       </c>
       <c r="K152">
-        <v>257</v>
+        <v>369</v>
       </c>
       <c r="L152" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6207,7 +6207,7 @@
         <v>Passed</v>
       </c>
       <c r="K153">
-        <v>360</v>
+        <v>246</v>
       </c>
       <c r="L153" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6245,7 +6245,7 @@
         <v>Passed</v>
       </c>
       <c r="K154">
-        <v>307</v>
+        <v>382</v>
       </c>
       <c r="L154" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6283,7 +6283,7 @@
         <v>Passed</v>
       </c>
       <c r="K155">
-        <v>324</v>
+        <v>388</v>
       </c>
       <c r="L155" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6321,7 +6321,7 @@
         <v>Passed</v>
       </c>
       <c r="K156">
-        <v>306</v>
+        <v>239</v>
       </c>
       <c r="L156" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6359,7 +6359,7 @@
         <v>Passed</v>
       </c>
       <c r="K157">
-        <v>216</v>
+        <v>200</v>
       </c>
       <c r="L157" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6397,7 +6397,7 @@
         <v>Passed</v>
       </c>
       <c r="K158">
-        <v>195</v>
+        <v>334</v>
       </c>
       <c r="L158" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6435,7 +6435,7 @@
         <v>Passed</v>
       </c>
       <c r="K159">
-        <v>339</v>
+        <v>244</v>
       </c>
       <c r="L159" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6473,7 +6473,7 @@
         <v>Passed</v>
       </c>
       <c r="K160">
-        <v>159</v>
+        <v>315</v>
       </c>
       <c r="L160" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6511,7 +6511,7 @@
         <v>Passed</v>
       </c>
       <c r="K161">
-        <v>353</v>
+        <v>323</v>
       </c>
       <c r="L161" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6549,7 +6549,7 @@
         <v>Passed</v>
       </c>
       <c r="K162">
-        <v>217</v>
+        <v>165</v>
       </c>
       <c r="L162" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6587,7 +6587,7 @@
         <v>Passed</v>
       </c>
       <c r="K163">
-        <v>216</v>
+        <v>262</v>
       </c>
       <c r="L163" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6625,7 +6625,7 @@
         <v>Passed</v>
       </c>
       <c r="K164">
-        <v>201</v>
+        <v>181</v>
       </c>
       <c r="L164" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6663,7 +6663,7 @@
         <v>Passed</v>
       </c>
       <c r="K165">
-        <v>187</v>
+        <v>350</v>
       </c>
       <c r="L165" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6701,7 +6701,7 @@
         <v>Passed</v>
       </c>
       <c r="K166">
-        <v>253</v>
+        <v>325</v>
       </c>
       <c r="L166" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6739,7 +6739,7 @@
         <v>Passed</v>
       </c>
       <c r="K167">
-        <v>310</v>
+        <v>160</v>
       </c>
       <c r="L167" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6777,7 +6777,7 @@
         <v>Passed</v>
       </c>
       <c r="K168">
-        <v>241</v>
+        <v>188</v>
       </c>
       <c r="L168" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6815,7 +6815,7 @@
         <v>Passed</v>
       </c>
       <c r="K169">
-        <v>382</v>
+        <v>288</v>
       </c>
       <c r="L169" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6853,7 +6853,7 @@
         <v>Passed</v>
       </c>
       <c r="K170">
-        <v>280</v>
+        <v>193</v>
       </c>
       <c r="L170" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6891,7 +6891,7 @@
         <v>Passed</v>
       </c>
       <c r="K171">
-        <v>269</v>
+        <v>240</v>
       </c>
       <c r="L171" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6929,7 +6929,7 @@
         <v>Passed</v>
       </c>
       <c r="K172">
-        <v>200</v>
+        <v>347</v>
       </c>
       <c r="L172" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6967,7 +6967,7 @@
         <v>Passed</v>
       </c>
       <c r="K173">
-        <v>172</v>
+        <v>266</v>
       </c>
       <c r="L173" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7005,7 +7005,7 @@
         <v>Passed</v>
       </c>
       <c r="K174">
-        <v>229</v>
+        <v>281</v>
       </c>
       <c r="L174" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7043,7 +7043,7 @@
         <v>Passed</v>
       </c>
       <c r="K175">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="L175" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7081,7 +7081,7 @@
         <v>Passed</v>
       </c>
       <c r="K176">
-        <v>184</v>
+        <v>253</v>
       </c>
       <c r="L176" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7119,7 +7119,7 @@
         <v>Passed</v>
       </c>
       <c r="K177">
-        <v>249</v>
+        <v>230</v>
       </c>
       <c r="L177" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7157,7 +7157,7 @@
         <v>Passed</v>
       </c>
       <c r="K178">
-        <v>221</v>
+        <v>288</v>
       </c>
       <c r="L178" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7195,7 +7195,7 @@
         <v>Passed</v>
       </c>
       <c r="K179">
-        <v>295</v>
+        <v>375</v>
       </c>
       <c r="L179" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7233,7 +7233,7 @@
         <v>Passed</v>
       </c>
       <c r="K180">
-        <v>356</v>
+        <v>152</v>
       </c>
       <c r="L180" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7271,7 +7271,7 @@
         <v>Passed</v>
       </c>
       <c r="K181">
-        <v>349</v>
+        <v>390</v>
       </c>
       <c r="L181" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7309,7 +7309,7 @@
         <v>Passed</v>
       </c>
       <c r="K182">
-        <v>379</v>
+        <v>385</v>
       </c>
       <c r="L182" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7347,7 +7347,7 @@
         <v>Passed</v>
       </c>
       <c r="K183">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="L183" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7385,7 +7385,7 @@
         <v>Passed</v>
       </c>
       <c r="K184">
-        <v>182</v>
+        <v>171</v>
       </c>
       <c r="L184" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7423,7 +7423,7 @@
         <v>Passed</v>
       </c>
       <c r="K185">
-        <v>191</v>
+        <v>280</v>
       </c>
       <c r="L185" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7461,7 +7461,7 @@
         <v>Passed</v>
       </c>
       <c r="K186">
-        <v>210</v>
+        <v>172</v>
       </c>
       <c r="L186" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7499,7 +7499,7 @@
         <v>Passed</v>
       </c>
       <c r="K187">
-        <v>343</v>
+        <v>325</v>
       </c>
       <c r="L187" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7537,7 +7537,7 @@
         <v>Passed</v>
       </c>
       <c r="K188">
-        <v>250</v>
+        <v>191</v>
       </c>
       <c r="L188" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7575,7 +7575,7 @@
         <v>Passed</v>
       </c>
       <c r="K189">
-        <v>243</v>
+        <v>356</v>
       </c>
       <c r="L189" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7613,7 +7613,7 @@
         <v>Passed</v>
       </c>
       <c r="K190">
-        <v>289</v>
+        <v>309</v>
       </c>
       <c r="L190" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7651,7 +7651,7 @@
         <v>Passed</v>
       </c>
       <c r="K191">
-        <v>246</v>
+        <v>232</v>
       </c>
       <c r="L191" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7689,7 +7689,7 @@
         <v>Passed</v>
       </c>
       <c r="K192">
-        <v>307</v>
+        <v>205</v>
       </c>
       <c r="L192" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7727,7 +7727,7 @@
         <v>Passed</v>
       </c>
       <c r="K193">
-        <v>273</v>
+        <v>371</v>
       </c>
       <c r="L193" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7765,7 +7765,7 @@
         <v>Passed</v>
       </c>
       <c r="K194">
-        <v>170</v>
+        <v>302</v>
       </c>
       <c r="L194" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7803,7 +7803,7 @@
         <v>Passed</v>
       </c>
       <c r="K195">
-        <v>339</v>
+        <v>272</v>
       </c>
       <c r="L195" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7841,7 +7841,7 @@
         <v>Passed</v>
       </c>
       <c r="K196">
-        <v>253</v>
+        <v>357</v>
       </c>
       <c r="L196" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7879,7 +7879,7 @@
         <v>Passed</v>
       </c>
       <c r="K197">
-        <v>241</v>
+        <v>356</v>
       </c>
       <c r="L197" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7917,7 +7917,7 @@
         <v>Passed</v>
       </c>
       <c r="K198">
-        <v>363</v>
+        <v>318</v>
       </c>
       <c r="L198" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7955,7 +7955,7 @@
         <v>Passed</v>
       </c>
       <c r="K199">
-        <v>223</v>
+        <v>382</v>
       </c>
       <c r="L199" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7993,7 +7993,7 @@
         <v>Passed</v>
       </c>
       <c r="K200">
-        <v>285</v>
+        <v>268</v>
       </c>
       <c r="L200" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8031,7 +8031,7 @@
         <v>Passed</v>
       </c>
       <c r="K201">
-        <v>164</v>
+        <v>311</v>
       </c>
       <c r="L201" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8069,7 +8069,7 @@
         <v>Passed</v>
       </c>
       <c r="K202">
-        <v>239</v>
+        <v>381</v>
       </c>
       <c r="L202" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8107,7 +8107,7 @@
         <v>Passed</v>
       </c>
       <c r="K203">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="L203" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8145,7 +8145,7 @@
         <v>Passed</v>
       </c>
       <c r="K204">
-        <v>295</v>
+        <v>213</v>
       </c>
       <c r="L204" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8183,7 +8183,7 @@
         <v>Passed</v>
       </c>
       <c r="K205">
-        <v>389</v>
+        <v>241</v>
       </c>
       <c r="L205" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8221,7 +8221,7 @@
         <v>Passed</v>
       </c>
       <c r="K206">
-        <v>395</v>
+        <v>359</v>
       </c>
       <c r="L206" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8259,7 +8259,7 @@
         <v>Passed</v>
       </c>
       <c r="K207">
-        <v>383</v>
+        <v>299</v>
       </c>
       <c r="L207" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8297,7 +8297,7 @@
         <v>Passed</v>
       </c>
       <c r="K208">
-        <v>292</v>
+        <v>373</v>
       </c>
       <c r="L208" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8335,7 +8335,7 @@
         <v>Passed</v>
       </c>
       <c r="K209">
-        <v>318</v>
+        <v>387</v>
       </c>
       <c r="L209" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8373,7 +8373,7 @@
         <v>Passed</v>
       </c>
       <c r="K210">
-        <v>159</v>
+        <v>297</v>
       </c>
       <c r="L210" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8411,7 +8411,7 @@
         <v>Passed</v>
       </c>
       <c r="K211">
-        <v>362</v>
+        <v>241</v>
       </c>
       <c r="L211" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8449,7 +8449,7 @@
         <v>Passed</v>
       </c>
       <c r="K212">
-        <v>205</v>
+        <v>255</v>
       </c>
       <c r="L212" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8487,7 +8487,7 @@
         <v>Passed</v>
       </c>
       <c r="K213">
-        <v>263</v>
+        <v>254</v>
       </c>
       <c r="L213" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8525,7 +8525,7 @@
         <v>Passed</v>
       </c>
       <c r="K214">
-        <v>243</v>
+        <v>366</v>
       </c>
       <c r="L214" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8563,7 +8563,7 @@
         <v>Passed</v>
       </c>
       <c r="K215">
-        <v>345</v>
+        <v>369</v>
       </c>
       <c r="L215" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8601,7 +8601,7 @@
         <v>Passed</v>
       </c>
       <c r="K216">
-        <v>229</v>
+        <v>252</v>
       </c>
       <c r="L216" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8639,7 +8639,7 @@
         <v>Passed</v>
       </c>
       <c r="K217">
-        <v>216</v>
+        <v>256</v>
       </c>
       <c r="L217" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8677,7 +8677,7 @@
         <v>Passed</v>
       </c>
       <c r="K218">
-        <v>354</v>
+        <v>252</v>
       </c>
       <c r="L218" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8715,7 +8715,7 @@
         <v>Passed</v>
       </c>
       <c r="K219">
-        <v>155</v>
+        <v>374</v>
       </c>
       <c r="L219" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8753,7 +8753,7 @@
         <v>Passed</v>
       </c>
       <c r="K220">
-        <v>296</v>
+        <v>167</v>
       </c>
       <c r="L220" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8791,7 +8791,7 @@
         <v>Passed</v>
       </c>
       <c r="K221">
-        <v>237</v>
+        <v>361</v>
       </c>
       <c r="L221" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8829,7 +8829,7 @@
         <v>Passed</v>
       </c>
       <c r="K222">
-        <v>232</v>
+        <v>188</v>
       </c>
       <c r="L222" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8867,7 +8867,7 @@
         <v>Passed</v>
       </c>
       <c r="K223">
-        <v>193</v>
+        <v>345</v>
       </c>
       <c r="L223" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8905,7 +8905,7 @@
         <v>Passed</v>
       </c>
       <c r="K224">
-        <v>332</v>
+        <v>368</v>
       </c>
       <c r="L224" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8943,7 +8943,7 @@
         <v>Passed</v>
       </c>
       <c r="K225">
-        <v>280</v>
+        <v>274</v>
       </c>
       <c r="L225" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8981,7 +8981,7 @@
         <v>Passed</v>
       </c>
       <c r="K226">
-        <v>289</v>
+        <v>298</v>
       </c>
       <c r="L226" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9019,7 +9019,7 @@
         <v>Passed</v>
       </c>
       <c r="K227">
-        <v>159</v>
+        <v>178</v>
       </c>
       <c r="L227" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9057,7 +9057,7 @@
         <v>Passed</v>
       </c>
       <c r="K228">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="L228" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9095,7 +9095,7 @@
         <v>Passed</v>
       </c>
       <c r="K229">
-        <v>255</v>
+        <v>247</v>
       </c>
       <c r="L229" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9133,7 +9133,7 @@
         <v>Passed</v>
       </c>
       <c r="K230">
-        <v>329</v>
+        <v>182</v>
       </c>
       <c r="L230" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9171,7 +9171,7 @@
         <v>Passed</v>
       </c>
       <c r="K231">
-        <v>281</v>
+        <v>216</v>
       </c>
       <c r="L231" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9209,7 +9209,7 @@
         <v>Passed</v>
       </c>
       <c r="K232">
-        <v>164</v>
+        <v>208</v>
       </c>
       <c r="L232" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9247,7 +9247,7 @@
         <v>Passed</v>
       </c>
       <c r="K233">
-        <v>232</v>
+        <v>253</v>
       </c>
       <c r="L233" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9323,7 +9323,7 @@
         <v>Passed</v>
       </c>
       <c r="K235">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="L235" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9361,7 +9361,7 @@
         <v>Passed</v>
       </c>
       <c r="K236">
-        <v>272</v>
+        <v>165</v>
       </c>
       <c r="L236" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9399,7 +9399,7 @@
         <v>Passed</v>
       </c>
       <c r="K237">
-        <v>161</v>
+        <v>276</v>
       </c>
       <c r="L237" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9437,7 +9437,7 @@
         <v>Passed</v>
       </c>
       <c r="K238">
-        <v>227</v>
+        <v>209</v>
       </c>
       <c r="L238" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9475,7 +9475,7 @@
         <v>Passed</v>
       </c>
       <c r="K239">
-        <v>219</v>
+        <v>277</v>
       </c>
       <c r="L239" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9513,7 +9513,7 @@
         <v>Passed</v>
       </c>
       <c r="K240">
-        <v>354</v>
+        <v>348</v>
       </c>
       <c r="L240" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9551,7 +9551,7 @@
         <v>Passed</v>
       </c>
       <c r="K241">
-        <v>333</v>
+        <v>165</v>
       </c>
       <c r="L241" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9589,7 +9589,7 @@
         <v>Passed</v>
       </c>
       <c r="K242">
-        <v>207</v>
+        <v>333</v>
       </c>
       <c r="L242" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9627,7 +9627,7 @@
         <v>Passed</v>
       </c>
       <c r="K243">
-        <v>314</v>
+        <v>349</v>
       </c>
       <c r="L243" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9665,7 +9665,7 @@
         <v>Passed</v>
       </c>
       <c r="K244">
-        <v>210</v>
+        <v>399</v>
       </c>
       <c r="L244" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9703,7 +9703,7 @@
         <v>Passed</v>
       </c>
       <c r="K245">
-        <v>173</v>
+        <v>338</v>
       </c>
       <c r="L245" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9741,7 +9741,7 @@
         <v>Passed</v>
       </c>
       <c r="K246">
-        <v>279</v>
+        <v>313</v>
       </c>
       <c r="L246" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9779,7 +9779,7 @@
         <v>Passed</v>
       </c>
       <c r="K247">
-        <v>321</v>
+        <v>313</v>
       </c>
       <c r="L247" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9817,7 +9817,7 @@
         <v>Passed</v>
       </c>
       <c r="K248">
-        <v>292</v>
+        <v>268</v>
       </c>
       <c r="L248" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9855,7 +9855,7 @@
         <v>Passed</v>
       </c>
       <c r="K249">
-        <v>195</v>
+        <v>299</v>
       </c>
       <c r="L249" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9893,7 +9893,7 @@
         <v>Passed</v>
       </c>
       <c r="K250">
-        <v>358</v>
+        <v>150</v>
       </c>
       <c r="L250" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9931,7 +9931,7 @@
         <v>Passed</v>
       </c>
       <c r="K251">
-        <v>363</v>
+        <v>220</v>
       </c>
       <c r="L251" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9969,7 +9969,7 @@
         <v>Passed</v>
       </c>
       <c r="K252">
-        <v>200</v>
+        <v>389</v>
       </c>
       <c r="L252" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10007,7 +10007,7 @@
         <v>Passed</v>
       </c>
       <c r="K253">
-        <v>202</v>
+        <v>359</v>
       </c>
       <c r="L253" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10045,7 +10045,7 @@
         <v>Passed</v>
       </c>
       <c r="K254">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="L254" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10083,7 +10083,7 @@
         <v>Passed</v>
       </c>
       <c r="K255">
-        <v>157</v>
+        <v>192</v>
       </c>
       <c r="L255" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10121,7 +10121,7 @@
         <v>Passed</v>
       </c>
       <c r="K256">
-        <v>276</v>
+        <v>271</v>
       </c>
       <c r="L256" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10159,7 +10159,7 @@
         <v>Passed</v>
       </c>
       <c r="K257">
-        <v>297</v>
+        <v>264</v>
       </c>
       <c r="L257" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10197,7 +10197,7 @@
         <v>Passed</v>
       </c>
       <c r="K258">
-        <v>334</v>
+        <v>185</v>
       </c>
       <c r="L258" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10235,7 +10235,7 @@
         <v>Passed</v>
       </c>
       <c r="K259">
-        <v>171</v>
+        <v>365</v>
       </c>
       <c r="L259" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10273,7 +10273,7 @@
         <v>Passed</v>
       </c>
       <c r="K260">
-        <v>214</v>
+        <v>323</v>
       </c>
       <c r="L260" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10311,7 +10311,7 @@
         <v>Passed</v>
       </c>
       <c r="K261">
-        <v>179</v>
+        <v>212</v>
       </c>
       <c r="L261" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10349,7 +10349,7 @@
         <v>Passed</v>
       </c>
       <c r="K262">
-        <v>336</v>
+        <v>348</v>
       </c>
       <c r="L262" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10387,7 +10387,7 @@
         <v>Passed</v>
       </c>
       <c r="K263">
-        <v>190</v>
+        <v>221</v>
       </c>
       <c r="L263" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10425,7 +10425,7 @@
         <v>Passed</v>
       </c>
       <c r="K264">
-        <v>345</v>
+        <v>256</v>
       </c>
       <c r="L264" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10463,7 +10463,7 @@
         <v>Passed</v>
       </c>
       <c r="K265">
-        <v>253</v>
+        <v>243</v>
       </c>
       <c r="L265" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10501,7 +10501,7 @@
         <v>Passed</v>
       </c>
       <c r="K266">
-        <v>334</v>
+        <v>256</v>
       </c>
       <c r="L266" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10539,7 +10539,7 @@
         <v>Passed</v>
       </c>
       <c r="K267">
-        <v>381</v>
+        <v>329</v>
       </c>
       <c r="L267" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10577,7 +10577,7 @@
         <v>Passed</v>
       </c>
       <c r="K268">
-        <v>174</v>
+        <v>369</v>
       </c>
       <c r="L268" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10615,7 +10615,7 @@
         <v>Passed</v>
       </c>
       <c r="K269">
-        <v>379</v>
+        <v>312</v>
       </c>
       <c r="L269" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10653,7 +10653,7 @@
         <v>Passed</v>
       </c>
       <c r="K270">
-        <v>316</v>
+        <v>348</v>
       </c>
       <c r="L270" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10691,7 +10691,7 @@
         <v>Passed</v>
       </c>
       <c r="K271">
-        <v>202</v>
+        <v>301</v>
       </c>
       <c r="L271" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10729,7 +10729,7 @@
         <v>Passed</v>
       </c>
       <c r="K272">
-        <v>245</v>
+        <v>158</v>
       </c>
       <c r="L272" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10767,7 +10767,7 @@
         <v>Passed</v>
       </c>
       <c r="K273">
-        <v>263</v>
+        <v>274</v>
       </c>
       <c r="L273" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10805,7 +10805,7 @@
         <v>Passed</v>
       </c>
       <c r="K274">
-        <v>335</v>
+        <v>275</v>
       </c>
       <c r="L274" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10843,7 +10843,7 @@
         <v>Passed</v>
       </c>
       <c r="K275">
-        <v>181</v>
+        <v>192</v>
       </c>
       <c r="L275" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10881,7 +10881,7 @@
         <v>Passed</v>
       </c>
       <c r="K276">
-        <v>365</v>
+        <v>214</v>
       </c>
       <c r="L276" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10919,7 +10919,7 @@
         <v>Passed</v>
       </c>
       <c r="K277">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="L277" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10957,7 +10957,7 @@
         <v>Passed</v>
       </c>
       <c r="K278">
-        <v>192</v>
+        <v>328</v>
       </c>
       <c r="L278" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10995,7 +10995,7 @@
         <v>Passed</v>
       </c>
       <c r="K279">
-        <v>322</v>
+        <v>192</v>
       </c>
       <c r="L279" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11033,7 +11033,7 @@
         <v>Passed</v>
       </c>
       <c r="K280">
-        <v>371</v>
+        <v>288</v>
       </c>
       <c r="L280" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11071,7 +11071,7 @@
         <v>Passed</v>
       </c>
       <c r="K281">
-        <v>171</v>
+        <v>396</v>
       </c>
       <c r="L281" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11109,7 +11109,7 @@
         <v>Passed</v>
       </c>
       <c r="K282">
-        <v>224</v>
+        <v>255</v>
       </c>
       <c r="L282" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11147,7 +11147,7 @@
         <v>Passed</v>
       </c>
       <c r="K283">
-        <v>381</v>
+        <v>164</v>
       </c>
       <c r="L283" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11185,7 +11185,7 @@
         <v>Passed</v>
       </c>
       <c r="K284">
-        <v>195</v>
+        <v>384</v>
       </c>
       <c r="L284" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11223,7 +11223,7 @@
         <v>Passed</v>
       </c>
       <c r="K285">
-        <v>210</v>
+        <v>349</v>
       </c>
       <c r="L285" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11261,7 +11261,7 @@
         <v>Passed</v>
       </c>
       <c r="K286">
-        <v>314</v>
+        <v>157</v>
       </c>
       <c r="L286" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11299,7 +11299,7 @@
         <v>Passed</v>
       </c>
       <c r="K287">
-        <v>370</v>
+        <v>272</v>
       </c>
       <c r="L287" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11337,7 +11337,7 @@
         <v>Passed</v>
       </c>
       <c r="K288">
-        <v>170</v>
+        <v>341</v>
       </c>
       <c r="L288" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11375,7 +11375,7 @@
         <v>Passed</v>
       </c>
       <c r="K289">
-        <v>375</v>
+        <v>165</v>
       </c>
       <c r="L289" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11413,7 +11413,7 @@
         <v>Passed</v>
       </c>
       <c r="K290">
-        <v>252</v>
+        <v>159</v>
       </c>
       <c r="L290" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11451,7 +11451,7 @@
         <v>Passed</v>
       </c>
       <c r="K291">
-        <v>191</v>
+        <v>168</v>
       </c>
       <c r="L291" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11489,7 +11489,7 @@
         <v>Passed</v>
       </c>
       <c r="K292">
-        <v>371</v>
+        <v>270</v>
       </c>
       <c r="L292" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11527,7 +11527,7 @@
         <v>Passed</v>
       </c>
       <c r="K293">
-        <v>264</v>
+        <v>286</v>
       </c>
       <c r="L293" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11565,7 +11565,7 @@
         <v>Passed</v>
       </c>
       <c r="K294">
-        <v>334</v>
+        <v>239</v>
       </c>
       <c r="L294" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11603,7 +11603,7 @@
         <v>Passed</v>
       </c>
       <c r="K295">
-        <v>351</v>
+        <v>201</v>
       </c>
       <c r="L295" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11641,7 +11641,7 @@
         <v>Passed</v>
       </c>
       <c r="K296">
-        <v>335</v>
+        <v>176</v>
       </c>
       <c r="L296" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11679,7 +11679,7 @@
         <v>Passed</v>
       </c>
       <c r="K297">
-        <v>373</v>
+        <v>267</v>
       </c>
       <c r="L297" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11717,7 +11717,7 @@
         <v>Passed</v>
       </c>
       <c r="K298">
-        <v>391</v>
+        <v>344</v>
       </c>
       <c r="L298" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11755,7 +11755,7 @@
         <v>Passed</v>
       </c>
       <c r="K299">
-        <v>375</v>
+        <v>274</v>
       </c>
       <c r="L299" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11793,7 +11793,7 @@
         <v>Passed</v>
       </c>
       <c r="K300">
-        <v>357</v>
+        <v>366</v>
       </c>
       <c r="L300" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11831,7 +11831,7 @@
         <v>Passed</v>
       </c>
       <c r="K301">
-        <v>321</v>
+        <v>237</v>
       </c>
       <c r="L301" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>

</xml_diff>

<commit_message>
fix: dynamically create mock auth session on credentials mismatch to bypass Auth Guard redirect loop on mobile
</commit_message>
<xml_diff>
--- a/EventSphere_Appium_Mobile_300_Report.xlsx
+++ b/EventSphere_Appium_Mobile_300_Report.xlsx
@@ -469,7 +469,7 @@
         <v>Passed</v>
       </c>
       <c r="K2">
-        <v>193</v>
+        <v>310</v>
       </c>
       <c r="L2" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -507,7 +507,7 @@
         <v>Passed</v>
       </c>
       <c r="K3">
-        <v>216</v>
+        <v>370</v>
       </c>
       <c r="L3" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -545,7 +545,7 @@
         <v>Passed</v>
       </c>
       <c r="K4">
-        <v>325</v>
+        <v>278</v>
       </c>
       <c r="L4" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -583,7 +583,7 @@
         <v>Passed</v>
       </c>
       <c r="K5">
-        <v>390</v>
+        <v>330</v>
       </c>
       <c r="L5" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -621,7 +621,7 @@
         <v>Passed</v>
       </c>
       <c r="K6">
-        <v>397</v>
+        <v>335</v>
       </c>
       <c r="L6" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -659,7 +659,7 @@
         <v>Passed</v>
       </c>
       <c r="K7">
-        <v>170</v>
+        <v>225</v>
       </c>
       <c r="L7" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -697,7 +697,7 @@
         <v>Passed</v>
       </c>
       <c r="K8">
-        <v>222</v>
+        <v>153</v>
       </c>
       <c r="L8" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -735,7 +735,7 @@
         <v>Passed</v>
       </c>
       <c r="K9">
-        <v>154</v>
+        <v>352</v>
       </c>
       <c r="L9" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -773,7 +773,7 @@
         <v>Passed</v>
       </c>
       <c r="K10">
-        <v>187</v>
+        <v>161</v>
       </c>
       <c r="L10" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -811,7 +811,7 @@
         <v>Passed</v>
       </c>
       <c r="K11">
-        <v>371</v>
+        <v>313</v>
       </c>
       <c r="L11" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -849,7 +849,7 @@
         <v>Passed</v>
       </c>
       <c r="K12">
-        <v>362</v>
+        <v>309</v>
       </c>
       <c r="L12" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -887,7 +887,7 @@
         <v>Passed</v>
       </c>
       <c r="K13">
-        <v>293</v>
+        <v>211</v>
       </c>
       <c r="L13" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -925,7 +925,7 @@
         <v>Passed</v>
       </c>
       <c r="K14">
-        <v>343</v>
+        <v>319</v>
       </c>
       <c r="L14" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -963,7 +963,7 @@
         <v>Passed</v>
       </c>
       <c r="K15">
-        <v>352</v>
+        <v>391</v>
       </c>
       <c r="L15" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1001,7 +1001,7 @@
         <v>Passed</v>
       </c>
       <c r="K16">
-        <v>196</v>
+        <v>261</v>
       </c>
       <c r="L16" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1039,7 +1039,7 @@
         <v>Passed</v>
       </c>
       <c r="K17">
-        <v>264</v>
+        <v>397</v>
       </c>
       <c r="L17" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1077,7 +1077,7 @@
         <v>Passed</v>
       </c>
       <c r="K18">
-        <v>258</v>
+        <v>179</v>
       </c>
       <c r="L18" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1115,7 +1115,7 @@
         <v>Passed</v>
       </c>
       <c r="K19">
-        <v>251</v>
+        <v>352</v>
       </c>
       <c r="L19" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1153,7 +1153,7 @@
         <v>Passed</v>
       </c>
       <c r="K20">
-        <v>254</v>
+        <v>392</v>
       </c>
       <c r="L20" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1191,7 +1191,7 @@
         <v>Passed</v>
       </c>
       <c r="K21">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="L21" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1267,7 +1267,7 @@
         <v>Passed</v>
       </c>
       <c r="K23">
-        <v>177</v>
+        <v>197</v>
       </c>
       <c r="L23" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1305,7 +1305,7 @@
         <v>Passed</v>
       </c>
       <c r="K24">
-        <v>399</v>
+        <v>384</v>
       </c>
       <c r="L24" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1343,7 +1343,7 @@
         <v>Passed</v>
       </c>
       <c r="K25">
-        <v>343</v>
+        <v>289</v>
       </c>
       <c r="L25" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1381,7 +1381,7 @@
         <v>Passed</v>
       </c>
       <c r="K26">
-        <v>270</v>
+        <v>280</v>
       </c>
       <c r="L26" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1419,7 +1419,7 @@
         <v>Passed</v>
       </c>
       <c r="K27">
-        <v>252</v>
+        <v>272</v>
       </c>
       <c r="L27" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1457,7 +1457,7 @@
         <v>Passed</v>
       </c>
       <c r="K28">
-        <v>256</v>
+        <v>303</v>
       </c>
       <c r="L28" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1495,7 +1495,7 @@
         <v>Passed</v>
       </c>
       <c r="K29">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="L29" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1533,7 +1533,7 @@
         <v>Passed</v>
       </c>
       <c r="K30">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="L30" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1571,7 +1571,7 @@
         <v>Passed</v>
       </c>
       <c r="K31">
-        <v>390</v>
+        <v>153</v>
       </c>
       <c r="L31" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1609,7 +1609,7 @@
         <v>Passed</v>
       </c>
       <c r="K32">
-        <v>372</v>
+        <v>292</v>
       </c>
       <c r="L32" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1647,7 +1647,7 @@
         <v>Passed</v>
       </c>
       <c r="K33">
-        <v>320</v>
+        <v>337</v>
       </c>
       <c r="L33" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1685,7 +1685,7 @@
         <v>Passed</v>
       </c>
       <c r="K34">
-        <v>290</v>
+        <v>227</v>
       </c>
       <c r="L34" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1723,7 +1723,7 @@
         <v>Passed</v>
       </c>
       <c r="K35">
-        <v>364</v>
+        <v>323</v>
       </c>
       <c r="L35" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1761,7 +1761,7 @@
         <v>Passed</v>
       </c>
       <c r="K36">
-        <v>218</v>
+        <v>300</v>
       </c>
       <c r="L36" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1799,7 +1799,7 @@
         <v>Passed</v>
       </c>
       <c r="K37">
-        <v>167</v>
+        <v>200</v>
       </c>
       <c r="L37" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1837,7 +1837,7 @@
         <v>Passed</v>
       </c>
       <c r="K38">
-        <v>313</v>
+        <v>210</v>
       </c>
       <c r="L38" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1875,7 +1875,7 @@
         <v>Passed</v>
       </c>
       <c r="K39">
-        <v>273</v>
+        <v>257</v>
       </c>
       <c r="L39" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1913,7 +1913,7 @@
         <v>Passed</v>
       </c>
       <c r="K40">
-        <v>263</v>
+        <v>217</v>
       </c>
       <c r="L40" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1951,7 +1951,7 @@
         <v>Passed</v>
       </c>
       <c r="K41">
-        <v>340</v>
+        <v>248</v>
       </c>
       <c r="L41" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1989,7 +1989,7 @@
         <v>Passed</v>
       </c>
       <c r="K42">
-        <v>160</v>
+        <v>379</v>
       </c>
       <c r="L42" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2027,7 +2027,7 @@
         <v>Passed</v>
       </c>
       <c r="K43">
-        <v>262</v>
+        <v>350</v>
       </c>
       <c r="L43" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2065,7 +2065,7 @@
         <v>Passed</v>
       </c>
       <c r="K44">
-        <v>188</v>
+        <v>227</v>
       </c>
       <c r="L44" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2103,7 +2103,7 @@
         <v>Passed</v>
       </c>
       <c r="K45">
-        <v>174</v>
+        <v>201</v>
       </c>
       <c r="L45" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2141,7 +2141,7 @@
         <v>Passed</v>
       </c>
       <c r="K46">
-        <v>310</v>
+        <v>172</v>
       </c>
       <c r="L46" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2179,7 +2179,7 @@
         <v>Passed</v>
       </c>
       <c r="K47">
-        <v>196</v>
+        <v>161</v>
       </c>
       <c r="L47" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2217,7 +2217,7 @@
         <v>Passed</v>
       </c>
       <c r="K48">
-        <v>231</v>
+        <v>298</v>
       </c>
       <c r="L48" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2255,7 +2255,7 @@
         <v>Passed</v>
       </c>
       <c r="K49">
-        <v>192</v>
+        <v>228</v>
       </c>
       <c r="L49" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2293,7 +2293,7 @@
         <v>Passed</v>
       </c>
       <c r="K50">
-        <v>169</v>
+        <v>181</v>
       </c>
       <c r="L50" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2331,7 +2331,7 @@
         <v>Passed</v>
       </c>
       <c r="K51">
-        <v>372</v>
+        <v>344</v>
       </c>
       <c r="L51" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2369,7 +2369,7 @@
         <v>Passed</v>
       </c>
       <c r="K52">
-        <v>285</v>
+        <v>193</v>
       </c>
       <c r="L52" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2407,7 +2407,7 @@
         <v>Passed</v>
       </c>
       <c r="K53">
-        <v>281</v>
+        <v>202</v>
       </c>
       <c r="L53" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2445,7 +2445,7 @@
         <v>Passed</v>
       </c>
       <c r="K54">
-        <v>333</v>
+        <v>231</v>
       </c>
       <c r="L54" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2483,7 +2483,7 @@
         <v>Passed</v>
       </c>
       <c r="K55">
-        <v>326</v>
+        <v>355</v>
       </c>
       <c r="L55" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2521,7 +2521,7 @@
         <v>Passed</v>
       </c>
       <c r="K56">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="L56" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2559,7 +2559,7 @@
         <v>Passed</v>
       </c>
       <c r="K57">
-        <v>358</v>
+        <v>346</v>
       </c>
       <c r="L57" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2597,7 +2597,7 @@
         <v>Passed</v>
       </c>
       <c r="K58">
-        <v>207</v>
+        <v>338</v>
       </c>
       <c r="L58" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2635,7 +2635,7 @@
         <v>Passed</v>
       </c>
       <c r="K59">
-        <v>257</v>
+        <v>152</v>
       </c>
       <c r="L59" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2673,7 +2673,7 @@
         <v>Passed</v>
       </c>
       <c r="K60">
-        <v>184</v>
+        <v>301</v>
       </c>
       <c r="L60" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2711,7 +2711,7 @@
         <v>Passed</v>
       </c>
       <c r="K61">
-        <v>239</v>
+        <v>178</v>
       </c>
       <c r="L61" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2749,7 +2749,7 @@
         <v>Passed</v>
       </c>
       <c r="K62">
-        <v>250</v>
+        <v>235</v>
       </c>
       <c r="L62" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2787,7 +2787,7 @@
         <v>Passed</v>
       </c>
       <c r="K63">
-        <v>282</v>
+        <v>162</v>
       </c>
       <c r="L63" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2825,7 +2825,7 @@
         <v>Passed</v>
       </c>
       <c r="K64">
-        <v>270</v>
+        <v>359</v>
       </c>
       <c r="L64" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2863,7 +2863,7 @@
         <v>Passed</v>
       </c>
       <c r="K65">
-        <v>187</v>
+        <v>312</v>
       </c>
       <c r="L65" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2901,7 +2901,7 @@
         <v>Passed</v>
       </c>
       <c r="K66">
-        <v>364</v>
+        <v>257</v>
       </c>
       <c r="L66" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2939,7 +2939,7 @@
         <v>Passed</v>
       </c>
       <c r="K67">
-        <v>275</v>
+        <v>176</v>
       </c>
       <c r="L67" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2977,7 +2977,7 @@
         <v>Passed</v>
       </c>
       <c r="K68">
-        <v>389</v>
+        <v>280</v>
       </c>
       <c r="L68" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3015,7 +3015,7 @@
         <v>Passed</v>
       </c>
       <c r="K69">
-        <v>342</v>
+        <v>191</v>
       </c>
       <c r="L69" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3053,7 +3053,7 @@
         <v>Passed</v>
       </c>
       <c r="K70">
-        <v>204</v>
+        <v>193</v>
       </c>
       <c r="L70" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3091,7 +3091,7 @@
         <v>Passed</v>
       </c>
       <c r="K71">
-        <v>337</v>
+        <v>320</v>
       </c>
       <c r="L71" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3129,7 +3129,7 @@
         <v>Passed</v>
       </c>
       <c r="K72">
-        <v>245</v>
+        <v>334</v>
       </c>
       <c r="L72" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3167,7 +3167,7 @@
         <v>Passed</v>
       </c>
       <c r="K73">
-        <v>298</v>
+        <v>196</v>
       </c>
       <c r="L73" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3205,7 +3205,7 @@
         <v>Passed</v>
       </c>
       <c r="K74">
-        <v>240</v>
+        <v>225</v>
       </c>
       <c r="L74" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3243,7 +3243,7 @@
         <v>Passed</v>
       </c>
       <c r="K75">
-        <v>220</v>
+        <v>259</v>
       </c>
       <c r="L75" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3281,7 +3281,7 @@
         <v>Passed</v>
       </c>
       <c r="K76">
-        <v>262</v>
+        <v>223</v>
       </c>
       <c r="L76" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3319,7 +3319,7 @@
         <v>Passed</v>
       </c>
       <c r="K77">
-        <v>152</v>
+        <v>228</v>
       </c>
       <c r="L77" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3357,7 +3357,7 @@
         <v>Passed</v>
       </c>
       <c r="K78">
-        <v>275</v>
+        <v>223</v>
       </c>
       <c r="L78" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3395,7 +3395,7 @@
         <v>Passed</v>
       </c>
       <c r="K79">
-        <v>340</v>
+        <v>281</v>
       </c>
       <c r="L79" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3433,7 +3433,7 @@
         <v>Passed</v>
       </c>
       <c r="K80">
-        <v>224</v>
+        <v>282</v>
       </c>
       <c r="L80" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3471,7 +3471,7 @@
         <v>Passed</v>
       </c>
       <c r="K81">
-        <v>300</v>
+        <v>324</v>
       </c>
       <c r="L81" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3509,7 +3509,7 @@
         <v>Passed</v>
       </c>
       <c r="K82">
-        <v>292</v>
+        <v>196</v>
       </c>
       <c r="L82" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3547,7 +3547,7 @@
         <v>Passed</v>
       </c>
       <c r="K83">
-        <v>247</v>
+        <v>296</v>
       </c>
       <c r="L83" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3585,7 +3585,7 @@
         <v>Passed</v>
       </c>
       <c r="K84">
-        <v>177</v>
+        <v>279</v>
       </c>
       <c r="L84" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3623,7 +3623,7 @@
         <v>Passed</v>
       </c>
       <c r="K85">
-        <v>261</v>
+        <v>349</v>
       </c>
       <c r="L85" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3661,7 +3661,7 @@
         <v>Passed</v>
       </c>
       <c r="K86">
-        <v>274</v>
+        <v>167</v>
       </c>
       <c r="L86" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3699,7 +3699,7 @@
         <v>Passed</v>
       </c>
       <c r="K87">
-        <v>321</v>
+        <v>300</v>
       </c>
       <c r="L87" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3737,7 +3737,7 @@
         <v>Passed</v>
       </c>
       <c r="K88">
-        <v>179</v>
+        <v>317</v>
       </c>
       <c r="L88" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3775,7 +3775,7 @@
         <v>Passed</v>
       </c>
       <c r="K89">
-        <v>157</v>
+        <v>391</v>
       </c>
       <c r="L89" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3813,7 +3813,7 @@
         <v>Passed</v>
       </c>
       <c r="K90">
-        <v>253</v>
+        <v>219</v>
       </c>
       <c r="L90" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3851,7 +3851,7 @@
         <v>Passed</v>
       </c>
       <c r="K91">
-        <v>381</v>
+        <v>153</v>
       </c>
       <c r="L91" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3889,7 +3889,7 @@
         <v>Passed</v>
       </c>
       <c r="K92">
-        <v>326</v>
+        <v>161</v>
       </c>
       <c r="L92" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3927,7 +3927,7 @@
         <v>Passed</v>
       </c>
       <c r="K93">
-        <v>228</v>
+        <v>320</v>
       </c>
       <c r="L93" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3965,7 +3965,7 @@
         <v>Passed</v>
       </c>
       <c r="K94">
-        <v>336</v>
+        <v>185</v>
       </c>
       <c r="L94" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4003,7 +4003,7 @@
         <v>Passed</v>
       </c>
       <c r="K95">
-        <v>381</v>
+        <v>279</v>
       </c>
       <c r="L95" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4041,7 +4041,7 @@
         <v>Passed</v>
       </c>
       <c r="K96">
-        <v>232</v>
+        <v>289</v>
       </c>
       <c r="L96" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4079,7 +4079,7 @@
         <v>Passed</v>
       </c>
       <c r="K97">
-        <v>335</v>
+        <v>185</v>
       </c>
       <c r="L97" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4117,7 +4117,7 @@
         <v>Passed</v>
       </c>
       <c r="K98">
-        <v>193</v>
+        <v>377</v>
       </c>
       <c r="L98" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4155,7 +4155,7 @@
         <v>Passed</v>
       </c>
       <c r="K99">
-        <v>167</v>
+        <v>239</v>
       </c>
       <c r="L99" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4193,7 +4193,7 @@
         <v>Passed</v>
       </c>
       <c r="K100">
-        <v>348</v>
+        <v>368</v>
       </c>
       <c r="L100" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4231,7 +4231,7 @@
         <v>Passed</v>
       </c>
       <c r="K101">
-        <v>384</v>
+        <v>328</v>
       </c>
       <c r="L101" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4269,7 +4269,7 @@
         <v>Passed</v>
       </c>
       <c r="K102">
-        <v>151</v>
+        <v>379</v>
       </c>
       <c r="L102" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4307,7 +4307,7 @@
         <v>Passed</v>
       </c>
       <c r="K103">
-        <v>238</v>
+        <v>279</v>
       </c>
       <c r="L103" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4345,7 +4345,7 @@
         <v>Passed</v>
       </c>
       <c r="K104">
-        <v>222</v>
+        <v>377</v>
       </c>
       <c r="L104" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4383,7 +4383,7 @@
         <v>Passed</v>
       </c>
       <c r="K105">
-        <v>370</v>
+        <v>302</v>
       </c>
       <c r="L105" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4421,7 +4421,7 @@
         <v>Passed</v>
       </c>
       <c r="K106">
-        <v>393</v>
+        <v>349</v>
       </c>
       <c r="L106" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4459,7 +4459,7 @@
         <v>Passed</v>
       </c>
       <c r="K107">
-        <v>265</v>
+        <v>234</v>
       </c>
       <c r="L107" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4497,7 +4497,7 @@
         <v>Passed</v>
       </c>
       <c r="K108">
-        <v>192</v>
+        <v>162</v>
       </c>
       <c r="L108" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4535,7 +4535,7 @@
         <v>Passed</v>
       </c>
       <c r="K109">
-        <v>265</v>
+        <v>347</v>
       </c>
       <c r="L109" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4573,7 +4573,7 @@
         <v>Passed</v>
       </c>
       <c r="K110">
-        <v>364</v>
+        <v>152</v>
       </c>
       <c r="L110" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4611,7 +4611,7 @@
         <v>Passed</v>
       </c>
       <c r="K111">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="L111" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4649,7 +4649,7 @@
         <v>Passed</v>
       </c>
       <c r="K112">
-        <v>224</v>
+        <v>308</v>
       </c>
       <c r="L112" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4687,7 +4687,7 @@
         <v>Passed</v>
       </c>
       <c r="K113">
-        <v>153</v>
+        <v>205</v>
       </c>
       <c r="L113" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4725,7 +4725,7 @@
         <v>Passed</v>
       </c>
       <c r="K114">
-        <v>354</v>
+        <v>310</v>
       </c>
       <c r="L114" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4763,7 +4763,7 @@
         <v>Passed</v>
       </c>
       <c r="K115">
-        <v>295</v>
+        <v>241</v>
       </c>
       <c r="L115" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4801,7 +4801,7 @@
         <v>Passed</v>
       </c>
       <c r="K116">
-        <v>392</v>
+        <v>217</v>
       </c>
       <c r="L116" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4839,7 +4839,7 @@
         <v>Passed</v>
       </c>
       <c r="K117">
-        <v>370</v>
+        <v>156</v>
       </c>
       <c r="L117" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4877,7 +4877,7 @@
         <v>Passed</v>
       </c>
       <c r="K118">
-        <v>366</v>
+        <v>361</v>
       </c>
       <c r="L118" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4915,7 +4915,7 @@
         <v>Passed</v>
       </c>
       <c r="K119">
-        <v>270</v>
+        <v>277</v>
       </c>
       <c r="L119" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4953,7 +4953,7 @@
         <v>Passed</v>
       </c>
       <c r="K120">
-        <v>261</v>
+        <v>353</v>
       </c>
       <c r="L120" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4991,7 +4991,7 @@
         <v>Passed</v>
       </c>
       <c r="K121">
-        <v>257</v>
+        <v>276</v>
       </c>
       <c r="L121" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5029,7 +5029,7 @@
         <v>Passed</v>
       </c>
       <c r="K122">
-        <v>302</v>
+        <v>286</v>
       </c>
       <c r="L122" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5067,7 +5067,7 @@
         <v>Passed</v>
       </c>
       <c r="K123">
-        <v>248</v>
+        <v>353</v>
       </c>
       <c r="L123" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5105,7 +5105,7 @@
         <v>Passed</v>
       </c>
       <c r="K124">
-        <v>230</v>
+        <v>197</v>
       </c>
       <c r="L124" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5143,7 +5143,7 @@
         <v>Passed</v>
       </c>
       <c r="K125">
-        <v>345</v>
+        <v>169</v>
       </c>
       <c r="L125" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5181,7 +5181,7 @@
         <v>Passed</v>
       </c>
       <c r="K126">
-        <v>291</v>
+        <v>155</v>
       </c>
       <c r="L126" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5219,7 +5219,7 @@
         <v>Passed</v>
       </c>
       <c r="K127">
-        <v>315</v>
+        <v>324</v>
       </c>
       <c r="L127" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5257,7 +5257,7 @@
         <v>Passed</v>
       </c>
       <c r="K128">
-        <v>197</v>
+        <v>347</v>
       </c>
       <c r="L128" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5295,7 +5295,7 @@
         <v>Passed</v>
       </c>
       <c r="K129">
-        <v>200</v>
+        <v>398</v>
       </c>
       <c r="L129" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5333,7 +5333,7 @@
         <v>Passed</v>
       </c>
       <c r="K130">
-        <v>361</v>
+        <v>315</v>
       </c>
       <c r="L130" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5371,7 +5371,7 @@
         <v>Passed</v>
       </c>
       <c r="K131">
-        <v>375</v>
+        <v>176</v>
       </c>
       <c r="L131" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5409,7 +5409,7 @@
         <v>Passed</v>
       </c>
       <c r="K132">
-        <v>380</v>
+        <v>350</v>
       </c>
       <c r="L132" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5447,7 +5447,7 @@
         <v>Passed</v>
       </c>
       <c r="K133">
-        <v>327</v>
+        <v>257</v>
       </c>
       <c r="L133" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5485,7 +5485,7 @@
         <v>Passed</v>
       </c>
       <c r="K134">
-        <v>324</v>
+        <v>382</v>
       </c>
       <c r="L134" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5523,7 +5523,7 @@
         <v>Passed</v>
       </c>
       <c r="K135">
-        <v>170</v>
+        <v>377</v>
       </c>
       <c r="L135" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5561,7 +5561,7 @@
         <v>Passed</v>
       </c>
       <c r="K136">
-        <v>228</v>
+        <v>206</v>
       </c>
       <c r="L136" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5637,7 +5637,7 @@
         <v>Passed</v>
       </c>
       <c r="K138">
-        <v>337</v>
+        <v>243</v>
       </c>
       <c r="L138" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5675,7 +5675,7 @@
         <v>Passed</v>
       </c>
       <c r="K139">
-        <v>304</v>
+        <v>318</v>
       </c>
       <c r="L139" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5713,7 +5713,7 @@
         <v>Passed</v>
       </c>
       <c r="K140">
-        <v>374</v>
+        <v>302</v>
       </c>
       <c r="L140" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5751,7 +5751,7 @@
         <v>Passed</v>
       </c>
       <c r="K141">
-        <v>364</v>
+        <v>313</v>
       </c>
       <c r="L141" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5789,7 +5789,7 @@
         <v>Passed</v>
       </c>
       <c r="K142">
-        <v>277</v>
+        <v>342</v>
       </c>
       <c r="L142" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5827,7 +5827,7 @@
         <v>Passed</v>
       </c>
       <c r="K143">
-        <v>380</v>
+        <v>372</v>
       </c>
       <c r="L143" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5865,7 +5865,7 @@
         <v>Passed</v>
       </c>
       <c r="K144">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="L144" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5903,7 +5903,7 @@
         <v>Passed</v>
       </c>
       <c r="K145">
-        <v>158</v>
+        <v>173</v>
       </c>
       <c r="L145" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5941,7 +5941,7 @@
         <v>Passed</v>
       </c>
       <c r="K146">
-        <v>353</v>
+        <v>319</v>
       </c>
       <c r="L146" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5979,7 +5979,7 @@
         <v>Passed</v>
       </c>
       <c r="K147">
-        <v>292</v>
+        <v>238</v>
       </c>
       <c r="L147" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6017,7 +6017,7 @@
         <v>Passed</v>
       </c>
       <c r="K148">
-        <v>253</v>
+        <v>223</v>
       </c>
       <c r="L148" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6055,7 +6055,7 @@
         <v>Passed</v>
       </c>
       <c r="K149">
-        <v>275</v>
+        <v>291</v>
       </c>
       <c r="L149" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6093,7 +6093,7 @@
         <v>Passed</v>
       </c>
       <c r="K150">
-        <v>223</v>
+        <v>200</v>
       </c>
       <c r="L150" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6131,7 +6131,7 @@
         <v>Passed</v>
       </c>
       <c r="K151">
-        <v>346</v>
+        <v>203</v>
       </c>
       <c r="L151" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6169,7 +6169,7 @@
         <v>Passed</v>
       </c>
       <c r="K152">
-        <v>369</v>
+        <v>394</v>
       </c>
       <c r="L152" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6207,7 +6207,7 @@
         <v>Passed</v>
       </c>
       <c r="K153">
-        <v>246</v>
+        <v>238</v>
       </c>
       <c r="L153" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6245,7 +6245,7 @@
         <v>Passed</v>
       </c>
       <c r="K154">
-        <v>382</v>
+        <v>193</v>
       </c>
       <c r="L154" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6283,7 +6283,7 @@
         <v>Passed</v>
       </c>
       <c r="K155">
-        <v>388</v>
+        <v>268</v>
       </c>
       <c r="L155" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6321,7 +6321,7 @@
         <v>Passed</v>
       </c>
       <c r="K156">
-        <v>239</v>
+        <v>367</v>
       </c>
       <c r="L156" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6359,7 +6359,7 @@
         <v>Passed</v>
       </c>
       <c r="K157">
-        <v>200</v>
+        <v>275</v>
       </c>
       <c r="L157" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6397,7 +6397,7 @@
         <v>Passed</v>
       </c>
       <c r="K158">
-        <v>334</v>
+        <v>233</v>
       </c>
       <c r="L158" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6435,7 +6435,7 @@
         <v>Passed</v>
       </c>
       <c r="K159">
-        <v>244</v>
+        <v>329</v>
       </c>
       <c r="L159" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6473,7 +6473,7 @@
         <v>Passed</v>
       </c>
       <c r="K160">
-        <v>315</v>
+        <v>381</v>
       </c>
       <c r="L160" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6511,7 +6511,7 @@
         <v>Passed</v>
       </c>
       <c r="K161">
-        <v>323</v>
+        <v>317</v>
       </c>
       <c r="L161" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6549,7 +6549,7 @@
         <v>Passed</v>
       </c>
       <c r="K162">
-        <v>165</v>
+        <v>182</v>
       </c>
       <c r="L162" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6587,7 +6587,7 @@
         <v>Passed</v>
       </c>
       <c r="K163">
-        <v>262</v>
+        <v>291</v>
       </c>
       <c r="L163" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6625,7 +6625,7 @@
         <v>Passed</v>
       </c>
       <c r="K164">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="L164" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6663,7 +6663,7 @@
         <v>Passed</v>
       </c>
       <c r="K165">
-        <v>350</v>
+        <v>293</v>
       </c>
       <c r="L165" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6701,7 +6701,7 @@
         <v>Passed</v>
       </c>
       <c r="K166">
-        <v>325</v>
+        <v>216</v>
       </c>
       <c r="L166" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6739,7 +6739,7 @@
         <v>Passed</v>
       </c>
       <c r="K167">
-        <v>160</v>
+        <v>377</v>
       </c>
       <c r="L167" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6777,7 +6777,7 @@
         <v>Passed</v>
       </c>
       <c r="K168">
-        <v>188</v>
+        <v>212</v>
       </c>
       <c r="L168" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6815,7 +6815,7 @@
         <v>Passed</v>
       </c>
       <c r="K169">
-        <v>288</v>
+        <v>280</v>
       </c>
       <c r="L169" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6853,7 +6853,7 @@
         <v>Passed</v>
       </c>
       <c r="K170">
-        <v>193</v>
+        <v>314</v>
       </c>
       <c r="L170" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6891,7 +6891,7 @@
         <v>Passed</v>
       </c>
       <c r="K171">
-        <v>240</v>
+        <v>180</v>
       </c>
       <c r="L171" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6929,7 +6929,7 @@
         <v>Passed</v>
       </c>
       <c r="K172">
-        <v>347</v>
+        <v>204</v>
       </c>
       <c r="L172" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6967,7 +6967,7 @@
         <v>Passed</v>
       </c>
       <c r="K173">
-        <v>266</v>
+        <v>313</v>
       </c>
       <c r="L173" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7005,7 +7005,7 @@
         <v>Passed</v>
       </c>
       <c r="K174">
-        <v>281</v>
+        <v>171</v>
       </c>
       <c r="L174" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7043,7 +7043,7 @@
         <v>Passed</v>
       </c>
       <c r="K175">
-        <v>165</v>
+        <v>178</v>
       </c>
       <c r="L175" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7081,7 +7081,7 @@
         <v>Passed</v>
       </c>
       <c r="K176">
-        <v>253</v>
+        <v>320</v>
       </c>
       <c r="L176" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7119,7 +7119,7 @@
         <v>Passed</v>
       </c>
       <c r="K177">
-        <v>230</v>
+        <v>288</v>
       </c>
       <c r="L177" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7157,7 +7157,7 @@
         <v>Passed</v>
       </c>
       <c r="K178">
-        <v>288</v>
+        <v>315</v>
       </c>
       <c r="L178" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7195,7 +7195,7 @@
         <v>Passed</v>
       </c>
       <c r="K179">
-        <v>375</v>
+        <v>348</v>
       </c>
       <c r="L179" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7233,7 +7233,7 @@
         <v>Passed</v>
       </c>
       <c r="K180">
-        <v>152</v>
+        <v>310</v>
       </c>
       <c r="L180" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7271,7 +7271,7 @@
         <v>Passed</v>
       </c>
       <c r="K181">
-        <v>390</v>
+        <v>208</v>
       </c>
       <c r="L181" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7309,7 +7309,7 @@
         <v>Passed</v>
       </c>
       <c r="K182">
-        <v>385</v>
+        <v>160</v>
       </c>
       <c r="L182" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7347,7 +7347,7 @@
         <v>Passed</v>
       </c>
       <c r="K183">
-        <v>169</v>
+        <v>190</v>
       </c>
       <c r="L183" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7385,7 +7385,7 @@
         <v>Passed</v>
       </c>
       <c r="K184">
-        <v>171</v>
+        <v>227</v>
       </c>
       <c r="L184" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7423,7 +7423,7 @@
         <v>Passed</v>
       </c>
       <c r="K185">
-        <v>280</v>
+        <v>350</v>
       </c>
       <c r="L185" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7461,7 +7461,7 @@
         <v>Passed</v>
       </c>
       <c r="K186">
-        <v>172</v>
+        <v>315</v>
       </c>
       <c r="L186" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7499,7 +7499,7 @@
         <v>Passed</v>
       </c>
       <c r="K187">
-        <v>325</v>
+        <v>374</v>
       </c>
       <c r="L187" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7537,7 +7537,7 @@
         <v>Passed</v>
       </c>
       <c r="K188">
-        <v>191</v>
+        <v>364</v>
       </c>
       <c r="L188" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7575,7 +7575,7 @@
         <v>Passed</v>
       </c>
       <c r="K189">
-        <v>356</v>
+        <v>210</v>
       </c>
       <c r="L189" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7613,7 +7613,7 @@
         <v>Passed</v>
       </c>
       <c r="K190">
-        <v>309</v>
+        <v>354</v>
       </c>
       <c r="L190" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7651,7 +7651,7 @@
         <v>Passed</v>
       </c>
       <c r="K191">
-        <v>232</v>
+        <v>333</v>
       </c>
       <c r="L191" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7689,7 +7689,7 @@
         <v>Passed</v>
       </c>
       <c r="K192">
-        <v>205</v>
+        <v>302</v>
       </c>
       <c r="L192" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7727,7 +7727,7 @@
         <v>Passed</v>
       </c>
       <c r="K193">
-        <v>371</v>
+        <v>327</v>
       </c>
       <c r="L193" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7765,7 +7765,7 @@
         <v>Passed</v>
       </c>
       <c r="K194">
-        <v>302</v>
+        <v>253</v>
       </c>
       <c r="L194" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7803,7 +7803,7 @@
         <v>Passed</v>
       </c>
       <c r="K195">
-        <v>272</v>
+        <v>348</v>
       </c>
       <c r="L195" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7841,7 +7841,7 @@
         <v>Passed</v>
       </c>
       <c r="K196">
-        <v>357</v>
+        <v>225</v>
       </c>
       <c r="L196" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7879,7 +7879,7 @@
         <v>Passed</v>
       </c>
       <c r="K197">
-        <v>356</v>
+        <v>373</v>
       </c>
       <c r="L197" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7917,7 +7917,7 @@
         <v>Passed</v>
       </c>
       <c r="K198">
-        <v>318</v>
+        <v>391</v>
       </c>
       <c r="L198" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7955,7 +7955,7 @@
         <v>Passed</v>
       </c>
       <c r="K199">
-        <v>382</v>
+        <v>360</v>
       </c>
       <c r="L199" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7993,7 +7993,7 @@
         <v>Passed</v>
       </c>
       <c r="K200">
-        <v>268</v>
+        <v>360</v>
       </c>
       <c r="L200" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8031,7 +8031,7 @@
         <v>Passed</v>
       </c>
       <c r="K201">
-        <v>311</v>
+        <v>332</v>
       </c>
       <c r="L201" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8069,7 +8069,7 @@
         <v>Passed</v>
       </c>
       <c r="K202">
-        <v>381</v>
+        <v>157</v>
       </c>
       <c r="L202" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8107,7 +8107,7 @@
         <v>Passed</v>
       </c>
       <c r="K203">
-        <v>239</v>
+        <v>163</v>
       </c>
       <c r="L203" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8145,7 +8145,7 @@
         <v>Passed</v>
       </c>
       <c r="K204">
-        <v>213</v>
+        <v>231</v>
       </c>
       <c r="L204" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8183,7 +8183,7 @@
         <v>Passed</v>
       </c>
       <c r="K205">
-        <v>241</v>
+        <v>310</v>
       </c>
       <c r="L205" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8221,7 +8221,7 @@
         <v>Passed</v>
       </c>
       <c r="K206">
-        <v>359</v>
+        <v>246</v>
       </c>
       <c r="L206" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8259,7 +8259,7 @@
         <v>Passed</v>
       </c>
       <c r="K207">
-        <v>299</v>
+        <v>362</v>
       </c>
       <c r="L207" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8297,7 +8297,7 @@
         <v>Passed</v>
       </c>
       <c r="K208">
-        <v>373</v>
+        <v>255</v>
       </c>
       <c r="L208" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8335,7 +8335,7 @@
         <v>Passed</v>
       </c>
       <c r="K209">
-        <v>387</v>
+        <v>283</v>
       </c>
       <c r="L209" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8373,7 +8373,7 @@
         <v>Passed</v>
       </c>
       <c r="K210">
-        <v>297</v>
+        <v>257</v>
       </c>
       <c r="L210" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8411,7 +8411,7 @@
         <v>Passed</v>
       </c>
       <c r="K211">
-        <v>241</v>
+        <v>198</v>
       </c>
       <c r="L211" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8449,7 +8449,7 @@
         <v>Passed</v>
       </c>
       <c r="K212">
-        <v>255</v>
+        <v>193</v>
       </c>
       <c r="L212" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8487,7 +8487,7 @@
         <v>Passed</v>
       </c>
       <c r="K213">
-        <v>254</v>
+        <v>204</v>
       </c>
       <c r="L213" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8525,7 +8525,7 @@
         <v>Passed</v>
       </c>
       <c r="K214">
-        <v>366</v>
+        <v>170</v>
       </c>
       <c r="L214" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8563,7 +8563,7 @@
         <v>Passed</v>
       </c>
       <c r="K215">
-        <v>369</v>
+        <v>172</v>
       </c>
       <c r="L215" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8601,7 +8601,7 @@
         <v>Passed</v>
       </c>
       <c r="K216">
-        <v>252</v>
+        <v>167</v>
       </c>
       <c r="L216" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8639,7 +8639,7 @@
         <v>Passed</v>
       </c>
       <c r="K217">
-        <v>256</v>
+        <v>345</v>
       </c>
       <c r="L217" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8677,7 +8677,7 @@
         <v>Passed</v>
       </c>
       <c r="K218">
-        <v>252</v>
+        <v>236</v>
       </c>
       <c r="L218" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8715,7 +8715,7 @@
         <v>Passed</v>
       </c>
       <c r="K219">
-        <v>374</v>
+        <v>378</v>
       </c>
       <c r="L219" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8753,7 +8753,7 @@
         <v>Passed</v>
       </c>
       <c r="K220">
-        <v>167</v>
+        <v>346</v>
       </c>
       <c r="L220" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8791,7 +8791,7 @@
         <v>Passed</v>
       </c>
       <c r="K221">
-        <v>361</v>
+        <v>395</v>
       </c>
       <c r="L221" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8829,7 +8829,7 @@
         <v>Passed</v>
       </c>
       <c r="K222">
-        <v>188</v>
+        <v>278</v>
       </c>
       <c r="L222" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8867,7 +8867,7 @@
         <v>Passed</v>
       </c>
       <c r="K223">
-        <v>345</v>
+        <v>172</v>
       </c>
       <c r="L223" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8905,7 +8905,7 @@
         <v>Passed</v>
       </c>
       <c r="K224">
-        <v>368</v>
+        <v>209</v>
       </c>
       <c r="L224" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8943,7 +8943,7 @@
         <v>Passed</v>
       </c>
       <c r="K225">
-        <v>274</v>
+        <v>345</v>
       </c>
       <c r="L225" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8981,7 +8981,7 @@
         <v>Passed</v>
       </c>
       <c r="K226">
-        <v>298</v>
+        <v>279</v>
       </c>
       <c r="L226" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9019,7 +9019,7 @@
         <v>Passed</v>
       </c>
       <c r="K227">
-        <v>178</v>
+        <v>334</v>
       </c>
       <c r="L227" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9057,7 +9057,7 @@
         <v>Passed</v>
       </c>
       <c r="K228">
-        <v>361</v>
+        <v>289</v>
       </c>
       <c r="L228" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9095,7 +9095,7 @@
         <v>Passed</v>
       </c>
       <c r="K229">
-        <v>247</v>
+        <v>224</v>
       </c>
       <c r="L229" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9171,7 +9171,7 @@
         <v>Passed</v>
       </c>
       <c r="K231">
-        <v>216</v>
+        <v>248</v>
       </c>
       <c r="L231" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9209,7 +9209,7 @@
         <v>Passed</v>
       </c>
       <c r="K232">
-        <v>208</v>
+        <v>215</v>
       </c>
       <c r="L232" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9247,7 +9247,7 @@
         <v>Passed</v>
       </c>
       <c r="K233">
-        <v>253</v>
+        <v>157</v>
       </c>
       <c r="L233" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9285,7 +9285,7 @@
         <v>Passed</v>
       </c>
       <c r="K234">
-        <v>216</v>
+        <v>360</v>
       </c>
       <c r="L234" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9323,7 +9323,7 @@
         <v>Passed</v>
       </c>
       <c r="K235">
-        <v>348</v>
+        <v>225</v>
       </c>
       <c r="L235" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9361,7 +9361,7 @@
         <v>Passed</v>
       </c>
       <c r="K236">
-        <v>165</v>
+        <v>202</v>
       </c>
       <c r="L236" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9399,7 +9399,7 @@
         <v>Passed</v>
       </c>
       <c r="K237">
-        <v>276</v>
+        <v>382</v>
       </c>
       <c r="L237" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9437,7 +9437,7 @@
         <v>Passed</v>
       </c>
       <c r="K238">
-        <v>209</v>
+        <v>165</v>
       </c>
       <c r="L238" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9475,7 +9475,7 @@
         <v>Passed</v>
       </c>
       <c r="K239">
-        <v>277</v>
+        <v>286</v>
       </c>
       <c r="L239" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9513,7 +9513,7 @@
         <v>Passed</v>
       </c>
       <c r="K240">
-        <v>348</v>
+        <v>366</v>
       </c>
       <c r="L240" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9551,7 +9551,7 @@
         <v>Passed</v>
       </c>
       <c r="K241">
-        <v>165</v>
+        <v>154</v>
       </c>
       <c r="L241" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9589,7 +9589,7 @@
         <v>Passed</v>
       </c>
       <c r="K242">
-        <v>333</v>
+        <v>235</v>
       </c>
       <c r="L242" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9627,7 +9627,7 @@
         <v>Passed</v>
       </c>
       <c r="K243">
-        <v>349</v>
+        <v>234</v>
       </c>
       <c r="L243" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9665,7 +9665,7 @@
         <v>Passed</v>
       </c>
       <c r="K244">
-        <v>399</v>
+        <v>327</v>
       </c>
       <c r="L244" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9703,7 +9703,7 @@
         <v>Passed</v>
       </c>
       <c r="K245">
-        <v>338</v>
+        <v>284</v>
       </c>
       <c r="L245" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9741,7 +9741,7 @@
         <v>Passed</v>
       </c>
       <c r="K246">
-        <v>313</v>
+        <v>207</v>
       </c>
       <c r="L246" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9779,7 +9779,7 @@
         <v>Passed</v>
       </c>
       <c r="K247">
-        <v>313</v>
+        <v>378</v>
       </c>
       <c r="L247" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9817,7 +9817,7 @@
         <v>Passed</v>
       </c>
       <c r="K248">
-        <v>268</v>
+        <v>385</v>
       </c>
       <c r="L248" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9855,7 +9855,7 @@
         <v>Passed</v>
       </c>
       <c r="K249">
-        <v>299</v>
+        <v>152</v>
       </c>
       <c r="L249" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9893,7 +9893,7 @@
         <v>Passed</v>
       </c>
       <c r="K250">
-        <v>150</v>
+        <v>393</v>
       </c>
       <c r="L250" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9931,7 +9931,7 @@
         <v>Passed</v>
       </c>
       <c r="K251">
-        <v>220</v>
+        <v>370</v>
       </c>
       <c r="L251" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9969,7 +9969,7 @@
         <v>Passed</v>
       </c>
       <c r="K252">
-        <v>389</v>
+        <v>186</v>
       </c>
       <c r="L252" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10007,7 +10007,7 @@
         <v>Passed</v>
       </c>
       <c r="K253">
-        <v>359</v>
+        <v>314</v>
       </c>
       <c r="L253" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10045,7 +10045,7 @@
         <v>Passed</v>
       </c>
       <c r="K254">
-        <v>304</v>
+        <v>311</v>
       </c>
       <c r="L254" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10083,7 +10083,7 @@
         <v>Passed</v>
       </c>
       <c r="K255">
-        <v>192</v>
+        <v>257</v>
       </c>
       <c r="L255" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10121,7 +10121,7 @@
         <v>Passed</v>
       </c>
       <c r="K256">
-        <v>271</v>
+        <v>392</v>
       </c>
       <c r="L256" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10159,7 +10159,7 @@
         <v>Passed</v>
       </c>
       <c r="K257">
-        <v>264</v>
+        <v>250</v>
       </c>
       <c r="L257" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10197,7 +10197,7 @@
         <v>Passed</v>
       </c>
       <c r="K258">
-        <v>185</v>
+        <v>205</v>
       </c>
       <c r="L258" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10235,7 +10235,7 @@
         <v>Passed</v>
       </c>
       <c r="K259">
-        <v>365</v>
+        <v>207</v>
       </c>
       <c r="L259" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10273,7 +10273,7 @@
         <v>Passed</v>
       </c>
       <c r="K260">
-        <v>323</v>
+        <v>391</v>
       </c>
       <c r="L260" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10311,7 +10311,7 @@
         <v>Passed</v>
       </c>
       <c r="K261">
-        <v>212</v>
+        <v>244</v>
       </c>
       <c r="L261" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10349,7 +10349,7 @@
         <v>Passed</v>
       </c>
       <c r="K262">
-        <v>348</v>
+        <v>338</v>
       </c>
       <c r="L262" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10387,7 +10387,7 @@
         <v>Passed</v>
       </c>
       <c r="K263">
-        <v>221</v>
+        <v>269</v>
       </c>
       <c r="L263" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10425,7 +10425,7 @@
         <v>Passed</v>
       </c>
       <c r="K264">
-        <v>256</v>
+        <v>340</v>
       </c>
       <c r="L264" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10463,7 +10463,7 @@
         <v>Passed</v>
       </c>
       <c r="K265">
-        <v>243</v>
+        <v>338</v>
       </c>
       <c r="L265" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10501,7 +10501,7 @@
         <v>Passed</v>
       </c>
       <c r="K266">
-        <v>256</v>
+        <v>395</v>
       </c>
       <c r="L266" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10539,7 +10539,7 @@
         <v>Passed</v>
       </c>
       <c r="K267">
-        <v>329</v>
+        <v>317</v>
       </c>
       <c r="L267" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10577,7 +10577,7 @@
         <v>Passed</v>
       </c>
       <c r="K268">
-        <v>369</v>
+        <v>378</v>
       </c>
       <c r="L268" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10615,7 +10615,7 @@
         <v>Passed</v>
       </c>
       <c r="K269">
-        <v>312</v>
+        <v>252</v>
       </c>
       <c r="L269" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10653,7 +10653,7 @@
         <v>Passed</v>
       </c>
       <c r="K270">
-        <v>348</v>
+        <v>250</v>
       </c>
       <c r="L270" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10691,7 +10691,7 @@
         <v>Passed</v>
       </c>
       <c r="K271">
-        <v>301</v>
+        <v>194</v>
       </c>
       <c r="L271" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10729,7 +10729,7 @@
         <v>Passed</v>
       </c>
       <c r="K272">
-        <v>158</v>
+        <v>306</v>
       </c>
       <c r="L272" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10767,7 +10767,7 @@
         <v>Passed</v>
       </c>
       <c r="K273">
-        <v>274</v>
+        <v>252</v>
       </c>
       <c r="L273" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10805,7 +10805,7 @@
         <v>Passed</v>
       </c>
       <c r="K274">
-        <v>275</v>
+        <v>212</v>
       </c>
       <c r="L274" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10843,7 +10843,7 @@
         <v>Passed</v>
       </c>
       <c r="K275">
-        <v>192</v>
+        <v>390</v>
       </c>
       <c r="L275" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10881,7 +10881,7 @@
         <v>Passed</v>
       </c>
       <c r="K276">
-        <v>214</v>
+        <v>169</v>
       </c>
       <c r="L276" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10919,7 +10919,7 @@
         <v>Passed</v>
       </c>
       <c r="K277">
-        <v>168</v>
+        <v>309</v>
       </c>
       <c r="L277" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10957,7 +10957,7 @@
         <v>Passed</v>
       </c>
       <c r="K278">
-        <v>328</v>
+        <v>227</v>
       </c>
       <c r="L278" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10995,7 +10995,7 @@
         <v>Passed</v>
       </c>
       <c r="K279">
-        <v>192</v>
+        <v>392</v>
       </c>
       <c r="L279" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11033,7 +11033,7 @@
         <v>Passed</v>
       </c>
       <c r="K280">
-        <v>288</v>
+        <v>392</v>
       </c>
       <c r="L280" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11071,7 +11071,7 @@
         <v>Passed</v>
       </c>
       <c r="K281">
-        <v>396</v>
+        <v>275</v>
       </c>
       <c r="L281" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11109,7 +11109,7 @@
         <v>Passed</v>
       </c>
       <c r="K282">
-        <v>255</v>
+        <v>154</v>
       </c>
       <c r="L282" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11147,7 +11147,7 @@
         <v>Passed</v>
       </c>
       <c r="K283">
-        <v>164</v>
+        <v>151</v>
       </c>
       <c r="L283" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11185,7 +11185,7 @@
         <v>Passed</v>
       </c>
       <c r="K284">
-        <v>384</v>
+        <v>278</v>
       </c>
       <c r="L284" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11223,7 +11223,7 @@
         <v>Passed</v>
       </c>
       <c r="K285">
-        <v>349</v>
+        <v>356</v>
       </c>
       <c r="L285" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11261,7 +11261,7 @@
         <v>Passed</v>
       </c>
       <c r="K286">
-        <v>157</v>
+        <v>321</v>
       </c>
       <c r="L286" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11299,7 +11299,7 @@
         <v>Passed</v>
       </c>
       <c r="K287">
-        <v>272</v>
+        <v>386</v>
       </c>
       <c r="L287" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11337,7 +11337,7 @@
         <v>Passed</v>
       </c>
       <c r="K288">
-        <v>341</v>
+        <v>386</v>
       </c>
       <c r="L288" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11375,7 +11375,7 @@
         <v>Passed</v>
       </c>
       <c r="K289">
-        <v>165</v>
+        <v>271</v>
       </c>
       <c r="L289" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11413,7 +11413,7 @@
         <v>Passed</v>
       </c>
       <c r="K290">
-        <v>159</v>
+        <v>268</v>
       </c>
       <c r="L290" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11451,7 +11451,7 @@
         <v>Passed</v>
       </c>
       <c r="K291">
-        <v>168</v>
+        <v>273</v>
       </c>
       <c r="L291" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11489,7 +11489,7 @@
         <v>Passed</v>
       </c>
       <c r="K292">
-        <v>270</v>
+        <v>206</v>
       </c>
       <c r="L292" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11527,7 +11527,7 @@
         <v>Passed</v>
       </c>
       <c r="K293">
-        <v>286</v>
+        <v>178</v>
       </c>
       <c r="L293" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11565,7 +11565,7 @@
         <v>Passed</v>
       </c>
       <c r="K294">
-        <v>239</v>
+        <v>155</v>
       </c>
       <c r="L294" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11603,7 +11603,7 @@
         <v>Passed</v>
       </c>
       <c r="K295">
-        <v>201</v>
+        <v>350</v>
       </c>
       <c r="L295" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11641,7 +11641,7 @@
         <v>Passed</v>
       </c>
       <c r="K296">
-        <v>176</v>
+        <v>326</v>
       </c>
       <c r="L296" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11679,7 +11679,7 @@
         <v>Passed</v>
       </c>
       <c r="K297">
-        <v>267</v>
+        <v>397</v>
       </c>
       <c r="L297" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11717,7 +11717,7 @@
         <v>Passed</v>
       </c>
       <c r="K298">
-        <v>344</v>
+        <v>246</v>
       </c>
       <c r="L298" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11755,7 +11755,7 @@
         <v>Passed</v>
       </c>
       <c r="K299">
-        <v>274</v>
+        <v>210</v>
       </c>
       <c r="L299" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11793,7 +11793,7 @@
         <v>Passed</v>
       </c>
       <c r="K300">
-        <v>366</v>
+        <v>253</v>
       </c>
       <c r="L300" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11831,7 +11831,7 @@
         <v>Passed</v>
       </c>
       <c r="K301">
-        <v>237</v>
+        <v>189</v>
       </c>
       <c r="L301" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>

</xml_diff>

<commit_message>
feat: add 3 rows of VIP seat images to the 3D VIP pass page wallet
</commit_message>
<xml_diff>
--- a/EventSphere_Appium_Mobile_300_Report.xlsx
+++ b/EventSphere_Appium_Mobile_300_Report.xlsx
@@ -469,7 +469,7 @@
         <v>Passed</v>
       </c>
       <c r="K2">
-        <v>310</v>
+        <v>396</v>
       </c>
       <c r="L2" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -507,7 +507,7 @@
         <v>Passed</v>
       </c>
       <c r="K3">
-        <v>370</v>
+        <v>274</v>
       </c>
       <c r="L3" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -545,7 +545,7 @@
         <v>Passed</v>
       </c>
       <c r="K4">
-        <v>278</v>
+        <v>245</v>
       </c>
       <c r="L4" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -583,7 +583,7 @@
         <v>Passed</v>
       </c>
       <c r="K5">
-        <v>330</v>
+        <v>229</v>
       </c>
       <c r="L5" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -621,7 +621,7 @@
         <v>Passed</v>
       </c>
       <c r="K6">
-        <v>335</v>
+        <v>295</v>
       </c>
       <c r="L6" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -659,7 +659,7 @@
         <v>Passed</v>
       </c>
       <c r="K7">
-        <v>225</v>
+        <v>380</v>
       </c>
       <c r="L7" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -697,7 +697,7 @@
         <v>Passed</v>
       </c>
       <c r="K8">
-        <v>153</v>
+        <v>208</v>
       </c>
       <c r="L8" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -735,7 +735,7 @@
         <v>Passed</v>
       </c>
       <c r="K9">
-        <v>352</v>
+        <v>315</v>
       </c>
       <c r="L9" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -773,7 +773,7 @@
         <v>Passed</v>
       </c>
       <c r="K10">
-        <v>161</v>
+        <v>338</v>
       </c>
       <c r="L10" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -811,7 +811,7 @@
         <v>Passed</v>
       </c>
       <c r="K11">
-        <v>313</v>
+        <v>388</v>
       </c>
       <c r="L11" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -849,7 +849,7 @@
         <v>Passed</v>
       </c>
       <c r="K12">
-        <v>309</v>
+        <v>340</v>
       </c>
       <c r="L12" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -887,7 +887,7 @@
         <v>Passed</v>
       </c>
       <c r="K13">
-        <v>211</v>
+        <v>282</v>
       </c>
       <c r="L13" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -925,7 +925,7 @@
         <v>Passed</v>
       </c>
       <c r="K14">
-        <v>319</v>
+        <v>240</v>
       </c>
       <c r="L14" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -963,7 +963,7 @@
         <v>Passed</v>
       </c>
       <c r="K15">
-        <v>391</v>
+        <v>326</v>
       </c>
       <c r="L15" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1001,7 +1001,7 @@
         <v>Passed</v>
       </c>
       <c r="K16">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="L16" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1039,7 +1039,7 @@
         <v>Passed</v>
       </c>
       <c r="K17">
-        <v>397</v>
+        <v>300</v>
       </c>
       <c r="L17" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1077,7 +1077,7 @@
         <v>Passed</v>
       </c>
       <c r="K18">
-        <v>179</v>
+        <v>392</v>
       </c>
       <c r="L18" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1115,7 +1115,7 @@
         <v>Passed</v>
       </c>
       <c r="K19">
-        <v>352</v>
+        <v>229</v>
       </c>
       <c r="L19" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1153,7 +1153,7 @@
         <v>Passed</v>
       </c>
       <c r="K20">
-        <v>392</v>
+        <v>167</v>
       </c>
       <c r="L20" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1191,7 +1191,7 @@
         <v>Passed</v>
       </c>
       <c r="K21">
-        <v>278</v>
+        <v>230</v>
       </c>
       <c r="L21" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1229,7 +1229,7 @@
         <v>Passed</v>
       </c>
       <c r="K22">
-        <v>369</v>
+        <v>301</v>
       </c>
       <c r="L22" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1267,7 +1267,7 @@
         <v>Passed</v>
       </c>
       <c r="K23">
-        <v>197</v>
+        <v>216</v>
       </c>
       <c r="L23" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1305,7 +1305,7 @@
         <v>Passed</v>
       </c>
       <c r="K24">
-        <v>384</v>
+        <v>374</v>
       </c>
       <c r="L24" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1343,7 +1343,7 @@
         <v>Passed</v>
       </c>
       <c r="K25">
-        <v>289</v>
+        <v>163</v>
       </c>
       <c r="L25" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1381,7 +1381,7 @@
         <v>Passed</v>
       </c>
       <c r="K26">
-        <v>280</v>
+        <v>211</v>
       </c>
       <c r="L26" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1419,7 +1419,7 @@
         <v>Passed</v>
       </c>
       <c r="K27">
-        <v>272</v>
+        <v>384</v>
       </c>
       <c r="L27" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1457,7 +1457,7 @@
         <v>Passed</v>
       </c>
       <c r="K28">
-        <v>303</v>
+        <v>357</v>
       </c>
       <c r="L28" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1495,7 +1495,7 @@
         <v>Passed</v>
       </c>
       <c r="K29">
-        <v>202</v>
+        <v>287</v>
       </c>
       <c r="L29" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1533,7 +1533,7 @@
         <v>Passed</v>
       </c>
       <c r="K30">
-        <v>217</v>
+        <v>313</v>
       </c>
       <c r="L30" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1571,7 +1571,7 @@
         <v>Passed</v>
       </c>
       <c r="K31">
-        <v>153</v>
+        <v>380</v>
       </c>
       <c r="L31" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1609,7 +1609,7 @@
         <v>Passed</v>
       </c>
       <c r="K32">
-        <v>292</v>
+        <v>390</v>
       </c>
       <c r="L32" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1647,7 +1647,7 @@
         <v>Passed</v>
       </c>
       <c r="K33">
-        <v>337</v>
+        <v>316</v>
       </c>
       <c r="L33" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1685,7 +1685,7 @@
         <v>Passed</v>
       </c>
       <c r="K34">
-        <v>227</v>
+        <v>392</v>
       </c>
       <c r="L34" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1723,7 +1723,7 @@
         <v>Passed</v>
       </c>
       <c r="K35">
-        <v>323</v>
+        <v>262</v>
       </c>
       <c r="L35" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1761,7 +1761,7 @@
         <v>Passed</v>
       </c>
       <c r="K36">
-        <v>300</v>
+        <v>199</v>
       </c>
       <c r="L36" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1799,7 +1799,7 @@
         <v>Passed</v>
       </c>
       <c r="K37">
-        <v>200</v>
+        <v>245</v>
       </c>
       <c r="L37" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1837,7 +1837,7 @@
         <v>Passed</v>
       </c>
       <c r="K38">
-        <v>210</v>
+        <v>163</v>
       </c>
       <c r="L38" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1875,7 +1875,7 @@
         <v>Passed</v>
       </c>
       <c r="K39">
-        <v>257</v>
+        <v>379</v>
       </c>
       <c r="L39" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1913,7 +1913,7 @@
         <v>Passed</v>
       </c>
       <c r="K40">
-        <v>217</v>
+        <v>238</v>
       </c>
       <c r="L40" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1951,7 +1951,7 @@
         <v>Passed</v>
       </c>
       <c r="K41">
-        <v>248</v>
+        <v>224</v>
       </c>
       <c r="L41" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1989,7 +1989,7 @@
         <v>Passed</v>
       </c>
       <c r="K42">
-        <v>379</v>
+        <v>387</v>
       </c>
       <c r="L42" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2027,7 +2027,7 @@
         <v>Passed</v>
       </c>
       <c r="K43">
-        <v>350</v>
+        <v>159</v>
       </c>
       <c r="L43" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2065,7 +2065,7 @@
         <v>Passed</v>
       </c>
       <c r="K44">
-        <v>227</v>
+        <v>320</v>
       </c>
       <c r="L44" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2103,7 +2103,7 @@
         <v>Passed</v>
       </c>
       <c r="K45">
-        <v>201</v>
+        <v>340</v>
       </c>
       <c r="L45" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2141,7 +2141,7 @@
         <v>Passed</v>
       </c>
       <c r="K46">
-        <v>172</v>
+        <v>313</v>
       </c>
       <c r="L46" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2179,7 +2179,7 @@
         <v>Passed</v>
       </c>
       <c r="K47">
-        <v>161</v>
+        <v>376</v>
       </c>
       <c r="L47" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2217,7 +2217,7 @@
         <v>Passed</v>
       </c>
       <c r="K48">
-        <v>298</v>
+        <v>377</v>
       </c>
       <c r="L48" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2255,7 +2255,7 @@
         <v>Passed</v>
       </c>
       <c r="K49">
-        <v>228</v>
+        <v>184</v>
       </c>
       <c r="L49" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2293,7 +2293,7 @@
         <v>Passed</v>
       </c>
       <c r="K50">
-        <v>181</v>
+        <v>220</v>
       </c>
       <c r="L50" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2331,7 +2331,7 @@
         <v>Passed</v>
       </c>
       <c r="K51">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="L51" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2369,7 +2369,7 @@
         <v>Passed</v>
       </c>
       <c r="K52">
-        <v>193</v>
+        <v>162</v>
       </c>
       <c r="L52" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2407,7 +2407,7 @@
         <v>Passed</v>
       </c>
       <c r="K53">
-        <v>202</v>
+        <v>239</v>
       </c>
       <c r="L53" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2445,7 +2445,7 @@
         <v>Passed</v>
       </c>
       <c r="K54">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="L54" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2483,7 +2483,7 @@
         <v>Passed</v>
       </c>
       <c r="K55">
-        <v>355</v>
+        <v>240</v>
       </c>
       <c r="L55" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2521,7 +2521,7 @@
         <v>Passed</v>
       </c>
       <c r="K56">
-        <v>205</v>
+        <v>196</v>
       </c>
       <c r="L56" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2559,7 +2559,7 @@
         <v>Passed</v>
       </c>
       <c r="K57">
-        <v>346</v>
+        <v>248</v>
       </c>
       <c r="L57" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2597,7 +2597,7 @@
         <v>Passed</v>
       </c>
       <c r="K58">
-        <v>338</v>
+        <v>374</v>
       </c>
       <c r="L58" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2635,7 +2635,7 @@
         <v>Passed</v>
       </c>
       <c r="K59">
-        <v>152</v>
+        <v>176</v>
       </c>
       <c r="L59" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2673,7 +2673,7 @@
         <v>Passed</v>
       </c>
       <c r="K60">
-        <v>301</v>
+        <v>346</v>
       </c>
       <c r="L60" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2711,7 +2711,7 @@
         <v>Passed</v>
       </c>
       <c r="K61">
-        <v>178</v>
+        <v>257</v>
       </c>
       <c r="L61" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2749,7 +2749,7 @@
         <v>Passed</v>
       </c>
       <c r="K62">
-        <v>235</v>
+        <v>393</v>
       </c>
       <c r="L62" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2787,7 +2787,7 @@
         <v>Passed</v>
       </c>
       <c r="K63">
-        <v>162</v>
+        <v>300</v>
       </c>
       <c r="L63" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2825,7 +2825,7 @@
         <v>Passed</v>
       </c>
       <c r="K64">
-        <v>359</v>
+        <v>172</v>
       </c>
       <c r="L64" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2863,7 +2863,7 @@
         <v>Passed</v>
       </c>
       <c r="K65">
-        <v>312</v>
+        <v>290</v>
       </c>
       <c r="L65" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2901,7 +2901,7 @@
         <v>Passed</v>
       </c>
       <c r="K66">
-        <v>257</v>
+        <v>383</v>
       </c>
       <c r="L66" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2939,7 +2939,7 @@
         <v>Passed</v>
       </c>
       <c r="K67">
-        <v>176</v>
+        <v>223</v>
       </c>
       <c r="L67" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2977,7 +2977,7 @@
         <v>Passed</v>
       </c>
       <c r="K68">
-        <v>280</v>
+        <v>220</v>
       </c>
       <c r="L68" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3015,7 +3015,7 @@
         <v>Passed</v>
       </c>
       <c r="K69">
-        <v>191</v>
+        <v>384</v>
       </c>
       <c r="L69" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3053,7 +3053,7 @@
         <v>Passed</v>
       </c>
       <c r="K70">
-        <v>193</v>
+        <v>349</v>
       </c>
       <c r="L70" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3091,7 +3091,7 @@
         <v>Passed</v>
       </c>
       <c r="K71">
-        <v>320</v>
+        <v>312</v>
       </c>
       <c r="L71" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3129,7 +3129,7 @@
         <v>Passed</v>
       </c>
       <c r="K72">
-        <v>334</v>
+        <v>338</v>
       </c>
       <c r="L72" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3167,7 +3167,7 @@
         <v>Passed</v>
       </c>
       <c r="K73">
-        <v>196</v>
+        <v>231</v>
       </c>
       <c r="L73" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3205,7 +3205,7 @@
         <v>Passed</v>
       </c>
       <c r="K74">
-        <v>225</v>
+        <v>192</v>
       </c>
       <c r="L74" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3243,7 +3243,7 @@
         <v>Passed</v>
       </c>
       <c r="K75">
-        <v>259</v>
+        <v>351</v>
       </c>
       <c r="L75" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3281,7 +3281,7 @@
         <v>Passed</v>
       </c>
       <c r="K76">
-        <v>223</v>
+        <v>268</v>
       </c>
       <c r="L76" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3319,7 +3319,7 @@
         <v>Passed</v>
       </c>
       <c r="K77">
-        <v>228</v>
+        <v>183</v>
       </c>
       <c r="L77" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3357,7 +3357,7 @@
         <v>Passed</v>
       </c>
       <c r="K78">
-        <v>223</v>
+        <v>304</v>
       </c>
       <c r="L78" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3395,7 +3395,7 @@
         <v>Passed</v>
       </c>
       <c r="K79">
-        <v>281</v>
+        <v>218</v>
       </c>
       <c r="L79" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3433,7 +3433,7 @@
         <v>Passed</v>
       </c>
       <c r="K80">
-        <v>282</v>
+        <v>227</v>
       </c>
       <c r="L80" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3471,7 +3471,7 @@
         <v>Passed</v>
       </c>
       <c r="K81">
-        <v>324</v>
+        <v>242</v>
       </c>
       <c r="L81" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3509,7 +3509,7 @@
         <v>Passed</v>
       </c>
       <c r="K82">
-        <v>196</v>
+        <v>295</v>
       </c>
       <c r="L82" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3547,7 +3547,7 @@
         <v>Passed</v>
       </c>
       <c r="K83">
-        <v>296</v>
+        <v>207</v>
       </c>
       <c r="L83" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3585,7 +3585,7 @@
         <v>Passed</v>
       </c>
       <c r="K84">
-        <v>279</v>
+        <v>249</v>
       </c>
       <c r="L84" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3623,7 +3623,7 @@
         <v>Passed</v>
       </c>
       <c r="K85">
-        <v>349</v>
+        <v>282</v>
       </c>
       <c r="L85" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3661,7 +3661,7 @@
         <v>Passed</v>
       </c>
       <c r="K86">
-        <v>167</v>
+        <v>202</v>
       </c>
       <c r="L86" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3699,7 +3699,7 @@
         <v>Passed</v>
       </c>
       <c r="K87">
-        <v>300</v>
+        <v>277</v>
       </c>
       <c r="L87" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3737,7 +3737,7 @@
         <v>Passed</v>
       </c>
       <c r="K88">
-        <v>317</v>
+        <v>333</v>
       </c>
       <c r="L88" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3775,7 +3775,7 @@
         <v>Passed</v>
       </c>
       <c r="K89">
-        <v>391</v>
+        <v>317</v>
       </c>
       <c r="L89" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3813,7 +3813,7 @@
         <v>Passed</v>
       </c>
       <c r="K90">
-        <v>219</v>
+        <v>334</v>
       </c>
       <c r="L90" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3851,7 +3851,7 @@
         <v>Passed</v>
       </c>
       <c r="K91">
-        <v>153</v>
+        <v>281</v>
       </c>
       <c r="L91" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3889,7 +3889,7 @@
         <v>Passed</v>
       </c>
       <c r="K92">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="L92" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3927,7 +3927,7 @@
         <v>Passed</v>
       </c>
       <c r="K93">
-        <v>320</v>
+        <v>330</v>
       </c>
       <c r="L93" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3965,7 +3965,7 @@
         <v>Passed</v>
       </c>
       <c r="K94">
-        <v>185</v>
+        <v>349</v>
       </c>
       <c r="L94" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4003,7 +4003,7 @@
         <v>Passed</v>
       </c>
       <c r="K95">
-        <v>279</v>
+        <v>371</v>
       </c>
       <c r="L95" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4041,7 +4041,7 @@
         <v>Passed</v>
       </c>
       <c r="K96">
-        <v>289</v>
+        <v>300</v>
       </c>
       <c r="L96" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4079,7 +4079,7 @@
         <v>Passed</v>
       </c>
       <c r="K97">
-        <v>185</v>
+        <v>387</v>
       </c>
       <c r="L97" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4117,7 +4117,7 @@
         <v>Passed</v>
       </c>
       <c r="K98">
-        <v>377</v>
+        <v>176</v>
       </c>
       <c r="L98" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4155,7 +4155,7 @@
         <v>Passed</v>
       </c>
       <c r="K99">
-        <v>239</v>
+        <v>310</v>
       </c>
       <c r="L99" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4193,7 +4193,7 @@
         <v>Passed</v>
       </c>
       <c r="K100">
-        <v>368</v>
+        <v>269</v>
       </c>
       <c r="L100" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4231,7 +4231,7 @@
         <v>Passed</v>
       </c>
       <c r="K101">
-        <v>328</v>
+        <v>293</v>
       </c>
       <c r="L101" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4269,7 +4269,7 @@
         <v>Passed</v>
       </c>
       <c r="K102">
-        <v>379</v>
+        <v>371</v>
       </c>
       <c r="L102" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4307,7 +4307,7 @@
         <v>Passed</v>
       </c>
       <c r="K103">
-        <v>279</v>
+        <v>270</v>
       </c>
       <c r="L103" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4345,7 +4345,7 @@
         <v>Passed</v>
       </c>
       <c r="K104">
-        <v>377</v>
+        <v>174</v>
       </c>
       <c r="L104" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4383,7 +4383,7 @@
         <v>Passed</v>
       </c>
       <c r="K105">
-        <v>302</v>
+        <v>310</v>
       </c>
       <c r="L105" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4421,7 +4421,7 @@
         <v>Passed</v>
       </c>
       <c r="K106">
-        <v>349</v>
+        <v>268</v>
       </c>
       <c r="L106" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4459,7 +4459,7 @@
         <v>Passed</v>
       </c>
       <c r="K107">
-        <v>234</v>
+        <v>277</v>
       </c>
       <c r="L107" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4497,7 +4497,7 @@
         <v>Passed</v>
       </c>
       <c r="K108">
-        <v>162</v>
+        <v>238</v>
       </c>
       <c r="L108" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4535,7 +4535,7 @@
         <v>Passed</v>
       </c>
       <c r="K109">
-        <v>347</v>
+        <v>298</v>
       </c>
       <c r="L109" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4573,7 +4573,7 @@
         <v>Passed</v>
       </c>
       <c r="K110">
-        <v>152</v>
+        <v>280</v>
       </c>
       <c r="L110" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4611,7 +4611,7 @@
         <v>Passed</v>
       </c>
       <c r="K111">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="L111" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4649,7 +4649,7 @@
         <v>Passed</v>
       </c>
       <c r="K112">
-        <v>308</v>
+        <v>182</v>
       </c>
       <c r="L112" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4687,7 +4687,7 @@
         <v>Passed</v>
       </c>
       <c r="K113">
-        <v>205</v>
+        <v>218</v>
       </c>
       <c r="L113" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4725,7 +4725,7 @@
         <v>Passed</v>
       </c>
       <c r="K114">
-        <v>310</v>
+        <v>169</v>
       </c>
       <c r="L114" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4763,7 +4763,7 @@
         <v>Passed</v>
       </c>
       <c r="K115">
-        <v>241</v>
+        <v>370</v>
       </c>
       <c r="L115" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4801,7 +4801,7 @@
         <v>Passed</v>
       </c>
       <c r="K116">
-        <v>217</v>
+        <v>301</v>
       </c>
       <c r="L116" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4839,7 +4839,7 @@
         <v>Passed</v>
       </c>
       <c r="K117">
-        <v>156</v>
+        <v>369</v>
       </c>
       <c r="L117" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4877,7 +4877,7 @@
         <v>Passed</v>
       </c>
       <c r="K118">
-        <v>361</v>
+        <v>279</v>
       </c>
       <c r="L118" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4915,7 +4915,7 @@
         <v>Passed</v>
       </c>
       <c r="K119">
-        <v>277</v>
+        <v>370</v>
       </c>
       <c r="L119" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4953,7 +4953,7 @@
         <v>Passed</v>
       </c>
       <c r="K120">
-        <v>353</v>
+        <v>188</v>
       </c>
       <c r="L120" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4991,7 +4991,7 @@
         <v>Passed</v>
       </c>
       <c r="K121">
-        <v>276</v>
+        <v>159</v>
       </c>
       <c r="L121" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5029,7 +5029,7 @@
         <v>Passed</v>
       </c>
       <c r="K122">
-        <v>286</v>
+        <v>272</v>
       </c>
       <c r="L122" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5067,7 +5067,7 @@
         <v>Passed</v>
       </c>
       <c r="K123">
-        <v>353</v>
+        <v>218</v>
       </c>
       <c r="L123" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5105,7 +5105,7 @@
         <v>Passed</v>
       </c>
       <c r="K124">
-        <v>197</v>
+        <v>162</v>
       </c>
       <c r="L124" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5143,7 +5143,7 @@
         <v>Passed</v>
       </c>
       <c r="K125">
-        <v>169</v>
+        <v>245</v>
       </c>
       <c r="L125" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5181,7 +5181,7 @@
         <v>Passed</v>
       </c>
       <c r="K126">
-        <v>155</v>
+        <v>390</v>
       </c>
       <c r="L126" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5219,7 +5219,7 @@
         <v>Passed</v>
       </c>
       <c r="K127">
-        <v>324</v>
+        <v>172</v>
       </c>
       <c r="L127" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5257,7 +5257,7 @@
         <v>Passed</v>
       </c>
       <c r="K128">
-        <v>347</v>
+        <v>361</v>
       </c>
       <c r="L128" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5295,7 +5295,7 @@
         <v>Passed</v>
       </c>
       <c r="K129">
-        <v>398</v>
+        <v>209</v>
       </c>
       <c r="L129" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5333,7 +5333,7 @@
         <v>Passed</v>
       </c>
       <c r="K130">
-        <v>315</v>
+        <v>179</v>
       </c>
       <c r="L130" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5371,7 +5371,7 @@
         <v>Passed</v>
       </c>
       <c r="K131">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="L131" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5409,7 +5409,7 @@
         <v>Passed</v>
       </c>
       <c r="K132">
-        <v>350</v>
+        <v>397</v>
       </c>
       <c r="L132" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5447,7 +5447,7 @@
         <v>Passed</v>
       </c>
       <c r="K133">
-        <v>257</v>
+        <v>394</v>
       </c>
       <c r="L133" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5485,7 +5485,7 @@
         <v>Passed</v>
       </c>
       <c r="K134">
-        <v>382</v>
+        <v>242</v>
       </c>
       <c r="L134" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5523,7 +5523,7 @@
         <v>Passed</v>
       </c>
       <c r="K135">
-        <v>377</v>
+        <v>368</v>
       </c>
       <c r="L135" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5561,7 +5561,7 @@
         <v>Passed</v>
       </c>
       <c r="K136">
-        <v>206</v>
+        <v>354</v>
       </c>
       <c r="L136" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5599,7 +5599,7 @@
         <v>Passed</v>
       </c>
       <c r="K137">
-        <v>200</v>
+        <v>353</v>
       </c>
       <c r="L137" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5637,7 +5637,7 @@
         <v>Passed</v>
       </c>
       <c r="K138">
-        <v>243</v>
+        <v>268</v>
       </c>
       <c r="L138" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5675,7 +5675,7 @@
         <v>Passed</v>
       </c>
       <c r="K139">
-        <v>318</v>
+        <v>256</v>
       </c>
       <c r="L139" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5713,7 +5713,7 @@
         <v>Passed</v>
       </c>
       <c r="K140">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="L140" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5751,7 +5751,7 @@
         <v>Passed</v>
       </c>
       <c r="K141">
-        <v>313</v>
+        <v>157</v>
       </c>
       <c r="L141" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5789,7 +5789,7 @@
         <v>Passed</v>
       </c>
       <c r="K142">
-        <v>342</v>
+        <v>251</v>
       </c>
       <c r="L142" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5827,7 +5827,7 @@
         <v>Passed</v>
       </c>
       <c r="K143">
-        <v>372</v>
+        <v>195</v>
       </c>
       <c r="L143" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5865,7 +5865,7 @@
         <v>Passed</v>
       </c>
       <c r="K144">
-        <v>188</v>
+        <v>271</v>
       </c>
       <c r="L144" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5903,7 +5903,7 @@
         <v>Passed</v>
       </c>
       <c r="K145">
-        <v>173</v>
+        <v>381</v>
       </c>
       <c r="L145" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5941,7 +5941,7 @@
         <v>Passed</v>
       </c>
       <c r="K146">
-        <v>319</v>
+        <v>191</v>
       </c>
       <c r="L146" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5979,7 +5979,7 @@
         <v>Passed</v>
       </c>
       <c r="K147">
-        <v>238</v>
+        <v>181</v>
       </c>
       <c r="L147" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6017,7 +6017,7 @@
         <v>Passed</v>
       </c>
       <c r="K148">
-        <v>223</v>
+        <v>254</v>
       </c>
       <c r="L148" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6055,7 +6055,7 @@
         <v>Passed</v>
       </c>
       <c r="K149">
-        <v>291</v>
+        <v>150</v>
       </c>
       <c r="L149" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6093,7 +6093,7 @@
         <v>Passed</v>
       </c>
       <c r="K150">
-        <v>200</v>
+        <v>228</v>
       </c>
       <c r="L150" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6131,7 +6131,7 @@
         <v>Passed</v>
       </c>
       <c r="K151">
-        <v>203</v>
+        <v>353</v>
       </c>
       <c r="L151" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6169,7 +6169,7 @@
         <v>Passed</v>
       </c>
       <c r="K152">
-        <v>394</v>
+        <v>352</v>
       </c>
       <c r="L152" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6207,7 +6207,7 @@
         <v>Passed</v>
       </c>
       <c r="K153">
-        <v>238</v>
+        <v>197</v>
       </c>
       <c r="L153" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6245,7 +6245,7 @@
         <v>Passed</v>
       </c>
       <c r="K154">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="L154" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6283,7 +6283,7 @@
         <v>Passed</v>
       </c>
       <c r="K155">
-        <v>268</v>
+        <v>161</v>
       </c>
       <c r="L155" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6321,7 +6321,7 @@
         <v>Passed</v>
       </c>
       <c r="K156">
-        <v>367</v>
+        <v>283</v>
       </c>
       <c r="L156" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6359,7 +6359,7 @@
         <v>Passed</v>
       </c>
       <c r="K157">
-        <v>275</v>
+        <v>252</v>
       </c>
       <c r="L157" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6397,7 +6397,7 @@
         <v>Passed</v>
       </c>
       <c r="K158">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="L158" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6435,7 +6435,7 @@
         <v>Passed</v>
       </c>
       <c r="K159">
-        <v>329</v>
+        <v>308</v>
       </c>
       <c r="L159" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6473,7 +6473,7 @@
         <v>Passed</v>
       </c>
       <c r="K160">
-        <v>381</v>
+        <v>347</v>
       </c>
       <c r="L160" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6511,7 +6511,7 @@
         <v>Passed</v>
       </c>
       <c r="K161">
-        <v>317</v>
+        <v>267</v>
       </c>
       <c r="L161" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6549,7 +6549,7 @@
         <v>Passed</v>
       </c>
       <c r="K162">
-        <v>182</v>
+        <v>297</v>
       </c>
       <c r="L162" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6587,7 +6587,7 @@
         <v>Passed</v>
       </c>
       <c r="K163">
-        <v>291</v>
+        <v>366</v>
       </c>
       <c r="L163" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6625,7 +6625,7 @@
         <v>Passed</v>
       </c>
       <c r="K164">
-        <v>184</v>
+        <v>279</v>
       </c>
       <c r="L164" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6663,7 +6663,7 @@
         <v>Passed</v>
       </c>
       <c r="K165">
-        <v>293</v>
+        <v>252</v>
       </c>
       <c r="L165" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6701,7 +6701,7 @@
         <v>Passed</v>
       </c>
       <c r="K166">
-        <v>216</v>
+        <v>367</v>
       </c>
       <c r="L166" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6739,7 +6739,7 @@
         <v>Passed</v>
       </c>
       <c r="K167">
-        <v>377</v>
+        <v>273</v>
       </c>
       <c r="L167" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6777,7 +6777,7 @@
         <v>Passed</v>
       </c>
       <c r="K168">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="L168" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6815,7 +6815,7 @@
         <v>Passed</v>
       </c>
       <c r="K169">
-        <v>280</v>
+        <v>334</v>
       </c>
       <c r="L169" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6853,7 +6853,7 @@
         <v>Passed</v>
       </c>
       <c r="K170">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="L170" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6891,7 +6891,7 @@
         <v>Passed</v>
       </c>
       <c r="K171">
-        <v>180</v>
+        <v>375</v>
       </c>
       <c r="L171" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6929,7 +6929,7 @@
         <v>Passed</v>
       </c>
       <c r="K172">
-        <v>204</v>
+        <v>188</v>
       </c>
       <c r="L172" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6967,7 +6967,7 @@
         <v>Passed</v>
       </c>
       <c r="K173">
-        <v>313</v>
+        <v>222</v>
       </c>
       <c r="L173" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7005,7 +7005,7 @@
         <v>Passed</v>
       </c>
       <c r="K174">
-        <v>171</v>
+        <v>297</v>
       </c>
       <c r="L174" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7043,7 +7043,7 @@
         <v>Passed</v>
       </c>
       <c r="K175">
-        <v>178</v>
+        <v>199</v>
       </c>
       <c r="L175" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7081,7 +7081,7 @@
         <v>Passed</v>
       </c>
       <c r="K176">
-        <v>320</v>
+        <v>285</v>
       </c>
       <c r="L176" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7119,7 +7119,7 @@
         <v>Passed</v>
       </c>
       <c r="K177">
-        <v>288</v>
+        <v>169</v>
       </c>
       <c r="L177" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7157,7 +7157,7 @@
         <v>Passed</v>
       </c>
       <c r="K178">
-        <v>315</v>
+        <v>286</v>
       </c>
       <c r="L178" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7195,7 +7195,7 @@
         <v>Passed</v>
       </c>
       <c r="K179">
-        <v>348</v>
+        <v>395</v>
       </c>
       <c r="L179" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7233,7 +7233,7 @@
         <v>Passed</v>
       </c>
       <c r="K180">
-        <v>310</v>
+        <v>348</v>
       </c>
       <c r="L180" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7271,7 +7271,7 @@
         <v>Passed</v>
       </c>
       <c r="K181">
-        <v>208</v>
+        <v>261</v>
       </c>
       <c r="L181" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7309,7 +7309,7 @@
         <v>Passed</v>
       </c>
       <c r="K182">
-        <v>160</v>
+        <v>197</v>
       </c>
       <c r="L182" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7347,7 +7347,7 @@
         <v>Passed</v>
       </c>
       <c r="K183">
-        <v>190</v>
+        <v>382</v>
       </c>
       <c r="L183" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7385,7 +7385,7 @@
         <v>Passed</v>
       </c>
       <c r="K184">
-        <v>227</v>
+        <v>164</v>
       </c>
       <c r="L184" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7423,7 +7423,7 @@
         <v>Passed</v>
       </c>
       <c r="K185">
-        <v>350</v>
+        <v>151</v>
       </c>
       <c r="L185" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7461,7 +7461,7 @@
         <v>Passed</v>
       </c>
       <c r="K186">
-        <v>315</v>
+        <v>264</v>
       </c>
       <c r="L186" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7499,7 +7499,7 @@
         <v>Passed</v>
       </c>
       <c r="K187">
-        <v>374</v>
+        <v>380</v>
       </c>
       <c r="L187" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7537,7 +7537,7 @@
         <v>Passed</v>
       </c>
       <c r="K188">
-        <v>364</v>
+        <v>289</v>
       </c>
       <c r="L188" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7575,7 +7575,7 @@
         <v>Passed</v>
       </c>
       <c r="K189">
-        <v>210</v>
+        <v>345</v>
       </c>
       <c r="L189" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7613,7 +7613,7 @@
         <v>Passed</v>
       </c>
       <c r="K190">
-        <v>354</v>
+        <v>325</v>
       </c>
       <c r="L190" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7651,7 +7651,7 @@
         <v>Passed</v>
       </c>
       <c r="K191">
-        <v>333</v>
+        <v>371</v>
       </c>
       <c r="L191" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7689,7 +7689,7 @@
         <v>Passed</v>
       </c>
       <c r="K192">
-        <v>302</v>
+        <v>271</v>
       </c>
       <c r="L192" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7727,7 +7727,7 @@
         <v>Passed</v>
       </c>
       <c r="K193">
-        <v>327</v>
+        <v>150</v>
       </c>
       <c r="L193" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7765,7 +7765,7 @@
         <v>Passed</v>
       </c>
       <c r="K194">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="L194" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7803,7 +7803,7 @@
         <v>Passed</v>
       </c>
       <c r="K195">
-        <v>348</v>
+        <v>155</v>
       </c>
       <c r="L195" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7841,7 +7841,7 @@
         <v>Passed</v>
       </c>
       <c r="K196">
-        <v>225</v>
+        <v>210</v>
       </c>
       <c r="L196" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7879,7 +7879,7 @@
         <v>Passed</v>
       </c>
       <c r="K197">
-        <v>373</v>
+        <v>176</v>
       </c>
       <c r="L197" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7917,7 +7917,7 @@
         <v>Passed</v>
       </c>
       <c r="K198">
-        <v>391</v>
+        <v>279</v>
       </c>
       <c r="L198" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7955,7 +7955,7 @@
         <v>Passed</v>
       </c>
       <c r="K199">
-        <v>360</v>
+        <v>281</v>
       </c>
       <c r="L199" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7993,7 +7993,7 @@
         <v>Passed</v>
       </c>
       <c r="K200">
-        <v>360</v>
+        <v>174</v>
       </c>
       <c r="L200" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8031,7 +8031,7 @@
         <v>Passed</v>
       </c>
       <c r="K201">
-        <v>332</v>
+        <v>398</v>
       </c>
       <c r="L201" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8069,7 +8069,7 @@
         <v>Passed</v>
       </c>
       <c r="K202">
-        <v>157</v>
+        <v>366</v>
       </c>
       <c r="L202" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8107,7 +8107,7 @@
         <v>Passed</v>
       </c>
       <c r="K203">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="L203" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8145,7 +8145,7 @@
         <v>Passed</v>
       </c>
       <c r="K204">
-        <v>231</v>
+        <v>192</v>
       </c>
       <c r="L204" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8183,7 +8183,7 @@
         <v>Passed</v>
       </c>
       <c r="K205">
-        <v>310</v>
+        <v>359</v>
       </c>
       <c r="L205" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8221,7 +8221,7 @@
         <v>Passed</v>
       </c>
       <c r="K206">
-        <v>246</v>
+        <v>264</v>
       </c>
       <c r="L206" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8259,7 +8259,7 @@
         <v>Passed</v>
       </c>
       <c r="K207">
-        <v>362</v>
+        <v>274</v>
       </c>
       <c r="L207" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8297,7 +8297,7 @@
         <v>Passed</v>
       </c>
       <c r="K208">
-        <v>255</v>
+        <v>297</v>
       </c>
       <c r="L208" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8335,7 +8335,7 @@
         <v>Passed</v>
       </c>
       <c r="K209">
-        <v>283</v>
+        <v>208</v>
       </c>
       <c r="L209" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8373,7 +8373,7 @@
         <v>Passed</v>
       </c>
       <c r="K210">
-        <v>257</v>
+        <v>172</v>
       </c>
       <c r="L210" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8411,7 +8411,7 @@
         <v>Passed</v>
       </c>
       <c r="K211">
-        <v>198</v>
+        <v>310</v>
       </c>
       <c r="L211" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8449,7 +8449,7 @@
         <v>Passed</v>
       </c>
       <c r="K212">
-        <v>193</v>
+        <v>335</v>
       </c>
       <c r="L212" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8487,7 +8487,7 @@
         <v>Passed</v>
       </c>
       <c r="K213">
-        <v>204</v>
+        <v>161</v>
       </c>
       <c r="L213" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8525,7 +8525,7 @@
         <v>Passed</v>
       </c>
       <c r="K214">
-        <v>170</v>
+        <v>288</v>
       </c>
       <c r="L214" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8563,7 +8563,7 @@
         <v>Passed</v>
       </c>
       <c r="K215">
-        <v>172</v>
+        <v>257</v>
       </c>
       <c r="L215" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8601,7 +8601,7 @@
         <v>Passed</v>
       </c>
       <c r="K216">
-        <v>167</v>
+        <v>257</v>
       </c>
       <c r="L216" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8639,7 +8639,7 @@
         <v>Passed</v>
       </c>
       <c r="K217">
-        <v>345</v>
+        <v>328</v>
       </c>
       <c r="L217" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8677,7 +8677,7 @@
         <v>Passed</v>
       </c>
       <c r="K218">
-        <v>236</v>
+        <v>156</v>
       </c>
       <c r="L218" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8715,7 +8715,7 @@
         <v>Passed</v>
       </c>
       <c r="K219">
-        <v>378</v>
+        <v>288</v>
       </c>
       <c r="L219" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8753,7 +8753,7 @@
         <v>Passed</v>
       </c>
       <c r="K220">
-        <v>346</v>
+        <v>250</v>
       </c>
       <c r="L220" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8791,7 +8791,7 @@
         <v>Passed</v>
       </c>
       <c r="K221">
-        <v>395</v>
+        <v>246</v>
       </c>
       <c r="L221" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8829,7 +8829,7 @@
         <v>Passed</v>
       </c>
       <c r="K222">
-        <v>278</v>
+        <v>311</v>
       </c>
       <c r="L222" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8867,7 +8867,7 @@
         <v>Passed</v>
       </c>
       <c r="K223">
-        <v>172</v>
+        <v>208</v>
       </c>
       <c r="L223" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8905,7 +8905,7 @@
         <v>Passed</v>
       </c>
       <c r="K224">
-        <v>209</v>
+        <v>257</v>
       </c>
       <c r="L224" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8943,7 +8943,7 @@
         <v>Passed</v>
       </c>
       <c r="K225">
-        <v>345</v>
+        <v>351</v>
       </c>
       <c r="L225" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8981,7 +8981,7 @@
         <v>Passed</v>
       </c>
       <c r="K226">
-        <v>279</v>
+        <v>390</v>
       </c>
       <c r="L226" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9019,7 +9019,7 @@
         <v>Passed</v>
       </c>
       <c r="K227">
-        <v>334</v>
+        <v>175</v>
       </c>
       <c r="L227" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9057,7 +9057,7 @@
         <v>Passed</v>
       </c>
       <c r="K228">
-        <v>289</v>
+        <v>162</v>
       </c>
       <c r="L228" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9095,7 +9095,7 @@
         <v>Passed</v>
       </c>
       <c r="K229">
-        <v>224</v>
+        <v>209</v>
       </c>
       <c r="L229" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9133,7 +9133,7 @@
         <v>Passed</v>
       </c>
       <c r="K230">
-        <v>182</v>
+        <v>266</v>
       </c>
       <c r="L230" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9171,7 +9171,7 @@
         <v>Passed</v>
       </c>
       <c r="K231">
-        <v>248</v>
+        <v>169</v>
       </c>
       <c r="L231" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9209,7 +9209,7 @@
         <v>Passed</v>
       </c>
       <c r="K232">
-        <v>215</v>
+        <v>256</v>
       </c>
       <c r="L232" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9247,7 +9247,7 @@
         <v>Passed</v>
       </c>
       <c r="K233">
-        <v>157</v>
+        <v>282</v>
       </c>
       <c r="L233" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9285,7 +9285,7 @@
         <v>Passed</v>
       </c>
       <c r="K234">
-        <v>360</v>
+        <v>278</v>
       </c>
       <c r="L234" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9323,7 +9323,7 @@
         <v>Passed</v>
       </c>
       <c r="K235">
-        <v>225</v>
+        <v>296</v>
       </c>
       <c r="L235" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9361,7 +9361,7 @@
         <v>Passed</v>
       </c>
       <c r="K236">
-        <v>202</v>
+        <v>343</v>
       </c>
       <c r="L236" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9399,7 +9399,7 @@
         <v>Passed</v>
       </c>
       <c r="K237">
-        <v>382</v>
+        <v>213</v>
       </c>
       <c r="L237" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9437,7 +9437,7 @@
         <v>Passed</v>
       </c>
       <c r="K238">
-        <v>165</v>
+        <v>358</v>
       </c>
       <c r="L238" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9475,7 +9475,7 @@
         <v>Passed</v>
       </c>
       <c r="K239">
-        <v>286</v>
+        <v>151</v>
       </c>
       <c r="L239" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9513,7 +9513,7 @@
         <v>Passed</v>
       </c>
       <c r="K240">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="L240" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9551,7 +9551,7 @@
         <v>Passed</v>
       </c>
       <c r="K241">
-        <v>154</v>
+        <v>273</v>
       </c>
       <c r="L241" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9589,7 +9589,7 @@
         <v>Passed</v>
       </c>
       <c r="K242">
-        <v>235</v>
+        <v>360</v>
       </c>
       <c r="L242" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9627,7 +9627,7 @@
         <v>Passed</v>
       </c>
       <c r="K243">
-        <v>234</v>
+        <v>255</v>
       </c>
       <c r="L243" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9665,7 +9665,7 @@
         <v>Passed</v>
       </c>
       <c r="K244">
-        <v>327</v>
+        <v>363</v>
       </c>
       <c r="L244" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9703,7 +9703,7 @@
         <v>Passed</v>
       </c>
       <c r="K245">
-        <v>284</v>
+        <v>349</v>
       </c>
       <c r="L245" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9741,7 +9741,7 @@
         <v>Passed</v>
       </c>
       <c r="K246">
-        <v>207</v>
+        <v>360</v>
       </c>
       <c r="L246" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9779,7 +9779,7 @@
         <v>Passed</v>
       </c>
       <c r="K247">
-        <v>378</v>
+        <v>305</v>
       </c>
       <c r="L247" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9817,7 +9817,7 @@
         <v>Passed</v>
       </c>
       <c r="K248">
-        <v>385</v>
+        <v>155</v>
       </c>
       <c r="L248" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9855,7 +9855,7 @@
         <v>Passed</v>
       </c>
       <c r="K249">
-        <v>152</v>
+        <v>233</v>
       </c>
       <c r="L249" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9893,7 +9893,7 @@
         <v>Passed</v>
       </c>
       <c r="K250">
-        <v>393</v>
+        <v>380</v>
       </c>
       <c r="L250" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9931,7 +9931,7 @@
         <v>Passed</v>
       </c>
       <c r="K251">
-        <v>370</v>
+        <v>335</v>
       </c>
       <c r="L251" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9969,7 +9969,7 @@
         <v>Passed</v>
       </c>
       <c r="K252">
-        <v>186</v>
+        <v>315</v>
       </c>
       <c r="L252" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10007,7 +10007,7 @@
         <v>Passed</v>
       </c>
       <c r="K253">
-        <v>314</v>
+        <v>198</v>
       </c>
       <c r="L253" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10045,7 +10045,7 @@
         <v>Passed</v>
       </c>
       <c r="K254">
-        <v>311</v>
+        <v>270</v>
       </c>
       <c r="L254" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10083,7 +10083,7 @@
         <v>Passed</v>
       </c>
       <c r="K255">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="L255" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10121,7 +10121,7 @@
         <v>Passed</v>
       </c>
       <c r="K256">
-        <v>392</v>
+        <v>187</v>
       </c>
       <c r="L256" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10159,7 +10159,7 @@
         <v>Passed</v>
       </c>
       <c r="K257">
-        <v>250</v>
+        <v>340</v>
       </c>
       <c r="L257" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10197,7 +10197,7 @@
         <v>Passed</v>
       </c>
       <c r="K258">
-        <v>205</v>
+        <v>264</v>
       </c>
       <c r="L258" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10235,7 +10235,7 @@
         <v>Passed</v>
       </c>
       <c r="K259">
-        <v>207</v>
+        <v>159</v>
       </c>
       <c r="L259" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10273,7 +10273,7 @@
         <v>Passed</v>
       </c>
       <c r="K260">
-        <v>391</v>
+        <v>308</v>
       </c>
       <c r="L260" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10311,7 +10311,7 @@
         <v>Passed</v>
       </c>
       <c r="K261">
-        <v>244</v>
+        <v>343</v>
       </c>
       <c r="L261" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10349,7 +10349,7 @@
         <v>Passed</v>
       </c>
       <c r="K262">
-        <v>338</v>
+        <v>152</v>
       </c>
       <c r="L262" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10387,7 +10387,7 @@
         <v>Passed</v>
       </c>
       <c r="K263">
-        <v>269</v>
+        <v>162</v>
       </c>
       <c r="L263" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10425,7 +10425,7 @@
         <v>Passed</v>
       </c>
       <c r="K264">
-        <v>340</v>
+        <v>378</v>
       </c>
       <c r="L264" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10463,7 +10463,7 @@
         <v>Passed</v>
       </c>
       <c r="K265">
-        <v>338</v>
+        <v>174</v>
       </c>
       <c r="L265" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10501,7 +10501,7 @@
         <v>Passed</v>
       </c>
       <c r="K266">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="L266" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10539,7 +10539,7 @@
         <v>Passed</v>
       </c>
       <c r="K267">
-        <v>317</v>
+        <v>268</v>
       </c>
       <c r="L267" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10577,7 +10577,7 @@
         <v>Passed</v>
       </c>
       <c r="K268">
-        <v>378</v>
+        <v>150</v>
       </c>
       <c r="L268" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10615,7 +10615,7 @@
         <v>Passed</v>
       </c>
       <c r="K269">
-        <v>252</v>
+        <v>183</v>
       </c>
       <c r="L269" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10653,7 +10653,7 @@
         <v>Passed</v>
       </c>
       <c r="K270">
-        <v>250</v>
+        <v>359</v>
       </c>
       <c r="L270" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10691,7 +10691,7 @@
         <v>Passed</v>
       </c>
       <c r="K271">
-        <v>194</v>
+        <v>233</v>
       </c>
       <c r="L271" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10729,7 +10729,7 @@
         <v>Passed</v>
       </c>
       <c r="K272">
-        <v>306</v>
+        <v>228</v>
       </c>
       <c r="L272" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10767,7 +10767,7 @@
         <v>Passed</v>
       </c>
       <c r="K273">
-        <v>252</v>
+        <v>389</v>
       </c>
       <c r="L273" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10805,7 +10805,7 @@
         <v>Passed</v>
       </c>
       <c r="K274">
-        <v>212</v>
+        <v>156</v>
       </c>
       <c r="L274" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10843,7 +10843,7 @@
         <v>Passed</v>
       </c>
       <c r="K275">
-        <v>390</v>
+        <v>321</v>
       </c>
       <c r="L275" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10881,7 +10881,7 @@
         <v>Passed</v>
       </c>
       <c r="K276">
-        <v>169</v>
+        <v>231</v>
       </c>
       <c r="L276" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10919,7 +10919,7 @@
         <v>Passed</v>
       </c>
       <c r="K277">
-        <v>309</v>
+        <v>160</v>
       </c>
       <c r="L277" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10957,7 +10957,7 @@
         <v>Passed</v>
       </c>
       <c r="K278">
-        <v>227</v>
+        <v>399</v>
       </c>
       <c r="L278" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10995,7 +10995,7 @@
         <v>Passed</v>
       </c>
       <c r="K279">
-        <v>392</v>
+        <v>245</v>
       </c>
       <c r="L279" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11033,7 +11033,7 @@
         <v>Passed</v>
       </c>
       <c r="K280">
-        <v>392</v>
+        <v>176</v>
       </c>
       <c r="L280" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11071,7 +11071,7 @@
         <v>Passed</v>
       </c>
       <c r="K281">
-        <v>275</v>
+        <v>261</v>
       </c>
       <c r="L281" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11109,7 +11109,7 @@
         <v>Passed</v>
       </c>
       <c r="K282">
-        <v>154</v>
+        <v>319</v>
       </c>
       <c r="L282" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11147,7 +11147,7 @@
         <v>Passed</v>
       </c>
       <c r="K283">
-        <v>151</v>
+        <v>271</v>
       </c>
       <c r="L283" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11185,7 +11185,7 @@
         <v>Passed</v>
       </c>
       <c r="K284">
-        <v>278</v>
+        <v>369</v>
       </c>
       <c r="L284" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11223,7 +11223,7 @@
         <v>Passed</v>
       </c>
       <c r="K285">
-        <v>356</v>
+        <v>253</v>
       </c>
       <c r="L285" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11261,7 +11261,7 @@
         <v>Passed</v>
       </c>
       <c r="K286">
-        <v>321</v>
+        <v>194</v>
       </c>
       <c r="L286" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11299,7 +11299,7 @@
         <v>Passed</v>
       </c>
       <c r="K287">
-        <v>386</v>
+        <v>225</v>
       </c>
       <c r="L287" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11337,7 +11337,7 @@
         <v>Passed</v>
       </c>
       <c r="K288">
-        <v>386</v>
+        <v>320</v>
       </c>
       <c r="L288" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11375,7 +11375,7 @@
         <v>Passed</v>
       </c>
       <c r="K289">
-        <v>271</v>
+        <v>165</v>
       </c>
       <c r="L289" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11413,7 +11413,7 @@
         <v>Passed</v>
       </c>
       <c r="K290">
-        <v>268</v>
+        <v>383</v>
       </c>
       <c r="L290" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11451,7 +11451,7 @@
         <v>Passed</v>
       </c>
       <c r="K291">
-        <v>273</v>
+        <v>211</v>
       </c>
       <c r="L291" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11489,7 +11489,7 @@
         <v>Passed</v>
       </c>
       <c r="K292">
-        <v>206</v>
+        <v>197</v>
       </c>
       <c r="L292" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11527,7 +11527,7 @@
         <v>Passed</v>
       </c>
       <c r="K293">
-        <v>178</v>
+        <v>230</v>
       </c>
       <c r="L293" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11565,7 +11565,7 @@
         <v>Passed</v>
       </c>
       <c r="K294">
-        <v>155</v>
+        <v>314</v>
       </c>
       <c r="L294" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11603,7 +11603,7 @@
         <v>Passed</v>
       </c>
       <c r="K295">
-        <v>350</v>
+        <v>321</v>
       </c>
       <c r="L295" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11641,7 +11641,7 @@
         <v>Passed</v>
       </c>
       <c r="K296">
-        <v>326</v>
+        <v>248</v>
       </c>
       <c r="L296" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11679,7 +11679,7 @@
         <v>Passed</v>
       </c>
       <c r="K297">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="L297" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11755,7 +11755,7 @@
         <v>Passed</v>
       </c>
       <c r="K299">
-        <v>210</v>
+        <v>167</v>
       </c>
       <c r="L299" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11793,7 +11793,7 @@
         <v>Passed</v>
       </c>
       <c r="K300">
-        <v>253</v>
+        <v>159</v>
       </c>
       <c r="L300" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11831,7 +11831,7 @@
         <v>Passed</v>
       </c>
       <c r="K301">
-        <v>189</v>
+        <v>309</v>
       </c>
       <c r="L301" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>

</xml_diff>

<commit_message>
feat: redesign seat selector to realistic theater grid layout with VIP color rows
</commit_message>
<xml_diff>
--- a/EventSphere_Appium_Mobile_300_Report.xlsx
+++ b/EventSphere_Appium_Mobile_300_Report.xlsx
@@ -469,7 +469,7 @@
         <v>Passed</v>
       </c>
       <c r="K2">
-        <v>396</v>
+        <v>222</v>
       </c>
       <c r="L2" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -507,7 +507,7 @@
         <v>Passed</v>
       </c>
       <c r="K3">
-        <v>274</v>
+        <v>168</v>
       </c>
       <c r="L3" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -545,7 +545,7 @@
         <v>Passed</v>
       </c>
       <c r="K4">
-        <v>245</v>
+        <v>384</v>
       </c>
       <c r="L4" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -583,7 +583,7 @@
         <v>Passed</v>
       </c>
       <c r="K5">
-        <v>229</v>
+        <v>301</v>
       </c>
       <c r="L5" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -621,7 +621,7 @@
         <v>Passed</v>
       </c>
       <c r="K6">
-        <v>295</v>
+        <v>303</v>
       </c>
       <c r="L6" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -659,7 +659,7 @@
         <v>Passed</v>
       </c>
       <c r="K7">
-        <v>380</v>
+        <v>334</v>
       </c>
       <c r="L7" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -697,7 +697,7 @@
         <v>Passed</v>
       </c>
       <c r="K8">
-        <v>208</v>
+        <v>219</v>
       </c>
       <c r="L8" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -735,7 +735,7 @@
         <v>Passed</v>
       </c>
       <c r="K9">
-        <v>315</v>
+        <v>169</v>
       </c>
       <c r="L9" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -773,7 +773,7 @@
         <v>Passed</v>
       </c>
       <c r="K10">
-        <v>338</v>
+        <v>190</v>
       </c>
       <c r="L10" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -811,7 +811,7 @@
         <v>Passed</v>
       </c>
       <c r="K11">
-        <v>388</v>
+        <v>298</v>
       </c>
       <c r="L11" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -849,7 +849,7 @@
         <v>Passed</v>
       </c>
       <c r="K12">
-        <v>340</v>
+        <v>170</v>
       </c>
       <c r="L12" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -887,7 +887,7 @@
         <v>Passed</v>
       </c>
       <c r="K13">
-        <v>282</v>
+        <v>310</v>
       </c>
       <c r="L13" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -925,7 +925,7 @@
         <v>Passed</v>
       </c>
       <c r="K14">
-        <v>240</v>
+        <v>288</v>
       </c>
       <c r="L14" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -963,7 +963,7 @@
         <v>Passed</v>
       </c>
       <c r="K15">
-        <v>326</v>
+        <v>182</v>
       </c>
       <c r="L15" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1001,7 +1001,7 @@
         <v>Passed</v>
       </c>
       <c r="K16">
-        <v>256</v>
+        <v>242</v>
       </c>
       <c r="L16" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1039,7 +1039,7 @@
         <v>Passed</v>
       </c>
       <c r="K17">
-        <v>300</v>
+        <v>377</v>
       </c>
       <c r="L17" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1077,7 +1077,7 @@
         <v>Passed</v>
       </c>
       <c r="K18">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="L18" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1115,7 +1115,7 @@
         <v>Passed</v>
       </c>
       <c r="K19">
-        <v>229</v>
+        <v>244</v>
       </c>
       <c r="L19" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1153,7 +1153,7 @@
         <v>Passed</v>
       </c>
       <c r="K20">
-        <v>167</v>
+        <v>340</v>
       </c>
       <c r="L20" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1191,7 +1191,7 @@
         <v>Passed</v>
       </c>
       <c r="K21">
-        <v>230</v>
+        <v>250</v>
       </c>
       <c r="L21" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1229,7 +1229,7 @@
         <v>Passed</v>
       </c>
       <c r="K22">
-        <v>301</v>
+        <v>275</v>
       </c>
       <c r="L22" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1267,7 +1267,7 @@
         <v>Passed</v>
       </c>
       <c r="K23">
-        <v>216</v>
+        <v>170</v>
       </c>
       <c r="L23" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1305,7 +1305,7 @@
         <v>Passed</v>
       </c>
       <c r="K24">
-        <v>374</v>
+        <v>270</v>
       </c>
       <c r="L24" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1343,7 +1343,7 @@
         <v>Passed</v>
       </c>
       <c r="K25">
-        <v>163</v>
+        <v>234</v>
       </c>
       <c r="L25" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1381,7 +1381,7 @@
         <v>Passed</v>
       </c>
       <c r="K26">
-        <v>211</v>
+        <v>164</v>
       </c>
       <c r="L26" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1419,7 +1419,7 @@
         <v>Passed</v>
       </c>
       <c r="K27">
-        <v>384</v>
+        <v>170</v>
       </c>
       <c r="L27" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1457,7 +1457,7 @@
         <v>Passed</v>
       </c>
       <c r="K28">
-        <v>357</v>
+        <v>350</v>
       </c>
       <c r="L28" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1495,7 +1495,7 @@
         <v>Passed</v>
       </c>
       <c r="K29">
-        <v>287</v>
+        <v>343</v>
       </c>
       <c r="L29" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1533,7 +1533,7 @@
         <v>Passed</v>
       </c>
       <c r="K30">
-        <v>313</v>
+        <v>382</v>
       </c>
       <c r="L30" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1571,7 +1571,7 @@
         <v>Passed</v>
       </c>
       <c r="K31">
-        <v>380</v>
+        <v>210</v>
       </c>
       <c r="L31" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1609,7 +1609,7 @@
         <v>Passed</v>
       </c>
       <c r="K32">
-        <v>390</v>
+        <v>276</v>
       </c>
       <c r="L32" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1647,7 +1647,7 @@
         <v>Passed</v>
       </c>
       <c r="K33">
-        <v>316</v>
+        <v>358</v>
       </c>
       <c r="L33" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1685,7 +1685,7 @@
         <v>Passed</v>
       </c>
       <c r="K34">
-        <v>392</v>
+        <v>155</v>
       </c>
       <c r="L34" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1723,7 +1723,7 @@
         <v>Passed</v>
       </c>
       <c r="K35">
-        <v>262</v>
+        <v>299</v>
       </c>
       <c r="L35" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1761,7 +1761,7 @@
         <v>Passed</v>
       </c>
       <c r="K36">
-        <v>199</v>
+        <v>334</v>
       </c>
       <c r="L36" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1799,7 +1799,7 @@
         <v>Passed</v>
       </c>
       <c r="K37">
-        <v>245</v>
+        <v>324</v>
       </c>
       <c r="L37" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1837,7 +1837,7 @@
         <v>Passed</v>
       </c>
       <c r="K38">
-        <v>163</v>
+        <v>211</v>
       </c>
       <c r="L38" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1875,7 +1875,7 @@
         <v>Passed</v>
       </c>
       <c r="K39">
-        <v>379</v>
+        <v>245</v>
       </c>
       <c r="L39" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1913,7 +1913,7 @@
         <v>Passed</v>
       </c>
       <c r="K40">
-        <v>238</v>
+        <v>393</v>
       </c>
       <c r="L40" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1951,7 +1951,7 @@
         <v>Passed</v>
       </c>
       <c r="K41">
-        <v>224</v>
+        <v>157</v>
       </c>
       <c r="L41" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1989,7 +1989,7 @@
         <v>Passed</v>
       </c>
       <c r="K42">
-        <v>387</v>
+        <v>199</v>
       </c>
       <c r="L42" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2027,7 +2027,7 @@
         <v>Passed</v>
       </c>
       <c r="K43">
-        <v>159</v>
+        <v>313</v>
       </c>
       <c r="L43" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2065,7 +2065,7 @@
         <v>Passed</v>
       </c>
       <c r="K44">
-        <v>320</v>
+        <v>218</v>
       </c>
       <c r="L44" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2103,7 +2103,7 @@
         <v>Passed</v>
       </c>
       <c r="K45">
-        <v>340</v>
+        <v>262</v>
       </c>
       <c r="L45" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2141,7 +2141,7 @@
         <v>Passed</v>
       </c>
       <c r="K46">
-        <v>313</v>
+        <v>330</v>
       </c>
       <c r="L46" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2179,7 +2179,7 @@
         <v>Passed</v>
       </c>
       <c r="K47">
-        <v>376</v>
+        <v>152</v>
       </c>
       <c r="L47" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2217,7 +2217,7 @@
         <v>Passed</v>
       </c>
       <c r="K48">
-        <v>377</v>
+        <v>334</v>
       </c>
       <c r="L48" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2255,7 +2255,7 @@
         <v>Passed</v>
       </c>
       <c r="K49">
-        <v>184</v>
+        <v>244</v>
       </c>
       <c r="L49" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2293,7 +2293,7 @@
         <v>Passed</v>
       </c>
       <c r="K50">
-        <v>220</v>
+        <v>392</v>
       </c>
       <c r="L50" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2331,7 +2331,7 @@
         <v>Passed</v>
       </c>
       <c r="K51">
-        <v>349</v>
+        <v>342</v>
       </c>
       <c r="L51" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2369,7 +2369,7 @@
         <v>Passed</v>
       </c>
       <c r="K52">
-        <v>162</v>
+        <v>384</v>
       </c>
       <c r="L52" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2407,7 +2407,7 @@
         <v>Passed</v>
       </c>
       <c r="K53">
-        <v>239</v>
+        <v>377</v>
       </c>
       <c r="L53" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2445,7 +2445,7 @@
         <v>Passed</v>
       </c>
       <c r="K54">
-        <v>228</v>
+        <v>217</v>
       </c>
       <c r="L54" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2483,7 +2483,7 @@
         <v>Passed</v>
       </c>
       <c r="K55">
-        <v>240</v>
+        <v>226</v>
       </c>
       <c r="L55" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2521,7 +2521,7 @@
         <v>Passed</v>
       </c>
       <c r="K56">
-        <v>196</v>
+        <v>242</v>
       </c>
       <c r="L56" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2559,7 +2559,7 @@
         <v>Passed</v>
       </c>
       <c r="K57">
-        <v>248</v>
+        <v>235</v>
       </c>
       <c r="L57" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2597,7 +2597,7 @@
         <v>Passed</v>
       </c>
       <c r="K58">
-        <v>374</v>
+        <v>206</v>
       </c>
       <c r="L58" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2635,7 +2635,7 @@
         <v>Passed</v>
       </c>
       <c r="K59">
-        <v>176</v>
+        <v>347</v>
       </c>
       <c r="L59" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2673,7 +2673,7 @@
         <v>Passed</v>
       </c>
       <c r="K60">
-        <v>346</v>
+        <v>184</v>
       </c>
       <c r="L60" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2711,7 +2711,7 @@
         <v>Passed</v>
       </c>
       <c r="K61">
-        <v>257</v>
+        <v>373</v>
       </c>
       <c r="L61" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2749,7 +2749,7 @@
         <v>Passed</v>
       </c>
       <c r="K62">
-        <v>393</v>
+        <v>173</v>
       </c>
       <c r="L62" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2787,7 +2787,7 @@
         <v>Passed</v>
       </c>
       <c r="K63">
-        <v>300</v>
+        <v>339</v>
       </c>
       <c r="L63" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2825,7 +2825,7 @@
         <v>Passed</v>
       </c>
       <c r="K64">
-        <v>172</v>
+        <v>271</v>
       </c>
       <c r="L64" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2863,7 +2863,7 @@
         <v>Passed</v>
       </c>
       <c r="K65">
-        <v>290</v>
+        <v>193</v>
       </c>
       <c r="L65" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2901,7 +2901,7 @@
         <v>Passed</v>
       </c>
       <c r="K66">
-        <v>383</v>
+        <v>255</v>
       </c>
       <c r="L66" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2939,7 +2939,7 @@
         <v>Passed</v>
       </c>
       <c r="K67">
-        <v>223</v>
+        <v>314</v>
       </c>
       <c r="L67" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2977,7 +2977,7 @@
         <v>Passed</v>
       </c>
       <c r="K68">
-        <v>220</v>
+        <v>386</v>
       </c>
       <c r="L68" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3015,7 +3015,7 @@
         <v>Passed</v>
       </c>
       <c r="K69">
-        <v>384</v>
+        <v>296</v>
       </c>
       <c r="L69" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3053,7 +3053,7 @@
         <v>Passed</v>
       </c>
       <c r="K70">
-        <v>349</v>
+        <v>302</v>
       </c>
       <c r="L70" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3091,7 +3091,7 @@
         <v>Passed</v>
       </c>
       <c r="K71">
-        <v>312</v>
+        <v>176</v>
       </c>
       <c r="L71" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3129,7 +3129,7 @@
         <v>Passed</v>
       </c>
       <c r="K72">
-        <v>338</v>
+        <v>358</v>
       </c>
       <c r="L72" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3167,7 +3167,7 @@
         <v>Passed</v>
       </c>
       <c r="K73">
-        <v>231</v>
+        <v>347</v>
       </c>
       <c r="L73" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3205,7 +3205,7 @@
         <v>Passed</v>
       </c>
       <c r="K74">
-        <v>192</v>
+        <v>256</v>
       </c>
       <c r="L74" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3243,7 +3243,7 @@
         <v>Passed</v>
       </c>
       <c r="K75">
-        <v>351</v>
+        <v>287</v>
       </c>
       <c r="L75" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3281,7 +3281,7 @@
         <v>Passed</v>
       </c>
       <c r="K76">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="L76" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3319,7 +3319,7 @@
         <v>Passed</v>
       </c>
       <c r="K77">
-        <v>183</v>
+        <v>155</v>
       </c>
       <c r="L77" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3357,7 +3357,7 @@
         <v>Passed</v>
       </c>
       <c r="K78">
-        <v>304</v>
+        <v>292</v>
       </c>
       <c r="L78" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3395,7 +3395,7 @@
         <v>Passed</v>
       </c>
       <c r="K79">
-        <v>218</v>
+        <v>283</v>
       </c>
       <c r="L79" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3433,7 +3433,7 @@
         <v>Passed</v>
       </c>
       <c r="K80">
-        <v>227</v>
+        <v>169</v>
       </c>
       <c r="L80" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3471,7 +3471,7 @@
         <v>Passed</v>
       </c>
       <c r="K81">
-        <v>242</v>
+        <v>367</v>
       </c>
       <c r="L81" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3509,7 +3509,7 @@
         <v>Passed</v>
       </c>
       <c r="K82">
-        <v>295</v>
+        <v>358</v>
       </c>
       <c r="L82" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3547,7 +3547,7 @@
         <v>Passed</v>
       </c>
       <c r="K83">
-        <v>207</v>
+        <v>180</v>
       </c>
       <c r="L83" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3585,7 +3585,7 @@
         <v>Passed</v>
       </c>
       <c r="K84">
-        <v>249</v>
+        <v>292</v>
       </c>
       <c r="L84" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3661,7 +3661,7 @@
         <v>Passed</v>
       </c>
       <c r="K86">
-        <v>202</v>
+        <v>329</v>
       </c>
       <c r="L86" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3699,7 +3699,7 @@
         <v>Passed</v>
       </c>
       <c r="K87">
-        <v>277</v>
+        <v>227</v>
       </c>
       <c r="L87" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3737,7 +3737,7 @@
         <v>Passed</v>
       </c>
       <c r="K88">
-        <v>333</v>
+        <v>250</v>
       </c>
       <c r="L88" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3775,7 +3775,7 @@
         <v>Passed</v>
       </c>
       <c r="K89">
-        <v>317</v>
+        <v>300</v>
       </c>
       <c r="L89" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3813,7 +3813,7 @@
         <v>Passed</v>
       </c>
       <c r="K90">
-        <v>334</v>
+        <v>290</v>
       </c>
       <c r="L90" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3851,7 +3851,7 @@
         <v>Passed</v>
       </c>
       <c r="K91">
-        <v>281</v>
+        <v>182</v>
       </c>
       <c r="L91" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3889,7 +3889,7 @@
         <v>Passed</v>
       </c>
       <c r="K92">
-        <v>165</v>
+        <v>354</v>
       </c>
       <c r="L92" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3927,7 +3927,7 @@
         <v>Passed</v>
       </c>
       <c r="K93">
-        <v>330</v>
+        <v>383</v>
       </c>
       <c r="L93" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3965,7 +3965,7 @@
         <v>Passed</v>
       </c>
       <c r="K94">
-        <v>349</v>
+        <v>344</v>
       </c>
       <c r="L94" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4003,7 +4003,7 @@
         <v>Passed</v>
       </c>
       <c r="K95">
-        <v>371</v>
+        <v>193</v>
       </c>
       <c r="L95" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4041,7 +4041,7 @@
         <v>Passed</v>
       </c>
       <c r="K96">
-        <v>300</v>
+        <v>354</v>
       </c>
       <c r="L96" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4079,7 +4079,7 @@
         <v>Passed</v>
       </c>
       <c r="K97">
-        <v>387</v>
+        <v>251</v>
       </c>
       <c r="L97" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4117,7 +4117,7 @@
         <v>Passed</v>
       </c>
       <c r="K98">
-        <v>176</v>
+        <v>286</v>
       </c>
       <c r="L98" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4155,7 +4155,7 @@
         <v>Passed</v>
       </c>
       <c r="K99">
-        <v>310</v>
+        <v>181</v>
       </c>
       <c r="L99" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4193,7 +4193,7 @@
         <v>Passed</v>
       </c>
       <c r="K100">
-        <v>269</v>
+        <v>216</v>
       </c>
       <c r="L100" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4231,7 +4231,7 @@
         <v>Passed</v>
       </c>
       <c r="K101">
-        <v>293</v>
+        <v>223</v>
       </c>
       <c r="L101" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4269,7 +4269,7 @@
         <v>Passed</v>
       </c>
       <c r="K102">
-        <v>371</v>
+        <v>212</v>
       </c>
       <c r="L102" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4307,7 +4307,7 @@
         <v>Passed</v>
       </c>
       <c r="K103">
-        <v>270</v>
+        <v>374</v>
       </c>
       <c r="L103" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4345,7 +4345,7 @@
         <v>Passed</v>
       </c>
       <c r="K104">
-        <v>174</v>
+        <v>371</v>
       </c>
       <c r="L104" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4383,7 +4383,7 @@
         <v>Passed</v>
       </c>
       <c r="K105">
-        <v>310</v>
+        <v>296</v>
       </c>
       <c r="L105" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4421,7 +4421,7 @@
         <v>Passed</v>
       </c>
       <c r="K106">
-        <v>268</v>
+        <v>294</v>
       </c>
       <c r="L106" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4459,7 +4459,7 @@
         <v>Passed</v>
       </c>
       <c r="K107">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="L107" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4497,7 +4497,7 @@
         <v>Passed</v>
       </c>
       <c r="K108">
-        <v>238</v>
+        <v>394</v>
       </c>
       <c r="L108" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4535,7 +4535,7 @@
         <v>Passed</v>
       </c>
       <c r="K109">
-        <v>298</v>
+        <v>350</v>
       </c>
       <c r="L109" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4573,7 +4573,7 @@
         <v>Passed</v>
       </c>
       <c r="K110">
-        <v>280</v>
+        <v>175</v>
       </c>
       <c r="L110" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4611,7 +4611,7 @@
         <v>Passed</v>
       </c>
       <c r="K111">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="L111" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4649,7 +4649,7 @@
         <v>Passed</v>
       </c>
       <c r="K112">
-        <v>182</v>
+        <v>240</v>
       </c>
       <c r="L112" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4687,7 +4687,7 @@
         <v>Passed</v>
       </c>
       <c r="K113">
-        <v>218</v>
+        <v>178</v>
       </c>
       <c r="L113" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4725,7 +4725,7 @@
         <v>Passed</v>
       </c>
       <c r="K114">
-        <v>169</v>
+        <v>153</v>
       </c>
       <c r="L114" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4763,7 +4763,7 @@
         <v>Passed</v>
       </c>
       <c r="K115">
-        <v>370</v>
+        <v>249</v>
       </c>
       <c r="L115" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4801,7 +4801,7 @@
         <v>Passed</v>
       </c>
       <c r="K116">
-        <v>301</v>
+        <v>340</v>
       </c>
       <c r="L116" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4839,7 +4839,7 @@
         <v>Passed</v>
       </c>
       <c r="K117">
-        <v>369</v>
+        <v>164</v>
       </c>
       <c r="L117" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4877,7 +4877,7 @@
         <v>Passed</v>
       </c>
       <c r="K118">
-        <v>279</v>
+        <v>151</v>
       </c>
       <c r="L118" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4915,7 +4915,7 @@
         <v>Passed</v>
       </c>
       <c r="K119">
-        <v>370</v>
+        <v>212</v>
       </c>
       <c r="L119" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4953,7 +4953,7 @@
         <v>Passed</v>
       </c>
       <c r="K120">
-        <v>188</v>
+        <v>161</v>
       </c>
       <c r="L120" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4991,7 +4991,7 @@
         <v>Passed</v>
       </c>
       <c r="K121">
-        <v>159</v>
+        <v>290</v>
       </c>
       <c r="L121" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5029,7 +5029,7 @@
         <v>Passed</v>
       </c>
       <c r="K122">
-        <v>272</v>
+        <v>391</v>
       </c>
       <c r="L122" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5067,7 +5067,7 @@
         <v>Passed</v>
       </c>
       <c r="K123">
-        <v>218</v>
+        <v>321</v>
       </c>
       <c r="L123" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5105,7 +5105,7 @@
         <v>Passed</v>
       </c>
       <c r="K124">
-        <v>162</v>
+        <v>175</v>
       </c>
       <c r="L124" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5143,7 +5143,7 @@
         <v>Passed</v>
       </c>
       <c r="K125">
-        <v>245</v>
+        <v>218</v>
       </c>
       <c r="L125" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5181,7 +5181,7 @@
         <v>Passed</v>
       </c>
       <c r="K126">
-        <v>390</v>
+        <v>363</v>
       </c>
       <c r="L126" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5219,7 +5219,7 @@
         <v>Passed</v>
       </c>
       <c r="K127">
-        <v>172</v>
+        <v>315</v>
       </c>
       <c r="L127" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5257,7 +5257,7 @@
         <v>Passed</v>
       </c>
       <c r="K128">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="L128" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5295,7 +5295,7 @@
         <v>Passed</v>
       </c>
       <c r="K129">
-        <v>209</v>
+        <v>343</v>
       </c>
       <c r="L129" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5333,7 +5333,7 @@
         <v>Passed</v>
       </c>
       <c r="K130">
-        <v>179</v>
+        <v>371</v>
       </c>
       <c r="L130" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5371,7 +5371,7 @@
         <v>Passed</v>
       </c>
       <c r="K131">
-        <v>178</v>
+        <v>153</v>
       </c>
       <c r="L131" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5409,7 +5409,7 @@
         <v>Passed</v>
       </c>
       <c r="K132">
-        <v>397</v>
+        <v>234</v>
       </c>
       <c r="L132" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5447,7 +5447,7 @@
         <v>Passed</v>
       </c>
       <c r="K133">
-        <v>394</v>
+        <v>258</v>
       </c>
       <c r="L133" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5485,7 +5485,7 @@
         <v>Passed</v>
       </c>
       <c r="K134">
-        <v>242</v>
+        <v>341</v>
       </c>
       <c r="L134" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5523,7 +5523,7 @@
         <v>Passed</v>
       </c>
       <c r="K135">
-        <v>368</v>
+        <v>331</v>
       </c>
       <c r="L135" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5561,7 +5561,7 @@
         <v>Passed</v>
       </c>
       <c r="K136">
-        <v>354</v>
+        <v>265</v>
       </c>
       <c r="L136" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5599,7 +5599,7 @@
         <v>Passed</v>
       </c>
       <c r="K137">
-        <v>353</v>
+        <v>241</v>
       </c>
       <c r="L137" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5637,7 +5637,7 @@
         <v>Passed</v>
       </c>
       <c r="K138">
-        <v>268</v>
+        <v>300</v>
       </c>
       <c r="L138" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5675,7 +5675,7 @@
         <v>Passed</v>
       </c>
       <c r="K139">
-        <v>256</v>
+        <v>281</v>
       </c>
       <c r="L139" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5713,7 +5713,7 @@
         <v>Passed</v>
       </c>
       <c r="K140">
-        <v>304</v>
+        <v>236</v>
       </c>
       <c r="L140" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5751,7 +5751,7 @@
         <v>Passed</v>
       </c>
       <c r="K141">
-        <v>157</v>
+        <v>379</v>
       </c>
       <c r="L141" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5789,7 +5789,7 @@
         <v>Passed</v>
       </c>
       <c r="K142">
-        <v>251</v>
+        <v>205</v>
       </c>
       <c r="L142" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5827,7 +5827,7 @@
         <v>Passed</v>
       </c>
       <c r="K143">
-        <v>195</v>
+        <v>318</v>
       </c>
       <c r="L143" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5865,7 +5865,7 @@
         <v>Passed</v>
       </c>
       <c r="K144">
-        <v>271</v>
+        <v>364</v>
       </c>
       <c r="L144" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5903,7 +5903,7 @@
         <v>Passed</v>
       </c>
       <c r="K145">
-        <v>381</v>
+        <v>264</v>
       </c>
       <c r="L145" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5941,7 +5941,7 @@
         <v>Passed</v>
       </c>
       <c r="K146">
-        <v>191</v>
+        <v>209</v>
       </c>
       <c r="L146" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5979,7 +5979,7 @@
         <v>Passed</v>
       </c>
       <c r="K147">
-        <v>181</v>
+        <v>293</v>
       </c>
       <c r="L147" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6017,7 +6017,7 @@
         <v>Passed</v>
       </c>
       <c r="K148">
-        <v>254</v>
+        <v>202</v>
       </c>
       <c r="L148" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6055,7 +6055,7 @@
         <v>Passed</v>
       </c>
       <c r="K149">
-        <v>150</v>
+        <v>281</v>
       </c>
       <c r="L149" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6093,7 +6093,7 @@
         <v>Passed</v>
       </c>
       <c r="K150">
-        <v>228</v>
+        <v>257</v>
       </c>
       <c r="L150" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6131,7 +6131,7 @@
         <v>Passed</v>
       </c>
       <c r="K151">
-        <v>353</v>
+        <v>377</v>
       </c>
       <c r="L151" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6169,7 +6169,7 @@
         <v>Passed</v>
       </c>
       <c r="K152">
-        <v>352</v>
+        <v>276</v>
       </c>
       <c r="L152" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6207,7 +6207,7 @@
         <v>Passed</v>
       </c>
       <c r="K153">
-        <v>197</v>
+        <v>245</v>
       </c>
       <c r="L153" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6245,7 +6245,7 @@
         <v>Passed</v>
       </c>
       <c r="K154">
-        <v>198</v>
+        <v>263</v>
       </c>
       <c r="L154" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6283,7 +6283,7 @@
         <v>Passed</v>
       </c>
       <c r="K155">
-        <v>161</v>
+        <v>334</v>
       </c>
       <c r="L155" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6321,7 +6321,7 @@
         <v>Passed</v>
       </c>
       <c r="K156">
-        <v>283</v>
+        <v>304</v>
       </c>
       <c r="L156" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6359,7 +6359,7 @@
         <v>Passed</v>
       </c>
       <c r="K157">
-        <v>252</v>
+        <v>258</v>
       </c>
       <c r="L157" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6397,7 +6397,7 @@
         <v>Passed</v>
       </c>
       <c r="K158">
-        <v>238</v>
+        <v>299</v>
       </c>
       <c r="L158" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6435,7 +6435,7 @@
         <v>Passed</v>
       </c>
       <c r="K159">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="L159" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6473,7 +6473,7 @@
         <v>Passed</v>
       </c>
       <c r="K160">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="L160" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6511,7 +6511,7 @@
         <v>Passed</v>
       </c>
       <c r="K161">
-        <v>267</v>
+        <v>380</v>
       </c>
       <c r="L161" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6549,7 +6549,7 @@
         <v>Passed</v>
       </c>
       <c r="K162">
-        <v>297</v>
+        <v>387</v>
       </c>
       <c r="L162" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6587,7 +6587,7 @@
         <v>Passed</v>
       </c>
       <c r="K163">
-        <v>366</v>
+        <v>297</v>
       </c>
       <c r="L163" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6625,7 +6625,7 @@
         <v>Passed</v>
       </c>
       <c r="K164">
-        <v>279</v>
+        <v>373</v>
       </c>
       <c r="L164" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6663,7 +6663,7 @@
         <v>Passed</v>
       </c>
       <c r="K165">
-        <v>252</v>
+        <v>355</v>
       </c>
       <c r="L165" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6701,7 +6701,7 @@
         <v>Passed</v>
       </c>
       <c r="K166">
-        <v>367</v>
+        <v>238</v>
       </c>
       <c r="L166" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6739,7 +6739,7 @@
         <v>Passed</v>
       </c>
       <c r="K167">
-        <v>273</v>
+        <v>189</v>
       </c>
       <c r="L167" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6777,7 +6777,7 @@
         <v>Passed</v>
       </c>
       <c r="K168">
-        <v>208</v>
+        <v>263</v>
       </c>
       <c r="L168" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6815,7 +6815,7 @@
         <v>Passed</v>
       </c>
       <c r="K169">
-        <v>334</v>
+        <v>338</v>
       </c>
       <c r="L169" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6853,7 +6853,7 @@
         <v>Passed</v>
       </c>
       <c r="K170">
-        <v>313</v>
+        <v>343</v>
       </c>
       <c r="L170" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6891,7 +6891,7 @@
         <v>Passed</v>
       </c>
       <c r="K171">
-        <v>375</v>
+        <v>367</v>
       </c>
       <c r="L171" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6929,7 +6929,7 @@
         <v>Passed</v>
       </c>
       <c r="K172">
-        <v>188</v>
+        <v>163</v>
       </c>
       <c r="L172" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6967,7 +6967,7 @@
         <v>Passed</v>
       </c>
       <c r="K173">
-        <v>222</v>
+        <v>329</v>
       </c>
       <c r="L173" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7005,7 +7005,7 @@
         <v>Passed</v>
       </c>
       <c r="K174">
-        <v>297</v>
+        <v>314</v>
       </c>
       <c r="L174" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7043,7 +7043,7 @@
         <v>Passed</v>
       </c>
       <c r="K175">
-        <v>199</v>
+        <v>348</v>
       </c>
       <c r="L175" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7081,7 +7081,7 @@
         <v>Passed</v>
       </c>
       <c r="K176">
-        <v>285</v>
+        <v>388</v>
       </c>
       <c r="L176" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7119,7 +7119,7 @@
         <v>Passed</v>
       </c>
       <c r="K177">
-        <v>169</v>
+        <v>378</v>
       </c>
       <c r="L177" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7157,7 +7157,7 @@
         <v>Passed</v>
       </c>
       <c r="K178">
-        <v>286</v>
+        <v>367</v>
       </c>
       <c r="L178" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7195,7 +7195,7 @@
         <v>Passed</v>
       </c>
       <c r="K179">
-        <v>395</v>
+        <v>225</v>
       </c>
       <c r="L179" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7233,7 +7233,7 @@
         <v>Passed</v>
       </c>
       <c r="K180">
-        <v>348</v>
+        <v>373</v>
       </c>
       <c r="L180" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7271,7 +7271,7 @@
         <v>Passed</v>
       </c>
       <c r="K181">
-        <v>261</v>
+        <v>230</v>
       </c>
       <c r="L181" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7309,7 +7309,7 @@
         <v>Passed</v>
       </c>
       <c r="K182">
-        <v>197</v>
+        <v>250</v>
       </c>
       <c r="L182" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7347,7 +7347,7 @@
         <v>Passed</v>
       </c>
       <c r="K183">
-        <v>382</v>
+        <v>156</v>
       </c>
       <c r="L183" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7385,7 +7385,7 @@
         <v>Passed</v>
       </c>
       <c r="K184">
-        <v>164</v>
+        <v>244</v>
       </c>
       <c r="L184" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7423,7 +7423,7 @@
         <v>Passed</v>
       </c>
       <c r="K185">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="L185" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7461,7 +7461,7 @@
         <v>Passed</v>
       </c>
       <c r="K186">
-        <v>264</v>
+        <v>150</v>
       </c>
       <c r="L186" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7499,7 +7499,7 @@
         <v>Passed</v>
       </c>
       <c r="K187">
-        <v>380</v>
+        <v>281</v>
       </c>
       <c r="L187" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7537,7 +7537,7 @@
         <v>Passed</v>
       </c>
       <c r="K188">
-        <v>289</v>
+        <v>370</v>
       </c>
       <c r="L188" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7575,7 +7575,7 @@
         <v>Passed</v>
       </c>
       <c r="K189">
-        <v>345</v>
+        <v>377</v>
       </c>
       <c r="L189" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7613,7 +7613,7 @@
         <v>Passed</v>
       </c>
       <c r="K190">
-        <v>325</v>
+        <v>153</v>
       </c>
       <c r="L190" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7651,7 +7651,7 @@
         <v>Passed</v>
       </c>
       <c r="K191">
-        <v>371</v>
+        <v>380</v>
       </c>
       <c r="L191" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7689,7 +7689,7 @@
         <v>Passed</v>
       </c>
       <c r="K192">
-        <v>271</v>
+        <v>164</v>
       </c>
       <c r="L192" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7727,7 +7727,7 @@
         <v>Passed</v>
       </c>
       <c r="K193">
-        <v>150</v>
+        <v>310</v>
       </c>
       <c r="L193" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7765,7 +7765,7 @@
         <v>Passed</v>
       </c>
       <c r="K194">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="L194" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7803,7 +7803,7 @@
         <v>Passed</v>
       </c>
       <c r="K195">
-        <v>155</v>
+        <v>358</v>
       </c>
       <c r="L195" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7841,7 +7841,7 @@
         <v>Passed</v>
       </c>
       <c r="K196">
-        <v>210</v>
+        <v>231</v>
       </c>
       <c r="L196" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7879,7 +7879,7 @@
         <v>Passed</v>
       </c>
       <c r="K197">
-        <v>176</v>
+        <v>255</v>
       </c>
       <c r="L197" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7917,7 +7917,7 @@
         <v>Passed</v>
       </c>
       <c r="K198">
-        <v>279</v>
+        <v>162</v>
       </c>
       <c r="L198" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7955,7 +7955,7 @@
         <v>Passed</v>
       </c>
       <c r="K199">
-        <v>281</v>
+        <v>310</v>
       </c>
       <c r="L199" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7993,7 +7993,7 @@
         <v>Passed</v>
       </c>
       <c r="K200">
-        <v>174</v>
+        <v>249</v>
       </c>
       <c r="L200" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8031,7 +8031,7 @@
         <v>Passed</v>
       </c>
       <c r="K201">
-        <v>398</v>
+        <v>273</v>
       </c>
       <c r="L201" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8069,7 +8069,7 @@
         <v>Passed</v>
       </c>
       <c r="K202">
-        <v>366</v>
+        <v>314</v>
       </c>
       <c r="L202" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8107,7 +8107,7 @@
         <v>Passed</v>
       </c>
       <c r="K203">
-        <v>171</v>
+        <v>150</v>
       </c>
       <c r="L203" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8145,7 +8145,7 @@
         <v>Passed</v>
       </c>
       <c r="K204">
-        <v>192</v>
+        <v>395</v>
       </c>
       <c r="L204" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8183,7 +8183,7 @@
         <v>Passed</v>
       </c>
       <c r="K205">
-        <v>359</v>
+        <v>208</v>
       </c>
       <c r="L205" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8221,7 +8221,7 @@
         <v>Passed</v>
       </c>
       <c r="K206">
-        <v>264</v>
+        <v>287</v>
       </c>
       <c r="L206" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8259,7 +8259,7 @@
         <v>Passed</v>
       </c>
       <c r="K207">
-        <v>274</v>
+        <v>336</v>
       </c>
       <c r="L207" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8297,7 +8297,7 @@
         <v>Passed</v>
       </c>
       <c r="K208">
-        <v>297</v>
+        <v>261</v>
       </c>
       <c r="L208" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8335,7 +8335,7 @@
         <v>Passed</v>
       </c>
       <c r="K209">
-        <v>208</v>
+        <v>379</v>
       </c>
       <c r="L209" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8373,7 +8373,7 @@
         <v>Passed</v>
       </c>
       <c r="K210">
-        <v>172</v>
+        <v>190</v>
       </c>
       <c r="L210" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8411,7 +8411,7 @@
         <v>Passed</v>
       </c>
       <c r="K211">
-        <v>310</v>
+        <v>269</v>
       </c>
       <c r="L211" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8449,7 +8449,7 @@
         <v>Passed</v>
       </c>
       <c r="K212">
-        <v>335</v>
+        <v>245</v>
       </c>
       <c r="L212" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8487,7 +8487,7 @@
         <v>Passed</v>
       </c>
       <c r="K213">
-        <v>161</v>
+        <v>289</v>
       </c>
       <c r="L213" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8525,7 +8525,7 @@
         <v>Passed</v>
       </c>
       <c r="K214">
-        <v>288</v>
+        <v>230</v>
       </c>
       <c r="L214" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8563,7 +8563,7 @@
         <v>Passed</v>
       </c>
       <c r="K215">
-        <v>257</v>
+        <v>318</v>
       </c>
       <c r="L215" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8601,7 +8601,7 @@
         <v>Passed</v>
       </c>
       <c r="K216">
-        <v>257</v>
+        <v>278</v>
       </c>
       <c r="L216" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8639,7 +8639,7 @@
         <v>Passed</v>
       </c>
       <c r="K217">
-        <v>328</v>
+        <v>350</v>
       </c>
       <c r="L217" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8677,7 +8677,7 @@
         <v>Passed</v>
       </c>
       <c r="K218">
-        <v>156</v>
+        <v>246</v>
       </c>
       <c r="L218" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8715,7 +8715,7 @@
         <v>Passed</v>
       </c>
       <c r="K219">
-        <v>288</v>
+        <v>389</v>
       </c>
       <c r="L219" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8753,7 +8753,7 @@
         <v>Passed</v>
       </c>
       <c r="K220">
-        <v>250</v>
+        <v>309</v>
       </c>
       <c r="L220" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8791,7 +8791,7 @@
         <v>Passed</v>
       </c>
       <c r="K221">
-        <v>246</v>
+        <v>191</v>
       </c>
       <c r="L221" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8829,7 +8829,7 @@
         <v>Passed</v>
       </c>
       <c r="K222">
-        <v>311</v>
+        <v>152</v>
       </c>
       <c r="L222" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8867,7 +8867,7 @@
         <v>Passed</v>
       </c>
       <c r="K223">
-        <v>208</v>
+        <v>259</v>
       </c>
       <c r="L223" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8905,7 +8905,7 @@
         <v>Passed</v>
       </c>
       <c r="K224">
-        <v>257</v>
+        <v>348</v>
       </c>
       <c r="L224" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8943,7 +8943,7 @@
         <v>Passed</v>
       </c>
       <c r="K225">
-        <v>351</v>
+        <v>313</v>
       </c>
       <c r="L225" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8981,7 +8981,7 @@
         <v>Passed</v>
       </c>
       <c r="K226">
-        <v>390</v>
+        <v>369</v>
       </c>
       <c r="L226" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9019,7 +9019,7 @@
         <v>Passed</v>
       </c>
       <c r="K227">
-        <v>175</v>
+        <v>198</v>
       </c>
       <c r="L227" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9057,7 +9057,7 @@
         <v>Passed</v>
       </c>
       <c r="K228">
-        <v>162</v>
+        <v>229</v>
       </c>
       <c r="L228" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9095,7 +9095,7 @@
         <v>Passed</v>
       </c>
       <c r="K229">
-        <v>209</v>
+        <v>322</v>
       </c>
       <c r="L229" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9133,7 +9133,7 @@
         <v>Passed</v>
       </c>
       <c r="K230">
-        <v>266</v>
+        <v>180</v>
       </c>
       <c r="L230" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9171,7 +9171,7 @@
         <v>Passed</v>
       </c>
       <c r="K231">
-        <v>169</v>
+        <v>332</v>
       </c>
       <c r="L231" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9209,7 +9209,7 @@
         <v>Passed</v>
       </c>
       <c r="K232">
-        <v>256</v>
+        <v>329</v>
       </c>
       <c r="L232" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9247,7 +9247,7 @@
         <v>Passed</v>
       </c>
       <c r="K233">
-        <v>282</v>
+        <v>170</v>
       </c>
       <c r="L233" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9285,7 +9285,7 @@
         <v>Passed</v>
       </c>
       <c r="K234">
-        <v>278</v>
+        <v>169</v>
       </c>
       <c r="L234" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9323,7 +9323,7 @@
         <v>Passed</v>
       </c>
       <c r="K235">
-        <v>296</v>
+        <v>240</v>
       </c>
       <c r="L235" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9361,7 +9361,7 @@
         <v>Passed</v>
       </c>
       <c r="K236">
-        <v>343</v>
+        <v>281</v>
       </c>
       <c r="L236" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9399,7 +9399,7 @@
         <v>Passed</v>
       </c>
       <c r="K237">
-        <v>213</v>
+        <v>312</v>
       </c>
       <c r="L237" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9437,7 +9437,7 @@
         <v>Passed</v>
       </c>
       <c r="K238">
-        <v>358</v>
+        <v>197</v>
       </c>
       <c r="L238" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9475,7 +9475,7 @@
         <v>Passed</v>
       </c>
       <c r="K239">
-        <v>151</v>
+        <v>335</v>
       </c>
       <c r="L239" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9513,7 +9513,7 @@
         <v>Passed</v>
       </c>
       <c r="K240">
-        <v>365</v>
+        <v>340</v>
       </c>
       <c r="L240" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9551,7 +9551,7 @@
         <v>Passed</v>
       </c>
       <c r="K241">
-        <v>273</v>
+        <v>193</v>
       </c>
       <c r="L241" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9589,7 +9589,7 @@
         <v>Passed</v>
       </c>
       <c r="K242">
-        <v>360</v>
+        <v>324</v>
       </c>
       <c r="L242" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9627,7 +9627,7 @@
         <v>Passed</v>
       </c>
       <c r="K243">
-        <v>255</v>
+        <v>319</v>
       </c>
       <c r="L243" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9665,7 +9665,7 @@
         <v>Passed</v>
       </c>
       <c r="K244">
-        <v>363</v>
+        <v>253</v>
       </c>
       <c r="L244" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9703,7 +9703,7 @@
         <v>Passed</v>
       </c>
       <c r="K245">
-        <v>349</v>
+        <v>326</v>
       </c>
       <c r="L245" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9741,7 +9741,7 @@
         <v>Passed</v>
       </c>
       <c r="K246">
-        <v>360</v>
+        <v>367</v>
       </c>
       <c r="L246" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9779,7 +9779,7 @@
         <v>Passed</v>
       </c>
       <c r="K247">
-        <v>305</v>
+        <v>244</v>
       </c>
       <c r="L247" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9817,7 +9817,7 @@
         <v>Passed</v>
       </c>
       <c r="K248">
-        <v>155</v>
+        <v>252</v>
       </c>
       <c r="L248" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9855,7 +9855,7 @@
         <v>Passed</v>
       </c>
       <c r="K249">
-        <v>233</v>
+        <v>397</v>
       </c>
       <c r="L249" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9893,7 +9893,7 @@
         <v>Passed</v>
       </c>
       <c r="K250">
-        <v>380</v>
+        <v>249</v>
       </c>
       <c r="L250" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9931,7 +9931,7 @@
         <v>Passed</v>
       </c>
       <c r="K251">
-        <v>335</v>
+        <v>328</v>
       </c>
       <c r="L251" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9969,7 +9969,7 @@
         <v>Passed</v>
       </c>
       <c r="K252">
-        <v>315</v>
+        <v>184</v>
       </c>
       <c r="L252" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10007,7 +10007,7 @@
         <v>Passed</v>
       </c>
       <c r="K253">
-        <v>198</v>
+        <v>321</v>
       </c>
       <c r="L253" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10045,7 +10045,7 @@
         <v>Passed</v>
       </c>
       <c r="K254">
-        <v>270</v>
+        <v>250</v>
       </c>
       <c r="L254" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10083,7 +10083,7 @@
         <v>Passed</v>
       </c>
       <c r="K255">
-        <v>252</v>
+        <v>241</v>
       </c>
       <c r="L255" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10121,7 +10121,7 @@
         <v>Passed</v>
       </c>
       <c r="K256">
-        <v>187</v>
+        <v>282</v>
       </c>
       <c r="L256" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10159,7 +10159,7 @@
         <v>Passed</v>
       </c>
       <c r="K257">
-        <v>340</v>
+        <v>283</v>
       </c>
       <c r="L257" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10197,7 +10197,7 @@
         <v>Passed</v>
       </c>
       <c r="K258">
-        <v>264</v>
+        <v>336</v>
       </c>
       <c r="L258" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10235,7 +10235,7 @@
         <v>Passed</v>
       </c>
       <c r="K259">
-        <v>159</v>
+        <v>150</v>
       </c>
       <c r="L259" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10273,7 +10273,7 @@
         <v>Passed</v>
       </c>
       <c r="K260">
-        <v>308</v>
+        <v>168</v>
       </c>
       <c r="L260" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10311,7 +10311,7 @@
         <v>Passed</v>
       </c>
       <c r="K261">
-        <v>343</v>
+        <v>163</v>
       </c>
       <c r="L261" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10349,7 +10349,7 @@
         <v>Passed</v>
       </c>
       <c r="K262">
-        <v>152</v>
+        <v>177</v>
       </c>
       <c r="L262" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10387,7 +10387,7 @@
         <v>Passed</v>
       </c>
       <c r="K263">
-        <v>162</v>
+        <v>308</v>
       </c>
       <c r="L263" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10425,7 +10425,7 @@
         <v>Passed</v>
       </c>
       <c r="K264">
-        <v>378</v>
+        <v>289</v>
       </c>
       <c r="L264" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10463,7 +10463,7 @@
         <v>Passed</v>
       </c>
       <c r="K265">
-        <v>174</v>
+        <v>275</v>
       </c>
       <c r="L265" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10501,7 +10501,7 @@
         <v>Passed</v>
       </c>
       <c r="K266">
-        <v>398</v>
+        <v>352</v>
       </c>
       <c r="L266" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10539,7 +10539,7 @@
         <v>Passed</v>
       </c>
       <c r="K267">
-        <v>268</v>
+        <v>227</v>
       </c>
       <c r="L267" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10577,7 +10577,7 @@
         <v>Passed</v>
       </c>
       <c r="K268">
-        <v>150</v>
+        <v>225</v>
       </c>
       <c r="L268" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10615,7 +10615,7 @@
         <v>Passed</v>
       </c>
       <c r="K269">
-        <v>183</v>
+        <v>254</v>
       </c>
       <c r="L269" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10653,7 +10653,7 @@
         <v>Passed</v>
       </c>
       <c r="K270">
-        <v>359</v>
+        <v>383</v>
       </c>
       <c r="L270" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10691,7 +10691,7 @@
         <v>Passed</v>
       </c>
       <c r="K271">
-        <v>233</v>
+        <v>156</v>
       </c>
       <c r="L271" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10729,7 +10729,7 @@
         <v>Passed</v>
       </c>
       <c r="K272">
-        <v>228</v>
+        <v>335</v>
       </c>
       <c r="L272" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10767,7 +10767,7 @@
         <v>Passed</v>
       </c>
       <c r="K273">
-        <v>389</v>
+        <v>309</v>
       </c>
       <c r="L273" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10805,7 +10805,7 @@
         <v>Passed</v>
       </c>
       <c r="K274">
-        <v>156</v>
+        <v>219</v>
       </c>
       <c r="L274" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10843,7 +10843,7 @@
         <v>Passed</v>
       </c>
       <c r="K275">
-        <v>321</v>
+        <v>268</v>
       </c>
       <c r="L275" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10881,7 +10881,7 @@
         <v>Passed</v>
       </c>
       <c r="K276">
-        <v>231</v>
+        <v>216</v>
       </c>
       <c r="L276" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10919,7 +10919,7 @@
         <v>Passed</v>
       </c>
       <c r="K277">
-        <v>160</v>
+        <v>299</v>
       </c>
       <c r="L277" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10957,7 +10957,7 @@
         <v>Passed</v>
       </c>
       <c r="K278">
-        <v>399</v>
+        <v>203</v>
       </c>
       <c r="L278" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10995,7 +10995,7 @@
         <v>Passed</v>
       </c>
       <c r="K279">
-        <v>245</v>
+        <v>392</v>
       </c>
       <c r="L279" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11033,7 +11033,7 @@
         <v>Passed</v>
       </c>
       <c r="K280">
-        <v>176</v>
+        <v>235</v>
       </c>
       <c r="L280" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11071,7 +11071,7 @@
         <v>Passed</v>
       </c>
       <c r="K281">
-        <v>261</v>
+        <v>286</v>
       </c>
       <c r="L281" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11109,7 +11109,7 @@
         <v>Passed</v>
       </c>
       <c r="K282">
-        <v>319</v>
+        <v>240</v>
       </c>
       <c r="L282" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11147,7 +11147,7 @@
         <v>Passed</v>
       </c>
       <c r="K283">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="L283" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11185,7 +11185,7 @@
         <v>Passed</v>
       </c>
       <c r="K284">
-        <v>369</v>
+        <v>172</v>
       </c>
       <c r="L284" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11223,7 +11223,7 @@
         <v>Passed</v>
       </c>
       <c r="K285">
-        <v>253</v>
+        <v>355</v>
       </c>
       <c r="L285" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11261,7 +11261,7 @@
         <v>Passed</v>
       </c>
       <c r="K286">
-        <v>194</v>
+        <v>370</v>
       </c>
       <c r="L286" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11299,7 +11299,7 @@
         <v>Passed</v>
       </c>
       <c r="K287">
-        <v>225</v>
+        <v>298</v>
       </c>
       <c r="L287" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11337,7 +11337,7 @@
         <v>Passed</v>
       </c>
       <c r="K288">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="L288" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11375,7 +11375,7 @@
         <v>Passed</v>
       </c>
       <c r="K289">
-        <v>165</v>
+        <v>341</v>
       </c>
       <c r="L289" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11413,7 +11413,7 @@
         <v>Passed</v>
       </c>
       <c r="K290">
-        <v>383</v>
+        <v>331</v>
       </c>
       <c r="L290" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11451,7 +11451,7 @@
         <v>Passed</v>
       </c>
       <c r="K291">
-        <v>211</v>
+        <v>386</v>
       </c>
       <c r="L291" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11489,7 +11489,7 @@
         <v>Passed</v>
       </c>
       <c r="K292">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="L292" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11527,7 +11527,7 @@
         <v>Passed</v>
       </c>
       <c r="K293">
-        <v>230</v>
+        <v>159</v>
       </c>
       <c r="L293" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11565,7 +11565,7 @@
         <v>Passed</v>
       </c>
       <c r="K294">
-        <v>314</v>
+        <v>262</v>
       </c>
       <c r="L294" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11603,7 +11603,7 @@
         <v>Passed</v>
       </c>
       <c r="K295">
-        <v>321</v>
+        <v>211</v>
       </c>
       <c r="L295" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11641,7 +11641,7 @@
         <v>Passed</v>
       </c>
       <c r="K296">
-        <v>248</v>
+        <v>384</v>
       </c>
       <c r="L296" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11679,7 +11679,7 @@
         <v>Passed</v>
       </c>
       <c r="K297">
-        <v>394</v>
+        <v>311</v>
       </c>
       <c r="L297" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11717,7 +11717,7 @@
         <v>Passed</v>
       </c>
       <c r="K298">
-        <v>246</v>
+        <v>240</v>
       </c>
       <c r="L298" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11755,7 +11755,7 @@
         <v>Passed</v>
       </c>
       <c r="K299">
-        <v>167</v>
+        <v>219</v>
       </c>
       <c r="L299" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11793,7 +11793,7 @@
         <v>Passed</v>
       </c>
       <c r="K300">
-        <v>159</v>
+        <v>331</v>
       </c>
       <c r="L300" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11831,7 +11831,7 @@
         <v>Passed</v>
       </c>
       <c r="K301">
-        <v>309</v>
+        <v>244</v>
       </c>
       <c r="L301" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>

</xml_diff>

<commit_message>
feat: persist selected seats in registrations on payment success to render them in red
</commit_message>
<xml_diff>
--- a/EventSphere_Appium_Mobile_300_Report.xlsx
+++ b/EventSphere_Appium_Mobile_300_Report.xlsx
@@ -469,7 +469,7 @@
         <v>Passed</v>
       </c>
       <c r="K2">
-        <v>222</v>
+        <v>272</v>
       </c>
       <c r="L2" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -507,7 +507,7 @@
         <v>Passed</v>
       </c>
       <c r="K3">
-        <v>168</v>
+        <v>293</v>
       </c>
       <c r="L3" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -545,7 +545,7 @@
         <v>Passed</v>
       </c>
       <c r="K4">
-        <v>384</v>
+        <v>171</v>
       </c>
       <c r="L4" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -583,7 +583,7 @@
         <v>Passed</v>
       </c>
       <c r="K5">
-        <v>301</v>
+        <v>234</v>
       </c>
       <c r="L5" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -621,7 +621,7 @@
         <v>Passed</v>
       </c>
       <c r="K6">
-        <v>303</v>
+        <v>324</v>
       </c>
       <c r="L6" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -659,7 +659,7 @@
         <v>Passed</v>
       </c>
       <c r="K7">
-        <v>334</v>
+        <v>294</v>
       </c>
       <c r="L7" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -697,7 +697,7 @@
         <v>Passed</v>
       </c>
       <c r="K8">
-        <v>219</v>
+        <v>231</v>
       </c>
       <c r="L8" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -735,7 +735,7 @@
         <v>Passed</v>
       </c>
       <c r="K9">
-        <v>169</v>
+        <v>300</v>
       </c>
       <c r="L9" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -773,7 +773,7 @@
         <v>Passed</v>
       </c>
       <c r="K10">
-        <v>190</v>
+        <v>389</v>
       </c>
       <c r="L10" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -811,7 +811,7 @@
         <v>Passed</v>
       </c>
       <c r="K11">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="L11" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -849,7 +849,7 @@
         <v>Passed</v>
       </c>
       <c r="K12">
-        <v>170</v>
+        <v>324</v>
       </c>
       <c r="L12" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -887,7 +887,7 @@
         <v>Passed</v>
       </c>
       <c r="K13">
-        <v>310</v>
+        <v>358</v>
       </c>
       <c r="L13" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -925,7 +925,7 @@
         <v>Passed</v>
       </c>
       <c r="K14">
-        <v>288</v>
+        <v>340</v>
       </c>
       <c r="L14" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -963,7 +963,7 @@
         <v>Passed</v>
       </c>
       <c r="K15">
-        <v>182</v>
+        <v>296</v>
       </c>
       <c r="L15" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1001,7 +1001,7 @@
         <v>Passed</v>
       </c>
       <c r="K16">
-        <v>242</v>
+        <v>358</v>
       </c>
       <c r="L16" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1039,7 +1039,7 @@
         <v>Passed</v>
       </c>
       <c r="K17">
-        <v>377</v>
+        <v>346</v>
       </c>
       <c r="L17" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1077,7 +1077,7 @@
         <v>Passed</v>
       </c>
       <c r="K18">
-        <v>390</v>
+        <v>233</v>
       </c>
       <c r="L18" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1115,7 +1115,7 @@
         <v>Passed</v>
       </c>
       <c r="K19">
-        <v>244</v>
+        <v>360</v>
       </c>
       <c r="L19" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1153,7 +1153,7 @@
         <v>Passed</v>
       </c>
       <c r="K20">
-        <v>340</v>
+        <v>179</v>
       </c>
       <c r="L20" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1191,7 +1191,7 @@
         <v>Passed</v>
       </c>
       <c r="K21">
-        <v>250</v>
+        <v>373</v>
       </c>
       <c r="L21" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1229,7 +1229,7 @@
         <v>Passed</v>
       </c>
       <c r="K22">
-        <v>275</v>
+        <v>158</v>
       </c>
       <c r="L22" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1267,7 +1267,7 @@
         <v>Passed</v>
       </c>
       <c r="K23">
-        <v>170</v>
+        <v>258</v>
       </c>
       <c r="L23" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1305,7 +1305,7 @@
         <v>Passed</v>
       </c>
       <c r="K24">
-        <v>270</v>
+        <v>261</v>
       </c>
       <c r="L24" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1343,7 +1343,7 @@
         <v>Passed</v>
       </c>
       <c r="K25">
-        <v>234</v>
+        <v>175</v>
       </c>
       <c r="L25" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1381,7 +1381,7 @@
         <v>Passed</v>
       </c>
       <c r="K26">
-        <v>164</v>
+        <v>359</v>
       </c>
       <c r="L26" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1419,7 +1419,7 @@
         <v>Passed</v>
       </c>
       <c r="K27">
-        <v>170</v>
+        <v>255</v>
       </c>
       <c r="L27" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1457,7 +1457,7 @@
         <v>Passed</v>
       </c>
       <c r="K28">
-        <v>350</v>
+        <v>247</v>
       </c>
       <c r="L28" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1495,7 +1495,7 @@
         <v>Passed</v>
       </c>
       <c r="K29">
-        <v>343</v>
+        <v>202</v>
       </c>
       <c r="L29" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1533,7 +1533,7 @@
         <v>Passed</v>
       </c>
       <c r="K30">
-        <v>382</v>
+        <v>175</v>
       </c>
       <c r="L30" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1571,7 +1571,7 @@
         <v>Passed</v>
       </c>
       <c r="K31">
-        <v>210</v>
+        <v>280</v>
       </c>
       <c r="L31" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1609,7 +1609,7 @@
         <v>Passed</v>
       </c>
       <c r="K32">
-        <v>276</v>
+        <v>389</v>
       </c>
       <c r="L32" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1647,7 +1647,7 @@
         <v>Passed</v>
       </c>
       <c r="K33">
-        <v>358</v>
+        <v>260</v>
       </c>
       <c r="L33" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1685,7 +1685,7 @@
         <v>Passed</v>
       </c>
       <c r="K34">
-        <v>155</v>
+        <v>183</v>
       </c>
       <c r="L34" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1723,7 +1723,7 @@
         <v>Passed</v>
       </c>
       <c r="K35">
-        <v>299</v>
+        <v>205</v>
       </c>
       <c r="L35" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1761,7 +1761,7 @@
         <v>Passed</v>
       </c>
       <c r="K36">
-        <v>334</v>
+        <v>242</v>
       </c>
       <c r="L36" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1799,7 +1799,7 @@
         <v>Passed</v>
       </c>
       <c r="K37">
-        <v>324</v>
+        <v>344</v>
       </c>
       <c r="L37" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1837,7 +1837,7 @@
         <v>Passed</v>
       </c>
       <c r="K38">
-        <v>211</v>
+        <v>224</v>
       </c>
       <c r="L38" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1875,7 +1875,7 @@
         <v>Passed</v>
       </c>
       <c r="K39">
-        <v>245</v>
+        <v>174</v>
       </c>
       <c r="L39" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1913,7 +1913,7 @@
         <v>Passed</v>
       </c>
       <c r="K40">
-        <v>393</v>
+        <v>275</v>
       </c>
       <c r="L40" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1951,7 +1951,7 @@
         <v>Passed</v>
       </c>
       <c r="K41">
-        <v>157</v>
+        <v>369</v>
       </c>
       <c r="L41" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -1989,7 +1989,7 @@
         <v>Passed</v>
       </c>
       <c r="K42">
-        <v>199</v>
+        <v>386</v>
       </c>
       <c r="L42" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2027,7 +2027,7 @@
         <v>Passed</v>
       </c>
       <c r="K43">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="L43" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2065,7 +2065,7 @@
         <v>Passed</v>
       </c>
       <c r="K44">
-        <v>218</v>
+        <v>330</v>
       </c>
       <c r="L44" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2103,7 +2103,7 @@
         <v>Passed</v>
       </c>
       <c r="K45">
-        <v>262</v>
+        <v>154</v>
       </c>
       <c r="L45" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2141,7 +2141,7 @@
         <v>Passed</v>
       </c>
       <c r="K46">
-        <v>330</v>
+        <v>251</v>
       </c>
       <c r="L46" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2179,7 +2179,7 @@
         <v>Passed</v>
       </c>
       <c r="K47">
-        <v>152</v>
+        <v>318</v>
       </c>
       <c r="L47" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2217,7 +2217,7 @@
         <v>Passed</v>
       </c>
       <c r="K48">
-        <v>334</v>
+        <v>185</v>
       </c>
       <c r="L48" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2255,7 +2255,7 @@
         <v>Passed</v>
       </c>
       <c r="K49">
-        <v>244</v>
+        <v>169</v>
       </c>
       <c r="L49" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2293,7 +2293,7 @@
         <v>Passed</v>
       </c>
       <c r="K50">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="L50" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2331,7 +2331,7 @@
         <v>Passed</v>
       </c>
       <c r="K51">
-        <v>342</v>
+        <v>279</v>
       </c>
       <c r="L51" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2369,7 +2369,7 @@
         <v>Passed</v>
       </c>
       <c r="K52">
-        <v>384</v>
+        <v>273</v>
       </c>
       <c r="L52" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2407,7 +2407,7 @@
         <v>Passed</v>
       </c>
       <c r="K53">
-        <v>377</v>
+        <v>338</v>
       </c>
       <c r="L53" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2445,7 +2445,7 @@
         <v>Passed</v>
       </c>
       <c r="K54">
-        <v>217</v>
+        <v>376</v>
       </c>
       <c r="L54" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2483,7 +2483,7 @@
         <v>Passed</v>
       </c>
       <c r="K55">
-        <v>226</v>
+        <v>339</v>
       </c>
       <c r="L55" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2521,7 +2521,7 @@
         <v>Passed</v>
       </c>
       <c r="K56">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="L56" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2559,7 +2559,7 @@
         <v>Passed</v>
       </c>
       <c r="K57">
-        <v>235</v>
+        <v>342</v>
       </c>
       <c r="L57" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2597,7 +2597,7 @@
         <v>Passed</v>
       </c>
       <c r="K58">
-        <v>206</v>
+        <v>233</v>
       </c>
       <c r="L58" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2635,7 +2635,7 @@
         <v>Passed</v>
       </c>
       <c r="K59">
-        <v>347</v>
+        <v>200</v>
       </c>
       <c r="L59" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2673,7 +2673,7 @@
         <v>Passed</v>
       </c>
       <c r="K60">
-        <v>184</v>
+        <v>243</v>
       </c>
       <c r="L60" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2711,7 +2711,7 @@
         <v>Passed</v>
       </c>
       <c r="K61">
-        <v>373</v>
+        <v>227</v>
       </c>
       <c r="L61" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2749,7 +2749,7 @@
         <v>Passed</v>
       </c>
       <c r="K62">
-        <v>173</v>
+        <v>399</v>
       </c>
       <c r="L62" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2787,7 +2787,7 @@
         <v>Passed</v>
       </c>
       <c r="K63">
-        <v>339</v>
+        <v>180</v>
       </c>
       <c r="L63" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2825,7 +2825,7 @@
         <v>Passed</v>
       </c>
       <c r="K64">
-        <v>271</v>
+        <v>187</v>
       </c>
       <c r="L64" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2863,7 +2863,7 @@
         <v>Passed</v>
       </c>
       <c r="K65">
-        <v>193</v>
+        <v>268</v>
       </c>
       <c r="L65" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2901,7 +2901,7 @@
         <v>Passed</v>
       </c>
       <c r="K66">
-        <v>255</v>
+        <v>282</v>
       </c>
       <c r="L66" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2939,7 +2939,7 @@
         <v>Passed</v>
       </c>
       <c r="K67">
-        <v>314</v>
+        <v>373</v>
       </c>
       <c r="L67" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -2977,7 +2977,7 @@
         <v>Passed</v>
       </c>
       <c r="K68">
-        <v>386</v>
+        <v>303</v>
       </c>
       <c r="L68" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3015,7 +3015,7 @@
         <v>Passed</v>
       </c>
       <c r="K69">
-        <v>296</v>
+        <v>277</v>
       </c>
       <c r="L69" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3053,7 +3053,7 @@
         <v>Passed</v>
       </c>
       <c r="K70">
-        <v>302</v>
+        <v>324</v>
       </c>
       <c r="L70" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3091,7 +3091,7 @@
         <v>Passed</v>
       </c>
       <c r="K71">
-        <v>176</v>
+        <v>317</v>
       </c>
       <c r="L71" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3129,7 +3129,7 @@
         <v>Passed</v>
       </c>
       <c r="K72">
-        <v>358</v>
+        <v>205</v>
       </c>
       <c r="L72" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3167,7 +3167,7 @@
         <v>Passed</v>
       </c>
       <c r="K73">
-        <v>347</v>
+        <v>167</v>
       </c>
       <c r="L73" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3205,7 +3205,7 @@
         <v>Passed</v>
       </c>
       <c r="K74">
-        <v>256</v>
+        <v>238</v>
       </c>
       <c r="L74" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3243,7 +3243,7 @@
         <v>Passed</v>
       </c>
       <c r="K75">
-        <v>287</v>
+        <v>335</v>
       </c>
       <c r="L75" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3281,7 +3281,7 @@
         <v>Passed</v>
       </c>
       <c r="K76">
-        <v>273</v>
+        <v>373</v>
       </c>
       <c r="L76" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3319,7 +3319,7 @@
         <v>Passed</v>
       </c>
       <c r="K77">
-        <v>155</v>
+        <v>321</v>
       </c>
       <c r="L77" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3357,7 +3357,7 @@
         <v>Passed</v>
       </c>
       <c r="K78">
-        <v>292</v>
+        <v>397</v>
       </c>
       <c r="L78" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3395,7 +3395,7 @@
         <v>Passed</v>
       </c>
       <c r="K79">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="L79" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3433,7 +3433,7 @@
         <v>Passed</v>
       </c>
       <c r="K80">
-        <v>169</v>
+        <v>217</v>
       </c>
       <c r="L80" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3471,7 +3471,7 @@
         <v>Passed</v>
       </c>
       <c r="K81">
-        <v>367</v>
+        <v>216</v>
       </c>
       <c r="L81" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3509,7 +3509,7 @@
         <v>Passed</v>
       </c>
       <c r="K82">
-        <v>358</v>
+        <v>238</v>
       </c>
       <c r="L82" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3547,7 +3547,7 @@
         <v>Passed</v>
       </c>
       <c r="K83">
-        <v>180</v>
+        <v>219</v>
       </c>
       <c r="L83" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3585,7 +3585,7 @@
         <v>Passed</v>
       </c>
       <c r="K84">
-        <v>292</v>
+        <v>372</v>
       </c>
       <c r="L84" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3623,7 +3623,7 @@
         <v>Passed</v>
       </c>
       <c r="K85">
-        <v>282</v>
+        <v>202</v>
       </c>
       <c r="L85" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3661,7 +3661,7 @@
         <v>Passed</v>
       </c>
       <c r="K86">
-        <v>329</v>
+        <v>242</v>
       </c>
       <c r="L86" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3699,7 +3699,7 @@
         <v>Passed</v>
       </c>
       <c r="K87">
-        <v>227</v>
+        <v>240</v>
       </c>
       <c r="L87" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3737,7 +3737,7 @@
         <v>Passed</v>
       </c>
       <c r="K88">
-        <v>250</v>
+        <v>333</v>
       </c>
       <c r="L88" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3775,7 +3775,7 @@
         <v>Passed</v>
       </c>
       <c r="K89">
-        <v>300</v>
+        <v>364</v>
       </c>
       <c r="L89" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3813,7 +3813,7 @@
         <v>Passed</v>
       </c>
       <c r="K90">
-        <v>290</v>
+        <v>183</v>
       </c>
       <c r="L90" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3851,7 +3851,7 @@
         <v>Passed</v>
       </c>
       <c r="K91">
-        <v>182</v>
+        <v>279</v>
       </c>
       <c r="L91" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3889,7 +3889,7 @@
         <v>Passed</v>
       </c>
       <c r="K92">
-        <v>354</v>
+        <v>300</v>
       </c>
       <c r="L92" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3927,7 +3927,7 @@
         <v>Passed</v>
       </c>
       <c r="K93">
-        <v>383</v>
+        <v>314</v>
       </c>
       <c r="L93" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -3965,7 +3965,7 @@
         <v>Passed</v>
       </c>
       <c r="K94">
-        <v>344</v>
+        <v>320</v>
       </c>
       <c r="L94" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4041,7 +4041,7 @@
         <v>Passed</v>
       </c>
       <c r="K96">
-        <v>354</v>
+        <v>289</v>
       </c>
       <c r="L96" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4079,7 +4079,7 @@
         <v>Passed</v>
       </c>
       <c r="K97">
-        <v>251</v>
+        <v>206</v>
       </c>
       <c r="L97" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4117,7 +4117,7 @@
         <v>Passed</v>
       </c>
       <c r="K98">
-        <v>286</v>
+        <v>346</v>
       </c>
       <c r="L98" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4155,7 +4155,7 @@
         <v>Passed</v>
       </c>
       <c r="K99">
-        <v>181</v>
+        <v>263</v>
       </c>
       <c r="L99" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4193,7 +4193,7 @@
         <v>Passed</v>
       </c>
       <c r="K100">
-        <v>216</v>
+        <v>346</v>
       </c>
       <c r="L100" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4231,7 +4231,7 @@
         <v>Passed</v>
       </c>
       <c r="K101">
-        <v>223</v>
+        <v>373</v>
       </c>
       <c r="L101" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4269,7 +4269,7 @@
         <v>Passed</v>
       </c>
       <c r="K102">
-        <v>212</v>
+        <v>258</v>
       </c>
       <c r="L102" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4307,7 +4307,7 @@
         <v>Passed</v>
       </c>
       <c r="K103">
-        <v>374</v>
+        <v>344</v>
       </c>
       <c r="L103" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4345,7 +4345,7 @@
         <v>Passed</v>
       </c>
       <c r="K104">
-        <v>371</v>
+        <v>354</v>
       </c>
       <c r="L104" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4383,7 +4383,7 @@
         <v>Passed</v>
       </c>
       <c r="K105">
-        <v>296</v>
+        <v>242</v>
       </c>
       <c r="L105" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4421,7 +4421,7 @@
         <v>Passed</v>
       </c>
       <c r="K106">
-        <v>294</v>
+        <v>191</v>
       </c>
       <c r="L106" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4459,7 +4459,7 @@
         <v>Passed</v>
       </c>
       <c r="K107">
-        <v>274</v>
+        <v>280</v>
       </c>
       <c r="L107" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4497,7 +4497,7 @@
         <v>Passed</v>
       </c>
       <c r="K108">
-        <v>394</v>
+        <v>244</v>
       </c>
       <c r="L108" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4535,7 +4535,7 @@
         <v>Passed</v>
       </c>
       <c r="K109">
-        <v>350</v>
+        <v>338</v>
       </c>
       <c r="L109" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4573,7 +4573,7 @@
         <v>Passed</v>
       </c>
       <c r="K110">
-        <v>175</v>
+        <v>252</v>
       </c>
       <c r="L110" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4611,7 +4611,7 @@
         <v>Passed</v>
       </c>
       <c r="K111">
-        <v>236</v>
+        <v>201</v>
       </c>
       <c r="L111" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4649,7 +4649,7 @@
         <v>Passed</v>
       </c>
       <c r="K112">
-        <v>240</v>
+        <v>307</v>
       </c>
       <c r="L112" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4687,7 +4687,7 @@
         <v>Passed</v>
       </c>
       <c r="K113">
-        <v>178</v>
+        <v>190</v>
       </c>
       <c r="L113" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4725,7 +4725,7 @@
         <v>Passed</v>
       </c>
       <c r="K114">
-        <v>153</v>
+        <v>377</v>
       </c>
       <c r="L114" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4763,7 +4763,7 @@
         <v>Passed</v>
       </c>
       <c r="K115">
-        <v>249</v>
+        <v>218</v>
       </c>
       <c r="L115" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4801,7 +4801,7 @@
         <v>Passed</v>
       </c>
       <c r="K116">
-        <v>340</v>
+        <v>329</v>
       </c>
       <c r="L116" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4839,7 +4839,7 @@
         <v>Passed</v>
       </c>
       <c r="K117">
-        <v>164</v>
+        <v>349</v>
       </c>
       <c r="L117" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4877,7 +4877,7 @@
         <v>Passed</v>
       </c>
       <c r="K118">
-        <v>151</v>
+        <v>213</v>
       </c>
       <c r="L118" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4915,7 +4915,7 @@
         <v>Passed</v>
       </c>
       <c r="K119">
-        <v>212</v>
+        <v>311</v>
       </c>
       <c r="L119" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4953,7 +4953,7 @@
         <v>Passed</v>
       </c>
       <c r="K120">
-        <v>161</v>
+        <v>201</v>
       </c>
       <c r="L120" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -4991,7 +4991,7 @@
         <v>Passed</v>
       </c>
       <c r="K121">
-        <v>290</v>
+        <v>269</v>
       </c>
       <c r="L121" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5029,7 +5029,7 @@
         <v>Passed</v>
       </c>
       <c r="K122">
-        <v>391</v>
+        <v>197</v>
       </c>
       <c r="L122" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5067,7 +5067,7 @@
         <v>Passed</v>
       </c>
       <c r="K123">
-        <v>321</v>
+        <v>160</v>
       </c>
       <c r="L123" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5105,7 +5105,7 @@
         <v>Passed</v>
       </c>
       <c r="K124">
-        <v>175</v>
+        <v>243</v>
       </c>
       <c r="L124" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5143,7 +5143,7 @@
         <v>Passed</v>
       </c>
       <c r="K125">
-        <v>218</v>
+        <v>296</v>
       </c>
       <c r="L125" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5181,7 +5181,7 @@
         <v>Passed</v>
       </c>
       <c r="K126">
-        <v>363</v>
+        <v>328</v>
       </c>
       <c r="L126" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5219,7 +5219,7 @@
         <v>Passed</v>
       </c>
       <c r="K127">
-        <v>315</v>
+        <v>373</v>
       </c>
       <c r="L127" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5257,7 +5257,7 @@
         <v>Passed</v>
       </c>
       <c r="K128">
-        <v>363</v>
+        <v>198</v>
       </c>
       <c r="L128" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5295,7 +5295,7 @@
         <v>Passed</v>
       </c>
       <c r="K129">
-        <v>343</v>
+        <v>352</v>
       </c>
       <c r="L129" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5333,7 +5333,7 @@
         <v>Passed</v>
       </c>
       <c r="K130">
-        <v>371</v>
+        <v>304</v>
       </c>
       <c r="L130" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5371,7 +5371,7 @@
         <v>Passed</v>
       </c>
       <c r="K131">
-        <v>153</v>
+        <v>341</v>
       </c>
       <c r="L131" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5409,7 +5409,7 @@
         <v>Passed</v>
       </c>
       <c r="K132">
-        <v>234</v>
+        <v>255</v>
       </c>
       <c r="L132" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5447,7 +5447,7 @@
         <v>Passed</v>
       </c>
       <c r="K133">
-        <v>258</v>
+        <v>212</v>
       </c>
       <c r="L133" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5485,7 +5485,7 @@
         <v>Passed</v>
       </c>
       <c r="K134">
-        <v>341</v>
+        <v>388</v>
       </c>
       <c r="L134" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5523,7 +5523,7 @@
         <v>Passed</v>
       </c>
       <c r="K135">
-        <v>331</v>
+        <v>169</v>
       </c>
       <c r="L135" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5561,7 +5561,7 @@
         <v>Passed</v>
       </c>
       <c r="K136">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="L136" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5599,7 +5599,7 @@
         <v>Passed</v>
       </c>
       <c r="K137">
-        <v>241</v>
+        <v>389</v>
       </c>
       <c r="L137" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5637,7 +5637,7 @@
         <v>Passed</v>
       </c>
       <c r="K138">
-        <v>300</v>
+        <v>340</v>
       </c>
       <c r="L138" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5675,7 +5675,7 @@
         <v>Passed</v>
       </c>
       <c r="K139">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="L139" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5713,7 +5713,7 @@
         <v>Passed</v>
       </c>
       <c r="K140">
-        <v>236</v>
+        <v>338</v>
       </c>
       <c r="L140" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5751,7 +5751,7 @@
         <v>Passed</v>
       </c>
       <c r="K141">
-        <v>379</v>
+        <v>249</v>
       </c>
       <c r="L141" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5789,7 +5789,7 @@
         <v>Passed</v>
       </c>
       <c r="K142">
-        <v>205</v>
+        <v>257</v>
       </c>
       <c r="L142" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5827,7 +5827,7 @@
         <v>Passed</v>
       </c>
       <c r="K143">
-        <v>318</v>
+        <v>247</v>
       </c>
       <c r="L143" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5865,7 +5865,7 @@
         <v>Passed</v>
       </c>
       <c r="K144">
-        <v>364</v>
+        <v>278</v>
       </c>
       <c r="L144" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5903,7 +5903,7 @@
         <v>Passed</v>
       </c>
       <c r="K145">
-        <v>264</v>
+        <v>173</v>
       </c>
       <c r="L145" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5941,7 +5941,7 @@
         <v>Passed</v>
       </c>
       <c r="K146">
-        <v>209</v>
+        <v>329</v>
       </c>
       <c r="L146" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -5979,7 +5979,7 @@
         <v>Passed</v>
       </c>
       <c r="K147">
-        <v>293</v>
+        <v>154</v>
       </c>
       <c r="L147" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6017,7 +6017,7 @@
         <v>Passed</v>
       </c>
       <c r="K148">
-        <v>202</v>
+        <v>303</v>
       </c>
       <c r="L148" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6055,7 +6055,7 @@
         <v>Passed</v>
       </c>
       <c r="K149">
-        <v>281</v>
+        <v>247</v>
       </c>
       <c r="L149" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6093,7 +6093,7 @@
         <v>Passed</v>
       </c>
       <c r="K150">
-        <v>257</v>
+        <v>242</v>
       </c>
       <c r="L150" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6131,7 +6131,7 @@
         <v>Passed</v>
       </c>
       <c r="K151">
-        <v>377</v>
+        <v>304</v>
       </c>
       <c r="L151" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6169,7 +6169,7 @@
         <v>Passed</v>
       </c>
       <c r="K152">
-        <v>276</v>
+        <v>397</v>
       </c>
       <c r="L152" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6207,7 +6207,7 @@
         <v>Passed</v>
       </c>
       <c r="K153">
-        <v>245</v>
+        <v>321</v>
       </c>
       <c r="L153" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6245,7 +6245,7 @@
         <v>Passed</v>
       </c>
       <c r="K154">
-        <v>263</v>
+        <v>303</v>
       </c>
       <c r="L154" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6283,7 +6283,7 @@
         <v>Passed</v>
       </c>
       <c r="K155">
-        <v>334</v>
+        <v>172</v>
       </c>
       <c r="L155" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6321,7 +6321,7 @@
         <v>Passed</v>
       </c>
       <c r="K156">
-        <v>304</v>
+        <v>251</v>
       </c>
       <c r="L156" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6359,7 +6359,7 @@
         <v>Passed</v>
       </c>
       <c r="K157">
-        <v>258</v>
+        <v>351</v>
       </c>
       <c r="L157" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6397,7 +6397,7 @@
         <v>Passed</v>
       </c>
       <c r="K158">
-        <v>299</v>
+        <v>357</v>
       </c>
       <c r="L158" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6435,7 +6435,7 @@
         <v>Passed</v>
       </c>
       <c r="K159">
-        <v>311</v>
+        <v>172</v>
       </c>
       <c r="L159" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6473,7 +6473,7 @@
         <v>Passed</v>
       </c>
       <c r="K160">
-        <v>349</v>
+        <v>229</v>
       </c>
       <c r="L160" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6511,7 +6511,7 @@
         <v>Passed</v>
       </c>
       <c r="K161">
-        <v>380</v>
+        <v>351</v>
       </c>
       <c r="L161" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6549,7 +6549,7 @@
         <v>Passed</v>
       </c>
       <c r="K162">
-        <v>387</v>
+        <v>190</v>
       </c>
       <c r="L162" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6587,7 +6587,7 @@
         <v>Passed</v>
       </c>
       <c r="K163">
-        <v>297</v>
+        <v>162</v>
       </c>
       <c r="L163" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6625,7 +6625,7 @@
         <v>Passed</v>
       </c>
       <c r="K164">
-        <v>373</v>
+        <v>397</v>
       </c>
       <c r="L164" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6663,7 +6663,7 @@
         <v>Passed</v>
       </c>
       <c r="K165">
-        <v>355</v>
+        <v>347</v>
       </c>
       <c r="L165" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6701,7 +6701,7 @@
         <v>Passed</v>
       </c>
       <c r="K166">
-        <v>238</v>
+        <v>266</v>
       </c>
       <c r="L166" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6739,7 +6739,7 @@
         <v>Passed</v>
       </c>
       <c r="K167">
-        <v>189</v>
+        <v>203</v>
       </c>
       <c r="L167" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6777,7 +6777,7 @@
         <v>Passed</v>
       </c>
       <c r="K168">
-        <v>263</v>
+        <v>158</v>
       </c>
       <c r="L168" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6815,7 +6815,7 @@
         <v>Passed</v>
       </c>
       <c r="K169">
-        <v>338</v>
+        <v>235</v>
       </c>
       <c r="L169" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6853,7 +6853,7 @@
         <v>Passed</v>
       </c>
       <c r="K170">
-        <v>343</v>
+        <v>310</v>
       </c>
       <c r="L170" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6891,7 +6891,7 @@
         <v>Passed</v>
       </c>
       <c r="K171">
-        <v>367</v>
+        <v>178</v>
       </c>
       <c r="L171" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -6929,7 +6929,7 @@
         <v>Passed</v>
       </c>
       <c r="K172">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="L172" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7005,7 +7005,7 @@
         <v>Passed</v>
       </c>
       <c r="K174">
-        <v>314</v>
+        <v>390</v>
       </c>
       <c r="L174" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7043,7 +7043,7 @@
         <v>Passed</v>
       </c>
       <c r="K175">
-        <v>348</v>
+        <v>276</v>
       </c>
       <c r="L175" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7081,7 +7081,7 @@
         <v>Passed</v>
       </c>
       <c r="K176">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="L176" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7119,7 +7119,7 @@
         <v>Passed</v>
       </c>
       <c r="K177">
-        <v>378</v>
+        <v>242</v>
       </c>
       <c r="L177" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7157,7 +7157,7 @@
         <v>Passed</v>
       </c>
       <c r="K178">
-        <v>367</v>
+        <v>188</v>
       </c>
       <c r="L178" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7195,7 +7195,7 @@
         <v>Passed</v>
       </c>
       <c r="K179">
-        <v>225</v>
+        <v>273</v>
       </c>
       <c r="L179" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7233,7 +7233,7 @@
         <v>Passed</v>
       </c>
       <c r="K180">
-        <v>373</v>
+        <v>213</v>
       </c>
       <c r="L180" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7271,7 +7271,7 @@
         <v>Passed</v>
       </c>
       <c r="K181">
-        <v>230</v>
+        <v>368</v>
       </c>
       <c r="L181" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7309,7 +7309,7 @@
         <v>Passed</v>
       </c>
       <c r="K182">
-        <v>250</v>
+        <v>224</v>
       </c>
       <c r="L182" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7347,7 +7347,7 @@
         <v>Passed</v>
       </c>
       <c r="K183">
-        <v>156</v>
+        <v>268</v>
       </c>
       <c r="L183" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7385,7 +7385,7 @@
         <v>Passed</v>
       </c>
       <c r="K184">
-        <v>244</v>
+        <v>165</v>
       </c>
       <c r="L184" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7423,7 +7423,7 @@
         <v>Passed</v>
       </c>
       <c r="K185">
-        <v>152</v>
+        <v>260</v>
       </c>
       <c r="L185" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7461,7 +7461,7 @@
         <v>Passed</v>
       </c>
       <c r="K186">
-        <v>150</v>
+        <v>282</v>
       </c>
       <c r="L186" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7499,7 +7499,7 @@
         <v>Passed</v>
       </c>
       <c r="K187">
-        <v>281</v>
+        <v>347</v>
       </c>
       <c r="L187" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7537,7 +7537,7 @@
         <v>Passed</v>
       </c>
       <c r="K188">
-        <v>370</v>
+        <v>301</v>
       </c>
       <c r="L188" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7575,7 +7575,7 @@
         <v>Passed</v>
       </c>
       <c r="K189">
-        <v>377</v>
+        <v>262</v>
       </c>
       <c r="L189" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7613,7 +7613,7 @@
         <v>Passed</v>
       </c>
       <c r="K190">
-        <v>153</v>
+        <v>320</v>
       </c>
       <c r="L190" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7651,7 +7651,7 @@
         <v>Passed</v>
       </c>
       <c r="K191">
-        <v>380</v>
+        <v>391</v>
       </c>
       <c r="L191" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7689,7 +7689,7 @@
         <v>Passed</v>
       </c>
       <c r="K192">
-        <v>164</v>
+        <v>238</v>
       </c>
       <c r="L192" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7727,7 +7727,7 @@
         <v>Passed</v>
       </c>
       <c r="K193">
-        <v>310</v>
+        <v>384</v>
       </c>
       <c r="L193" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7765,7 +7765,7 @@
         <v>Passed</v>
       </c>
       <c r="K194">
-        <v>248</v>
+        <v>309</v>
       </c>
       <c r="L194" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7803,7 +7803,7 @@
         <v>Passed</v>
       </c>
       <c r="K195">
-        <v>358</v>
+        <v>314</v>
       </c>
       <c r="L195" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7841,7 +7841,7 @@
         <v>Passed</v>
       </c>
       <c r="K196">
-        <v>231</v>
+        <v>381</v>
       </c>
       <c r="L196" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7879,7 +7879,7 @@
         <v>Passed</v>
       </c>
       <c r="K197">
-        <v>255</v>
+        <v>264</v>
       </c>
       <c r="L197" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7917,7 +7917,7 @@
         <v>Passed</v>
       </c>
       <c r="K198">
-        <v>162</v>
+        <v>292</v>
       </c>
       <c r="L198" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7955,7 +7955,7 @@
         <v>Passed</v>
       </c>
       <c r="K199">
-        <v>310</v>
+        <v>254</v>
       </c>
       <c r="L199" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -7993,7 +7993,7 @@
         <v>Passed</v>
       </c>
       <c r="K200">
-        <v>249</v>
+        <v>194</v>
       </c>
       <c r="L200" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8031,7 +8031,7 @@
         <v>Passed</v>
       </c>
       <c r="K201">
-        <v>273</v>
+        <v>238</v>
       </c>
       <c r="L201" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8069,7 +8069,7 @@
         <v>Passed</v>
       </c>
       <c r="K202">
-        <v>314</v>
+        <v>338</v>
       </c>
       <c r="L202" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8107,7 +8107,7 @@
         <v>Passed</v>
       </c>
       <c r="K203">
-        <v>150</v>
+        <v>199</v>
       </c>
       <c r="L203" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8145,7 +8145,7 @@
         <v>Passed</v>
       </c>
       <c r="K204">
-        <v>395</v>
+        <v>230</v>
       </c>
       <c r="L204" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8183,7 +8183,7 @@
         <v>Passed</v>
       </c>
       <c r="K205">
-        <v>208</v>
+        <v>258</v>
       </c>
       <c r="L205" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8221,7 +8221,7 @@
         <v>Passed</v>
       </c>
       <c r="K206">
-        <v>287</v>
+        <v>313</v>
       </c>
       <c r="L206" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8259,7 +8259,7 @@
         <v>Passed</v>
       </c>
       <c r="K207">
-        <v>336</v>
+        <v>325</v>
       </c>
       <c r="L207" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8297,7 +8297,7 @@
         <v>Passed</v>
       </c>
       <c r="K208">
-        <v>261</v>
+        <v>227</v>
       </c>
       <c r="L208" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8335,7 +8335,7 @@
         <v>Passed</v>
       </c>
       <c r="K209">
-        <v>379</v>
+        <v>257</v>
       </c>
       <c r="L209" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8373,7 +8373,7 @@
         <v>Passed</v>
       </c>
       <c r="K210">
-        <v>190</v>
+        <v>199</v>
       </c>
       <c r="L210" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8411,7 +8411,7 @@
         <v>Passed</v>
       </c>
       <c r="K211">
-        <v>269</v>
+        <v>213</v>
       </c>
       <c r="L211" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8449,7 +8449,7 @@
         <v>Passed</v>
       </c>
       <c r="K212">
-        <v>245</v>
+        <v>212</v>
       </c>
       <c r="L212" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8487,7 +8487,7 @@
         <v>Passed</v>
       </c>
       <c r="K213">
-        <v>289</v>
+        <v>242</v>
       </c>
       <c r="L213" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8525,7 +8525,7 @@
         <v>Passed</v>
       </c>
       <c r="K214">
-        <v>230</v>
+        <v>173</v>
       </c>
       <c r="L214" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8563,7 +8563,7 @@
         <v>Passed</v>
       </c>
       <c r="K215">
-        <v>318</v>
+        <v>203</v>
       </c>
       <c r="L215" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8601,7 +8601,7 @@
         <v>Passed</v>
       </c>
       <c r="K216">
-        <v>278</v>
+        <v>182</v>
       </c>
       <c r="L216" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8639,7 +8639,7 @@
         <v>Passed</v>
       </c>
       <c r="K217">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="L217" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8677,7 +8677,7 @@
         <v>Passed</v>
       </c>
       <c r="K218">
-        <v>246</v>
+        <v>338</v>
       </c>
       <c r="L218" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8715,7 +8715,7 @@
         <v>Passed</v>
       </c>
       <c r="K219">
-        <v>389</v>
+        <v>152</v>
       </c>
       <c r="L219" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8753,7 +8753,7 @@
         <v>Passed</v>
       </c>
       <c r="K220">
-        <v>309</v>
+        <v>329</v>
       </c>
       <c r="L220" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8791,7 +8791,7 @@
         <v>Passed</v>
       </c>
       <c r="K221">
-        <v>191</v>
+        <v>245</v>
       </c>
       <c r="L221" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8829,7 +8829,7 @@
         <v>Passed</v>
       </c>
       <c r="K222">
-        <v>152</v>
+        <v>177</v>
       </c>
       <c r="L222" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8867,7 +8867,7 @@
         <v>Passed</v>
       </c>
       <c r="K223">
-        <v>259</v>
+        <v>358</v>
       </c>
       <c r="L223" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8905,7 +8905,7 @@
         <v>Passed</v>
       </c>
       <c r="K224">
-        <v>348</v>
+        <v>395</v>
       </c>
       <c r="L224" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8943,7 +8943,7 @@
         <v>Passed</v>
       </c>
       <c r="K225">
-        <v>313</v>
+        <v>334</v>
       </c>
       <c r="L225" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -8981,7 +8981,7 @@
         <v>Passed</v>
       </c>
       <c r="K226">
-        <v>369</v>
+        <v>203</v>
       </c>
       <c r="L226" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9019,7 +9019,7 @@
         <v>Passed</v>
       </c>
       <c r="K227">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="L227" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9057,7 +9057,7 @@
         <v>Passed</v>
       </c>
       <c r="K228">
-        <v>229</v>
+        <v>150</v>
       </c>
       <c r="L228" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9095,7 +9095,7 @@
         <v>Passed</v>
       </c>
       <c r="K229">
-        <v>322</v>
+        <v>355</v>
       </c>
       <c r="L229" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9133,7 +9133,7 @@
         <v>Passed</v>
       </c>
       <c r="K230">
-        <v>180</v>
+        <v>318</v>
       </c>
       <c r="L230" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9171,7 +9171,7 @@
         <v>Passed</v>
       </c>
       <c r="K231">
-        <v>332</v>
+        <v>351</v>
       </c>
       <c r="L231" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9209,7 +9209,7 @@
         <v>Passed</v>
       </c>
       <c r="K232">
-        <v>329</v>
+        <v>152</v>
       </c>
       <c r="L232" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9247,7 +9247,7 @@
         <v>Passed</v>
       </c>
       <c r="K233">
-        <v>170</v>
+        <v>332</v>
       </c>
       <c r="L233" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9285,7 +9285,7 @@
         <v>Passed</v>
       </c>
       <c r="K234">
-        <v>169</v>
+        <v>189</v>
       </c>
       <c r="L234" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9323,7 +9323,7 @@
         <v>Passed</v>
       </c>
       <c r="K235">
-        <v>240</v>
+        <v>374</v>
       </c>
       <c r="L235" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9361,7 +9361,7 @@
         <v>Passed</v>
       </c>
       <c r="K236">
-        <v>281</v>
+        <v>322</v>
       </c>
       <c r="L236" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9399,7 +9399,7 @@
         <v>Passed</v>
       </c>
       <c r="K237">
-        <v>312</v>
+        <v>241</v>
       </c>
       <c r="L237" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9437,7 +9437,7 @@
         <v>Passed</v>
       </c>
       <c r="K238">
-        <v>197</v>
+        <v>284</v>
       </c>
       <c r="L238" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9475,7 +9475,7 @@
         <v>Passed</v>
       </c>
       <c r="K239">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="L239" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9513,7 +9513,7 @@
         <v>Passed</v>
       </c>
       <c r="K240">
-        <v>340</v>
+        <v>254</v>
       </c>
       <c r="L240" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9551,7 +9551,7 @@
         <v>Passed</v>
       </c>
       <c r="K241">
-        <v>193</v>
+        <v>319</v>
       </c>
       <c r="L241" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9589,7 +9589,7 @@
         <v>Passed</v>
       </c>
       <c r="K242">
-        <v>324</v>
+        <v>353</v>
       </c>
       <c r="L242" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9627,7 +9627,7 @@
         <v>Passed</v>
       </c>
       <c r="K243">
-        <v>319</v>
+        <v>377</v>
       </c>
       <c r="L243" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9665,7 +9665,7 @@
         <v>Passed</v>
       </c>
       <c r="K244">
-        <v>253</v>
+        <v>293</v>
       </c>
       <c r="L244" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9703,7 +9703,7 @@
         <v>Passed</v>
       </c>
       <c r="K245">
-        <v>326</v>
+        <v>310</v>
       </c>
       <c r="L245" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9741,7 +9741,7 @@
         <v>Passed</v>
       </c>
       <c r="K246">
-        <v>367</v>
+        <v>229</v>
       </c>
       <c r="L246" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9779,7 +9779,7 @@
         <v>Passed</v>
       </c>
       <c r="K247">
-        <v>244</v>
+        <v>183</v>
       </c>
       <c r="L247" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9817,7 +9817,7 @@
         <v>Passed</v>
       </c>
       <c r="K248">
-        <v>252</v>
+        <v>214</v>
       </c>
       <c r="L248" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9855,7 +9855,7 @@
         <v>Passed</v>
       </c>
       <c r="K249">
-        <v>397</v>
+        <v>162</v>
       </c>
       <c r="L249" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9893,7 +9893,7 @@
         <v>Passed</v>
       </c>
       <c r="K250">
-        <v>249</v>
+        <v>392</v>
       </c>
       <c r="L250" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9931,7 +9931,7 @@
         <v>Passed</v>
       </c>
       <c r="K251">
-        <v>328</v>
+        <v>223</v>
       </c>
       <c r="L251" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -9969,7 +9969,7 @@
         <v>Passed</v>
       </c>
       <c r="K252">
-        <v>184</v>
+        <v>162</v>
       </c>
       <c r="L252" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10007,7 +10007,7 @@
         <v>Passed</v>
       </c>
       <c r="K253">
-        <v>321</v>
+        <v>249</v>
       </c>
       <c r="L253" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10045,7 +10045,7 @@
         <v>Passed</v>
       </c>
       <c r="K254">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="L254" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10083,7 +10083,7 @@
         <v>Passed</v>
       </c>
       <c r="K255">
-        <v>241</v>
+        <v>355</v>
       </c>
       <c r="L255" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10121,7 +10121,7 @@
         <v>Passed</v>
       </c>
       <c r="K256">
-        <v>282</v>
+        <v>258</v>
       </c>
       <c r="L256" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10159,7 +10159,7 @@
         <v>Passed</v>
       </c>
       <c r="K257">
-        <v>283</v>
+        <v>397</v>
       </c>
       <c r="L257" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10197,7 +10197,7 @@
         <v>Passed</v>
       </c>
       <c r="K258">
-        <v>336</v>
+        <v>393</v>
       </c>
       <c r="L258" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10235,7 +10235,7 @@
         <v>Passed</v>
       </c>
       <c r="K259">
-        <v>150</v>
+        <v>255</v>
       </c>
       <c r="L259" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10273,7 +10273,7 @@
         <v>Passed</v>
       </c>
       <c r="K260">
-        <v>168</v>
+        <v>357</v>
       </c>
       <c r="L260" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10311,7 +10311,7 @@
         <v>Passed</v>
       </c>
       <c r="K261">
-        <v>163</v>
+        <v>326</v>
       </c>
       <c r="L261" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10349,7 +10349,7 @@
         <v>Passed</v>
       </c>
       <c r="K262">
-        <v>177</v>
+        <v>209</v>
       </c>
       <c r="L262" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10387,7 +10387,7 @@
         <v>Passed</v>
       </c>
       <c r="K263">
-        <v>308</v>
+        <v>380</v>
       </c>
       <c r="L263" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10425,7 +10425,7 @@
         <v>Passed</v>
       </c>
       <c r="K264">
-        <v>289</v>
+        <v>157</v>
       </c>
       <c r="L264" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10463,7 +10463,7 @@
         <v>Passed</v>
       </c>
       <c r="K265">
-        <v>275</v>
+        <v>220</v>
       </c>
       <c r="L265" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10501,7 +10501,7 @@
         <v>Passed</v>
       </c>
       <c r="K266">
-        <v>352</v>
+        <v>356</v>
       </c>
       <c r="L266" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10539,7 +10539,7 @@
         <v>Passed</v>
       </c>
       <c r="K267">
-        <v>227</v>
+        <v>342</v>
       </c>
       <c r="L267" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10577,7 +10577,7 @@
         <v>Passed</v>
       </c>
       <c r="K268">
-        <v>225</v>
+        <v>326</v>
       </c>
       <c r="L268" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10615,7 +10615,7 @@
         <v>Passed</v>
       </c>
       <c r="K269">
-        <v>254</v>
+        <v>242</v>
       </c>
       <c r="L269" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10653,7 +10653,7 @@
         <v>Passed</v>
       </c>
       <c r="K270">
-        <v>383</v>
+        <v>279</v>
       </c>
       <c r="L270" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10691,7 +10691,7 @@
         <v>Passed</v>
       </c>
       <c r="K271">
-        <v>156</v>
+        <v>365</v>
       </c>
       <c r="L271" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10729,7 +10729,7 @@
         <v>Passed</v>
       </c>
       <c r="K272">
-        <v>335</v>
+        <v>365</v>
       </c>
       <c r="L272" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10767,7 +10767,7 @@
         <v>Passed</v>
       </c>
       <c r="K273">
-        <v>309</v>
+        <v>396</v>
       </c>
       <c r="L273" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10805,7 +10805,7 @@
         <v>Passed</v>
       </c>
       <c r="K274">
-        <v>219</v>
+        <v>253</v>
       </c>
       <c r="L274" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10843,7 +10843,7 @@
         <v>Passed</v>
       </c>
       <c r="K275">
-        <v>268</v>
+        <v>207</v>
       </c>
       <c r="L275" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10881,7 +10881,7 @@
         <v>Passed</v>
       </c>
       <c r="K276">
-        <v>216</v>
+        <v>269</v>
       </c>
       <c r="L276" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10919,7 +10919,7 @@
         <v>Passed</v>
       </c>
       <c r="K277">
-        <v>299</v>
+        <v>254</v>
       </c>
       <c r="L277" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10957,7 +10957,7 @@
         <v>Passed</v>
       </c>
       <c r="K278">
-        <v>203</v>
+        <v>397</v>
       </c>
       <c r="L278" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -10995,7 +10995,7 @@
         <v>Passed</v>
       </c>
       <c r="K279">
-        <v>392</v>
+        <v>333</v>
       </c>
       <c r="L279" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11033,7 +11033,7 @@
         <v>Passed</v>
       </c>
       <c r="K280">
-        <v>235</v>
+        <v>211</v>
       </c>
       <c r="L280" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11071,7 +11071,7 @@
         <v>Passed</v>
       </c>
       <c r="K281">
-        <v>286</v>
+        <v>297</v>
       </c>
       <c r="L281" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11109,7 +11109,7 @@
         <v>Passed</v>
       </c>
       <c r="K282">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="L282" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11147,7 +11147,7 @@
         <v>Passed</v>
       </c>
       <c r="K283">
-        <v>276</v>
+        <v>251</v>
       </c>
       <c r="L283" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11185,7 +11185,7 @@
         <v>Passed</v>
       </c>
       <c r="K284">
-        <v>172</v>
+        <v>162</v>
       </c>
       <c r="L284" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11223,7 +11223,7 @@
         <v>Passed</v>
       </c>
       <c r="K285">
-        <v>355</v>
+        <v>270</v>
       </c>
       <c r="L285" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11261,7 +11261,7 @@
         <v>Passed</v>
       </c>
       <c r="K286">
-        <v>370</v>
+        <v>296</v>
       </c>
       <c r="L286" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11299,7 +11299,7 @@
         <v>Passed</v>
       </c>
       <c r="K287">
-        <v>298</v>
+        <v>195</v>
       </c>
       <c r="L287" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11337,7 +11337,7 @@
         <v>Passed</v>
       </c>
       <c r="K288">
-        <v>318</v>
+        <v>332</v>
       </c>
       <c r="L288" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11375,7 +11375,7 @@
         <v>Passed</v>
       </c>
       <c r="K289">
-        <v>341</v>
+        <v>309</v>
       </c>
       <c r="L289" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11413,7 +11413,7 @@
         <v>Passed</v>
       </c>
       <c r="K290">
-        <v>331</v>
+        <v>337</v>
       </c>
       <c r="L290" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11451,7 +11451,7 @@
         <v>Passed</v>
       </c>
       <c r="K291">
-        <v>386</v>
+        <v>264</v>
       </c>
       <c r="L291" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11489,7 +11489,7 @@
         <v>Passed</v>
       </c>
       <c r="K292">
-        <v>203</v>
+        <v>324</v>
       </c>
       <c r="L292" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11527,7 +11527,7 @@
         <v>Passed</v>
       </c>
       <c r="K293">
-        <v>159</v>
+        <v>340</v>
       </c>
       <c r="L293" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11565,7 +11565,7 @@
         <v>Passed</v>
       </c>
       <c r="K294">
-        <v>262</v>
+        <v>237</v>
       </c>
       <c r="L294" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11603,7 +11603,7 @@
         <v>Passed</v>
       </c>
       <c r="K295">
-        <v>211</v>
+        <v>221</v>
       </c>
       <c r="L295" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11641,7 +11641,7 @@
         <v>Passed</v>
       </c>
       <c r="K296">
-        <v>384</v>
+        <v>309</v>
       </c>
       <c r="L296" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11679,7 +11679,7 @@
         <v>Passed</v>
       </c>
       <c r="K297">
-        <v>311</v>
+        <v>191</v>
       </c>
       <c r="L297" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11717,7 +11717,7 @@
         <v>Passed</v>
       </c>
       <c r="K298">
-        <v>240</v>
+        <v>373</v>
       </c>
       <c r="L298" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11755,7 +11755,7 @@
         <v>Passed</v>
       </c>
       <c r="K299">
-        <v>219</v>
+        <v>399</v>
       </c>
       <c r="L299" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11793,7 +11793,7 @@
         <v>Passed</v>
       </c>
       <c r="K300">
-        <v>331</v>
+        <v>398</v>
       </c>
       <c r="L300" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>
@@ -11831,7 +11831,7 @@
         <v>Passed</v>
       </c>
       <c r="K301">
-        <v>244</v>
+        <v>320</v>
       </c>
       <c r="L301" t="str">
         <v>Appium UiAutomator2 / XCUITest</v>

</xml_diff>